<commit_message>
chore: ensure punkt corpora available for TextBlob/NRCLex
</commit_message>
<xml_diff>
--- a/notebooks/merged_stock_news.xlsx
+++ b/notebooks/merged_stock_news.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,7 +593,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>why you should get your boot to beyonces cowboy carter tour a sermon for the weary while you can chinese battery giant and tesla supplier catl is expanding globally here why it matter how to stay on top of google search faraday x preparation are in the final stage for the private preview and cocreation launch event on june th for the groundbreaking fx super one mpv biocon biologics receives health canada approval for yesafilitm aflibercept first global launch scheduled for july china factory activity expected to shrink for third month amid trade tension reuters poll nike vomero quietly became a million franchise in day a ceo say it time to turn the page investor gary black cheer afterhours rally ap technology summarybrief at am edt ap technology summarybrief at am edt ap technology summarybrief at am edt ap technology summarybrief at am edt amazon google not far behind but dan ives say microsoft clearly leading in these segment price target is probably conservative why your to feel more like report say analysisin dovish tilt boj zoom in on obscure underlying inflation trend find the best crypto to join for emerging project reshaping the digital economy tesla shakeup who is omead afshar senior executive reportedly fired by elon musk amid slumping sale i time of india ap business summarybrief at am edt ap business summarybrief at am edt asian share are mostly higher after u stock rise to the brink of a record trump tariff have unsettled thailand pet food exporter germany tell apple google to block deepseek a the chinese ai app face rising pressure in europe hugging face cofounder challenge ai optimist model cant ask original scientific question you might not have bezoslevel buck but you still might consider a prenup vertex founder boger donates m to boston art academy trump big beautiful bill might be unloved and a mess but it will still probably pas here how the luxury real estate market is splitting up how company profit from your data without consent full circle boy leap forward with debut ep jete and official music video this go out to you out now increase of share capital in connection with realization of the employee option programm and subscription result more than an ev charger it peace of mind wherever the road take you cutting u energy credit doesnt save money it steal it from ratepayer local government ansi officially approves two new seia standard on consumer protection and operation and maintenance kymera therapeutic announces pricing of million public offering kymera therapeutic announces pricing of million public offering solaredge expands u manufacturing in salt lake city utah why denver homeowner are investing more in renovation project leap power national grid virtual power plant initiative in massachusetts hawaiian airline report cybersecurity event no flight disruption kitv boeing dreamliner black box recovered data under scrutiny to provide insight into fatal air india crash cso receives grant from mt charitable foundation achieve life science announces pricing of million underwritten public offering the mobility house and schneider electric unveil solar charging depot for turlock unifieds electric school bus fleet trump crypto advisor david sack say july will be a big month say president support legislation on market structure and stablecoins amazon grocery chief blame ridiculous red tape for holding back initiative at whole food were wasting time year old driver from tripura treated with eastern india firstever bachmanns bundle pacing vdh in the end everyone hated the iranian theocracy oklahoma governor kevin stitt and u secretary of health and human service robert f kennedy jr visit mom meal to highlight food a medicine leadership japan executes twitter killer who murdered and dismembered nine people saratoga county celebrates m airport revitalization ap business summarybrief at pm edt ap business summarybrief at pm edt ap business summarybrief at pm edt ap business summarybrief at pm edt ap technology summarybrief at pm edt driver crash nearly plummet over san mateo county cliff north korea just opened a beach resort for people but who will visit jeep gladiator rank first in midsize pickup segment in jd power u initial quality study chrysler jeep and dodge brand improve iq score over thailand will hold trade talk with u next week finance minister say meta say it winning the talent war with openai the verge china u agree on detail of london trade framework beijing say saratogians remember mark straus a pioneer sp cut colombia debt rating to bb over declining fiscal result why lumen technology stock wa winning this week annovis bio to present key finding at alzheimers association international conference iraq war veteran hegseths news conference wa conduct unbecoming chinese influence in climate change lawsuit threatens to derail u energy industry asia fx muted dollar struggle at yr low with pce data on tap demolition start at former kera hq clearing way for new uptown tower european stock extend gain after white house hint at tariff extension baseball player wander franco found guilty in sexual abuse case imposed twoyear suspended sentence china skirt u sanction a top buyer of iranian oil here how and why thats unlikely to change soon china may industrial profit slip back into sharp decline reuters gold head for weekly loss a middle east truce sap demand uk auto production for may slump to lowest level since a trump tariff hit hard mgi announces partnership with negedia enhance genomic sequencing technology at the service of scientific research and precision medicine in italy mgi announces partnership with negedia enhance genomic sequencing technology at the service of scientific research and precision medicine in italy informal mining boom is biggest fear for peru copper investor best cryptos to buy now one already up and climbing bill gate say he know for a fact that more child will die due to u health aid cut and he taking the proof to congress cancer patient recover by taking repurposed antiparasitic drug india economy to hold top spot for growth but underlying weakness remain reuters poll cnbc daily open wall street is tuning out the noise and catching ray turkish farmer pioneer xag agricultural drone for watersmart practice treasury yield inch higher a investor await the fed preferred inflation print bitcoin ethereum rangebound dogecoin dip amid potential july tariff deadline extension analyst predicts btcs next big move once it break out of this range softbank ceo say he all in on openai reveals he long wanted microsofts spot a main backer mexico investigating contamination from spacex explosion debris sandia national laboratory to cut up to workforce by early fall canada approves law to fasttrack resource project face indigenous opposition lithium industry bemoans paradox of low price rising demand china industrial profit slip back into sharp decline in may two north texas school board increase teacher pay in final budget confusion a trump say deal with china signed yet both side violate term of ceasefire share rally but dollar weakens with fed independence seen under threat courtney b vance on book ban protest in los angeles and narrating the audiobook of the biography of web du bois atlantic strategic mineral start commercial production at virginia operation u food and drug administration approves streamlined patient monitoring requirement and removal of rem program within bristol myers squibbs cell therapy label u food and drug administration approves streamlined patient monitoring requirement and removal of rem program within bristol myers squibbs cell therapy label u food and drug administration approves streamlined patient monitoring requirement and removal of rem program within bristol myers squibbs cell therapy label u food and drug administration approves streamlined patient monitoring requirement and removal of rem program within bristol myers squibbs cell therapy label why you should get your boot to beyonces cowboy carter tour a sermon for the weary while you can clarence page did you miss a holiday mr president arthur cyr bombing iran mideast stability and the role of the u former minnesota house speaker melissa hortman to lie in state a suspect face court date former minnesota house speaker melissa hortman to lie in state a suspect face court date democrat are trying to figure out what to do about john fetterman one of them is stepping up democrat are trying to figure out what to do about john fetterman one of them is stepping up democrat are trying to figure out what to do about john fetterman one of them is stepping up supreme court meet friday to decide remaining case including birthright citizenship supreme court meet friday to decide remaining case including birthright citizenship supreme court meet friday to decide remaining case including birthright citizenship supreme court meet friday to decide remaining case including birthright citizenship you might not have bezoslevel buck but you still might consider a prenup summer league basketball islander rattler trump big beautiful bill might be unloved and a mess but it will still probably pas edward d shanshala ii billion in waste fraud and abuse maybe but look in the right place editorial go slow on waymo several caution before selfdriving car arrive rev allison palm rev jonathan hopkins gov ayotte reneged on promise to meet with faith leader senator diverge sharply on damage done by iran strike after classified briefing japan executes twitter killer who murdered and dismembered nine people oregon senate vote to override governor veto a first since dallas place future of the franchise in cooper flagg a southwest division get better north korea just opened a beach resort for people but who will visit panton named johnstown knox elementary school principal former top aide to jill biden subpoenaed in house gop biden age probe iraq war veteran hegseths news conference wa conduct unbecoming selling public land isnt the answer to affordable housing title lx protection matter more than ever trump appointing a shadow chair at the fed ha put dollar under pressure meanwhile china is dumping the greenback and hoarding gold baseball player wander franco found guilty in sexual abuse case imposed twoyear suspended sentence abbott trump approval rating poll show economy thc reduce favorability among texan family file for release in lawsuit considered first involving child challenging arrest at court family file for release in lawsuit considered first involving child challenging arrest at court family sue over u detention in what may be first challenge to courthouse arrest involving kid gov ferguson warns medicaid cut could devastate washington health care system review gloversvilles stump city brewing is modern version of oldtime public house pintsized louisiana is latest state to redefine natural gas a planetwarming fossil fuel a green energy change coming for wilco voter courtney b vance on book ban protest in los angeles and narrating the audiobook of the biography of web du bois critical rce flaw in cisco ise and isepic allow unauthenticated attacker to gain root access pete hegseth air medium coverage grievance towards cnn and others the latest pretrial development in the idaho student killing case green leader larissa water on holding the labor government to account australian politics podcast labor must protect environment while rewriting law written to facilitate development larissa water say wife of minnesota suspect say she wa blindsided by shooting of state politician cnn this is your brain on chatgpt white house confirms u china have reached additional trade agreement trump threatens cnn and new york time with lawsuit over iran report senate parliamentarian ok gop cut to federal food assistance former trail blazer ben mclemore say sex wa consensual while taking the stand during rape trial woman accused of stealing from jewelry store in washington oregon former defense secy iranian nuclear facility damage assessment will take week community rally in massive show of support for caesar palace time square u tariff may sideline youth sport for many family making it harder for kid to stay active rep josh gottheimer american dont like trump big policy bill court issue opinion on centennial at tejon ranch cnn medium analyst responds to false attack on iranian nuclear site report let go through it zohran mamdani tell erin burnett how he plan to pay for his policy fireball fly across the sky and cause sonic boom america controversial iran airstrike letter to the editor june china on alert a nato boost defense spending mamdani vow to stand up to trump border czar and ice canadian official press u government for detail on canadian citizen who died in ice custody at a florida detention center former montana u rep pat williams who won a liberal conservative showdown dy at portland city council pass resolution to strengthen portland street response a look at legal threat facing samesex marriage year after obergefell decision it judgement time for john thune on the big beautiful bill guest commentary rtc targeting senior with displacement former pantagraph building get positive recommendation for landmark status eu leader on wto we need to come up with something else senate democrat question obliteration of iran nuclear site after classified briefing on strike officer placed on leave after shooting in bangor at least orgs urge senator to support iran war power resolution lawsuit filed on behalf of nex benedict estate against owasso public school trump spotlight parent who have lost kid due to open border during big beautiful bill event former trump lawyer kenneth chesebro disbarred in new york over election interference case donald trump say uschina trade truce ha been signed hegseth defends success of u strike on iran nuclear site amid doubt over impact standing up to bullying unscientific transgender activist mob canadian man held by immigration official dy in south florida federal facility official say canadian man held by immigration official dy in south florida federal facility official say canadian man held by immigration official dy in south florida federal facility official say canadian man held by immigration official dy in south florida federal facility official say canadian man held by immigration official dy in south florida federal facility official say canadian man held by immigration official dy in south florida federal facility official say illinois gov jb pritzker announces bid for historic third term amidst presidential buzz interior secretary doug burgum answer question about the big beautiful bill and public land trump doj is targeting daily ko agent mental health passport led to push for secured bond famous preston night rodeo gearing up for it th annual community experience plan unveiled for story link at boca at west yamato road in boca raton fact check trump make big false claim about his big domestic policy bill biogen genentech may stay mum on damage at trial inside the trading desk that surfed day of oil market mayhem bloomberg trader bet on interest rate cut from jay powell successor at the fed financial time etf are booming mutual fund want in on the action analyst amd stock will close the gap with nvidia by should you buy amd stock here leadership style arent staticheres why that myth is costing you good manager microservices in healthcare market size to hit usd million by driven by cloud adoption and healthcare digitization sn insider meme coin like pepe and wif lose steamozak ai gain investor attention brilliant stock that could soar by to according to wall street balfour beatty community foundation award over in scholarship hims hers stock investor need to know this before buying or selling this growth stock whats going on with adobe stock nyt wordle hint and answer for june puzzle lpro investor have the opportunity to lead the open lending security fraud lawsuit with faruqi faruqi llp ftre investor deadline fortrea holding inc investor with loss may have been affected by fraud contact bfa law by august court deadline nasdaqftre ogn investor deadline organon co investor with loss may have been affected by fraud contact bfa law by july court deadline nyseogn breaking hims news a security fraud class action ha been filed on behalf of hims hers health inc nysehims investor contact bfa law if you lost money aapl investor deadline apple inc investor with loss may have been affected by fraud contact bfa law by august court deadline nasdaqaapl civi investor deadline civitas resource inc investor with loss may have been affected by fraud contact bfa law by july court deadline nysecivi rddt investor deadline reddit inc investor with loss may have been affected by fraud contact bfa law by august court deadline nyserddt breaking codi news compass diversified holding nysecodi announces nonreliance on financial statement for contact bfa law by july iova investor deadline iovance biotherapeutics investor with loss may have been affected by fraud contact bfa law by july court deadline nasdaqiova womens sober housing along the mississippi ha a bright future following troubled past this stock is up since it ipo here reason it could still be a smart buy oppenheimer co inc raise stock position in marsh mclennan company inc nysemmc kremlin reacts to nato defense spending hike no significant effect house republican don bacon of nebraska will not seek reelection stock market pullback coming etf to buy meta platform inc nasdaqmeta share bought by pinnacle bancorp inc golden state wealth management llc boost stock position in lam research corporation nasdaqlrcx hims hers stock financial analysis following huge stock price crash incredible news for quantumscape stock investor this blackrock etf could soar according to billionaire michael saylor new owner to keep childrens exchange open for rochester family how to start learning math for data science a simple guide at bezos venetian wedding buzz bling and backlash the new york time spire wealth management purchase share of doordash inc nasdaqdash bessemer group inc sell share of ameriprise financial inc nyseamp cambridge investment research advisor inc cut position in huntington bancshares incorporated nasdaqhban beloved grocery chain better than costco to open new store a part of expansion after buying closed winndixie site amd v arista network which artificial intelligence ai stock is a better buy right now tariff drive up firework price ahead of fourth of july tip to save for your celebration tariff drive up firework price ahead of fourth of july tip to save for your celebration tariff drive up firework price ahead of fourth of july tip to save for your celebration agg is a great choice for most but i like this vanguard etf better can disney stock keep rising after hitting a new week high memory of muscatine a post card of the golden state tampa outsource call center firm name new ceo whats going on with micron stock america newest space ipo wa a smashing success reigning ballon dor winner aitana bonmati hospitalized with meningitis less than a week before euro i make a year and want to retire at should i invest more in stock or focus on real estate jeff bezos lauren sanchez join list of richest married couple here how prenups for wealthiest people take place hindustan time hindustan time farm labor land cost dominate discussion at inaugural lake county agricultural summit here what the new condo law requires is it too much to handle here what the new condo law requires is it too much to handle developer file preapplication for mixeduse project at nw th st miami florida debt is a growing force influencing jobseekers choice career expert say here how im year old and the father of functional medicine here my daily routine for a healthy life target face serious challenge a ceo cornell retirement nears walmart slash price on popular summer essential to just and it even cheaper than target version the end of bank branch how europe digital euro and stablecoins are reshaping finance luvmes independence day wig sale limitedtime countdown deal old navy is selling americana flip flop for just theyre identical to havaianas but and nearly cheaper new la trader joes open across the street from another trader joes amid messiness at the social security administration more people are taking benefit early asking the right question can reframe how you respond to challenge grandfather k seized by chase in sudden account closure it destroyed his credit forced him to delay retirement macro trend likely to send bitcoin and xrp skyrocketing in how to budget weekly pay when freight is inconsistent why ai resume are overwhelming recruiter and manager after lahaina burned an experiment in housing the most vulnerable golden state wealth management llc purchase share of diageo plc nysedeo rob biederman join the stage at all stage family and business are concerned about the effect of tariff on youth sport share in meta platform inc nasdaqmeta acquired by mokan wealth management inc meta platform inc nasdaqmeta share sold by moran wealth management llc bessemer group inc reduces stake in tmobile u inc nasdaqtmus bessemer group inc lower stock holding in stryker corporation nysesyk aurora private wealth inc purchase share of meta platform inc nasdaqmeta first pacific financial trim position in meta platform inc nasdaqmeta meta platform inc nasdaqmeta stake lifted by symmetry partner llc gamma investing llc ha million stock holding in meta platform inc nasdaqmeta share in carnival corporation nyseccl bought by oppenheimer asset management inc which stock will dominate the weight management market through thing every tesla investor need to watch right now asset management one co ltd sell share of expeditors international of washington inc nasdaqexpd sch financial advisor inc ha million position in alphabet inc nasdaqgoogl walkner condon financial advisor llc acquires share of alphabet inc nasdaqgoogl fidelity national financial inc nysefnf stake increased by oppenheimer co inc nobrainer stock to buy for under right now house republican don bacon of nebraska will not seek reelection wealth enhancement advisory service llc ha million stock holding in darden restaurant inc nysedri llm project every ai enthusiast should build for a stronger resume how europe can mitigate it mighty defence cost challenge ing which cryptocurrency is more likely to be a millionaire maker xrp v shiba inu mortgage rate hit lowest level since early may why you should drop this phrase from your business email colorado health official brace for layoff amid loss of federal funding from trump administration broadcast bias network shield nyc socialist mamdani from extreme label they apply to conservative fact check trump make big false claim about his big domestic policy bill why donald trump is trying to make an example out of this one house republican colorado play about israelgaza debate explores difficult conversation a crisis deepens editorial cartoon for saturday june letter dial back the false rhetoric that inspires violence memory of firework lyon fall and a childhood fueled by curiosity and imagination albemarle look to add more school zone speed camera after initial success column limit of free speech shouldnt be condoned why it time to make america think again deportation nation trump is gunning for new record in immigration prosecution person rescued friday from the penobscot river supreme court limit judge power to block trump order take a stand against the fascist takeover of america policy change could have big consequence for veteran va care drop the charade when it come to social security medicare tesla say it made it first driverless delivery of a new car to a customer this stock is up since it ipo here reason it could still be a smart buy developer lay out their latest vision for the former pleasant hill golf course opinion what doe it mean to be a patriot reader view protect minnesota resource from data center reader view u hypocritical when sending troop senate to hold initial vote today on trump big beautiful bill senate to hold initial vote today on trump big beautiful bill fall river school employee out after arrest on serious charge how psychiatry and activism created the dangerous concept of transgender child reigning ballon dor winner aitana bonmati hospitalized with meningitis less than a week before euro fbi attack on fentanyl is working to reduce overdose death opinion democrat are trying to figure out what to do about john fetterman conor lamb is stepping up letter to the editor truth aint what it used to be why wouldnt there be a regime change what if a hurricane hit alligator alcatraz florida drawing up evacuation plan opinion john tayer that uncomfortable situation where economic and social interest converge opinion max boykoff what will we say in community editorial board considering the sale of public land who is mitchell berger the fort lauderdale democrat chairing david jolly governor campaign canadian man who died in miami detention lived in daytona beach kenosha festivity to change parking traffic downtown old bogeyman reunite maga after explosive iran divide colorado supreme court accepts case on parole revocation debt collection congressional candidate allard see little need for campaign spending limit a look back colorado republican jeff crank get up close look at fire station air base and a convenience store bridging the lgbtq wealth gap the left political philosophy persuasion with a government club roger koopman thing you need to know about new idf chief canceled screening stalled grant federal cut hit iowa group fighting cancer new ut tyler poll reflects texas voter view on current issue political matchup keep our public land public letter hitching a flight tell your story hitching a flight tell your story letter to the editor flag day deserves to be a federal holiday more than other holiday lost in translation off the record lost in translation off the record i dont shy away from a fight pritzkers run for atypical third term fit unprecedented time what happens if wisconsin budget isnt passed on time i dont shy away from a fight pritzkers run for atypical third term fit unprecedented time i dont shy away from a fight pritzkers run for atypical third term fit unprecedented time abbott paxton can withhold uvalde jan related record texas supreme court rule uw nurse bid to reclaim union status rejected by wisconsin supreme court unanimously dont take me out to the ballgame editorial cartoon for saturday june walter five year on the pandemic still plague california employee safety net legislator review kurth disappointed by republican education funding plan legislator review kurth disappointed by republican education funding plan editorial veto speed cam tax credit bill measure to protect hawaii fishing industry one of five food and farm bill signed friday mayor name nominee to future ocean safety commission gop leader boost rural hospital fund rewrite medicaid provision to save trump megabill gop leader boost rural hospital fund rewrite medicaid provision to save trump megabill gop leader boost rural hospital fund rewrite medicaid provision to save trump megabill republican race toward crucial vote on trump megabill despite uncertainty republican race toward crucial vote on trump megabill despite uncertainty republican race toward crucial vote on trump megabill despite uncertainty gop leader boost rural hospital fund rewrite medicaid provision to save trump megabill gop leader boost rural hospital fund rewrite medicaid provision to save trump megabill gop leader boost rural hospital fund rewrite medicaid provision to save trump megabill republican race toward crucial vote on trump megabill despite uncertainty republican race toward crucial vote on trump megabill despite uncertainty republican race toward crucial vote on trump megabill despite uncertainty the tribune quote of the week quiz for june letter route series neglect to capture the beauty along the road in new mexico final day of scotus decision brings wave of historymaking ruling trump nato turnaround from threatening to pull u out to daddy of the alliance msgr charles j dubois is travis decker alive a fruitless week manhunt ha produced no certain evidence republican plan to overhaul medicaid are already shaking up the midterm trump immigration arrest are seeing a wave of resistance wanda ammons regina gina marie williams baccigalopi letter trump like staging spectacle more than he like helping people heat dome pass but climatefueled wave arent going anywhere word of the week eudaimonia what is the meaning of the pursuit of happiness tom sawyer fence painting closed to girl the jackpod taking a break cnn report from the huge crowd attending state funeral in tehran oreo is bringing back a fanfavorite flavor after year stop yelling at u biden join thousand paying final respect to slain minnesota lawmaker and husband ge appliance moving production from china to republican state matthew schaefer honor late mother after getting selected first overall by new york islander in nhl draft letter city could do better to help north tulsa grow thing every rivian investor need to watch right now shiba inu and cardano price prediction leave investor nervous many are joining the remittix train after gain walmart is selling an excellent soundbar for and shopper say it quite impressive bigfoot stomp in from east county mountain it your business bigfoot stomp in from east county mountain it your business unpacking the content strategy definition a modern marketer guide delta operation recovering through weekend more delay and cancellation sunday alivecom la vega strip casino cant escape troubling trend in their shoe what is life like a an olympic longdistance runner the type of load board when and how to use each bart improves in safety cleanliness and satisfaction yet ridership recovery remains slow uptown aventura planned for biscayne blvd miami fl house gop leadership discussing new way to limit classified information on capitol hill from hallucination to hardware lesson from a realworld computer vision project gone sideways this psychedelic drug flopped on trial result should you buy the dip ai stock up to in that should continue moving higher this ridiculously cheap warren buffett stock could make you richer iranian hacker could become more active after military strike here how to protect your business im not putting on a fing hijab uk singer refuse to virtue signal for palestine pull out of festival three sneaky way sam club trick you into buying a tv worth plus easy tip to maximize your home viewing marktomarket middle east conflict whipsaw energy price cheer to year abc fine wine spirit renews support for pediatric cancer research marktomarket middle east conflict whipsaw energy price xrp price prediction payment token surge incoming xrp rtx xlm expected to outperform in july trump tax bill conflict with trump trade goal editorial supreme court ruling restores right to parent walmart is selling a burner expert grill for just and it cheaper than the lowes version borderland mexico winner in global tariff war could be mexico report say global sport medicine leader smithnephew to sponsor select player competing at wimbledon highlighting advanced solution for joint repair an energy star inside u home is under attack from trump with the cost to homeowner uncertain costco branded insane and archaic a shopper beg chain to speed up roll out of popular checkout method used by rival autodesk inc nasdaqadsk share acquired by spire wealth management spire wealth management raise stock holding in autodesk inc nasdaqadsk alphabet inc nasdaqgoogl is apeiron capital ltds th largest position promising robotics stock to consider june th ameriprise financial inc nyseamp share bought by spire wealth management sequoia financial advisor llc buy share of yum brand inc nyseyum elevance health inc nyseelv share bought by sequoia financial advisor llc robeco institutional asset management bv ha million stock position in paychex inc nasdaqpayx top streaming stock worth watching june th steele capital management inc ha million holding in nvidia corporation nasdaqnvda amphenol corporation nyseaph share purchased by cambridge investment research advisor inc robeco institutional asset management bv purchase share of the charles schwab corporation nyseschw sequoia financial advisor llc buy share of public storage nysepsa nvidia corporation nasdaqnvda share purchased by ipswich investment management co inc spire wealth management boost stock position in ameriprise financial inc nyseamp nvidia cor</t>
+          <t>why you should get your boot to beyonces cowboy carter tour a sermon for the weary while you can chinese battery giant and tesla supplier catl is expanding globally here why it matter how to stay on top of google search faraday x preparation are in the final stage for the private preview and cocreation launch event on june th for the groundbreaking fx super one mpv biocon biologics receives health canada approval for yesafilitm aflibercept first global launch scheduled for july china factory activity expected to shrink for third month amid trade tension reuters poll nike vomero quietly became a million franchise in day a ceo say it time to turn the page investor gary black cheer afterhours rally ap technology summarybrief at am edt ap technology summarybrief at am edt ap technology summarybrief at am edt ap technology summarybrief at am edt amazon google not far behind but dan ives say microsoft clearly leading in these segment price target is probably conservative why your to feel more like report say analysisin dovish tilt boj zoom in on obscure underlying inflation trend find the best crypto to join for emerging project reshaping the digital economy tesla shakeup who is omead afshar senior executive reportedly fired by elon musk amid slumping sale i time of india ap business summarybrief at am edt ap business summarybrief at am edt asian share are mostly higher after u stock rise to the brink of a record trump tariff have unsettled thailand pet food exporter germany tell apple google to block deepseek a the chinese ai app face rising pressure in europe hugging face cofounder challenge ai optimist model cant ask original scientific question you might not have bezoslevel buck but you still might consider a prenup vertex founder boger donates m to boston art academy trump big beautiful bill might be unloved and a mess but it will still probably pas here how the luxury real estate market is splitting up how company profit from your data without consent full circle boy leap forward with debut ep jete and official music video this go out to you out now increase of share capital in connection with realization of the employee option programm and subscription result more than an ev charger it peace of mind wherever the road take you cutting u energy credit doesnt save money it steal it from ratepayer local government ansi officially approves two new seia standard on consumer protection and operation and maintenance kymera therapeutic announces pricing of million public offering kymera therapeutic announces pricing of million public offering solaredge expands u manufacturing in salt lake city utah why denver homeowner are investing more in renovation project leap power national grid virtual power plant initiative in massachusetts hawaiian airline report cybersecurity event no flight disruption kitv boeing dreamliner black box recovered data under scrutiny to provide insight into fatal air india crash cso receives grant from mt charitable foundation achieve life science announces pricing of million underwritten public offering the mobility house and schneider electric unveil solar charging depot for turlock unifieds electric school bus fleet trump crypto advisor david sack say july will be a big month say president support legislation on market structure and stablecoins amazon grocery chief blame ridiculous red tape for holding back initiative at whole food were wasting time year old driver from tripura treated with eastern india firstever bachmanns bundle pacing vdh in the end everyone hated the iranian theocracy oklahoma governor kevin stitt and u secretary of health and human service robert f kennedy jr visit mom meal to highlight food a medicine leadership japan executes twitter killer who murdered and dismembered nine people saratoga county celebrates m airport revitalization ap business summarybrief at pm edt ap business summarybrief at pm edt ap business summarybrief at pm edt ap business summarybrief at pm edt ap technology summarybrief at pm edt driver crash nearly plummet over san mateo county cliff north korea just opened a beach resort for people but who will visit jeep gladiator rank first in midsize pickup segment in jd power u initial quality study chrysler jeep and dodge brand improve iq score over thailand will hold trade talk with u next week finance minister say meta say it winning the talent war with openai the verge china u agree on detail of london trade framework beijing say saratogians remember mark straus a pioneer sp cut colombia debt rating to bb over declining fiscal result why lumen technology stock wa winning this week annovis bio to present key finding at alzheimers association international conference iraq war veteran hegseths news conference wa conduct unbecoming chinese influence in climate change lawsuit threatens to derail u energy industry asia fx muted dollar struggle at yr low with pce data on tap demolition start at former kera hq clearing way for new uptown tower european stock extend gain after white house hint at tariff extension baseball player wander franco found guilty in sexual abuse case imposed twoyear suspended sentence china skirt u sanction a top buyer of iranian oil here how and why thats unlikely to change soon china may industrial profit slip back into sharp decline reuters gold head for weekly loss a middle east truce sap demand uk auto production for may slump to lowest level since a trump tariff hit hard mgi announces partnership with negedia enhance genomic sequencing technology at the service of scientific research and precision medicine in italy mgi announces partnership with negedia enhance genomic sequencing technology at the service of scientific research and precision medicine in italy informal mining boom is biggest fear for peru copper investor best cryptos to buy now one already up and climbing bill gate say he know for a fact that more child will die due to u health aid cut and he taking the proof to congress cancer patient recover by taking repurposed antiparasitic drug india economy to hold top spot for growth but underlying weakness remain reuters poll cnbc daily open wall street is tuning out the noise and catching ray turkish farmer pioneer xag agricultural drone for watersmart practice treasury yield inch higher a investor await the fed preferred inflation print bitcoin ethereum rangebound dogecoin dip amid potential july tariff deadline extension analyst predicts btcs next big move once it break out of this range softbank ceo say he all in on openai reveals he long wanted microsofts spot a main backer mexico investigating contamination from spacex explosion debris sandia national laboratory to cut up to workforce by early fall canada approves law to fasttrack resource project face indigenous opposition lithium industry bemoans paradox of low price rising demand china industrial profit slip back into sharp decline in may two north texas school board increase teacher pay in final budget confusion a trump say deal with china signed yet both side violate term of ceasefire share rally but dollar weakens with fed independence seen under threat courtney b vance on book ban protest in los angeles and narrating the audiobook of the biography of web du bois atlantic strategic mineral start commercial production at virginia operation u food and drug administration approves streamlined patient monitoring requirement and removal of rem program within bristol myers squibbs cell therapy label u food and drug administration approves streamlined patient monitoring requirement and removal of rem program within bristol myers squibbs cell therapy label u food and drug administration approves streamlined patient monitoring requirement and removal of rem program within bristol myers squibbs cell therapy label u food and drug administration approves streamlined patient monitoring requirement and removal of rem program within bristol myers squibbs cell therapy label why you should get your boot to beyonces cowboy carter tour a sermon for the weary while you can clarence page did you miss a holiday mr president arthur cyr bombing iran mideast stability and the role of the u former minnesota house speaker melissa hortman to lie in state a suspect face court date former minnesota house speaker melissa hortman to lie in state a suspect face court date democrat are trying to figure out what to do about john fetterman one of them is stepping up democrat are trying to figure out what to do about john fetterman one of them is stepping up democrat are trying to figure out what to do about john fetterman one of them is stepping up supreme court meet friday to decide remaining case including birthright citizenship supreme court meet friday to decide remaining case including birthright citizenship supreme court meet friday to decide remaining case including birthright citizenship supreme court meet friday to decide remaining case including birthright citizenship you might not have bezoslevel buck but you still might consider a prenup summer league basketball islander rattler trump big beautiful bill might be unloved and a mess but it will still probably pas edward d shanshala ii billion in waste fraud and abuse maybe but look in the right place editorial go slow on waymo several caution before selfdriving car arrive rev allison palm rev jonathan hopkins gov ayotte reneged on promise to meet with faith leader senator diverge sharply on damage done by iran strike after classified briefing japan executes twitter killer who murdered and dismembered nine people oregon senate vote to override governor veto a first since dallas place future of the franchise in cooper flagg a southwest division get better north korea just opened a beach resort for people but who will visit panton named johnstown knox elementary school principal former top aide to jill biden subpoenaed in house gop biden age probe iraq war veteran hegseths news conference wa conduct unbecoming selling public land isnt the answer to affordable housing title lx protection matter more than ever trump appointing a shadow chair at the fed ha put dollar under pressure meanwhile china is dumping the greenback and hoarding gold baseball player wander franco found guilty in sexual abuse case imposed twoyear suspended sentence abbott trump approval rating poll show economy thc reduce favorability among texan family file for release in lawsuit considered first involving child challenging arrest at court family file for release in lawsuit considered first involving child challenging arrest at court family sue over u detention in what may be first challenge to courthouse arrest involving kid gov ferguson warns medicaid cut could devastate washington health care system review gloversvilles stump city brewing is modern version of oldtime public house pintsized louisiana is latest state to redefine natural gas a planetwarming fossil fuel a green energy change coming for wilco voter courtney b vance on book ban protest in los angeles and narrating the audiobook of the biography of web du bois critical rce flaw in cisco ise and isepic allow unauthenticated attacker to gain root access pete hegseth air medium coverage grievance towards cnn and others the latest pretrial development in the idaho student killing case green leader larissa water on holding the labor government to account australian politics podcast labor must protect environment while rewriting law written to facilitate development larissa water say wife of minnesota suspect say she wa blindsided by shooting of state politician cnn this is your brain on chatgpt white house confirms u china have reached additional trade agreement trump threatens cnn and new york time with lawsuit over iran report senate parliamentarian ok gop cut to federal food assistance former trail blazer ben mclemore say sex wa consensual while taking the stand during rape trial woman accused of stealing from jewelry store in washington oregon former defense secy iranian nuclear facility damage assessment will take week community rally in massive show of support for caesar palace time square u tariff may sideline youth sport for many family making it harder for kid to stay active rep josh gottheimer american dont like trump big policy bill court issue opinion on centennial at tejon ranch cnn medium analyst responds to false attack on iranian nuclear site report let go through it zohran mamdani tell erin burnett how he plan to pay for his policy fireball fly across the sky and cause sonic boom america controversial iran airstrike letter to the editor june china on alert a nato boost defense spending mamdani vow to stand up to trump border czar and ice canadian official press u government for detail on canadian citizen who died in ice custody at a florida detention center former montana u rep pat williams who won a liberal conservative showdown dy at portland city council pass resolution to strengthen portland street response a look at legal threat facing samesex marriage year after obergefell decision it judgement time for john thune on the big beautiful bill guest commentary rtc targeting senior with displacement former pantagraph building get positive recommendation for landmark status eu leader on wto we need to come up with something else senate democrat question obliteration of iran nuclear site after classified briefing on strike officer placed on leave after shooting in bangor at least orgs urge senator to support iran war power resolution lawsuit filed on behalf of nex benedict estate against owasso public school trump spotlight parent who have lost kid due to open border during big beautiful bill event former trump lawyer kenneth chesebro disbarred in new york over election interference case donald trump say uschina trade truce ha been signed hegseth defends success of u strike on iran nuclear site amid doubt over impact standing up to bullying unscientific transgender activist mob canadian man held by immigration official dy in south florida federal facility official say canadian man held by immigration official dy in south florida federal facility official say canadian man held by immigration official dy in south florida federal facility official say canadian man held by immigration official dy in south florida federal facility official say canadian man held by immigration official dy in south florida federal facility official say canadian man held by immigration official dy in south florida federal facility official say illinois gov jb pritzker announces bid for historic third term amidst presidential buzz interior secretary doug burgum answer question about the big beautiful bill and public land trump doj is targeting daily ko agent mental health passport led to push for secured bond famous preston night rodeo gearing up for it th annual community experience plan unveiled for story link at boca at west yamato road in boca raton fact check trump make big false claim about his big domestic policy bill biogen genentech may stay mum on damage at trial inside the trading desk that surfed day of oil market mayhem bloomberg trader bet on interest rate cut from jay powell successor at the fed financial time etf are booming mutual fund want in on the action analyst amd stock will close the gap with nvidia by should you buy amd stock here leadership style arent staticheres why that myth is costing you good manager microservices in healthcare market size to hit usd million by driven by cloud adoption and healthcare digitization sn insider meme coin like pepe and wif lose steamozak ai gain investor attention brilliant stock that could soar by to according to wall street balfour beatty community foundation award over in scholarship hims hers stock investor need to know this before buying or selling this growth stock whats going on with adobe stock nyt wordle hint and answer for june puzzle lpro investor have the opportunity to lead the open lending security fraud lawsuit with faruqi faruqi llp ftre investor deadline fortrea holding inc investor with loss may have been affected by fraud contact bfa law by august court deadline nasdaqftre ogn investor deadline organon co investor with loss may have been affected by fraud contact bfa law by july court deadline nyseogn breaking hims news a security fraud class action ha been filed on behalf of hims hers health inc nysehims investor contact bfa law if you lost money aapl investor deadline apple inc investor with loss may have been affected by fraud contact bfa law by august court deadline nasdaqaapl civi investor deadline civitas resource inc investor with loss may have been affected by fraud contact bfa law by july court deadline nysecivi rddt investor deadline reddit inc investor with loss may have been affected by fraud contact bfa law by august court deadline nyserddt breaking codi news compass diversified holding nysecodi announces nonreliance on financial statement for contact bfa law by july iova investor deadline iovance biotherapeutics investor with loss may have been affected by fraud contact bfa law by july court deadline nasdaqiova woman sober housing along the mississippi ha a bright future following troubled past this stock is up since it ipo here reason it could still be a smart buy oppenheimer co inc raise stock position in marsh mclennan company inc nysemmc kremlin reacts to nato defense spending hike no significant effect house republican don bacon of nebraska will not seek reelection stock market pullback coming etf to buy meta platform inc nasdaqmeta share bought by pinnacle bancorp inc golden state wealth management llc boost stock position in lam research corporation nasdaqlrcx hims hers stock financial analysis following huge stock price crash incredible news for quantumscape stock investor this blackrock etf could soar according to billionaire michael saylor new owner to keep childrens exchange open for rochester family how to start learning math for data science a simple guide at bezos venetian wedding buzz bling and backlash the new york time spire wealth management purchase share of doordash inc nasdaqdash bessemer group inc sell share of ameriprise financial inc nyseamp cambridge investment research advisor inc cut position in huntington bancshares incorporated nasdaqhban beloved grocery chain better than costco to open new store a part of expansion after buying closed winndixie site amd v arista network which artificial intelligence ai stock is a better buy right now tariff drive up firework price ahead of fourth of july tip to save for your celebration tariff drive up firework price ahead of fourth of july tip to save for your celebration tariff drive up firework price ahead of fourth of july tip to save for your celebration agg is a great choice for most but i like this vanguard etf better can disney stock keep rising after hitting a new week high memory of muscatine a post card of the golden state tampa outsource call center firm name new ceo whats going on with micron stock america newest space ipo wa a smashing success reigning ballon dor winner aitana bonmati hospitalized with meningitis le than a week before euro i make a year and want to retire at should i invest more in stock or focus on real estate jeff bezos lauren sanchez join list of richest married couple here how prenups for wealthiest people take place hindustan time hindustan time farm labor land cost dominate discussion at inaugural lake county agricultural summit here what the new condo law requires is it too much to handle here what the new condo law requires is it too much to handle developer file preapplication for mixeduse project at nw th st miami florida debt is a growing force influencing jobseekers choice career expert say here how im year old and the father of functional medicine here my daily routine for a healthy life target face serious challenge a ceo cornell retirement nears walmart slash price on popular summer essential to just and it even cheaper than target version the end of bank branch how europe digital euro and stablecoins are reshaping finance luvmes independence day wig sale limitedtime countdown deal old navy is selling americana flip flop for just theyre identical to havaianas but and nearly cheaper new la trader joes open across the street from another trader joes amid messiness at the social security administration more people are taking benefit early asking the right question can reframe how you respond to challenge grandfather k seized by chase in sudden account closure it destroyed his credit forced him to delay retirement macro trend likely to send bitcoin and xrp skyrocketing in how to budget weekly pay when freight is inconsistent why ai resume are overwhelming recruiter and manager after lahaina burned an experiment in housing the most vulnerable golden state wealth management llc purchase share of diageo plc nysedeo rob biederman join the stage at all stage family and business are concerned about the effect of tariff on youth sport share in meta platform inc nasdaqmeta acquired by mokan wealth management inc meta platform inc nasdaqmeta share sold by moran wealth management llc bessemer group inc reduces stake in tmobile u inc nasdaqtmus bessemer group inc lower stock holding in stryker corporation nysesyk aurora private wealth inc purchase share of meta platform inc nasdaqmeta first pacific financial trim position in meta platform inc nasdaqmeta meta platform inc nasdaqmeta stake lifted by symmetry partner llc gamma investing llc ha million stock holding in meta platform inc nasdaqmeta share in carnival corporation nyseccl bought by oppenheimer asset management inc which stock will dominate the weight management market through thing every tesla investor need to watch right now asset management one co ltd sell share of expeditors international of washington inc nasdaqexpd sch financial advisor inc ha million position in alphabet inc nasdaqgoogl walkner condon financial advisor llc acquires share of alphabet inc nasdaqgoogl fidelity national financial inc nysefnf stake increased by oppenheimer co inc nobrainer stock to buy for under right now house republican don bacon of nebraska will not seek reelection wealth enhancement advisory service llc ha million stock holding in darden restaurant inc nysedri llm project every ai enthusiast should build for a stronger resume how europe can mitigate it mighty defence cost challenge ing which cryptocurrency is more likely to be a millionaire maker xrp v shiba inu mortgage rate hit lowest level since early may why you should drop this phrase from your business email colorado health official brace for layoff amid loss of federal funding from trump administration broadcast bias network shield nyc socialist mamdani from extreme label they apply to conservative fact check trump make big false claim about his big domestic policy bill why donald trump is trying to make an example out of this one house republican colorado play about israelgaza debate explores difficult conversation a crisis deepens editorial cartoon for saturday june letter dial back the false rhetoric that inspires violence memory of firework lyon fall and a childhood fueled by curiosity and imagination albemarle look to add more school zone speed camera after initial success column limit of free speech shouldnt be condoned why it time to make america think again deportation nation trump is gunning for new record in immigration prosecution person rescued friday from the penobscot river supreme court limit judge power to block trump order take a stand against the fascist takeover of america policy change could have big consequence for veteran va care drop the charade when it come to social security medicare tesla say it made it first driverless delivery of a new car to a customer this stock is up since it ipo here reason it could still be a smart buy developer lay out their latest vision for the former pleasant hill golf course opinion what doe it mean to be a patriot reader view protect minnesota resource from data center reader view u hypocritical when sending troop senate to hold initial vote today on trump big beautiful bill senate to hold initial vote today on trump big beautiful bill fall river school employee out after arrest on serious charge how psychiatry and activism created the dangerous concept of transgender child reigning ballon dor winner aitana bonmati hospitalized with meningitis le than a week before euro fbi attack on fentanyl is working to reduce overdose death opinion democrat are trying to figure out what to do about john fetterman conor lamb is stepping up letter to the editor truth aint what it used to be why wouldnt there be a regime change what if a hurricane hit alligator alcatraz florida drawing up evacuation plan opinion john tayer that uncomfortable situation where economic and social interest converge opinion max boykoff what will we say in community editorial board considering the sale of public land who is mitchell berger the fort lauderdale democrat chairing david jolly governor campaign canadian man who died in miami detention lived in daytona beach kenosha festivity to change parking traffic downtown old bogeyman reunite maga after explosive iran divide colorado supreme court accepts case on parole revocation debt collection congressional candidate allard see little need for campaign spending limit a look back colorado republican jeff crank get up close look at fire station air base and a convenience store bridging the lgbtq wealth gap the left political philosophy persuasion with a government club roger koopman thing you need to know about new idf chief canceled screening stalled grant federal cut hit iowa group fighting cancer new ut tyler poll reflects texas voter view on current issue political matchup keep our public land public letter hitching a flight tell your story hitching a flight tell your story letter to the editor flag day deserves to be a federal holiday more than other holiday lost in translation off the record lost in translation off the record i dont shy away from a fight pritzkers run for atypical third term fit unprecedented time what happens if wisconsin budget isnt passed on time i dont shy away from a fight pritzkers run for atypical third term fit unprecedented time i dont shy away from a fight pritzkers run for atypical third term fit unprecedented time abbott paxton can withhold uvalde jan related record texas supreme court rule uw nurse bid to reclaim union status rejected by wisconsin supreme court unanimously dont take me out to the ballgame editorial cartoon for saturday june walter five year on the pandemic still plague california employee safety net legislator review kurth disappointed by republican education funding plan legislator review kurth disappointed by republican education funding plan editorial veto speed cam tax credit bill measure to protect hawaii fishing industry one of five food and farm bill signed friday mayor name nominee to future ocean safety commission gop leader boost rural hospital fund rewrite medicaid provision to save trump megabill gop leader boost rural hospital fund rewrite medicaid provision to save trump megabill gop leader boost rural hospital fund rewrite medicaid provision to save trump megabill republican race toward crucial vote on trump megabill despite uncertainty republican race toward crucial vote on trump megabill despite uncertainty republican race toward crucial vote on trump megabill despite uncertainty gop leader boost rural hospital fund rewrite medicaid provision to save trump megabill gop leader boost rural hospital fund rewrite medicaid provision to save trump megabill gop leader boost rural hospital fund rewrite medicaid provision to save trump megabill republican race toward crucial vote on trump megabill despite uncertainty republican race toward crucial vote on trump megabill despite uncertainty republican race toward crucial vote on trump megabill despite uncertainty the tribune quote of the week quiz for june letter route series neglect to capture the beauty along the road in new mexico final day of scotus decision brings wave of historymaking ruling trump nato turnaround from threatening to pull u out to daddy of the alliance msgr charles j dubois is travis decker alive a fruitless week manhunt ha produced no certain evidence republican plan to overhaul medicaid are already shaking up the midterm trump immigration arrest are seeing a wave of resistance wanda ammons regina gina marie williams baccigalopi letter trump like staging spectacle more than he like helping people heat dome pass but climatefueled wave arent going anywhere word of the week eudaimonia what is the meaning of the pursuit of happiness tom sawyer fence painting closed to girl the jackpod taking a break cnn report from the huge crowd attending state funeral in tehran oreo is bringing back a fanfavorite flavor after year stop yelling at u biden join thousand paying final respect to slain minnesota lawmaker and husband ge appliance moving production from china to republican state matthew schaefer honor late mother after getting selected first overall by new york islander in nhl draft letter city could do better to help north tulsa grow thing every rivian investor need to watch right now shiba inu and cardano price prediction leave investor nervous many are joining the remittix train after gain walmart is selling an excellent soundbar for and shopper say it quite impressive bigfoot stomp in from east county mountain it your business bigfoot stomp in from east county mountain it your business unpacking the content strategy definition a modern marketer guide delta operation recovering through weekend more delay and cancellation sunday alivecom la vega strip casino cant escape troubling trend in their shoe what is life like a an olympic longdistance runner the type of load board when and how to use each bart improves in safety cleanliness and satisfaction yet ridership recovery remains slow uptown aventura planned for biscayne blvd miami fl house gop leadership discussing new way to limit classified information on capitol hill from hallucination to hardware lesson from a realworld computer vision project gone sideways this psychedelic drug flopped on trial result should you buy the dip ai stock up to in that should continue moving higher this ridiculously cheap warren buffett stock could make you richer iranian hacker could become more active after military strike here how to protect your business im not putting on a fing hijab uk singer refuse to virtue signal for palestine pull out of festival three sneaky way sam club trick you into buying a tv worth plus easy tip to maximize your home viewing marktomarket middle east conflict whipsaw energy price cheer to year abc fine wine spirit renews support for pediatric cancer research marktomarket middle east conflict whipsaw energy price xrp price prediction payment token surge incoming xrp rtx xlm expected to outperform in july trump tax bill conflict with trump trade goal editorial supreme court ruling restores right to parent walmart is selling a burner expert grill for just and it cheaper than the lowes version borderland mexico winner in global tariff war could be mexico report say global sport medicine leader smithnephew to sponsor select player competing at wimbledon highlighting advanced solution for joint repair an energy star inside u home is under attack from trump with the cost to homeowner uncertain costco branded insane and archaic a shopper beg chain to speed up roll out of popular checkout method used by rival autodesk inc nasdaqadsk share acquired by spire wealth management spire wealth management raise stock holding in autodesk inc nasdaqadsk alphabet inc nasdaqgoogl is apeiron capital ltds th largest position promising robotics stock to consider june th ameriprise financial inc nyseamp share bought by spire wealth management sequoia financial advisor llc buy share of yum brand inc nyseyum elevance health inc nyseelv share bought by sequoia financial advisor llc robeco institutional asset management bv ha million stock position in paychex inc nasdaqpayx top streaming stock worth watching june th steele capital management inc ha million holding in nvidia corporation nasdaqnvda amphenol corporation nyseaph share purchased by cambridge investment research advisor inc robeco institutional asset management bv purchase share of the charles schwab corporation nyseschw sequoia financial advisor llc buy share of public storage nysepsa nvidia corporation nasdaqnvda share purchased by ipswich investment management co inc spire wealth management boost stock position in ameriprise financial inc nyseamp nvidia corporat</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>esperion appoints craig thompson to board of director mercadolibre applied material and a healthcare stock on cnbcs final trade ap business summarybrief at am edt ap business summarybrief at am edt how to plan in an uncertain economy senate churn through overnight session a republican seek support for trump big bill senate churn through overnight session a republican seek support for trump big bill bbg launch data center specialty practice appoints industry veteran chris fudacz to lead new specialty practice mara report june bitcoin production and mining operation update issue midyear outlook the bond canary in the big beautiful coal mine nasdaq welcome ipo in the first half of ameresco receives frost sullivan global company of the year award for excellence in energy service nasdaq welcome ipo in the first half of outlook therapeutic appoints biopharmaceutical industry and commercial leader bob jahr a chief executive officer outlook therapeutic appoints biopharmaceutical industry and commercial leader bob jahr a chief executive officer beyond the number analyst discus taysha gene therapy stock deep dive into new fortress energy stock analyst perspective rating trevi therapeutic to attend leerink partner therapeutic forum ii and metabolism beyond the number analyst discus lineage stock stock market today dow jones fall ahead of powell talk tesla dive on trumpmusk feud live coverage analyst assess ionis pharmaceutical what you need to know where robinhood market stand with analyst deep dive into weyerhaeuser stock analyst perspective rating should you expect demand growth in range resource rrc alphyns zabalafin hydrogel for atopic dermatitis highlighted in leading peerreviewed journal oppo reno pro price availability spec more qapel medical appoints stewart strong a president and chief executive officer highspring and vaco by highspring earn top honor from staffing industry analyst what make pinnacle financial partner pnfp a longterm bet ap technology summarybrief at am edt july is flush smart month who need a refresher on potty training basic historic hip hop def jam memorabilia auction to benefit rush philanthropic art foundation bidding close july july is flush smart month who need a refresher on potty training basic bounce empire debut world largest indoor circular transparent led screen surpasses visitor in two year rohrer aesthetic unveils new clinical study highlighting pixe a the future of regenerative aesthetic can community health launch susan terry foundation to empower individual living with hiv blackrock esg capital allocation term trust ecat certified result of annual meeting announced td synnex acquires apptium to accelerate innovation breadth of cloud and everythingasaservice offering masco corporation announces date for earnings release and conference call for second quarter fifth third wealth advisor surpasses billion in net new asset under management expands platform capability thredd expands global footprint with new office in the u intrabio inc completes recruitment for ib at pivotal clinical trial dakota announces formation of advisory board to accelerate strategic growth and product evolution uber eats expands partnership with beloved local grocer marea therapeutic appoints shishir gadam phd a chief technical officer lynq set july th launch date for realtime interestbearing settlement network retail investor use ethransaction btc xrp usdc and other mainstream currency for cloud mining earning a stable income of per day cordia pittsburgh win system of the year award at idea senate strike ai provision from gop bill after uproar from the state senate strike ai provision from gop bill after uproar from the state senate strike ai provision from gop bill after uproar from the state senate strike ai provision from gop bill after uproar from the state thermo fisher scientific to hold earnings conference call on wednesday july amentum to host third quarter fiscal year earnings conference call on august momentus and orbit fab partner to advance space servicing with podracer and rafti demonstration flight this stock is still the very best place you can put your money tailor expands series a to m with privatepublic support operation hope and georgia state university launch groundbreaking ai literacy program for underserved youth levelblue to acquire trustwave becoming largest pureplay managed security service provider this stock is still the very best place you can put your money nline energy and penn state health milton s hershey medical center win joseph m brillhart innovation award at idea pepper launch the first open and extensible endless aisle platform in the foodservice industry fresenius expands biosimilars portfolio with the launch of denosumab biosimilars in the u sofi schedule conference call to discus q result valley national bancorp announces new general counsel unnatural product tap argenxs help for ringed molecule expands internal work into obesity brightspring health lead company in line for tripledigit profit growth brightspring health lead company in line for tripledigit profit growth i tried amazon bestselling beckham hotel collection pillow to see if theyre actually any good transcript velina peneva swiss re chief investment officer elon musk and donald trump are fighting again miami beach city commission grant final approval to terras redevelopment of the historic deauville hotel site canadian cuisine food that reflect the country size and diversity is nvidia stock a buy at new record high jewelry sale outperform a u spending for most luxury good falter citi report find cnbc oportun responds to comment by findell capital actelis network announces private placement priced atthemarket under nasdaq rule deepki accelerates u operation to help commercial real estate tackle sustainability challenge manage risk and drive financial performance duo technology added to russell microcap index dih appoints rehazentrum valens a a dih center of excellence lendmark financial service announces expiration and result of it tender offer for it senior note due cole engineering awarded m u army production contract for nextgeneration stinger training system zohran mamdanis primary win is a warning to every legacy brand travtus partner with engrain to bring spatial intelligence to it everyday ai platform jd martin expands partnership with nvent eriflex to florida north carolina and south carolina radius recycling report third quarter fiscal financial result stryker to announce financial result for it second quarter of fiscal year richtech robotics announces inclusion in u smallcap russell and russell index oncternal therapeutic announces the sale of select development program and the winddown of it operation arevon secures million credit facility to accelerate renewable energy growth in the united state dih appoints rehazentrum valens a a dih center of excellence kavalan blitz iwc taking trio of whisky distillery and master distiller of the year prize inriver research reveals widespread ai deployment in pim of company have moved beyond pilot randamu and chengdu university of information technology collaborate to advance cryptographic research and web coordination infrastructure kestra medical technology ltd to report fourth quarter and fiscal year result on july genmab announces change to it executive committee document available regarding ramacos brook mine rare earth and critical mineral project condo price dropped in maythe second largest decline on record independent preliminary economic assessment report from fluor corporation confirms commercial and technical feasibility of ramacos brook mine rare earth deposit realme series set to shake up india midrange smartphone market aocs childhood nickname revealed amid bronx girl claim second democrat announces campaign to unseat gop congressman in competitive michigan district these new colorado law take effect tuesday regulating gun shop sexual assault case youth detention and more these new colorado law take effect tuesday regulating gun shop sexual assault case youth detention and more the multiverse scandal how academia is redefining science to avoid god senate strike ai provision from gop bill after uproar from the state senate strike ai provision from gop bill after uproar from the state i tried amazon bestselling beckham hotel collection pillow to see if theyre actually any good elon musk and donald trump are fighting again dan gainor the good the bad and the absurd june wildest political moment and celebrity meltdown canadian cuisine food that reflect the country size and diversity la new budget kick in today here what your tax dollar are paying for montana leader need to protect our export economy mark noland letter bad outcome if medicare is cut editorial cartoon for tuesday july cant wait for saturday today texas state to the pac then what james walkinshaw win democratic contest to likely replace u rep connolly in northern virginia mystery surround the jeffrey epstein file after bondi claim ten of thousand of video amendment targeting medicaid expansion wont get a senate vote trump say doge might have to go back and eat elon musk after his criticism of the gop bill president lee jaemyung hope for a better interkorean relationship hickory public housing authority officially abolished after final meeting monday well break your leg un accused of mafiatype response to usled gaza relief effort usaid cut could cause staggering number of avoidable death study say how iran lost the short war with israel and america republican struggle to pas trump massive tax bill after hour of drama opinion senate bill undermines decade of progress in disability service thousand of cancer patient fear disruption in care due to insurance contract dispute supreme court medina ruling free state to defund planned parenthood muscatine contingent visit china trump blame att after conference call with faith leader disrupted takeaway from aps report on attorney general bondis comment about evidence in epstein case takeaway from aps report on attorney general bondis comment about evidence in epstein case texas democrat who lost to ted cruz month ago jump into senate race watching area near florida for possible tropical development saudi arabia alhilal had to climb mount everest without oxygen in shock club world cup win over manchester city trump score major victory a vance help push big beautiful bill through senate maybe he ha a knife yulia putintseva asks for crazy wimbledon spectator to be ejected over safety fear senate hold votearama on trump big beautiful bill senate votearama on gop megabill go all night most american feel democracy is theatened poll show and mamdani speaks with npr new jersey phil murphy take heat from all side in final budget a governor south korea energy policy under lee jaemyung american opinion deportation alone cant fix u immigration problem can south korea achieve peace in a chaotic world trump big beautiful bill awaits final senate vote opinion spense havlick scam are everywhere these day dont be fooled the future of air combat how long will the u military still need pilot california new consumer protection law go into effect july amc theater will start placing even more ad in cinema nationwide starting today letter to the editor power must be maintained at all cost extend freedom beyond our own specie we need a shared morality major insurance change are coming to glp drug for weight loss here how that could affect patient editorial american deserve clearer explanation of what happened in iran maglite pedestrian safety institute and additional partner to promote traffic and pedestrian safety during national roadside traffic safety awareness month egg harbor township approves year affordable housing plan remembering the men and woman who serve our country do the saint have their qb of the future in the building this season should decide that trump relief for farmer look like control by fear guest commentary florida resident get a new roof now and receive free exterior painting just in time for hurricane season letter democrat seem incapable of praising trump for anything whats the point of being a u senator if you dont have gut bob brown the most undervalued asset for a leader it these hour the bully pulpit ron waterman what sdas latest win signal for military space republican still pushing to pas trump big beautiful bill he hasnt played in mlb for more than two decade one team is paying him million a year until senate republican closing in on final vote on gop spending bill more republican than dems vote to raise tax on billionaire in latenight senate vote house democrat announces he wont seek reelection in trump doge is the monster that might have to go back and eat elon will state assembly save energy independence california focus will state assembly save energy independence california focus watch out for weirdo facebook scammer promising the world scam of the week letter obama policy necessitated u strike on nuclear site opinion state bill pausing new building code risk climate change progress public health expert trump big beautiful bill will cause misery and death my turn we need to be a twohospital town my turn thanks extremist for making me reexamine who i want to be and what our nation should be my turn state democrat play dirty trick with legislation my turn another four year of the idiot council doofus thing to know for july trump megabill israelgaza alligator alcatraz idaho shooting hurricane data debate over trump big bill continues tuesday morning in u senate hundred of national guard force deployed to la by trump could be returned to calif wildfire duty editorial cartoon for july reader view congress must reject any cut to medicaid who to say anybodys vote is safe trump doj target north carolina voter roll here how president trump mega tax bill would impact illinois council lower real estate tax rate yet restores funding for service program concern in north dakota grow about increased aca cost medical debt flood drown out lancaster county roadway in aftermath of monday storm hundred of child told to test for disease in australia after childcare worker charged with child sex abuse here are offensive player who can contribute for southern football in wisconsin governor gop reach budget deal to cut tax fund university maha report call for fighting chronic disease but trump and kennedy have yanked funding local expert detail potential effect of federal funding cut lagniappe next up the steve miller band jay take isolation a doubleedged sword letter catholic must stand in unity and sacrifice a jesus did letter america most beautiful wild land are in grave danger burke catawba mcdowell iredell city county close for july see garbage impact</t>
+          <t>esperion appoints craig thompson to board of director mercadolibre applied material and a healthcare stock on cnbcs final trade ap business summarybrief at am edt ap business summarybrief at am edt how to plan in an uncertain economy senate churn through overnight session a republican seek support for trump big bill senate churn through overnight session a republican seek support for trump big bill bbg launch data center specialty practice appoints industry veteran chris fudacz to lead new specialty practice mara report june bitcoin production and mining operation update issue midyear outlook the bond canary in the big beautiful coal mine nasdaq welcome ipo in the first half of ameresco receives frost sullivan global company of the year award for excellence in energy service nasdaq welcome ipo in the first half of outlook therapeutic appoints biopharmaceutical industry and commercial leader bob jahr a chief executive officer outlook therapeutic appoints biopharmaceutical industry and commercial leader bob jahr a chief executive officer beyond the number analyst discus taysha gene therapy stock deep dive into new fortress energy stock analyst perspective rating trevi therapeutic to attend leerink partner therapeutic forum ii and metabolism beyond the number analyst discus lineage stock stock market today dow jones fall ahead of powell talk tesla dive on trumpmusk feud live coverage analyst ass ionis pharmaceutical what you need to know where robinhood market stand with analyst deep dive into weyerhaeuser stock analyst perspective rating should you expect demand growth in range resource rrc alphyns zabalafin hydrogel for atopic dermatitis highlighted in leading peerreviewed journal oppo reno pro price availability spec more qapel medical appoints stewart strong a president and chief executive officer highspring and vaco by highspring earn top honor from staffing industry analyst what make pinnacle financial partner pnfp a longterm bet ap technology summarybrief at am edt july is flush smart month who need a refresher on potty training basic historic hip hop def jam memorabilia auction to benefit rush philanthropic art foundation bidding close july july is flush smart month who need a refresher on potty training basic bounce empire debut world largest indoor circular transparent led screen surpasses visitor in two year rohrer aesthetic unveils new clinical study highlighting pixe a the future of regenerative aesthetic can community health launch susan terry foundation to empower individual living with hiv blackrock esg capital allocation term trust ecat certified result of annual meeting announced td synnex acquires apptium to accelerate innovation breadth of cloud and everythingasaservice offering masco corporation announces date for earnings release and conference call for second quarter fifth third wealth advisor surpasses billion in net new asset under management expands platform capability thredd expands global footprint with new office in the u intrabio inc completes recruitment for ib at pivotal clinical trial dakota announces formation of advisory board to accelerate strategic growth and product evolution uber eats expands partnership with beloved local grocer marea therapeutic appoints shishir gadam phd a chief technical officer lynq set july th launch date for realtime interestbearing settlement network retail investor use ethransaction btc xrp usdc and other mainstream currency for cloud mining earning a stable income of per day cordia pittsburgh win system of the year award at idea senate strike ai provision from gop bill after uproar from the state senate strike ai provision from gop bill after uproar from the state senate strike ai provision from gop bill after uproar from the state senate strike ai provision from gop bill after uproar from the state thermo fisher scientific to hold earnings conference call on wednesday july amentum to host third quarter fiscal year earnings conference call on august momentus and orbit fab partner to advance space servicing with podracer and rafti demonstration flight this stock is still the very best place you can put your money tailor expands series a to m with privatepublic support operation hope and georgia state university launch groundbreaking ai literacy program for underserved youth levelblue to acquire trustwave becoming largest pureplay managed security service provider this stock is still the very best place you can put your money nline energy and penn state health milton s hershey medical center win joseph m brillhart innovation award at idea pepper launch the first open and extensible endless aisle platform in the foodservice industry fresenius expands biosimilars portfolio with the launch of denosumab biosimilars in the u sofi schedule conference call to discus q result valley national bancorp announces new general counsel unnatural product tap argenxs help for ringed molecule expands internal work into obesity brightspring health lead company in line for tripledigit profit growth brightspring health lead company in line for tripledigit profit growth i tried amazon bestselling beckham hotel collection pillow to see if theyre actually any good transcript velina peneva swiss re chief investment officer elon musk and donald trump are fighting again miami beach city commission grant final approval to terras redevelopment of the historic deauville hotel site canadian cuisine food that reflect the country size and diversity is nvidia stock a buy at new record high jewelry sale outperform a u spending for most luxury good falter citi report find cnbc oportun responds to comment by findell capital actelis network announces private placement priced atthemarket under nasdaq rule deepki accelerates u operation to help commercial real estate tackle sustainability challenge manage risk and drive financial performance duo technology added to russell microcap index dih appoints rehazentrum valens a a dih center of excellence lendmark financial service announces expiration and result of it tender offer for it senior note due cole engineering awarded m u army production contract for nextgeneration stinger training system zohran mamdanis primary win is a warning to every legacy brand travtus partner with engrain to bring spatial intelligence to it everyday ai platform jd martin expands partnership with nvent eriflex to florida north carolina and south carolina radius recycling report third quarter fiscal financial result stryker to announce financial result for it second quarter of fiscal year richtech robotics announces inclusion in u smallcap russell and russell index oncternal therapeutic announces the sale of select development program and the winddown of it operation arevon secures million credit facility to accelerate renewable energy growth in the united state dih appoints rehazentrum valens a a dih center of excellence kavalan blitz iwc taking trio of whisky distillery and master distiller of the year prize inriver research reveals widespread ai deployment in pim of company have moved beyond pilot randamu and chengdu university of information technology collaborate to advance cryptographic research and web coordination infrastructure kestra medical technology ltd to report fourth quarter and fiscal year result on july genmab announces change to it executive committee document available regarding ramacos brook mine rare earth and critical mineral project condo price dropped in maythe second largest decline on record independent preliminary economic assessment report from fluor corporation confirms commercial and technical feasibility of ramacos brook mine rare earth deposit realme series set to shake up india midrange smartphone market aocs childhood nickname revealed amid bronx girl claim second democrat announces campaign to unseat gop congressman in competitive michigan district these new colorado law take effect tuesday regulating gun shop sexual assault case youth detention and more these new colorado law take effect tuesday regulating gun shop sexual assault case youth detention and more the multiverse scandal how academia is redefining science to avoid god senate strike ai provision from gop bill after uproar from the state senate strike ai provision from gop bill after uproar from the state i tried amazon bestselling beckham hotel collection pillow to see if theyre actually any good elon musk and donald trump are fighting again dan gainor the good the bad and the absurd june wildest political moment and celebrity meltdown canadian cuisine food that reflect the country size and diversity la new budget kick in today here what your tax dollar are paying for montana leader need to protect our export economy mark noland letter bad outcome if medicare is cut editorial cartoon for tuesday july cant wait for saturday today texas state to the pac then what james walkinshaw win democratic contest to likely replace u rep connolly in northern virginia mystery surround the jeffrey epstein file after bondi claim ten of thousand of video amendment targeting medicaid expansion wont get a senate vote trump say doge might have to go back and eat elon musk after his criticism of the gop bill president lee jaemyung hope for a better interkorean relationship hickory public housing authority officially abolished after final meeting monday well break your leg un accused of mafiatype response to usled gaza relief effort usaid cut could cause staggering number of avoidable death study say how iran lost the short war with israel and america republican struggle to pas trump massive tax bill after hour of drama opinion senate bill undermines decade of progress in disability service thousand of cancer patient fear disruption in care due to insurance contract dispute supreme court medina ruling free state to defund planned parenthood muscatine contingent visit china trump blame att after conference call with faith leader disrupted takeaway from aps report on attorney general bondis comment about evidence in epstein case takeaway from aps report on attorney general bondis comment about evidence in epstein case texas democrat who lost to ted cruz month ago jump into senate race watching area near florida for possible tropical development saudi arabia alhilal had to climb mount everest without oxygen in shock club world cup win over manchester city trump score major victory a vance help push big beautiful bill through senate maybe he ha a knife yulia putintseva asks for crazy wimbledon spectator to be ejected over safety fear senate hold votearama on trump big beautiful bill senate votearama on gop megabill go all night most american feel democracy is theatened poll show and mamdani speaks with npr new jersey phil murphy take heat from all side in final budget a governor south korea energy policy under lee jaemyung american opinion deportation alone cant fix u immigration problem can south korea achieve peace in a chaotic world trump big beautiful bill awaits final senate vote opinion spense havlick scam are everywhere these day dont be fooled the future of air combat how long will the u military still need pilot california new consumer protection law go into effect july amc theater will start placing even more ad in cinema nationwide starting today letter to the editor power must be maintained at all cost extend freedom beyond our own specie we need a shared morality major insurance change are coming to glp drug for weight loss here how that could affect patient editorial american deserve clearer explanation of what happened in iran maglite pedestrian safety institute and additional partner to promote traffic and pedestrian safety during national roadside traffic safety awareness month egg harbor township approves year affordable housing plan remembering the men and woman who serve our country do the saint have their qb of the future in the building this season should decide that trump relief for farmer look like control by fear guest commentary florida resident get a new roof now and receive free exterior painting just in time for hurricane season letter democrat seem incapable of praising trump for anything whats the point of being a u senator if you dont have gut bob brown the most undervalued asset for a leader it these hour the bully pulpit ron waterman what sdas latest win signal for military space republican still pushing to pas trump big beautiful bill he hasnt played in mlb for more than two decade one team is paying him million a year until senate republican closing in on final vote on gop spending bill more republican than dems vote to raise tax on billionaire in latenight senate vote house democrat announces he wont seek reelection in trump doge is the monster that might have to go back and eat elon will state assembly save energy independence california focus will state assembly save energy independence california focus watch out for weirdo facebook scammer promising the world scam of the week letter obama policy necessitated u strike on nuclear site opinion state bill pausing new building code risk climate change progress public health expert trump big beautiful bill will cause misery and death my turn we need to be a twohospital town my turn thanks extremist for making me reexamine who i want to be and what our nation should be my turn state democrat play dirty trick with legislation my turn another four year of the idiot council doofus thing to know for july trump megabill israelgaza alligator alcatraz idaho shooting hurricane data debate over trump big bill continues tuesday morning in u senate hundred of national guard force deployed to la by trump could be returned to calif wildfire duty editorial cartoon for july reader view congress must reject any cut to medicaid who to say anybodys vote is safe trump doj target north carolina voter roll here how president trump mega tax bill would impact illinois council lower real estate tax rate yet restores funding for service program concern in north dakota grow about increased aca cost medical debt flood drown out lancaster county roadway in aftermath of monday storm hundred of child told to test for disease in australia after childcare worker charged with child sex abuse here are offensive player who can contribute for southern football in wisconsin governor gop reach budget deal to cut tax fund university maha report call for fighting chronic disease but trump and kennedy have yanked funding local expert detail potential effect of federal funding cut lagniappe next up the steve miller band jay take isolation a doubleedged sword letter catholic must stand in unity and sacrifice a jesus did letter america most beautiful wild land are in grave danger burke catawba mcdowell iredell city county close for july see garbage impact</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>halftime show icon take big fall get injured during wnba commissioner cup championship after paying u tariff on it product busy baby look to europe and australia a future market dan ives urge apple to make a move saying that perplexity acquisition is a nobrainer it a matter of when and not if centene stock plummet what sparked the brutal selloff centene stock plummet what sparked the brutal selloff barrons iran president approves law suspending cooperation with un nuclear watchdog invivyd and leading researcher form spear spike protein elimination and recovery study group first horizon corporation announces redemption of series b preferred stock and corresponding series b depositary share new study reveals brutal hit that u employer face from trump tariff huffpost fortnite how to get the battle bus suv try this trick wildfire kill people in spain a part of europe bake in heat wave think you missed the ai rally these gridbacked play are just getting warmed up tech billionaire launch erebor bank to fill svbs gap invivyd and leading researcher form spear spike protein elimination and recovery study group to assess the effect of monoclonal antibody therapy for long covid and covid postvaccination syndrome diversified energy promotes michael garrett to chief accounting officer diversified energy promotes michael garrett to chief accounting officer uk investor see not one but two pathway to rail merger developer acquire land for westgate village at north congress avenue west palm beach florida argon ai raise m to build the ai workspace powering the future of life science nationsbenefits integrates with dollar general to enable greater access to healthy food and wellness essential for million of healthcare consumer nationwide nationsbenefits integrates with dollar general to enable greater access to healthy food and wellness essential for million of healthcare consumer nationwide trump to cut protection for home health aide migrant farmworkers is atlantic hurricane season behind schedule here whats really going on a striking trend after texas banned abortion more woman nearly bled to death during miscarriage america tariffdriven buying spree leaf household saddled with debt and financially vulnerable elon musk want to create a new political party building rocket may be easier ge aerospace bear put spread could return in the next few month the humn etf let you invest in humanoid robotics stock should you buy in now the humn etf let you invest in humanoid robotics stock should you buy in now ge aerospace bear put spread could return in the next few month mortgage refinance demand surge a interest rate drop further cnbc u of m health care consulting fee adding up at rate of to per hour mortgage refinance demand surge a interest rate drop further certik hackd fortress building product accelerates fencing and steel framing growth strategy divests railing and lighting business to primesource brand inventus sign milling agreement with mcewen mining alta equipment group announces preferred stock dividend erdene commences trading on the otcqb riley permian announces closing of new mexico acquisition tonix pharmaceutical announces peerreviewed publication in cancer cell journal highlighting positive preclinical data of mtnx in gastric cancer animal model have an allamerican fourth of july with beef on the grill greystone logistics share information on stock buyback this is the key to building a personal brand that resonates with others olipops latest marketing stunt drew a person waitlistand sold out immediately alta equipment group announces preferred stock dividend pasinex announces annual and q financial result green thumb industry to hold second quarter earnings conference call on august whitestone reit announces second quarter earnings webcast and conference call the bestperforming sp stock of the last year have key commonality other than being ai stock can you guess it whitestone reit announces second quarter earnings webcast and conference call cipher mining surpasses hashrate growth forecast at black pearl and announces june operational update inventus sign milling agreement with mcewen mining riley permian announces closing of new mexico acquisition amc network announces early result and upsizing of tender offer for it senior note due amc network announces early result and upsizing of tender offer for it senior note due cardano price prediction ada price struggle to surpass a newcomer remittix gain ground with ico surge the bestperforming sp stock of the last year have key commonality other than being ai stock can you guess it token crypto presale go live price prediction x potential and what early buyer need to know now is bitcoin getting ready for a big price move in july water way technology enters strategic partnership for exclusive tomato hybrid development for vertical farming editorial stop the bleeding for colorado medicaid paramount resource ltd announces renewal of normal course issuer bid and july dividend pyrogenesis sign contract targeting plastic waste management problem in europe mda space completes acquisition of satixfy communication cipher mining surpasses hashrate growth forecast at black pearl and announces june operational update valore report result from successful hole trado auger drilling campaign at pedra branca including m at gt pgeau from surface dr phone fix expands partnership with assurant to accelerate certified preowned phone sale across canada what are the best vanguard etf for a wellrounded portfolio first horizon corporation announces redemption of series b preferred stock and corresponding series b depositary share what are the best vanguard etf for a wellrounded portfolio wallbridge exploration drilling continues to intercept highgrade gold mineralization at martiniere consumertech brand nothing tap cevas realspace software to bring immersive spatial audio to headphone and earbuds primesource brand acquires fortress railing product shattuck lab announces participation in upcoming leerink partner therapeutic forum ii and metabolism pyrogenesis sign contract targeting plastic waste management problem in europe dayforce empowers canadian small and midsized business with powerpay by dayforce identiv partner with narravero to accelerate digital product passport adoption and compliance blue sky uranium acquires key subsurface data for corcovo uranium project mendoza province argentina verkkokauppacom to publish januaryjune halfyear report on july crypto loss surpass billion in h certik report reveals alarming rise in phishing attack blue sky uranium acquires key subsurface data for corcovo uranium project mendoza province argentina main street announces followon portfolio investment paramount global and donald trump settle for million inside america department store tarifftriggered price hike are picking up robeco institutional asset management bv ha million position in dollar general corporation nysedg after trump warns elon musk to close up shop china rally behind world richest man there no need to keep putting up with it year old grocery store staple file for bankruptcy northisle announces near surface intercept and highergrade intercept at depth at west goodspeed on it north island project stock market news dow set to open higher after senate pass spending bill barrons meeka metal begin gold production at murchison project australia seeking stable passive income in crypto quid miner offer a sustainable new cloud mining solution democrat the last holdout bear could be the key to a new stockmarket rally marketwatch smart gas meter market worth billion by marketsandmarketstm yieldmax etf announces distribution on smcy ulty msty wntr lfgy and others yieldmax etf announces distribution on smcy ulty msty wntr lfgy and others aldi is selling a comfort sandal for just it a perfect oofos dupe but cheaper kkr bet on sustainable protein demand with proten investment in australia kitron receive eur million contract for defense airborne radar application northern trust q earnings what to expect northern trust q earnings what to expect murkowski got to yes on t megabill thanks to spending for alaska how the megabill will limit health care access and plan to ease gun regulation iran president approves law suspending cooperation with un nuclear watchdog new study reveals brutal hit that u employer face from trump tariff another one bite the dust cbs settle with trump over infamous kamala minute segment letter to the editor a plea to boulder earbud hiker no excuse for not repaying student loan guthrie song is a relevant a ever guest opinion stuart c lord education wa my way out this bill slam that door shut house republican race toward a final vote on trump tax bill daring critic to oppose guest opinion christopher schweitzer the siren song of unreason is a dangerous plunge into darkness hollywood lost the plot now rebel are making movie great again what the rd budget proposal say about the future of war is atlantic hurricane season behind schedule here whats really going on trump immigration crackdown ripple through economy a striking trend after texas banned abortion more woman nearly bled to death during miscarriage america tariffdriven buying spree leaf household saddled with debt and financially vulnerable elon musk want to create a new political party building rocket may be easier politician push jobkilling minimum wage hike while ignoring the devastating economic reality editorial attacking zohran mamdanis u citizenship is contemptible and dangerous republican rep jim jordan discusses trumpbacked megabill after senate passage rash kid have been abducted from ukraine these midwest senator want to find them a welcome shift in federal financial reporting wednesday letter sen budd where is your courage where is your honesty grow keep an eye out for brown patch disease in coolseason grass american opinion instead of ice raid on farmworkers overhaul this visa program cytosorbents provides u fda and health canada regulatory update for drugsorbatr best of the babylon bee defeated cuomo left groping for answer berry tramel rising valuation of nba franchise will prompt thunder ownership to sell opinion minneapolis police chief brian ohara is getting a bum rap over lake street raid year old grocery store staple file for bankruptcy democratic gov janet mill discusses how the gop megabill will impact maine maine cant afford to lose federal funding governor say modestly bipartisan budget could go to full wisconsin legislature wednesday gop megabill head back to the house for final approval u wont send some weapon pledged to ukraine following a pentagon review of military aid what the mar elia church bombing mean for syria future artificial intelligence saving you money and helping massdot build faster republican holdout head to the white house to discus trump bill letter patriot not saying much on ice treatment of veteran opinion a july approach supreme court sign away american democracy trump put senate in play in wall street journal new jersey gubernatorial candidate to speak at made in nj manufacturing day trump put senate in play in wall street journal nelly denies he maga say kamala harris locked up black ha white husband trump put senate in play in wall street journal trump put senate in play in wall street journal trump put senate in play in wall street journal trump put senate in play in wall street journal trump put senate in play in wall street journal trump put senate in play in wall street journal lawrence odonnells unfiltered reaction to bonkers trump presser moment say it all how ai can help ease the strain on health care service man charged in deadly brockton stabbing pleads not guilty house republican race toward a final vote on trump tax bill sen ron johnson a yes on trump budget bill sen tammy baldwin disgusted by it holy cow history happy july whatever green bay prison would close by under republican budget proposal gen z is the worst at work right wrong thing to know for july usaid ukraine munition trump megabill climate change paramount settlement former insurance commissioner say lara should go california focus former insurance commissioner say lara should go california focus letter spending choice make republican leader priority clear incredible growth stock poised for longterm gain win an ar old state saloon present conspiracy theory trivia and salooncast with ian carroll a twonight blast of truth tech and patriotism analysis show trump tariff would cost u employer billion if elon stick to rocket i will stick to finance bessent shrug off musk debt drama lancashire need to set investment priority to get biggest bang for buck can south korea deescalate north korea without u support how to be editor for a day notorious husband and wife professional tenant indicted on criminal charge we will not let hate win provincetown town manager say following second incident protect your pet on the fourth of july editor for a day letter constitutional system seems abandoned the u military cant quit the middle east another voice financial restitution is necessary but not sufficient for abuse survivor letter war against diversity education in unjust and disrespect history sean diddy comb found guilty on count acquitted of most serious charge firework warehouse explodes in california dalai lama say he intends to reincarnate after death ukraine look to jointly produce weapon with ally while u halt some shipment honolulu board of water supply sue navy for b over red hill fuel leak governor state budget veto trim public school maintenance new hawaii firework law take effect today hooser walking through my thought and value federal climate website go dark a trump administration promise policy reset house gop leader scrambling to rally holdout behind trump megabill house gop leader scrambling to rally holdout behind trump megabill house gop leader scrambling to rally holdout behind trump megabill house gop leader scrambling to rally holdout behind trump megabill house gop leader scrambling to rally holdout behind trump megabill house gop leader scrambling to rally holdout behind trump megabill leore james kowarsch liz shulman will big tech transform school into an ai video game jerald mcnair doe student use of ai spell the end for homework trump lit a fire under nato but more need to be done to contain the russiachina axis north korea to send a many a troop to bolster russia force ukrainian official say trump pick to run federal watchdog a yearold who once shared a conspiracy video and ha tie to a holocaust denier letter keep an eye on what matter not just what seems exciting editorial financial hit keep on coming and city hall only response is excuse steve chapman congress and the supreme court approve donald trump drive for absolute power letter why centrism doesnt have enough bite to make an impact</t>
+          <t>halftime show icon take big fall get injured during wnba commissioner cup championship after paying u tariff on it product busy baby look to europe and australia a future market dan ives urge apple to make a move saying that perplexity acquisition is a nobrainer it a matter of when and not if centene stock plummet what sparked the brutal selloff centene stock plummet what sparked the brutal selloff barrons iran president approves law suspending cooperation with un nuclear watchdog invivyd and leading researcher form spear spike protein elimination and recovery study group first horizon corporation announces redemption of series b preferred stock and corresponding series b depositary share new study reveals brutal hit that u employer face from trump tariff huffpost fortnite how to get the battle bus suv try this trick wildfire kill people in spain a part of europe bake in heat wave think you missed the ai rally these gridbacked play are just getting warmed up tech billionaire launch erebor bank to fill svbs gap invivyd and leading researcher form spear spike protein elimination and recovery study group to ass the effect of monoclonal antibody therapy for long covid and covid postvaccination syndrome diversified energy promotes michael garrett to chief accounting officer diversified energy promotes michael garrett to chief accounting officer uk investor see not one but two pathway to rail merger developer acquire land for westgate village at north congress avenue west palm beach florida argon ai raise m to build the ai workspace powering the future of life science nationsbenefits integrates with dollar general to enable greater access to healthy food and wellness essential for million of healthcare consumer nationwide nationsbenefits integrates with dollar general to enable greater access to healthy food and wellness essential for million of healthcare consumer nationwide trump to cut protection for home health aide migrant farmworkers is atlantic hurricane season behind schedule here whats really going on a striking trend after texas banned abortion more woman nearly bled to death during miscarriage america tariffdriven buying spree leaf household saddled with debt and financially vulnerable elon musk want to create a new political party building rocket may be easier ge aerospace bear put spread could return in the next few month the humn etf let you invest in humanoid robotics stock should you buy in now the humn etf let you invest in humanoid robotics stock should you buy in now ge aerospace bear put spread could return in the next few month mortgage refinance demand surge a interest rate drop further cnbc u of m health care consulting fee adding up at rate of to per hour mortgage refinance demand surge a interest rate drop further certik hackd fortress building product accelerates fencing and steel framing growth strategy divests railing and lighting business to primesource brand inventus sign milling agreement with mcewen mining alta equipment group announces preferred stock dividend erdene commences trading on the otcqb riley permian announces closing of new mexico acquisition tonix pharmaceutical announces peerreviewed publication in cancer cell journal highlighting positive preclinical data of mtnx in gastric cancer animal model have an allamerican fourth of july with beef on the grill greystone logistics share information on stock buyback this is the key to building a personal brand that resonates with others olipops latest marketing stunt drew a person waitlistand sold out immediately alta equipment group announces preferred stock dividend pasinex announces annual and q financial result green thumb industry to hold second quarter earnings conference call on august whitestone reit announces second quarter earnings webcast and conference call the bestperforming sp stock of the last year have key commonality other than being ai stock can you guess it whitestone reit announces second quarter earnings webcast and conference call cipher mining surpasses hashrate growth forecast at black pearl and announces june operational update inventus sign milling agreement with mcewen mining riley permian announces closing of new mexico acquisition amc network announces early result and upsizing of tender offer for it senior note due amc network announces early result and upsizing of tender offer for it senior note due cardano price prediction ada price struggle to surpass a newcomer remittix gain ground with ico surge the bestperforming sp stock of the last year have key commonality other than being ai stock can you guess it token crypto presale go live price prediction x potential and what early buyer need to know now is bitcoin getting ready for a big price move in july water way technology enters strategic partnership for exclusive tomato hybrid development for vertical farming editorial stop the bleeding for colorado medicaid paramount resource ltd announces renewal of normal course issuer bid and july dividend pyrogenesis sign contract targeting plastic waste management problem in europe mda space completes acquisition of satixfy communication cipher mining surpasses hashrate growth forecast at black pearl and announces june operational update valore report result from successful hole trado auger drilling campaign at pedra branca including m at gt pgeau from surface dr phone fix expands partnership with assurant to accelerate certified preowned phone sale across canada what are the best vanguard etf for a wellrounded portfolio first horizon corporation announces redemption of series b preferred stock and corresponding series b depositary share what are the best vanguard etf for a wellrounded portfolio wallbridge exploration drilling continues to intercept highgrade gold mineralization at martiniere consumertech brand nothing tap cevas realspace software to bring immersive spatial audio to headphone and earbuds primesource brand acquires fortress railing product shattuck lab announces participation in upcoming leerink partner therapeutic forum ii and metabolism pyrogenesis sign contract targeting plastic waste management problem in europe dayforce empowers canadian small and midsized business with powerpay by dayforce identiv partner with narravero to accelerate digital product passport adoption and compliance blue sky uranium acquires key subsurface data for corcovo uranium project mendoza province argentina verkkokauppacom to publish januaryjune halfyear report on july crypto loss surpass billion in h certik report reveals alarming rise in phishing attack blue sky uranium acquires key subsurface data for corcovo uranium project mendoza province argentina main street announces followon portfolio investment paramount global and donald trump settle for million inside america department store tarifftriggered price hike are picking up robeco institutional asset management bv ha million position in dollar general corporation nysedg after trump warns elon musk to close up shop china rally behind world richest man there no need to keep putting up with it year old grocery store staple file for bankruptcy northisle announces near surface intercept and highergrade intercept at depth at west goodspeed on it north island project stock market news dow set to open higher after senate pass spending bill barrons meeka metal begin gold production at murchison project australia seeking stable passive income in crypto quid miner offer a sustainable new cloud mining solution democrat the last holdout bear could be the key to a new stockmarket rally marketwatch smart gas meter market worth billion by marketsandmarketstm yieldmax etf announces distribution on smcy ulty msty wntr lfgy and others yieldmax etf announces distribution on smcy ulty msty wntr lfgy and others aldi is selling a comfort sandal for just it a perfect oofos dupe but cheaper kkr bet on sustainable protein demand with proten investment in australia kitron receive eur million contract for defense airborne radar application northern trust q earnings what to expect northern trust q earnings what to expect murkowski got to yes on t megabill thanks to spending for alaska how the megabill will limit health care access and plan to ease gun regulation iran president approves law suspending cooperation with un nuclear watchdog new study reveals brutal hit that u employer face from trump tariff another one bite the dust cbs settle with trump over infamous kamala minute segment letter to the editor a plea to boulder earbud hiker no excuse for not repaying student loan guthrie song is a relevant a ever guest opinion stuart c lord education wa my way out this bill slam that door shut house republican race toward a final vote on trump tax bill daring critic to oppose guest opinion christopher schweitzer the siren song of unreason is a dangerous plunge into darkness hollywood lost the plot now rebel are making movie great again what the rd budget proposal say about the future of war is atlantic hurricane season behind schedule here whats really going on trump immigration crackdown ripple through economy a striking trend after texas banned abortion more woman nearly bled to death during miscarriage america tariffdriven buying spree leaf household saddled with debt and financially vulnerable elon musk want to create a new political party building rocket may be easier politician push jobkilling minimum wage hike while ignoring the devastating economic reality editorial attacking zohran mamdanis u citizenship is contemptible and dangerous republican rep jim jordan discus trumpbacked megabill after senate passage rash kid have been abducted from ukraine these midwest senator want to find them a welcome shift in federal financial reporting wednesday letter sen budd where is your courage where is your honesty grow keep an eye out for brown patch disease in coolseason grass american opinion instead of ice raid on farmworkers overhaul this visa program cytosorbents provides u fda and health canada regulatory update for drugsorbatr best of the babylon bee defeated cuomo left groping for answer berry tramel rising valuation of nba franchise will prompt thunder ownership to sell opinion minneapolis police chief brian ohara is getting a bum rap over lake street raid year old grocery store staple file for bankruptcy democratic gov janet mill discus how the gop megabill will impact maine maine cant afford to lose federal funding governor say modestly bipartisan budget could go to full wisconsin legislature wednesday gop megabill head back to the house for final approval u wont send some weapon pledged to ukraine following a pentagon review of military aid what the mar elia church bombing mean for syria future artificial intelligence saving you money and helping massdot build faster republican holdout head to the white house to discus trump bill letter patriot not saying much on ice treatment of veteran opinion a july approach supreme court sign away american democracy trump put senate in play in wall street journal new jersey gubernatorial candidate to speak at made in nj manufacturing day trump put senate in play in wall street journal nelly denies he maga say kamala harris locked up black ha white husband trump put senate in play in wall street journal trump put senate in play in wall street journal trump put senate in play in wall street journal trump put senate in play in wall street journal trump put senate in play in wall street journal trump put senate in play in wall street journal lawrence odonnells unfiltered reaction to bonkers trump presser moment say it all how ai can help ease the strain on health care service man charged in deadly brockton stabbing pleads not guilty house republican race toward a final vote on trump tax bill sen ron johnson a yes on trump budget bill sen tammy baldwin disgusted by it holy cow history happy july whatever green bay prison would close by under republican budget proposal gen z is the worst at work right wrong thing to know for july usaid ukraine munition trump megabill climate change paramount settlement former insurance commissioner say lara should go california focus former insurance commissioner say lara should go california focus letter spending choice make republican leader priority clear incredible growth stock poised for longterm gain win an ar old state saloon present conspiracy theory trivia and salooncast with ian carroll a twonight blast of truth tech and patriotism analysis show trump tariff would cost u employer billion if elon stick to rocket i will stick to finance bessent shrug off musk debt drama lancashire need to set investment priority to get biggest bang for buck can south korea deescalate north korea without u support how to be editor for a day notorious husband and wife professional tenant indicted on criminal charge we will not let hate win provincetown town manager say following second incident protect your pet on the fourth of july editor for a day letter constitutional system seems abandoned the u military cant quit the middle east another voice financial restitution is necessary but not sufficient for abuse survivor letter war against diversity education in unjust and disrespect history sean diddy comb found guilty on count acquitted of most serious charge firework warehouse explodes in california dalai lama say he intends to reincarnate after death ukraine look to jointly produce weapon with ally while u halt some shipment honolulu board of water supply sue navy for b over red hill fuel leak governor state budget veto trim public school maintenance new hawaii firework law take effect today hooser walking through my thought and value federal climate website go dark a trump administration promise policy reset house gop leader scrambling to rally holdout behind trump megabill house gop leader scrambling to rally holdout behind trump megabill house gop leader scrambling to rally holdout behind trump megabill house gop leader scrambling to rally holdout behind trump megabill house gop leader scrambling to rally holdout behind trump megabill house gop leader scrambling to rally holdout behind trump megabill leore james kowarsch liz shulman will big tech transform school into an ai video game jerald mcnair doe student use of ai spell the end for homework trump lit a fire under nato but more need to be done to contain the russiachina axis north korea to send a many a troop to bolster russia force ukrainian official say trump pick to run federal watchdog a yearold who once shared a conspiracy video and ha tie to a holocaust denier letter keep an eye on what matter not just what seems exciting editorial financial hit keep on coming and city hall only response is excuse steve chapman congress and the supreme court approve donald trump drive for absolute power letter why centrism doesnt have enough bite to make an impact</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t xml:space="preserve">u employer added a surprising job last month despite uncertainty over economic policy canada trade deficit in may narrow export to u drop millionaire renter surge in nyc a high earner opt for luxury lease report trader pare bet on fed rate cut after job report here lindsell train global equity fund comment on nintendo co ltd ntdoy stock market today dow sp and nasdaq future advance after strong payroll data trump tax and spending bill face vote marketwatch new online casino canada reddit user share the leading real money online casino for tcl csot exclusively supply display for xiaomi mix flip and xiaomi yu powering xiaomis new beginning blowout june payroll k job added smashing expectation unemployment rate drop to avdx alert monsey firm of wohl fruchter investigating fairness of the sale of avidxchange holding to tpg global and corpay dune awakening drop massive july update fix exploit and rebalances pvp zone clearmind medicine announces irb approval for phase a clinical trial for alcohol use disorder at tel aviv sourasky medical center u stock and bond market are open on eve of july but they close early trump want the world to squeeze out china he starting with vietnam u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low trader pare bet on fed rate cut after job report yahoo finance u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low parazero receives a recurring bulk order of safeair system from an australian distributor nyt strand july serf a sweet scoop with icecream a spangram half yearly report on lvmhs liquidity contract with oddo bhf sca half yearly report on lvmhs liquidity contract with oddo bhf sca these fossil fuel stock rallied a senate passed trump tax spending plan deep tristate layoff leave continuing jobless claim stuck at highest since canada trade deficit narrow in may a export rise these fossil fuel stock rallied a senate passed trump tax spending plan investor business daily ford jpmorgan amazon executive predict deep job cut a ai advance u weekly firsttime unemployment claim fewest since may ap business summarybrief at am edt u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low review liquid death on fire plus one of the most unique thc drink yet hog look to close thing out ahead of holiday break cotton mixed in early thursday trade corn pushing gain into thursday morning trade cattle look to round out short week wheat sneaking out gain ahead of threeday weekend soybean strength continuing on thursday am top financial stock you may want to dump this quarter house beat and hidden venue a new sound is emerging in abu dhabi u employer added a surprising job last month despite uncertainty over economic policy u employer added a surprising job last month despite uncertainty over economic policy starbucks offer million stock bonus to exec but should you buy it share here what technical analysis show fed rate cut appears less likely after strongerthanforecast june payroll data green science alliance established an electric vehicle ev company utilizing next generation inwheel motor technology developed by a japanese engineer who pioneered supercar ev named eliica over year ago u economy add new job unemployment rate dip to percent in june stock market today dow sp nasdaq future hit pause after a solid job report liveone synervoz partner for nextgen voice experience u employer added job in june strategy stock rise after key trading signal jobless claim fall to lowest level since midmay sp build on record high future rising after strong job report barrons my parent gifted me what should i do with it u economy add job in june more than expected popular restaurant chain close all location no bankruptcy u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low trade deficit widens surpassing both forecast and previous figure u job growth beat expectation in june celebrate independence wilmatm set aba practice free from manual workflow with powerful patient relationship management nike is back in the race billionaire bill ackman urge tired subdued andrew cuomo to drop out of nyc mayoral race begrudgingly endorses eric adam u payroll increased by in june more than expected navitas semiconductor to participate in upcoming cjs security conference u add k job in june beating expectation u initial jobless claim dip below expectation bolstering usd u employer added job in june a labor market show resilience despite uncertainty over trump economic policy u employer added job in june a labor market show resilience despite uncertainty over trump economic policy labor market stay afloat a hiring top forecastsagain u employer added job in june a labor market show resilience despite uncertainty over trump economic policy airline face investor after strong but cheaper july holiday cnbc lamplight luxury rv park invite traveler to discover their perfect texas getaway at holiday road rv park dsh hotel advisor close jacksonville fl candlewood suite sale a hospitality market heat up lamplight luxury rv park invite traveler to discover their perfect texas getaway at holiday road rv park navitas semiconductor to participate in upcoming cjs security conference dsh hotel advisor close jacksonville fl candlewood suite sale a hospitality market heat up nonfarm payroll beat expectation indicating robust u job market coinex research june report bitcoin in the crossfire u payroll increased by in june more than expected cnbc etoro appoints former sec commissioner laura unger and wix cfo lior shemesh a board member beauty and the bear michael burry estee lauder snub china smci stock get price target bump but it still below current share price agf announces passing of kevin mccreadie ceo and cio coreweave is the first cloud provider to deploy nvidias latest ai chip why kelly slater moved headquarters of his sustainable clothing brand from la to san diego why kelly slater moved headquarters of his sustainable clothing brand from la to san diego why kelly slater moved headquarters of his sustainable clothing brand from la to san diego why kelly slater moved headquarters of his sustainable clothing brand from la to san diego why kelly slater moved headquarters of his sustainable clothing brand from la to san diego why kelly slater moved headquarters of his sustainable clothing brand from la to san diego why kelly slater moved headquarters of his sustainable clothing brand from la to san diego can california democrat require ice agent to unmask and show id trump show america wont tolerate nuclear threat james fitzpatrick trump show america wont tolerate nuclear threat james fitzpatrick texas internet porn law is constitutional common sense prevails dallas morning news texas internet porn law is constitutional common sense prevails dallas morning news texas internet porn law is constitutional common sense prevails dallas morning news trump show america wont tolerate nuclear threat james fitzpatrick trump show america wont tolerate nuclear threat james fitzpatrick texas internet porn law is constitutional common sense prevails dallas morning news trump show america wont tolerate nuclear threat james fitzpatrick texas internet porn law is constitutional common sense prevails dallas morning news texas internet porn law is constitutional common sense prevails dallas morning news trump show america wont tolerate nuclear threat james fitzpatrick texas internet porn law is constitutional common sense prevails dallas morning news texas internet porn law is constitutional common sense prevails dallas morning news texas internet porn law is constitutional common sense prevails dallas morning news trump show america wont tolerate nuclear threat james fitzpatrick trump show america wont tolerate nuclear threat james fitzpatrick trump show america wont tolerate nuclear threat james fitzpatrick texas internet porn law is constitutional common sense prevails dallas morning news congressional intern killed in dc shooting scrum alliance ranked on comparablys list of best leadership team among small company judge strike down trump policy that deleted transgender page from govt website house beat and hidden venue a new sound is emerging in abu dhabi federal judge rule noncalifornia resident can apply for concealedcarry gun permit the latest house leader rush toward a final vote a democrat hold the floor what maga mean to american u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low aclu sue to block ice raid in southern california alleging constitutional violation u employer added job in june a labor market show resilience despite uncertainty over trump economic policy u employer added job in june a labor market show resilience despite uncertainty over trump economic policy california boost film and tv tax credit to million to preserve job attorney general tap politically connected billing lawyer for judicial discipline panel dnrcs drought outlook for montana is grim going into hot dry summer attorney general tap politically connected billing lawyer for judicial discipline panel attorney general tap politically connected billing lawyer for judicial discipline panel double standard no no standard did the pentagon spread false ufo story were skeptical trump t megabill set house record for longest vote in history number of megarounds drop in first half a biotech struggle against worsening slump california school official say video show immigration agent urinating in public view homeland security investigating iran suspends cooperation with un nuclear monitoring agency a slider a milestone and a heartfelt thank you kershaws th strikeout federal funding for contraceptive access return to missouri nonprofit after threemonth freeze dan walter california lawmaker finally achieve holy grail reform of state key environmental law jeffries us magic minute to delay vote on trump megabill after settling with trump cbs news staffer fear what come next some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say family of slain police officer krystal rivera shot by a fellow officer want an independent investigation vance boelter man charged in minnesota lawmaker shooting due back in federal court how george washington america reluctant leader contrast with today frederic j fransen choosing war over diplomacy increase danger for u elizabeth shackelford choosing war over diplomacy increase danger for u elizabeth shackelford choosing war over diplomacy increase danger for u elizabeth shackelford how george washington america reluctant leader contrast with today frederic j fransen choosing war over diplomacy increase danger for u elizabeth shackelford how george washington america reluctant leader contrast with today frederic j fransen choosing war over diplomacy increase danger for u elizabeth shackelford choosing war over diplomacy increase danger for u elizabeth shackelford how george washington america reluctant leader contrast with today frederic j fransen how george washington america reluctant leader contrast with today frederic j fransen how george washington america reluctant leader contrast with today frederic j fransen choosing war over diplomacy increase danger for u elizabeth shackelford choosing war over diplomacy increase danger for u elizabeth shackelford how george washington america reluctant leader contrast with today frederic j fransen choosing war over diplomacy increase danger for u elizabeth shackelford choosing war over diplomacy increase danger for u elizabeth shackelford choosing war over diplomacy increase danger for u elizabeth shackelford how george washington america reluctant leader contrast with today frederic j fransen how george washington america reluctant leader contrast with today frederic j fransen how george washington america reluctant leader contrast with today frederic j fransen how can azerbaijan be ally with iran and israel nova ukraine earns platinum seal of transparency from candid ukraine kill one of the highestranking russian officer of the conflict federal budget megabill would shift billion in cost to missouri taxpayer ups violates teamster national contract with plan for buyout chile cut up to of red tape promise streamlined mining approval colorado education leader urge trump to release million in k school funding capitol walkway backed by gov polis is a bridge to nowhere key lawmaker say a project face criticism colorado education leader urge trump to release million in k school funding capitol walkway backed by gov polis is a bridge to nowhere key lawmaker say a project face criticism colorado education leader urge trump to release million in k school funding colorado education leader urge trump to release million in k school funding opinion pb is a national treasure worthy of government support the best american express credit card for picked by a frequent traveler trump cut are squeezing america most popular national park in peak season here what mental health study should look like at a christian college steven eng a christian crisis across our nation and in our backyard the united state just cut off key defense aid to ukraine stock to buy with less than nordstrom rack is selling a gorgeous kendra scott necklace for and shopper get so many compliment openai ceo sam altman say he politically homeless in july post bashing democrat what to expect from boston scientifics next quarterly earnings report buttonwood financial advisor inc ha million holding in meta platform inc nasdaqmeta crown wealth group llc buy share of meta platform inc nasdaqmeta bankplus wealth management llc grows position in meta platform inc nasdaqmeta shilanski associate inc raise holding in meta platform inc nasdaqmeta amalgamated bank acquires share of meta platform inc nasdaqmeta monument capital management buy share of meta platform inc nasdaqmeta best car insurance company of july risk remains of uschina trade truce breakdown capital economics say ups make drastic change it never done before in year history a part of major overhaul the secret to great grilled kabob it all in the cut prediction this magnificent artificial intelligence ai stock will skyrocket to new high in july bitcoin price on the brink a congress introduces a new groundbreaking crypto bill forbes veraltos quarterly earnings preview what you need to know oppo pad se india launch check variant spec price breakdown sofi stock skyrocket in a year how high can it go in consolidated lithium metal announces exposure of a new libearing pegmatite at it preissac project and close financing bmo announces special cash distribution for etf series unit of bmo money market fund consolidated lithium metal announces exposure of a new libearing pegmatite at it preissac project and close financing niurstour i utboi rikisbrefa riks is trader joes open on the th of july best podcast headphone of auction result of treasury bond riks rtx corporation q earnings what to expect how to fix lenovo fingerprint scanner issue fast quick easy guide what to expect from dover q earnings report what you need to know ahead of erie indemnity earnings release petrovictory energy corp and azevedo travassos energia sa sign binding memorandum of understanding petrovictory energy corp and azevedo travassos energia sa sign binding memorandum of understanding sakana ai treequest deploy multimodel team that outperform individual llm by sony break exclusivity helldivers land on xbox this august tesla ha a problem and it not just the elon musk backlash bloombergcom eu stick with timeline for ai rule reuters lot of speculation is swirling around the sumy front wildfire cripple alberta oil production this is why tesla robotaxi launch needed human babysitter what to expect from raymond james financials q earnings report which store are open and closed on independence day kusacom btc hit k why pro trader arent fully confident yet the fiscal treadmill is speeding up and washington keep jogging after year of grinding i have million but am burned out what are my option these catalyst could lift micron stock higher in and beyond costco stock analysis buy sell or hold every breath you take affect how you move here how to fix both my smartest dividend stock to buy today earnings preview what to expect from globe life report here what to expect from ameriprise financials next earnings report key headwind facing usdc cme group quarterly earnings preview what you need to know is subway open on the fourth of july west fargo new herbz and spicez store offer customer allnatural alternative be resilient by accepting adversity and learning from it why black unemployment just rose to it highest level since january littleknown item in trump big agenda bill riley gaines ha been one of lia thomas most vocal critic she just scored two major win in her antitrans effort who the coolest person at your july barbecue they got six thing goin on according to a new study construction start on beacon at princeton hill at s dixie hwy homestead fl i visited universal studio and people were on their phone everywhereeven rollercoasters that habit is really hard to break expert say company in the new york city metro area that are great place to work the strategy that will make your sale call more successful editorial today we celebrate the real no king holiday how glen powell condiment brand made more than million in it first month azi announces receipt of minimum bid price notice from nasdaq fourth of july weekend lotterycom and sportscom driver revved up for midohio challenge stoneform launch a tokenized real estate platform to open up investment opportunity northwest copper announces closing of oversubscribed private placement bybit tradfi x crypto report regulatory tailwind drive coinbase outperformance despite premium valuation stoneform launch a tokenized real estate platform to open up investment opportunity esg hitgen release it inaugural sustainability report is chickfila closed on july northwest copper announces closing of oversubscribed private placement china using tiktok a a pawn to squeeze trump in trade talk source net zero now clear key milestone on acre energy campus accelerating alberta lowcarbon data center infrastructure build out whats open whats closed on july th what grocery store are open walmart costco target more alcom u future slide after trump say hell start sending tariff letter today setting levy up to musk back sen paul criticism of trump megabill in first comment since it passed cf cfrp market worth billion in exclusive report by marketsandmarketstm cf cfrp market worth billion in exclusive report by marketsandmarketstm trump vietnam pact take aim at china but it raise more question than answer cnbc new york state teacher retirement system sell share of avery dennison corporation nyseavy ameritas advisory service llc buy share of ulta beauty inc nasdaqulta these were the bestperforming stock in the dow jones industrial average in june hot dog eating contest host share prediction for this year winner partner value investment lp announces tenforone unit split xrp and ozak ai price prediction which token ha the clearer path to massive gain american flight diverts after nosy passenger cause bomb scare one mile at a time trump bill secures billion for u arctic surge six new icebreaker to counter russian and chinese dominance ethereum is powering wall street future the crypto scene at cannes show how far it come apex group appoints wang a chief ai and data science officer kinterra score small win in new world copper takeover fight new york state teacher retirement system reduces position in oge energy corporation nyseoge u patriotism among democrat crash a marxist demand grow louder birdie for charity in the final stretch to reach m milestone what oracle meta platform and nvidia stock investor should know about recent ai update amber international raise m to enhance m crypto ecosystem reserve best horror game that test your morality marsden launch workplace saving with charity pledge for first business in today gop there is no choice at all multiple suspect charged in separate drug dealing case in billing the secret to great grilled kabob it all in the cut is central asia the next target of russian aggression opinion congress making big mistake with energy tax credit what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean the house just did our patriotic duty to deliver tax relief and uphold our value what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean controversy a staggering amount of usmexico border is now militarized what is trump new realism in foreign policy to celebrate july fully consider the context of the declaration of independence selfevident truth every breath you take affect how you move here how to fix both my smartest dividend stock to buy today army experiment with integrating attack drone into artillery formation trump admin to adjust national park fee to prioritize american family over foreign tourist flooding in texas cause multiple fatality a guadalupe river surge to record level jocko willink in a sea of imperfect voice i heard the anthem and the spirit of a nation this july th a family wait american hostage father pleads for son freedom from hamas terrorist opinion bill lueders reason to celebrate july th why black unemployment just rose to it highest level since january littleknown item in trump big agenda bill riley gaines ha been one of lia thomas most vocal critic she just scored two major win in her antitrans effort guest opinion bj and brecken jones u supreme court got it right on parental right and education who the coolest person at your july barbecue they got six thing goin on according to a new study trump ha big plan for america next birthday historian have question trump to sign big beautiful bill in july fourth ceremony at white house editorial after year righteousness and truth must prevail letter to the editor county should be compensated for iris field honoring superintendent extraordinary service trump crowning moment is ammo for dems in america nonstop birthday party watt happening tonis weekly energy highlight hot dog eating contest host share prediction for this year winner opinion supreme court unitary executive theory threatens our balance of power trump concedes he made no progress on achieving top campaign promise democratic rep katherine clark discusses gop megabill heading for trump signature president trump take victory lap after congress pass tax cut and policy bill elote churrasco and churros alligator alcatraz worker fed by miami food truck scientist issue warning after detecting concerning surge in infection in domestic cat should be closely monitored chef who feed penn state student make summer shift helping family with meal are the worst of the storm behind u hateful trump trashed over fking disgusting line about half the country for th of july the allamerican director you dont know by name katy perry and orlando bloom confirm split what we know about the death of liverpool soccer star diogo jota and his brother la activist indicted after handing out face shield to antiice protester president trump to honor iran strike flight team at the white house glenn eden who is chicago greatest ambassador you editorial on july of all day a naturalized citizen is not less than a u citizen editorial america is soon to turn remember the warmth of the bicentennial heidi stevens on long list of thing being cut art may seem inconsequential it not zohran mamdani ha big housing plan here what stand in the way letter what july fourth mean to me a an ahmadi muslim american rep bob morgan what patriotism mean to me three year after the highland park mass shooting this artist hope to be chosen to make a sculpture for trump garden of american hero how ice raid turned part of los angeles into ghost town maggie mulqueen what doe summer mean for my family and me the beach and book a declaration of independence for these time trump pardon cost at least billion in restitution tax hike in december is helping local library raise worker wage and restore lost position ny official react to passage of big beautiful bill through congress impending signature into law who broke george washington walking stick at the sc statehouse yankee rebel an exgovernor hegseth halted weapon for ukraine despite military analysis that the aid wouldnt jeopardize u readiness legislature should act on the pernicious effect of cellphone in school trump success rate in the court so far letter budget cut harmful for health nutrition letter budget cut harmful for health nutrition think youre smarter than a slate associate writer find out with this week news quiz editorial cartoon for july world share are mostly down a trump tariff deadline loom while u stock set record trump pitch plan allowing farmer to vouch for illegal immigrant worker facing deportation blaze engulfs four home in la amid active firework a strike by air traffic controller is disrupting travel to from and over france trump ag secretary ha irony meter exploding left right and center with beyond parody spin trump decision to end taxfree loophole for lowvalue good from china lead to a sharp decline in air cargo shipment cyber school facing wrongful death suit say it unreasonable for teacher to see student weekly opinion blockbuster made me do it questionable advice from big summer movie pa republican gamble on rural health care a megabill push through cumberland county official optimistic that new memo will improve coordination with library system galasso look forward to tomorrow expectantly beyond current circumstance joey chestnut return to coney island expected to dominate hot dog eating contest trump proposes ufc fight at white house to celebrate year of independence will new england sky stay clear for friday night big firework show u colombia announce recall of envoy amid diplomatic rift lucas trump should demand the unconditional surrender of the democrat party food hygiene rating handed to four doncaster establishment one need major improvement elephant kill two female tourist from the uk and new zealand in zambian national park many missouri law restricting abortion blocked again by state judge iredell county name rodney harris a the new deputy county manager iran try keeping new military commander a secret mossad offer guessing game confirms winner atlanta clogged road bring out the rage in motorist opinion challenge opportunity and bright future in ct for dairy farming trump tear into marxist lunatic mamdani honor american hero in bold rebuke play these p plus free game in july xrp hold market confidence while lightchain ai latejuly launch prepares to broaden investor option rosen nationally regarded investor counsel encourages reckitt benckiser group plc investor to secure counsel before important deadline in security class action rbgly robinhood want to redo wall street on the blockchain gizmodo why tempus ai stock soared in june japan brace for more quake authority dismiss doomsday hype opec plus agrees to pump more oil in august the new york time trump reportedly told iran it wa ok to strike back after u attack i said go ahead i understand poland blast trumpputin dialogue after drone strike escalation walmart is selling calvin klein eternity perfume for only and shopper say it an unbeatable deal ap business summarybrief at pm edt ap business summarybrief at pm edt ap business summarybrief at pm edt ap business summarybrief at pm edt the newest stock in the sp ha soared since it ipo and it a buy right now according to wall street the newest stock in the sp ha soared since it ipo and it a buy right now according to wall street were watching a brain drain in real time openai hit hard a top researcher defect to rival tech giant meta rude baguette the best amazon prime day deal under save on gear from blink anker samsung and others engadget nextgen ai and social startup backed by thrive capital and y combinator shaping were on the brink of another big consumer wave click like sugar gambling in a world of quick pleasure an addiction expert say it might be time for a dopamine fast a amazon double down on robotaxis is amzn stock a buy charlize theron is choosing to be single she told call her daddy that can be a sign of strength say relationship expert the future of ai selfdriving car mechanical weeding health care assistant and more patriotic parade at the park the market hidden current delivering fast gain top romantic drama on ott to watch this weekend daily habit that separate high achiever from everyone else best altcoins for next bull run blockdags m summer raffle roi feature alongside inj rndr tia a forgotten megatrend that could be key to the ai economy quality nonus stock to buy in simply staggering cnn correspondent describes floodwater impact in texas good stock still worth buying in this market matt mower after nato summit europe free ride is on the line archer aviation the bet that could take off sooner than you think oneofakind brewery taproom closing no bankruptcy oneofakind brewery taproom closing no bankruptcy trump hit with backlash over use of antisemitic slur at iowa rally stage almost over arctic pablos price hike imminent a myro and housecoin push forward shopper race to get off all item in major closing down sale after iconic activewear brand shuts store investor deadline robbins geller rudman dowd llp announces that sarepta therapeutic inc srpt investor with substantial loss have opportunity to lead class action lawsuit one big beautiful budget deficit opec to increase output by barrel a day in august what it mean for oil market btc miner cloud mining platform strives to offer stability security a bitcoin recently crossed k amazon prime day the best deal live right now plus everything else you need to know engadget an iowa law rolling back trans civil right protection in the state ha taken effect here what to know thinkcarebelieve week of america victory walmart is selling a sleek digital camera for and shopper say it look professional subaru launch killer legacy lease offer for july top short anime to watch this weekend odd taxi death parade more safeway strike end a albertsons and local union reach agreement colorado public radio headed for sentencing sean diddy comb lawyer aim to show he no longer a bad boy for life the average american family is a millionaire how you can join them your kid is </t>
+          <t>u employer added a surprising job last month despite uncertainty over economic policy canada trade deficit in may narrow export to u drop millionaire renter surge in nyc a high earner opt for luxury lease report trader pare bet on fed rate cut after job report here lindsell train global equity fund comment on nintendo co ltd ntdoy stock market today dow sp and nasdaq future advance after strong payroll data trump tax and spending bill face vote marketwatch new online casino canada reddit user share the leading real money online casino for tcl csot exclusively supply display for xiaomi mix flip and xiaomi yu powering xiaomis new beginning blowout june payroll k job added smashing expectation unemployment rate drop to avdx alert monsey firm of wohl fruchter investigating fairness of the sale of avidxchange holding to tpg global and corpay dune awakening drop massive july update fix exploit and rebalances pvp zone clearmind medicine announces irb approval for phase a clinical trial for alcohol use disorder at tel aviv sourasky medical center u stock and bond market are open on eve of july but they close early trump want the world to squeeze out china he starting with vietnam u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low trader pare bet on fed rate cut after job report yahoo finance u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low parazero receives a recurring bulk order of safeair system from an australian distributor nyt strand july serf a sweet scoop with icecream a spangram half yearly report on lvmhs liquidity contract with oddo bhf sca half yearly report on lvmhs liquidity contract with oddo bhf sca these fossil fuel stock rallied a senate passed trump tax spending plan deep tristate layoff leave continuing jobless claim stuck at highest since canada trade deficit narrow in may a export rise these fossil fuel stock rallied a senate passed trump tax spending plan investor business daily ford jpmorgan amazon executive predict deep job cut a ai advance u weekly firsttime unemployment claim fewest since may ap business summarybrief at am edt u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low review liquid death on fire plus one of the most unique thc drink yet hog look to close thing out ahead of holiday break cotton mixed in early thursday trade corn pushing gain into thursday morning trade cattle look to round out short week wheat sneaking out gain ahead of threeday weekend soybean strength continuing on thursday am top financial stock you may want to dump this quarter house beat and hidden venue a new sound is emerging in abu dhabi u employer added a surprising job last month despite uncertainty over economic policy u employer added a surprising job last month despite uncertainty over economic policy starbucks offer million stock bonus to exec but should you buy it share here what technical analysis show fed rate cut appears le likely after strongerthanforecast june payroll data green science alliance established an electric vehicle ev company utilizing next generation inwheel motor technology developed by a japanese engineer who pioneered supercar ev named eliica over year ago u economy add new job unemployment rate dip to percent in june stock market today dow sp nasdaq future hit pause after a solid job report liveone synervoz partner for nextgen voice experience u employer added job in june strategy stock rise after key trading signal jobless claim fall to lowest level since midmay sp build on record high future rising after strong job report barrons my parent gifted me what should i do with it u economy add job in june more than expected popular restaurant chain close all location no bankruptcy u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low trade deficit widens surpassing both forecast and previous figure u job growth beat expectation in june celebrate independence wilmatm set aba practice free from manual workflow with powerful patient relationship management nike is back in the race billionaire bill ackman urge tired subdued andrew cuomo to drop out of nyc mayoral race begrudgingly endorses eric adam u payroll increased by in june more than expected navitas semiconductor to participate in upcoming cjs security conference u add k job in june beating expectation u initial jobless claim dip below expectation bolstering usd u employer added job in june a labor market show resilience despite uncertainty over trump economic policy u employer added job in june a labor market show resilience despite uncertainty over trump economic policy labor market stay afloat a hiring top forecastsagain u employer added job in june a labor market show resilience despite uncertainty over trump economic policy airline face investor after strong but cheaper july holiday cnbc lamplight luxury rv park invite traveler to discover their perfect texas getaway at holiday road rv park dsh hotel advisor close jacksonville fl candlewood suite sale a hospitality market heat up lamplight luxury rv park invite traveler to discover their perfect texas getaway at holiday road rv park navitas semiconductor to participate in upcoming cjs security conference dsh hotel advisor close jacksonville fl candlewood suite sale a hospitality market heat up nonfarm payroll beat expectation indicating robust u job market coinex research june report bitcoin in the crossfire u payroll increased by in june more than expected cnbc etoro appoints former sec commissioner laura unger and wix cfo lior shemesh a board member beauty and the bear michael burry estee lauder snub china smci stock get price target bump but it still below current share price agf announces passing of kevin mccreadie ceo and cio coreweave is the first cloud provider to deploy nvidias latest ai chip why kelly slater moved headquarters of his sustainable clothing brand from la to san diego why kelly slater moved headquarters of his sustainable clothing brand from la to san diego why kelly slater moved headquarters of his sustainable clothing brand from la to san diego why kelly slater moved headquarters of his sustainable clothing brand from la to san diego why kelly slater moved headquarters of his sustainable clothing brand from la to san diego why kelly slater moved headquarters of his sustainable clothing brand from la to san diego why kelly slater moved headquarters of his sustainable clothing brand from la to san diego can california democrat require ice agent to unmask and show id trump show america wont tolerate nuclear threat james fitzpatrick trump show america wont tolerate nuclear threat james fitzpatrick texas internet porn law is constitutional common sense prevails dallas morning news texas internet porn law is constitutional common sense prevails dallas morning news texas internet porn law is constitutional common sense prevails dallas morning news trump show america wont tolerate nuclear threat james fitzpatrick trump show america wont tolerate nuclear threat james fitzpatrick texas internet porn law is constitutional common sense prevails dallas morning news trump show america wont tolerate nuclear threat james fitzpatrick texas internet porn law is constitutional common sense prevails dallas morning news texas internet porn law is constitutional common sense prevails dallas morning news trump show america wont tolerate nuclear threat james fitzpatrick texas internet porn law is constitutional common sense prevails dallas morning news texas internet porn law is constitutional common sense prevails dallas morning news texas internet porn law is constitutional common sense prevails dallas morning news trump show america wont tolerate nuclear threat james fitzpatrick trump show america wont tolerate nuclear threat james fitzpatrick trump show america wont tolerate nuclear threat james fitzpatrick texas internet porn law is constitutional common sense prevails dallas morning news congressional intern killed in dc shooting scrum alliance ranked on comparablys list of best leadership team among small company judge strike down trump policy that deleted transgender page from govt website house beat and hidden venue a new sound is emerging in abu dhabi federal judge rule noncalifornia resident can apply for concealedcarry gun permit the latest house leader rush toward a final vote a democrat hold the floor what maga mean to american u application for jobless aid fell to last week a layoff remain low u application for jobless aid fell to last week a layoff remain low aclu sue to block ice raid in southern california alleging constitutional violation u employer added job in june a labor market show resilience despite uncertainty over trump economic policy u employer added job in june a labor market show resilience despite uncertainty over trump economic policy california boost film and tv tax credit to million to preserve job attorney general tap politically connected billing lawyer for judicial discipline panel dnrcs drought outlook for montana is grim going into hot dry summer attorney general tap politically connected billing lawyer for judicial discipline panel attorney general tap politically connected billing lawyer for judicial discipline panel double standard no no standard did the pentagon spread false ufo story were skeptical trump t megabill set house record for longest vote in history number of megarounds drop in first half a biotech struggle against worsening slump california school official say video show immigration agent urinating in public view homeland security investigating iran suspends cooperation with un nuclear monitoring agency a slider a milestone and a heartfelt thank you kershaws th strikeout federal funding for contraceptive access return to missouri nonprofit after threemonth freeze dan walter california lawmaker finally achieve holy grail reform of state key environmental law jeffries us magic minute to delay vote on trump megabill after settling with trump cbs news staffer fear what come next some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say some education grant in limbo were used for leftwing agenda trump administration say family of slain police officer krystal rivera shot by a fellow officer want an independent investigation vance boelter man charged in minnesota lawmaker shooting due back in federal court how george washington america reluctant leader contrast with today frederic j fransen choosing war over diplomacy increase danger for u elizabeth shackelford choosing war over diplomacy increase danger for u elizabeth shackelford choosing war over diplomacy increase danger for u elizabeth shackelford how george washington america reluctant leader contrast with today frederic j fransen choosing war over diplomacy increase danger for u elizabeth shackelford how george washington america reluctant leader contrast with today frederic j fransen choosing war over diplomacy increase danger for u elizabeth shackelford choosing war over diplomacy increase danger for u elizabeth shackelford how george washington america reluctant leader contrast with today frederic j fransen how george washington america reluctant leader contrast with today frederic j fransen how george washington america reluctant leader contrast with today frederic j fransen choosing war over diplomacy increase danger for u elizabeth shackelford choosing war over diplomacy increase danger for u elizabeth shackelford how george washington america reluctant leader contrast with today frederic j fransen choosing war over diplomacy increase danger for u elizabeth shackelford choosing war over diplomacy increase danger for u elizabeth shackelford choosing war over diplomacy increase danger for u elizabeth shackelford how george washington america reluctant leader contrast with today frederic j fransen how george washington america reluctant leader contrast with today frederic j fransen how george washington america reluctant leader contrast with today frederic j fransen how can azerbaijan be ally with iran and israel nova ukraine earns platinum seal of transparency from candid ukraine kill one of the highestranking russian officer of the conflict federal budget megabill would shift billion in cost to missouri taxpayer ups violates teamster national contract with plan for buyout chile cut up to of red tape promise streamlined mining approval colorado education leader urge trump to release million in k school funding capitol walkway backed by gov polis is a bridge to nowhere key lawmaker say a project face criticism colorado education leader urge trump to release million in k school funding capitol walkway backed by gov polis is a bridge to nowhere key lawmaker say a project face criticism colorado education leader urge trump to release million in k school funding colorado education leader urge trump to release million in k school funding opinion pb is a national treasure worthy of government support the best american express credit card for picked by a frequent traveler trump cut are squeezing america most popular national park in peak season here what mental health study should look like at a christian college steven eng a christian crisis across our nation and in our backyard the united state just cut off key defense aid to ukraine stock to buy with le than nordstrom rack is selling a gorgeous kendra scott necklace for and shopper get so many compliment openai ceo sam altman say he politically homeless in july post bashing democrat what to expect from boston scientifics next quarterly earnings report buttonwood financial advisor inc ha million holding in meta platform inc nasdaqmeta crown wealth group llc buy share of meta platform inc nasdaqmeta bankplus wealth management llc grows position in meta platform inc nasdaqmeta shilanski associate inc raise holding in meta platform inc nasdaqmeta amalgamated bank acquires share of meta platform inc nasdaqmeta monument capital management buy share of meta platform inc nasdaqmeta best car insurance company of july risk remains of uschina trade truce breakdown capital economics say ups make drastic change it never done before in year history a part of major overhaul the secret to great grilled kabob it all in the cut prediction this magnificent artificial intelligence ai stock will skyrocket to new high in july bitcoin price on the brink a congress introduces a new groundbreaking crypto bill forbes veraltos quarterly earnings preview what you need to know oppo pad se india launch check variant spec price breakdown sofi stock skyrocket in a year how high can it go in consolidated lithium metal announces exposure of a new libearing pegmatite at it preissac project and close financing bmo announces special cash distribution for etf series unit of bmo money market fund consolidated lithium metal announces exposure of a new libearing pegmatite at it preissac project and close financing niurstour i utboi rikisbrefa riks is trader joes open on the th of july best podcast headphone of auction result of treasury bond riks rtx corporation q earnings what to expect how to fix lenovo fingerprint scanner issue fast quick easy guide what to expect from dover q earnings report what you need to know ahead of erie indemnity earnings release petrovictory energy corp and azevedo travassos energia sa sign binding memorandum of understanding petrovictory energy corp and azevedo travassos energia sa sign binding memorandum of understanding sakana ai treequest deploy multimodel team that outperform individual llm by sony break exclusivity helldivers land on xbox this august tesla ha a problem and it not just the elon musk backlash bloombergcom eu stick with timeline for ai rule reuters lot of speculation is swirling around the sumy front wildfire cripple alberta oil production this is why tesla robotaxi launch needed human babysitter what to expect from raymond james financials q earnings report which store are open and closed on independence day kusacom btc hit k why pro trader arent fully confident yet the fiscal treadmill is speeding up and washington keep jogging after year of grinding i have million but am burned out what are my option these catalyst could lift micron stock higher in and beyond costco stock analysis buy sell or hold every breath you take affect how you move here how to fix both my smartest dividend stock to buy today earnings preview what to expect from globe life report here what to expect from ameriprise financials next earnings report key headwind facing usdc cme group quarterly earnings preview what you need to know is subway open on the fourth of july west fargo new herbz and spicez store offer customer allnatural alternative be resilient by accepting adversity and learning from it why black unemployment just rose to it highest level since january littleknown item in trump big agenda bill riley gaines ha been one of lia thomas most vocal critic she just scored two major win in her antitrans effort who the coolest person at your july barbecue they got six thing goin on according to a new study construction start on beacon at princeton hill at s dixie hwy homestead fl i visited universal studio and people were on their phone everywhereeven rollercoasters that habit is really hard to break expert say company in the new york city metro area that are great place to work the strategy that will make your sale call more successful editorial today we celebrate the real no king holiday how glen powell condiment brand made more than million in it first month azi announces receipt of minimum bid price notice from nasdaq fourth of july weekend lotterycom and sportscom driver revved up for midohio challenge stoneform launch a tokenized real estate platform to open up investment opportunity northwest copper announces closing of oversubscribed private placement bybit tradfi x crypto report regulatory tailwind drive coinbase outperformance despite premium valuation stoneform launch a tokenized real estate platform to open up investment opportunity esg hitgen release it inaugural sustainability report is chickfila closed on july northwest copper announces closing of oversubscribed private placement china using tiktok a a pawn to squeeze trump in trade talk source net zero now clear key milestone on acre energy campus accelerating alberta lowcarbon data center infrastructure build out whats open whats closed on july th what grocery store are open walmart costco target more alcom u future slide after trump say hell start sending tariff letter today setting levy up to musk back sen paul criticism of trump megabill in first comment since it passed cf cfrp market worth billion in exclusive report by marketsandmarketstm cf cfrp market worth billion in exclusive report by marketsandmarketstm trump vietnam pact take aim at china but it raise more question than answer cnbc new york state teacher retirement system sell share of avery dennison corporation nyseavy ameritas advisory service llc buy share of ulta beauty inc nasdaqulta these were the bestperforming stock in the dow jones industrial average in june hot dog eating contest host share prediction for this year winner partner value investment lp announces tenforone unit split xrp and ozak ai price prediction which token ha the clearer path to massive gain american flight diverts after nosy passenger cause bomb scare one mile at a time trump bill secures billion for u arctic surge six new icebreaker to counter russian and chinese dominance ethereum is powering wall street future the crypto scene at cannes show how far it come apex group appoints wang a chief ai and data science officer kinterra score small win in new world copper takeover fight new york state teacher retirement system reduces position in oge energy corporation nyseoge u patriotism among democrat crash a marxist demand grow louder birdie for charity in the final stretch to reach m milestone what oracle meta platform and nvidia stock investor should know about recent ai update amber international raise m to enhance m crypto ecosystem reserve best horror game that test your morality marsden launch workplace saving with charity pledge for first business in today gop there is no choice at all multiple suspect charged in separate drug dealing case in billing the secret to great grilled kabob it all in the cut is central asia the next target of russian aggression opinion congress making big mistake with energy tax credit what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean the house just did our patriotic duty to deliver tax relief and uphold our value what the justice department push to bring denaturalization case mean what the justice department push to bring denaturalization case mean controversy a staggering amount of usmexico border is now militarized what is trump new realism in foreign policy to celebrate july fully consider the context of the declaration of independence selfevident truth every breath you take affect how you move here how to fix both my smartest dividend stock to buy today army experiment with integrating attack drone into artillery formation trump admin to adjust national park fee to prioritize american family over foreign tourist flooding in texas cause multiple fatality a guadalupe river surge to record level jocko willink in a sea of imperfect voice i heard the anthem and the spirit of a nation this july th a family wait american hostage father pleads for son freedom from hamas terrorist opinion bill lueders reason to celebrate july th why black unemployment just rose to it highest level since january littleknown item in trump big agenda bill riley gaines ha been one of lia thomas most vocal critic she just scored two major win in her antitrans effort guest opinion bj and brecken jones u supreme court got it right on parental right and education who the coolest person at your july barbecue they got six thing goin on according to a new study trump ha big plan for america next birthday historian have question trump to sign big beautiful bill in july fourth ceremony at white house editorial after year righteousness and truth must prevail letter to the editor county should be compensated for iris field honoring superintendent extraordinary service trump crowning moment is ammo for dems in america nonstop birthday party watt happening tonis weekly energy highlight hot dog eating contest host share prediction for this year winner opinion supreme court unitary executive theory threatens our balance of power trump concedes he made no progress on achieving top campaign promise democratic rep katherine clark discus gop megabill heading for trump signature president trump take victory lap after congress pass tax cut and policy bill elote churrasco and churros alligator alcatraz worker fed by miami food truck scientist issue warning after detecting concerning surge in infection in domestic cat should be closely monitored chef who feed penn state student make summer shift helping family with meal are the worst of the storm behind u hateful trump trashed over fking disgusting line about half the country for th of july the allamerican director you dont know by name katy perry and orlando bloom confirm split what we know about the death of liverpool soccer star diogo jota and his brother la activist indicted after handing out face shield to antiice protester president trump to honor iran strike flight team at the white house glenn eden who is chicago greatest ambassador you editorial on july of all day a naturalized citizen is not le than a u citizen editorial america is soon to turn remember the warmth of the bicentennial heidi stevens on long list of thing being cut art may seem inconsequential it not zohran mamdani ha big housing plan here what stand in the way letter what july fourth mean to me a an ahmadi muslim american rep bob morgan what patriotism mean to me three year after the highland park mass shooting this artist hope to be chosen to make a sculpture for trump garden of american hero how ice raid turned part of los angeles into ghost town maggie mulqueen what doe summer mean for my family and me the beach and book a declaration of independence for these time trump pardon cost at least billion in restitution tax hike in december is helping local library raise worker wage and restore lost position ny official react to passage of big beautiful bill through congress impending signature into law who broke george washington walking stick at the sc statehouse yankee rebel an exgovernor hegseth halted weapon for ukraine despite military analysis that the aid wouldnt jeopardize u readiness legislature should act on the pernicious effect of cellphone in school trump success rate in the court so far letter budget cut harmful for health nutrition letter budget cut harmful for health nutrition think youre smarter than a slate associate writer find out with this week news quiz editorial cartoon for july world share are mostly down a trump tariff deadline loom while u stock set record trump pitch plan allowing farmer to vouch for illegal immigrant worker facing deportation blaze engulfs four home in la amid active firework a strike by air traffic controller is disrupting travel to from and over france trump ag secretary ha irony meter exploding left right and center with beyond parody spin trump decision to end taxfree loophole for lowvalue good from china lead to a sharp decline in air cargo shipment cyber school facing wrongful death suit say it unreasonable for teacher to see student weekly opinion blockbuster made me do it questionable advice from big summer movie pa republican gamble on rural health care a megabill push through cumberland county official optimistic that new memo will improve coordination with library system galasso look forward to tomorrow expectantly beyond current circumstance joey chestnut return to coney island expected to dominate hot dog eating contest trump proposes ufc fight at white house to celebrate year of independence will new england sky stay clear for friday night big firework show u colombia announce recall of envoy amid diplomatic rift lucas trump should demand the unconditional surrender of the democrat party food hygiene rating handed to four doncaster establishment one need major improvement elephant kill two female tourist from the uk and new zealand in zambian national park many missouri law restricting abortion blocked again by state judge iredell county name rodney harris a the new deputy county manager iran try keeping new military commander a secret mossad offer guessing game confirms winner atlanta clogged road bring out the rage in motorist opinion challenge opportunity and bright future in ct for dairy farming trump tear into marxist lunatic mamdani honor american hero in bold rebuke play these p plus free game in july xrp hold market confidence while lightchain ai latejuly launch prepares to broaden investor option rosen nationally regarded investor counsel encourages reckitt benckiser group plc investor to secure counsel before important deadline in security class action rbgly robinhood want to redo wall street on the blockchain gizmodo why tempus ai stock soared in june japan brace for more quake authority dismiss doomsday hype opec plus agrees to pump more oil in august the new york time trump reportedly told iran it wa ok to strike back after u attack i said go ahead i understand poland blast trumpputin dialogue after drone strike escalation walmart is selling calvin klein eternity perfume for only and shopper say it an unbeatable deal ap business summarybrief at pm edt ap business summarybrief at pm edt ap business summarybrief at pm edt ap business summarybrief at pm edt the newest stock in the sp ha soared since it ipo and it a buy right now according to wall street the newest stock in the sp ha soared since it ipo and it a buy right now according to wall street were watching a brain drain in real time openai hit hard a top researcher defect to rival tech giant meta rude baguette the best amazon prime day deal under save on gear from blink anker samsung and others engadget nextgen ai and social startup backed by thrive capital and y combinator shaping were on the brink of another big consumer wave click like sugar gambling in a world of quick pleasure an addiction expert say it might be time for a dopamine fast a amazon double down on robotaxis is amzn stock a buy charlize theron is choosing to be single she told call her daddy that can be a sign of strength say relationship expert the future of ai selfdriving car mechanical weeding health care assistant and more patriotic parade at the park the market hidden current delivering fast gain top romantic drama on ott to watch this weekend daily habit that separate high achiever from everyone else best altcoins for next bull run blockdags m summer raffle roi feature alongside inj rndr tia a forgotten megatrend that could be key to the ai economy quality nonus stock to buy in simply staggering cnn correspondent describes floodwater impact in texas good stock still worth buying in this market matt mower after nato summit europe free ride is on the line archer aviation the bet that could take off sooner than you think oneofakind brewery taproom closing no bankruptcy oneofakind brewery taproom closing no bankruptcy trump hit with backlash over use of antisemitic slur at iowa rally stage almost over arctic pablos price hike imminent a myro and housecoin push forward shopper race to get off all item in major closing down sale after iconic activewear brand shuts store investor deadline robbins geller rudman dowd llp announces that sarepta therapeutic inc srpt investor with substantial loss have opportunity to lead class action lawsuit one big beautiful budget deficit opec to increase output by barrel a day in august what it mean for oil market btc miner cloud mining platform strives to offer stability security a bitcoin recently crossed k amazon prime day the best deal live right now plus everything else you need to know engadget an iowa law rolling back trans civil right protection in the state ha taken effect here what to know thinkcarebelieve week of america victory walmart is selling a sleek digital camera for and shopper say it look professional subaru launch killer legacy lease offer for july top short anime to watch this weekend odd taxi death parade more safeway strike end a albertsons and local union reach agreement colorado public radio headed for sentencing sean diddy comb lawyer aim to show he no longer a bad boy for life the average american family is a millionaire how you can join them your kid is getting a</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>tribe property technology announces closing of best effort public offering of unit with full exercise of overallotment option for gross proceeds of approximately will recent event dent palantir technology stock growth sinopec launch new floating solar project with green hydrogen in play storen leading the future of home energy storage scottscott attorney at law llp file security class action against reckitt benckiser group plc otc rbgly chime financial first internetnative juggernaut focused on consumer banking say bullish analyst stock making big midday move tesla uber royal gold stellantis wns and more jeldwen expands cradle to cradle certification expanding portfolio of certified sustainable door energy demand optimism and houthi rebel attack on red sea shipping boost crude price nombase powered by bevnet launch new data hub a centralized resource for food beverage beer industry report iceland seafood international hf refinancing completed big beautiful bill may help some senior on social security but it doesnt eliminate tax on benefit noridian renews commitment to continuous improvement with the promotion of jeremiah mckay nvidias ai chip rival groq launch first european data center top ai growth stock to buy in july amazon prime day is here what it mean for the stock barrons fella it time to spice up your life with the help of lynks sexual wellness collection oneoncology appoints dr michael byrne a medical director for cellular therapy investing veteran see market pricing maseratis like ford tune in at noon workplace have embraced mindfulness and selfcompassionbut did capitalism hijack their true purpose google want to hit net zero by so it signed a massive deal with a bill gatesbacked startup thats still year away from making energy could amd and nvidia face new ai chip export restriction petco health and wellness company inc nasdaq woof shareholder alert bernstein liebhard llp reminds petco health and wellness company inc investor of upcoming deadline dhls german postal unit aim to increase use of parcel locker noridian renews commitment to continuous improvement with the promotion of jeremiah mckay rubis halfyear statement on rubis liquidity agreement with exane bnp paribas gtt monthly disclosure of the total number of voting right and share composing the share capital top trending meme coin breaking the internet arctic pablo freeze out the competition a fartboy and mubarak coin rise noridian renews commitment to continuous improvement with the promotion of jeremiah mckay kpn report on progress of m share buyback gtt halfyear liquidity contract statement asm share buyback update june july fnac darty disclosure of trading in own share june to july in french only this solanafocused etf by rexosprey offer a new way to earn from crypto wmo weather forecast for come true year early sarepta therapeutic inc nasdaq srpt shareholder alert bernstein liebhard llp reminds sarepta therapeutic inc investor of upcoming deadline thread is nearing x daily app user new data show techcrunch brazil to return to global bond market this year treasury secretary say planned parenthood sue trump administration over planned defunding gold price retreat to oneweek low on u tariff delay microstrategy paused it bitcoinbuying spree last week california bill seek to rein in debt settlement company that target mcas business loan borrower ageas report on the progress of share buyback programme luxury housing market no longer out of reach for some moveup buyer report homebuyers given new way to pay for a house after gamechanging policy switch and it not with cash up in a month should you buy plug power stock here yearold ran a one direction fan account a a teennow she run a medium brand with m follower including lorde and bella hadid i love my job rarely offered donut selling for off at krispy kreme on world chocolate day what will happen to the housing market during a baby dust taste radio one of the best trade show weve ever attended fancy that strait of hormuz in the spotlight forvia total number of voting right and share forming the share capital rite aid in ashland closing this summer gray and scripps to swap station and create more duopolies were booking profit in a topperforming bank stock in an extremely overbought market can trump run it hot plan trap the fed and jolt the bond market u child are much more likely to die than kid in similar country study find here how much invested in rtx year ago would be worth today best credit card for amazon of why everyones wrong about xrps real value a spacepay aim to become a top crypto payment solution weekly report share buyback from june to july weekly report share buyback from june to july historic yes could be better how to access perplexity ai free version fake image detection market is poised to expand beyond u million by say astute analytica uk fund invests million in carbon capture project hipgnosis founder talk new venture eye buying back catalog from blackstone the best amazon prime day deal under save on gear from samsung blink anker and others engadget lululemon v dupe texas flood live update death roll rise to a nw warns of more flooding trump say he will begin announcing trade deal and tariff rate at noon sinclair name narinder sahai evp and cfo sonar enhances oracle otm integration and launch shipper consortium for unmatched supply chain benchmarking palantir stock go warp speed but there a caveat walmart sam club and the walmart foundation commit up to to support texas flood relief effort explaining assessing the digital service tax dilemma gunman ambush border patrol agent in texas amid antiice rhetoric from democrat unmanned saildrones track russian shadow fleet during nato baltic sea operation jeldwen expands cradle to cradle certification expanding portfolio of certified sustainable door chase sapphire reserve lounge access in whats actually included tesla stock price fall after elon musk plan new political party micron meteoric rise can mu stock hit in ai is the new oil and america is laying the pipeline dow industrials intraday decline now exceeds point live update which worker will ai hurt most the young or the experienced the new york time will ai replace new hire or middle manager your job interviewer is not a person it ai catch up on your reading list this prime day with up to off kindles tesla trouble amplified by musk party politics etf on edge yemen houthi rebel say bulk carrier magic sea that they attacked sunday ha sunk starbucks launch new frappuccino kusacom hims hers navigates novo nordisk breakup and compounding lawsuit italy shipbuilder appoints new u chief trump administration move to terminate a form of humanitarian relief for nicaraguan and honduran in the u global wet chemical in semiconductor market forecast usd b by driven by advanced node manufacturing valuates report st elizabeth hospital and flight for life celebrate one year in fort morgan almonty industry applies for nasdaq listing elon musk realized too late how badly tesla will hurt from trump bill electrek ascendion win gold a the artificial intelligence service provider of the year in globee award borr drilling announces first settlement of the offering of common share brcevichelivjpg trump and netanyahu may take a victory lap on iran but the gaza war loom over their meeting alaskan lng the future of natural gas brcevichelivjpg brcevichelivjpg brcevichelivjpg brcevichelivjpg opinion reclaiming my time what in the hell happened bannon blast doj over epstein announcement daily beast try to use texas tragedy to attack ted cruz man killed after shooting at a u border patrol facility in southern texas u will make several trade announcement in next hour bessent hakeem jeffries roasted for obviously photoshopped instagram post a man ha been killed after opening fire at a u border patrol facility in texas authority say musk say he forming a new political party after split with trump over tax cut law strait of hormuz in the spotlight first look swapping beer for pisco sour see dive bar new life a madisonville restaurant society of st vincent de paul usa president john berry say work to protect the poor must go on after reconciliation bill passage liberal critic question why architect of failed biden foreign policy is advising project man killed after shooting at a u border patrol facility in southern texas american kid have become increasingly unhealthy over nearly two decade new study find patricia lopez ice doesnt need another billion surprise dems medium lie blame trump for storm death ken morris you may not be a diversified a you think rep carlos barron elected a state house minority whip tiktok user try to make texas flood all about race u child are much more likely to die than kid in similar country study find carnival cruise update rule critic cry racism trump threatens not to chicken out yet again over tariff democrat trying to field candidate slate to win first statewide race in year dccc target house republican over budget law impact on rural hospital dem lawmaker say their voter are threatening blood and violence over inability to hinder trump report dhs terminates temporary protected status for around k honduran nicaraguan migrant top maga voice stunned by trump administration debunking epstein theory jesse jackson jr explores a house comeback bid california expands automatic renewal law new requirement now in effect louisiana state police arrest woman in connection with motorcycle death of shreveport man gang burn down famous haitian hotel trump administration move to terminate a form of humanitarian relief for nicaraguan and honduran in the u leave bolsonaro alone trump furious a brazil exleader face coup trial mainer need to do what democracy demand letter maga influencers scream coverup following release of doj memo closing the book on jeffrey epstein case editorial chicago mourns with texas and the parent of the camp mystic girl schumer demand investigation of trump weather service vacancy in wake of texas flooding schumer demand investigation of trump weather service vacancy in wake of texas flooding schumer demand investigation of trump weather service vacancy in wake of texas flooding yemen houthi rebel say bulk carrier magic sea that they attacked sunday ha sunk schumer demand investigation of trump weather service vacancy in wake of texas flooding schumer demand investigation of trump weather service vacancy in wake of texas flooding schumer demand investigation of trump weather service vacancy in wake of texas flooding holy cross cattleman asks for permit to kill copper creek wolf u to revoke protected status for immigrant from honduras and nicaragua u chamber of commerce discusses how tariff will raise the cost of summer fun with yourupdatetv u cancel contract save million in day doge former librarian of congress fired by trump vow to improve public information in new mellon role former librarian of congress fired by trump vow to improve public information in new mellon role trump say he will visit texas probably on friday to tour flash flood damage mcafees summer shopping study reveals it prime time for smart shopping team technology an arlington capital partner portfolio company expands medical device manufacturing capability with acquisition of duke empirical inc trump th week in office set to include visit to texas devastated hill country third netanyahu meeting i dont use credit card point to shop for prime day here what i do instead this senator just sold up to k in unitedhealth group stock recent filing show that rep john rose sold over m worth of alphabet stock u lobby group urge tariff retaliation against australia socialised medicine face the nation stoltenberg panel wear it or resist anne hanson time to reboot lucy k wyman peacham th of july dave edward michael paul williams maga turn back the clock at uva proposed radio tower cynthia krieble abm announces new board of director and executive committee member threat to freedom of religion denise fontaine court release cctv footage shown during mushroom murder trial maine ban floating camp another big week for nepa new federal procedure and a big beautiful bill benefit the mindful minute by jon heydenreich my menu correction osisko development announces positive bulk tonnage ore sorting result for the project worldwide bolster indiasouth asia leadership with strategic appointment educator view throw a book at your kid to avoid summer slide jeffery epstein died by suicide and there no client list justice department say houston official fired over raciallytinged tiktok rant about search for missing girl man with rifle and tactical gear killed after exchange of fire with border patrol in texas prominent west bank sheikh face violent threat after proposing peace with israel zelenskyy spoke with trump on replacing kyivs envoy to u israel and hamas are inching toward a new ceasefire deal for gaza this is how it might look chrome day ivanti exploit macos stealer crypto heist and more russia exminister found dead hour after being fired in an apparent suicide official said don davis eye open north carolina senate seat white house asks american to pray after deadly texas flooding planned parenthood challenge gop reconciliation law north carolina also hit with lifethreatening flash flood governor murphy mansion tax modification breaking leo source report active shooter with rifle and tactical gear ambushed border patrol agent french gameshow contestant epic month winning streak finally end a reignited trumpmusk feud burn tesla investor share of ev company tumble a reignited trumpmusk feud burn tesla investor share of ev company tumble p miner launch the world first xrp liquid mining aidriven multiasset putting up the closed sign trump policy have cost vital u business b see what first responder are facing in texas a they search for victim airwavz solution appoints monte dube to market advisory board to strengthen healthcare wireless strategy hidden megabill clause hand taxpayer bill for huge gift to private jet owner church street closed for new sewer line trump administration revoke terrorism designation of new syrian leader group mayor adam hears community concern on housing ebikes education at bayside town hall flatbread barbecue and more best thing we ate this week in baton rouge and acadiana faimon robert how this la rural sheriff is remaking his office and redefining progressive the battle over the big beautiful bill move from capitol hill to the campaign trail global trade is back in limbo revealed white house email show desperate rush to punish university</t>
+          <t>tribe property technology announces closing of best effort public offering of unit with full exercise of overallotment option for gross proceeds of approximately will recent event dent palantir technology stock growth sinopec launch new floating solar project with green hydrogen in play storen leading the future of home energy storage scottscott attorney at law llp file security class action against reckitt benckiser group plc otc rbgly chime financial first internetnative juggernaut focused on consumer banking say bullish analyst stock making big midday move tesla uber royal gold stellantis wns and more jeldwen expands cradle to cradle certification expanding portfolio of certified sustainable door energy demand optimism and houthi rebel attack on red sea shipping boost crude price nombase powered by bevnet launch new data hub a centralized resource for food beverage beer industry report iceland seafood international hf refinancing completed big beautiful bill may help some senior on social security but it doesnt eliminate tax on benefit noridian renews commitment to continuous improvement with the promotion of jeremiah mckay nvidias ai chip rival groq launch first european data center top ai growth stock to buy in july amazon prime day is here what it mean for the stock barrons fella it time to spice up your life with the help of lynks sexual wellness collection oneoncology appoints dr michael byrne a medical director for cellular therapy investing veteran see market pricing maseratis like ford tune in at noon workplace have embraced mindfulness and selfcompassionbut did capitalism hijack their true purpose google want to hit net zero by so it signed a massive deal with a bill gatesbacked startup thats still year away from making energy could amd and nvidia face new ai chip export restriction petco health and wellness company inc nasdaq woof shareholder alert bernstein liebhard llp reminds petco health and wellness company inc investor of upcoming deadline dhls german postal unit aim to increase use of parcel locker noridian renews commitment to continuous improvement with the promotion of jeremiah mckay rubis halfyear statement on rubis liquidity agreement with exane bnp paribas gtt monthly disclosure of the total number of voting right and share composing the share capital top trending meme coin breaking the internet arctic pablo freeze out the competition a fartboy and mubarak coin rise noridian renews commitment to continuous improvement with the promotion of jeremiah mckay kpn report on progress of m share buyback gtt halfyear liquidity contract statement asm share buyback update june july fnac darty disclosure of trading in own share june to july in french only this solanafocused etf by rexosprey offer a new way to earn from crypto wmo weather forecast for come true year early sarepta therapeutic inc nasdaq srpt shareholder alert bernstein liebhard llp reminds sarepta therapeutic inc investor of upcoming deadline thread is nearing x daily app user new data show techcrunch brazil to return to global bond market this year treasury secretary say planned parenthood sue trump administration over planned defunding gold price retreat to oneweek low on u tariff delay microstrategy paused it bitcoinbuying spree last week california bill seek to rein in debt settlement company that target mcas business loan borrower ageas report on the progress of share buyback programme luxury housing market no longer out of reach for some moveup buyer report homebuyers given new way to pay for a house after gamechanging policy switch and it not with cash up in a month should you buy plug power stock here yearold ran a one direction fan account a a teennow she run a medium brand with m follower including lorde and bella hadid i love my job rarely offered donut selling for off at krispy kreme on world chocolate day what will happen to the housing market during a baby dust taste radio one of the best trade show weve ever attended fancy that strait of hormuz in the spotlight forvia total number of voting right and share forming the share capital rite aid in ashland closing this summer gray and scripps to swap station and create more duopolies were booking profit in a topperforming bank stock in an extremely overbought market can trump run it hot plan trap the fed and jolt the bond market u child are much more likely to die than kid in similar country study find here how much invested in rtx year ago would be worth today best credit card for amazon of why everyones wrong about xrps real value a spacepay aim to become a top crypto payment solution weekly report share buyback from june to july weekly report share buyback from june to july historic yes could be better how to access perplexity ai free version fake image detection market is poised to expand beyond u million by say astute analytica uk fund invests million in carbon capture project hipgnosis founder talk new venture eye buying back catalog from blackstone the best amazon prime day deal under save on gear from samsung blink anker and others engadget lululemon v dupe texas flood live update death roll rise to a nw warns of more flooding trump say he will begin announcing trade deal and tariff rate at noon sinclair name narinder sahai evp and cfo sonar enhances oracle otm integration and launch shipper consortium for unmatched supply chain benchmarking palantir stock go warp speed but there a caveat walmart sam club and the walmart foundation commit up to to support texas flood relief effort explaining assessing the digital service tax dilemma gunman ambush border patrol agent in texas amid antiice rhetoric from democrat unmanned saildrones track russian shadow fleet during nato baltic sea operation jeldwen expands cradle to cradle certification expanding portfolio of certified sustainable door chase sapphire reserve lounge access in whats actually included tesla stock price fall after elon musk plan new political party micron meteoric rise can mu stock hit in ai is the new oil and america is laying the pipeline dow industrials intraday decline now exceeds point live update which worker will ai hurt most the young or the experienced the new york time will ai replace new hire or middle manager your job interviewer is not a person it ai catch up on your reading list this prime day with up to off kindles tesla trouble amplified by musk party politics etf on edge yemen houthi rebel say bulk carrier magic sea that they attacked sunday ha sunk starbucks launch new frappuccino kusacom hims hers navigates novo nordisk breakup and compounding lawsuit italy shipbuilder appoints new u chief trump administration move to terminate a form of humanitarian relief for nicaraguan and honduran in the u global wet chemical in semiconductor market forecast usd b by driven by advanced node manufacturing valuates report st elizabeth hospital and flight for life celebrate one year in fort morgan almonty industry applies for nasdaq listing elon musk realized too late how badly tesla will hurt from trump bill electrek ascendion win gold a the artificial intelligence service provider of the year in globee award borr drilling announces first settlement of the offering of common share brcevichelivjpg trump and netanyahu may take a victory lap on iran but the gaza war loom over their meeting alaskan lng the future of natural gas brcevichelivjpg brcevichelivjpg brcevichelivjpg brcevichelivjpg opinion reclaiming my time what in the hell happened bannon blast doj over epstein announcement daily beast try to use texas tragedy to attack ted cruz man killed after shooting at a u border patrol facility in southern texas u will make several trade announcement in next hour bessent hakeem jeffries roasted for obviously photoshopped instagram post a man ha been killed after opening fire at a u border patrol facility in texas authority say musk say he forming a new political party after split with trump over tax cut law strait of hormuz in the spotlight first look swapping beer for pisco sour see dive bar new life a madisonville restaurant society of st vincent de paul usa president john berry say work to protect the poor must go on after reconciliation bill passage liberal critic question why architect of failed biden foreign policy is advising project man killed after shooting at a u border patrol facility in southern texas american kid have become increasingly unhealthy over nearly two decade new study find patricia lopez ice doesnt need another billion surprise dems medium lie blame trump for storm death ken morris you may not be a diversified a you think rep carlos barron elected a state house minority whip tiktok user try to make texas flood all about race u child are much more likely to die than kid in similar country study find carnival cruise update rule critic cry racism trump threatens not to chicken out yet again over tariff democrat trying to field candidate slate to win first statewide race in year dccc target house republican over budget law impact on rural hospital dem lawmaker say their voter are threatening blood and violence over inability to hinder trump report dhs terminates temporary protected status for around k honduran nicaraguan migrant top maga voice stunned by trump administration debunking epstein theory jesse jackson jr explores a house comeback bid california expands automatic renewal law new requirement now in effect louisiana state police arrest woman in connection with motorcycle death of shreveport man gang burn down famous haitian hotel trump administration move to terminate a form of humanitarian relief for nicaraguan and honduran in the u leave bolsonaro alone trump furious a brazil exleader face coup trial mainer need to do what democracy demand letter maga influencers scream coverup following release of doj memo closing the book on jeffrey epstein case editorial chicago mourns with texas and the parent of the camp mystic girl schumer demand investigation of trump weather service vacancy in wake of texas flooding schumer demand investigation of trump weather service vacancy in wake of texas flooding schumer demand investigation of trump weather service vacancy in wake of texas flooding yemen houthi rebel say bulk carrier magic sea that they attacked sunday ha sunk schumer demand investigation of trump weather service vacancy in wake of texas flooding schumer demand investigation of trump weather service vacancy in wake of texas flooding schumer demand investigation of trump weather service vacancy in wake of texas flooding holy cross cattleman asks for permit to kill copper creek wolf u to revoke protected status for immigrant from honduras and nicaragua u chamber of commerce discus how tariff will raise the cost of summer fun with yourupdatetv u cancel contract save million in day doge former librarian of congress fired by trump vow to improve public information in new mellon role former librarian of congress fired by trump vow to improve public information in new mellon role trump say he will visit texas probably on friday to tour flash flood damage mcafees summer shopping study reveals it prime time for smart shopping team technology an arlington capital partner portfolio company expands medical device manufacturing capability with acquisition of duke empirical inc trump th week in office set to include visit to texas devastated hill country third netanyahu meeting i dont use credit card point to shop for prime day here what i do instead this senator just sold up to k in unitedhealth group stock recent filing show that rep john rose sold over m worth of alphabet stock u lobby group urge tariff retaliation against australia socialised medicine face the nation stoltenberg panel wear it or resist anne hanson time to reboot lucy k wyman peacham th of july dave edward michael paul williams maga turn back the clock at uva proposed radio tower cynthia krieble abm announces new board of director and executive committee member threat to freedom of religion denise fontaine court release cctv footage shown during mushroom murder trial maine ban floating camp another big week for nepa new federal procedure and a big beautiful bill benefit the mindful minute by jon heydenreich my menu correction osisko development announces positive bulk tonnage ore sorting result for the project worldwide bolster indiasouth asia leadership with strategic appointment educator view throw a book at your kid to avoid summer slide jeffery epstein died by suicide and there no client list justice department say houston official fired over raciallytinged tiktok rant about search for missing girl man with rifle and tactical gear killed after exchange of fire with border patrol in texas prominent west bank sheikh face violent threat after proposing peace with israel zelenskyy spoke with trump on replacing kyivs envoy to u israel and hamas are inching toward a new ceasefire deal for gaza this is how it might look chrome day ivanti exploit macos stealer crypto heist and more russia exminister found dead hour after being fired in an apparent suicide official said don davis eye open north carolina senate seat white house asks american to pray after deadly texas flooding planned parenthood challenge gop reconciliation law north carolina also hit with lifethreatening flash flood governor murphy mansion tax modification breaking leo source report active shooter with rifle and tactical gear ambushed border patrol agent french gameshow contestant epic month winning streak finally end a reignited trumpmusk feud burn tesla investor share of ev company tumble a reignited trumpmusk feud burn tesla investor share of ev company tumble p miner launch the world first xrp liquid mining aidriven multiasset putting up the closed sign trump policy have cost vital u business b see what first responder are facing in texas a they search for victim airwavz solution appoints monte dube to market advisory board to strengthen healthcare wireless strategy hidden megabill clause hand taxpayer bill for huge gift to private jet owner church street closed for new sewer line trump administration revoke terrorism designation of new syrian leader group mayor adam hears community concern on housing ebikes education at bayside town hall flatbread barbecue and more best thing we ate this week in baton rouge and acadiana faimon robert how this la rural sheriff is remaking his office and redefining progressive the battle over the big beautiful bill move from capitol hill to the campaign trail global trade is back in limbo revealed white house email show desperate rush to punish university</t>
         </is>
       </c>
     </row>
@@ -810,7 +810,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>what you need to know ahead of arch capital earnings release what really killed the mill reason to buy ethereum before what to expect from leidos holding q earnings report successful couple do these thing in the morning that little hello go a long way relationship expert say in a world of bull and bear be the tiger s ai launch agentic capability in latest molecular universe release to increase value proposition for rd a a service we found the best amazon prime day deal after shopping thousand of offer cnn most fed official see rate cut coming but opinion vary widely on how many minute show fury intercept m of lio at the ninaaskumuwin discovery incorporation of boerne in lawmaker will investigate response to flood covered call screener result for july th texas just passed quantum computing legislation how should you play ionq stock here homebuyers finally responded after mortgage rate hit lowest level in three month cnbc palantir technology ha been the sp s hottest stock over the past year and it not even close can it incredible rally continue cybersecurity stock you can buy and hold for the next decade business newsline july amazon extends prime day discount to day trump medium file for crypto blue chip etf vibe coding ha arrived for business wsj this bigname adviser say avoiding crypto is now a more speculative investment move than buying it marketwatch trump threatened to bomb the s out of moscow to deter putin cnn trump big beautiful bill promise no tax on tip and overtime but there a limitheres who qualifies droit launch explore mode on it adept platform h room for optimism risk for complacency aes freeportmcmoran verona pharma intel aehr penguin solution and more mover barrons michelle obama i learned this great parenting tip from my mom and dadthey did a beautiful job modeling it bmw v mercedes u sale race there a clear leader in linda yaccarino step down a ceo of elon musk x dax push higher a eu edge closer to tariff deal with u the prime day deal you can still get the verge eli manning say he no longer interested in buying a piece of the nfls giant it too expensive for me merck to acquire verona pharma expanding it portfolio to include ohtuvayre ensifentrine a firstinclass copd maintenance treatment for adult and expected to drive growth into the next decade merck to acquire verona pharma expanding it portfolio to include ohtuvayre ensifentrine a firstinclass copd maintenance treatment for adult and expected to drive growth into the next decade merckcom walmart is selling a fantastic chromebook laptop for just and shopper love the touchscreen feature these word help teach kid critical thinking say michelle obama and psychologist malaysian pm warns southeast asia that trade war is not a passing storm quadmotor rivians arrive with wild power and wilder price apple can it catch up in the ai race a rival turn up the heat boomer are buying the highestyielding dividend champion handoverfist a o smith corporation nyseaos share purchased by private trust co na elon musk grok ai chatbot denies that it praised hitler and made antisemitic comment daily vickers top insider pick for hudson edge investment partner inc ha million stock position in jpmorgan chase co nysejpm private trust co na ha stock holding in coterra energy inc nysectra rosalia is new balance newest brand ambassador russia launch another record drone attack on ukraine ukrainian official say beware of scam that promise good pay for completing easy online task beware of scam that promise good pay for completing easy online task today top money market account rate for july rate hit current heloc home equity loan rate july highyield saving account rate today july rate are steady beware of scam that promise good pay for completing easy online task ap news bank of england flag global debt pressure despite market stabilization goldman demand an oath from junior banker to fend off private equity poaching bloomberg court block rule that would let you cancel subscription easily sp future tick higher a investor shrug off trump tariff threat fomc minute on tap today mortgage refinance rate july rate increase mortgage rate today july rate move up cd rate today july rate rise uae say the oil market is thirsty for more opec barrel proposed clermont subdivision would redesign deadly lakeshore drive exact science announces medicare coverage for oncodetecttm molecular residual disease test in colorectal cancer fresh del monte produce inc to report second quarter financial result trump trade blitz produce few deal but lot of uncertainty trump trade blitz produce few deal but lot of uncertainty trump trade blitz produce few deal but lot of uncertainty trump trade blitz produce few deal but lot of uncertainty trump trade blitz produce few deal but lot of uncertainty trump trade blitz produce few deal but lot of uncertainty a new era of restaurant worker may earn sixfigure salary and benefit that no other industry can provide tesla board need ground rule for musk political activism analyst say samsung launch three new foldable smartphones a it fends off chinese rival trump tariff extension leaf bank fed in limbo hbo max is back prestige brand return to streaming corra group see rising demand from global investor for due diligence investigation market sputter after trump push tariff deadline xrp price forecast hit but insider are loading up on the new xrp that could go x auddia announces leadership change and special committee to evaluate business combination and restructuring a ai native holding company senate gop gear up for test on trump doge cut inside information orion upgrade fullyear outlook for social security sends million of american a misleading and blatantly political message see this shreveport director awardwinning screenplay red carpet premiere here how first atlantic nickel expands rpm zone awaruite nickelalloy nife discovery meter northern extension yield nickel concentrate over meter in dtr metallurgical recovery testing shreveport to kick off return of eleven store to louisiana more site planned two ragnarok ip title achieved top game ranking in taiwan hong kong and macau toast inc nysetost share acquired by da davidson co private trust co na ha stock holding in ge healthcare technology inc nasdaqgehc trump big beautiful bill slash cfpb funding what it mean for you davenport co llc sell share of fortive corporation nyseftv private trust co na acquires share of emcor group inc nyseeme you have less than month to claim the ev tax credit now is the time to buy say car expert this legend cross time zone with just pound of gear here are his favorite principal financial group inc increase stock position in zimmer biomet holding inc nysezbh mutual advisor llc buy share of trane technology plc nysett mutual advisor llc grows stock holding in decker outdoor corporation nysedeck first malaria drug for newborn and young infant expected to be approved in africa within week former rapid city anchor given suspended sentence in domestic assault case bank of england warns of high financial market risk despite easing tension kisti secures funding for national quantum center of excellence name ionq a primary quantum partner our opinion when the president punishes patriot wednesday letter a the world burn eye turn to diddy european court russia wa behind downing of mh watch popular podcaster discusses how kamala episode wa scrapped because she talked gibberish her own campaign wanted it canned fbi bust chinese national for multimillion dollar drug ring exploiting immigration system the president mean business trump admin sue california over transgender athlete policy other view state congressional delegation must fight cut to noaa burke county company say hildebran wont issue permit for train cabin business another voice buffalo garden vibrantly express a community soul trump admin subpoena harvard over foreign student misconduct campus radicalism george conway flag trump awkward new admission a fresh proof he a fool eu seek to finalize trade deal with trump by end of the month hawaii lawmaker demand immigration arrest briefing haleiwa development under council review state road usage charge begin for electric vehicle on july governor state budget veto trim public school maintenance hooser sbcd a travesty of process and policy senate gop gear up for test on trump doge cut senate gop gear up for test on trump doge cut jewish democrat in congress sound the alarm on mamdani tea party patriot to push lawmaker on noncitizen voting jewish democrat in congress sound the alarm on mamdani tea party patriot to push lawmaker on noncitizen voting senate gop gear up for test on trump doge cut larger fight rage on but trump racking up win against college tea party patriot to push lawmaker on noncitizen voting jewish democrat in congress sound the alarm on mamdani larger fight rage on but trump racking up win against college larger fight rage on but trump racking up win against college senate gop gear up for test on trump doge cut senate gop gear up for test on trump doge cut tea party patriot to push lawmaker on noncitizen voting jewish democrat in congress sound the alarm on mamdani tea party patriot to push lawmaker on noncitizen voting jewish democrat in congress sound the alarm on mamdani senate gop gear up for test on trump doge cut larger fight rage on but trump racking up win against college tea party patriot to push lawmaker on noncitizen voting larger fight rage on but trump racking up win against college jewish democrat in congress sound the alarm on mamdani larger fight rage on but trump racking up win against college candace cameron bure say son biblebased pep talk helped save her marriage antiviolence advocate why not hold gun manufacturer accountable for mass shooting like river north tragedy letter chicago allows people to be who they want to be trump trade blitz produce few deal but lot of uncertainty laura washington the art institute is slowly getting back to normal georgia police arrest farmworkers then get warrant from dhs firearm testing and ballistics unit could be open in september at county forensics lab former dc fire official want to cut tax increase police presence with city council bid my view trekking pole can lend some mountainclimber swagger steve corbin give me liberty or a tinpot dictator scare buying reported in rochester why should legislator favor legal pot business california focus why should legislator favor legal pot business california focus editorial cartoon for july this legend cross time zone with just pound of gear here are his favorite which u president had wife named ellen and edith first malaria drug for newborn and young infant expected to be approved in africa within week red bull team principal christian horner fired after year with team after month stuck in the south north korean go home letter billion not served by trump big bill letter billion not served by trump big bill supreme court reject shielding identity of police attending jan capitol rally trump slam democrat over inflation narrative say he cut cost more than any president in history red bull team principal christan horner sacked after year with team letter no one is voting after result are known letter no one is voting after result are known here everything to expect at this family fun day in colnes alkincoates park robinhood ceo tokenization is a major innovation in capital market here who will and wont qualify for the new car loan interest deduction allegheny county council approves innamorato choice for shuman advisory board pittsburgh city council pass further protection for lgbtq people elon musk grok remove politically incorrect instruction after it praise hitler wa the flash flooding in texas preventable trump say tariff on pharmaceutical import could increase to percent threetime mvp nikola jokic will delay signing extension with nugget this summer ap source say trump boast about threat to bomb the st out of moscow in leaked audio charles warns small boat crisis is a profound challenge a he host macron at state banquet ahead of migrant deal newsom go big on holy grail reform other view newsom go big on holy grail reform other view supreme court allows trump administration to resume mass federal layoff for now suit challenge government effort to deport supporter of propalestinian protest invest america act give to every u newborn investment account dell ceo call it futureproofing prosperity sam altman asks for more stuff like this reader speak why i say thank you to uconn health center off the rail trump ramble in the middle of cabinet meeting is karat nonsense wall street trump taco trade ha a chicken and an egg problem meet the new national police force mamdanis farleft ally want to primary hakeem jeffries and other nyc democrat reader speak american tragedy is that those who are in power are inhumane congressional democrat push for new watchdog to oversee trump white house american need to work together to fix education weve both done it before on opposite side the search for the old lady pony continues tariff are already squeezing corporate margin new survey find ai is changing the world faster than most realize fencing wa a chore that we enjoyed texas is relying on fema state leader said it should be cut letter trump usaid action are evil letter trump usaid action are evil microsoft patch vulnerability including critical flaw in spnego and sql server</t>
+          <t>what you need to know ahead of arch capital earnings release what really killed the mill reason to buy ethereum before what to expect from leidos holding q earnings report successful couple do these thing in the morning that little hello go a long way relationship expert say in a world of bull and bear be the tiger s ai launch agentic capability in latest molecular universe release to increase value proposition for rd a a service we found the best amazon prime day deal after shopping thousand of offer cnn most fed official see rate cut coming but opinion vary widely on how many minute show fury intercept m of lio at the ninaaskumuwin discovery incorporation of boerne in lawmaker will investigate response to flood covered call screener result for july th texas just passed quantum computing legislation how should you play ionq stock here homebuyers finally responded after mortgage rate hit lowest level in three month cnbc palantir technology ha been the sp s hottest stock over the past year and it not even close can it incredible rally continue cybersecurity stock you can buy and hold for the next decade business newsline july amazon extends prime day discount to day trump medium file for crypto blue chip etf vibe coding ha arrived for business wsj this bigname adviser say avoiding crypto is now a more speculative investment move than buying it marketwatch trump threatened to bomb the s out of moscow to deter putin cnn trump big beautiful bill promise no tax on tip and overtime but there a limitheres who qualifies droit launch explore mode on it adept platform h room for optimism risk for complacency aes freeportmcmoran verona pharma intel aehr penguin solution and more mover barrons michelle obama i learned this great parenting tip from my mom and dadthey did a beautiful job modeling it bmw v mercedes u sale race there a clear leader in linda yaccarino step down a ceo of elon musk x dax push higher a eu edge closer to tariff deal with u the prime day deal you can still get the verge eli manning say he no longer interested in buying a piece of the nfls giant it too expensive for me merck to acquire verona pharma expanding it portfolio to include ohtuvayre ensifentrine a firstinclass copd maintenance treatment for adult and expected to drive growth into the next decade merck to acquire verona pharma expanding it portfolio to include ohtuvayre ensifentrine a firstinclass copd maintenance treatment for adult and expected to drive growth into the next decade merckcom walmart is selling a fantastic chromebook laptop for just and shopper love the touchscreen feature these word help teach kid critical thinking say michelle obama and psychologist malaysian pm warns southeast asia that trade war is not a passing storm quadmotor rivians arrive with wild power and wilder price apple can it catch up in the ai race a rival turn up the heat boomer are buying the highestyielding dividend champion handoverfist a o smith corporation nyseaos share purchased by private trust co na elon musk grok ai chatbot denies that it praised hitler and made antisemitic comment daily vickers top insider pick for hudson edge investment partner inc ha million stock position in jpmorgan chase co nysejpm private trust co na ha stock holding in coterra energy inc nysectra rosalia is new balance newest brand ambassador russia launch another record drone attack on ukraine ukrainian official say beware of scam that promise good pay for completing easy online task beware of scam that promise good pay for completing easy online task today top money market account rate for july rate hit current heloc home equity loan rate july highyield saving account rate today july rate are steady beware of scam that promise good pay for completing easy online task ap news bank of england flag global debt pressure despite market stabilization goldman demand an oath from junior banker to fend off private equity poaching bloomberg court block rule that would let you cancel subscription easily sp future tick higher a investor shrug off trump tariff threat fomc minute on tap today mortgage refinance rate july rate increase mortgage rate today july rate move up cd rate today july rate rise uae say the oil market is thirsty for more opec barrel proposed clermont subdivision would redesign deadly lakeshore drive exact science announces medicare coverage for oncodetecttm molecular residual disease test in colorectal cancer fresh del monte produce inc to report second quarter financial result trump trade blitz produce few deal but lot of uncertainty trump trade blitz produce few deal but lot of uncertainty trump trade blitz produce few deal but lot of uncertainty trump trade blitz produce few deal but lot of uncertainty trump trade blitz produce few deal but lot of uncertainty trump trade blitz produce few deal but lot of uncertainty a new era of restaurant worker may earn sixfigure salary and benefit that no other industry can provide tesla board need ground rule for musk political activism analyst say samsung launch three new foldable smartphones a it fends off chinese rival trump tariff extension leaf bank fed in limbo hbo max is back prestige brand return to streaming corra group see rising demand from global investor for due diligence investigation market sputter after trump push tariff deadline xrp price forecast hit but insider are loading up on the new xrp that could go x auddia announces leadership change and special committee to evaluate business combination and restructuring a ai native holding company senate gop gear up for test on trump doge cut inside information orion upgrade fullyear outlook for social security sends million of american a misleading and blatantly political message see this shreveport director awardwinning screenplay red carpet premiere here how first atlantic nickel expands rpm zone awaruite nickelalloy nife discovery meter northern extension yield nickel concentrate over meter in dtr metallurgical recovery testing shreveport to kick off return of eleven store to louisiana more site planned two ragnarok ip title achieved top game ranking in taiwan hong kong and macau toast inc nysetost share acquired by da davidson co private trust co na ha stock holding in ge healthcare technology inc nasdaqgehc trump big beautiful bill slash cfpb funding what it mean for you davenport co llc sell share of fortive corporation nyseftv private trust co na acquires share of emcor group inc nyseeme you have le than month to claim the ev tax credit now is the time to buy say car expert this legend cross time zone with just pound of gear here are his favorite principal financial group inc increase stock position in zimmer biomet holding inc nysezbh mutual advisor llc buy share of trane technology plc nysett mutual advisor llc grows stock holding in decker outdoor corporation nysedeck first malaria drug for newborn and young infant expected to be approved in africa within week former rapid city anchor given suspended sentence in domestic assault case bank of england warns of high financial market risk despite easing tension kisti secures funding for national quantum center of excellence name ionq a primary quantum partner our opinion when the president punishes patriot wednesday letter a the world burn eye turn to diddy european court russia wa behind downing of mh watch popular podcaster discus how kamala episode wa scrapped because she talked gibberish her own campaign wanted it canned fbi bust chinese national for multimillion dollar drug ring exploiting immigration system the president mean business trump admin sue california over transgender athlete policy other view state congressional delegation must fight cut to noaa burke county company say hildebran wont issue permit for train cabin business another voice buffalo garden vibrantly express a community soul trump admin subpoena harvard over foreign student misconduct campus radicalism george conway flag trump awkward new admission a fresh proof he a fool eu seek to finalize trade deal with trump by end of the month hawaii lawmaker demand immigration arrest briefing haleiwa development under council review state road usage charge begin for electric vehicle on july governor state budget veto trim public school maintenance hooser sbcd a travesty of process and policy senate gop gear up for test on trump doge cut senate gop gear up for test on trump doge cut jewish democrat in congress sound the alarm on mamdani tea party patriot to push lawmaker on noncitizen voting jewish democrat in congress sound the alarm on mamdani tea party patriot to push lawmaker on noncitizen voting senate gop gear up for test on trump doge cut larger fight rage on but trump racking up win against college tea party patriot to push lawmaker on noncitizen voting jewish democrat in congress sound the alarm on mamdani larger fight rage on but trump racking up win against college larger fight rage on but trump racking up win against college senate gop gear up for test on trump doge cut senate gop gear up for test on trump doge cut tea party patriot to push lawmaker on noncitizen voting jewish democrat in congress sound the alarm on mamdani tea party patriot to push lawmaker on noncitizen voting jewish democrat in congress sound the alarm on mamdani senate gop gear up for test on trump doge cut larger fight rage on but trump racking up win against college tea party patriot to push lawmaker on noncitizen voting larger fight rage on but trump racking up win against college jewish democrat in congress sound the alarm on mamdani larger fight rage on but trump racking up win against college candace cameron bure say son biblebased pep talk helped save her marriage antiviolence advocate why not hold gun manufacturer accountable for mass shooting like river north tragedy letter chicago allows people to be who they want to be trump trade blitz produce few deal but lot of uncertainty laura washington the art institute is slowly getting back to normal georgia police arrest farmworkers then get warrant from dhs firearm testing and ballistics unit could be open in september at county forensics lab former dc fire official want to cut tax increase police presence with city council bid my view trekking pole can lend some mountainclimber swagger steve corbin give me liberty or a tinpot dictator scare buying reported in rochester why should legislator favor legal pot business california focus why should legislator favor legal pot business california focus editorial cartoon for july this legend cross time zone with just pound of gear here are his favorite which u president had wife named ellen and edith first malaria drug for newborn and young infant expected to be approved in africa within week red bull team principal christian horner fired after year with team after month stuck in the south north korean go home letter billion not served by trump big bill letter billion not served by trump big bill supreme court reject shielding identity of police attending jan capitol rally trump slam democrat over inflation narrative say he cut cost more than any president in history red bull team principal christan horner sacked after year with team letter no one is voting after result are known letter no one is voting after result are known here everything to expect at this family fun day in colnes alkincoates park robinhood ceo tokenization is a major innovation in capital market here who will and wont qualify for the new car loan interest deduction allegheny county council approves innamorato choice for shuman advisory board pittsburgh city council pass further protection for lgbtq people elon musk grok remove politically incorrect instruction after it praise hitler wa the flash flooding in texas preventable trump say tariff on pharmaceutical import could increase to percent threetime mvp nikola jokic will delay signing extension with nugget this summer ap source say trump boast about threat to bomb the st out of moscow in leaked audio charles warns small boat crisis is a profound challenge a he host macron at state banquet ahead of migrant deal newsom go big on holy grail reform other view newsom go big on holy grail reform other view supreme court allows trump administration to resume mass federal layoff for now suit challenge government effort to deport supporter of propalestinian protest invest america act give to every u newborn investment account dell ceo call it futureproofing prosperity sam altman asks for more stuff like this reader speak why i say thank you to uconn health center off the rail trump ramble in the middle of cabinet meeting is karat nonsense wall street trump taco trade ha a chicken and an egg problem meet the new national police force mamdanis farleft ally want to primary hakeem jeffries and other nyc democrat reader speak american tragedy is that those who are in power are inhumane congressional democrat push for new watchdog to oversee trump white house american need to work together to fix education weve both done it before on opposite side the search for the old lady pony continues tariff are already squeezing corporate margin new survey find ai is changing the world faster than most realize fencing wa a chore that we enjoyed texas is relying on fema state leader said it should be cut letter trump usaid action are evil letter trump usaid action are evil microsoft patch vulnerability including critical flaw in spnego and sql server</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>time run out for nearly centuryold michigan clock company due to tariff other factor ap news sage rhino capital llc sell share of shell plc unsponsored adr nyseshel vanguard total stock market etf nysearcavti position increased by seamount financial group inc sage rhino capital llc acquires share of vanguard total stock market etf nysearcavti kesler norman wride llc boost stake in broadcom inc nasdaqavgo genus capital management inc invests million in ishares msci eafe etf nysearcaefa sage rhino capital llc buy share of broadcom inc nasdaqavgo vanguard total stock market etf nysearcavti is clarity wealth advisor llcs rd largest position seamount financial group inc buy share of vanguard dividend appreciation etf nysearcavig state of michigan retirement system ha million stock holding in chubb limited nysecb state of michigan retirement system ha million position in lam research corporation nasdaqlrcx clarity wealth advisor llc reduces holding in the walt disney company nysedis genus capital management inc make new investment in ishares msci eafe etf nysearcaefa kesler norman wride llc buy share of vanguard information technology etf nysearcavgt chubb limited nysecb share sold by state of michigan retirement system sage rhino capital llc purchase share of broadcom inc nasdaqavgo state of michigan retirement system decrease stake in lam research corporation nasdaqlrcx seamount financial group inc raise stock holding in vanguard dividend appreciation etf nysearcavig think quantum computing will be the next big thing these are the stock to buy today boss quietly veto devastating law that may pull the rug out on american and thousand would lose cash ford recall vehicle over fuel pump defect manufacturing layoff at pacira oak hill bios phase angelman data france launch criminal investigation into musk x over algorithm manipulation politicoeu trump million crypto mystery man reuters buy the dip win again for stock investor rockwell automation pharmasuite power sinteticas swiss drug production teledyne raymarine acquires maretron asset to boost marine automation cummins unveils new hydrogen turbocharger for european heavyduty engine dover techcon unveils new precision dispensing cartridge for key industry carrier global enhances aipowered abound app for proactive building management trane technology debut first u dynamic closed loop geothermal system in chicago school district johnson control sensormatic solution launch aipowered shopper tracking with privacyfirst reid technology goldman sachs mustbuy chip stock and a few you should forget honeywell explores sale of two division ahead of planned split raytheon from rtx demonstrates autonomous barracuda mine neutralization vehicle gmbacked energyx expands lithium holding in u smackover formation with pantera acquisition boeing win b space force contract for nextgen nuclear comms satellite penguin solution launch nextgen stratus ztc endurance for ultrahigh availability ai workload clarivate unveils enhanced g research innovation scorecard with expanded data ai insight xerox completes b lexmark acquisition support print market position globant suntory global spirit partner to deploy gen ai commercial insight agent concentrix half carbon emission target by detail progress in sustainability report dxc technology aipowered tendia solution slash bid writing time for ventia genpact launch aipowered ap suite to revolutionize account payable process kyndryl launch new aipowered service to accelerate mainframe migration to aws saic awarded m air force contract for rapid warfighting prototype development shopper can now buy a bjs membership for just a year in new deal it cheaper than rival sam club u bank set to post trading gain on trump tariff turmoil cognizant pledge to white house ai education initiative aim to train m by education department to resume interest accrual on million student loan borrower rtx corporation nysertx stake reduced by cfolife group llc fonville wealth management llc cut stake in costco wholesale corporation nasdaqcost kesler norman wride llc acquires share of invesco qqq nasdaqqqq bernardo wealth planning llc cut stock holding in alphabet inc nasdaqgoog nextera energy inc nysenee holding lifted by cerity partner llc leavell investment management inc reduces position in ishares core u aggregate bond etf nysearcaagg leavell investment management inc raise stake in uber technology inc nyseuber fonville wealth management llc sell share of southern company the nyseso cerity partner llc boost holding in invesco qqq nasdaqqqq capital insight partner llc raise stock holding in freeportmcmoran inc nysefcx kesler norman wride llc sell share of stryker corporation nysesyk costco wholesale corporation nasdaqcost share sold by alp advisor inc fonville wealth management llc increase stake in vanguard growth etf nysearcavug capital insight partner llc acquires share of freeportmcmoran inc nysefcx kesler norman wride llc increase stock holding in linde plc nasdaqlin phillips financial management llc sell share of schwab u largecap etf nysearcaschx financial gravity asset management inc purchase new position in costco wholesale corporation nasdaqcost kesler norman wride llc sell share of stryker corporation nysesyk parr mcknight wealth management group llc trim holding in spdr gold share nysearcagld cerity partner llc trim stock position in adobe inc nasdaqadbe uk business confidence plummet to threeyear low icaew walmart recall water bottle after two consumer suffer vision loss from ejecting lid walmart recall water bottle after two consumer suffer vision loss from ejecting lid walmart recall water bottle after two consumer suffer vision loss from ejecting lid walmart recall water bottle after two consumer suffer vision loss from ejecting lid wall street giant issue stark message on sp walmart recall water bottle after two consumer suffer vision loss from ejecting lid ap news nikki bella discusses wwe evolution looking at ge vernovas recent unusual option activity check out what whale are doing with citigroup analyzing broadcom in comparison to competitor in semiconductor semiconductor equipment industry chief executive officer of integral ad science holdi sold k in stock italianstyle villa in south minneapolis linden hill listed for m sell alert aaron yeon ho lee cash out m in acushnet holding stock sell alert kevin chang keun yoon cash out m in acushnet holding stock allworth financial lp raise holding in pepsico inc nasdaqpep state of michigan retirement system ha million holding in philip morris international inc nysepm state of michigan retirement system sell share of intuit inc nasdaqintu cisco system inc nasdaqcsco share sold by state of michigan retirement system state of michigan retirement system sell share of pepsico inc nasdaqpep leavell investment management inc sell share of merck co inc nysemrk mjp associate inc adv increase stake in invesco sp equal weight etf nysearcarsp state of michigan retirement system cut stake in merck co inc nysemrk state of michigan retirement system reduces holding in ishares core sp midcap etf nysearcaijh merck co inc nysemrk stake reduced by leavell investment management inc insider decision gene soo yoon yoon offloads m worth of acushnet holding stock lacroix announces new partnership with the dallas wing wnba team royal caribbean take delivery of world largest cruise ship insider decision tod e carpenter exercise option at donaldson for m evaluating apple against peer in technology hardware storage peripheral industry clarity wealth advisor llc sell share of the walt disney company nysedis state of michigan retirement system reduces stock holding in cme group inc nasdaqcme state of michigan retirement system ha million stock holding in palo alto network inc nasdaqpanw sage rhino capital llc cut position in vanguard ftse allworld exus etf nysearcaveu cfc planning co llc ha million stake in the walt disney company nysedis parr mcknight wealth management group llc sell share of spdr gold share nysearcagld kesler norman wride llc ha million position in fortinet inc nasdaqftnt round rock advisor llc purchase share of verizon communication inc nysevz financial gravity asset management inc buy share of costco wholesale corporation nasdaqcost phillips financial management llc sell share of schwab u largecap etf nysearcaschx round rock advisor llc ha stock holding in salesforce inc nysecrm kesler norman wride llc buy share of linde plc nasdaqlin omb director question powell over fed hq renovation spending perfektblue bluetooth vulnerability expose million of vehicle to remote code execution trump doing all the thing he said he would bondi or bongino bongino wont remain at fbi if bondi keep job source say u is selling weapon to nato ally to give to ukraine trump say ishares core sp midcap etf nysearcaijh share sold by state of michigan retirement system kla corporation nasdaqklac share bought by mjp associate inc adv state of michigan retirement system ha million stock position in merck co inc nysemrk veteran political reporter reveals what the medium missed about trump appeal to american in back to back barrie could the antisemitism plan be used to silence dissent podcast the special envoy plan is the latest push to weaponise antisemitism a a relentless campaign pay off louise adler albanese must be careful that tackling antisemitism doesnt curb free speech tom mcilroy virginia rep john mcguire bought over k worth of meta platform stock here what you should know congressional trading report rep susie lee sold over k in full house resort stock state right to sue over medical privacy state right to sue over medical privacy state right to sue over medical privacy california rep gilbert ray cisneros sold over k worth of springworks therapeutic inc ordinary share stock here what you should know laurel libby stood strong in the face of tyranny letter beth claybourn interior trump new front in the war on drug the bank the u air force want million to double production of the aim missile new themed playground equipment officially open for use in two lake charles park steve mann more on the aftermath of magees time in san bruno new england professional planning group inc reduces holding in international business machine corporation nyseibm pfizer inc nysepfe share sold by new england professional planning group inc diversify wealth management llc buy share of cocacola company the nyseko bipartisan legislation aim to legalize adultuse cannabis in pennsylvania cerity partner llc boost holding in mcdonalds corporation nysemcd mjp associate inc adv raise stock position in mcdonalds corporation nysemcd mcdonalds corporation nysemcd share purchased by freedom day solution llc moloney security asset management llc buy share of vanguard total bond market etf nasdaqbnd benny blanco ha made so much music he ha to shazam his own tune elv deadline today rosen leading trial attorney encourages elevance health inc investor epstein conspiracy just isnt there teacher union reveals true color and more from fox news opinion stratos wealth advisor llc trim stock position in the goldman sachs group inc nysegs freedom day solution llc decrease stock holding in amgen inc nasdaqamgn lbp am sa sell share of visa inc nysev the mindful minute by jon heydenreich that martini and megaburger u is selling weapon to nato ally to give to ukraine trump say u is selling weapon to nato ally to give to ukraine trump say u is selling weapon to nato ally to give to ukraine trump say u is selling weapon to nato ally to give to ukraine trump say u is selling weapon to nato ally to give to ukraine trump say greater midwest financial group llc purchase share of vanguard sp etf nysearcavoo barry investment advisor llc sell share of vanguard ftse emerging market etf nysearcavwo state department is firing over employee under trump administration plan rubio and wang stress cooperation after talk in malaysia a uschina tension simmer diversify wealth management llc buy share of ishares u treasury bond etf batsgovt cromwell holding llc decrease stake in micron technology inc nasdaqmu vanguard value etf nysearcavtv share sold by ade llc chevron corporation nysecvx share purchased by diversify wealth management llc cromwell holding llc raise stake in monolithic power system inc nasdaqmpwr church street road closure extended in brattleboro u is selling weapon to nato ally to give to ukraine trump say noqualifyjpg bill to clarify st louis sheriff duty stall in committee strategist flag very unusual trump admin loyalty test on cnn fidelis capital partner llc ha million stake in thermo fisher scientific inc nysetmo pkk fighter pile up their weapon in arm amnesty in northern iraq brazil vow retaliatory tariff against u if trump follows through on import tax new pac form to back mamdani nyc mayoral bid a business community rally to defeat him history program highlight the map and stone wall of dummerson financial gravity asset management inc buy new position in ishares tip bond etf nysearcatip phillips financial management llc increase holding in vanguard ftse developed market etf nysearcavea trump plan to hike tariff on canadian good to trump plan to tour texas flood damage a the scope of the disaster test his pledge to shutter fema trump plan to hike tariff on canadian good to ishares msci emerging market etf nysearcaeem share sold by ramsay stattman vela price inc burford brother inc raise position in the sherwinwilliams company nyseshw spdr dow jones industrial average etf trust nysearcadia position lifted by christopher j hasenberg inc genus capital management inc invests million in the sherwinwilliams company nyseshw state department to axe employee state of michigan retirement system boost stock position in prologis inc nysepld advanced micro device inc nasdaqamd share purchased by clarity wealth advisor llc seamount financial group inc sell share of vanguard total world stock etf nysearcavt share in vaneck gold miner etf nysearcagdx acquired by sage rhino capital llc vestia personal wealth advisor increase position in dimensional u marketwide value etf nysearcadfuv milwaukee remove fonzie statue amid reckoning with greaser past noqualifyingjpg exxon mobil corporation nysexom share sold by pineridge advisor llc cfolife group llc buy share of ge aerospace nysege stonebrook private inc buy share of vanguard total stock market etf nysearcavti allworth financial lp grows position in united parcel service inc nyseups cerity partner llc sell share of adobe inc nasdaqadbe adobe inc nasdaqadbe holding lowered by xponance inc honeywell international inc nasdaqhon share bought by kesler norman wride llc amphenol corporation nyseaph position boosted by cerity partner llc b t capital management dba alpha capital management make new investment in taiwan semiconductor manufacturing company ltd nysetsm vanguard midcap etf nysearcavo is beirne wealth consulting service llcs th largest position vanguard smallcap etf nysearcavb share sold by b t capital management dba alpha capital management walmart inc nysewmt position increased by fort sheridan advisor llc kathmere capital management llc buy share of vanguard smallcap etf nysearcavb kathmere capital management llc purchase share of walmart inc nysewmt ishares core sp smallcap etf nysearcaijr share sold by forum private client group llc kathmere capital management llc purchase share of vanguard smallcap etf nysearcavb b t capital management dba alpha capital management boost position in honeywell international inc nasdaqhon fort sheridan advisor llc boost stake in walmart inc nysewmt ifc advisor llc sell share of the home depot inc nysehd ifc advisor llc ha million holding in pepsico inc nasdaqpep quest wealth builder inc sell share of eli lilly and company nyselly caterpillar inc nysecat share sold by ifc advisor llc ballentine partner llc lower position in invesco qqq nasdaqqqq quest wealth builder inc sell share of pepsico inc nasdaqpep ballentine partner llc sell share of invesco qqq nasdaqqqq caterpillar inc nysecat share sold by ifc advisor llc eureka business weather economic uncertainty ap business summarybrief at pm edt ap business summarybrief at pm edt why share of the metal company skyrocketed in the first half of why share of the metal company skyrocketed in the first half of is circle internet stock a millionaire maker another large grocery chain follows kroger in closing store is circle internet stock a millionaire maker another large grocery chain follows kroger in closing store fulcrum equity management ha stake in broadcom inc nasdaqavgo why nvidia partner navitas semiconductor surged in the first half of why nvidia partner navitas semiconductor surged in the first half of a bitcoin matures volatility dropsso expect slower climb say expert decrypt crypto top gainer why blockdag solana pepe and render are leading in growth and utility how ai notetakers can become the black box of business the low altitude market could be worth trillion by according to morgan stanley this cathie wood stock is my top pick to dominate the opportunity hint it not archer aviation the low altitude market could be worth trillion by according to morgan stanley this cathie wood stock is my top pick to dominate the opportunity hint it not archer aviation iron ore price surge amid china industrial crackdown northwest capital management inc buy share of ishares core sp midcap etf nysearcaijh rational advisor inc invests million in mcdonalds corporation nysemcd superman smash box office expectation soaring towards million opening pam bondi fire doj staffer who worked on trump case amid chaos at agency nikulski financial inc buy share of lowes company inc nyselow mjp associate inc adv ha holding in blackstone inc nysebx cerity partner llc grows stock position in palantir technology inc nasdaqpltr trump to impose tariff on eu mexico starting aug trump to impose eu tariff on aug trumnp to impose eu tariff on august trump announces tariff on import from mexico eu eu say it still want u trade deal will defend interest tucker carlson reveals who he think funded jeffrey epstein crime focused wealth management inc increase stock position in merck co inc nysemrk roger wittlin investment advisory llc acquires share of vanguard sp etf nysearcavoo family firm inc ha million stock holding in ishares russell etf nysearcaiwm schwab u smallcap etf nysearcascha share sold by family firm inc roger wittlin investment advisory llc purchase share of vanguard sp etf nysearcavoo quest wealth builder inc ha stock holding in parkerhannifin corporation nyseph share in vanguard high dividend yield etf nysearcavym acquired by stillwater wealth management group ishares russell etf nysearcaiwm share sold by family firm inc well fargo company nysewfc share sold by family firm inc bank of america corporation nysebac share acquired by fortem financial group llc fortem financial group llc boost stock position in att inc nyset unitedhealth down is the dividend still safe netflix inc nasdaqnflx share acquired by martin capital advisor llp vanguard ftse developed market etf nysearcavea share purchased by bridge generation wealth management llc riversedge advisor llc grows holding in vanguard ftse emerging market etf nysearcavwo american financial advisor llc reduces stock holding in ge vernova inc nysegev crowdstrike nasdaqcrwd share acquired by american financial advisor llc riversedge advisor llc purchase share of alphabet inc nasdaqgoog vanguard value etf nysearcavtv share purchased by riversedge advisor llc vanguard value etf nysearcavtv share purchased by riversedge advisor llc crowdstrike nasdaqcrwd share bought by american financial advisor llc tesla inc nasdaqtsla share bought by riversedge advisor llc riversedge advisor llc ha holding in salesforce inc nysecrm american financial advisor llc ha million position in ishares core sp etf nysearcaivv vanguard ftse developed market etf nysearcavea position decreased by riversedge advisor llc grant grossmendelsohn llc ha holding in vanguard ftse developed market etf nysearcavea dogecoins doge holder are shifting to ruvi ai ruvi passed audit and early entry bonus make it the smarter bet auour investment llc ha million stake in ishares core msci eafe etf batsiefa fort sheridan advisor llc raise stock holding in abbott laboratory nyseabt beirne wealth consulting service llc increase stock position in ishares core msci eafe etf batsiefa b t capital management dba alpha capital management buy share of schwab u largecap growth etf nysearcaschg b t capital management dba alpha capital management purchase share of schwab u largecap growth etf nysearcaschg quest wealth builder inc cut stock position in walmart inc nysewmt ifc advisor llc reduces position in vanguard midcap etf nysearcavo spdr gold share nysearcagld share purchased by acorn wealth advisor llc ballentine partner llc increase position in chevron corporation nysecvx acorn wealth advisor llc sell share of ishares core sp smallcap etf nysearcaijr acorn wealth advisor llc ha stock position in vanguard midcap etf nysearcavo acorn wealth advisor llc reduces stock position in ishares core sp smallcap etf nysearcaijr ballentine partner llc acquires share of walmart inc nysewmt history say these stock could be big winner in the second half history say these stock could be big winner in the second half alp advisor inc ha million stock position in kkr co inc nysekkr eli lilly and company nyselly share sold by wealthtrust asset management llc eli lilly and company nyselly is harmony asset management llcs th largest position the home depot inc nysehd share purchased by lane associate llc fulcrum equity management lower stock holding in eli lilly and company nyselly fulcrum equity management sell share of eli lilly and company nyselly servicenow inc nysenow share acquired by steelpeak wealth llc trump target mexico eu with tariff hartford bakery inc voluntarily recall hundred of loaf of artisanal bread sold in state cbs news reader view we can all reduce greenhouse gas shes great trump back bondi want top official to end conflict over epstein ishares core sp smallcap etf nysearcaijr share sold by forum private client group llc chevron corporation nysecvx share acquired by b t capital management dba alpha capital management forum private client group llc ha million position in vanguard midcap etf nysearcavo b t capital management dba alpha capital management increase stake in honeywell international inc nasdaqhon beirne wealth consulting service llc acquires share of vanguard smallcap etf nysearcavb ifc advisor llc boost holding in kkr co inc nysekkr ballentine partner llc grows holding in eli lilly and company nyselly young democrat have called for a rebrand theyre vying to replace the party old guard temperance in cabinetry climate change helped fuel heavy rain that led to devastating texas flood former pentagon insider could trump big beautiful bill finally unlock america longforgotten resource archaeolgists find largestever ceremony hall weapon hoard the democratic party is missing an opportunity to engage christian voter northwest capital management inc purchase share of ishares core sp midcap etf nysearcaijh rational advisor inc take position in mcdonalds corporation nysemcd superman smash box office expectation soaring towards million opening pam bondi fire doj staffer who worked on trump case amid chaos at agency nikulski financial inc acquires share of lowes company inc nyselow parkerhannifin corporation nyseph share sold by quest wealth builder inc family firm inc lower stock holding in schwab u smallcap etf nysearcascha family firm inc reduces stock holding in well fargo company nysewfc stillwater wealth management group invests in vanguard high dividend yield etf nysearcavym extrump lawyer dershowitz claim knowledge of epstein client list i know the name but im bound by confidentiality grant grossmendelsohn llc purchase share of vanguard ftse developed market etf nysearcavea riversedge advisor llc cut stake in vanguard ftse developed market etf nysearcavea piper sandler issue positive forecast for netflix nasdaqnflx stock price riversedge advisor llc ha holding in salesforce inc nysecrm american financial advisor llc ha million stake in ishares core sp etf nysearcaivv riversedge advisor llc increase stake in ishares core sp etf nysearcaivv start exploring cloud mining for free from the new winnermining app and get visible daily reward forum private client group llc trim position in vanguard growth etf nysearcavug fort sheridan advisor llc buy share of vanguard growth etf nysearcavug the big beautiful bill and mlp qualifying income acorn wealth advisor llc lower holding in chevron corporation nysecvx ballentine partner llc buy share of walmart inc nysewmt ballentine partner llc sell share of ishares core sp smallcap etf nysearcaijr lane associate llc sell share of eli lilly and company nyselly harmony asset management llc ha million holding in the home depot inc nysehd steelpeak wealth llc ha million stake in the progressive corporation nysepgr servicenow inc nysenow share acquired by steelpeak wealth llc trump threatens rosie odonnells citizenship she is a threat to humanity annual new london to new brighton antique car run to take place aug coyle financial counsel llc invests in qualcomm incorporated nasdaqqcom broadcom inc nasdaqavgo share sold by skyoak wealth llc forum private client group llc take position in elevance health inc nyseelv a major red flag for republican a trump policy threatens their future fbi director kash patel responds to controversy surrounding epstein file stillwater wealth management group grows position in amgen inc nasdaqamgn riversedge advisor llc grows stake in tesla inc nasdaqtsla fort sheridan advisor llc ha position in kla corporation nasdaqklac kathmere capital management llc grows holding in vanguard value etf nysearcavtv nycs broken election system need far more than these bandaid fix ballentine partner llc ha million position in abbott laboratory nyseabt abbott laboratory nyseabt share acquired by ifc advisor llc trump post support for embattled attorney general pam bondi ma private wealth take position in bristol myers squibb company nysebmy parkerhannifin corporation nyseph share sold by lbp am sa harmony asset management llc reduces stock position in chevron corporation nysecvx bonus editorial cartoon for july federal employee bracing after supreme court greenlights widespread layoff federal employee bracing after supreme court greenlights widespread layoff federal employee bracing after supreme court greenlights widespread layoff lawmaker visit alligator alcatraz but some wonder how much theyll get to see man convicted of meredith kerchers murder facing trial for sexual assault federal employee bracing after supreme court greenlights widespread layoff federal employee bracing after supreme court greenlights widespread layoff federal employee bracing after supreme court greenlights widespread layoff focused wealth management inc ha million stake in walmart inc nysewmt berbice capital management llc grows position in kkr co inc nysekkr coyle financial counsel llc raise holding in invesco qqq nasdaqqqq meet china man in lima who jetted over to u to collect train donated by biden admin amazon prime day delivers record sale and saving in expanded fourday shopping event how new tax legislation impact clean energy tax credit the dalai lama is planning his succession a the ultimate protest against china the u army m vulcan air defense system wa a beast in the vietnam war the us john f kennedy fordclass carrier may miss it delivery date comcast corporation nasdaqcmcsa share sold by sage rhino capital llc kesler norman wride llc sell share of comcast corporation nasdaqcmcsa exchange capital management inc sell share of servicenow inc nysenow fukoku mutual life insurance co sell share of duke energy corporation nyseduk cerity partner llc buy share of asml holding nv nasdaqasml mjp associate inc adv take position in elevance health inc nyseelv fidelis capital partner llc boost stock position in elevance health inc nyseelv reader view u must invest in our independence candidate view localgovernment focus would benefit school board stillwater wealth management group reduces position in unitedhealth group incorporated nyseunh martin capital advisor llp sell share of oracle corporation nyseorcl park square financial group llc decrease stock position in ishares core sp midcap etf nysearcaijh fortem financial group llc purchase share of blackstone inc nysebx pya waltman capital llc ha million stake in mcdonalds corporation nysemcd massachusetts police officer shot by colleague victim of campaign to criminalize her lawyer horrified by alligator alcatraz letter coyle financial counsel llc ha million stake in ishares core sp etf nysearcaivv vanguard high dividend yield etf nysearcavym stock holding decreased by auour investment llc ifc advisor llc increase position in ishares russell etf nysearcaiwm forum private client group llc purchase new stake in cummins inc nysecmi fortem financial group llc grows holding in tesla inc nasdaqtsla vanguard ftse developed market etf nysearcavea share purchased by beirne wealth consulting service llc schear investment adviser llc buy share of tmobile u inc nasdaqtmus jrmc recognized for infection control rate wall street pro drop bold price target on circle stock bitcoin hit new alltime high above k a trader eye week uptrend cointelegraph cardinal strategic wealth guidance cut position in alphabet inc nasdaqgoog bradley co private wealth management llc reduces position in costco wholesale corporation nasdaqcost pointe capital management llc grows holding in the walt disney company nysedis westmount partner llc sell share of amgen inc nasdaqamgn westmount partner llc sell share of starbucks corporation nasdaqsbux westmount partner llc trim holding in lockheed martin corporation nyselmt q asset management buy share of williams company inc the nysewmb westmount partner llc trim holding in lockheed martin corporation nyselmt westmount partner llc trim stock position in amgen inc nasdaqamgn zullo investment group inc lower stock position in alphabet inc nasdaqgoog trunorth capital management llc acquires share of vanguard sp etf nysearcavoo pointe capital management llc boost holding in linde plc nasdaqlin ishares core u aggregate bond etf nysearcaagg share acquired by pointe capital management llc nextera energy inc nysenee share sold by pointe capital management llc bristol myers squibb company nysebmy stock holding lifted by prudent man advisor llc mqs management llc buy new position in nextera energy inc nysenee prudent man advisor llc acquires new position in blackrock nyseblk zullo investment group inc buy share of eli lilly and company nyselly zullo investment group inc acquires share of eli lilly and company nyselly zullo investment group inc cut stake in m company nysemmm prudent man advisor llc make new million investment in blackrock nyseblk mqs management llc take position in nextera energy inc nysenee ai financial service llc boost holding in eli lilly and company nyselly u tomato price could jump a soon a monday xrp break out near gain yet blockdags coin unlock chance at steal market focus top altcoins still lag while bitcoin stay strong promising outdoor stock to add to your watchlist july th kathmere capital management llc sell share of kimberlyclark co nysekmb citigroup inc nysec share purchased by ballentine partner llc cigna group nyseci share bought by ballentine partner llc ballentine partner llc purchase share of the sherwinwilliams company nyseshw arizona state retirement system purchase share of kimberlyclark co nysekmb bankplus trust department grows holding in ishares core sp smallcap etf nysearcaijr berkeley inc ha million holding in schwab u largecap etf nysearcaschx arizona state retirement system increase stake in kimberlyclark co nysekmb fdx advisor inc invests in medtronic plc nysemdt how trump latest tariff threat risk deeper damage to europe economy fort sheridan advisor llc increase stock position in cocacola company the nyseko fortem financial group llc sell share of conocophillips nysecop blackstone inc nysebx share bought by louisiana state employee retirement system eaton corporation plc nyseetn share sold by stephen inc ar taiwan semiconductor manufacturing company ltd nysetsm share sold by fulton breakefield broenniman llc why broadcoms avgo ai momentum ha goldman sachs backing the stock on gps nvidia ceo on the overwhelmingly positive effect of ai isthmus partner llc sell share of thermo fisher scientific inc nysetmo whitener ca</t>
+          <t>time run out for nearly centuryold michigan clock company due to tariff other factor ap news sage rhino capital llc sell share of shell plc unsponsored adr nyseshel vanguard total stock market etf nysearcavti position increased by seamount financial group inc sage rhino capital llc acquires share of vanguard total stock market etf nysearcavti kesler norman wride llc boost stake in broadcom inc nasdaqavgo genus capital management inc invests million in ishares msci eafe etf nysearcaefa sage rhino capital llc buy share of broadcom inc nasdaqavgo vanguard total stock market etf nysearcavti is clarity wealth advisor llcs rd largest position seamount financial group inc buy share of vanguard dividend appreciation etf nysearcavig state of michigan retirement system ha million stock holding in chubb limited nysecb state of michigan retirement system ha million position in lam research corporation nasdaqlrcx clarity wealth advisor llc reduces holding in the walt disney company nysedis genus capital management inc make new investment in ishares msci eafe etf nysearcaefa kesler norman wride llc buy share of vanguard information technology etf nysearcavgt chubb limited nysecb share sold by state of michigan retirement system sage rhino capital llc purchase share of broadcom inc nasdaqavgo state of michigan retirement system decrease stake in lam research corporation nasdaqlrcx seamount financial group inc raise stock holding in vanguard dividend appreciation etf nysearcavig think quantum computing will be the next big thing these are the stock to buy today boss quietly veto devastating law that may pull the rug out on american and thousand would lose cash ford recall vehicle over fuel pump defect manufacturing layoff at pacira oak hill bios phase angelman data france launch criminal investigation into musk x over algorithm manipulation politicoeu trump million crypto mystery man reuters buy the dip win again for stock investor rockwell automation pharmasuite power sinteticas swiss drug production teledyne raymarine acquires maretron asset to boost marine automation cummins unveils new hydrogen turbocharger for european heavyduty engine dover techcon unveils new precision dispensing cartridge for key industry carrier global enhances aipowered abound app for proactive building management trane technology debut first u dynamic closed loop geothermal system in chicago school district johnson control sensormatic solution launch aipowered shopper tracking with privacyfirst reid technology goldman sachs mustbuy chip stock and a few you should forget honeywell explores sale of two division ahead of planned split raytheon from rtx demonstrates autonomous barracuda mine neutralization vehicle gmbacked energyx expands lithium holding in u smackover formation with pantera acquisition boeing win b space force contract for nextgen nuclear comms satellite penguin solution launch nextgen stratus ztc endurance for ultrahigh availability ai workload clarivate unveils enhanced g research innovation scorecard with expanded data ai insight xerox completes b lexmark acquisition support print market position globant suntory global spirit partner to deploy gen ai commercial insight agent concentrix half carbon emission target by detail progress in sustainability report dxc technology aipowered tendia solution slash bid writing time for ventia genpact launch aipowered ap suite to revolutionize account payable process kyndryl launch new aipowered service to accelerate mainframe migration to aws saic awarded m air force contract for rapid warfighting prototype development shopper can now buy a bjs membership for just a year in new deal it cheaper than rival sam club u bank set to post trading gain on trump tariff turmoil cognizant pledge to white house ai education initiative aim to train m by education department to resume interest accrual on million student loan borrower rtx corporation nysertx stake reduced by cfolife group llc fonville wealth management llc cut stake in costco wholesale corporation nasdaqcost kesler norman wride llc acquires share of invesco qqq nasdaqqqq bernardo wealth planning llc cut stock holding in alphabet inc nasdaqgoog nextera energy inc nysenee holding lifted by cerity partner llc leavell investment management inc reduces position in ishares core u aggregate bond etf nysearcaagg leavell investment management inc raise stake in uber technology inc nyseuber fonville wealth management llc sell share of southern company the nyseso cerity partner llc boost holding in invesco qqq nasdaqqqq capital insight partner llc raise stock holding in freeportmcmoran inc nysefcx kesler norman wride llc sell share of stryker corporation nysesyk costco wholesale corporation nasdaqcost share sold by alp advisor inc fonville wealth management llc increase stake in vanguard growth etf nysearcavug capital insight partner llc acquires share of freeportmcmoran inc nysefcx kesler norman wride llc increase stock holding in linde plc nasdaqlin phillips financial management llc sell share of schwab u largecap etf nysearcaschx financial gravity asset management inc purchase new position in costco wholesale corporation nasdaqcost kesler norman wride llc sell share of stryker corporation nysesyk parr mcknight wealth management group llc trim holding in spdr gold share nysearcagld cerity partner llc trim stock position in adobe inc nasdaqadbe uk business confidence plummet to threeyear low icaew walmart recall water bottle after two consumer suffer vision loss from ejecting lid walmart recall water bottle after two consumer suffer vision loss from ejecting lid walmart recall water bottle after two consumer suffer vision loss from ejecting lid walmart recall water bottle after two consumer suffer vision loss from ejecting lid wall street giant issue stark message on sp walmart recall water bottle after two consumer suffer vision loss from ejecting lid ap news nikki bella discus wwe evolution looking at ge vernovas recent unusual option activity check out what whale are doing with citigroup analyzing broadcom in comparison to competitor in semiconductor semiconductor equipment industry chief executive officer of integral ad science holdi sold k in stock italianstyle villa in south minneapolis linden hill listed for m sell alert aaron yeon ho lee cash out m in acushnet holding stock sell alert kevin chang keun yoon cash out m in acushnet holding stock allworth financial lp raise holding in pepsico inc nasdaqpep state of michigan retirement system ha million holding in philip morris international inc nysepm state of michigan retirement system sell share of intuit inc nasdaqintu cisco system inc nasdaqcsco share sold by state of michigan retirement system state of michigan retirement system sell share of pepsico inc nasdaqpep leavell investment management inc sell share of merck co inc nysemrk mjp associate inc adv increase stake in invesco sp equal weight etf nysearcarsp state of michigan retirement system cut stake in merck co inc nysemrk state of michigan retirement system reduces holding in ishares core sp midcap etf nysearcaijh merck co inc nysemrk stake reduced by leavell investment management inc insider decision gene soo yoon yoon offloads m worth of acushnet holding stock lacroix announces new partnership with the dallas wing wnba team royal caribbean take delivery of world largest cruise ship insider decision tod e carpenter exercise option at donaldson for m evaluating apple against peer in technology hardware storage peripheral industry clarity wealth advisor llc sell share of the walt disney company nysedis state of michigan retirement system reduces stock holding in cme group inc nasdaqcme state of michigan retirement system ha million stock holding in palo alto network inc nasdaqpanw sage rhino capital llc cut position in vanguard ftse allworld exus etf nysearcaveu cfc planning co llc ha million stake in the walt disney company nysedis parr mcknight wealth management group llc sell share of spdr gold share nysearcagld kesler norman wride llc ha million position in fortinet inc nasdaqftnt round rock advisor llc purchase share of verizon communication inc nysevz financial gravity asset management inc buy share of costco wholesale corporation nasdaqcost phillips financial management llc sell share of schwab u largecap etf nysearcaschx round rock advisor llc ha stock holding in salesforce inc nysecrm kesler norman wride llc buy share of linde plc nasdaqlin omb director question powell over fed hq renovation spending perfektblue bluetooth vulnerability expose million of vehicle to remote code execution trump doing all the thing he said he would bondi or bongino bongino wont remain at fbi if bondi keep job source say u is selling weapon to nato ally to give to ukraine trump say ishares core sp midcap etf nysearcaijh share sold by state of michigan retirement system kla corporation nasdaqklac share bought by mjp associate inc adv state of michigan retirement system ha million stock position in merck co inc nysemrk veteran political reporter reveals what the medium missed about trump appeal to american in back to back barrie could the antisemitism plan be used to silence dissent podcast the special envoy plan is the latest push to weaponise antisemitism a a relentless campaign pay off louise adler albanese must be careful that tackling antisemitism doesnt curb free speech tom mcilroy virginia rep john mcguire bought over k worth of meta platform stock here what you should know congressional trading report rep susie lee sold over k in full house resort stock state right to sue over medical privacy state right to sue over medical privacy state right to sue over medical privacy california rep gilbert ray cisneros sold over k worth of springworks therapeutic inc ordinary share stock here what you should know laurel libby stood strong in the face of tyranny letter beth claybourn interior trump new front in the war on drug the bank the u air force want million to double production of the aim missile new themed playground equipment officially open for use in two lake charles park steve mann more on the aftermath of magees time in san bruno new england professional planning group inc reduces holding in international business machine corporation nyseibm pfizer inc nysepfe share sold by new england professional planning group inc diversify wealth management llc buy share of cocacola company the nyseko bipartisan legislation aim to legalize adultuse cannabis in pennsylvania cerity partner llc boost holding in mcdonalds corporation nysemcd mjp associate inc adv raise stock position in mcdonalds corporation nysemcd mcdonalds corporation nysemcd share purchased by freedom day solution llc moloney security asset management llc buy share of vanguard total bond market etf nasdaqbnd benny blanco ha made so much music he ha to shazam his own tune elv deadline today rosen leading trial attorney encourages elevance health inc investor epstein conspiracy just isnt there teacher union reveals true color and more from fox news opinion stratos wealth advisor llc trim stock position in the goldman sachs group inc nysegs freedom day solution llc decrease stock holding in amgen inc nasdaqamgn lbp am sa sell share of visa inc nysev the mindful minute by jon heydenreich that martini and megaburger u is selling weapon to nato ally to give to ukraine trump say u is selling weapon to nato ally to give to ukraine trump say u is selling weapon to nato ally to give to ukraine trump say u is selling weapon to nato ally to give to ukraine trump say u is selling weapon to nato ally to give to ukraine trump say greater midwest financial group llc purchase share of vanguard sp etf nysearcavoo barry investment advisor llc sell share of vanguard ftse emerging market etf nysearcavwo state department is firing over employee under trump administration plan rubio and wang stress cooperation after talk in malaysia a uschina tension simmer diversify wealth management llc buy share of ishares u treasury bond etf batsgovt cromwell holding llc decrease stake in micron technology inc nasdaqmu vanguard value etf nysearcavtv share sold by ade llc chevron corporation nysecvx share purchased by diversify wealth management llc cromwell holding llc raise stake in monolithic power system inc nasdaqmpwr church street road closure extended in brattleboro u is selling weapon to nato ally to give to ukraine trump say noqualifyjpg bill to clarify st louis sheriff duty stall in committee strategist flag very unusual trump admin loyalty test on cnn fidelis capital partner llc ha million stake in thermo fisher scientific inc nysetmo pkk fighter pile up their weapon in arm amnesty in northern iraq brazil vow retaliatory tariff against u if trump follows through on import tax new pac form to back mamdani nyc mayoral bid a business community rally to defeat him history program highlight the map and stone wall of dummerson financial gravity asset management inc buy new position in ishares tip bond etf nysearcatip phillips financial management llc increase holding in vanguard ftse developed market etf nysearcavea trump plan to hike tariff on canadian good to trump plan to tour texas flood damage a the scope of the disaster test his pledge to shutter fema trump plan to hike tariff on canadian good to ishares msci emerging market etf nysearcaeem share sold by ramsay stattman vela price inc burford brother inc raise position in the sherwinwilliams company nyseshw spdr dow jones industrial average etf trust nysearcadia position lifted by christopher j hasenberg inc genus capital management inc invests million in the sherwinwilliams company nyseshw state department to axe employee state of michigan retirement system boost stock position in prologis inc nysepld advanced micro device inc nasdaqamd share purchased by clarity wealth advisor llc seamount financial group inc sell share of vanguard total world stock etf nysearcavt share in vaneck gold miner etf nysearcagdx acquired by sage rhino capital llc vestia personal wealth advisor increase position in dimensional u marketwide value etf nysearcadfuv milwaukee remove fonzie statue amid reckoning with greaser past noqualifyingjpg exxon mobil corporation nysexom share sold by pineridge advisor llc cfolife group llc buy share of ge aerospace nysege stonebrook private inc buy share of vanguard total stock market etf nysearcavti allworth financial lp grows position in united parcel service inc nyseups cerity partner llc sell share of adobe inc nasdaqadbe adobe inc nasdaqadbe holding lowered by xponance inc honeywell international inc nasdaqhon share bought by kesler norman wride llc amphenol corporation nyseaph position boosted by cerity partner llc b t capital management dba alpha capital management make new investment in taiwan semiconductor manufacturing company ltd nysetsm vanguard midcap etf nysearcavo is beirne wealth consulting service llcs th largest position vanguard smallcap etf nysearcavb share sold by b t capital management dba alpha capital management walmart inc nysewmt position increased by fort sheridan advisor llc kathmere capital management llc buy share of vanguard smallcap etf nysearcavb kathmere capital management llc purchase share of walmart inc nysewmt ishares core sp smallcap etf nysearcaijr share sold by forum private client group llc kathmere capital management llc purchase share of vanguard smallcap etf nysearcavb b t capital management dba alpha capital management boost position in honeywell international inc nasdaqhon fort sheridan advisor llc boost stake in walmart inc nysewmt ifc advisor llc sell share of the home depot inc nysehd ifc advisor llc ha million holding in pepsico inc nasdaqpep quest wealth builder inc sell share of eli lilly and company nyselly caterpillar inc nysecat share sold by ifc advisor llc ballentine partner llc lower position in invesco qqq nasdaqqqq quest wealth builder inc sell share of pepsico inc nasdaqpep ballentine partner llc sell share of invesco qqq nasdaqqqq caterpillar inc nysecat share sold by ifc advisor llc eureka business weather economic uncertainty ap business summarybrief at pm edt ap business summarybrief at pm edt why share of the metal company skyrocketed in the first half of why share of the metal company skyrocketed in the first half of is circle internet stock a millionaire maker another large grocery chain follows kroger in closing store is circle internet stock a millionaire maker another large grocery chain follows kroger in closing store fulcrum equity management ha stake in broadcom inc nasdaqavgo why nvidia partner navitas semiconductor surged in the first half of why nvidia partner navitas semiconductor surged in the first half of a bitcoin matures volatility dropsso expect slower climb say expert decrypt crypto top gainer why blockdag solana pepe and render are leading in growth and utility how ai notetakers can become the black box of business the low altitude market could be worth trillion by according to morgan stanley this cathie wood stock is my top pick to dominate the opportunity hint it not archer aviation the low altitude market could be worth trillion by according to morgan stanley this cathie wood stock is my top pick to dominate the opportunity hint it not archer aviation iron ore price surge amid china industrial crackdown northwest capital management inc buy share of ishares core sp midcap etf nysearcaijh rational advisor inc invests million in mcdonalds corporation nysemcd superman smash box office expectation soaring towards million opening pam bondi fire doj staffer who worked on trump case amid chaos at agency nikulski financial inc buy share of lowes company inc nyselow mjp associate inc adv ha holding in blackstone inc nysebx cerity partner llc grows stock position in palantir technology inc nasdaqpltr trump to impose tariff on eu mexico starting aug trump to impose eu tariff on aug trumnp to impose eu tariff on august trump announces tariff on import from mexico eu eu say it still want u trade deal will defend interest tucker carlson reveals who he think funded jeffrey epstein crime focused wealth management inc increase stock position in merck co inc nysemrk roger wittlin investment advisory llc acquires share of vanguard sp etf nysearcavoo family firm inc ha million stock holding in ishares russell etf nysearcaiwm schwab u smallcap etf nysearcascha share sold by family firm inc roger wittlin investment advisory llc purchase share of vanguard sp etf nysearcavoo quest wealth builder inc ha stock holding in parkerhannifin corporation nyseph share in vanguard high dividend yield etf nysearcavym acquired by stillwater wealth management group ishares russell etf nysearcaiwm share sold by family firm inc well fargo company nysewfc share sold by family firm inc bank of america corporation nysebac share acquired by fortem financial group llc fortem financial group llc boost stock position in att inc nyset unitedhealth down is the dividend still safe netflix inc nasdaqnflx share acquired by martin capital advisor llp vanguard ftse developed market etf nysearcavea share purchased by bridge generation wealth management llc riversedge advisor llc grows holding in vanguard ftse emerging market etf nysearcavwo american financial advisor llc reduces stock holding in ge vernova inc nysegev crowdstrike nasdaqcrwd share acquired by american financial advisor llc riversedge advisor llc purchase share of alphabet inc nasdaqgoog vanguard value etf nysearcavtv share purchased by riversedge advisor llc vanguard value etf nysearcavtv share purchased by riversedge advisor llc crowdstrike nasdaqcrwd share bought by american financial advisor llc tesla inc nasdaqtsla share bought by riversedge advisor llc riversedge advisor llc ha holding in salesforce inc nysecrm american financial advisor llc ha million position in ishares core sp etf nysearcaivv vanguard ftse developed market etf nysearcavea position decreased by riversedge advisor llc grant grossmendelsohn llc ha holding in vanguard ftse developed market etf nysearcavea dogecoins doge holder are shifting to ruvi ai ruvi passed audit and early entry bonus make it the smarter bet auour investment llc ha million stake in ishares core msci eafe etf batsiefa fort sheridan advisor llc raise stock holding in abbott laboratory nyseabt beirne wealth consulting service llc increase stock position in ishares core msci eafe etf batsiefa b t capital management dba alpha capital management buy share of schwab u largecap growth etf nysearcaschg b t capital management dba alpha capital management purchase share of schwab u largecap growth etf nysearcaschg quest wealth builder inc cut stock position in walmart inc nysewmt ifc advisor llc reduces position in vanguard midcap etf nysearcavo spdr gold share nysearcagld share purchased by acorn wealth advisor llc ballentine partner llc increase position in chevron corporation nysecvx acorn wealth advisor llc sell share of ishares core sp smallcap etf nysearcaijr acorn wealth advisor llc ha stock position in vanguard midcap etf nysearcavo acorn wealth advisor llc reduces stock position in ishares core sp smallcap etf nysearcaijr ballentine partner llc acquires share of walmart inc nysewmt history say these stock could be big winner in the second half history say these stock could be big winner in the second half alp advisor inc ha million stock position in kkr co inc nysekkr eli lilly and company nyselly share sold by wealthtrust asset management llc eli lilly and company nyselly is harmony asset management llcs th largest position the home depot inc nysehd share purchased by lane associate llc fulcrum equity management lower stock holding in eli lilly and company nyselly fulcrum equity management sell share of eli lilly and company nyselly servicenow inc nysenow share acquired by steelpeak wealth llc trump target mexico eu with tariff hartford bakery inc voluntarily recall hundred of loaf of artisanal bread sold in state cbs news reader view we can all reduce greenhouse gas shes great trump back bondi want top official to end conflict over epstein ishares core sp smallcap etf nysearcaijr share sold by forum private client group llc chevron corporation nysecvx share acquired by b t capital management dba alpha capital management forum private client group llc ha million position in vanguard midcap etf nysearcavo b t capital management dba alpha capital management increase stake in honeywell international inc nasdaqhon beirne wealth consulting service llc acquires share of vanguard smallcap etf nysearcavb ifc advisor llc boost holding in kkr co inc nysekkr ballentine partner llc grows holding in eli lilly and company nyselly young democrat have called for a rebrand theyre vying to replace the party old guard temperance in cabinetry climate change helped fuel heavy rain that led to devastating texas flood former pentagon insider could trump big beautiful bill finally unlock america longforgotten resource archaeolgists find largestever ceremony hall weapon hoard the democratic party is missing an opportunity to engage christian voter northwest capital management inc purchase share of ishares core sp midcap etf nysearcaijh rational advisor inc take position in mcdonalds corporation nysemcd superman smash box office expectation soaring towards million opening pam bondi fire doj staffer who worked on trump case amid chaos at agency nikulski financial inc acquires share of lowes company inc nyselow parkerhannifin corporation nyseph share sold by quest wealth builder inc family firm inc lower stock holding in schwab u smallcap etf nysearcascha family firm inc reduces stock holding in well fargo company nysewfc stillwater wealth management group invests in vanguard high dividend yield etf nysearcavym extrump lawyer dershowitz claim knowledge of epstein client list i know the name but im bound by confidentiality grant grossmendelsohn llc purchase share of vanguard ftse developed market etf nysearcavea riversedge advisor llc cut stake in vanguard ftse developed market etf nysearcavea piper sandler issue positive forecast for netflix nasdaqnflx stock price riversedge advisor llc ha holding in salesforce inc nysecrm american financial advisor llc ha million stake in ishares core sp etf nysearcaivv riversedge advisor llc increase stake in ishares core sp etf nysearcaivv start exploring cloud mining for free from the new winnermining app and get visible daily reward forum private client group llc trim position in vanguard growth etf nysearcavug fort sheridan advisor llc buy share of vanguard growth etf nysearcavug the big beautiful bill and mlp qualifying income acorn wealth advisor llc lower holding in chevron corporation nysecvx ballentine partner llc buy share of walmart inc nysewmt ballentine partner llc sell share of ishares core sp smallcap etf nysearcaijr lane associate llc sell share of eli lilly and company nyselly harmony asset management llc ha million holding in the home depot inc nysehd steelpeak wealth llc ha million stake in the progressive corporation nysepgr servicenow inc nysenow share acquired by steelpeak wealth llc trump threatens rosie odonnells citizenship she is a threat to humanity annual new london to new brighton antique car run to take place aug coyle financial counsel llc invests in qualcomm incorporated nasdaqqcom broadcom inc nasdaqavgo share sold by skyoak wealth llc forum private client group llc take position in elevance health inc nyseelv a major red flag for republican a trump policy threatens their future fbi director kash patel responds to controversy surrounding epstein file stillwater wealth management group grows position in amgen inc nasdaqamgn riversedge advisor llc grows stake in tesla inc nasdaqtsla fort sheridan advisor llc ha position in kla corporation nasdaqklac kathmere capital management llc grows holding in vanguard value etf nysearcavtv nycs broken election system need far more than these bandaid fix ballentine partner llc ha million position in abbott laboratory nyseabt abbott laboratory nyseabt share acquired by ifc advisor llc trump post support for embattled attorney general pam bondi ma private wealth take position in bristol myers squibb company nysebmy parkerhannifin corporation nyseph share sold by lbp am sa harmony asset management llc reduces stock position in chevron corporation nysecvx bonus editorial cartoon for july federal employee bracing after supreme court greenlights widespread layoff federal employee bracing after supreme court greenlights widespread layoff federal employee bracing after supreme court greenlights widespread layoff lawmaker visit alligator alcatraz but some wonder how much theyll get to see man convicted of meredith kerchers murder facing trial for sexual assault federal employee bracing after supreme court greenlights widespread layoff federal employee bracing after supreme court greenlights widespread layoff federal employee bracing after supreme court greenlights widespread layoff focused wealth management inc ha million stake in walmart inc nysewmt berbice capital management llc grows position in kkr co inc nysekkr coyle financial counsel llc raise holding in invesco qqq nasdaqqqq meet china man in lima who jetted over to u to collect train donated by biden admin amazon prime day delivers record sale and saving in expanded fourday shopping event how new tax legislation impact clean energy tax credit the dalai lama is planning his succession a the ultimate protest against china the u army m vulcan air defense system wa a beast in the vietnam war the us john f kennedy fordclass carrier may miss it delivery date comcast corporation nasdaqcmcsa share sold by sage rhino capital llc kesler norman wride llc sell share of comcast corporation nasdaqcmcsa exchange capital management inc sell share of servicenow inc nysenow fukoku mutual life insurance co sell share of duke energy corporation nyseduk cerity partner llc buy share of asml holding nv nasdaqasml mjp associate inc adv take position in elevance health inc nyseelv fidelis capital partner llc boost stock position in elevance health inc nyseelv reader view u must invest in our independence candidate view localgovernment focus would benefit school board stillwater wealth management group reduces position in unitedhealth group incorporated nyseunh martin capital advisor llp sell share of oracle corporation nyseorcl park square financial group llc decrease stock position in ishares core sp midcap etf nysearcaijh fortem financial group llc purchase share of blackstone inc nysebx pya waltman capital llc ha million stake in mcdonalds corporation nysemcd massachusetts police officer shot by colleague victim of campaign to criminalize her lawyer horrified by alligator alcatraz letter coyle financial counsel llc ha million stake in ishares core sp etf nysearcaivv vanguard high dividend yield etf nysearcavym stock holding decreased by auour investment llc ifc advisor llc increase position in ishares russell etf nysearcaiwm forum private client group llc purchase new stake in cummins inc nysecmi fortem financial group llc grows holding in tesla inc nasdaqtsla vanguard ftse developed market etf nysearcavea share purchased by beirne wealth consulting service llc schear investment adviser llc buy share of tmobile u inc nasdaqtmus jrmc recognized for infection control rate wall street pro drop bold price target on circle stock bitcoin hit new alltime high above k a trader eye week uptrend cointelegraph cardinal strategic wealth guidance cut position in alphabet inc nasdaqgoog bradley co private wealth management llc reduces position in costco wholesale corporation nasdaqcost pointe capital management llc grows holding in the walt disney company nysedis westmount partner llc sell share of amgen inc nasdaqamgn westmount partner llc sell share of starbucks corporation nasdaqsbux westmount partner llc trim holding in lockheed martin corporation nyselmt q asset management buy share of williams company inc the nysewmb westmount partner llc trim holding in lockheed martin corporation nyselmt westmount partner llc trim stock position in amgen inc nasdaqamgn zullo investment group inc lower stock position in alphabet inc nasdaqgoog trunorth capital management llc acquires share of vanguard sp etf nysearcavoo pointe capital management llc boost holding in linde plc nasdaqlin ishares core u aggregate bond etf nysearcaagg share acquired by pointe capital management llc nextera energy inc nysenee share sold by pointe capital management llc bristol myers squibb company nysebmy stock holding lifted by prudent man advisor llc mqs management llc buy new position in nextera energy inc nysenee prudent man advisor llc acquires new position in blackrock nyseblk zullo investment group inc buy share of eli lilly and company nyselly zullo investment group inc acquires share of eli lilly and company nyselly zullo investment group inc cut stake in m company nysemmm prudent man advisor llc make new million investment in blackrock nyseblk mqs management llc take position in nextera energy inc nysenee ai financial service llc boost holding in eli lilly and company nyselly u tomato price could jump a soon a monday xrp break out near gain yet blockdags coin unlock chance at steal market focus top altcoins still lag while bitcoin stay strong promising outdoor stock to add to your watchlist july th kathmere capital management llc sell share of kimberlyclark co nysekmb citigroup inc nysec share purchased by ballentine partner llc cigna group nyseci share bought by ballentine partner llc ballentine partner llc purchase share of the sherwinwilliams company nyseshw arizona state retirement system purchase share of kimberlyclark co nysekmb bankplus trust department grows holding in ishares core sp smallcap etf nysearcaijr berkeley inc ha million holding in schwab u largecap etf nysearcaschx arizona state retirement system increase stake in kimberlyclark co nysekmb fdx advisor inc invests in medtronic plc nysemdt how trump latest tariff threat risk deeper damage to europe economy fort sheridan advisor llc increase stock position in cocacola company the nyseko fortem financial group llc sell share of conocophillips nysecop blackstone inc nysebx share bought by louisiana state employee retirement system eaton corporation plc nyseetn share sold by stephen inc ar taiwan semiconductor manufacturing company ltd nysetsm share sold by fulton breakefield broenniman llc why broadcoms avgo ai momentum ha goldman sachs backing the stock on gps nvidia ceo on the overwhelmingly positive effect of ai isthmus partner llc sell share of thermo fisher scientific inc nysetmo whitener capit</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>axecap investment llc sell share of apple inc nasdaqaapl fifth third bancorp sell share of apple inc nasdaqaapl sagace wealth management llc sell share of microsoft corporation nasdaqmsft microsoft corporation nasdaqmsft stake lowered by tran capital management lp define financial llc buy share of microsoft corporation nasdaqmsft sapient capital llc sell share of microsoft corporation nasdaqmsft teacher retirement system of texas sell share of safety insurance group inc nasdaqsaft teacher retirement system of texas sell share of organon co nyseogn teacher retirement system of texas cut stock holding in artisan partner asset management inc nyseapam teacher retirement system of texas buy new share in a o smith corporation nyseaos rev group inc nyserevg position trimmed by teacher retirement system of texas share in lamb weston nyselw acquired by teacher retirement system of texas bridgebio pharma inc nasdaqbbio share sold by teacher retirement system of texas two west capital advisor llc trim position in apple inc nasdaqaapl teacher retirement system of texas take million position in community health system inc nysecyh teacher retirement system of texas ha million position in portland general electric company nysepor teacher retirement system of texas buy share of ugi corporation nyseugi teacher retirement system of texas ha million stake in ziff davis inc nasdaqzd teacher retirement system of texas purchase new stake in the campbell company nasdaqcpb asian heat squeeze lng flow to europe borgwarner inc nysebwa share sold by cambridge investment research advisor inc teacher retirement system of texas ha million stake in madrigal pharmaceutical inc nasdaqmdgl exclusive interview the future belongs to nocodes with deep ai integration abhinav girdhar ceo founder appy pie european trade minister meet to forge strategy after trump surprise tariff european trade minister meet to forge strategy after trump surprise tariff european trade minister meet to forge strategy after trump surprise tariff relx nyserelx rating lowered to hold at wall street zen southside bancshares nysesbsi rating lowered to sell at wall street zen wall street zen downgrade vista energy nysevist to sell bank of america cut primo brand nyseprmb price target to silgan nyseslgn price target raised to stifel financial nysesf price target raised to ubiquitis ui buy rating reiterated at bw financial wall street zen upgrade rafael nyserfl to hold charles schwab nyseschw price target raised to sea nysese stock rating lowered by wall street zen sealed air nysesee price target raised to wall street zen upgrade te connectivity nysetel to buy telus digital nysetixt stock rating upgraded by wall street zen sealed air nysesee price target raised to telephone and data system nysetds stock rating upgraded by wall street zen synovus financial nysesnv price target raised to truist financial cut sonoco product nyseson price target to att nyset price target raised to wec energy group nysewec rating lowered to sell at wall street zen exxon mobil nysexom price target raised to at scotiabank truist financial raise webster financial nysewbs price target to top ai stock to buy this week the place report surge in company relocation driving demand for flexible office space in dubai and riyadh rockfire resource lonrock stock price up still a buy rockfire resource lonrock trading up should you buy new zealand energy cvenz trading down here what happened argentina lithium energy cvelit share down should you sell silver spruce resource cvesse share down here what happened silver spruce resource cvesse trading down time to sell new zealand energy cvenz trading down should you sell argentina lithium energy cvelit stock price down here why geomega resource cvegma stock price up whats next geomega resource cvegma trading higher still a buy geomega resource cvegma stock price up here what happened geomega resource cvegma share up time to buy geomega resource cvegma trading higher should you buy form eptriricardo plc advanced drainage system inc nysewms share bought by teacher retirement system of texas teacher retirement system of texas purchase share of lxp industrial trust nyselxp teacher retirement system of texas purchase new stake in exact science corporation nasdaqexas teacher retirement system of texas raise holding in advanced drainage system inc nysewms amentum holding inc nyseamtm share sold by teacher retirement system of texas teacher retirement system of texas boost stock position in sprinklr inc nysecxm teacher retirement system of texas acquires share of lxp industrial trust nyselxp ola electric share rise to r a market reacts to q update aktietilbagekbsprogram uge share buyback programme week bunge global earnings preview what to expect robinhood eu wont retaliate to trump tariff countermeasure on hold until august avis budget group car v it peer head to head analysis contrasting cps technology cpsh the competition head to head analysis better home finance betr and it peer analyzing greif bros gefb the competition head to head review better home finance betr the competition cps technology cpsh it competitor head to head survey avis budget group car it peer financial comparison how doe nvidias reaching trillion in market cap impact the sp nasdaq and dow jones marc benioff dismisses ai panic say whitecollar workforce wont be wiped out market week ahead strong bank earnings sticky inflation could jolt summer lull china exporter rush to beat trump next big tariff deadline bp nysebp stock price expected to rise scotiabank analyst say ladenburg thalmsh sh initiate coverage on kala bio nasdaqkala franklin resource nyseben given new price target at well fargo company kkrs quarterly earnings preview what you need to know wall street zen upgrade wintrust financial nasdaqwtfc to hold botswana diamond lonbod trading higher still a buy botswana diamond lonbod share up here what happened botswana diamond lonbod trading higher whats next majestic ideal holding refiled mjid plan to raise million in july th ipo tower resource cvetwr trading up here what happened tower resource cvetwr trading up here why botswana diamond lonbod share up here what happened tower resource cvetwr trading up time to buy trump envoy meet with ukraine zelenskyy a u pledge more patriot missile for kyiv trump threatens russia with tariff and boost u weapon for ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump threatens russia with tariff and boost u weapon for ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump threatens russia with tariff and boost u weapon for ukraine trump threatens russia with tariff if war on ukraine isnt resolved within day trump envoy meet with ukraine zelenskyy a u weighs next step on russia invasion trump envoy meet with ukraine zelenskyy a u weighs next step on russia invasion trump threatens russia with tariff if war on ukraine isnt resolved within day trump threatens russia with tariff if war on ukraine isnt resolved within day spin cycle theyre throwing spaghetti at the wall bbc dump masterchef host over sex misconduct report eu want no trade war a trade minister mull new u tariff threat new review ordered into nh murdersuicide case amid criticism of shooter bail morning brief the epstein firestorm ice raid riot california v trump aquestive therapeutic inc nasdaqaqst given consensus recommendation of buy by analyst astera lab inc nasdaqalab receives consensus target price from analyst mplx lp nysemplx receives consensus recommendation of moderate buy from analyst brokerage set altria group inc nysemo price target at kornit digital ltd nasdaqkrnt receives average price target from brokerage exwhite house aide reveals why trump panicking right now brokerage set triple flag precious metal corp nysetfpm price target at lionsgate studio corp nyselion receives average price target from brokerage agnico eagle mine limited tseaem receives c consensus pt from analyst democrat already lining up for presidential race in early voting state these state are america best for quality of life in letter for monday july a bitcoin rush past k whats next for ether xrp dogecoin elkem asa elkef to release earnings on tuesday america movil amx expected to announce quarterly earnings on tuesday nikki wegner understanding big beautiful bill impact on long term care in nd why not hold gun manufacturer accountable for mass shooting boston herald will democrat reembrace musk now that he feuding with trump guest view bipartisan push to strengthen pa disability care system must succeed house debate pentagon spending crypto a rescission head to senate hancock whitney hwc projected to post quarterly earnings on tuesday omnicom group omc expected to announce quarterly earnings on tuesday what is bastille day what to know about the french holiday and why it is celebrated insider buying schroders plc lonsdr insider purchase share of stock cv group plc loncvsg insider buy in stock crest nicholson holding plc loncrst insider acquires in stock nextdecade nasdaqnext hit new month high on analyst upgrade trump mark anniversary of assassination attempt at the fifa club world cup final historic grand canyon lodge destroyed a wildfire force evacuation in northern arizona today in history july the storming of the bastille invisible rural homelessness grows in the shadow of a maine tourism mecca education notebook bond result child nutrition change and federal consultation orrington trash plant at risk of permanent closure if judge freeze funding susan collins start lining up money for maine that may not actually arrive hungary oldest library is fighting to save book from a beetle infestation trump to meet nato secretarygeneral a plan take shape for ukraine weapon sale chris christie say trump not pam bondi pulled the plug on epstein memo when you start the fire sometimes you cant put it out iyo sue former engineer after io founder tang yew tan admits to receiving trade secret from him poll show support for immigration is rising in u amid president trump crackdown trial will be very difficult for sen nicole mitchell to win minneapolis attorney say who got next democrat already lining up for presidential race in early voting state who got next democrat already lining up for presidential race in early voting state who got next democrat already lining up for presidential race in early voting state a nicotine pouch popularity soar theyre also responsible for more poisoning in young kid study find the biden doj tried to imprison a trump supporter over meme now he fighting back gop infighting over trump doge cut to take center stage a deadline loom how much trump big beautiful bill could raise electricity cost in every u state over the next year claudia istel ken barnes budget ayotte signed is designed to perpetuate inequality letter to the editor response to a response william hinkle eversource customer deserve more stable electric bill letter to the editor resident deserve more information about data center a look at a new poll showing support for immigration is rising in the u bitcoin top for the first time peter schiff give trump tariff threat on mexico eu a reality check america relies on deficit to make up for excess debt and consumption trump say he spoke to bongino amid report of infighting over epstein file trump reflects on surviving pennsylvania rally shooting year on god alone saved me one year after trump assassination attempt change at secret service but question remain jim chalmers insists labor can meet target of m new home despite department warning trump to meet nato secretary general a plan take shape for ukraine weapon sale tragedy in fall river read the full press release on sunday deadly fire amd warns of new transient scheduler attack impacting a wide range of cpu cambodia khmer rouge torture site added to unesco heritage list cant contain debris then forget about starbase dont allow hidden tax on energy producer hydrogen is a pipe dream dont be fooled the epstein list still remain relevant immigrant in overcapacity ice detention say theyre hungry raise food quality concern miranda devine shocking new poll reveals majority of deluded dems still believe the russia collusion hoax wa real live update trump threatens russia with tariff if war on ukraine isnt resolved dhs secretary kristi noem say trump want fema remade not dismantled homicide investigation underway after stabbing in southeast portland trump to announce aggressive ukraine weapon plan houston astros select lsus ethan frey in the third round of the mlb draft here when trump say american spirit triumph over force of evil on anniversary of butler assassination attempt trump brazil tariff imposed because they jail insurrectionist say economist your next coffee come with an insurrection infusion fee christie say trump benefited from epstein conspiracy theory boston red sox select lsus anthony eyanson in third round of mlb draft here when biden say he had to use autopen because he simply granted too many pardon company cast party biden defends frequent autopen use at end of term alex jose padilla say trump is to blame for violence against ice carried out by dems foot soldier fulltime mayor is unnecessary appendage an lsu baseball signee ha been picked by the tampa bay ray in the mlb draft here who portland police seize pound of cannabis in traffic stop florida financial advisor llc grows position in spdr sp small cap value etf nysearcaslyv share in united therapeutic corporation nasdaquthr bought by aurora investment counsel aurora investment counsel take million position in globe life inc nysegl florida financial advisor llc acquires share of spdr sp mid cap growth etf nysearcamdyg bhk investment advisor llc ha stake in eli lilly and company nyselly bleakley financial group llc boost stock position in bank of america corporation nysebac bleakley financial group llc sell share of ishares silver trust nysearcaslv rice hall james associate llc boost holding in green brick partner inc nasdaqgrbk jpmorgan betabuilders u equity etf batsbbus is florida financial advisor llcs rd largest position securian asset management inc sell share of servicenow inc nysenow florida financial advisor llc acquires new holding in ishares core high dividend etf nysearcahdv bleakley financial group llc sell share of ishares year treasury bond etf nasdaqshy securian asset management inc ha million stock holding in merck co inc nysemrk florida financial advisor llc buy share of ishares core high dividend etf nysearcahdv focused investor llc decrease stock holding in the home depot inc nysehd the pnc financial service group inc nysepnc share sold by bhk investment advisor llc rice hall james associate llc sell share of griffon corporation nysegff florida financial advisor llc sell share of fidelity msci information technology index etf nysearcaftec bleakley financial group llc buy share of vanguard total world stock etf nysearcavt charity fraud alert how to donate safely to texas flood victim charity fraud alert how to donate safely to texas flood victim tight oil market shrug off supply surge heartland advisor value plus fund q investor letter boy girl club program threatened by trump grant freeze serve thousand of family sun pharma announces launch of leqselvitm deuruxolitinib in the united state for the treatment of severe alopecia areata texas roadhouse inc nasdaqtxrh given consensus recommendation of moderate buy by analyst mqs management llc make new investment in rli corp nyserli stephen investment management group llc buy share of autodesk inc nasdaqadsk lri investment llc acquires share of newmont corporation nysenem lri investment llc sell share of teledyne technology incorporated nysetdy lri investment llc take position in spdr portfolio sp growth etf nysearcaspyg mqs management llc invests in centene corporation nysecnc eaton corporation plc nyseetn stock position lowered by lri investment llc stephen investment management group llc increase position in roper technology inc nyserop mtm investment management llc ha holding in ishares russell midcap etf nysearcaiwr lri investment llc acquires share of union pacific corporation nyseunp lri investment llc sell share of ameriprise financial inc nyseamp mtm investment management llc sell share of kinder morgan inc nysekmi mtm investment management llc buy share of vanguard sp etf nysearcavoo stephen inc ar boost stock position in hp inc nysehpq church dwight co inc nysechd share acquired by key financial inc lri investment llc reduces holding in kenvue inc nysekvue lri investment llc reduces position in ferrari nv nyserace lri investment llc buy share of spdr portfolio sp growth etf nysearcaspyg prudent man advisor llc sell share of vanguard intermediateterm bond etf nysearcabiv cme group inc nasdaqcme share purchased by key financial inc eaton corporation plc nyseetn share sold by lri investment llc mqs management llc buy new position in astrazeneca plc nasdaqazn kinder morgan inc nysekmi is mtm investment management llcs th largest position analyst set regeneron pharmaceutical inc nasdaqregn pt at catalyst financial partner llc grows stock position in linde plc nasdaqlin evergreen private wealth llc boost stock position in zoetis inc nysezts schwab u largecap etf nysearcaschx share sold by slow capital inc catalyst financial partner llc buy share of att inc nyset catalyst financial partner llc raise position in lowes company inc nyselow shore capital reiterates house stock rating for touchstone exploration lontxp cohen capital management inc sell share of ishares europe etf nysearcaiev vanguard ftse allworld exus etf nysearcaveu share sold by slow capital inc signaturefd llc reduces holding in rollins inc nyserol braime group lonbmt announces quarterly earnings result catalyst financial partner llc ha stock holding in sp global inc nysespgi beeks financial cloud group lonbks receives buy rating from canaccord genuity group catalyst financial partner llc increase holding in att inc nyset slow capital inc sell share of jpmorgan ultrashort municipal etf batsjmst catalyst financial partner llc ha stock position in intuitive surgical inc nasdaqisrg creightons loncrl trading higher still a buy dewhurst group londwha announces earnings result signaturefd llc boost stake in cisco system inc nasdaqcsco beeks financial cloud group lonbks receives buy rating from canaccord genuity group dunelm group londnlm receives buy rating from deutsche bank aktiengesellschaft catalyst financial partner llc ha position in capital group global growth equity etf nysearcacggo ariana resource lonaau trading up whats next simec atlantis energy lonsae trading down time to sell creightons loncrl trading higher still a buy what make uber technology uber a great business to invest in nearly half of u child are without summer learning program a cost rise study say world chess lonchss stock price down time to sell catalyst financial partner llc ha holding in the tjx company inc nysetjx a tariff on europe would effectively knock out transatlantic trade say eu trade chief promising cybersecurity stock to keep an eye on july th stratos wealth partner ltd sell share of universal display corporation nasdaqoled ge vernova inc nysegev share sold by mutual of america capital management llc bleakley financial group llc acquires share of marsh mclennan company inc nysemmc owen corning inc nyseoc given average recommendation of moderate buy by brokerage schechter investment advisor llc sell share of morgan stanley nysems corrado advisor llc raise stock position in vici property inc nysevici new york state common retirement fund trim position in ansys inc nasdaqanss arizona state retirement system sell share of raymond james financial inc nyserjf new york state common retirement fund sell share of mondelez international inc nasdaqmdlz diversify wealth management llc raise stock position in appfolio inc nasdaqappf emerald adviser llc decrease stock position in lharris technology inc nyselhx stephen inc ar boost stock position in automatic data processing inc nasdaqadp m mmm hold c rating reaffirmed at weiss rating weatherly asset management l p take position in chubb limited nysecb emerald adviser llc ha stock position in msci inc nysemsci bleakley financial group llc acquires share of marsh mclennan company inc nysemmc arizona state retirement system reduces stock position in ansys inc nasdaqanss fortinet inc nasdaqftnt share sold by new york state common retirement fund new york state common retirement fund sell share of cognizant technology solution corporation nasdaqctsh key financial inc increase stock position in kinsale capital group inc nyseknsl focused investor llc sell share of the home depot inc nysehd aurora investment counsel take position in elf beauty nyseelf bleakley financial group llc purchase share of vanguard total world stock etf nysearcavt trump adviser say this is how the president could certainly fire powell regeneron pharmaceutical inc nasdaqregn given average recommendation of moderate buy by brokerage mtm investment management llc acquires new position in american electric power company inc nasdaqaep lri investment llc trim stock position in kenvue inc nysekvue key financial inc purchase share of kla corporation nasdaqklac alp advisor inc purchase share of global payment inc nysegpn lri investment llc reduces stock position in ferrari nv nyserace cme group inc nasdaqcme share purchased by key financial inc mtm investment management llc ha position in hershey company the nysehsy signaturefd llc raise stock position in ishares msci usa value factor etf batsvlue slow capital inc sell share of jpmorgan ultrashort municipal etf batsjmst catalyst financial partner llc boost stock position in intuitive surgical inc nasdaqisrg pulsar group lonpuls post quarterly earnings result evergreen private wealth llc ha million position in vaneck long muni etf batsmln world chess lonchss stock price down time to sell rockfire resource lonrock trading up still a buy catalyst financial partner llc ha holding in capital group global growth equity etf nysearcacggo catalyst financial partner llc purchase share of deere company nysede dunelm group londnlm receives buy rating from deutsche bank aktiengesellschaft a tariff on europe would effectively knock out transatlantic trade say eu trade chief kathmere capital management llc cut stake in ge vernova inc nysegev arthur j gallagher co nyseajg share purchased by new york state common retirement fund analyst set wex inc nysewex target price at corrado advisor llc sell share of corning incorporated nyseglw dominion energy inc nysed share acquired by new york state common retirement fund kathmere capital management llc trim holding in dell technology inc nysedell new york state common retirement fund sell share of nike inc nysenke new york state common retirement fund sell share of marvell technology inc nasdaqmrvl kinsale capital group inc nyseknsl given consensus rating of hold by brokerage emerald adviser llc sell share of xpo inc nysexpo emerald adviser llc ha stake in burlington store inc nyseburl invmun incom oia to go exdividend on july th doubleline yield opportunity fund plan monthly dividend of nysedly inv vk invt ny announces monthly dividend of nysevtn gladstone land co announces monthly dividend of nasdaqlandp regency center co declares quarterly dividend of nasdaqregcp thor exploration lonthx given buy rating at canaccord genuity group berenberg bank issue positive forecast for volex lonvlx stock price gladstone commercial co nasdaqgoodn plan monthly dividend trump give russia a day deadline on ukraine signaturefd llc ha million stock position in ishares msci acwi ex u etf nasdaqacwx signaturefd llc buy share of toyota motor corporation nysetm cheems cheemspet cheems price hit on exchange reviewing cyclo therapeutic nasdaqcyth sorrento therapeutic nasdaqsrne financial contrast cemtrex nasdaqcetx versus omron otcmktsomrny empower self reported market capitalization top thousand mpwr animecoin anime hit day volume of million dignity gold digau trading higher over last day share in howmet aerospace inc nysehwm bought by florida financial advisor llc florida financial advisor llc sell share of unitedhealth group incorporated nyseunh aercap holding nv nyseaer stake cut by check capital management inc ca headtohead contrast insight enterprise nasdaqnsit v flowerscom nasdaqflws slow capital inc sell share of ishares global consumer staple etf nysearcakxi fidelity national information service inc nysefis position boosted by isthmus partner llc gould asset management llc ca reduces stock holding in ishares select dividend etf nasdaqdvy abbvie inc nyseabbv share sold by florida financial advisor llc slow capital inc cut stake in ishares global comm service etf nysearcaixp top renewable energy stock to research july th gould asset management llc ca lower position in ishares msci acwi low carbon target etf nysearcacrbn alta foundation donates k toward texas flood relief trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine rice hall james associate llc lower stock position in lantheus holding inc nasdaqlnth aurora investment counsel buy share of euronet worldwide inc nasdaqeeft slow capital inc raise stock position in cadence design system inc nasdaqcdns moody corporation nysemco share purchased by slow capital inc corteva inc nysectva share sold by lri investment llc top fintech stock to keep an eye on july th first bancorp nysefbp share bought by edgestream partner lp revolution medicine inc nasdaqrvmd share acquired by edgestream partner lp rithm capital corp nyseritm share bought by edgestream partner lp edgestream partner lp raise holding in ncino inc nasdaqncno antisemitic post appear on elmos x account after hack bleakley financial group llc purchase share of schwab u smallcap etf nysearcascha bleakley financial group llc boost stock holding in dimensional u small cap etf nysearcadfas edgestream partner lp acquires share of simpson manufacturing company inc nysessd edgestream partner lp ha million stake in nmi holding inc nasdaqnmih edgestream partner lp make new investment in exlservice holding inc nasdaqexls hartford schroders taxaware bond etf nysearcahtab share acquired by leelyn smith llc edgestream partner lp increase stock holding in cno financial group inc nysecno invesco sp high dividend low volatility etf nysearcasphd share sold by leelyn smith llc edgestream partner lp buy new position in bentley system incorporated nasdaqbsy fortress financial solution llc decrease holding in avantis emerging market equity etf nysearcaavem share in ishares future ai tech etf nysearcaarty acquired by mitchell mcleod pugh williams inc eu trade minister meet in brussels after u announces percent tariff private capital advisor inc take position in relay therapeutic inc nasdaqrlay mutual of america capital management llc ha million holding in ametek inc nyseame mitchell mcleod pugh williams inc purchase share of becton dickinson and company nysebdx</t>
+          <t>axecap investment llc sell share of apple inc nasdaqaapl fifth third bancorp sell share of apple inc nasdaqaapl sagace wealth management llc sell share of microsoft corporation nasdaqmsft microsoft corporation nasdaqmsft stake lowered by tran capital management lp define financial llc buy share of microsoft corporation nasdaqmsft sapient capital llc sell share of microsoft corporation nasdaqmsft teacher retirement system of texas sell share of safety insurance group inc nasdaqsaft teacher retirement system of texas sell share of organon co nyseogn teacher retirement system of texas cut stock holding in artisan partner asset management inc nyseapam teacher retirement system of texas buy new share in a o smith corporation nyseaos rev group inc nyserevg position trimmed by teacher retirement system of texas share in lamb weston nyselw acquired by teacher retirement system of texas bridgebio pharma inc nasdaqbbio share sold by teacher retirement system of texas two west capital advisor llc trim position in apple inc nasdaqaapl teacher retirement system of texas take million position in community health system inc nysecyh teacher retirement system of texas ha million position in portland general electric company nysepor teacher retirement system of texas buy share of ugi corporation nyseugi teacher retirement system of texas ha million stake in ziff davis inc nasdaqzd teacher retirement system of texas purchase new stake in the campbell company nasdaqcpb asian heat squeeze lng flow to europe borgwarner inc nysebwa share sold by cambridge investment research advisor inc teacher retirement system of texas ha million stake in madrigal pharmaceutical inc nasdaqmdgl exclusive interview the future belongs to nocodes with deep ai integration abhinav girdhar ceo founder appy pie european trade minister meet to forge strategy after trump surprise tariff european trade minister meet to forge strategy after trump surprise tariff european trade minister meet to forge strategy after trump surprise tariff relx nyserelx rating lowered to hold at wall street zen southside bancshares nysesbsi rating lowered to sell at wall street zen wall street zen downgrade vista energy nysevist to sell bank of america cut primo brand nyseprmb price target to silgan nyseslgn price target raised to stifel financial nysesf price target raised to ubiquitis ui buy rating reiterated at bw financial wall street zen upgrade rafael nyserfl to hold charles schwab nyseschw price target raised to sea nysese stock rating lowered by wall street zen sealed air nysesee price target raised to wall street zen upgrade te connectivity nysetel to buy telus digital nysetixt stock rating upgraded by wall street zen sealed air nysesee price target raised to telephone and data system nysetds stock rating upgraded by wall street zen synovus financial nysesnv price target raised to truist financial cut sonoco product nyseson price target to att nyset price target raised to wec energy group nysewec rating lowered to sell at wall street zen exxon mobil nysexom price target raised to at scotiabank truist financial raise webster financial nysewbs price target to top ai stock to buy this week the place report surge in company relocation driving demand for flexible office space in dubai and riyadh rockfire resource lonrock stock price up still a buy rockfire resource lonrock trading up should you buy new zealand energy cvenz trading down here what happened argentina lithium energy cvelit share down should you sell silver spruce resource cvesse share down here what happened silver spruce resource cvesse trading down time to sell new zealand energy cvenz trading down should you sell argentina lithium energy cvelit stock price down here why geomega resource cvegma stock price up whats next geomega resource cvegma trading higher still a buy geomega resource cvegma stock price up here what happened geomega resource cvegma share up time to buy geomega resource cvegma trading higher should you buy form eptriricardo plc advanced drainage system inc nysewms share bought by teacher retirement system of texas teacher retirement system of texas purchase share of lxp industrial trust nyselxp teacher retirement system of texas purchase new stake in exact science corporation nasdaqexas teacher retirement system of texas raise holding in advanced drainage system inc nysewms amentum holding inc nyseamtm share sold by teacher retirement system of texas teacher retirement system of texas boost stock position in sprinklr inc nysecxm teacher retirement system of texas acquires share of lxp industrial trust nyselxp ola electric share rise to r a market reacts to q update aktietilbagekbsprogram uge share buyback programme week bunge global earnings preview what to expect robinhood eu wont retaliate to trump tariff countermeasure on hold until august avis budget group car v it peer head to head analysis contrasting cps technology cpsh the competition head to head analysis better home finance betr and it peer analyzing greif bros gefb the competition head to head review better home finance betr the competition cps technology cpsh it competitor head to head survey avis budget group car it peer financial comparison how doe nvidias reaching trillion in market cap impact the sp nasdaq and dow jones marc benioff dismisses ai panic say whitecollar workforce wont be wiped out market week ahead strong bank earnings sticky inflation could jolt summer lull china exporter rush to beat trump next big tariff deadline bp nysebp stock price expected to rise scotiabank analyst say ladenburg thalmsh sh initiate coverage on kala bio nasdaqkala franklin resource nyseben given new price target at well fargo company kkrs quarterly earnings preview what you need to know wall street zen upgrade wintrust financial nasdaqwtfc to hold botswana diamond lonbod trading higher still a buy botswana diamond lonbod share up here what happened botswana diamond lonbod trading higher whats next majestic ideal holding refiled mjid plan to raise million in july th ipo tower resource cvetwr trading up here what happened tower resource cvetwr trading up here why botswana diamond lonbod share up here what happened tower resource cvetwr trading up time to buy trump envoy meet with ukraine zelenskyy a u pledge more patriot missile for kyiv trump threatens russia with tariff and boost u weapon for ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump threatens russia with tariff and boost u weapon for ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump threatens russia with tariff and boost u weapon for ukraine trump threatens russia with tariff if war on ukraine isnt resolved within day trump envoy meet with ukraine zelenskyy a u weighs next step on russia invasion trump envoy meet with ukraine zelenskyy a u weighs next step on russia invasion trump threatens russia with tariff if war on ukraine isnt resolved within day trump threatens russia with tariff if war on ukraine isnt resolved within day spin cycle theyre throwing spaghetti at the wall bbc dump masterchef host over sex misconduct report eu want no trade war a trade minister mull new u tariff threat new review ordered into nh murdersuicide case amid criticism of shooter bail morning brief the epstein firestorm ice raid riot california v trump aquestive therapeutic inc nasdaqaqst given consensus recommendation of buy by analyst astera lab inc nasdaqalab receives consensus target price from analyst mplx lp nysemplx receives consensus recommendation of moderate buy from analyst brokerage set altria group inc nysemo price target at kornit digital ltd nasdaqkrnt receives average price target from brokerage exwhite house aide reveals why trump panicking right now brokerage set triple flag precious metal corp nysetfpm price target at lionsgate studio corp nyselion receives average price target from brokerage agnico eagle mine limited tseaem receives c consensus pt from analyst democrat already lining up for presidential race in early voting state these state are america best for quality of life in letter for monday july a bitcoin rush past k whats next for ether xrp dogecoin elkem asa elkef to release earnings on tuesday america movil amx expected to announce quarterly earnings on tuesday nikki wegner understanding big beautiful bill impact on long term care in nd why not hold gun manufacturer accountable for mass shooting boston herald will democrat reembrace musk now that he feuding with trump guest view bipartisan push to strengthen pa disability care system must succeed house debate pentagon spending crypto a rescission head to senate hancock whitney hwc projected to post quarterly earnings on tuesday omnicom group omc expected to announce quarterly earnings on tuesday what is bastille day what to know about the french holiday and why it is celebrated insider buying schroders plc lonsdr insider purchase share of stock cv group plc loncvsg insider buy in stock crest nicholson holding plc loncrst insider acquires in stock nextdecade nasdaqnext hit new month high on analyst upgrade trump mark anniversary of assassination attempt at the fifa club world cup final historic grand canyon lodge destroyed a wildfire force evacuation in northern arizona today in history july the storming of the bastille invisible rural homelessness grows in the shadow of a maine tourism mecca education notebook bond result child nutrition change and federal consultation orrington trash plant at risk of permanent closure if judge freeze funding susan collins start lining up money for maine that may not actually arrive hungary oldest library is fighting to save book from a beetle infestation trump to meet nato secretarygeneral a plan take shape for ukraine weapon sale chris christie say trump not pam bondi pulled the plug on epstein memo when you start the fire sometimes you cant put it out iyo sue former engineer after io founder tang yew tan admits to receiving trade secret from him poll show support for immigration is rising in u amid president trump crackdown trial will be very difficult for sen nicole mitchell to win minneapolis attorney say who got next democrat already lining up for presidential race in early voting state who got next democrat already lining up for presidential race in early voting state who got next democrat already lining up for presidential race in early voting state a nicotine pouch popularity soar theyre also responsible for more poisoning in young kid study find the biden doj tried to imprison a trump supporter over meme now he fighting back gop infighting over trump doge cut to take center stage a deadline loom how much trump big beautiful bill could raise electricity cost in every u state over the next year claudia istel ken barnes budget ayotte signed is designed to perpetuate inequality letter to the editor response to a response william hinkle eversource customer deserve more stable electric bill letter to the editor resident deserve more information about data center a look at a new poll showing support for immigration is rising in the u bitcoin top for the first time peter schiff give trump tariff threat on mexico eu a reality check america relies on deficit to make up for excess debt and consumption trump say he spoke to bongino amid report of infighting over epstein file trump reflects on surviving pennsylvania rally shooting year on god alone saved me one year after trump assassination attempt change at secret service but question remain jim chalmers insists labor can meet target of m new home despite department warning trump to meet nato secretary general a plan take shape for ukraine weapon sale tragedy in fall river read the full press release on sunday deadly fire amd warns of new transient scheduler attack impacting a wide range of cpu cambodia khmer rouge torture site added to unesco heritage list cant contain debris then forget about starbase dont allow hidden tax on energy producer hydrogen is a pipe dream dont be fooled the epstein list still remain relevant immigrant in overcapacity ice detention say theyre hungry raise food quality concern miranda devine shocking new poll reveals majority of deluded dems still believe the russia collusion hoax wa real live update trump threatens russia with tariff if war on ukraine isnt resolved dhs secretary kristi noem say trump want fema remade not dismantled homicide investigation underway after stabbing in southeast portland trump to announce aggressive ukraine weapon plan houston astros select lsus ethan frey in the third round of the mlb draft here when trump say american spirit triumph over force of evil on anniversary of butler assassination attempt trump brazil tariff imposed because they jail insurrectionist say economist your next coffee come with an insurrection infusion fee christie say trump benefited from epstein conspiracy theory boston red sox select lsus anthony eyanson in third round of mlb draft here when biden say he had to use autopen because he simply granted too many pardon company cast party biden defends frequent autopen use at end of term alex jose padilla say trump is to blame for violence against ice carried out by dems foot soldier fulltime mayor is unnecessary appendage an lsu baseball signee ha been picked by the tampa bay ray in the mlb draft here who portland police seize pound of cannabis in traffic stop florida financial advisor llc grows position in spdr sp small cap value etf nysearcaslyv share in united therapeutic corporation nasdaquthr bought by aurora investment counsel aurora investment counsel take million position in globe life inc nysegl florida financial advisor llc acquires share of spdr sp mid cap growth etf nysearcamdyg bhk investment advisor llc ha stake in eli lilly and company nyselly bleakley financial group llc boost stock position in bank of america corporation nysebac bleakley financial group llc sell share of ishares silver trust nysearcaslv rice hall james associate llc boost holding in green brick partner inc nasdaqgrbk jpmorgan betabuilders u equity etf batsbbus is florida financial advisor llcs rd largest position securian asset management inc sell share of servicenow inc nysenow florida financial advisor llc acquires new holding in ishares core high dividend etf nysearcahdv bleakley financial group llc sell share of ishares year treasury bond etf nasdaqshy securian asset management inc ha million stock holding in merck co inc nysemrk florida financial advisor llc buy share of ishares core high dividend etf nysearcahdv focused investor llc decrease stock holding in the home depot inc nysehd the pnc financial service group inc nysepnc share sold by bhk investment advisor llc rice hall james associate llc sell share of griffon corporation nysegff florida financial advisor llc sell share of fidelity msci information technology index etf nysearcaftec bleakley financial group llc buy share of vanguard total world stock etf nysearcavt charity fraud alert how to donate safely to texas flood victim charity fraud alert how to donate safely to texas flood victim tight oil market shrug off supply surge heartland advisor value plus fund q investor letter boy girl club program threatened by trump grant freeze serve thousand of family sun pharma announces launch of leqselvitm deuruxolitinib in the united state for the treatment of severe alopecia areata texas roadhouse inc nasdaqtxrh given consensus recommendation of moderate buy by analyst mqs management llc make new investment in rli corp nyserli stephen investment management group llc buy share of autodesk inc nasdaqadsk lri investment llc acquires share of newmont corporation nysenem lri investment llc sell share of teledyne technology incorporated nysetdy lri investment llc take position in spdr portfolio sp growth etf nysearcaspyg mqs management llc invests in centene corporation nysecnc eaton corporation plc nyseetn stock position lowered by lri investment llc stephen investment management group llc increase position in roper technology inc nyserop mtm investment management llc ha holding in ishares russell midcap etf nysearcaiwr lri investment llc acquires share of union pacific corporation nyseunp lri investment llc sell share of ameriprise financial inc nyseamp mtm investment management llc sell share of kinder morgan inc nysekmi mtm investment management llc buy share of vanguard sp etf nysearcavoo stephen inc ar boost stock position in hp inc nysehpq church dwight co inc nysechd share acquired by key financial inc lri investment llc reduces holding in kenvue inc nysekvue lri investment llc reduces position in ferrari nv nyserace lri investment llc buy share of spdr portfolio sp growth etf nysearcaspyg prudent man advisor llc sell share of vanguard intermediateterm bond etf nysearcabiv cme group inc nasdaqcme share purchased by key financial inc eaton corporation plc nyseetn share sold by lri investment llc mqs management llc buy new position in astrazeneca plc nasdaqazn kinder morgan inc nysekmi is mtm investment management llcs th largest position analyst set regeneron pharmaceutical inc nasdaqregn pt at catalyst financial partner llc grows stock position in linde plc nasdaqlin evergreen private wealth llc boost stock position in zoetis inc nysezts schwab u largecap etf nysearcaschx share sold by slow capital inc catalyst financial partner llc buy share of att inc nyset catalyst financial partner llc raise position in lowes company inc nyselow shore capital reiterates house stock rating for touchstone exploration lontxp cohen capital management inc sell share of ishares europe etf nysearcaiev vanguard ftse allworld exus etf nysearcaveu share sold by slow capital inc signaturefd llc reduces holding in rollins inc nyserol braime group lonbmt announces quarterly earnings result catalyst financial partner llc ha stock holding in sp global inc nysespgi beeks financial cloud group lonbks receives buy rating from canaccord genuity group catalyst financial partner llc increase holding in att inc nyset slow capital inc sell share of jpmorgan ultrashort municipal etf batsjmst catalyst financial partner llc ha stock position in intuitive surgical inc nasdaqisrg creightons loncrl trading higher still a buy dewhurst group londwha announces earnings result signaturefd llc boost stake in cisco system inc nasdaqcsco beeks financial cloud group lonbks receives buy rating from canaccord genuity group dunelm group londnlm receives buy rating from deutsche bank aktiengesellschaft catalyst financial partner llc ha position in capital group global growth equity etf nysearcacggo ariana resource lonaau trading up whats next simec atlantis energy lonsae trading down time to sell creightons loncrl trading higher still a buy what make uber technology uber a great business to invest in nearly half of u child are without summer learning program a cost rise study say world chess lonchss stock price down time to sell catalyst financial partner llc ha holding in the tjx company inc nysetjx a tariff on europe would effectively knock out transatlantic trade say eu trade chief promising cybersecurity stock to keep an eye on july th stratos wealth partner ltd sell share of universal display corporation nasdaqoled ge vernova inc nysegev share sold by mutual of america capital management llc bleakley financial group llc acquires share of marsh mclennan company inc nysemmc owen corning inc nyseoc given average recommendation of moderate buy by brokerage schechter investment advisor llc sell share of morgan stanley nysems corrado advisor llc raise stock position in vici property inc nysevici new york state common retirement fund trim position in ansys inc nasdaqanss arizona state retirement system sell share of raymond james financial inc nyserjf new york state common retirement fund sell share of mondelez international inc nasdaqmdlz diversify wealth management llc raise stock position in appfolio inc nasdaqappf emerald adviser llc decrease stock position in lharris technology inc nyselhx stephen inc ar boost stock position in automatic data processing inc nasdaqadp m mmm hold c rating reaffirmed at wei rating weatherly asset management l p take position in chubb limited nysecb emerald adviser llc ha stock position in msci inc nysemsci bleakley financial group llc acquires share of marsh mclennan company inc nysemmc arizona state retirement system reduces stock position in ansys inc nasdaqanss fortinet inc nasdaqftnt share sold by new york state common retirement fund new york state common retirement fund sell share of cognizant technology solution corporation nasdaqctsh key financial inc increase stock position in kinsale capital group inc nyseknsl focused investor llc sell share of the home depot inc nysehd aurora investment counsel take position in elf beauty nyseelf bleakley financial group llc purchase share of vanguard total world stock etf nysearcavt trump adviser say this is how the president could certainly fire powell regeneron pharmaceutical inc nasdaqregn given average recommendation of moderate buy by brokerage mtm investment management llc acquires new position in american electric power company inc nasdaqaep lri investment llc trim stock position in kenvue inc nysekvue key financial inc purchase share of kla corporation nasdaqklac alp advisor inc purchase share of global payment inc nysegpn lri investment llc reduces stock position in ferrari nv nyserace cme group inc nasdaqcme share purchased by key financial inc mtm investment management llc ha position in hershey company the nysehsy signaturefd llc raise stock position in ishares msci usa value factor etf batsvlue slow capital inc sell share of jpmorgan ultrashort municipal etf batsjmst catalyst financial partner llc boost stock position in intuitive surgical inc nasdaqisrg pulsar group lonpuls post quarterly earnings result evergreen private wealth llc ha million position in vaneck long muni etf batsmln world chess lonchss stock price down time to sell rockfire resource lonrock trading up still a buy catalyst financial partner llc ha holding in capital group global growth equity etf nysearcacggo catalyst financial partner llc purchase share of deere company nysede dunelm group londnlm receives buy rating from deutsche bank aktiengesellschaft a tariff on europe would effectively knock out transatlantic trade say eu trade chief kathmere capital management llc cut stake in ge vernova inc nysegev arthur j gallagher co nyseajg share purchased by new york state common retirement fund analyst set wex inc nysewex target price at corrado advisor llc sell share of corning incorporated nyseglw dominion energy inc nysed share acquired by new york state common retirement fund kathmere capital management llc trim holding in dell technology inc nysedell new york state common retirement fund sell share of nike inc nysenke new york state common retirement fund sell share of marvell technology inc nasdaqmrvl kinsale capital group inc nyseknsl given consensus rating of hold by brokerage emerald adviser llc sell share of xpo inc nysexpo emerald adviser llc ha stake in burlington store inc nyseburl invmun incom oia to go exdividend on july th doubleline yield opportunity fund plan monthly dividend of nysedly inv vk invt ny announces monthly dividend of nysevtn gladstone land co announces monthly dividend of nasdaqlandp regency center co declares quarterly dividend of nasdaqregcp thor exploration lonthx given buy rating at canaccord genuity group berenberg bank issue positive forecast for volex lonvlx stock price gladstone commercial co nasdaqgoodn plan monthly dividend trump give russia a day deadline on ukraine signaturefd llc ha million stock position in ishares msci acwi ex u etf nasdaqacwx signaturefd llc buy share of toyota motor corporation nysetm cheems cheemspet cheems price hit on exchange reviewing cyclo therapeutic nasdaqcyth sorrento therapeutic nasdaqsrne financial contrast cemtrex nasdaqcetx versus omron otcmktsomrny empower self reported market capitalization top thousand mpwr animecoin anime hit day volume of million dignity gold digau trading higher over last day share in howmet aerospace inc nysehwm bought by florida financial advisor llc florida financial advisor llc sell share of unitedhealth group incorporated nyseunh aercap holding nv nyseaer stake cut by check capital management inc ca headtohead contrast insight enterprise nasdaqnsit v flowerscom nasdaqflws slow capital inc sell share of ishares global consumer staple etf nysearcakxi fidelity national information service inc nysefis position boosted by isthmus partner llc gould asset management llc ca reduces stock holding in ishares select dividend etf nasdaqdvy abbvie inc nyseabbv share sold by florida financial advisor llc slow capital inc cut stake in ishares global comm service etf nysearcaixp top renewable energy stock to research july th gould asset management llc ca lower position in ishares msci acwi low carbon target etf nysearcacrbn alta foundation donates k toward texas flood relief trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine trump envoy arrives in kyiv a u pledge more patriot missile to ukraine rice hall james associate llc lower stock position in lantheus holding inc nasdaqlnth aurora investment counsel buy share of euronet worldwide inc nasdaqeeft slow capital inc raise stock position in cadence design system inc nasdaqcdns moody corporation nysemco share purchased by slow capital inc corteva inc nysectva share sold by lri investment llc top fintech stock to keep an eye on july th first bancorp nysefbp share bought by edgestream partner lp revolution medicine inc nasdaqrvmd share acquired by edgestream partner lp rithm capital corp nyseritm share bought by edgestream partner lp edgestream partner lp raise holding in ncino inc nasdaqncno antisemitic post appear on elmos x account after hack bleakley financial group llc purchase share of schwab u smallcap etf nysearcascha bleakley financial group llc boost stock holding in dimensional u small cap etf nysearcadfas edgestream partner lp acquires share of simpson manufacturing company inc nysessd edgestream partner lp ha million stake in nmi holding inc nasdaqnmih edgestream partner lp make new investment in exlservice holding inc nasdaqexls hartford schroders taxaware bond etf nysearcahtab share acquired by leelyn smith llc edgestream partner lp increase stock holding in cno financial group inc nysecno invesco sp high dividend low volatility etf nysearcasphd share sold by leelyn smith llc edgestream partner lp buy new position in bentley system incorporated nasdaqbsy fortress financial solution llc decrease holding in avantis emerging market equity etf nysearcaavem share in ishares future ai tech etf nysearcaarty acquired by mitchell mcleod pugh williams inc eu trade minister meet in brussels after u announces percent tariff private capital advisor inc take position in relay therapeutic inc nasdaqrlay mutual of america capital management llc ha million holding in ametek inc nyseame mitchell mcleod pugh williams inc purchase share of becton dickinson and company nysebdx</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>promising biotech stock to consider july th best travel stock worth watching july th top small cap stock to follow now july th bailard inc buy share of axon enterprise inc nasdaqaxon airline stock to follow now july th how trump tax law will reshape benefit qa is this the end of the magnificent seven boss stop trying to flatter your worker say leadership expertit doesnt make them like you verkkokauppacom oyj manager transaction nina anttila what separate successful manager from the pack come down to their oneonones here how to do it right today quordle hint and answer for july verkkokauppacom oyj manager transaction pekka litmanen sp signal the u stock rally momentum is waning bloomberg what would you like to leave behind a financial planner guide to family wealth discussion prediction stock that will be worth more than annaly capital year from now top budget gaming phone built for speed top pick under r autohome inc to announce second quarter and interim financial result on july massachusetts financial service co ma sell share of quidelortho corporation nasdaqqdel sbi security co ltd purchase share of fabrinet nysefn apollon wealth management llc acquires share of franklin bsp realty trust inc nysefbrt massachusetts financial service co ma ha million position in royal gold inc nasdaqrgld bitcoin miner iren could surge a sotp valuation peg target hedge fund manager eric jackson say were cooking with gas stock to watch monday verizon bp stellantis block she got the last seat on a flight next to a stranger theyve been married for year zwsoft launch zwcad flex in the u and canada powerful cad performance meet purchasing flexibility cwm llc grows position in lamar advertising company nasdaqlamr top chinese stock to add to your watchlist july th bailard inc sell share of mineral technology inc nysemtx ranger energy service rngr to release earnings on monday hacker exploit microsoft software vulnerability to reportedly target government and businesseswhat to know cwm llc take position in millrose property inc nysemrp acuity inc nyseayi share purchased by cwm llc massachusetts financial service co ma decrease position in select water solution inc nysewttr louisiana state employee retirement system ha stock position in apogee enterprise inc nasdaqapog signaturefd llc lower stock holding in interpublic group of company inc the nyseipg envestnet asset management inc grows holding in yeti holding inc nyseyeti protagonist therapeutic inc nasdaqptgx share sold by massachusetts financial service co ma sbi security co ltd lower position in immunitybio inc nasdaqibrx massachusetts financial service co ma sell share of zurn elkay water solution cor nysezws reynolds consumer product inc nasdaqreyn share sold by massachusetts financial service co ma cwm llc acquires share of spdr sp biotech etf nysearcaxbi edgestream partner lp sell share of the traveler company inc nysetrv sbi security co ltd purchase share of fluor corporation nyseflr st bancorp nasdaqstba rating increased to hold at wall street zen sbi security co ltd ha holding in first trust buywrite income etf nasdaqfthi copa holding sa nysecpa position boosted by massachusetts financial service co ma cemex nysecx cut to hold at wall street zen american asset trust nyseaat upgraded by wall street zen to buy rating massachusetts financial service co ma sell share of kiniksa pharmaceutical international plc nasdaqknsa fg annuity life nysefg upgraded by wall street zen to hold rating brookdale senior living nysebkd downgraded by wall street zen to sell westlake corp nysewlk given consensus rating of moderate buy by brokerage upland software nasdaqupld stock rating upgraded by wall street zen envestnet asset management inc raise stock position in yeti holding inc nyseyeti upland software nasdaqupld rating increased to strongbuy at wall street zen dxc technology nysedxc upgraded by wall street zen to buy rating coupang nysecpng lowered to hold rating by wall street zen dxc technology nysedxc upgraded by wall street zen to buy rating ap business summarybrief at am edt rincon broadcasting buy seven local station from imagicomm rep jonathan l jackson buy international business machine corporation nyseibm share grupo aeroportuario del pacifico nysepac upgraded to buy at wall street zen infineon technology otcmktsifnny stock rating upgraded by wall street zen kennedywilson nysekw upgraded to hold at wall street zen neumora therapeutic inc nasdaqnmra receives consensus rating of hold from analyst insteel industry nyseiiin rating increased to strongbuy at wall street zen world share mostly gain after wall street log a rd straight winning week world share mostly gain after wall street log a rd straight winning week telus digital nysetixt rating lowered to hold at wall street zen nuveen churchill direct lending nysencdl upgraded at wall street zen world share mostly gain after wall street log a rd straight winning week orange otcmktsorany lowered to hold rating by wall street zen wall street zen downgrade irsa inversiones y representaciones nyseirs to buy vista energy nysevist upgraded by wall street zen to hold rating nuveen churchill direct lending nysencdl rating increased to hold at wall street zen telus digital nysetixt downgraded by wall street zen to hold orange otcmktsorany lowered to hold rating by wall street zen gold start the week on the upside a investor weigh trump tariff threat sl green realty nyseslg price target raised to karen kwan sell share of aritzia inc tseatz stock nexxen international nasdaqnexn downgraded by wall street zen to buy nexxen international nasdaqnexn downgraded to buy rating by wall street zen david o watson sell share of apellis pharmaceutical inc nasdaqapls stock victory capital management inc purchase share of sally beauty holding inc nysesbh larson financial group llc acquires share of centerpoint energy inc nysecnp victory capital management inc ha million holding in reddit inc nyserddt larson financial group llc buy share of centerpoint energy inc nysecnp victory capital management inc ha million stock position in highwoods property inc nysehiw microsoft hit with sharepoint attack one version still vulnerable apollon wealth management llc sell share of vaneck oil service etf nysearcaoih apollon wealth management llc grows position in netapp inc nasdaqntap biotechne nasdaqtech and neurogene nasdaqngne financial survey hormel food nysehrl versus china marine food group otcmktscmfo head to head survey sentinelone inc nyse share bought by signaturefd llc sigma planning corp ha million holding in jpmorgan chase co nysejpm cohen capital management inc sell share of jpmorgan chase co nysejpm sigma planning corp ha position in invesco rafi u smallmid etf nasdaqprfz apollon wealth management llc ha position in ppl corporation nyseppl signaturefd llc sell share of illumina inc nasdaqilmn visa inc nysev share sold by edgestream partner lp altman plan dc push to democratize ai economic benefit airline stock to follow now july th blue chip stock worth watching july th doj request for voter data from pa other swing state raise concern among election law expert malcolmjamal warner former cosby show star dy at in costa rica drowning there one thing no one know about trump vladimir tenev sell share of robinhood market inc nasdaqhood stock she got the last seat on a flight next to a stranger theyve been married for year insider selling garrett motion inc nysegtx major shareholder sell share of stock top chinese stock to add to your watchlist july th keith a goldan sell share of syndax pharmaceutical inc nasdaqsndx stock insider selling sintana energy inc cvesei director sell share of stock mineral technology inc nysemtx share sold by bailard inc ford motor nysef upgraded by wall street zen to hold rating performance food group company nysepfgc holding cut by massachusetts financial service co ma echostar corporation nasdaqsats receives consensus recommendation of hold from brokerage the tjx company inc nysetjx receives average pt from brokerage zevra therapeutic nasdaqzvra rating lowered to buy at wall street zen coupang nysecpng downgraded to hold rating by wall street zen irsa inversiones y representaciones nyseirs lowered to buy rating by wall street zen internet initiative japan otcmktsiijiy downgraded to hold rating by wall street zen ofg bancorp nyseofg upgraded by wall street zen to hold rating vista energy nysevist rating increased to hold at wall street zen syrian government start evacuating bedouin family from sweida getting antivaxxers to roll up their sleeve akamai technology nasdaqakam downgraded to hold rating by wall street zen victory capital management inc ha million stock position in yum brand inc nyseyum highwoods property inc nysehiw holding raised by victory capital management inc reviewing hormel food nysehrl and china marine food group otcmktscmfo u envoy double down on support for syria government and criticizes israel intervention larson financial group llc acquires share of ct corporation nysects new parliament seating chart show how labor election win shifted the tectonic plate of federal politics data show more than mbta employee made over k in overtime in cullen frost banker inc invests in sea limited sponsored adr nysese cullen frost banker inc ha holding in howmet aerospace inc nysehwm safehold inc nysesafe given consensus rating of hold by brokerage thomson reuters co nysetri stock position raised by cullen frost banker inc ishares core year usd bond etf nasdaqistb share acquired by cullen frost banker inc apollo global management inc nyseapo share acquired by cullen frost banker inc share in fortis nysefts purchased by cullen frost banker inc costar group inc nasdaqcsgp share acquired by cullen frost banker inc verdence capital advisor llc boost stock position in ishares russell midcap value etf nysearcaiws verdence capital advisor llc ha stake in schwab u midcap etf nysearcaschm verdence capital advisor llc ha stake in medpace holding inc nasdaqmedp verdence capital advisor llc sell share of teck resource ltd nyseteck hillenbrand inc nysehi share acquired by verdence capital advisor llc goldman sachs bdc inc nysegsbd share sold by verdence capital advisor llc verdence capital advisor llc buy new stake in ishares sp value etf nysearcaive tetra tech inc nasdaqttek share acquired by verdence capital advisor llc you can walk between the louvre and the guggenheim in this new art district councilor boston mass and cass drug crisis is worsening the city rat infestation verdence capital advisor llc sell share of target corporation nysetgt bailard inc take position in universal insurance holding inc nyseuve bailard inc ha position in agilent technology inc nysea verdence capital advisor llc buy share of axos financial inc nyseax verdence capital advisor llc purchase new holding in dutch bros inc nysebros verdence capital advisor llc ha holding in millerknoll inc nasdaqmlkn bailard inc grows position in umh property inc nyseumh share in mach natural resource lp nysemnr bought by verdence capital advisor llc victory capital management inc boost stock position in dollar tree inc nasdaqdltr victory capital management inc decrease position in charter communication inc nasdaqchtr larson financial group llc increase position in electronic art inc nasdaqea larson financial group llc raise stock position in airbnb inc nasdaqabnb larson financial group llc sell share of rockwell automation inc nyserok oi glass inc nyseoi receives average recommendation of moderate buy from analyst regret thy name is hawley and murkowski and musk sirius xm holding inc nasdaqsiri share sold by cullen frost banker inc wealthfront adviser llc sell share of ishares russell etf nysearcaiwm wealthfront adviser llc purchase share of the chemours company nysecc wealthfront adviser llc ha holding in first trust senior loan etf nasdaqftsl ast spacemobile inc nasdaqasts share acquired by wealthfront adviser llc pvh corp nysepvh share sold by wealthfront adviser llc emerging market internet etf nysearcaemqq share acquired by wealthfront adviser llc wealthfront adviser llc buy share of f inc nasdaqffiv wealthfront adviser llc boost position in invitation home nyseinvh avantis emerging market equity etf nysearcaavem share purchased by wealthfront adviser llc texas republican want to redraw congressional district in special session inside idaho only maximum security prison where bryan kohberger may spend the rest of his life what to expect a harvard take on the trump administration in federal court vances and marco rubios senate successor avoid gop primary drama independent voter in nyc must count is pakistan moving to join the abraham accord wary democratic establishment keeping new york mamdani at arm length how trump gameplanning for the midterm ai chatbots cocreating a matrix of unreality what i won in a staring contest with a lava heron on san cristobal island vances and marco rubios senate successor avoid gop primary drama bailard inc make new investment in pagaya technology ltd nasdaqpgy share in ge vernova inc nysegev acquired by bailard inc bailard inc sell share of philip morris international inc nysepm promising home improvement stock to research july th bailard inc make new investment in angiodynamics inc nasdaqango best ecommerce stock to watch now july th battery technology stock to research july th nanotechnology stock to consider july th value stock to follow today july th syros pharmaceutical inc nasdaqsyrs receives consensus rating of hold from brokerage massachusetts financial service co ma ha holding in vanguard value etf nysearcavtv arcus bioscience inc nysercus share sold by massachusetts financial service co ma massachusetts financial service co ma sell share of anika therapeutic inc nasdaqanik matson suspends electric vehicle shipment over battery fire concern inside pure fuel partnershipsoverretail strategy sleeper dividend stock to buy for massive upside builder mortgage aid contributing to higher home price morgan stanley say notice on the general meeting of shareholder of the auga group ab entity under restructuring on august to approve the company draft restructuring plan gries financial llc ha million position in procter gamble company the nysepg vanguard growth etf nysearcavug set new year high here why vanguard sp etf nysearcavoo is arrow financial corp largest position gries financial llc ha million stake in bristol myers squibb company nysebmy global bond yield come under pressure obama foundation add outgoing ford foundation president to board of director why opendoor stock is skyrocketing today investopedia jpm high crowding lends risk to stock not involved in ai nucleus security steve carter named a security business innovator hydrograph launch compounding partner program to expand grapheneenhanced thermoplastic klp official deny claim made in civil right lawsuit filed against them lighting precinct reject claim made in civil right lawsuit cornerstone bancorp inc quarterly report june deutsche bank aktiengesellschaft raise american express nyseaxp price target to treasure coast financial planning invests in costco wholesale corporation nasdaqcost share in costco wholesale corporation nasdaqcost purchased by tabor asset management lp costco wholesale corporation nasdaqcost holding trimmed by crestwood advisor group llc im able foundation get donation from firstenergy im able foundation get donation from firstenergy im able foundation get donation from firstenergy rosen law firm encourages vera bradley inc investor to inquire about security class action investigation vra ripple xrp trader who made m earlier this year buy again after month but it not xrp hii summer intern research top use case for ai present finding to company leadership samsung galaxy watch why it the best ai wearable wnba allstar player pay move began well before shirt and sign the pulse business new research suggests rising pr ethic problem with organizational gaslighting best samsung smart tv under r in cnbc daily open investor dismiss trump administration beef with the fed sp hit new high ap technology summarybrief at pm edt delta plane from minneapolis avoids near collision with b bomber iran sends a rocket designed to carry satellite into a suborbital test flight iran sends a rocket designed to carry satellite into a suborbital test flight wex tap ai for faster fsa reimbursement ap business summarybrief at pm edt biogen bet big on billion expansion to boost u drug manufacturing retail speculation is back with a vengeance heat pump industry on the rise global market to expand significantly by senior connection receives innovative achievement award for care express weekly analyst rating update for metlife met hazlett burt watson inc boost stock position in schwab u dividend equity etf nysearcaschd hazlett burt watson inc grows holding in salesforce inc nysecrm verus financial partner inc raise stock position in schwab u dividend equity etf nysearcaschd western montana mental health center wmmhc data breach expose personal information murphy law firm investigates legal claim appeal court order new trial for man convicted in etan patz case animal science expertise honored at international conference it end with u insurer file lawsuit say it doesnt have to pay justin baldonis legal fee jonas brother sell portion of music catalog to dad company i dont know that anybody can love your music more silicon lab announces second quarter earnings webcast head to head review ge aerospace nysege v northrop grumman nysenoc van strum towne inc boost holding in mcdonalds corporation nysemcd analyzing storage computer otcmktssoso teradata nysetdc financial review crh crh v it rival gauzy nasdaqgauz versus kla nasdaqklac head to head comparison netflix inc nasdaqnflx share sold by lewis asset management llc replimune group nasdaqrepl see large volume increase should you buy pacific wealth management sell share of abbott laboratory nyseabt walker dunlop nysewd v rocket company nyserkt headtohead survey zegona communication lonzeg hit new year high following analyst upgrade dwave quantum stock is trading higher monday whats going on rogers returning to bargaining table tomorrow usw local member call for real action toward a fair deal southwest airline announces start date for assigned seating cnn democrat try to dissect themselves with autopsy show theyre riddled with disease vista capital partner inc trim stock position in nike inc nysenke van strum towne inc ha million position in pepsico inc nasdaqpep van strum towne inc sell share of ishares core sp etf nysearcaivv integrity investment advisor llc acquires share of ishares core sp etf nysearcaivv unit apartment project proposed for virginia ave in hollywood integrity investment advisor llc buy new stake in ishares core sp etf nysearcaivv astronomer ceo kiss cam controversy sparked over million in prediction market bet on his ouster whataburger saddle up with the new bacon wrangler double a burger a big and bold a the lone star state rosen a ranked and leading law firm encourages petco health and wellness company inc investor to secure counsel before important deadline in security class action woof critical comparison finwise bancorp nasdaqfinw and texas capital bancshares nasdaqtcbi analyzing kuehne nagel international khngy it competitor rd lewis holding inc acquires share of walmart inc nysewmt comparing rayonier advanced material nyseryam and suzano nysesuz comparing osisko mining otcmktsobnnf aris mining nysearmn analyzing elme community nyseelme sun community nysesui marinemax hzo v it competitor headtohead analysis contrasting williamssonoma wsm and it competitor oneascent wealth management llc increase stake in walmart inc nysewmt reviewing ivanhoe mine ivpaf and it competitor contrasting senstar technology nasdaqsnt applied dna science nasdaqapdn ivanhoe mine ivpaf and it competitor financial comparison headtohead analysis suzano nysesuz versus rayonier advanced material nyseryam lewis asset management llc increase stake in cisco system inc nasdaqcsco unifirst nyseunf and vestis nysevsts financial analysis virgin galactic nysespce v safran otcmktssafry critical contrast amazon ups quantum game with new qubit qpu eye commercial future perception that tariff will be pulled back if market react is alive and well say cfrs patterson skip brittenham hollywood lawyer to the star dy at rogers announces pricing of cash tender offer for canadian dollar debt security rep gilbert ray cisneros jr buy northrop grumman corporation nysenoc stock rep gilbert ray cisneros jr sell prologis inc nysepld stock rep robert bresnahan jr sell off share of arista network inc nyseanet rep gilbert ray cisneros jr purchase share of okta inc nasdaqokta aire advisor llc cut stock position in abbvie inc nyseabbv lauterbach financial advisor llc invests in vanguard sp etf nysearcavoo minnesota lawmaker to resign after being convicted of felony burglary research offer link between burn pit smoke and serious brain injury gop megabills final score t in red ink and million kicked off health insurance cbo say gop megabills final score t in red ink and million kicked off health insurance cbo say trump wade into bryan kohberger murder case demand answer on why he did it there are no explanation sentencing hearing set for exkentucky officer convicted in breonna taylor raid treasure coast financial planning purchase share of costco wholesale corporation nasdaqcost ge vernova gev versus it peer critical contrast tabor asset management lp make new investment in costco wholesale corporation nasdaqcost wealth dimension group ltd ha stake in cocacola company the nyseko trump team throw nyc mayor eric adam under the bus the public deserves to know dcfs withholds detail in illinois girl death miller financial service llc sell share of vanguard value etf nysearcavtv maine need to brace for natural disaster opinion maine need to brace for natural disaster opinion maine need to brace for natural disaster opinion appeal court order new trial for man convicted in etan patz case hunter biden go off on george clooney f him and everybody around him activeduty marine will be leaving los angeles pentagon confirms encountering a bear on the trail yieldmax ultra option income strategy etf nysearcaulty see strong trading volume still a buy contrasting cosan csan it rival rollins nyserol versus limbach nasdaqlmb critical comparison southwest airline announces start date for assigned seating rogers returning to bargaining table tomorrow usw local member call for real action toward a fair deal bruker nasdaqbrkr share gap down whats next irobot nasdaqirbt v robogroup tek otcmktsrobof head to head analysis headtohead contrast kuehne nagel international khngy and it peer srh advisor llc cut holding in the charles schwab corporation nyseschw lewis asset management llc sell share of pfizer inc nysepfe limoneira nasdaqlmnr and forafric global nasdaqafri headtohead review analyzing samsonite group smsey it competitor senstar technology nasdaqsnt and applied dna science nasdaqapdn head to head survey malcolmjamal warner cosby show star dy of drowning at okta nasdaqokta stock unloaded rep robert bresnahan jr travis county commissioner margaret gomez to retire after more than year of service resecurity and braly insurance group announce strategic partnership to drive innovation in cybersecurity and insurance risk management pb and npr are generally unbiased independent of government propaganda and provide key benefit to u democracy this analyst just returned from ukraine frontlines here what he saw judge weighs reality of trump ideological deportation policy a activist crackdown trial end judge weighs reality of trump ideological deportation policy a activist crackdown trial end judge weighs reality of trump ideological deportation policy a activist crackdown trial end top metaverse stock to follow today july st judge weighs reality of trump ideological deportation policy a activist crackdown trial end judge weighs reality of trump ideological deportation policy a activist crackdown trial end lowering the voting age is a call to trust young people with democracy likely new owner of paramount pledge to snuff out bias at cbs lawyer tell fcc that cbs news will practice unbiased journalism judge weighs reality of trump ideological deportation policy a activist crackdown trial end no fk you hunter julio rosa wallop hunter biden for whining about illegals not cleaning his toilet the day niagara fall ran dry here what it looked like highpoint advisor group llc boost stock holding in johnson johnson nysejnj highpoint advisor group llc purchase share of uber technology inc nyseuber hotel stock to add to your watchlist july st highpoint advisor group llc ha million stake in bank of america corporation nysebac promising g stock to add to your watchlist july st peterson wealth service purchase share of johnson johnson nysejnj promising digital medium stock to follow today july st best gold stock to watch today july st verizon communication nysevz release quarterly earnings result beat expectation by eps exxon mobil nysexom braskem nysebak headtohead contrast financial stock to keep an eye on july st johnson johnson nysejnj stock holding decreased by peregrine asset adviser inc this pb station in boston sign is going viral after trump defunded them mark herr communication issue statement regarding the sentencing of anne pramaggiore mastercard incorporated nysema share sold by gries financial llc trump say make indian great again year ago he tried to buy and move the cleveland indian hunter biden suggests ambien contributed to joe bidens poor debate performance hunter biden suggests ambien contributed to joe bidens poor debate performance hunter biden suggests ambien contributed to joe bidens poor debate performance hunter biden suggests ambien contributed to joe bidens poor debate performance hunter biden suggests ambien contributed to joe bidens poor debate performance hunter biden suggests ambien contributed to joe bidens poor debate performance visa inc nysev stock position lowered by miller financial service llc arrow financial corp reduces stock holding in the home depot inc nysehd peterson wealth service purchase share of visa inc nysev jw cole advisor inc purchase share of oracle corporation nyseorcl harvard argues against trump admins funding freeze in court hearing future generation global limited asxfgg insider geoff wilson purchase share d boral capital reiterates buy rating for biomea fusion nasdaqbmea pepsi is betting a popular health trend can get more people to drink it soda america golden age is over letter epstein ghost is haunting trump and america enemy could summon more how did being a sport fan get so expensive wealth dimension group ltd boost position in well fargo company nysewfc environmentalist lawsuit to halt alligator alcatraz filed in wrong court florida official say trump official who hold more than one job malcolmjamal warner actor who starred a theo in the cosby show dead at young kim draw another democratic challenger in california hazlett burt watson inc acquires share of caterpillar inc nysecat hazlett burt watson inc ha million stock holding in lockheed martin corporation nyselmt gop house majority shrink after big beautiful victory dhs release video showing attempted robbery of offduty federal officer in nyc update dare bioscience to host august webinar the dare to playtm difference the winch advisory service llc ha million holding in salesforce inc nysecrm clinton email investigation omitted crucial piece of evidence declassified report find sei select international equity etf nasdaqseie see strong trading volume should you buy head to head comparison hydrofarm holding group nasdaqhyfm one bio otcmktsonbi concord medical service nyseccm versus brookdale senior living nysebkd critical contrast</t>
+          <t>promising biotech stock to consider july th best travel stock worth watching july th top small cap stock to follow now july th bailard inc buy share of axon enterprise inc nasdaqaxon airline stock to follow now july th how trump tax law will reshape benefit qa is this the end of the magnificent seven boss stop trying to flatter your worker say leadership expertit doesnt make them like you verkkokauppacom oyj manager transaction nina anttila what separate successful manager from the pack come down to their oneonones here how to do it right today quordle hint and answer for july verkkokauppacom oyj manager transaction pekka litmanen sp signal the u stock rally momentum is waning bloomberg what would you like to leave behind a financial planner guide to family wealth discussion prediction stock that will be worth more than annaly capital year from now top budget gaming phone built for speed top pick under r autohome inc to announce second quarter and interim financial result on july massachusetts financial service co ma sell share of quidelortho corporation nasdaqqdel sbi security co ltd purchase share of fabrinet nysefn apollon wealth management llc acquires share of franklin bsp realty trust inc nysefbrt massachusetts financial service co ma ha million position in royal gold inc nasdaqrgld bitcoin miner iren could surge a sotp valuation peg target hedge fund manager eric jackson say were cooking with gas stock to watch monday verizon bp stellantis block she got the last seat on a flight next to a stranger theyve been married for year zwsoft launch zwcad flex in the u and canada powerful cad performance meet purchasing flexibility cwm llc grows position in lamar advertising company nasdaqlamr top chinese stock to add to your watchlist july th bailard inc sell share of mineral technology inc nysemtx ranger energy service rngr to release earnings on monday hacker exploit microsoft software vulnerability to reportedly target government and businesseswhat to know cwm llc take position in millrose property inc nysemrp acuity inc nyseayi share purchased by cwm llc massachusetts financial service co ma decrease position in select water solution inc nysewttr louisiana state employee retirement system ha stock position in apogee enterprise inc nasdaqapog signaturefd llc lower stock holding in interpublic group of company inc the nyseipg envestnet asset management inc grows holding in yeti holding inc nyseyeti protagonist therapeutic inc nasdaqptgx share sold by massachusetts financial service co ma sbi security co ltd lower position in immunitybio inc nasdaqibrx massachusetts financial service co ma sell share of zurn elkay water solution cor nysezws reynolds consumer product inc nasdaqreyn share sold by massachusetts financial service co ma cwm llc acquires share of spdr sp biotech etf nysearcaxbi edgestream partner lp sell share of the traveler company inc nysetrv sbi security co ltd purchase share of fluor corporation nyseflr st bancorp nasdaqstba rating increased to hold at wall street zen sbi security co ltd ha holding in first trust buywrite income etf nasdaqfthi copa holding sa nysecpa position boosted by massachusetts financial service co ma cemex nysecx cut to hold at wall street zen american asset trust nyseaat upgraded by wall street zen to buy rating massachusetts financial service co ma sell share of kiniksa pharmaceutical international plc nasdaqknsa fg annuity life nysefg upgraded by wall street zen to hold rating brookdale senior living nysebkd downgraded by wall street zen to sell westlake corp nysewlk given consensus rating of moderate buy by brokerage upland software nasdaqupld stock rating upgraded by wall street zen envestnet asset management inc raise stock position in yeti holding inc nyseyeti upland software nasdaqupld rating increased to strongbuy at wall street zen dxc technology nysedxc upgraded by wall street zen to buy rating coupang nysecpng lowered to hold rating by wall street zen dxc technology nysedxc upgraded by wall street zen to buy rating ap business summarybrief at am edt rincon broadcasting buy seven local station from imagicomm rep jonathan l jackson buy international business machine corporation nyseibm share grupo aeroportuario del pacifico nysepac upgraded to buy at wall street zen infineon technology otcmktsifnny stock rating upgraded by wall street zen kennedywilson nysekw upgraded to hold at wall street zen neumora therapeutic inc nasdaqnmra receives consensus rating of hold from analyst insteel industry nyseiiin rating increased to strongbuy at wall street zen world share mostly gain after wall street log a rd straight winning week world share mostly gain after wall street log a rd straight winning week telus digital nysetixt rating lowered to hold at wall street zen nuveen churchill direct lending nysencdl upgraded at wall street zen world share mostly gain after wall street log a rd straight winning week orange otcmktsorany lowered to hold rating by wall street zen wall street zen downgrade irsa inversiones y representaciones nyseirs to buy vista energy nysevist upgraded by wall street zen to hold rating nuveen churchill direct lending nysencdl rating increased to hold at wall street zen telus digital nysetixt downgraded by wall street zen to hold orange otcmktsorany lowered to hold rating by wall street zen gold start the week on the upside a investor weigh trump tariff threat sl green realty nyseslg price target raised to karen kwan sell share of aritzia inc tseatz stock nexxen international nasdaqnexn downgraded by wall street zen to buy nexxen international nasdaqnexn downgraded to buy rating by wall street zen david o watson sell share of apellis pharmaceutical inc nasdaqapls stock victory capital management inc purchase share of sally beauty holding inc nysesbh larson financial group llc acquires share of centerpoint energy inc nysecnp victory capital management inc ha million holding in reddit inc nyserddt larson financial group llc buy share of centerpoint energy inc nysecnp victory capital management inc ha million stock position in highwoods property inc nysehiw microsoft hit with sharepoint attack one version still vulnerable apollon wealth management llc sell share of vaneck oil service etf nysearcaoih apollon wealth management llc grows position in netapp inc nasdaqntap biotechne nasdaqtech and neurogene nasdaqngne financial survey hormel food nysehrl versus china marine food group otcmktscmfo head to head survey sentinelone inc nyse share bought by signaturefd llc sigma planning corp ha million holding in jpmorgan chase co nysejpm cohen capital management inc sell share of jpmorgan chase co nysejpm sigma planning corp ha position in invesco rafi u smallmid etf nasdaqprfz apollon wealth management llc ha position in ppl corporation nyseppl signaturefd llc sell share of illumina inc nasdaqilmn visa inc nysev share sold by edgestream partner lp altman plan dc push to democratize ai economic benefit airline stock to follow now july th blue chip stock worth watching july th doj request for voter data from pa other swing state raise concern among election law expert malcolmjamal warner former cosby show star dy at in costa rica drowning there one thing no one know about trump vladimir tenev sell share of robinhood market inc nasdaqhood stock she got the last seat on a flight next to a stranger theyve been married for year insider selling garrett motion inc nysegtx major shareholder sell share of stock top chinese stock to add to your watchlist july th keith a goldan sell share of syndax pharmaceutical inc nasdaqsndx stock insider selling sintana energy inc cvesei director sell share of stock mineral technology inc nysemtx share sold by bailard inc ford motor nysef upgraded by wall street zen to hold rating performance food group company nysepfgc holding cut by massachusetts financial service co ma echostar corporation nasdaqsats receives consensus recommendation of hold from brokerage the tjx company inc nysetjx receives average pt from brokerage zevra therapeutic nasdaqzvra rating lowered to buy at wall street zen coupang nysecpng downgraded to hold rating by wall street zen irsa inversiones y representaciones nyseirs lowered to buy rating by wall street zen internet initiative japan otcmktsiijiy downgraded to hold rating by wall street zen ofg bancorp nyseofg upgraded by wall street zen to hold rating vista energy nysevist rating increased to hold at wall street zen syrian government start evacuating bedouin family from sweida getting antivaxxers to roll up their sleeve akamai technology nasdaqakam downgraded to hold rating by wall street zen victory capital management inc ha million stock position in yum brand inc nyseyum highwoods property inc nysehiw holding raised by victory capital management inc reviewing hormel food nysehrl and china marine food group otcmktscmfo u envoy double down on support for syria government and criticizes israel intervention larson financial group llc acquires share of ct corporation nysects new parliament seating chart show how labor election win shifted the tectonic plate of federal politics data show more than mbta employee made over k in overtime in cullen frost banker inc invests in sea limited sponsored adr nysese cullen frost banker inc ha holding in howmet aerospace inc nysehwm safehold inc nysesafe given consensus rating of hold by brokerage thomson reuters co nysetri stock position raised by cullen frost banker inc ishares core year usd bond etf nasdaqistb share acquired by cullen frost banker inc apollo global management inc nyseapo share acquired by cullen frost banker inc share in fortis nysefts purchased by cullen frost banker inc costar group inc nasdaqcsgp share acquired by cullen frost banker inc verdence capital advisor llc boost stock position in ishares russell midcap value etf nysearcaiws verdence capital advisor llc ha stake in schwab u midcap etf nysearcaschm verdence capital advisor llc ha stake in medpace holding inc nasdaqmedp verdence capital advisor llc sell share of teck resource ltd nyseteck hillenbrand inc nysehi share acquired by verdence capital advisor llc goldman sachs bdc inc nysegsbd share sold by verdence capital advisor llc verdence capital advisor llc buy new stake in ishares sp value etf nysearcaive tetra tech inc nasdaqttek share acquired by verdence capital advisor llc you can walk between the louvre and the guggenheim in this new art district councilor boston mass and ca drug crisis is worsening the city rat infestation verdence capital advisor llc sell share of target corporation nysetgt bailard inc take position in universal insurance holding inc nyseuve bailard inc ha position in agilent technology inc nysea verdence capital advisor llc buy share of axos financial inc nyseax verdence capital advisor llc purchase new holding in dutch bros inc nysebros verdence capital advisor llc ha holding in millerknoll inc nasdaqmlkn bailard inc grows position in umh property inc nyseumh share in mach natural resource lp nysemnr bought by verdence capital advisor llc victory capital management inc boost stock position in dollar tree inc nasdaqdltr victory capital management inc decrease position in charter communication inc nasdaqchtr larson financial group llc increase position in electronic art inc nasdaqea larson financial group llc raise stock position in airbnb inc nasdaqabnb larson financial group llc sell share of rockwell automation inc nyserok oi glass inc nyseoi receives average recommendation of moderate buy from analyst regret thy name is hawley and murkowski and musk sirius xm holding inc nasdaqsiri share sold by cullen frost banker inc wealthfront adviser llc sell share of ishares russell etf nysearcaiwm wealthfront adviser llc purchase share of the chemours company nysecc wealthfront adviser llc ha holding in first trust senior loan etf nasdaqftsl ast spacemobile inc nasdaqasts share acquired by wealthfront adviser llc pvh corp nysepvh share sold by wealthfront adviser llc emerging market internet etf nysearcaemqq share acquired by wealthfront adviser llc wealthfront adviser llc buy share of f inc nasdaqffiv wealthfront adviser llc boost position in invitation home nyseinvh avantis emerging market equity etf nysearcaavem share purchased by wealthfront adviser llc texas republican want to redraw congressional district in special session inside idaho only maximum security prison where bryan kohberger may spend the rest of his life what to expect a harvard take on the trump administration in federal court vances and marco rubios senate successor avoid gop primary drama independent voter in nyc must count is pakistan moving to join the abraham accord wary democratic establishment keeping new york mamdani at arm length how trump gameplanning for the midterm ai chatbots cocreating a matrix of unreality what i won in a staring contest with a lava heron on san cristobal island vances and marco rubios senate successor avoid gop primary drama bailard inc make new investment in pagaya technology ltd nasdaqpgy share in ge vernova inc nysegev acquired by bailard inc bailard inc sell share of philip morris international inc nysepm promising home improvement stock to research july th bailard inc make new investment in angiodynamics inc nasdaqango best ecommerce stock to watch now july th battery technology stock to research july th nanotechnology stock to consider july th value stock to follow today july th syros pharmaceutical inc nasdaqsyrs receives consensus rating of hold from brokerage massachusetts financial service co ma ha holding in vanguard value etf nysearcavtv arcus bioscience inc nysercus share sold by massachusetts financial service co ma massachusetts financial service co ma sell share of anika therapeutic inc nasdaqanik matson suspends electric vehicle shipment over battery fire concern inside pure fuel partnershipsoverretail strategy sleeper dividend stock to buy for massive upside builder mortgage aid contributing to higher home price morgan stanley say notice on the general meeting of shareholder of the auga group ab entity under restructuring on august to approve the company draft restructuring plan gries financial llc ha million position in procter gamble company the nysepg vanguard growth etf nysearcavug set new year high here why vanguard sp etf nysearcavoo is arrow financial corp largest position gries financial llc ha million stake in bristol myers squibb company nysebmy global bond yield come under pressure obama foundation add outgoing ford foundation president to board of director why opendoor stock is skyrocketing today investopedia jpm high crowding lends risk to stock not involved in ai nucleus security steve carter named a security business innovator hydrograph launch compounding partner program to expand grapheneenhanced thermoplastic klp official deny claim made in civil right lawsuit filed against them lighting precinct reject claim made in civil right lawsuit cornerstone bancorp inc quarterly report june deutsche bank aktiengesellschaft raise american express nyseaxp price target to treasure coast financial planning invests in costco wholesale corporation nasdaqcost share in costco wholesale corporation nasdaqcost purchased by tabor asset management lp costco wholesale corporation nasdaqcost holding trimmed by crestwood advisor group llc im able foundation get donation from firstenergy im able foundation get donation from firstenergy im able foundation get donation from firstenergy rosen law firm encourages vera bradley inc investor to inquire about security class action investigation vra ripple xrp trader who made m earlier this year buy again after month but it not xrp hii summer intern research top use case for ai present finding to company leadership samsung galaxy watch why it the best ai wearable wnba allstar player pay move began well before shirt and sign the pulse business new research suggests rising pr ethic problem with organizational gaslighting best samsung smart tv under r in cnbc daily open investor dismiss trump administration beef with the fed sp hit new high ap technology summarybrief at pm edt delta plane from minneapolis avoids near collision with b bomber iran sends a rocket designed to carry satellite into a suborbital test flight iran sends a rocket designed to carry satellite into a suborbital test flight wex tap ai for faster fsa reimbursement ap business summarybrief at pm edt biogen bet big on billion expansion to boost u drug manufacturing retail speculation is back with a vengeance heat pump industry on the rise global market to expand significantly by senior connection receives innovative achievement award for care express weekly analyst rating update for metlife met hazlett burt watson inc boost stock position in schwab u dividend equity etf nysearcaschd hazlett burt watson inc grows holding in salesforce inc nysecrm verus financial partner inc raise stock position in schwab u dividend equity etf nysearcaschd western montana mental health center wmmhc data breach expose personal information murphy law firm investigates legal claim appeal court order new trial for man convicted in etan patz case animal science expertise honored at international conference it end with u insurer file lawsuit say it doesnt have to pay justin baldonis legal fee jonas brother sell portion of music catalog to dad company i dont know that anybody can love your music more silicon lab announces second quarter earnings webcast head to head review ge aerospace nysege v northrop grumman nysenoc van strum towne inc boost holding in mcdonalds corporation nysemcd analyzing storage computer otcmktssoso teradata nysetdc financial review crh crh v it rival gauzy nasdaqgauz versus kla nasdaqklac head to head comparison netflix inc nasdaqnflx share sold by lewis asset management llc replimune group nasdaqrepl see large volume increase should you buy pacific wealth management sell share of abbott laboratory nyseabt walker dunlop nysewd v rocket company nyserkt headtohead survey zegona communication lonzeg hit new year high following analyst upgrade dwave quantum stock is trading higher monday whats going on rogers returning to bargaining table tomorrow usw local member call for real action toward a fair deal southwest airline announces start date for assigned seating cnn democrat try to dissect themselves with autopsy show theyre riddled with disease vista capital partner inc trim stock position in nike inc nysenke van strum towne inc ha million position in pepsico inc nasdaqpep van strum towne inc sell share of ishares core sp etf nysearcaivv integrity investment advisor llc acquires share of ishares core sp etf nysearcaivv unit apartment project proposed for virginia ave in hollywood integrity investment advisor llc buy new stake in ishares core sp etf nysearcaivv astronomer ceo kiss cam controversy sparked over million in prediction market bet on his ouster whataburger saddle up with the new bacon wrangler double a burger a big and bold a the lone star state rosen a ranked and leading law firm encourages petco health and wellness company inc investor to secure counsel before important deadline in security class action woof critical comparison finwise bancorp nasdaqfinw and texas capital bancshares nasdaqtcbi analyzing kuehne nagel international khngy it competitor rd lewis holding inc acquires share of walmart inc nysewmt comparing rayonier advanced material nyseryam and suzano nysesuz comparing osisko mining otcmktsobnnf aris mining nysearmn analyzing elme community nyseelme sun community nysesui marinemax hzo v it competitor headtohead analysis contrasting williamssonoma wsm and it competitor oneascent wealth management llc increase stake in walmart inc nysewmt reviewing ivanhoe mine ivpaf and it competitor contrasting senstar technology nasdaqsnt applied dna science nasdaqapdn ivanhoe mine ivpaf and it competitor financial comparison headtohead analysis suzano nysesuz versus rayonier advanced material nyseryam lewis asset management llc increase stake in cisco system inc nasdaqcsco unifirst nyseunf and vestis nysevsts financial analysis virgin galactic nysespce v safran otcmktssafry critical contrast amazon ups quantum game with new qubit qpu eye commercial future perception that tariff will be pulled back if market react is alive and well say cfrs patterson skip brittenham hollywood lawyer to the star dy at rogers announces pricing of cash tender offer for canadian dollar debt security rep gilbert ray cisneros jr buy northrop grumman corporation nysenoc stock rep gilbert ray cisneros jr sell prologis inc nysepld stock rep robert bresnahan jr sell off share of arista network inc nyseanet rep gilbert ray cisneros jr purchase share of okta inc nasdaqokta aire advisor llc cut stock position in abbvie inc nyseabbv lauterbach financial advisor llc invests in vanguard sp etf nysearcavoo minnesota lawmaker to resign after being convicted of felony burglary research offer link between burn pit smoke and serious brain injury gop megabills final score t in red ink and million kicked off health insurance cbo say gop megabills final score t in red ink and million kicked off health insurance cbo say trump wade into bryan kohberger murder case demand answer on why he did it there are no explanation sentencing hearing set for exkentucky officer convicted in breonna taylor raid treasure coast financial planning purchase share of costco wholesale corporation nasdaqcost ge vernova gev versus it peer critical contrast tabor asset management lp make new investment in costco wholesale corporation nasdaqcost wealth dimension group ltd ha stake in cocacola company the nyseko trump team throw nyc mayor eric adam under the bus the public deserves to know dcfs withholds detail in illinois girl death miller financial service llc sell share of vanguard value etf nysearcavtv maine need to brace for natural disaster opinion maine need to brace for natural disaster opinion maine need to brace for natural disaster opinion appeal court order new trial for man convicted in etan patz case hunter biden go off on george clooney f him and everybody around him activeduty marine will be leaving los angeles pentagon confirms encountering a bear on the trail yieldmax ultra option income strategy etf nysearcaulty see strong trading volume still a buy contrasting cosan csan it rival rollins nyserol versus limbach nasdaqlmb critical comparison southwest airline announces start date for assigned seating rogers returning to bargaining table tomorrow usw local member call for real action toward a fair deal bruker nasdaqbrkr share gap down whats next irobot nasdaqirbt v robogroup tek otcmktsrobof head to head analysis headtohead contrast kuehne nagel international khngy and it peer srh advisor llc cut holding in the charles schwab corporation nyseschw lewis asset management llc sell share of pfizer inc nysepfe limoneira nasdaqlmnr and forafric global nasdaqafri headtohead review analyzing samsonite group smsey it competitor senstar technology nasdaqsnt and applied dna science nasdaqapdn head to head survey malcolmjamal warner cosby show star dy of drowning at okta nasdaqokta stock unloaded rep robert bresnahan jr travis county commissioner margaret gomez to retire after more than year of service resecurity and braly insurance group announce strategic partnership to drive innovation in cybersecurity and insurance risk management pb and npr are generally unbiased independent of government propaganda and provide key benefit to u democracy this analyst just returned from ukraine frontlines here what he saw judge weighs reality of trump ideological deportation policy a activist crackdown trial end judge weighs reality of trump ideological deportation policy a activist crackdown trial end judge weighs reality of trump ideological deportation policy a activist crackdown trial end top metaverse stock to follow today july st judge weighs reality of trump ideological deportation policy a activist crackdown trial end judge weighs reality of trump ideological deportation policy a activist crackdown trial end lowering the voting age is a call to trust young people with democracy likely new owner of paramount pledge to snuff out bias at cbs lawyer tell fcc that cbs news will practice unbiased journalism judge weighs reality of trump ideological deportation policy a activist crackdown trial end no fk you hunter julio rosa wallop hunter biden for whining about illegals not cleaning his toilet the day niagara fall ran dry here what it looked like highpoint advisor group llc boost stock holding in johnson johnson nysejnj highpoint advisor group llc purchase share of uber technology inc nyseuber hotel stock to add to your watchlist july st highpoint advisor group llc ha million stake in bank of america corporation nysebac promising g stock to add to your watchlist july st peterson wealth service purchase share of johnson johnson nysejnj promising digital medium stock to follow today july st best gold stock to watch today july st verizon communication nysevz release quarterly earnings result beat expectation by eps exxon mobil nysexom braskem nysebak headtohead contrast financial stock to keep an eye on july st johnson johnson nysejnj stock holding decreased by peregrine asset adviser inc this pb station in boston sign is going viral after trump defunded them mark herr communication issue statement regarding the sentencing of anne pramaggiore mastercard incorporated nysema share sold by gries financial llc trump say make indian great again year ago he tried to buy and move the cleveland indian hunter biden suggests ambien contributed to joe bidens poor debate performance hunter biden suggests ambien contributed to joe bidens poor debate performance hunter biden suggests ambien contributed to joe bidens poor debate performance hunter biden suggests ambien contributed to joe bidens poor debate performance hunter biden suggests ambien contributed to joe bidens poor debate performance hunter biden suggests ambien contributed to joe bidens poor debate performance visa inc nysev stock position lowered by miller financial service llc arrow financial corp reduces stock holding in the home depot inc nysehd peterson wealth service purchase share of visa inc nysev jw cole advisor inc purchase share of oracle corporation nyseorcl harvard argues against trump admins funding freeze in court hearing future generation global limited asxfgg insider geoff wilson purchase share d boral capital reiterates buy rating for biomea fusion nasdaqbmea pepsi is betting a popular health trend can get more people to drink it soda america golden age is over letter epstein ghost is haunting trump and america enemy could summon more how did being a sport fan get so expensive wealth dimension group ltd boost position in well fargo company nysewfc environmentalist lawsuit to halt alligator alcatraz filed in wrong court florida official say trump official who hold more than one job malcolmjamal warner actor who starred a theo in the cosby show dead at young kim draw another democratic challenger in california hazlett burt watson inc acquires share of caterpillar inc nysecat hazlett burt watson inc ha million stock holding in lockheed martin corporation nyselmt gop house majority shrink after big beautiful victory dhs release video showing attempted robbery of offduty federal officer in nyc update dare bioscience to host august webinar the dare to playtm difference the winch advisory service llc ha million holding in salesforce inc nysecrm clinton email investigation omitted crucial piece of evidence declassified report find sei select international equity etf nasdaqseie see strong trading volume should you buy head to head comparison hydrofarm holding group nasdaqhyfm one bio otcmktsonbi concord medical service nyseccm versus brookdale senior living nysebkd critical contrast</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>neon bloom inc announces successful launch of aidriven backend software facebook parent meta to halt political ad in eu citing unworkable new regulation education department say it will release billion in remaining withheld grant money for school education department say it will release billion in remaining withheld grant money for school education department say it will release billion in remaining withheld grant money for school education department say it will release billion in remaining withheld grant money for school rd place at southbridge celebrates retail anchor with grand opening ribboncutting tempus wealth planning llc ha position in alphabet inc nasdaqgoog neo ivy capital management cut stock holding in johnson johnson nysejnj nicholas wealth llc trim position in alphabet inc nasdaqgoog aldi trader joes adding store in pennsylvania here where when cocoa price sharply higher on belownormal rain in west africa everything you need to know about relocating part everything you need to know about relocating part everything you need to know about relocating part everything you need to know about relocating part palantir join list of most valuable u company with stock more than doubling in coffee price slump a brazil coffee harvest accelerates chicago police blew past dnc overtime budget foreign investor in charlotte eagle lake jf project obtain conditional green card approval it will be a tidal wave of earning and data next week ap sport summarybrief at pm edt ap sport summarybrief at pm edt nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in kpn completes m share buyback walmart is selling a dresser for only and it stackable design is so versatile bill creating new wheatfield pendleton zip code pass house walmart is selling a dresser for only and it stackable design is so versatile planner approve latest section of tracy hill kpn completes m share buyback how to send bulk email in gmail easily and quickly integrate reward into the saas customer journey luxury yacht company continues to sail smoothly despite trump trade tariff partner with palm beach hotel nfl fining more than player for selling super bowl ticket above face value visa inc nysev share sold by panoramic investment advisor llc foreign investor in charlotte eagle lake jf project obtain conditional green card approval remy cointreau invests in nonalc spirit brand jnpr elbow to the face what canada risk by embracing economic nationalism special council meeting tuesday on capital improvement priority when to apply for social security jeff bezos is considering major cable channel purchase report trump float rebate for american thanks to tariff revenue berger montague pc investigates security claim against rxsight inc nasdaq rxst trump say he considering rebate check for american based on tariff expert discus state of american manufacturing at daily caller live event apple share edge higher ahead of q earnings release from epstein to exponential debt sign of a system unraveling openais gpt expected next month could steal the vibecoding crown from anthropic are healthcare customer service job at risk in ai automation era can you close on a heloc in less than two week here what to know now education department say it will release billion in remaining withheld grant money for school education department say it will release billion in remaining withheld grant money for school trump administration approves controversial acquisition of paramount by skydance medium discovery announces detail of second quarter conference call and webcast discovery announces detail of second quarter conference call and webcast behind trump war with powell a battering ram with million follower mcdonalds to test drink from shuttering cosmcs spinoff at some restaurant longbow finance sa acquires share of abbvie inc nyseabbv prospect financial group llc acquires share of abbvie inc nyseabbv hedeker wealth llc trim stake in vanguard sp etf nysearcavoo longbow finance sa buy share of abbvie inc nyseabbv longbow finance sa boost stock holding in intuitive surgical inc nasdaqisrg curb the splurge prominent chiropractor accused of sending indecent material cbnnws plan carbondale cheapening genocide strip the nea of it charter and other commentary uk germany france call for immediate ceasefire in gaza yurachek alphabet inc nasdaqgoog share sold by elefante mark b nicholas wealth llc trim stock position in alphabet inc nasdaqgoog ice begin deportation flight from florida alligator alcatraz detention facility elon musk hit back at trump after president said he didnt want to strip tesla bos of subsidy ap news summary at pm edt sylacauga voter can hear their candidate idea aug trump official hit with fascist accusation over stephen colbert ouster pharaoh maharaja and the making of a multipolar world house ethic committee order aoc to pay additional for met gala showing countryrap star gain upper hand in custody battle over daughter trump team want to rewrite history by axing book on slavery letter to the editor wallis for black peterson nichols in longview race dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge park county man allegedly plotted mass shooting at chico hot spring dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge woodsonia ready to proceed with grand island good life application president say illinois state fair upping security measure this year dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge illinois state fair upping security measure this year dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge gordon melville mackenzie dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge central florida daca recipient released from alligator alcatraz attorney say he still jailed trump sign executive order clamping down on homeless trump sign executive order clamping down on homeless nfl fining more than player for selling super bowl ticket above face value caterpillar inc nysecat share sold by ae wealth management llc hospital chaplain fired after supporting former coworker detained by ice hospital chaplain fired after supporting former coworker detained by ice hospital chaplain fired after supporting former coworker detained by ice hospital chaplain fired after supporting former coworker detained by ice hospital chaplain fired after supporting former coworker detained by ice house ethic panel tell aoc to pay another for met gala dress ucsf worker on strike over layoff in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked ae wealth management llc raise holding in vanguard midcap etf nysearcavo ae wealth management llc sell share of general mill inc nysegis ae wealth management llc acquires share of the charles schwab corporation nyseschw burney co sell share of zoetis inc nysezts two longterm dividend stock to secure your financial future molina healthcare inc nysemoh share purchased by tempus wealth planning llc dimensional emerging core equity market etf nysearcadfae share acquired by avantax advisory service inc tempus wealth planning llc buy share of vanguard information technology etf nysearcavgt gilbert cook inc acquires new holding in ovintiv inc nyseovv ishares year treasury bond etf nasdaqtlt stake cut by avantax advisory service inc royce associate lp buy share of pattersonuti energy inc nasdaqpten first trust managed municipal etf nasdaqfmb share sold by tempus wealth planning llc royce associate lp trim stake in silvercrest asset management group inc nasdaqsamg tempus wealth planning llc ha stock holding in vanguard information technology etf nysearcavgt avantax advisory service inc grows position in oracle corporation nyseorcl avantax advisory service inc trim holding in ishares year treasury bond etf nasdaqtlt gilbert cook inc buy new stake in ovintiv inc nyseovv amazon is selling a slender smartwatch for and shopper love it accurate fitness tracking channel rewind traffic chaos growth safety upgrade video vault future file consumer not beefing about these price brookwood investment group llc make new investment in kinder morgan inc nysekmi brookwood investment group llc buy share of first trust short duration managed municipal etf nysearcafsmb brookwood investment group llc take position in cigna group nyseci brookwood investment group llc acquires share of ishares core sp smallcap etf nysearcaijr organon co nyseogn share sold by royce associate lp royce associate lp lower stake in powell industry inc nasdaqpowl brookwood investment group llc buy share of southern company the nyseso organon co nyseogn share sold by royce associate lp brookwood investment group llc invests in kinder morgan inc nysekmi royce associate lp ha million stock position in ishares russell value etf nysearcaiwn brookwood investment group llc acquires share of crown castle inc nysecci brookwood investment group llc acquires share of vanguard consumer discretionary etf nysearcavcr usjapan trade deal give trump control over billion it could be vapor ware fortune globalt investment llc ga cut stock holding in uber technology inc nyseuber nikko asset management america inc sell share of alphabet inc nasdaqgoog marietta investment partner llc invests in costco wholesale corporation nasdaqcost journey strategic wealth llc sell share of chipotle mexican grill inc nysecmg journey strategic wealth llc ha position in morgan stanley nysems share in gsk plc sponsored adr nysegsk purchased by lifework advisor llc freeportmcmoran inc nysefcx share sold by journey strategic wealth llc journey strategic wealth llc ha stock position in msci inc nysemsci brookwood investment group llc purchase share of philip morris international inc nysepm journey strategic wealth llc ha stake in vanguard smallcap value etf nysearcavbr mgm resort international nysemgm share acquired by journey strategic wealth llc advisor o llc raise position in morgan stanley nysems lifework advisor llc make new investment in steel dynamic inc nasdaqstld advisor o llc purchase share of broadridge financial solution inc nysebr lifework advisor llc sell share of spdr portfolio long term treasury etf nysearcasptl one wealth advisor llc grows position in emerson electric co nyseemr journey strategic wealth llc purchase share of msci inc nysemsci advisor o llc ha stock position in trane technology plc nysett advisor o llc sell share of charles river laboratory international inc nysecrl brookwood investment group llc buy share of philip morris international inc nysepm dimensional international value etf nysearcadfiv share sold by journey strategic wealth llc advanced micro device inc nasdaqamd stock position lifted by lifework advisor llc freeportmcmoran inc nysefcx share sold by journey strategic wealth llc journey strategic wealth llc ha position in ford motor company nysef brandywine oak private wealth llc decrease stake in international business machine corporation nyseibm hb wealth management llc grows stock position in johnson johnson nysejnj washington gas customer in virginia to see a surcharge this summer aurora facing significant hole in budget mayor say advisor o llc increase stock position in bristol myers squibb company nysebmy wec energy group inc nysewec share acquired by carnegie investment counsel advisor o llc decrease stock holding in teledyne technology incorporated nysetdy carnegie investment counsel cut stock position in invesco bulletshares high yield corporate bond etf nasdaqbsjq advisor o llc lower stock holding in becton dickinson and company nysebdx advisor o llc ha stock position in ishares msci usa quality factor etf batsqual advisor o llc buy share of arista network inc nyseanet archer daniel midland company nyseadm share purchased by advisor o llc intuit inc nasdaqintu share purchased by carnegie investment counsel adobe inc nasdaqadbe share bought by advisor o llc advisor o llc sell share of equifax inc nyseefx kovack advisor inc buy share of invesco aerospace defense etf nysearcappa fair isaac corporation nysefico share sold by advisor o llc advisor o llc ha stock position in ge vernova inc nysegev eversource energy nysees share bought by advisor o llc honeywell international inc nasdaqhon share acquired by advisor o llc advisor o llc acquires share of arista network inc nyseanet carnegie investment counsel invests in equifax inc nyseefx advisor o llc ha position in sei investment company nasdaqseic carnegie investment counsel ha million holding in fiserv inc nysefi advisor o llc sell share of ishares msci usa quality factor etf batsqual wedbush security inc decrease position in capital group u multisector income etf nysearcacgms phoenix financial ltd increase stock holding in barrick mining corporation nyseb carnegie investment counsel invests million in bank of montreal nysebmo machina capital sa make new investment in marvell technology inc nasdaqmrvl phoenix financial ltd invests in tmobile u inc nasdaqtmus carnegie investment counsel ha million stock position in ishares global tech etf nysearcaixn carnegie investment counsel sell share of ishares msci eafe etf nysearcaefa schwab u largecap etf nysearcaschx share acquired by carnegie investment counsel carnegie investment counsel acquires share of the walt disney company nysedis machina capital sa cut stock position in workday inc nasdaqwday carnegie investment counsel purchase share of dover corporation nysedov carnegie investment counsel sell share of comcast corporation nasdaqcmcsa phoenix financial ltd invests in tmobile u inc nasdaqtmus carnegie investment counsel acquires share of american express company nyseaxp phoenix financial ltd cut stake in synopsys inc nasdaqsnps ishares russell growth etf nysearcaiwf share bought by carnegie investment counsel carnegie investment counsel raise stock position in american electric power company inc nasdaqaep carnegie investment counsel purchase share of vanguard smallcap growth etf nysearcavbk letter bzdok pinnacle associate ltd acquires share of ishares russell midcap growth etf nysearcaiwp tempus wealth planning llc decrease stock position in first trust managed municipal etf nasdaqfmb avantax advisory service inc raise position in oracle corporation nyseorcl house democrat look to get copy of late sex offender jeffrey epstein birthday book astronomer hire gwyneth paltrow to be temporary spokesperson after kiss cam drama child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born watch a the company that employed the coldplay cheater run an absolute clinic on damage control child who starved to death in gaza weighed less than when she wa born youth delegate represent polk county at th tennessee h congress child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born child who starved to death in gaza weighed less than when she wa born share in the kroger co nysekr acquired by brookwood investment group llc royce associate lp ha million stock holding in ishares russell value etf nysearcaiwn brookwood investment group llc make new investment in crown castle inc nysecci clash over a promotion put hegseth at odds with his general horror upon horror how u congress responded to mass hunger in gaza lifework advisor llc boost stake in advanced micro device inc nasdaqamd journey strategic wealth llc ha stock position in ford motor company nysef drugpanel member who resigned lament ignoring of expert advice role of politics bc eaton corporation plc nyseetn share sold by advisor o llc carnegie investment counsel boost holding in cdw corporation nasdaqcdw sei investment company nasdaqseic stock position boosted by advisor o llc carnegie investment counsel ha million position in fiserv inc nysefi advisor o llc purchase share of eog resource inc nyseeog ap news summary at pm edt ap news summary at pm edt woman in legislature across the u fight for potty parity woman in legislature across the u fight for potty parity woman in legislature across the u fight for potty parity woman in legislature across the u fight for potty parity woman in legislature across the u fight for potty parity woman in legislature across the u fight for potty parity woman in legislature across the u fight for potty parity woman in legislature across the u fight for potty parity president donald trump say japan will invest billion in u at his direction it may not be a sure thing forum epstein case dont look away from this controversy letter president trump vision for america will have calamitous consequence woman in legislature across the u fight for potty parity quentin and carnell lake team up to tackle heart valve disease ishares russell growth etf nysearcaiwf share acquired by carnegie investment counsel phoenix financial ltd sell share of synopsys inc nasdaqsnps carnegie investment counsel trim stock position in booking holding inc nasdaqbkng carnegie investment counsel purchase share of american express company nyseaxp carnegie investment counsel increase stake in american electric power company inc nasdaqaep omnicom group inc nyseomc share sold by carnegie investment counsel analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal amazon backtoschool apple sale is live airpods ipads and macbooks from your source for insightful business news and analysis bedel financial consulting inc sell share of vanguard total stock market etf nysearcavti nisource inc nyseni share sold by spectrum wealth counsel llc kapitalo investimentos ltda purchase share of flower food inc nyseflo spectrum wealth counsel llc buy share of verizon communication inc nysevz spectrum wealth counsel llc purchase new share in ishares russell value etf nysearcaiwd spectrum wealth counsel llc trim position in ishares msci eafe growth etf batsefg kapitalo investimentos ltda acquires share of hess corporation nysehes exelon corporation nasdaqexc share sold by kapitalo investimentos ltda kapitalo investimentos ltda lower position in fox corporation nasdaqfoxa kapitalo investimentos ltda raise stock position in nrg energy inc nysenrg bedel financial consulting inc increase stock holding in pacer u cash cow etf batscowz kapitalo investimentos ltda buy share of taiwan semiconductor manufacturing company ltd nysetsm spectrum wealth counsel llc ha million stake in illinois tool work inc nyseitw kapitalo investimentos ltda purchase share of regency center corporation nasdaqreg trump announces trade agreement with eu to set tariff at ask eartha how can home energy assessment help save money charge because i unplugged a cord paris la vega hotel tiny print fee sum up why visitor are fleeing the city view from the wing nextera energy inc nysenee share bought by mrp capital investment llc advantage trust co decrease stake in first trust smid cap rising dividend achiever etf nasdaqsdvy customer data stolen at u branch of german insurer allianz carmax inc nysekmx share bought by assetmark inc ap news summary at pm edt ap news summary at pm edt ap news summary at pm edt urgent recall of popular cheeseburger that can trigger lifethreatening allergic reaction daily mail bay bank of virginia otcmktsbayk and renasant nasdaqrnst critical contrast intellus advisor llc reduces stock position in raymond james financial inc nyserjf intellus advisor llc ha million holding in alphabet inc nasdaqgoog applied finance capital management llc grows stock position in cardinal health inc nysecah otis worldwide corporation nyseotis share acquired by empirical finance llc intellus advisor llc acquires share of tesla inc nasdaqtsla paccar inc nasdaqpcar receives average recommendation of moderate buy from brokerage ishares silver trust nysearcaslv share bought by intellus advisor llc avantax advisory service inc buy share of servicenow inc nysenow what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke walmart is selling a weatherresistant deck box for and shopper say it storage space is impressive what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke accretive wealth partner llc take position in shell plc unsponsored adr nyseshel ark investment management llc ha million holding in ptc inc nasdaqptc delta air line inc nysedal share acquired by empirical finance llc ark investment management llc sell share of faro technology inc nasdaqfaro ark investment management llc ha million holding in</t>
+          <t>neon bloom inc announces successful launch of aidriven backend software facebook parent meta to halt political ad in eu citing unworkable new regulation education department say it will release billion in remaining withheld grant money for school education department say it will release billion in remaining withheld grant money for school education department say it will release billion in remaining withheld grant money for school education department say it will release billion in remaining withheld grant money for school rd place at southbridge celebrates retail anchor with grand opening ribboncutting tempus wealth planning llc ha position in alphabet inc nasdaqgoog neo ivy capital management cut stock holding in johnson johnson nysejnj nicholas wealth llc trim position in alphabet inc nasdaqgoog aldi trader joes adding store in pennsylvania here where when cocoa price sharply higher on belownormal rain in west africa everything you need to know about relocating part everything you need to know about relocating part everything you need to know about relocating part everything you need to know about relocating part palantir join list of most valuable u company with stock more than doubling in coffee price slump a brazil coffee harvest accelerates chicago police blew past dnc overtime budget foreign investor in charlotte eagle lake jf project obtain conditional green card approval it will be a tidal wave of earning and data next week ap sport summarybrief at pm edt ap sport summarybrief at pm edt nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in nearshoring a smart way to cut cost and scale your business in kpn completes m share buyback walmart is selling a dresser for only and it stackable design is so versatile bill creating new wheatfield pendleton zip code pass house walmart is selling a dresser for only and it stackable design is so versatile planner approve latest section of tracy hill kpn completes m share buyback how to send bulk email in gmail easily and quickly integrate reward into the saas customer journey luxury yacht company continues to sail smoothly despite trump trade tariff partner with palm beach hotel nfl fining more than player for selling super bowl ticket above face value visa inc nysev share sold by panoramic investment advisor llc foreign investor in charlotte eagle lake jf project obtain conditional green card approval remy cointreau invests in nonalc spirit brand jnpr elbow to the face what canada risk by embracing economic nationalism special council meeting tuesday on capital improvement priority when to apply for social security jeff bezos is considering major cable channel purchase report trump float rebate for american thanks to tariff revenue berger montague pc investigates security claim against rxsight inc nasdaq rxst trump say he considering rebate check for american based on tariff expert discus state of american manufacturing at daily caller live event apple share edge higher ahead of q earnings release from epstein to exponential debt sign of a system unraveling openais gpt expected next month could steal the vibecoding crown from anthropic are healthcare customer service job at risk in ai automation era can you close on a heloc in le than two week here what to know now education department say it will release billion in remaining withheld grant money for school education department say it will release billion in remaining withheld grant money for school trump administration approves controversial acquisition of paramount by skydance medium discovery announces detail of second quarter conference call and webcast discovery announces detail of second quarter conference call and webcast behind trump war with powell a battering ram with million follower mcdonalds to test drink from shuttering cosmcs spinoff at some restaurant longbow finance sa acquires share of abbvie inc nyseabbv prospect financial group llc acquires share of abbvie inc nyseabbv hedeker wealth llc trim stake in vanguard sp etf nysearcavoo longbow finance sa buy share of abbvie inc nyseabbv longbow finance sa boost stock holding in intuitive surgical inc nasdaqisrg curb the splurge prominent chiropractor accused of sending indecent material cbnnws plan carbondale cheapening genocide strip the nea of it charter and other commentary uk germany france call for immediate ceasefire in gaza yurachek alphabet inc nasdaqgoog share sold by elefante mark b nicholas wealth llc trim stock position in alphabet inc nasdaqgoog ice begin deportation flight from florida alligator alcatraz detention facility elon musk hit back at trump after president said he didnt want to strip tesla bos of subsidy ap news summary at pm edt sylacauga voter can hear their candidate idea aug trump official hit with fascist accusation over stephen colbert ouster pharaoh maharaja and the making of a multipolar world house ethic committee order aoc to pay additional for met gala showing countryrap star gain upper hand in custody battle over daughter trump team want to rewrite history by axing book on slavery letter to the editor wallis for black peterson nichols in longview race dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge park county man allegedly plotted mass shooting at chico hot spring dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge woodsonia ready to proceed with grand island good life application president say illinois state fair upping security measure this year dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge illinois state fair upping security measure this year dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge gordon melville mackenzie dozen of kid and adult in gaza have starved to death in july a hunger surge dozen of kid and adult in gaza have starved to death in july a hunger surge central florida daca recipient released from alligator alcatraz attorney say he still jailed trump sign executive order clamping down on homeless trump sign executive order clamping down on homeless nfl fining more than player for selling super bowl ticket above face value caterpillar inc nysecat share sold by ae wealth management llc hospital chaplain fired after supporting former coworker detained by ice hospital chaplain fired after supporting former coworker detained by ice hospital chaplain fired after supporting former coworker detained by ice hospital chaplain fired after supporting former coworker detained by ice hospital chaplain fired after supporting former coworker detained by ice house ethic panel tell aoc to pay another for met gala dress ucsf worker on strike over layoff in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked in epstein furor trump struggle to shake off a controversy his ally once stoked ae wealth management llc raise holding in vanguard midcap etf nysearcavo ae wealth management llc sell share of general mill inc nysegis ae wealth management llc acquires share of the charles schwab corporation nyseschw burney co sell share of zoetis inc nysezts two longterm dividend stock to secure your financial future molina healthcare inc nysemoh share purchased by tempus wealth planning llc dimensional emerging core equity market etf nysearcadfae share acquired by avantax advisory service inc tempus wealth planning llc buy share of vanguard information technology etf nysearcavgt gilbert cook inc acquires new holding in ovintiv inc nyseovv ishares year treasury bond etf nasdaqtlt stake cut by avantax advisory service inc royce associate lp buy share of pattersonuti energy inc nasdaqpten first trust managed municipal etf nasdaqfmb share sold by tempus wealth planning llc royce associate lp trim stake in silvercrest asset management group inc nasdaqsamg tempus wealth planning llc ha stock holding in vanguard information technology etf nysearcavgt avantax advisory service inc grows position in oracle corporation nyseorcl avantax advisory service inc trim holding in ishares year treasury bond etf nasdaqtlt gilbert cook inc buy new stake in ovintiv inc nyseovv amazon is selling a slender smartwatch for and shopper love it accurate fitness tracking channel rewind traffic chaos growth safety upgrade video vault future file consumer not beefing about these price brookwood investment group llc make new investment in kinder morgan inc nysekmi brookwood investment group llc buy share of first trust short duration managed municipal etf nysearcafsmb brookwood investment group llc take position in cigna group nyseci brookwood investment group llc acquires share of ishares core sp smallcap etf nysearcaijr organon co nyseogn share sold by royce associate lp royce associate lp lower stake in powell industry inc nasdaqpowl brookwood investment group llc buy share of southern company the nyseso organon co nyseogn share sold by royce associate lp brookwood investment group llc invests in kinder morgan inc nysekmi royce associate lp ha million stock position in ishares russell value etf nysearcaiwn brookwood investment group llc acquires share of crown castle inc nysecci brookwood investment group llc acquires share of vanguard consumer discretionary etf nysearcavcr usjapan trade deal give trump control over billion it could be vapor ware fortune globalt investment llc ga cut stock holding in uber technology inc nyseuber nikko asset management america inc sell share of alphabet inc nasdaqgoog marietta investment partner llc invests in costco wholesale corporation nasdaqcost journey strategic wealth llc sell share of chipotle mexican grill inc nysecmg journey strategic wealth llc ha position in morgan stanley nysems share in gsk plc sponsored adr nysegsk purchased by lifework advisor llc freeportmcmoran inc nysefcx share sold by journey strategic wealth llc journey strategic wealth llc ha stock position in msci inc nysemsci brookwood investment group llc purchase share of philip morris international inc nysepm journey strategic wealth llc ha stake in vanguard smallcap value etf nysearcavbr mgm resort international nysemgm share acquired by journey strategic wealth llc advisor o llc raise position in morgan stanley nysems lifework advisor llc make new investment in steel dynamic inc nasdaqstld advisor o llc purchase share of broadridge financial solution inc nysebr lifework advisor llc sell share of spdr portfolio long term treasury etf nysearcasptl one wealth advisor llc grows position in emerson electric co nyseemr journey strategic wealth llc purchase share of msci inc nysemsci advisor o llc ha stock position in trane technology plc nysett advisor o llc sell share of charles river laboratory international inc nysecrl brookwood investment group llc buy share of philip morris international inc nysepm dimensional international value etf nysearcadfiv share sold by journey strategic wealth llc advanced micro device inc nasdaqamd stock position lifted by lifework advisor llc freeportmcmoran inc nysefcx share sold by journey strategic wealth llc journey strategic wealth llc ha position in ford motor company nysef brandywine oak private wealth llc decrease stake in international business machine corporation nyseibm hb wealth management llc grows stock position in johnson johnson nysejnj washington gas customer in virginia to see a surcharge this summer aurora facing significant hole in budget mayor say advisor o llc increase stock position in bristol myers squibb company nysebmy wec energy group inc nysewec share acquired by carnegie investment counsel advisor o llc decrease stock holding in teledyne technology incorporated nysetdy carnegie investment counsel cut stock position in invesco bulletshares high yield corporate bond etf nasdaqbsjq advisor o llc lower stock holding in becton dickinson and company nysebdx advisor o llc ha stock position in ishares msci usa quality factor etf batsqual advisor o llc buy share of arista network inc nyseanet archer daniel midland company nyseadm share purchased by advisor o llc intuit inc nasdaqintu share purchased by carnegie investment counsel adobe inc nasdaqadbe share bought by advisor o llc advisor o llc sell share of equifax inc nyseefx kovack advisor inc buy share of invesco aerospace defense etf nysearcappa fair isaac corporation nysefico share sold by advisor o llc advisor o llc ha stock position in ge vernova inc nysegev eversource energy nysees share bought by advisor o llc honeywell international inc nasdaqhon share acquired by advisor o llc advisor o llc acquires share of arista network inc nyseanet carnegie investment counsel invests in equifax inc nyseefx advisor o llc ha position in sei investment company nasdaqseic carnegie investment counsel ha million holding in fiserv inc nysefi advisor o llc sell share of ishares msci usa quality factor etf batsqual wedbush security inc decrease position in capital group u multisector income etf nysearcacgms phoenix financial ltd increase stock holding in barrick mining corporation nyseb carnegie investment counsel invests million in bank of montreal nysebmo machina capital sa make new investment in marvell technology inc nasdaqmrvl phoenix financial ltd invests in tmobile u inc nasdaqtmus carnegie investment counsel ha million stock position in ishares global tech etf nysearcaixn carnegie investment counsel sell share of ishares msci eafe etf nysearcaefa schwab u largecap etf nysearcaschx share acquired by carnegie investment counsel carnegie investment counsel acquires share of the walt disney company nysedis machina capital sa cut stock position in workday inc nasdaqwday carnegie investment counsel purchase share of dover corporation nysedov carnegie investment counsel sell share of comcast corporation nasdaqcmcsa phoenix financial ltd invests in tmobile u inc nasdaqtmus carnegie investment counsel acquires share of american express company nyseaxp phoenix financial ltd cut stake in synopsys inc nasdaqsnps ishares russell growth etf nysearcaiwf share bought by carnegie investment counsel carnegie investment counsel raise stock position in american electric power company inc nasdaqaep carnegie investment counsel purchase share of vanguard smallcap growth etf nysearcavbk letter bzdok pinnacle associate ltd acquires share of ishares russell midcap growth etf nysearcaiwp tempus wealth planning llc decrease stock position in first trust managed municipal etf nasdaqfmb avantax advisory service inc raise position in oracle corporation nyseorcl house democrat look to get copy of late sex offender jeffrey epstein birthday book astronomer hire gwyneth paltrow to be temporary spokesperson after kiss cam drama child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born watch a the company that employed the coldplay cheater run an absolute clinic on damage control child who starved to death in gaza weighed le than when she wa born youth delegate represent polk county at th tennessee h congress child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born child who starved to death in gaza weighed le than when she wa born share in the kroger co nysekr acquired by brookwood investment group llc royce associate lp ha million stock holding in ishares russell value etf nysearcaiwn brookwood investment group llc make new investment in crown castle inc nysecci clash over a promotion put hegseth at odds with his general horror upon horror how u congress responded to mass hunger in gaza lifework advisor llc boost stake in advanced micro device inc nasdaqamd journey strategic wealth llc ha stock position in ford motor company nysef drugpanel member who resigned lament ignoring of expert advice role of politics bc eaton corporation plc nyseetn share sold by advisor o llc carnegie investment counsel boost holding in cdw corporation nasdaqcdw sei investment company nasdaqseic stock position boosted by advisor o llc carnegie investment counsel ha million position in fiserv inc nysefi advisor o llc purchase share of eog resource inc nyseeog ap news summary at pm edt ap news summary at pm edt woman in legislature across the u fight for potty parity woman in legislature across the u fight for potty parity woman in legislature across the u fight for potty parity woman in legislature across the u fight for potty parity woman in legislature across the u fight for potty parity woman in legislature across the u fight for potty parity woman in legislature across the u fight for potty parity woman in legislature across the u fight for potty parity president donald trump say japan will invest billion in u at his direction it may not be a sure thing forum epstein case dont look away from this controversy letter president trump vision for america will have calamitous consequence woman in legislature across the u fight for potty parity quentin and carnell lake team up to tackle heart valve disease ishares russell growth etf nysearcaiwf share acquired by carnegie investment counsel phoenix financial ltd sell share of synopsys inc nasdaqsnps carnegie investment counsel trim stock position in booking holding inc nasdaqbkng carnegie investment counsel purchase share of american express company nyseaxp carnegie investment counsel increase stake in american electric power company inc nasdaqaep omnicom group inc nyseomc share sold by carnegie investment counsel analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal analyst ending digital service tax strict regulation must be part of eu trade deal amazon backtoschool apple sale is live airpods ipads and macbooks from your source for insightful business news and analysis bedel financial consulting inc sell share of vanguard total stock market etf nysearcavti nisource inc nyseni share sold by spectrum wealth counsel llc kapitalo investimentos ltda purchase share of flower food inc nyseflo spectrum wealth counsel llc buy share of verizon communication inc nysevz spectrum wealth counsel llc purchase new share in ishares russell value etf nysearcaiwd spectrum wealth counsel llc trim position in ishares msci eafe growth etf batsefg kapitalo investimentos ltda acquires share of hess corporation nysehes exelon corporation nasdaqexc share sold by kapitalo investimentos ltda kapitalo investimentos ltda lower position in fox corporation nasdaqfoxa kapitalo investimentos ltda raise stock position in nrg energy inc nysenrg bedel financial consulting inc increase stock holding in pacer u cash cow etf batscowz kapitalo investimentos ltda buy share of taiwan semiconductor manufacturing company ltd nysetsm spectrum wealth counsel llc ha million stake in illinois tool work inc nyseitw kapitalo investimentos ltda purchase share of regency center corporation nasdaqreg trump announces trade agreement with eu to set tariff at ask eartha how can home energy assessment help save money charge because i unplugged a cord paris la vega hotel tiny print fee sum up why visitor are fleeing the city view from the wing nextera energy inc nysenee share bought by mrp capital investment llc advantage trust co decrease stake in first trust smid cap rising dividend achiever etf nasdaqsdvy customer data stolen at u branch of german insurer allianz carmax inc nysekmx share bought by assetmark inc ap news summary at pm edt ap news summary at pm edt ap news summary at pm edt urgent recall of popular cheeseburger that can trigger lifethreatening allergic reaction daily mail bay bank of virginia otcmktsbayk and renasant nasdaqrnst critical contrast intellus advisor llc reduces stock position in raymond james financial inc nyserjf intellus advisor llc ha million holding in alphabet inc nasdaqgoog applied finance capital management llc grows stock position in cardinal health inc nysecah otis worldwide corporation nyseotis share acquired by empirical finance llc intellus advisor llc acquires share of tesla inc nasdaqtsla paccar inc nasdaqpcar receives average recommendation of moderate buy from brokerage ishares silver trust nysearcaslv share bought by intellus advisor llc avantax advisory service inc buy share of servicenow inc nysenow what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke walmart is selling a weatherresistant deck box for and shopper say it storage space is impressive what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke what to know about soda sweetener a sugar return to american coke accretive wealth partner llc take position in shell plc unsponsored adr nyseshel ark investment management llc ha million holding in ptc inc nasdaqptc delta air line inc nysedal share acquired by empirical finance llc ark investment management llc sell share of faro technology inc nasdaqfaro ark investment management llc ha million holding in nano dimension ltd nasdaqnndm empirical finance llc acquires share of fidelity national infor</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>nintendo break sale record did delayed gta release save switch fedex corporation fdxs ceo is a hitter say jim cramer inside gamesxs ai revolution can india become the next global gamechanger intel corporation intc taught me not to trust ai chatbots say jim cramer ipo stock of the week china stock leader atour test buy point amid market fall the procter gamble company pg it just not great say jim cramer espn obtains redzone other medium asset from nfl in blockbuster deal per report this week in ai key to agentic ai adoption plus ai action plan from u china mcdonalds plan major ai expansion to streamline customer order executive say paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame oil major beat back billion fine in kazakhstan paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame the outdated management mindset holding your business back paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame i worked in the building where people were killed here how to make your building more secure paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame columbia is selling a stylish quilted jacket for and reviewer say it is wellmade paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame top action comedy anime series in paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame already hit your k limit in here what to do next cadence design system inc cdnss number show nvidia is in great shape in china say jim cramer alnylams amvuttra make powerful entrance eye firstline dominance president trump seek firing of government official overseeing job data after weak employment report president trump seek firing of government official overseeing job data after weak employment report nvidia corporation nvda could be in great shape in china say jim cramer the boeing company ba a horse it ceo ha done a great job say jim cramer doj identifies tariff fraud a enforcement priority waste management inc wms ceo is doing a remarkable job say jim cramer merck co inc mrk need to move on from talking about it animal division say jim cramer starbucks corporation sbux dont worry about luckin coffee say jim cramer sarah jessica parker announces emotional and poetic end to and just like that carrier global corporation carr delivered a good quarter say jim cramer iphone pro launch in september new colour a pro chip expected india price and more otis worldwide corporation otis had a tough quarter china wa horrible say jim cramer a apple watch series is just one click away at stacksocial celestica inc cl is up huge say jim cramer ai evolution prompt sense of urgency among cfo oracle jury say tesla wa partly to blame for fatal crash trump issue nuclear threat to russiaand wall street fear gauge go vertical crypto founder take note these sec roundtable could decide the rule that govern you sugar price pressured a brazil ramp up sugar production this week in stablecoins building nextgen rail for enterprise finance tesla must pay million in damage after fatal autopilot crash jury say cnbc miami jury find tesla partly liable in autopilot crash award million in punitive damage nbc news bond etf could catch a tailwind from job data tesla tsla is found liable in fatal autopilot crash ha to pay million the latest u stock market and global trade partner react to trump new tariff no one can be that wrong trump fire labor statistic bos after weak revised job data the green revolution anand chandra cofounder executive director aryaag on fixing india agri gap with tech cocoa price sharply lower on the outlook for adequate supply what ghislaine maxwell move to a lowersecurity federal prison camp could signal reddit want to replace google a the internet top search engine investor are all in ct bond commission approves m to lower electric bill republican say it not enough coffee price plunge a supply concern ease the latest business and u trading partner worldwide respond to trump new tariff the latest business and u trading partner worldwide respond to trump new tariff nextnav and oscilloquartz partner to advance g based timing solution for critical infrastructure resmed analyst increase their forecast after strong q earnings hedge fund and insider trading news william heard warren buffett ray dalio bill ackman rokos capital management alden global capital clear channel outdoor holding inc cco and more here are reason we are not going to buy stock in friday nosediving market this is why coinbase stock coin is cratering today tipranks phoenix az lemonade stand squeeze success expands into western state with over million in sale top cryptos to join now for that could deliver big return a new bowling center wa big news in west valley bowl face endofmonth deadline corporation for public broadcasting will shutter after trump funding cut the best trader in congress how to track politician stock trade a dallas bank is confident it loss will pay off best gold stock to watch in midtiers and junior beat the major online creator led by mrbeast and mark rober want to raise million for clean water access online creator led by mrbeast and mark rober want to raise million for clean water access online creator led by mrbeast and mark rober want to raise million for clean water access former chairman of savannah economic development dy jury order tesla to pay m in autopilot crash case opening it up to other costly lawsuit jury order tesla to pay m in autopilot crash case opening it up to other costly lawsuit online creator led by mrbeast and mark rober want to raise million for clean water access tesla found partially liable for fatal crash involving driverassistance technology jury order million in damage the washington post india secret weapon for defence sovereignty through ai and zerochina tech trump injects a new dose of uncertainty in tariff a he push start date back to aug trump injects a new dose of uncertainty in tariff a he push start date back to aug these analyst boost their forecast on microstrategy following q result trump injects a new dose of uncertainty in tariff a he push start date back to aug unit moving and portable storage return a primary sponsor for timmy hill at watkins glen nascar truck series race tech stock lead selloff a soft labor data fuel fed cut bet the eye of the hurricane why the u job market ha soured economist say here what could get more expensive from trump massive tariff hike here what could get more expensive from trump massive tariff hike trump seek to leave his goldplated stain on the white house beatrice police department hosting national night out nicole leone former executive director erie humane society ha september trial date president trump seek firing of government official overseeing job data after weak employment report president trump seek firing of government official overseeing job data after weak employment report president trump seek firing of government official overseeing job data after weak employment report president trump seek firing of government official overseeing job data after weak employment report president trump seek firing of government official overseeing job data after weak employment report president trump seek firing of government official overseeing job data after weak employment report north carolina u senate race turn into a battle for the middle class sarah jessica parker announces emotional and poetic end to and just like that ghislaine maxwell join famous prisoner in move to texas prison camp wave of fake credential spark political fallout in spain gop congressman suggests hed lose money and go broke if adviser stop stock trade gop congressman suggests hed lose money and go broke if adviser stop stock trade gop congressman suggests hed lose money and go broke if adviser stop stock trade jeffrey epstein former girlfriend ghislaine maxwell is transferred to a prison camp in texas jeffrey epstein former girlfriend ghislaine maxwell is transferred to a prison camp in texas jeffrey epstein former girlfriend ghislaine maxwell is transferred to a prison camp in texas jeffrey epstein former girlfriend ghislaine maxwell is transferred to a prison camp in texas gop congressman suggests hed lose money and go broke if adviser stop stock trade gop congressman suggests hed lose money and go broke if adviser stop stock trade gop congressman suggests hed lose money and go broke if adviser stop stock trade corporation for public broadcasting which fund pb npr to close after federal aid cut nyc subway nightmare flood trap commuter in filth and failure the latest u stock market and global trade partner react to trump new tariff what ghislaine maxwell move to a lowersecurity federal prison camp could signal what new public comment rule mean for speaking at local meeting in bismarckmandan area corporation for public broadcasting will shutter after trump funding cut congressman view here the truth about impact of beautiful bill on st louis county trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev state college rally planned a another local health system cut youth trans care more american couple are turning to italy dolce vita in a quest for memorable wedding city say thursday odor came from construction of city new industrial water plant trump announces nuclear submarine positioned near russia trump announces nuclear submarine positioned near russia trump announces nuclear submarine positioned near russia cult of cruelty ghastly photo video of emaciated israeli hostage released by gaza terrorist here what could get more expensive from trump massive tariff hike red state move to slash medicaid funding for planned parenthood trump announces nuclear submarine positioned near russia trump announces nuclear submarine positioned near russia trump announces nuclear submarine positioned near russia trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev guest columnist we must empower support girl and boy trump order nuclear submarine repositioned after provocative statement from russia editorial maxwell talk giving more life to a conspiracy shribman who a hero in the age of trump brown fulfilling the promise of the ada a trophy hunter killed a lion in zimbabwe that wa part of a research project sparking anger pensacola man traveled to orlando stealing smokey bear sign along the way official say kamala harris insufferably cackle over the government spying on american through wireless earpods western country speak of a future palestinian state a the nightmare unfolding in gaza worsens western country speak of a future palestinian state a the nightmare unfolding in gaza worsens western country speak of a future palestinian state a the nightmare unfolding in gaza worsens western country speak of a future palestinian state a the nightmare unfolding in gaza worsens western country speak of a future palestinian state a the nightmare unfolding in gaza worsens trump say he deploying two nuclear sub after provocative comment from exrussian leader democrat are struggling to block trump texas power grab the healing power of sunlight office cleaner who came facetoface with the manhattan gunman detail his deadly rampage corporation for public broadcasting funder of npr and pb say it will end operation within month after federal budget cut dozen of protester swarm chuck schumer kirsten gillibrands nyc office to let gaza live fourth circuit rule unanimously in favor of employee in two case involving employer allegation of breach of restrictive covenant city county official talk about animal control a texas researcher wa held at an airport for over a week now he face deportation a texas researcher wa held at an airport for over a week now he face deportation a texas researcher wa held at an airport for over a week now he face deportation a texas researcher wa held at an airport for over a week now he face deportation a texas researcher wa held at an airport for over a week now he face deportation trump plan to build million white house party room america rising part a federal judge just called out the trump administration for lying to the supreme court k nieth to retire fbi official reportedly redacted reference to trump from epstein file trump positioning two nuclear submarine near russia following russian official threat of war how immigration legislation is dangerous to immigrant judge pause removal of k migrant from honduras nicaragua and nepal in overthetop ruling democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan trump weighs in on american eagle sydney sweeney ad shiba inu and cardano set to breakout a one new token set sight on gain top cryptos to buy in trimiq weight loss official launched in uk and ireland with green tea probiotic complex free spin no deposit bonus casino online real money casino no deposit by wild casino the shock job report set off this recession alert and hold fresh clue that ai may be boosting unemployment jpmorgan say fortune crypto presale that could make you a millionaire in dogecoin ada xrp cant match ozak ai potential arialief for neuropathy supplement official launch of a new hope for sciatic nerve discomfort relief the ig choice ha gone off the rail reader commentary what to know if youre at risk of having your wage garnished over student loan debt m raised and climbing ruvi ai ruvi called ripple xrp a coinmarketcap listing made it token one of the highest in demand why parent are suing snapchat over fentanyl death tea encouraged it user to spill then the apps data got leaked npr federal reserve governor resigns creating vacancy for trump federal reserve governor resigns creating vacancy for trump upicom bragar eagel squire pc is reminds investor of class action against neogen alto bragar eagel squire pc is reminds investor of class action against neogen alto rxsight and replimune and encourages investor to contact the firm audizen drop officially launched natural tinnitus support inspired by audifort europe ev sale report tesla ha plus win in a ev share market matsato knife official launch in australia usa redefining precision and power in the kitchen warren buffett dividend stock you can buy and hold forever crushed q earnings luka doncic agrees to a threeyear million contract extension through with the la lakers the financial swamp of banking regulator who decide which american get their bank account shut down sam altman compare openai to the manhattan projectand he not joking about the risk the democrat have a mamdani problem editorial toncoin at ondo cross while cold wallet entry crypto reward outclass both weekend gaming best ipad game to try in little pepe lilpepe price prediction for show strong potential to beat solana sol and cardano ada sluggish summer in sin city la vega see big drop in tourist ap business summarybrief at pm edt ap business summarybrief at pm edt from lao to brazil trump tariff leave a lot of loser but even the winner will pay a price from lao to brazil trump tariff leave a lot of loser but even the winner will pay a price from lao to brazil trump tariff leave a lot of loser but even the winner will pay a price from lao to brazil trump tariff leave a lot of loser but even the winner will pay a price texas panel advance redrawn congressional map that could take democratic seat your money exit a business or equity position without regret pepes chart turn positive litecoin gather whale support blockdag expands web reach with devs a day workweek isnt good just for team moral it also good for the bottom line teleflex raise outlook following strong q and biotronik acquisition tucson trolley tour operator seek to expand reach former trump prosecutor jack smith probed for alleged election interference u hiring slowed sharply over the summer the wall street journal mstr news michael saylor explains why strategy strc preferred stock is the firm iphone moment coindesk harvard say it will comply with dhs request to hand over employment form missed binance coin bnb expert say ruvi ai ruvi audited token is next millionaire maker a coinmarketcap listing spark high demand what to know if youre at risk of having your wage garnished over student loan debt how to safely download and install game on your laptop shib find support ondo hold while cold wallet price gas rebate make it a top crypto to watch little pepe lilpepe gather momentum with gain ahead while cardano ada nears run the trump administration take a very orwellian turn how this week avalanche of news from washington to wall street kept investor guessing westchester capital management inc trim stake in valero energy corporation nysevlo united super pty ltd in it capacity a trustee for the construction building union superannuation fund make new investment in valero energy corporation nysevlo decadeold bitcoin wallet emptied million in btc moved amid market correction how florida quietly surpassed california in solar growth ukrainian longrange drone hit multiple russian refinery factory overnight journointerior designer jim acosta guarantee trump wh ballroom is going to look like st americu appoints new community relation manager mitsubishi ufj trust banking corp purchase share of ge aerospace nysege j safra sarasin holding ag purchase share of thermo fisher scientific inc nysetmo mitsubishi ufj trust banking corp sell share of thermo fisher scientific inc nysetmo banco santander sa ha million stake in thermo fisher scientific inc nysetmo the walt disney company nysedis share bought by bank of nova scotia trust co the walt disney company nysedis stake lifted by r squared ltd the walt disney company nysedis share acquired by j safra sarasin holding ag the walt disney company nysedis share bought by j safra sarasin holding ag banco santander sa increase stock holding in the walt disney company nysedis this ai is set to flip every major altcoinare you in figma ipo surprise winner is a charity with million sharesand a famous backstory that sparked a bitter feud over an oil fortune decade ago fortune the hidden signal in oil market moor cabot inc ha million stock holding in the goldman sachs group inc nysegs moor cabot inc buy share of the goldman sachs group inc nysegs hartford investment management co cut stock position in zoetis inc nysezts how florida quietly surpassed california in solar growth cnbc lesson from a decade of empowering woman entrepreneur to lead boldly best trucking bookkeeping service three stock to consider today blockdags no vesting pas with roi end soon eth eye jup drop just of smallbusiness owner say the child care crisis is a critical problem here why pepeto price forecast will this presale meme coin surpass dogecoin shiba inu and ethereum editorial beyond the number study into subminimum must consider all ramification thing to know about palantir pltr before it report q earnings best trucking bookkeeping service it super disrespectful wnba player exasperated after sex toy thrown onto court for second time in a week claude cutoff anthropic revoke openais api access ahead of gpt launch malaga cove capital llc sell share of abbott laboratory nyseabt bayforest capital ltd ha stake in fidelity national financial inc nysefnf vestcor inc buy share of fidelity national financial inc nysefnf modera wealth management llc sell share of arista network inc nyseanet bank of nova scotia sell share of procter gamble company the nysepg bank of nova scotia increase stock holding in arista network inc nyseanet aviso wealth management acquires share of procter gamble company the nysepg aviso wealth management cut position in the boeing company nyseba j safra sarasin holding ag purchase share of abbott laboratory nyseabt pathway financial adviser llc purchase share of eli lilly and company nyselly aviso wealth management lower stock position in the boeing company nyseba procter gamble company the nysepg share bought by j safra sarasin holding ag what are the best dividend growth stock i should invest in right now hims alert bragar eagel squire pc announces that a class action lawsuit ha been steve witkoff meet with hostage family in tel aviv susan estrich the harvard fight money v principle jet holiday ad audio used in ice deportation video shes so cringe christine pelosi tease that shes running but not the way youd think video from the dream of dr king to the nightmare that is donald trump opinion from the dream of dr king to the nightmare that is donald trump opinion from the dream of dr king to the nightmare that is donald trump opinion guam d printing facility to enhance navy maintenance capability the ig choice ha gone off the rail reader commentary trump motif can be opaque i asked a feminist economist to bare them india stand firm on russian oil import despite trump sanction threat pedaling dei cycling weekly demand bike community include fat black woman or theyre racist the u military just launched it largest air exercise in year pennsylvania lawmaker say child care is broken but dont agree on how to fix it yet twice told tale city council attends team building workshop if trump save maxwell he will destroy everything he promised pope thrill hundred of thousand of young catholic at holy year youth festival pope thrill hundred of thousand of young catholic at holy year youth festival are republican doing enough to confirm trump nominee conservative critic say no texas panel advance redrawn congressional map that could take democratic seat trump wa asked about his press secretary performance his answer took a weird turn a i see it corvallis ha done nothing to help gazans how top democrat are already gearing up for online texas is moving forward with it radical redistricting plan america trucker need a place to park george mason university president keep job get a raise despite trump admins probe in which way is the bls biased donna brazile say nprpbsdefunding maga cannot compete with idea cue a hard trip over hillary right degree wrong time new graduate face discouraging odds of landing a job trump administration move to ban abortion care for veteran unspeakably cruel manhunt intensifies for suspect in montana bar mass shooting texas panel advance redrawn congressional map that could take democratic seat bill maher know trump losing credibility when these supporter smell bullst kevin oleary slam trump for whacking bls chief after disappointing job report you dont shoot the messenger trump administration halted civil right lawsuit targeting abuse of prisoner and the mentally ill it wa never about safety one week in here whats blocked by the uk orwellian online bill these three country dominate the fighter jet export marketfor now tiktok can shape america next generation and beijing know it former trump prosecutor jack smith probed for alleged election interference virginia end fiscal year with million surplus for next budget bonus editorial cartoon for aug other voice conserving enhancing agricultural resource with solar energy trump alum share chilling google message from before secondterm return lawfare at it finest texas house panel advance redrawn congressional map that would add more gop seat letter nd representative helping put our nation closer to fiscal crisis tracey weiss our ocean backyard coming soon opening the gate to cotonicoast dairy senate make progress in averting government shutdown much earlier than usual no piecemeal deal witkoff tell hostage family trump want full gaza agreement will the wnba approve record m deal to bring connecticut sun to boston proud democrat call into chris cuomos show admits she wa wrong about trump shes not the only one texas house committee advance gopfriendly map texas house committee advance gopfriendly map texas house committee advance gopfriendly map release the epstein file and end the coverup texas house committee advance gopfriendly map texas house committee advance gopfriendly map texas house committee advance gopfriendly map the trump administration take a very orwellian turn new photo reveal iconic white house rose garden paved over after trump makeover the nfls new kickoff rule is here to stay with a slight tweak what else is changing oversea chinese banking corp ltd raise position in ecolab inc nyseecl westchester capital management inc ha million stake in becton dickinson and company nysebdx ecolab inc nyseecl share purchased by mirabaud cie sa limited option for democrat to retaliate if texas republican redraw congressional map trump hit brazilian product with tariff over bolsonaro sign that someone you know is secretly broke do they apply to the people around you party poopers less than of american friendship cross political line texas house committee advance redrawn congressional map congressional redistricting map pass house committee pushing dems towards quorum break how trump became the new master of the senate luka doncic lakers agree to year million extension banco santander sa grows stock position in the walt disney company nysedis union pacific corporation nyseunp share sold by mitsubishi ufj trust banking corp moor cabot inc ha million stock holding in zoetis inc nysezts black swimmer teach others to help end history of aquatic segregation laduke let the sun shine so say former intelligence agent rolling stone claim the kremlin made up russiagate evidence can donald trump f diplomacy keep everyone happy laduke let the sun shine laduke let the sun shine in japan launched a second strike on pearl harborsort of laduke let the sun shine your view people have the right to sign recall petition laduke let the sun shine letter to the editor the generosity of kentuckian laduke let the sun shine laduke let the sun shine it super disrespectful wnba player exasperated after sex toy thrown onto court for second time in a week it trump economy now the latest financial number offer some warning sign aviso wealth management sell share of eli lilly and company nyselly j safra sarasin holding ag buy share of procter gamble company the nysepg steve witkoff meet with hostage family in tel aviv u court upholds order blocking indiscriminate targeting by immigration patrol u court upholds order blocking indiscriminate targeting by immigration patrol oversea chinese banking corp ltd reduces stock position in welltower inc nysewell here what we know about the anaconda shooter the victim and ongoing search effort banque cantonale vaudoise purchase new position in entergy corporation nyseetr the sherwinwilliams company nyseshw position lifted by banco santander sa lsv asset management sell share of phillips nysepsx profit drop at warren buffetts berkshire hathaway a it writes down it kraft heinz investment moor cabot inc sell share of thermo fisher scientific inc nysetmo trump tariff are making money that may make them hard to quit the new york time revolution camp unhinged white liberal spend weekend smashing junk in antitrump fury sen josh hawleys longshot stock trading ban bill advance rankles trump larimer county restaurant inspection made july st louis boeing worker again reject contract strike to begin at midnight former associate executive director file lawsuit against ahsaa boeings st louis union worker will strike on monday boeing defense union poised for it first strike since bloombergcom mahjong the latest networking opp for woman entrepreneur why analyst say this audited ai token is the next big thing coinmarketcap listing spark daily sale in the million luxury label lose their luster amid changing vibe gucci sale plunge and lvmh disappoints best crypto to buy now and secure early gain north texas father of win million at choctaw casino this cookware maker is bracing for steel tariff behind a wall of pot and pan nbc news opec country to boost oil production by barrel per day opec country to boost oil production by barrel per day opec country to boost oil production by barrel per day opec country to boost oil production by barrel per day opec country to boost oil production by barrel per day trump live update white house defends firing bls commissioner over weak job number the new york time opec country to boost oil production by barrel per day opec country to boost oil production by barrel per day white house official defend firing of labor official a critic warn of trust erosion clickbait and clean water youtubers are the new philanthropist palantir advanced micro walt disney pfizer zoominfo and more stock to watch this week barrons sen blackburn to introduce bill to root out embedded foreign interest free iq test online with instant result reliable accurate free realiqonline roll out new iq testing experience himerex pro this himerex pro uk app set new standard in aidriven trading with unmatched security and user approval ev lead vehicle category in california berkshire earnings key takeaway strong profit no buyback high cash level barrons steam and itchio pull hundred of adult game over alleged visa mastercard pressure pauline ferrandprevot win tour de france femmes becoming first french rider to win event since iam district member in st louis reject latest boeing offer strike for fair contract iam union bmw sue teen entrepreneur twice over alibaba trademark infringement top trader see ripple xrp hitting binance coin bnb and little pepe lilpepe when to buy for maximum roi starbucks to close pickup store in back to starbucks pivot citigroup launch stratum elite card to rival chase sapphire reserve disney world ferry crash into dock in stormy weather injuring rider u manufacturing resurgence foreign firm relocate amid tariff the fantastic four first step hold it lead atop the box office the fantastic four first step hold it lead atop the box office the fantastic four first step hold it lead atop the box office la vega unemployment at amid tourism drop and visitor de</t>
+          <t>nintendo break sale record did delayed gta release save switch fedex corporation fdxs ceo is a hitter say jim cramer inside gamesxs ai revolution can india become the next global gamechanger intel corporation intc taught me not to trust ai chatbots say jim cramer ipo stock of the week china stock leader atour test buy point amid market fall the procter gamble company pg it just not great say jim cramer espn obtains redzone other medium asset from nfl in blockbuster deal per report this week in ai key to agentic ai adoption plus ai action plan from u china mcdonalds plan major ai expansion to streamline customer order executive say paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame oil major beat back billion fine in kazakhstan paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame the outdated management mindset holding your business back paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame i worked in the building where people were killed here how to make your building more secure paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame columbia is selling a stylish quilted jacket for and reviewer say it is wellmade paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame top action comedy anime series in paula deen ha abruptly closed the savannah restaurant that launched her to food network fame paula deen ha abruptly closed the savannah restaurant that launched her to food network fame already hit your k limit in here what to do next cadence design system inc cdnss number show nvidia is in great shape in china say jim cramer alnylams amvuttra make powerful entrance eye firstline dominance president trump seek firing of government official overseeing job data after weak employment report president trump seek firing of government official overseeing job data after weak employment report nvidia corporation nvda could be in great shape in china say jim cramer the boeing company ba a horse it ceo ha done a great job say jim cramer doj identifies tariff fraud a enforcement priority waste management inc wms ceo is doing a remarkable job say jim cramer merck co inc mrk need to move on from talking about it animal division say jim cramer starbucks corporation sbux dont worry about luckin coffee say jim cramer sarah jessica parker announces emotional and poetic end to and just like that carrier global corporation carr delivered a good quarter say jim cramer iphone pro launch in september new colour a pro chip expected india price and more otis worldwide corporation otis had a tough quarter china wa horrible say jim cramer a apple watch series is just one click away at stacksocial celestica inc cl is up huge say jim cramer ai evolution prompt sense of urgency among cfo oracle jury say tesla wa partly to blame for fatal crash trump issue nuclear threat to russiaand wall street fear gauge go vertical crypto founder take note these sec roundtable could decide the rule that govern you sugar price pressured a brazil ramp up sugar production this week in stablecoins building nextgen rail for enterprise finance tesla must pay million in damage after fatal autopilot crash jury say cnbc miami jury find tesla partly liable in autopilot crash award million in punitive damage nbc news bond etf could catch a tailwind from job data tesla tsla is found liable in fatal autopilot crash ha to pay million the latest u stock market and global trade partner react to trump new tariff no one can be that wrong trump fire labor statistic bos after weak revised job data the green revolution anand chandra cofounder executive director aryaag on fixing india agri gap with tech cocoa price sharply lower on the outlook for adequate supply what ghislaine maxwell move to a lowersecurity federal prison camp could signal reddit want to replace google a the internet top search engine investor are all in ct bond commission approves m to lower electric bill republican say it not enough coffee price plunge a supply concern ease the latest business and u trading partner worldwide respond to trump new tariff the latest business and u trading partner worldwide respond to trump new tariff nextnav and oscilloquartz partner to advance g based timing solution for critical infrastructure resmed analyst increase their forecast after strong q earnings hedge fund and insider trading news william heard warren buffett ray dalio bill ackman rokos capital management alden global capital clear channel outdoor holding inc cco and more here are reason we are not going to buy stock in friday nosediving market this is why coinbase stock coin is cratering today tipranks phoenix az lemonade stand squeeze success expands into western state with over million in sale top cryptos to join now for that could deliver big return a new bowling center wa big news in west valley bowl face endofmonth deadline corporation for public broadcasting will shutter after trump funding cut the best trader in congress how to track politician stock trade a dallas bank is confident it loss will pay off best gold stock to watch in midtiers and junior beat the major online creator led by mrbeast and mark rober want to raise million for clean water access online creator led by mrbeast and mark rober want to raise million for clean water access online creator led by mrbeast and mark rober want to raise million for clean water access former chairman of savannah economic development dy jury order tesla to pay m in autopilot crash case opening it up to other costly lawsuit jury order tesla to pay m in autopilot crash case opening it up to other costly lawsuit online creator led by mrbeast and mark rober want to raise million for clean water access tesla found partially liable for fatal crash involving driverassistance technology jury order million in damage the washington post india secret weapon for defence sovereignty through ai and zerochina tech trump injects a new dose of uncertainty in tariff a he push start date back to aug trump injects a new dose of uncertainty in tariff a he push start date back to aug these analyst boost their forecast on microstrategy following q result trump injects a new dose of uncertainty in tariff a he push start date back to aug unit moving and portable storage return a primary sponsor for timmy hill at watkins glen nascar truck series race tech stock lead selloff a soft labor data fuel fed cut bet the eye of the hurricane why the u job market ha soured economist say here what could get more expensive from trump massive tariff hike here what could get more expensive from trump massive tariff hike trump seek to leave his goldplated stain on the white house beatrice police department hosting national night out nicole leone former executive director erie humane society ha september trial date president trump seek firing of government official overseeing job data after weak employment report president trump seek firing of government official overseeing job data after weak employment report president trump seek firing of government official overseeing job data after weak employment report president trump seek firing of government official overseeing job data after weak employment report president trump seek firing of government official overseeing job data after weak employment report president trump seek firing of government official overseeing job data after weak employment report north carolina u senate race turn into a battle for the middle class sarah jessica parker announces emotional and poetic end to and just like that ghislaine maxwell join famous prisoner in move to texas prison camp wave of fake credential spark political fallout in spain gop congressman suggests hed lose money and go broke if adviser stop stock trade gop congressman suggests hed lose money and go broke if adviser stop stock trade gop congressman suggests hed lose money and go broke if adviser stop stock trade jeffrey epstein former girlfriend ghislaine maxwell is transferred to a prison camp in texas jeffrey epstein former girlfriend ghislaine maxwell is transferred to a prison camp in texas jeffrey epstein former girlfriend ghislaine maxwell is transferred to a prison camp in texas jeffrey epstein former girlfriend ghislaine maxwell is transferred to a prison camp in texas gop congressman suggests hed lose money and go broke if adviser stop stock trade gop congressman suggests hed lose money and go broke if adviser stop stock trade gop congressman suggests hed lose money and go broke if adviser stop stock trade corporation for public broadcasting which fund pb npr to close after federal aid cut nyc subway nightmare flood trap commuter in filth and failure the latest u stock market and global trade partner react to trump new tariff what ghislaine maxwell move to a lowersecurity federal prison camp could signal what new public comment rule mean for speaking at local meeting in bismarckmandan area corporation for public broadcasting will shutter after trump funding cut congressman view here the truth about impact of beautiful bill on st louis county trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev state college rally planned a another local health system cut youth trans care more american couple are turning to italy dolce vita in a quest for memorable wedding city say thursday odor came from construction of city new industrial water plant trump announces nuclear submarine positioned near russia trump announces nuclear submarine positioned near russia trump announces nuclear submarine positioned near russia cult of cruelty ghastly photo video of emaciated israeli hostage released by gaza terrorist here what could get more expensive from trump massive tariff hike red state move to slash medicaid funding for planned parenthood trump announces nuclear submarine positioned near russia trump announces nuclear submarine positioned near russia trump announces nuclear submarine positioned near russia trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev trump order u nuclear sub repositioned over statement from exrussian leader medvedev guest columnist we must empower support girl and boy trump order nuclear submarine repositioned after provocative statement from russia editorial maxwell talk giving more life to a conspiracy shribman who a hero in the age of trump brown fulfilling the promise of the ada a trophy hunter killed a lion in zimbabwe that wa part of a research project sparking anger pensacola man traveled to orlando stealing smokey bear sign along the way official say kamala harris insufferably cackle over the government spying on american through wireless earpods western country speak of a future palestinian state a the nightmare unfolding in gaza worsens western country speak of a future palestinian state a the nightmare unfolding in gaza worsens western country speak of a future palestinian state a the nightmare unfolding in gaza worsens western country speak of a future palestinian state a the nightmare unfolding in gaza worsens western country speak of a future palestinian state a the nightmare unfolding in gaza worsens trump say he deploying two nuclear sub after provocative comment from exrussian leader democrat are struggling to block trump texas power grab the healing power of sunlight office cleaner who came facetoface with the manhattan gunman detail his deadly rampage corporation for public broadcasting funder of npr and pb say it will end operation within month after federal budget cut dozen of protester swarm chuck schumer kirsten gillibrands nyc office to let gaza live fourth circuit rule unanimously in favor of employee in two case involving employer allegation of breach of restrictive covenant city county official talk about animal control a texas researcher wa held at an airport for over a week now he face deportation a texas researcher wa held at an airport for over a week now he face deportation a texas researcher wa held at an airport for over a week now he face deportation a texas researcher wa held at an airport for over a week now he face deportation a texas researcher wa held at an airport for over a week now he face deportation trump plan to build million white house party room america rising part a federal judge just called out the trump administration for lying to the supreme court k nieth to retire fbi official reportedly redacted reference to trump from epstein file trump positioning two nuclear submarine near russia following russian official threat of war how immigration legislation is dangerous to immigrant judge pause removal of k migrant from honduras nicaragua and nepal in overthetop ruling democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan democrat launching summer blitz to press republican on trump spending plan trump weighs in on american eagle sydney sweeney ad shiba inu and cardano set to breakout a one new token set sight on gain top cryptos to buy in trimiq weight loss official launched in uk and ireland with green tea probiotic complex free spin no deposit bonus casino online real money casino no deposit by wild casino the shock job report set off this recession alert and hold fresh clue that ai may be boosting unemployment jpmorgan say fortune crypto presale that could make you a millionaire in dogecoin ada xrp cant match ozak ai potential arialief for neuropathy supplement official launch of a new hope for sciatic nerve discomfort relief the ig choice ha gone off the rail reader commentary what to know if youre at risk of having your wage garnished over student loan debt m raised and climbing ruvi ai ruvi called ripple xrp a coinmarketcap listing made it token one of the highest in demand why parent are suing snapchat over fentanyl death tea encouraged it user to spill then the apps data got leaked npr federal reserve governor resigns creating vacancy for trump federal reserve governor resigns creating vacancy for trump upicom bragar eagel squire pc is reminds investor of class action against neogen alto bragar eagel squire pc is reminds investor of class action against neogen alto rxsight and replimune and encourages investor to contact the firm audizen drop officially launched natural tinnitus support inspired by audifort europe ev sale report tesla ha plus win in a ev share market matsato knife official launch in australia usa redefining precision and power in the kitchen warren buffett dividend stock you can buy and hold forever crushed q earnings luka doncic agrees to a threeyear million contract extension through with the la lakers the financial swamp of banking regulator who decide which american get their bank account shut down sam altman compare openai to the manhattan projectand he not joking about the risk the democrat have a mamdani problem editorial toncoin at ondo cross while cold wallet entry crypto reward outclass both weekend gaming best ipad game to try in little pepe lilpepe price prediction for show strong potential to beat solana sol and cardano ada sluggish summer in sin city la vega see big drop in tourist ap business summarybrief at pm edt ap business summarybrief at pm edt from lao to brazil trump tariff leave a lot of loser but even the winner will pay a price from lao to brazil trump tariff leave a lot of loser but even the winner will pay a price from lao to brazil trump tariff leave a lot of loser but even the winner will pay a price from lao to brazil trump tariff leave a lot of loser but even the winner will pay a price texas panel advance redrawn congressional map that could take democratic seat your money exit a business or equity position without regret pepes chart turn positive litecoin gather whale support blockdag expands web reach with devs a day workweek isnt good just for team moral it also good for the bottom line teleflex raise outlook following strong q and biotronik acquisition tucson trolley tour operator seek to expand reach former trump prosecutor jack smith probed for alleged election interference u hiring slowed sharply over the summer the wall street journal mstr news michael saylor explains why strategy strc preferred stock is the firm iphone moment coindesk harvard say it will comply with dhs request to hand over employment form missed binance coin bnb expert say ruvi ai ruvi audited token is next millionaire maker a coinmarketcap listing spark high demand what to know if youre at risk of having your wage garnished over student loan debt how to safely download and install game on your laptop shib find support ondo hold while cold wallet price gas rebate make it a top crypto to watch little pepe lilpepe gather momentum with gain ahead while cardano ada nears run the trump administration take a very orwellian turn how this week avalanche of news from washington to wall street kept investor guessing westchester capital management inc trim stake in valero energy corporation nysevlo united super pty ltd in it capacity a trustee for the construction building union superannuation fund make new investment in valero energy corporation nysevlo decadeold bitcoin wallet emptied million in btc moved amid market correction how florida quietly surpassed california in solar growth ukrainian longrange drone hit multiple russian refinery factory overnight journointerior designer jim acosta guarantee trump wh ballroom is going to look like st americu appoints new community relation manager mitsubishi ufj trust banking corp purchase share of ge aerospace nysege j safra sarasin holding ag purchase share of thermo fisher scientific inc nysetmo mitsubishi ufj trust banking corp sell share of thermo fisher scientific inc nysetmo banco santander sa ha million stake in thermo fisher scientific inc nysetmo the walt disney company nysedis share bought by bank of nova scotia trust co the walt disney company nysedis stake lifted by r squared ltd the walt disney company nysedis share acquired by j safra sarasin holding ag the walt disney company nysedis share bought by j safra sarasin holding ag banco santander sa increase stock holding in the walt disney company nysedis this ai is set to flip every major altcoinare you in figma ipo surprise winner is a charity with million sharesand a famous backstory that sparked a bitter feud over an oil fortune decade ago fortune the hidden signal in oil market moor cabot inc ha million stock holding in the goldman sachs group inc nysegs moor cabot inc buy share of the goldman sachs group inc nysegs hartford investment management co cut stock position in zoetis inc nysezts how florida quietly surpassed california in solar growth cnbc lesson from a decade of empowering woman entrepreneur to lead boldly best trucking bookkeeping service three stock to consider today blockdags no vesting pas with roi end soon eth eye jup drop just of smallbusiness owner say the child care crisis is a critical problem here why pepeto price forecast will this presale meme coin surpass dogecoin shiba inu and ethereum editorial beyond the number study into subminimum must consider all ramification thing to know about palantir pltr before it report q earnings best trucking bookkeeping service it super disrespectful wnba player exasperated after sex toy thrown onto court for second time in a week claude cutoff anthropic revoke openais api access ahead of gpt launch malaga cove capital llc sell share of abbott laboratory nyseabt bayforest capital ltd ha stake in fidelity national financial inc nysefnf vestcor inc buy share of fidelity national financial inc nysefnf modera wealth management llc sell share of arista network inc nyseanet bank of nova scotia sell share of procter gamble company the nysepg bank of nova scotia increase stock holding in arista network inc nyseanet aviso wealth management acquires share of procter gamble company the nysepg aviso wealth management cut position in the boeing company nyseba j safra sarasin holding ag purchase share of abbott laboratory nyseabt pathway financial adviser llc purchase share of eli lilly and company nyselly aviso wealth management lower stock position in the boeing company nyseba procter gamble company the nysepg share bought by j safra sarasin holding ag what are the best dividend growth stock i should invest in right now hims alert bragar eagel squire pc announces that a class action lawsuit ha been steve witkoff meet with hostage family in tel aviv susan estrich the harvard fight money v principle jet holiday ad audio used in ice deportation video shes so cringe christine pelosi tease that shes running but not the way youd think video from the dream of dr king to the nightmare that is donald trump opinion from the dream of dr king to the nightmare that is donald trump opinion from the dream of dr king to the nightmare that is donald trump opinion guam d printing facility to enhance navy maintenance capability the ig choice ha gone off the rail reader commentary trump motif can be opaque i asked a feminist economist to bare them india stand firm on russian oil import despite trump sanction threat pedaling dei cycling weekly demand bike community include fat black woman or theyre racist the u military just launched it largest air exercise in year pennsylvania lawmaker say child care is broken but dont agree on how to fix it yet twice told tale city council attends team building workshop if trump save maxwell he will destroy everything he promised pope thrill hundred of thousand of young catholic at holy year youth festival pope thrill hundred of thousand of young catholic at holy year youth festival are republican doing enough to confirm trump nominee conservative critic say no texas panel advance redrawn congressional map that could take democratic seat trump wa asked about his press secretary performance his answer took a weird turn a i see it corvallis ha done nothing to help gazans how top democrat are already gearing up for online texas is moving forward with it radical redistricting plan america trucker need a place to park george mason university president keep job get a raise despite trump admins probe in which way is the bls biased donna brazile say nprpbsdefunding maga cannot compete with idea cue a hard trip over hillary right degree wrong time new graduate face discouraging odds of landing a job trump administration move to ban abortion care for veteran unspeakably cruel manhunt intensifies for suspect in montana bar mass shooting texas panel advance redrawn congressional map that could take democratic seat bill maher know trump losing credibility when these supporter smell bullst kevin oleary slam trump for whacking bls chief after disappointing job report you dont shoot the messenger trump administration halted civil right lawsuit targeting abuse of prisoner and the mentally ill it wa never about safety one week in here whats blocked by the uk orwellian online bill these three country dominate the fighter jet export marketfor now tiktok can shape america next generation and beijing know it former trump prosecutor jack smith probed for alleged election interference virginia end fiscal year with million surplus for next budget bonus editorial cartoon for aug other voice conserving enhancing agricultural resource with solar energy trump alum share chilling google message from before secondterm return lawfare at it finest texas house panel advance redrawn congressional map that would add more gop seat letter nd representative helping put our nation closer to fiscal crisis tracey wei our ocean backyard coming soon opening the gate to cotonicoast dairy senate make progress in averting government shutdown much earlier than usual no piecemeal deal witkoff tell hostage family trump want full gaza agreement will the wnba approve record m deal to bring connecticut sun to boston proud democrat call into chris cuomos show admits she wa wrong about trump shes not the only one texas house committee advance gopfriendly map texas house committee advance gopfriendly map texas house committee advance gopfriendly map release the epstein file and end the coverup texas house committee advance gopfriendly map texas house committee advance gopfriendly map texas house committee advance gopfriendly map the trump administration take a very orwellian turn new photo reveal iconic white house rose garden paved over after trump makeover the nfls new kickoff rule is here to stay with a slight tweak what else is changing oversea chinese banking corp ltd raise position in ecolab inc nyseecl westchester capital management inc ha million stake in becton dickinson and company nysebdx ecolab inc nyseecl share purchased by mirabaud cie sa limited option for democrat to retaliate if texas republican redraw congressional map trump hit brazilian product with tariff over bolsonaro sign that someone you know is secretly broke do they apply to the people around you party poopers le than of american friendship cross political line texas house committee advance redrawn congressional map congressional redistricting map pass house committee pushing dems towards quorum break how trump became the new master of the senate luka doncic lakers agree to year million extension banco santander sa grows stock position in the walt disney company nysedis union pacific corporation nyseunp share sold by mitsubishi ufj trust banking corp moor cabot inc ha million stock holding in zoetis inc nysezts black swimmer teach others to help end history of aquatic segregation laduke let the sun shine so say former intelligence agent rolling stone claim the kremlin made up russiagate evidence can donald trump f diplomacy keep everyone happy laduke let the sun shine laduke let the sun shine in japan launched a second strike on pearl harborsort of laduke let the sun shine your view people have the right to sign recall petition laduke let the sun shine letter to the editor the generosity of kentuckian laduke let the sun shine laduke let the sun shine it super disrespectful wnba player exasperated after sex toy thrown onto court for second time in a week it trump economy now the latest financial number offer some warning sign aviso wealth management sell share of eli lilly and company nyselly j safra sarasin holding ag buy share of procter gamble company the nysepg steve witkoff meet with hostage family in tel aviv u court upholds order blocking indiscriminate targeting by immigration patrol u court upholds order blocking indiscriminate targeting by immigration patrol oversea chinese banking corp ltd reduces stock position in welltower inc nysewell here what we know about the anaconda shooter the victim and ongoing search effort banque cantonale vaudoise purchase new position in entergy corporation nyseetr the sherwinwilliams company nyseshw position lifted by banco santander sa lsv asset management sell share of phillips nysepsx profit drop at warren buffetts berkshire hathaway a it writes down it kraft heinz investment moor cabot inc sell share of thermo fisher scientific inc nysetmo trump tariff are making money that may make them hard to quit the new york time revolution camp unhinged white liberal spend weekend smashing junk in antitrump fury sen josh hawleys longshot stock trading ban bill advance rankles trump larimer county restaurant inspection made july st louis boeing worker again reject contract strike to begin at midnight former associate executive director file lawsuit against ahsaa boeings st louis union worker will strike on monday boeing defense union poised for it first strike since bloombergcom mahjong the latest networking opp for woman entrepreneur why analyst say this audited ai token is the next big thing coinmarketcap listing spark daily sale in the million luxury label lose their luster amid changing vibe gucci sale plunge and lvmh disappoints best crypto to buy now and secure early gain north texas father of win million at choctaw casino this cookware maker is bracing for steel tariff behind a wall of pot and pan nbc news opec country to boost oil production by barrel per day opec country to boost oil production by barrel per day opec country to boost oil production by barrel per day opec country to boost oil production by barrel per day opec country to boost oil production by barrel per day trump live update white house defends firing bls commissioner over weak job number the new york time opec country to boost oil production by barrel per day opec country to boost oil production by barrel per day white house official defend firing of labor official a critic warn of trust erosion clickbait and clean water youtubers are the new philanthropist palantir advanced micro walt disney pfizer zoominfo and more stock to watch this week barrons sen blackburn to introduce bill to root out embedded foreign interest free iq test online with instant result reliable accurate free realiqonline roll out new iq testing experience himerex pro this himerex pro uk app set new standard in aidriven trading with unmatched security and user approval ev lead vehicle category in california berkshire earnings key takeaway strong profit no buyback high cash level barrons steam and itchio pull hundred of adult game over alleged visa mastercard pressure pauline ferrandprevot win tour de france femmes becoming first french rider to win event since iam district member in st louis reject latest boeing offer strike for fair contract iam union bmw sue teen entrepreneur twice over alibaba trademark infringement top trader see ripple xrp hitting binance coin bnb and little pepe lilpepe when to buy for maximum roi starbucks to close pickup store in back to starbucks pivot citigroup launch stratum elite card to rival chase sapphire reserve disney world ferry crash into dock in stormy weather injuring rider u manufacturing resurgence foreign firm relocate amid tariff the fantastic four first step hold it lead atop the box office the fantastic four first step hold it lead atop the box office the fantastic four first step hold it lead atop the box office la vega unemployment at amid tourism drop and visitor declin</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>tpg re finance trust q eps beat prologis see narrow window before warehouse rent increase ap business summarybrief at pm edt tesla award ceo musk million of share valued at about billion fox nation greenlights two new season of god family football tesla award ceo musk million of share valued at about billion ap news nyse martin say ipo market open for pretty much all sector exxonmobil q eps beat but stock fell magnera announces participation at the ubs global material conference magnera announces participation at the ubs global material conference danville cvb award in tourism grant panama port challenge could turn into trump win man accused in atm robbery bombing arrested in newport beach wipfli secures strategic investment from new mountain capital wild brawl erupts between ton of parent during youth football game all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend poltreg dos first patient in phase ii trial for presymptomatic type diabetes with ptg what a september rate cut would mean for stock plus a bullish call on ai spending clash of trade reality show aim to boost prestige of u manufacturing why gen z driver suffer the highest rate of crash injury why gen z driver suffer the highest rate of crash injury why gen z driver suffer the highest rate of crash injury why gen z driver suffer the highest rate of crash injury why gen z driver suffer the highest rate of crash injury palantir earnings due a nvidia broadcom shake off trump tariff investor business daily bitcoin news today m outflow hit digital asset amid fed rate fear fanzone scoreboard the ultimate gameday upgrade for nfl fan amazon metal water hose is absolutely a life changer apple io why you should update your iphone today naphtha cushion china q oil demand decline oxford bank corporation announces six month and second quarter operating result fanzone scoreboard the ultimate gameday upgrade for nfl fan thousand of boeing worker who build fighter jet and weapon go on strike palantirs ultraexpensive valuation spark worry into result yahoo finance agibank raise brl billion in debenture offering to strengthen it funding strategy and support sustainable growth kremlin urge careful use of nuclear rhetoric a medvedev pivot to saying trump blackmailed by mossad recent home sale in the area bond yield continue to decline to lowest level since april healthcare workforce management market surge amid drive for operational efficiency and cost reduction tx rail product inc report financial result for third quarter of fiscal delta say ai speed up market analysis to price airfare letter potential for a repeat firefly aerospace lift ipo range that would value company at over billion cftc issue noaction relief for sefs on order book obligation sarat sethi inflation not coming down ha put fed in quandary nyse texas tap former abbott official a president shareholder investigation halper sadeh llc investigates sptn base rkda on behalf of shareholder how is the trump bill changing plan bnb integration announced for q in apirones cryptogateway search for suspect in tennessee killing focus near university source say a rd arrest announced hhi water quality laboratory receives excellence recognition shareholder investigation halper sadeh llc investigates sptn base rkda on behalf of shareholder all major la vega strip casino are unionized defying national trend homestyle direct medically tailored meal delivery score high in pennsylvania all major la vega strip casino are unionized defying national trend homestyle direct expands access to medically tailored meal in california hireright appoints jim desmond a chief information security officer what may happen to stock market next pridestaff launch new fort worth west office to strengthen workforce solution in north texas live will palantir post a big earnings beat after the bell local husbandandwife team to lead pridestaff asheville office the ultimate guide to top cryptos to join now for massive roi ww grainger analyst cut their forecast after q earnings skylight health launch valuebased multispecialty platform mark herr communication issue statement regarding the notice of appeal by anne pramaggiore mark herr communication issue statement regarding the notice of appeal by anne pramaggiore stock that soared the last time market were this wobbly tesla gain on elon musk new pay package is tsla stock a buy euro strengthens a postpayroll fallout set stage for fed september rate cut legendary investor vinod khosla advises gen z to invest in this one skill because chatgpt can teach you everything else fortune roadwork to alter traffic on ssu campus these analyst raise their forecast on nvent electric after strong q earnings ap business summarybrief at pm edt wall street rally and u stock recover much of friday wipeout wall street rally and u stock recover much of friday wipeout wall street rally and u stock recover much of friday wipeout wall street rally and u stock recover much of friday wipeout microbiome sequencing market on the rise cagr forecast why opendoor technology stock wa soaring again today trump will raise india tariff rate substantially over russian oil purchasesheres why india might not budge these analyst increase their forecast on regeneron pharmaceutical after betterthanexpected earnings fed rate cut now likely a soft data erodes confidence in economic resilience elon musk unveils grok update after controversial post by the ai chatbot why nvidia is the biggest risk to the stock marketnot tariff barrons dude perfect partner with regal cinema to launch dude perfect the hero tour movie in hundred of theater worldwide sp could plummet say morgan stanley tipranks cal thomas starvation in gaza whom to blame former football coach enters georgia senate race european union say it pausing retaliatory tariff against the u amid trade talk gerken named sterling professor of law dhs say daca recipient are illegal alien tell them to selfdeport ap news summary at pm edt cbo republican megabill to cost t due to higher borrowing cost state department may require visa applicant to post bond of up to to enter the u state department may require visa applicant to post bond of up to to enter the u state department may require visa applicant to post bond of up to to enter the u all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend mitch mcconnells legacy come under fire in kentucky race to replace him in the senate davenport open application for round of dream home improvement funding davenport open application for round of dream home improvement funding trump say sweeneys ad is hottest american eagle stock go wild a the great new jersey denizen yogi berra observed it deja vu all over again noncompete clause are under fire in new jersey once more how many woman on the board fewer company are saying mtg sour on republican party claim gop turned it back on america first for tax paid minnesota offer a taxpayer receipt for where dollar go pic of woman at tx capitol fighting to use womens bathroom sum up how dumb transmovement really is search for suspect in tennessee killing focus near university source say a rd arrest announced all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend sex offender harassed marjorie taylor greene turn on gop for abandoning maga base officer find teen girl when arresting man for sex trafficking mpd say mamdani study america worst mayor brandon johnson to avoid his political pitfall report now i love her ad trump praise sydney sweeney amid jean ad fallout ap news summary at pm edt ap news summary at pm edt donald trump and the deconstruction of america mitch mcconnells legacy come under fire in kentucky race to replace him in the senate men accused of shooting up woman glenburn home and car trump shootthemessenger tactic will only hurt the economy more america best idea is under fierce attack u rep kelly morrison introduces legislation to boost police recruitment funding these epstein revelation show the deep state is real and it work for trump mary moriarty dont accept simplistic narrative on carjacking prosecution texas dems flee to illinois to block redistricting vote texas dems flee to illinois to block redistricting vote copy famine in gaza ocean city mayor vow further effort on ebike safety after nearly hitting rider with democrat out of state whats next for texas special session trump threatens to substantially raise tariff on indian good a it continues to buy russian oil trump threatens to substantially raise tariff on indian good a it continues to buy russian oil mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate every minute is crucial here israeli journalist on hostage held inside gaza michta published in realcleardefense and featured in realclearworld on nato and european security nyt claim many jewish voter back mamdani you wont believe who they interviewed college grad compete with ai for entrylevel job guest commentary cpuc dont saddle monterey peninsula ratepayer with desalination project celtic minority owner offer recordbreaking amount to buy move wnba team report mr william bill sander dubose sr how the supreme court kickstarted the redistricting arm race minnesota department of correction expands online application for visitor at adult facility state department may require visa applicant to post bond of up to to enter the u trump administration wont say why it transferred ghislaine maxwell to a minimumsecurity prison new law to make new hampshire library record available to parent grammywinner doechii bringing tour to san diego mortgage lender stick with bidenera reappraisal guidance white south african farm owner on trial for allegedly murdering two black woman and feeding their body to pig trump to substantially raise tariff on india for buying russian oil banana republic stuff top economist react to trump firing bls statistic chief ghislaine maxwell prison transfer add to trump epstein morass look on cnn host face a lee zeldin politely take her climate change b apart is priceless watch texas hold em gov abbott threatens legal action for absent dems mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate letter ballroom location not a good idea ap news summary at pm edt new u visa rule could require bond from visitor it feel less like advertising and more like brainwashing mainer injured when their utv rolled over in nh gravel pit former ct chief state attorney fined in ethic case what to know texas house issue arrest warrant for rogue democrat who fled to blue state rep nancy mace is latest republican to announce bid for south carolina governor minnesota congresswoman call for more police recruitment funding why dozen of democrat left texas and how republican want to punish them why dozen of democrat left texas and how republican want to punish them why dozen of democrat left texas and how republican want to punish them why dozen of democrat left texas and how republican want to punish them</t>
+          <t>tpg re finance trust q eps beat prologis see narrow window before warehouse rent increase ap business summarybrief at pm edt tesla award ceo musk million of share valued at about billion fox nation greenlights two new season of god family football tesla award ceo musk million of share valued at about billion ap news nyse martin say ipo market open for pretty much all sector exxonmobil q eps beat but stock fell magnera announces participation at the ubs global material conference magnera announces participation at the ubs global material conference danville cvb award in tourism grant panama port challenge could turn into trump win man accused in atm robbery bombing arrested in newport beach wipfli secures strategic investment from new mountain capital wild brawl erupts between ton of parent during youth football game all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend poltreg dos first patient in phase ii trial for presymptomatic type diabetes with ptg what a september rate cut would mean for stock plus a bullish call on ai spending clash of trade reality show aim to boost prestige of u manufacturing why gen z driver suffer the highest rate of crash injury why gen z driver suffer the highest rate of crash injury why gen z driver suffer the highest rate of crash injury why gen z driver suffer the highest rate of crash injury why gen z driver suffer the highest rate of crash injury palantir earnings due a nvidia broadcom shake off trump tariff investor business daily bitcoin news today m outflow hit digital asset amid fed rate fear fanzone scoreboard the ultimate gameday upgrade for nfl fan amazon metal water hose is absolutely a life changer apple io why you should update your iphone today naphtha cushion china q oil demand decline oxford bank corporation announces six month and second quarter operating result fanzone scoreboard the ultimate gameday upgrade for nfl fan thousand of boeing worker who build fighter jet and weapon go on strike palantirs ultraexpensive valuation spark worry into result yahoo finance agibank raise brl billion in debenture offering to strengthen it funding strategy and support sustainable growth kremlin urge careful use of nuclear rhetoric a medvedev pivot to saying trump blackmailed by mossad recent home sale in the area bond yield continue to decline to lowest level since april healthcare workforce management market surge amid drive for operational efficiency and cost reduction tx rail product inc report financial result for third quarter of fiscal delta say ai speed up market analysis to price airfare letter potential for a repeat firefly aerospace lift ipo range that would value company at over billion cftc issue noaction relief for sefs on order book obligation sarat sethi inflation not coming down ha put fed in quandary nyse texas tap former abbott official a president shareholder investigation halper sadeh llc investigates sptn base rkda on behalf of shareholder how is the trump bill changing plan bnb integration announced for q in apirones cryptogateway search for suspect in tennessee killing focus near university source say a rd arrest announced hhi water quality laboratory receives excellence recognition shareholder investigation halper sadeh llc investigates sptn base rkda on behalf of shareholder all major la vega strip casino are unionized defying national trend homestyle direct medically tailored meal delivery score high in pennsylvania all major la vega strip casino are unionized defying national trend homestyle direct expands access to medically tailored meal in california hireright appoints jim desmond a chief information security officer what may happen to stock market next pridestaff launch new fort worth west office to strengthen workforce solution in north texas live will palantir post a big earnings beat after the bell local husbandandwife team to lead pridestaff asheville office the ultimate guide to top cryptos to join now for massive roi ww grainger analyst cut their forecast after q earnings skylight health launch valuebased multispecialty platform mark herr communication issue statement regarding the notice of appeal by anne pramaggiore mark herr communication issue statement regarding the notice of appeal by anne pramaggiore stock that soared the last time market were this wobbly tesla gain on elon musk new pay package is tsla stock a buy euro strengthens a postpayroll fallout set stage for fed september rate cut legendary investor vinod khosla advises gen z to invest in this one skill because chatgpt can teach you everything else fortune roadwork to alter traffic on ssu campus these analyst raise their forecast on nvent electric after strong q earnings ap business summarybrief at pm edt wall street rally and u stock recover much of friday wipeout wall street rally and u stock recover much of friday wipeout wall street rally and u stock recover much of friday wipeout wall street rally and u stock recover much of friday wipeout microbiome sequencing market on the rise cagr forecast why opendoor technology stock wa soaring again today trump will raise india tariff rate substantially over russian oil purchasesheres why india might not budge these analyst increase their forecast on regeneron pharmaceutical after betterthanexpected earnings fed rate cut now likely a soft data erodes confidence in economic resilience elon musk unveils grok update after controversial post by the ai chatbot why nvidia is the biggest risk to the stock marketnot tariff barrons dude perfect partner with regal cinema to launch dude perfect the hero tour movie in hundred of theater worldwide sp could plummet say morgan stanley tipranks cal thomas starvation in gaza whom to blame former football coach enters georgia senate race european union say it pausing retaliatory tariff against the u amid trade talk gerken named sterling professor of law dhs say daca recipient are illegal alien tell them to selfdeport ap news summary at pm edt cbo republican megabill to cost t due to higher borrowing cost state department may require visa applicant to post bond of up to to enter the u state department may require visa applicant to post bond of up to to enter the u state department may require visa applicant to post bond of up to to enter the u all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend mitch mcconnells legacy come under fire in kentucky race to replace him in the senate davenport open application for round of dream home improvement funding davenport open application for round of dream home improvement funding trump say sweeneys ad is hottest american eagle stock go wild a the great new jersey denizen yogi berra observed it deja vu all over again noncompete clause are under fire in new jersey once more how many woman on the board fewer company are saying mtg sour on republican party claim gop turned it back on america first for tax paid minnesota offer a taxpayer receipt for where dollar go pic of woman at tx capitol fighting to use woman bathroom sum up how dumb transmovement really is search for suspect in tennessee killing focus near university source say a rd arrest announced all major la vega strip casino are unionized defying national trend all major la vega strip casino are unionized defying national trend sex offender harassed marjorie taylor greene turn on gop for abandoning maga base officer find teen girl when arresting man for sex trafficking mpd say mamdani study america worst mayor brandon johnson to avoid his political pitfall report now i love her ad trump praise sydney sweeney amid jean ad fallout ap news summary at pm edt ap news summary at pm edt donald trump and the deconstruction of america mitch mcconnells legacy come under fire in kentucky race to replace him in the senate men accused of shooting up woman glenburn home and car trump shootthemessenger tactic will only hurt the economy more america best idea is under fierce attack u rep kelly morrison introduces legislation to boost police recruitment funding these epstein revelation show the deep state is real and it work for trump mary moriarty dont accept simplistic narrative on carjacking prosecution texas dems flee to illinois to block redistricting vote texas dems flee to illinois to block redistricting vote copy famine in gaza ocean city mayor vow further effort on ebike safety after nearly hitting rider with democrat out of state whats next for texas special session trump threatens to substantially raise tariff on indian good a it continues to buy russian oil trump threatens to substantially raise tariff on indian good a it continues to buy russian oil mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate every minute is crucial here israeli journalist on hostage held inside gaza michta published in realcleardefense and featured in realclearworld on nato and european security nyt claim many jewish voter back mamdani you wont believe who they interviewed college grad compete with ai for entrylevel job guest commentary cpuc dont saddle monterey peninsula ratepayer with desalination project celtic minority owner offer recordbreaking amount to buy move wnba team report mr william bill sander dubose sr how the supreme court kickstarted the redistricting arm race minnesota department of correction expands online application for visitor at adult facility state department may require visa applicant to post bond of up to to enter the u trump administration wont say why it transferred ghislaine maxwell to a minimumsecurity prison new law to make new hampshire library record available to parent grammywinner doechii bringing tour to san diego mortgage lender stick with bidenera reappraisal guidance white south african farm owner on trial for allegedly murdering two black woman and feeding their body to pig trump to substantially raise tariff on india for buying russian oil banana republic stuff top economist react to trump firing bls statistic chief ghislaine maxwell prison transfer add to trump epstein morass look on cnn host face a lee zeldin politely take her climate change b apart is priceless watch texas hold em gov abbott threatens legal action for absent dems mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate mitch mcconnells legacy come under fire in kentucky race to replace him in the senate letter ballroom location not a good idea ap news summary at pm edt new u visa rule could require bond from visitor it feel le like advertising and more like brainwashing mainer injured when their utv rolled over in nh gravel pit former ct chief state attorney fined in ethic case what to know texas house issue arrest warrant for rogue democrat who fled to blue state rep nancy mace is latest republican to announce bid for south carolina governor minnesota congresswoman call for more police recruitment funding why dozen of democrat left texas and how republican want to punish them why dozen of democrat left texas and how republican want to punish them why dozen of democrat left texas and how republican want to punish them why dozen of democrat left texas and how republican want to punish them</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>when independent contractor are actually employee lesson from the m steadfast medical staffing judgment coursera cour q earnings call transcript ap business summarybrief at pm edt cohu q revenue rise wayfair post m q profit revenue up to b trump narrow fed chair candidate to four excluding treasury secretary bessent trump narrow fed chair candidate to four excluding treasury secretary bessent service sector slows down in july rural grocery store pilot project aim to prevent food desert in north dakota rural grocery store pilot project aim to prevent food desert in north dakota texas community q net jump trump say bank discriminate against conservativesincluding him the wall street journal microsoft cloud and ai revenue soar tevogenai expands collaboration with databricks and microsoft to build the beta version of it predictcelltm model with a focus on oncology trump administration officially end thing email for federal employee cbs news citizen bet on open banking to ease account switching best free tech book to read online cftc eye spot crypto trading on future market public opinion due august arabica coffee price sharply higher on brazil coffee crop concern danica mason named among top female entrepreneur build equity from the ground up with red team go franklin resource q revenue beat fincen seeing scam urge bank beware crypto atm mel gordon appointed ceo of chronicle heritage signaling a new era of stability and scalable growth cardano ada face new challenger a rollblock presale heat up with x speculation weave q revenue jump ensign ensg q earnings call transcript real estate expert kim nicols offer insight on buying luxury real estate in granite bay in hellonation magazine former x ceo yaccarino take helm at glp focused telehealth firm emed reuters california marijuana grower said employee were among hundred detained in immigration raid california marijuana grower said employee were among hundred detained in immigration raid u pressure tsmc to buy intel stake for taiwan tariff relief vertical aerospace move beyond can it fly with aciturri deal in focus linda yaccarino join health tech platform emed a ceo after leaving x techcrunch intels a chip woe low yield delay panther lake production gold technical setup turn bullish with job miss and cpi ahead michael novogratz say bitcoin ethereum treasury frenzy may be over what now join sdccu for free resource on national financial awareness day investor alert investigation of bellring brand inc brbr announced by holzer holzer llc gainey mckenna egleston announces a class action lawsuit ha been filed against lineage bed bath beyond could be headed your way here whats next for the revived retail chain bed bath beyond could be headed your way here whats next for the revived retail chain real good food announces corporate action requesting transfer of share to transfer agent johnson fistel investigates fairness of proposed sale of staar surgical johnson fistel commences investigation of agilon health inc birdie bringing froyo back with plan for location in west village week of july morning news rating today move back to first in demo ethereum news today ethereum etf see record m outflow a blackrock lead withdrawal gainey mckenna egleston announces a class action lawsuit ha been filed against lineage inc line sprott inc declares second quarter dividend featuring locus control report find landfill methane monitoring and tuning system among lowest cost ghg reduction sprott inc declares second quarter dividend middleton co inc ma sell share of procter gamble company the nysepg thoroughbred financial service llc acquires share of procter gamble company the nysepg palantir ceo warns of america ai danger zone a he plan to bring superpower to bluecollar worker fortune roku expands streaming option with new adfree service at month century complete expands to nevada with new home in pahrump replenish nutrient announces beiseker facility update crypto news today sharplink boost eth holding figure plan public listing galaxy mull tokenized stock paramount skydance board to include david ellison sherry lansing oracle safra catz the fda is targeting orange juice here why and what the science say the washington post introducing transparent lab grassfed protein shake the protein shake thor drink built to scale how barak diskin bridge real estate and startup growth westfield capital management co lp decrease stock position in alphabet inc nasdaqgoog alphabet inc nasdaqgoog position cut by atrium wealth solution inc syntegra private wealth group llc ha position in alphabet inc nasdaqgoog inspire medical system analyst lower their forecast after q result meta illegally collected data from flo period and pregnancy app jury find ar technica examining the future niagen bioscience earnings outlook earnings outlook for jack in the box a look ahead innovative ind props earnings forecast insight into helmerich paynes upcoming earnings a look ahead horace mann educatorss earnings forecast whats next honest co earnings preview what are the best smart glass of herbalife earnings preview rosen law firm urge novo nordisk a nyse nvo investor with loss in excess of k to contact the firm for information about their right a glimpse of genco shipping trading earnings potential a look ahead fastlys earnings forecast examining the future national vision holdingss earnings outlook earnings outlook for oscar health spotlight on mercadolibre analyzing the surge in option activity this is what whale are betting on philip morris intl a look into citigroup inc price over earnings is the market bullish or bearish on msc industrial direct co how is the market feeling about alphabet infoblox appoints joshua husk a chief revenue officer to accelerate global growth whats driving the market sentiment around caretrust reit bullet blockchain announces strategic initiative to accelerate growth and cement market leadership wyoming average gas price fall by cent per gallon in past week shiba inu shib may miss the mark but analyst say ruvi ai ruvi coinmarketcap listing powered surge ha it closer than ever novo nordisk expands legal action to protect u patient from unsafe nonfdaapproved compounded semaglutide pr newswire infoblox appoints joshua husk a chief revenue officer to accelerate global growth bullet blockchain announces strategic initiative to accelerate growth and cement market leadership beer institute release june taxable removal estimate report porsche gt r with manthey package arrives at porsche track experience buzz wear off for michigan marijuana business best meme coin to invest in today little pepe lilpepe to rally like pepe coin pepe did in cold wallet cashback utility set new standard while sol aim for doge eye target william raveis named top luxury brokerage at inman golden i club award beer institute release june taxable removal estimate report trump administration end musk controversial five thing email for federal worker live now ncsl hold discussion on citizenship and voting ag completes expansion of cold case unit trump give coal a boost gut renewables and will return haze to the four corner opinion trump narrow fed chair candidate to four excluding treasury secretary bessent track live update michigan primary election result track live result detroit mayoral primary election endoflease eviction allowed under new state law editorial quire served community with honor compassion texas ag asks judge to officially remove awol dems from seat this texas republican stalked trump to get his endorsementand flopped trump firing of bureau of labor statistic commissioner will prove damaging woof watch don lemon bonkers trumptrashing therapy session with the runaway texas dem disaster video federal judge blast republican for trying to pas obviously unconstitutional law city council approves limited shortterm rental in centertown overlay sjc confines zoning standing analysis to actual proposed use speculation a to future us is irrelevant time for yall to love america again texas dems in illinois call on republican to be brave ap news summary at pm edt trump take an unexpected walk on the white house roof to survey new project trump plan to take over gaza aid effort u official say opinion with harris out who lead california governor race pentagon keep a lid on golden dome marjorie taylor greene call for george santos year sentence to be commuted editorial the fed wa right to say no on interest rate banihashemi what possibility is there for true reform in iran garrity boiled frog syndrome they decided to cheat national democrat gov jb pritzker vow to do whatever it take to win redistricting battle well well what do we have here ethic committee rip aoc for spouse shenanigan and hooboy thread ayotte sign bill to tighten absentee voting ensure accessible voting exportsmouth teen pleads guilty to charge related to hatemotivated vandalism spree trump admin unveils rule to unleash american drone dominance eagle running back saquon barkley decline invitation to join trump sport council tulsi gabbard tell pod force one she belief there may be alien and still ha a lot of question on nj drone trump will restore a confederate monument in the nation capital justice department to seek federal hate crime charge and death penalty in killing of israeli embassy staffer the state of america judiciary with judge j michael luttig there it is jasmine crockett admits dems lose when voter id is the law of the land watch election is on democrat see opportunity and a wide open primary why spanish fighter jet are patrolling iceland sky raising deposit insurance limit would cost consumer over billion henderson state lawmaker running for dina titus house seat ct put back on federal list of sanctuary jurisdiction why the state top lawyer disagrees house committee issue subpoena for epstein file and deposition with the clinton republican next redistricting target missouri port will kirsten baesler be confirmed for a spot in the trump administration trump jack smith probe isnt just hypocritical it could backfire spectacularly u government proposes easing some restriction on drone traveling long distance live now state department spokesperson hold press briefing aug marjorie taylor greene call for george santos year sentence to be commuted marjorie taylor greene call for george santos year sentence to be commuted trump creates white house task force for los angeles olympics chuck todd worry democratic party hasnt lost enough to learn lesson change course aws announces general availability of amazon elastic vmware service trump plan drug tariff of up to live now texas house hold legislative session day after democrat flee state gop congressman face heated town hall where hundred boo him for supporting trump big bill the latest house committee issue subpoena for epstein file deposition with clinton and others palantir book it first billion in quarterly sale and dodge doge axe elizabeth warren go to the mat for mamdani but it the new york post with the takedown eazy grease accelerates multiregional expansion with liquid recovery solution merger building dominant uco collection network african nation have agreed to take deportee from the u what we know about the secretive deal african nation have agreed to take deportee from the u what we know about the secretive deal african nation have agreed to take deportee from the u what we know about the secretive deal african nation have agreed to take deportee from the u what we know about the secretive deal african nation have agreed to take deportee from the u what we know about the secretive deal african nation have agreed to take deportee from the u what we know about the secretive deal african nation have agreed to take deportee from the u what we know about the secretive deal african nation have agreed to take deportee from the u what we know about the secretive deal a former rolling stone say the met ha his stolen guitar the museum dispute it sterlington welcome leading private wealth team from morgan lewis new snap rule candy and soda no longer covered in additional state trump and democrat turn rival texas and california into proxy for national power struggle tariff trade and tension donald trump central asia policy massachusetts police training material classify mom for liberty a hate group alongside antifa the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance aug might be one of the shortest day of the year here why from the publisher how to gain enemy and sow mistrust trump take an unexpected walk on the white house roof to survey new project trump take an unexpected walk on the white house roof to survey new project mayor brandon johnson say police fire pension sweetener will make chicago finance far more difficult staa alert monsey firm of wohl fruchter investigating fairness of the sale of staar surgical to alcon justice department open grand jury probe into investigation of trump and russia report nato to coordinate regular and largescale arm delivery to ukraine most will be bought in the u alligator alcatraz ha some new competition the speedway slammer pbgh announces aurora chen a vice president of advisory service sen michael bennet asks fed to allow colorado plan that would let toddler stay on medicaid tesla billion muskcentric gamble marjorie taylor greene urge trump to commute george santos sentence illinois gov pritzker commends texas democrat who fled state to block gop redistricting plan illinois gov pritzker commends texas democrat who fled state to block gop redistricting plan trump tour white house roof hint at further renovation woke men mocked by woman for obnoxious performative drinking habit you guy ruined matcha</t>
+          <t>when independent contractor are actually employee lesson from the m steadfast medical staffing judgment coursera cour q earnings call transcript ap business summarybrief at pm edt cohu q revenue rise wayfair post m q profit revenue up to b trump narrow fed chair candidate to four excluding treasury secretary bessent trump narrow fed chair candidate to four excluding treasury secretary bessent service sector slows down in july rural grocery store pilot project aim to prevent food desert in north dakota rural grocery store pilot project aim to prevent food desert in north dakota texas community q net jump trump say bank discriminate against conservativesincluding him the wall street journal microsoft cloud and ai revenue soar tevogenai expands collaboration with databricks and microsoft to build the beta version of it predictcelltm model with a focus on oncology trump administration officially end thing email for federal employee cbs news citizen bet on open banking to ease account switching best free tech book to read online cftc eye spot crypto trading on future market public opinion due august arabica coffee price sharply higher on brazil coffee crop concern danica mason named among top female entrepreneur build equity from the ground up with red team go franklin resource q revenue beat fincen seeing scam urge bank beware crypto atm mel gordon appointed ceo of chronicle heritage signaling a new era of stability and scalable growth cardano ada face new challenger a rollblock presale heat up with x speculation weave q revenue jump ensign ensg q earnings call transcript real estate expert kim nicols offer insight on buying luxury real estate in granite bay in hellonation magazine former x ceo yaccarino take helm at glp focused telehealth firm emed reuters california marijuana grower said employee were among hundred detained in immigration raid california marijuana grower said employee were among hundred detained in immigration raid u pressure tsmc to buy intel stake for taiwan tariff relief vertical aerospace move beyond can it fly with aciturri deal in focus linda yaccarino join health tech platform emed a ceo after leaving x techcrunch intels a chip woe low yield delay panther lake production gold technical setup turn bullish with job miss and cpi ahead michael novogratz say bitcoin ethereum treasury frenzy may be over what now join sdccu for free resource on national financial awareness day investor alert investigation of bellring brand inc brbr announced by holzer holzer llc gainey mckenna egleston announces a class action lawsuit ha been filed against lineage bed bath beyond could be headed your way here whats next for the revived retail chain bed bath beyond could be headed your way here whats next for the revived retail chain real good food announces corporate action requesting transfer of share to transfer agent johnson fistel investigates fairness of proposed sale of staar surgical johnson fistel commences investigation of agilon health inc birdie bringing froyo back with plan for location in west village week of july morning news rating today move back to first in demo ethereum news today ethereum etf see record m outflow a blackrock lead withdrawal gainey mckenna egleston announces a class action lawsuit ha been filed against lineage inc line sprott inc declares second quarter dividend featuring locus control report find landfill methane monitoring and tuning system among lowest cost ghg reduction sprott inc declares second quarter dividend middleton co inc ma sell share of procter gamble company the nysepg thoroughbred financial service llc acquires share of procter gamble company the nysepg palantir ceo warns of america ai danger zone a he plan to bring superpower to bluecollar worker fortune roku expands streaming option with new adfree service at month century complete expands to nevada with new home in pahrump replenish nutrient announces beiseker facility update crypto news today sharplink boost eth holding figure plan public listing galaxy mull tokenized stock paramount skydance board to include david ellison sherry lansing oracle safra catz the fda is targeting orange juice here why and what the science say the washington post introducing transparent lab grassfed protein shake the protein shake thor drink built to scale how barak diskin bridge real estate and startup growth westfield capital management co lp decrease stock position in alphabet inc nasdaqgoog alphabet inc nasdaqgoog position cut by atrium wealth solution inc syntegra private wealth group llc ha position in alphabet inc nasdaqgoog inspire medical system analyst lower their forecast after q result meta illegally collected data from flo period and pregnancy app jury find ar technica examining the future niagen bioscience earnings outlook earnings outlook for jack in the box a look ahead innovative ind props earnings forecast insight into helmerich paynes upcoming earnings a look ahead horace mann educator earnings forecast whats next honest co earnings preview what are the best smart glass of herbalife earnings preview rosen law firm urge novo nordisk a nyse nvo investor with loss in excess of k to contact the firm for information about their right a glimpse of genco shipping trading earnings potential a look ahead fastlys earnings forecast examining the future national vision holding earnings outlook earnings outlook for oscar health spotlight on mercadolibre analyzing the surge in option activity this is what whale are betting on philip morris intl a look into citigroup inc price over earnings is the market bullish or bearish on msc industrial direct co how is the market feeling about alphabet infoblox appoints joshua husk a chief revenue officer to accelerate global growth whats driving the market sentiment around caretrust reit bullet blockchain announces strategic initiative to accelerate growth and cement market leadership wyoming average gas price fall by cent per gallon in past week shiba inu shib may miss the mark but analyst say ruvi ai ruvi coinmarketcap listing powered surge ha it closer than ever novo nordisk expands legal action to protect u patient from unsafe nonfdaapproved compounded semaglutide pr newswire infoblox appoints joshua husk a chief revenue officer to accelerate global growth bullet blockchain announces strategic initiative to accelerate growth and cement market leadership beer institute release june taxable removal estimate report porsche gt r with manthey package arrives at porsche track experience buzz wear off for michigan marijuana business best meme coin to invest in today little pepe lilpepe to rally like pepe coin pepe did in cold wallet cashback utility set new standard while sol aim for doge eye target william raveis named top luxury brokerage at inman golden i club award beer institute release june taxable removal estimate report trump administration end musk controversial five thing email for federal worker live now ncsl hold discussion on citizenship and voting ag completes expansion of cold case unit trump give coal a boost gut renewables and will return haze to the four corner opinion trump narrow fed chair candidate to four excluding treasury secretary bessent track live update michigan primary election result track live result detroit mayoral primary election endoflease eviction allowed under new state law editorial quire served community with honor compassion texas ag asks judge to officially remove awol dems from seat this texas republican stalked trump to get his endorsementand flopped trump firing of bureau of labor statistic commissioner will prove damaging woof watch don lemon bonkers trumptrashing therapy session with the runaway texas dem disaster video federal judge blast republican for trying to pas obviously unconstitutional law city council approves limited shortterm rental in centertown overlay sjc confines zoning standing analysis to actual proposed use speculation a to future us is irrelevant time for yall to love america again texas dems in illinois call on republican to be brave ap news summary at pm edt trump take an unexpected walk on the white house roof to survey new project trump plan to take over gaza aid effort u official say opinion with harris out who lead california governor race pentagon keep a lid on golden dome marjorie taylor greene call for george santos year sentence to be commuted editorial the fed wa right to say no on interest rate banihashemi what possibility is there for true reform in iran garrity boiled frog syndrome they decided to cheat national democrat gov jb pritzker vow to do whatever it take to win redistricting battle well well what do we have here ethic committee rip aoc for spouse shenanigan and hooboy thread ayotte sign bill to tighten absentee voting ensure accessible voting exportsmouth teen pleads guilty to charge related to hatemotivated vandalism spree trump admin unveils rule to unleash american drone dominance eagle running back saquon barkley decline invitation to join trump sport council tulsi gabbard tell pod force one she belief there may be alien and still ha a lot of question on nj drone trump will restore a confederate monument in the nation capital justice department to seek federal hate crime charge and death penalty in killing of israeli embassy staffer the state of america judiciary with judge j michael luttig there it is jasmine crockett admits dems lose when voter id is the law of the land watch election is on democrat see opportunity and a wide open primary why spanish fighter jet are patrolling iceland sky raising deposit insurance limit would cost consumer over billion henderson state lawmaker running for dina titus house seat ct put back on federal list of sanctuary jurisdiction why the state top lawyer disagrees house committee issue subpoena for epstein file and deposition with the clinton republican next redistricting target missouri port will kirsten baesler be confirmed for a spot in the trump administration trump jack smith probe isnt just hypocritical it could backfire spectacularly u government proposes easing some restriction on drone traveling long distance live now state department spokesperson hold press briefing aug marjorie taylor greene call for george santos year sentence to be commuted marjorie taylor greene call for george santos year sentence to be commuted trump creates white house task force for los angeles olympics chuck todd worry democratic party hasnt lost enough to learn lesson change course aws announces general availability of amazon elastic vmware service trump plan drug tariff of up to live now texas house hold legislative session day after democrat flee state gop congressman face heated town hall where hundred boo him for supporting trump big bill the latest house committee issue subpoena for epstein file deposition with clinton and others palantir book it first billion in quarterly sale and dodge doge axe elizabeth warren go to the mat for mamdani but it the new york post with the takedown eazy grease accelerates multiregional expansion with liquid recovery solution merger building dominant uco collection network african nation have agreed to take deportee from the u what we know about the secretive deal african nation have agreed to take deportee from the u what we know about the secretive deal african nation have agreed to take deportee from the u what we know about the secretive deal african nation have agreed to take deportee from the u what we know about the secretive deal african nation have agreed to take deportee from the u what we know about the secretive deal african nation have agreed to take deportee from the u what we know about the secretive deal african nation have agreed to take deportee from the u what we know about the secretive deal african nation have agreed to take deportee from the u what we know about the secretive deal a former rolling stone say the met ha his stolen guitar the museum dispute it sterlington welcome leading private wealth team from morgan lewis new snap rule candy and soda no longer covered in additional state trump and democrat turn rival texas and california into proxy for national power struggle tariff trade and tension donald trump central asia policy massachusetts police training material classify mom for liberty a hate group alongside antifa the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance the trump administration dismisses most on a federal board overseeing puerto rico finance aug might be one of the shortest day of the year here why from the publisher how to gain enemy and sow mistrust trump take an unexpected walk on the white house roof to survey new project trump take an unexpected walk on the white house roof to survey new project mayor brandon johnson say police fire pension sweetener will make chicago finance far more difficult staa alert monsey firm of wohl fruchter investigating fairness of the sale of staar surgical to alcon justice department open grand jury probe into investigation of trump and russia report nato to coordinate regular and largescale arm delivery to ukraine most will be bought in the u alligator alcatraz ha some new competition the speedway slammer pbgh announces aurora chen a vice president of advisory service sen michael bennet asks fed to allow colorado plan that would let toddler stay on medicaid tesla billion muskcentric gamble marjorie taylor greene urge trump to commute george santos sentence illinois gov pritzker commends texas democrat who fled state to block gop redistricting plan illinois gov pritzker commends texas democrat who fled state to block gop redistricting plan trump tour white house roof hint at further renovation woke men mocked by woman for obnoxious performative drinking habit you guy ruined matcha</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>u tariff on asian mining rig slow bitcoin growth a firm eye canada domestic production outfront medium out q eps drop u auctioning seized m russian superyacht with state room helipad gym spa millennials lead the coffee badging revolt to protest return to office a business push to fill empty seat fortune castleinspired home from metal icon list for million global payment gpn q eps jump blazing new trail minnesota city are considering municipal cannabis store whats going on with ionq share today one gas ogs q net income jump ofsis enforcement overhaul what the july consultation mean for uk sanction compliance titus pressing for information on commodity commission nominee earnings season make it clear ai is the only game in town general dynamic board declares dividend myth about metabolism could be holding you back allegiant algt q earnings call transcript sm entertainment revenue up on new release from riize nct wish strong merch sale chatham cldt eps drop wall street oil gas lending down ytd niit learning system limited niit mt announces q fy apriljune result why opendoor technology stock wa tumbling today rosen a ranked and leading law firm encourages irobot corporation investor to secure counsel before important deadline in security class action irbt deloitte india and embark form a strategic alliance to offer endtoend solution for global capability centre how workplace toxicity played a role in the titan submersible disaster mcdonalds announces nostalgic mcdonaldland meal organic avocado mattress are up to off ahead of labor day phone jewelry linen which product could cost more due to trump india tariff jeff wood join patriot growth insurance service a premier client practice leader claires known for piercing million of teen ear file for chapter nd time since a catastrophic funding model court sends sec back to the drawing board tyson beck celebrity mint release first ever coin design featuring basketball icon dennis rodman new york city board denies mayor adam m in matching campaign fund best hp business laptop in strong pick for smart work beloved brooklyn restaurant from chef baxtrom close august claires known for piercing million of teen ear again file for chapter cliq digital ag dylan medium to vote against proposed share buyback and cliq digital currently no longer considers delisting latest global arabinogalactan market sizeshare worth usd million by at a cagr custom market insight analysis outlook leader report trend forecast segmentation growth rate value swot analysis coupa add tariff impact planning to supply chain tool amgen stock sink a market eye maritides next move how can you borrow less for grad school live will q earnings fuel doordashs dash next rally jenavalve responds to ftc action against proposed edward lifesciences acquisition roger williams university school of law named to best law school for by the princeton review israeli society is living in trauma say frenchisraeli journalist pioneer realty capital secures million dollar bond refinancing for texas student housing project from event to improvement step for turning dash cam alert into driver coaching a cautionary tale state ag prevail with a lump of coal for major investment firm a rally for apple lead wall street higher tween jewelry retailer claires file for second bankruptcy bloombergcom brazil request consultation at world trade organization over trump tariff brazil request consultation at world trade organization over trump tariff smart payment solution launch mony a revolutionary upi app for tourist and nris visiting india apple share pop ahead of trumpcook investment announcement at white house best crypto to buy today arctic pablos entry might be the last golden ticket a shiba inu and cheems revive interest c o r r e c t i o n enercom inc enercom announces andrew rapp senior advisor in the u department of energy a keynote speaker on august th at enercoms th anniversary energy investment conference rhode island writes it own cybersecurity rule for nonbanks ap trending summarybrief at pm edt rosen skilled investor counsel encourages lockheed martin corporation investor to secure rosen skilled investor counsel encourages lockheed martin corporation investor to secure counsel before important deadline in security class action lmt china fight mosquitoborne chikungunya virus with drone fine and net a thousand fall ill a preview of sabre earnings preview relay therapeutics earnings direct equity source featured in exclusive qa with two time emmy award winner jim knox a look ahead realreals earnings forecast claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since a look ahead advanced drainage systemss earnings forecast earnings outlook for warby parker snap stock is falling wednesday whats going on u is auctioning a seized m russian superyacht with state room a helipad a gym and a spa cloudsquare unveils new website and brand direction cementing it role a the leading lending platform for alternative finance we want to get there first and claim that for america nasa chief explains push for nuclear reactor on the moon video space walker dunlops earnings a preview exploring construction partnerss earnings expectation tesla cfo taneja excfo kirkhorn named in robotaxi shareholder suit altura join kuviai to enable ai agent in blockchain gaming earnings preview for peloton interactive mapped america hottest zip code revealed region by region realtorcom a peek at dwave quantum future earnings preview penn entertainment earnings rdo equipment co announces layoff delta exchange launch tracker a gamechanging alternative to spot crypto trading behind the scene of caterpillar latest option trend volatility isnt just a metric anymore it driving market structure cava group option frenzy what you need to know jen pawol will be major league baseball first woman to umpire in a regularseason game this weekend mother issue heartbreaking warning after son dy taking popular natural supplement ladbible best hacking surveillance game in origis energy and pioneer community energy announce year solar battery storage agreement richmond american community hosting open house in saratoga spring glencore scrap london listing move missed binance coin bnb roi analyst say ruvi ai ruvi could be your last chance to catch similar gain a phase nears end ethena gain vechain expands but cold wallet cwt token could be the hidden x crypto for adam zyglis cook getting messy suspected south american gang member arrested in maine by border patrol opinion with trump and ice involved los angeles shouldnt host the olympics midair skydiving collision over flathead county leaf one dead moran and marshall lied by omission myth about metabolism could be holding you back pekin restaurant currently closed due to unexpected plumbing issue should professional athlete still be role model the ethical life podcast return national park service to reinstall confederate statue felled by blm mob in should professional athlete still be role model the ethical life podcast gop rep cory mill accused by exgirlfriend of threatening to release sexually explicit image video of her cnn politics texas democrat loses touch with reality compare redistricting to the holocaust rosen a ranked and leading law firm encourages irobot corporation investor to secure counsel before important deadline in security class action irbt cincinnati brawl victim want onlooker who didnt help prosecuted rfk jr launch crackdown on kratom legal morphine substance often found in smoke shop product jonah goldberg kamala harris wont cure what ail the democratic party tim burchett signal hed take blackburn senate seat if she becomes governor once again demanding answer mahmoud khalils terrorist support and his unjustified presence in america former state worker and environmental advocate launch independent run for maine governor roger williams university school of law named to best law school for by the princeton review israeli society is living in trauma say frenchisraeli journalist ucla in talk with trump administration to end m freeze analysis lebanon decision on weapon corner hezbollah watch fox news rave about trump weird white house roof walk james city county police announces school zone speed camera installation former ct criminal justice official pay to resolve ethic complaint denies wrongdoing rosen skilled investor counsel encourages lockheed martin corporation investor to secure counsel before important deadline in security class action lmt china fight mosquitoborne chikungunya virus with drone fine and net a thousand fall ill the latest putin host trump envoy witkoff for crucial talk on ukraine peace deal rep jolanda jones apologizes for comparing texas redistricting plan to holocaust political analyst say if kamala slam biden in her book his team will level her crisp trump suit perfectly our national cognitive dissonance trump say he may deploy national guard in dc editorial redistricting a cynical power play by politician rowley six month into his presidency donald trump ha created a police state se cupp to trump truth is only what he want it be trump envoy witkoff meet putin ahead of russiaukraine peace deadline trump envoy witkoff meet putin ahead of russiaukraine peace deadline jen pawol will be major league baseball first woman to umpire in a regularseason game this weekend the death of highspeed rail not so fast editorial ai help rapidly crack yearlong mystery in alp platte county senator nominated by trump to serve in administration ocean city to consider declaring condemned condo in need of rehabilitation what are cool roof and how do they work india paid the price for underestimating china pl missile disgusting tom homan skewer farleft dem declaring her allegiance to foreign nation over her own country will doj crackdown prompt sanctuary jurisdiction to alter immigration policy democratic politician at iowa state fair john seiler next state school chief will follow delinquent thurmond despite court order federal official use penske truck to trick and arrest immigrant in la several state threaten to redraw congressional map after texas kick off fight several state threaten to redraw congressional map after texas kick off fight several state threaten to redraw congressional map after texas kick off fight several state threaten to redraw congressional map after texas kick off fight several state threaten to redraw congressional map after texas kick off fight several state threaten to redraw congressional map after texas kick off fight several state threaten to redraw congressional map after texas kick off fight democracy be damned texas and california plot dueling congressional gerrymander raap policy study release solving for access and affordability pdabs are not the answer several state threaten to redraw congressional map after texas kick off fight soldier shot before arrest made at army fort stewart in georgia soldier wounded in mass shooting at fort stewart in georgia independentminor party candidate join luzerne county ballot to woody allen epstein wa dracula serviced by young female vampire u sanction narcorapper el makabelico who laundered streaming proceeds to bloodthirsty mexican drug lord a massive u measles outbreak ha slowed but the start of the school year brings renewed risk of spread stanford student newspaper sue trump administration over use of immigration law to target propalestinian student why moderate dems scapegoat bibi dems should drop green energy and other commentary appeal court directs jeffco judge to reconsider releasing man car from lakewood police custody how trump is exploiting musk big ball pritzker democrat vow to win redistricting battle in the wild of the anaconda range expert say elusive gunman ha advantage over searcher pritzker democrat vow to win redistricting battle copy missouri gop see redistricting call a opening for limiting constitutional amendment rising dem star say party isnt playing dead amid gerrymandering chaos from gop bully fort stewart lockdown five soldier shot in active shooter incident dozen killed seeking aid in gaza a israel weighs further military action lawrence odonnell shred trump for playing dumb on ghislaine maxwell prison transfer drill sergeant are back hegseth reinstates practice to make basic great again bridge result for aug tribal group assert sovereignty a fed crack down on genderaffirming care tribal group assert sovereignty a fed crack down on genderaffirming care what to know about mrna vaccine what to know about mrna vaccine lunar lunacy cbs morning host worried colonization could harm the moon indigenous population wut openai is practically giving chatgpt to the government for free trump hate all democrat not just mamdani reader commentary leftist agitator disrupt trump official at student event in washington dc the mindful minute by jon heydenreich funny dozen killed seeking aid in gaza a israel weighs further military action dozen killed seeking aid in gaza a israel weighs further military action indycar distance itself from speedway slammer immigration detention facility defiance over compliance harvard med school continuing to use racial preference complaint say opinion trump destroys our source of information about job this is beyond irresponsible how form of pay got issued to exst louis comptroller mistake and bigger mistake the u dragon lady celebrated it th anniversary with a historic flight america is prepared for a strike on our nuclear weapon deadline alert faruqi faruqi llp investigates claim on behalf of investor of altimmune the real reason democrat are panicking about redistricting support at work central ohio workforce development network launch employee resource network to help employee thrive</t>
+          <t>u tariff on asian mining rig slow bitcoin growth a firm eye canada domestic production outfront medium out q eps drop u auctioning seized m russian superyacht with state room helipad gym spa millennials lead the coffee badging revolt to protest return to office a business push to fill empty seat fortune castleinspired home from metal icon list for million global payment gpn q eps jump blazing new trail minnesota city are considering municipal cannabis store whats going on with ionq share today one gas ogs q net income jump ofsis enforcement overhaul what the july consultation mean for uk sanction compliance titus pressing for information on commodity commission nominee earnings season make it clear ai is the only game in town general dynamic board declares dividend myth about metabolism could be holding you back allegiant algt q earnings call transcript sm entertainment revenue up on new release from riize nct wish strong merch sale chatham cldt eps drop wall street oil gas lending down ytd niit learning system limited niit mt announces q fy apriljune result why opendoor technology stock wa tumbling today rosen a ranked and leading law firm encourages irobot corporation investor to secure counsel before important deadline in security class action irbt deloitte india and embark form a strategic alliance to offer endtoend solution for global capability centre how workplace toxicity played a role in the titan submersible disaster mcdonalds announces nostalgic mcdonaldland meal organic avocado mattress are up to off ahead of labor day phone jewelry linen which product could cost more due to trump india tariff jeff wood join patriot growth insurance service a premier client practice leader claires known for piercing million of teen ear file for chapter nd time since a catastrophic funding model court sends sec back to the drawing board tyson beck celebrity mint release first ever coin design featuring basketball icon dennis rodman new york city board denies mayor adam m in matching campaign fund best hp business laptop in strong pick for smart work beloved brooklyn restaurant from chef baxtrom close august claires known for piercing million of teen ear again file for chapter cliq digital ag dylan medium to vote against proposed share buyback and cliq digital currently no longer considers delisting latest global arabinogalactan market sizeshare worth usd million by at a cagr custom market insight analysis outlook leader report trend forecast segmentation growth rate value swot analysis coupa add tariff impact planning to supply chain tool amgen stock sink a market eye maritides next move how can you borrow le for grad school live will q earnings fuel doordashs dash next rally jenavalve responds to ftc action against proposed edward lifesciences acquisition roger williams university school of law named to best law school for by the princeton review israeli society is living in trauma say frenchisraeli journalist pioneer realty capital secures million dollar bond refinancing for texas student housing project from event to improvement step for turning dash cam alert into driver coaching a cautionary tale state ag prevail with a lump of coal for major investment firm a rally for apple lead wall street higher tween jewelry retailer claires file for second bankruptcy bloombergcom brazil request consultation at world trade organization over trump tariff brazil request consultation at world trade organization over trump tariff smart payment solution launch mony a revolutionary upi app for tourist and nris visiting india apple share pop ahead of trumpcook investment announcement at white house best crypto to buy today arctic pablos entry might be the last golden ticket a shiba inu and cheems revive interest c o r r e c t i o n enercom inc enercom announces andrew rapp senior advisor in the u department of energy a keynote speaker on august th at enercoms th anniversary energy investment conference rhode island writes it own cybersecurity rule for nonbanks ap trending summarybrief at pm edt rosen skilled investor counsel encourages lockheed martin corporation investor to secure rosen skilled investor counsel encourages lockheed martin corporation investor to secure counsel before important deadline in security class action lmt china fight mosquitoborne chikungunya virus with drone fine and net a thousand fall ill a preview of sabre earnings preview relay therapeutics earnings direct equity source featured in exclusive qa with two time emmy award winner jim knox a look ahead realreals earnings forecast claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since claires known for piercing million of teen ear file for chapter nd time since a look ahead advanced drainage system earnings forecast earnings outlook for warby parker snap stock is falling wednesday whats going on u is auctioning a seized m russian superyacht with state room a helipad a gym and a spa cloudsquare unveils new website and brand direction cementing it role a the leading lending platform for alternative finance we want to get there first and claim that for america nasa chief explains push for nuclear reactor on the moon video space walker dunlops earnings a preview exploring construction partner earnings expectation tesla cfo taneja excfo kirkhorn named in robotaxi shareholder suit altura join kuviai to enable ai agent in blockchain gaming earnings preview for peloton interactive mapped america hottest zip code revealed region by region realtorcom a peek at dwave quantum future earnings preview penn entertainment earnings rdo equipment co announces layoff delta exchange launch tracker a gamechanging alternative to spot crypto trading behind the scene of caterpillar latest option trend volatility isnt just a metric anymore it driving market structure cava group option frenzy what you need to know jen pawol will be major league baseball first woman to umpire in a regularseason game this weekend mother issue heartbreaking warning after son dy taking popular natural supplement ladbible best hacking surveillance game in origis energy and pioneer community energy announce year solar battery storage agreement richmond american community hosting open house in saratoga spring glencore scrap london listing move missed binance coin bnb roi analyst say ruvi ai ruvi could be your last chance to catch similar gain a phase nears end ethena gain vechain expands but cold wallet cwt token could be the hidden x crypto for adam zyglis cook getting messy suspected south american gang member arrested in maine by border patrol opinion with trump and ice involved los angeles shouldnt host the olympics midair skydiving collision over flathead county leaf one dead moran and marshall lied by omission myth about metabolism could be holding you back pekin restaurant currently closed due to unexpected plumbing issue should professional athlete still be role model the ethical life podcast return national park service to reinstall confederate statue felled by blm mob in should professional athlete still be role model the ethical life podcast gop rep cory mill accused by exgirlfriend of threatening to release sexually explicit image video of her cnn politics texas democrat loses touch with reality compare redistricting to the holocaust rosen a ranked and leading law firm encourages irobot corporation investor to secure counsel before important deadline in security class action irbt cincinnati brawl victim want onlooker who didnt help prosecuted rfk jr launch crackdown on kratom legal morphine substance often found in smoke shop product jonah goldberg kamala harris wont cure what ail the democratic party tim burchett signal hed take blackburn senate seat if she becomes governor once again demanding answer mahmoud khalils terrorist support and his unjustified presence in america former state worker and environmental advocate launch independent run for maine governor roger williams university school of law named to best law school for by the princeton review israeli society is living in trauma say frenchisraeli journalist ucla in talk with trump administration to end m freeze analysis lebanon decision on weapon corner hezbollah watch fox news rave about trump weird white house roof walk james city county police announces school zone speed camera installation former ct criminal justice official pay to resolve ethic complaint denies wrongdoing rosen skilled investor counsel encourages lockheed martin corporation investor to secure counsel before important deadline in security class action lmt china fight mosquitoborne chikungunya virus with drone fine and net a thousand fall ill the latest putin host trump envoy witkoff for crucial talk on ukraine peace deal rep jolanda jones apologizes for comparing texas redistricting plan to holocaust political analyst say if kamala slam biden in her book his team will level her crisp trump suit perfectly our national cognitive dissonance trump say he may deploy national guard in dc editorial redistricting a cynical power play by politician rowley six month into his presidency donald trump ha created a police state se cupp to trump truth is only what he want it be trump envoy witkoff meet putin ahead of russiaukraine peace deadline trump envoy witkoff meet putin ahead of russiaukraine peace deadline jen pawol will be major league baseball first woman to umpire in a regularseason game this weekend the death of highspeed rail not so fast editorial ai help rapidly crack yearlong mystery in alp platte county senator nominated by trump to serve in administration ocean city to consider declaring condemned condo in need of rehabilitation what are cool roof and how do they work india paid the price for underestimating china pl missile disgusting tom homan skewer farleft dem declaring her allegiance to foreign nation over her own country will doj crackdown prompt sanctuary jurisdiction to alter immigration policy democratic politician at iowa state fair john seiler next state school chief will follow delinquent thurmond despite court order federal official use penske truck to trick and arrest immigrant in la several state threaten to redraw congressional map after texas kick off fight several state threaten to redraw congressional map after texas kick off fight several state threaten to redraw congressional map after texas kick off fight several state threaten to redraw congressional map after texas kick off fight several state threaten to redraw congressional map after texas kick off fight several state threaten to redraw congressional map after texas kick off fight several state threaten to redraw congressional map after texas kick off fight democracy be damned texas and california plot dueling congressional gerrymander raap policy study release solving for access and affordability pdabs are not the answer several state threaten to redraw congressional map after texas kick off fight soldier shot before arrest made at army fort stewart in georgia soldier wounded in mass shooting at fort stewart in georgia independentminor party candidate join luzerne county ballot to woody allen epstein wa dracula serviced by young female vampire u sanction narcorapper el makabelico who laundered streaming proceeds to bloodthirsty mexican drug lord a massive u measles outbreak ha slowed but the start of the school year brings renewed risk of spread stanford student newspaper sue trump administration over use of immigration law to target propalestinian student why moderate dems scapegoat bibi dems should drop green energy and other commentary appeal court directs jeffco judge to reconsider releasing man car from lakewood police custody how trump is exploiting musk big ball pritzker democrat vow to win redistricting battle in the wild of the anaconda range expert say elusive gunman ha advantage over searcher pritzker democrat vow to win redistricting battle copy missouri gop see redistricting call a opening for limiting constitutional amendment rising dem star say party isnt playing dead amid gerrymandering chaos from gop bully fort stewart lockdown five soldier shot in active shooter incident dozen killed seeking aid in gaza a israel weighs further military action lawrence odonnell shred trump for playing dumb on ghislaine maxwell prison transfer drill sergeant are back hegseth reinstates practice to make basic great again bridge result for aug tribal group assert sovereignty a fed crack down on genderaffirming care tribal group assert sovereignty a fed crack down on genderaffirming care what to know about mrna vaccine what to know about mrna vaccine lunar lunacy cbs morning host worried colonization could harm the moon indigenous population wut openai is practically giving chatgpt to the government for free trump hate all democrat not just mamdani reader commentary leftist agitator disrupt trump official at student event in washington dc the mindful minute by jon heydenreich funny dozen killed seeking aid in gaza a israel weighs further military action dozen killed seeking aid in gaza a israel weighs further military action indycar distance itself from speedway slammer immigration detention facility defiance over compliance harvard med school continuing to use racial preference complaint say opinion trump destroys our source of information about job this is beyond irresponsible how form of pay got issued to exst louis comptroller mistake and bigger mistake the u dragon lady celebrated it th anniversary with a historic flight america is prepared for a strike on our nuclear weapon deadline alert faruqi faruqi llp investigates claim on behalf of investor of altimmune the real reason democrat are panicking about redistricting support at work central ohio workforce development network launch employee resource network to help employee thrive</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>spirit of halloweentown is calling festival ticket go on sale august passenger injured in icon of the sea water slide panel shatter kate spade outlet shopper say this crossbody bag is a timeless accessory and it on sale for only nvr inc announces share repurchase authorization car coffee and clothing are poised to get pricier with new tariff bitcoin news today bitcoin auction for dogwifhat meme cap hit k amid growing nft interest nvr inc announces share repurchase authorization top cryptos to invest before end of august best rakshabandhan tech gift under r taketwo q net booking up fran drescher wont run for sagaftra president a candidate line up for race gold miner earn double the profit of yet still undervalued trump warns of great depression a court weighs billion tariff rollback this small city ha managed to keep rent down since and it a quick train ride from nyc sec end lawsuit against ripple company to pay million fine reuters dow jones today stock surge a major index on track to post solid weekly gain apple extends rally gold at record high level investopedia investor alert morris kandinov llp investigating phh wai pcla and epwk stockholder are encouraged to contact the firm a florida woman posed a a nurse and treated thousand of unsuspecting patient official say gold price jump to record high following surprise u tariff ruling apple stock retake key level after dodging tariff bullet apple stock retake key level after dodging tariff bullet investor business daily trump pursues record billion settlement from ucla over antisemitism claim dwave quantum cash hoard fuel aggressive expansion analyst report parkerhannifin corp minsud announces option grant fat brand open first cobranded round table pizza and fatburger in california openstore shift focus from shopify aggregator to menswear brand run to samsung now for up to off a new tv score off your first order at small the purrfect cat meal service rosen a ranked and leading law firm encourages fiserv inc investor to secure counsel denver employee no longer with the city after incident at cannabis club rosen a ranked and leading law firm encourages fiserv inc investor to secure counsel before important deadline in security class action fi examining the future growgenerations earnings outlook a look at perasos upcoming earnings report a peek at teloss future earnings apple aapl confirms billion u investment after white house tease shore living welcome new realtor to team u global investor launch it smart beta sea etf on the mexican stock exchange joining jet and goau earnings preview for quest resource holding insight into quipt home medical upcoming earnings a preview of hf food group earnings examining the future virtras earnings outlook a look ahead gaia earnings forecast connex credit union data breach expose personal information murphy law firm investigates legal claim a glimpse of synchronoss technologiess earnings potential rosen a ranked and leading law firm encourages flywire corporation investor to secure uncovering potential microvast holdingss earnings preview analyst have this to say about elanco animal health an overview of aris water solutionss earnings deep dive into mirum pharmaceutical stock analyst perspective rating expert outlook abcellera biologics through the eye of analyst demystifying penn entertainment insight from analyst review what analyst rating have to say about iovance biotherapeutics tmobile u unusual option activity unpacking the latest option trading trend in cai unpacking the latest option trading trend in ford motor whats driving the market sentiment around affirm holding what doe the market think about paylocity holding pe ratio insight for jdcom taketwo interactive stock a deep dive into analyst perspective rating what doe the market think about ubs gr popular grocery store supplier file chapter bankruptcy how doe a k hardship withdrawal work and is it smart to take one ripple xrp tron trx poised for gain but trader are watching this crypto for a bigger run in samsung galaxy z fold what make it the best foldable phone cardanos ada lead in the race is in danger ruvi ai ruvi coinmarketcap listing get it industry spotlight a analyst call it the top summer play bofa reiterates buy on alphabet googl a gemini gain traction and kpis hold steady xrp news today xrp rally hit with institutional buying and legal victory in play rosen a ranked and leading law firm encourages flywire corporation investor to secure counsel before important deadline in security class action flyw fed president issue stern warning on lasting price increase trump clash with intels ceo is a crucial test for u chip making market update cmcsa cv expe msi pgr ph unh yum hims final deadline rosen a top ranked law firm encourages hims hers health inc fannie freddie stock offering could come a soon a this year barrons amazon amzn aws unveils amazon evsa new way to run vmware workload in the cloud recordhigh gold price push jeweler to offer gilded veneer to prevent sticker shock best ev penny stock to buy according to hedge fund royal expert reveal hypocrisy of william kates secret greek holiday electric vehicle supply equipment market size will attain usd billion by growing at cagr exclusive report by zion market research global electric vehicle supply equipment market size share trend analysis report electric vehicle supply equipment market size will attain usd billion by growing at cagr exclusive report by zion market research global electric vehicle supply equipment market size share trend analysis report san mateo burger popup start this weekend at coyote point best canadian gold stock to buy according to hedge fund doj asks court to release epstein grand jury evidencebut unclear how much may already be public trump approval rating drop in poll this week but rise slightly in retailer tariffbattered import volume to be weaker in gear for the great outdoors is up to off for this great sale at backcountry cool down anywhere save on this ultra cooling shark fan celebrate cbd day with off sitewide at sunday scaries qqq and friend hit high tech etf thrive despite trade turbulence parent trap star reunite in new movie freakier friday deutsche bank reiterates buy on microsoft msftai driving doubledigit efficiency gain ap business summarybrief at pm edt boar head plan to reopen troubled deli meat plant but report of sanitation problem persist boar head plan to reopen troubled deli meat plant but report of sanitation problem persist intel ceo fire back at trump demand to resign mcdonalds menu brings back classic character for shake meal nvidia nvda get overweight rating a ai capex stay strong into mexican authority accuse adidas of cultural appropriation over new sandal design gold future jump to record high a u imposes tariff on swiss gold bar import amd ai growth story gain steambarclays see room for more upside montgomery county democratic state rep call on senate republican to pas funding for septum friday assorted link opinion direct primary care provides medical treatment the oldfashioned way not sure whats more humiliating meidastouch pushing fake jd vance story or the obama bro who bought it report trump seek billion from ucla over antisemitism claim texas state rep isnt backing down from fighting overtly racist redistricting map investigation stalled while georgia state election board tried to change voting rule justice department subpoena new york ag james a it probe whether she violated trump right photo show israeli demonstrating for the release of hostage and ending the gaza war photo show israeli demonstrating for the release of hostage and ending the gaza war gov gavin newsom appoints new judge to bay area superior court kristi noem slam south park for petty and lazy spoof of her only the liberal nuclear energy now reactor on the moon and at denver airport bauer south carolina former lieutenant governor end gop primary challenge to sen graham bauer south carolina former lieutenant governor end gop primary challenge to sen graham bauer south carolina former lieutenant governor end gop primary challenge to sen graham watchdog group asks for probe of acquisition of qatari jet on trump behalf mandan approves preliminary budget with small property tax increase ap news summary at pm edt israel plan to take over gaza city stir fear for civilian and hostage the latest trump will host armenia and azerbaijan for a white house peace summit exclusive full video show leadup to brutal attack of elderly prolifers by man who dodged prison u global investor launch it smart beta sea etf on the mexican stock exchange exclusive federal law enforcement to begin interviewing unaccompanied migrant child in government custody texas republican vow to go nuclear in redistricting row trump action unlikely to affect fed independence trump tariff are killing f sale is there a better way to manage grizzly bear state urged to step up in matching federal momentum for developing nuclear energy trump considering use of military force against mexican drug cartel what doe occupying gaza accomplish for israel live now texas hold legislative session after democrat lawmaker depart doj asks court to release epstein grand jury evidencebut unclear how much may already be public trump approval rating drop in poll this week but rise slightly in plane cabin fill with toxic smoke a power bank catch fire over the ocean hour away from landing how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very president trump sign debanking executive order horizontal review for bank and credit union are next parent trap star reunite in new movie freakier friday boar head plan to reopen troubled deli meat plant but report of sanitation problem persist intel ceo fire back at trump demand to resign how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very city can make do with fewer public employee florida updated agreement on handling detainee at alligator alcatraz but a month after it opened florida updated agreement on handling alligator alcatraz detainee but a month after it opened trump is asking the supreme court to bless stephen miller racial profiling white house pause public tour amid ballroom construction landrum police chief resigns after year of service minute before gunfire erupted at fort stewart the shooting suspect texted his family saying i love yall uncle say what to know about israel plan to retake gaza city what to know about israel plan to retake gaza city update labrynth launch the red tape index to help america build smarter faster other view millennials are avoiding divorce but their american dream ha changed house republican try to defend medicaid cutsand it go poorly dhs secretary kristi noem truth nuke a reporter pushing dem talking point disguised a question ice family separation are forcing child to parent themselves ap news summary at pm edt columnist helen ubinas my philadelphia inquirer farewell lt governor kounalakis announces switch for governor race to treasurer thomas financial group and phoenix lender service close million usda business possible outcome of a gerrymandering battle royale reason republican redistricting power grab might backfire doe your state have official drink if so what is it here the answer warren call on fed to activate additional capital charge special prosecutor ag bondi assigns to letitia james and adam schiff should scare the hell out of them trumpappointed judge toss contempt finding against administration doj informs judge it will ask supreme court to quickly rule on trump birthright citizenship order epa terminates billion solar for all program what to know about past meeting between putin and his american counterpart germany halt military export to israel for use in gaza amid outcry over netanyahu plan when real life feel like a jurassic park moment pete davidson thought the starstudded audience at the snl special wa terrible just peachy fema tell staff to work for ice or risk getting fired letter to the editor leave the judging to jesus tarantula overcome southwest during mating season right now the worst thing you can be is a racist marc maron fire back at howie mandels comment using donald trump a an example dam if you do dam if dont private berk lake murky future opinion opinion to keep finest city title san diego must clean up it act russia mediterranean flotilla is in a sorry state aquaculture can help produce more u seafood pennsylvania advocate call for shutdown of moshannon after ice detainee death putin say hell end war with ukraine with one major concession trump double reward to million for arrest of venezuela president to face u drug charge blue state throw tantrum over trump food stamp fraud crackdown couple welcome baby born from yearold embryo sen kelly bill help military medic enter civilian career b bombed a smiley face into the ground because it ran out of target jd vance go fishing for trout with uk lammy germany halt military export to israel for use in gaza amid outcry over netanyahu plan germany halt military export to israel for use in gaza amid outcry over netanyahu plan appeal court remove boasbergs contempt order in trump admin deportation case why trump tariff hit poor country with higher rate than rich one diana taurasi endorses caitlin clark joining shortlist of wnba player with signature shoe mixedbreed dog buddy is a sweetheart ready for a welcoming new home a top federal reserve official say dour job data back the case for rate cut a top federal reserve official say dour job data back the case for rate cut a top federal reserve official say dour job data back the case for rate cut common lead a strong opening night for san jose jazz summer fest a top federal reserve official say dour job data back the case for rate cut ap news morton meyerson texas businessman and perot lieutenant dy at why xiaomi succeeded at making electric car but apple failed jim cramer delivers straight talk on tricky sp market top crypto token under that could see big gain in fastestgrowing cryptos in blockdag toncoin cronos tron gaining fast top cryptos under to buy nowozak ai lead the list while nearing m presale momentum and x token growth potential cardano price prediction ada eye x growth but this cheaper crypto might soar x in why clean energy fuel stock raced nearly higher today here why joby aviation stock flew higher in july china ev tipping point racing from to new sale in record time rethinking state government presence in baltimore editorial massachusetts makarevich understandable separation agreement language aid employer in unpaid wage case building growth lane that work in any market weekend binge best family series to watch on hotstar from low market cap to big ambition most promising cryptos in landlord say ruby lius plan for bay property defies commercial common sense rosie odonnell claim abc gonna cancel the view michigan governor tell president trump tariff are hurting auto job fda official return to agency after loomerled ouster cnn lula and putin discus peace in ukraine before u summit after the mustang ford is teasing the return of another beloved car a an ev gizmodo apple ai momentum is building here what it mean for investor top crypto gainer today blockdag stellar uniswap hedera are the one to watch ukraine drone revolution ha exposed a u military vulnerability how to trade in corporate life for your next big idea best meme coin to buy new pepe coin rival is growing faster than pepe when it gained billion market cap in day court rule pension fund position wa not so baseless a to mandate an award of attorney fee new art cafe community space to open in camp washington this summer whistleblower tie clinton campaign to fake russia hack sperry trump meeting with putin pose high stake for the ukraine war and his legacy investor alert pomerantz law firm investigates claim on behalf of investor of agilon health inc agl investor alert pomerantz law firm investigates claim on behalf of investor of inspire medical system inc insp dol resurrects paid program employer can selfreport resolve violation rosen recognized investor counsel encourages lockheed martin corporation investor to secure investor alert pomerantz law firm investigates claim on behalf of investor of national grid rosen recognized investor counsel encourages lockheed martin corporation investor to secure counsel before important deadline in security class action lmt trump pick for the fed fuel an existential threat a central bank independence is targeted jpmorgan say fortune what to know about instagram map location sharing and privacy concern the new york time a gpt launch openai loyalist pushed altman for gptos return citing performance and reliability flipkart freedom sale huge discount on ipad oneplus pad samsung tab top presale cryptos in this month that are breaking funding record cold wallet dexboss aurealone lightchain ai taxloss harvesting part iii investment strategy u fed bowman latest job data stiffens support for three rate cut in california rooftop solar rule in limbo after state supreme court ruling top altcoins to buy blockchainfx presale at might dwarf polkadot and cosmos gain speech by vice chair for supervision bowman on the economic outlook and community banking federal reserve board gov irs white house clashed over immigrant data before tax chief wa ousted u fed bowman latest job data stiffens support for three rate cut in reuters fed bowman call for community bank reform favor rate cut these are dead decision zelensky reject ceding territory after trump talk landswap fed bowman back a september rate cut the wall street journal thumzup medium corporation announces update to the term of it proposed public offering im what is the perfect growth etf to pair with voo for longterm wealth reddit stock pop after a blowout quarter but is it a buy best crypto to buy this month magacoin finance gain whale support from solana and doge polk county chamber of commerce ha new home from hollywood to silicon valley how eventbrites ceo bet k on a phone closet startup is qualcomm the best semiconductor stock to buy right now best crypto to buy now blockdag shiba inu cardano xrp stand out fpl reach potential rate settlement deep dive american havent saved for retirement state are creating automatic saving plan ai can solve the genz and millennial engagement crisis put yourself in front of the next major investing trend trump tariff are making international stock market great again reason why ozak ai could be the best investment this august x growth still on the table investor alert pomerantz law firm investigates claim on behalf of investor of barnes noble education inc bned why burger cost so much right now trump announces white house press conference to stop violent crime in washington dcdespite historically low rate whitmer told trump in private that michigan auto job depend on a tariff change of course whitmer told trump in private that michigan auto job depend on a tariff change of course how a cia hit on al qaeda ensnared a u citizen in afghanistan byd ev struck by lightning hold up fine your daily dose of insightful news and perspective investor alert pomerantz law firm investigates claim on behalf of investor of exelixis inc exel ai can be used to develop biological and chemical weapon investor alert pomerantz law firm investigates claim on behalf of investor of anika investor alert pomerantz law firm investigates claim on behalf of investor of anika therapeutic inc anik investor alert pomerantz law firm investigates claim on behalf of investor of neogenomics inc neo investor alert pomerantz law firm investigates claim on behalf of investor of praxis precision medicine inc prax how compounding return can help you retire a millionaire even on a modest income investor alert pomerantz law firm investigates claim on behalf of investor of albany international corp ain top new cryptocurrencies to buy in top presale coin to buy today before price jump in the next stage investor alert pomerantz law firm investigates claim on behalf of investor of tronox holding plc trox investor alert pomerantz law firm investigates claim on behalf of investor of confluent inc cflt crew splash down in pacific after return from iss if youd invested in nvidia stock year ago here how much youd have today vinay prasad return to the fda week after his ouster statnewscom farmer consider the good and bad of incorporating artificial intelligence on the farm farmer consider the good and bad of incorporating artificial intelligence on the farm only a blink left to buy in arctic pablo shock market with b toke burned a shiba inu and pudgy penguin rally bathroom tool that save money and water all you need is this simple upgrade reader view essentia aspirus need to do more for duluth laguna niguel man pleads guilty to firing semiautomatic rifle at sheriff helicopter justice department target new york attorney general a trump foe here what to know justice department target new york attorney general a trump foe here what to know man suckerpunched during argument at eureka sport bar charge filed end of racial consent decree poised to change federal hiring sin city economic slump signal wider slowdown the soviet union yakk fighter wa too powerful for it own design wnba coach say female athlete have been subjected to adult toy projectile for century wut trump team push for ouster of top iea official california poverty crisis will hamper newsoms national climb avoid buying this canned coconut milk brand our taste test show it the absolute worst security flaw in web server enables remote code execution cve london police arrest people a propalestinian protester defy new law london police arrest people a propalestinian protester defy new law trump narcos strategy collides with mexico strong opposition to u deployment oc man sentenced to year for la street takeover that left nursing student dead extrump lawyer call president middecade redistricting scheme more brazen than watergate welcome to the next phase of american heist secretary duffy host press conference on one big beautiful bill act and air traffic control trump warns of new great depression if court block his tariff plan it would be all over again why did judge throw out conviction in murder of chris paul grandfather in winstonsalem beto orourke trash texas republican these motherfkers are panicking beto orourke trash texas republican these motherfkers are panicking trump to host news conference to stop violent crime and make dc one of the safest city in the world mexican president rule out trump reported military plan against mexico drug cartel kelly army arrival worried the town fda official return to agency after loomerled ouster illinois gov jb pritzker forgets map exist when slamming antidemocracy gopers over redistricting nyc limit housing discrimination based on criminal background is criminal history history breastfeeding at work redefined puerto rico new code usher in major change to save animal county must mobilize more volunteer to save animal county must mobilize more volunteer diddy lawyer mark geragos say diddy would be trump supporter if pardoned clip of the week old man wanders around on a roofand more the soviet union insane first attempt at an aircraft carrier ag paxton call on california to aid texas in arresting house democrat that left the state ai the road to utopia or dystopia man charged with raping unconscious woman multiple time in irvine trump meeting with putin pose high stake for the ukraine war and his legacy homeland security secretary kristi noem blast illinois leader during visit ambassador mike huckabee slam british pm keir starmer for for condemning israel did uk surrender to nazi and drop food to them doj seek to unseal jeffrey epstein ghislaine maxwell grand jury record chairlift collapse at a resort and leaf at least hurt including person who sustained a spinal cord injury watt rebellion th anniversary renews call for kerner report plan to fight poverty court order reinstatement and back pay for pittsburgh officer fired after taser arrest death restored nagasaki bell ring in year since abomb strong march demand britain break tie with israel howie carr suffolk high sheriff steven tompkins earns his democrat credential government house repair wont break taxpayer reader commentary california focus require id from federal agent end some fear israel face growing global condemnation over military expansion in gaza founder of trump burger chain could be deported after ice arrest bernie sander kick off fighting the oligarchy tour in west virginia the dred scott dissent lincoln loved the three strategic bomber the u air force cant live without la county evacuation warning lifted a canyon fire continues burning national perspective newton third law rule washington politics artifact in u museum explain the outsized role of racism in the nation history did i miss a memo adam schiffs lawyer say mortgage fraud allegation have been debunked trump announces white house press conference to stop violent crime in washington dcdespite historically low rate fda leader resigned after push from big pharma now he back live now texas house hold legislative session on aug for democrat lawmaker to come back investor alert pomerantz law firm investigates claim on behalf of investor of exelixis inc exel hundred defy police brutality to oppose palestine action ban investor alert pomerantz law firm investigates claim on behalf of investor of anika therapeutic inc anik investor alert pomerantz law firm investigates claim on behalf of investor of neogenomics inc neo investor alert pomerantz law firm investigates claim on behalf of investor of praxis precision medicine inc prax the nation capital wait for trump next move a a federal takeover threat loom investor alert pomerantz law firm investigates claim on behalf of investor of albany international corp ain trump planned computer chip tariff spark confusion among business and trading partner investor alert pomerantz law firm investigates claim on behalf of investor of tronox holding plc trox investor alert pomerantz law firm investigates claim on behalf of investor of confluent inc cflt how to keep hezbollah away from power gop seek to game system thats not a noble cause reader commentary larimer county restaurant inspection made aug iran wont allow trumpbacked azerbaijan corridor top aide say he wa on the fbi most wanted list now he running for congress this physicianscientist is taking on trump on behalf of disadvantaged community we are at war bring it on democrat ready to fight dirty to stop trump gerrymandering is despicable chase empsall the time is now to speak out rick hausman the f lightning ii is still the greatest fighter jet in the world france sends crew to keep fatal wildfire from reigniting shaw walz shouldnt run for reelection and fargo poor communication david cone drop new country album if you dont count the money im the richest man in town grand haven twp to discus pair of development past page for august to accused in death of manchester emt retired firefighter ordered held on unrelated charge susan shelley good riddance to cafe penalty lawmaker urge meta to shut down instagram map abysmal at protecting child politics without shame gerrymandering make hypocrisy a political punch line judge block beto orourke from financially supporting texas democrat who left the state local view like caesar rome u feeling more vulnerable pomerantz law firm announces the filing of a class action against tesla inc and certain officer tsla bonior a tribute to the courageous ukrainian people london police arrest demonstrator supporting the banned palestine action group pomerantz law firm announces the filing of a class action against irobot corporation and certain officer irbt brickner navalny an american hero letter to the editor geothermal is way to go letter to the editor pritzker just a hypocrite white house mull inviting zelensky to trumpputin talk in alaska d printing and ai cut nuclear reactor build time to day google test ai finance platform with chatbot and live insight stanford forgoes m cal grant to keep legacy admission boar head to reopen virginia plant after fatal listeria outbreak concern why cold wallet top the list of top crypto to buy with x roi outpacing shiba inus and toncoins gain twenty suspected mossad spy arrested in iran top meme coin in august with massive roi potential aveo capital partner llc decrease position in exxon mobil corporation nysexom shaquille oneal admits family mistake left him lonely in squarefoot home i know i messed up and when i didnt have that i wa lost owner connected to monster energy announce plan to expand thrifty ice cream gasket market is forecasted to reach u billion in say stratview research microelectronics vacuum valve market is forecasted to reach u billion in say stratview research semiconductor fluid conveyance market is forecasted to reach u billion in say stratview research semiconductor seal market is forecasted to reach u billion in say stratview research the debt and deficit problem isnt what you think microelectronics vacuum valve market is forecasted to reach u billion in say stratview research forget shiba inu shib and pepe coin pepe the best meme coin to buy in is still very undervalued semiconductor vacuum valve market is forecasted to reach u billion in say stratview research semiconductor fluid conveyance market is forecasted to reach u billion in say stratview research semiconductor seal market is forecasted to reach u billion in say stratview research gasket market is forecasted to reach u billion in say stratview research last hour to grab blockdag at before price change xrp hype reach key level semiconductor vacuum valve market is forecasted to reach u billion in say stratview research weapon horror film score a box office victory weapon horror film score a box office victory tesla cybertruck is suddenly sold out sort of gizmodo cobblestone capital advisor llc ny decrease stock position in oracle corporation nyseorcl ccm investment group llc purchase new position in chevron corporation nysecvx third ave outlook brightening cbre say largest u retailer to pay million for overcharging customer newsnation new offshore wind study confirms the obvious a malevolently incompetent clown is steering the u clown car financial literacy key term every firstgeneration american should know luxury houseboat rental a growing trend in virginia beach solana price prediction suggests modest gainsozak ai could leave it behind strengthening family community llc acquires share of mcdonalds corporation nysemcd accenture plc nyseacn share bought by covington investment advisor inc coin gaining steam the best altcoin to buy now for major growth largest stock exchange in the world by market cap in designing a weekly financial health check for your truck or fleet best ethereum ecosystem coin by market cap in connor clark lunn investment management ltd acquires new share in eaton corporation plc nyseetn eye on atlantic basin a tropical development likely next week more than half of industry are already shedding worker a telling sign thats accompanied past recession top economist say fortune united flight ua is declaring an emergency and diverting to new york airlive chevron corporation nysecvx share acquired by first american trust fsb linscomb wealth inc ha million stock holding in visa inc nysev northeast financial group inc ha holding in eli lilly and company nyselly business people coborns exec david best tapped to lead cub food nina roza longquan the dragon spring and dark chocolate scoop prize at locarno pro industry award king luther capital management corp trim stake in exxon mobil corporation nysexom a robot cop named parker spark controversy in wealthy maryland county the washington post inflation fed leadership and other key thing to watch this week blockdag achieves m presale milestone in record time solana hold at bnb near bessent say tariff should melt if trade rebalances nik</t>
+          <t xml:space="preserve">spirit of halloweentown is calling festival ticket go on sale august passenger injured in icon of the sea water slide panel shatter kate spade outlet shopper say this crossbody bag is a timeless accessory and it on sale for only nvr inc announces share repurchase authorization car coffee and clothing are poised to get pricier with new tariff bitcoin news today bitcoin auction for dogwifhat meme cap hit k amid growing nft interest nvr inc announces share repurchase authorization top cryptos to invest before end of august best rakshabandhan tech gift under r taketwo q net booking up fran drescher wont run for sagaftra president a candidate line up for race gold miner earn double the profit of yet still undervalued trump warns of great depression a court weighs billion tariff rollback this small city ha managed to keep rent down since and it a quick train ride from nyc sec end lawsuit against ripple company to pay million fine reuters dow jones today stock surge a major index on track to post solid weekly gain apple extends rally gold at record high level investopedia investor alert morris kandinov llp investigating phh wai pcla and epwk stockholder are encouraged to contact the firm a florida woman posed a a nurse and treated thousand of unsuspecting patient official say gold price jump to record high following surprise u tariff ruling apple stock retake key level after dodging tariff bullet apple stock retake key level after dodging tariff bullet investor business daily trump pursues record billion settlement from ucla over antisemitism claim dwave quantum cash hoard fuel aggressive expansion analyst report parkerhannifin corp minsud announces option grant fat brand open first cobranded round table pizza and fatburger in california openstore shift focus from shopify aggregator to menswear brand run to samsung now for up to off a new tv score off your first order at small the purrfect cat meal service rosen a ranked and leading law firm encourages fiserv inc investor to secure counsel denver employee no longer with the city after incident at cannabis club rosen a ranked and leading law firm encourages fiserv inc investor to secure counsel before important deadline in security class action fi examining the future growgenerations earnings outlook a look at perasos upcoming earnings report a peek at teloss future earnings apple aapl confirms billion u investment after white house tease shore living welcome new realtor to team u global investor launch it smart beta sea etf on the mexican stock exchange joining jet and goau earnings preview for quest resource holding insight into quipt home medical upcoming earnings a preview of hf food group earnings examining the future virtras earnings outlook a look ahead gaia earnings forecast connex credit union data breach expose personal information murphy law firm investigates legal claim a glimpse of synchronoss technology earnings potential rosen a ranked and leading law firm encourages flywire corporation investor to secure uncovering potential microvast holding earnings preview analyst have this to say about elanco animal health an overview of aris water solution earnings deep dive into mirum pharmaceutical stock analyst perspective rating expert outlook abcellera biologics through the eye of analyst demystifying penn entertainment insight from analyst review what analyst rating have to say about iovance biotherapeutics tmobile u unusual option activity unpacking the latest option trading trend in cai unpacking the latest option trading trend in ford motor whats driving the market sentiment around affirm holding what doe the market think about paylocity holding pe ratio insight for jdcom taketwo interactive stock a deep dive into analyst perspective rating what doe the market think about ubs gr popular grocery store supplier file chapter bankruptcy how doe a k hardship withdrawal work and is it smart to take one ripple xrp tron trx poised for gain but trader are watching this crypto for a bigger run in samsung galaxy z fold what make it the best foldable phone cardanos ada lead in the race is in danger ruvi ai ruvi coinmarketcap listing get it industry spotlight a analyst call it the top summer play bofa reiterates buy on alphabet googl a gemini gain traction and kpis hold steady xrp news today xrp rally hit with institutional buying and legal victory in play rosen a ranked and leading law firm encourages flywire corporation investor to secure counsel before important deadline in security class action flyw fed president issue stern warning on lasting price increase trump clash with intels ceo is a crucial test for u chip making market update cmcsa cv expe msi pgr ph unh yum hims final deadline rosen a top ranked law firm encourages hims hers health inc fannie freddie stock offering could come a soon a this year barrons amazon amzn aws unveils amazon evsa new way to run vmware workload in the cloud recordhigh gold price push jeweler to offer gilded veneer to prevent sticker shock best ev penny stock to buy according to hedge fund royal expert reveal hypocrisy of william kates secret greek holiday electric vehicle supply equipment market size will attain usd billion by growing at cagr exclusive report by zion market research global electric vehicle supply equipment market size share trend analysis report electric vehicle supply equipment market size will attain usd billion by growing at cagr exclusive report by zion market research global electric vehicle supply equipment market size share trend analysis report san mateo burger popup start this weekend at coyote point best canadian gold stock to buy according to hedge fund doj asks court to release epstein grand jury evidencebut unclear how much may already be public trump approval rating drop in poll this week but rise slightly in retailer tariffbattered import volume to be weaker in gear for the great outdoors is up to off for this great sale at backcountry cool down anywhere save on this ultra cooling shark fan celebrate cbd day with off sitewide at sunday scaries qqq and friend hit high tech etf thrive despite trade turbulence parent trap star reunite in new movie freakier friday deutsche bank reiterates buy on microsoft msftai driving doubledigit efficiency gain ap business summarybrief at pm edt boar head plan to reopen troubled deli meat plant but report of sanitation problem persist boar head plan to reopen troubled deli meat plant but report of sanitation problem persist intel ceo fire back at trump demand to resign mcdonalds menu brings back classic character for shake meal nvidia nvda get overweight rating a ai capex stay strong into mexican authority accuse adidas of cultural appropriation over new sandal design gold future jump to record high a u imposes tariff on swiss gold bar import amd ai growth story gain steambarclays see room for more upside montgomery county democratic state rep call on senate republican to pas funding for septum friday assorted link opinion direct primary care provides medical treatment the oldfashioned way not sure whats more humiliating meidastouch pushing fake jd vance story or the obama bro who bought it report trump seek billion from ucla over antisemitism claim texas state rep isnt backing down from fighting overtly racist redistricting map investigation stalled while georgia state election board tried to change voting rule justice department subpoena new york ag james a it probe whether she violated trump right photo show israeli demonstrating for the release of hostage and ending the gaza war photo show israeli demonstrating for the release of hostage and ending the gaza war gov gavin newsom appoints new judge to bay area superior court kristi noem slam south park for petty and lazy spoof of her only the liberal nuclear energy now reactor on the moon and at denver airport bauer south carolina former lieutenant governor end gop primary challenge to sen graham bauer south carolina former lieutenant governor end gop primary challenge to sen graham bauer south carolina former lieutenant governor end gop primary challenge to sen graham watchdog group asks for probe of acquisition of qatari jet on trump behalf mandan approves preliminary budget with small property tax increase ap news summary at pm edt israel plan to take over gaza city stir fear for civilian and hostage the latest trump will host armenia and azerbaijan for a white house peace summit exclusive full video show leadup to brutal attack of elderly prolifers by man who dodged prison u global investor launch it smart beta sea etf on the mexican stock exchange exclusive federal law enforcement to begin interviewing unaccompanied migrant child in government custody texas republican vow to go nuclear in redistricting row trump action unlikely to affect fed independence trump tariff are killing f sale is there a better way to manage grizzly bear state urged to step up in matching federal momentum for developing nuclear energy trump considering use of military force against mexican drug cartel what doe occupying gaza accomplish for israel live now texas hold legislative session after democrat lawmaker depart doj asks court to release epstein grand jury evidencebut unclear how much may already be public trump approval rating drop in poll this week but rise slightly in plane cabin fill with toxic smoke a power bank catch fire over the ocean hour away from landing how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very president trump sign debanking executive order horizontal review for bank and credit union are next parent trap star reunite in new movie freakier friday boar head plan to reopen troubled deli meat plant but report of sanitation problem persist intel ceo fire back at trump demand to resign how closely do congressional delegation reflect how people vote not very how closely do congressional delegation reflect how people vote not very city can make do with fewer public employee florida updated agreement on handling detainee at alligator alcatraz but a month after it opened florida updated agreement on handling alligator alcatraz detainee but a month after it opened trump is asking the supreme court to bless stephen miller racial profiling white house pause public tour amid ballroom construction landrum police chief resigns after year of service minute before gunfire erupted at fort stewart the shooting suspect texted his family saying i love yall uncle say what to know about israel plan to retake gaza city what to know about israel plan to retake gaza city update labrynth launch the red tape index to help america build smarter faster other view millennials are avoiding divorce but their american dream ha changed house republican try to defend medicaid cutsand it go poorly dhs secretary kristi noem truth nuke a reporter pushing dem talking point disguised a question ice family separation are forcing child to parent themselves ap news summary at pm edt columnist helen ubinas my philadelphia inquirer farewell lt governor kounalakis announces switch for governor race to treasurer thomas financial group and phoenix lender service close million usda business possible outcome of a gerrymandering battle royale reason republican redistricting power grab might backfire doe your state have official drink if so what is it here the answer warren call on fed to activate additional capital charge special prosecutor ag bondi assigns to letitia james and adam schiff should scare the hell out of them trumpappointed judge toss contempt finding against administration doj informs judge it will ask supreme court to quickly rule on trump birthright citizenship order epa terminates billion solar for all program what to know about past meeting between putin and his american counterpart germany halt military export to israel for use in gaza amid outcry over netanyahu plan when real life feel like a jurassic park moment pete davidson thought the starstudded audience at the snl special wa terrible just peachy fema tell staff to work for ice or risk getting fired letter to the editor leave the judging to jesus tarantula overcome southwest during mating season right now the worst thing you can be is a racist marc maron fire back at howie mandels comment using donald trump a an example dam if you do dam if dont private berk lake murky future opinion opinion to keep finest city title san diego must clean up it act russia mediterranean flotilla is in a sorry state aquaculture can help produce more u seafood pennsylvania advocate call for shutdown of moshannon after ice detainee death putin say hell end war with ukraine with one major concession trump double reward to million for arrest of venezuela president to face u drug charge blue state throw tantrum over trump food stamp fraud crackdown couple welcome baby born from yearold embryo sen kelly bill help military medic enter civilian career b bombed a smiley face into the ground because it ran out of target jd vance go fishing for trout with uk lammy germany halt military export to israel for use in gaza amid outcry over netanyahu plan germany halt military export to israel for use in gaza amid outcry over netanyahu plan appeal court remove boasbergs contempt order in trump admin deportation case why trump tariff hit poor country with higher rate than rich one diana taurasi endorses caitlin clark joining shortlist of wnba player with signature shoe mixedbreed dog buddy is a sweetheart ready for a welcoming new home a top federal reserve official say dour job data back the case for rate cut a top federal reserve official say dour job data back the case for rate cut a top federal reserve official say dour job data back the case for rate cut common lead a strong opening night for san jose jazz summer fest a top federal reserve official say dour job data back the case for rate cut ap news morton meyerson texas businessman and perot lieutenant dy at why xiaomi succeeded at making electric car but apple failed jim cramer delivers straight talk on tricky sp market top crypto token under that could see big gain in fastestgrowing cryptos in blockdag toncoin cronos tron gaining fast top cryptos under to buy nowozak ai lead the list while nearing m presale momentum and x token growth potential cardano price prediction ada eye x growth but this cheaper crypto might soar x in why clean energy fuel stock raced nearly higher today here why joby aviation stock flew higher in july china ev tipping point racing from to new sale in record time rethinking state government presence in baltimore editorial massachusetts makarevich understandable separation agreement language aid employer in unpaid wage case building growth lane that work in any market weekend binge best family series to watch on hotstar from low market cap to big ambition most promising cryptos in landlord say ruby lius plan for bay property defies commercial common sense rosie odonnell claim abc gonna cancel the view michigan governor tell president trump tariff are hurting auto job fda official return to agency after loomerled ouster cnn lula and putin discus peace in ukraine before u summit after the mustang ford is teasing the return of another beloved car a an ev gizmodo apple ai momentum is building here what it mean for investor top crypto gainer today blockdag stellar uniswap hedera are the one to watch ukraine drone revolution ha exposed a u military vulnerability how to trade in corporate life for your next big idea best meme coin to buy new pepe coin rival is growing faster than pepe when it gained billion market cap in day court rule pension fund position wa not so baseless a to mandate an award of attorney fee new art cafe community space to open in camp washington this summer whistleblower tie clinton campaign to fake russia hack sperry trump meeting with putin pose high stake for the ukraine war and his legacy investor alert pomerantz law firm investigates claim on behalf of investor of agilon health inc agl investor alert pomerantz law firm investigates claim on behalf of investor of inspire medical system inc insp dol resurrects paid program employer can selfreport resolve violation rosen recognized investor counsel encourages lockheed martin corporation investor to secure investor alert pomerantz law firm investigates claim on behalf of investor of national grid rosen recognized investor counsel encourages lockheed martin corporation investor to secure counsel before important deadline in security class action lmt trump pick for the fed fuel an existential threat a central bank independence is targeted jpmorgan say fortune what to know about instagram map location sharing and privacy concern the new york time a gpt launch openai loyalist pushed altman for gptos return citing performance and reliability flipkart freedom sale huge discount on ipad oneplus pad samsung tab top presale cryptos in this month that are breaking funding record cold wallet dexboss aurealone lightchain ai taxloss harvesting part iii investment strategy u fed bowman latest job data stiffens support for three rate cut in california rooftop solar rule in limbo after state supreme court ruling top altcoins to buy blockchainfx presale at might dwarf polkadot and cosmos gain speech by vice chair for supervision bowman on the economic outlook and community banking federal reserve board gov irs white house clashed over immigrant data before tax chief wa ousted u fed bowman latest job data stiffens support for three rate cut in reuters fed bowman call for community bank reform favor rate cut these are dead decision zelensky reject ceding territory after trump talk landswap fed bowman back a september rate cut the wall street journal thumzup medium corporation announces update to the term of it proposed public offering im what is the perfect growth etf to pair with voo for longterm wealth reddit stock pop after a blowout quarter but is it a buy best crypto to buy this month magacoin finance gain whale support from solana and doge polk county chamber of commerce ha new home from hollywood to silicon valley how eventbrites ceo bet k on a phone closet startup is qualcomm the best semiconductor stock to buy right now best crypto to buy now blockdag shiba inu cardano xrp stand out fpl reach potential rate settlement deep dive american havent saved for retirement state are creating automatic saving plan ai can solve the genz and millennial engagement crisis put yourself in front of the next major investing trend trump tariff are making international stock market great again reason why ozak ai could be the best investment this august x growth still on the table investor alert pomerantz law firm investigates claim on behalf of investor of barnes noble education inc bned why burger cost so much right now trump announces white house press conference to stop violent crime in washington dcdespite historically low rate whitmer told trump in private that michigan auto job depend on a tariff change of course whitmer told trump in private that michigan auto job depend on a tariff change of course how a cia hit on al qaeda ensnared a u citizen in afghanistan byd ev struck by lightning hold up fine your daily dose of insightful news and perspective investor alert pomerantz law firm investigates claim on behalf of investor of exelixis inc exel ai can be used to develop biological and chemical weapon investor alert pomerantz law firm investigates claim on behalf of investor of anika investor alert pomerantz law firm investigates claim on behalf of investor of anika therapeutic inc anik investor alert pomerantz law firm investigates claim on behalf of investor of neogenomics inc neo investor alert pomerantz law firm investigates claim on behalf of investor of praxis precision medicine inc prax how compounding return can help you retire a millionaire even on a modest income investor alert pomerantz law firm investigates claim on behalf of investor of albany international corp ain top new cryptocurrencies to buy in top presale coin to buy today before price jump in the next stage investor alert pomerantz law firm investigates claim on behalf of investor of tronox holding plc trox investor alert pomerantz law firm investigates claim on behalf of investor of confluent inc cflt crew splash down in pacific after return from i if youd invested in nvidia stock year ago here how much youd have today vinay prasad return to the fda week after his ouster statnewscom farmer consider the good and bad of incorporating artificial intelligence on the farm farmer consider the good and bad of incorporating artificial intelligence on the farm only a blink left to buy in arctic pablo shock market with b toke burned a shiba inu and pudgy penguin rally bathroom tool that save money and water all you need is this simple upgrade reader view essentia aspirus need to do more for duluth laguna niguel man pleads guilty to firing semiautomatic rifle at sheriff helicopter justice department target new york attorney general a trump foe here what to know justice department target new york attorney general a trump foe here what to know man suckerpunched during argument at eureka sport bar charge filed end of racial consent decree poised to change federal hiring sin city economic slump signal wider slowdown the soviet union yakk fighter wa too powerful for it own design wnba coach say female athlete have been subjected to adult toy projectile for century wut trump team push for ouster of top iea official california poverty crisis will hamper newsoms national climb avoid buying this canned coconut milk brand our taste test show it the absolute worst security flaw in web server enables remote code execution cve london police arrest people a propalestinian protester defy new law london police arrest people a propalestinian protester defy new law trump narcos strategy collides with mexico strong opposition to u deployment oc man sentenced to year for la street takeover that left nursing student dead extrump lawyer call president middecade redistricting scheme more brazen than watergate welcome to the next phase of american heist secretary duffy host press conference on one big beautiful bill act and air traffic control trump warns of new great depression if court block his tariff plan it would be all over again why did judge throw out conviction in murder of chris paul grandfather in winstonsalem beto orourke trash texas republican these motherfkers are panicking beto orourke trash texas republican these motherfkers are panicking trump to host news conference to stop violent crime and make dc one of the safest city in the world mexican president rule out trump reported military plan against mexico drug cartel kelly army arrival worried the town fda official return to agency after loomerled ouster illinois gov jb pritzker forgets map exist when slamming antidemocracy gopers over redistricting nyc limit housing discrimination based on criminal background is criminal history history breastfeeding at work redefined puerto rico new code usher in major change to save animal county must mobilize more volunteer to save animal county must mobilize more volunteer diddy lawyer mark geragos say diddy would be trump supporter if pardoned clip of the week old man wanders around on a roofand more the soviet union insane first attempt at an aircraft carrier ag paxton call on california to aid texas in arresting house democrat that left the state ai the road to utopia or dystopia man charged with raping unconscious woman multiple time in irvine trump meeting with putin pose high stake for the ukraine war and his legacy homeland security secretary kristi noem blast illinois leader during visit ambassador mike huckabee slam british pm keir starmer for for condemning israel did uk surrender to nazi and drop food to them doj seek to unseal jeffrey epstein ghislaine maxwell grand jury record chairlift collapse at a resort and leaf at least hurt including person who sustained a spinal cord injury watt rebellion th anniversary renews call for kerner report plan to fight poverty court order reinstatement and back pay for pittsburgh officer fired after taser arrest death restored nagasaki bell ring in year since abomb strong march demand britain break tie with israel howie carr suffolk high sheriff steven tompkins earns his democrat credential government house repair wont break taxpayer reader commentary california focus require id from federal agent end some fear israel face growing global condemnation over military expansion in gaza founder of trump burger chain could be deported after ice arrest bernie sander kick off fighting the oligarchy tour in west virginia the dred scott dissent lincoln loved the three strategic bomber the u air force cant live without la county evacuation warning lifted a canyon fire continues burning national perspective newton third law rule washington politics artifact in u museum explain the outsized role of racism in the nation history did i miss a memo adam schiffs lawyer say mortgage fraud allegation have been debunked trump announces white house press conference to stop violent crime in washington dcdespite historically low rate fda leader resigned after push from big pharma now he back live now texas house hold legislative session on aug for democrat lawmaker to come back investor alert pomerantz law firm investigates claim on behalf of investor of exelixis inc exel hundred defy police brutality to oppose palestine action ban investor alert pomerantz law firm investigates claim on behalf of investor of anika therapeutic inc anik investor alert pomerantz law firm investigates claim on behalf of investor of neogenomics inc neo investor alert pomerantz law firm investigates claim on behalf of investor of praxis precision medicine inc prax the nation capital wait for trump next move a a federal takeover threat loom investor alert pomerantz law firm investigates claim on behalf of investor of albany international corp ain trump planned computer chip tariff spark confusion among business and trading partner investor alert pomerantz law firm investigates claim on behalf of investor of tronox holding plc trox investor alert pomerantz law firm investigates claim on behalf of investor of confluent inc cflt how to keep hezbollah away from power gop seek to game system thats not a noble cause reader commentary larimer county restaurant inspection made aug iran wont allow trumpbacked azerbaijan corridor top aide say he wa on the fbi most wanted list now he running for congress this physicianscientist is taking on trump on behalf of disadvantaged community we are at war bring it on democrat ready to fight dirty to stop trump gerrymandering is despicable chase empsall the time is now to speak out rick hausman the f lightning ii is still the greatest fighter jet in the world france sends crew to keep fatal wildfire from reigniting shaw walz shouldnt run for reelection and fargo poor communication david cone drop new country album if you dont count the money im the richest man in town grand haven twp to discus pair of development past page for august to accused in death of manchester emt retired firefighter ordered held on unrelated charge susan shelley good riddance to cafe penalty lawmaker urge meta to shut down instagram map abysmal at protecting child politics without shame gerrymandering make hypocrisy a political punch line judge block beto orourke from financially supporting texas democrat who left the state local view like caesar rome u feeling more vulnerable pomerantz law firm announces the filing of a class action against tesla inc and certain officer tsla bonior a tribute to the courageous ukrainian people london police arrest demonstrator supporting the banned palestine action group pomerantz law firm announces the filing of a class action against irobot corporation and certain officer irbt brickner navalny an american hero letter to the editor geothermal is way to go letter to the editor pritzker just a hypocrite white house mull inviting zelensky to trumpputin talk in alaska d printing and ai cut nuclear reactor build time to day google test ai finance platform with chatbot and live insight stanford forgoes m cal grant to keep legacy admission boar head to reopen virginia plant after fatal listeria outbreak concern why cold wallet top the list of top crypto to buy with x roi outpacing shiba inus and toncoins gain twenty suspected mossad spy arrested in iran top meme coin in august with massive roi potential aveo capital partner llc decrease position in exxon mobil corporation nysexom shaquille oneal admits family mistake left him lonely in squarefoot home i know i messed up and when i didnt have that i wa lost owner connected to monster energy announce plan to expand thrifty ice cream gasket market is forecasted to reach u billion in say stratview research microelectronics vacuum valve market is forecasted to reach u billion in say stratview research semiconductor fluid conveyance market is forecasted to reach u billion in say stratview research semiconductor seal market is forecasted to reach u billion in say stratview research the debt and deficit problem isnt what you think microelectronics vacuum valve market is forecasted to reach u billion in say stratview research forget shiba inu shib and pepe coin pepe the best meme coin to buy in is still very undervalued semiconductor vacuum valve market is forecasted to reach u billion in say stratview research semiconductor fluid conveyance market is forecasted to reach u billion in say stratview research semiconductor seal market is forecasted to reach u billion in say stratview research gasket market is forecasted to reach u billion in say stratview research last hour to grab blockdag at before price change xrp hype reach key level semiconductor vacuum valve market is forecasted to reach u billion in say stratview research weapon horror film score a box office victory weapon horror film score a box office victory tesla cybertruck is suddenly sold out sort of gizmodo cobblestone capital advisor llc ny decrease stock position in oracle corporation nyseorcl ccm investment group llc purchase new position in chevron corporation nysecvx third ave outlook brightening cbre say largest u retailer to pay million for overcharging customer newsnation new offshore wind study confirms the obvious a malevolently incompetent clown is steering the u clown car financial literacy key term every firstgeneration american should know luxury houseboat rental a growing trend in virginia beach solana price prediction suggests modest gainsozak ai could leave it behind strengthening family community llc acquires share of mcdonalds corporation nysemcd accenture plc nyseacn share bought by covington investment advisor inc coin gaining steam the best altcoin to buy now for major growth largest stock exchange in the world by market cap in designing a weekly financial health check for your truck or fleet best ethereum ecosystem coin by market cap in connor clark lunn investment management ltd acquires new share in eaton corporation plc nyseetn eye on atlantic basin a tropical development likely next week more than half of industry are already shedding worker a telling sign thats accompanied past recession top economist say fortune united flight ua is declaring an emergency and diverting to new york airlive chevron corporation nysecvx share acquired by first american trust fsb linscomb wealth inc ha million stock holding in visa inc nysev northeast financial group inc ha holding in eli lilly and company nyselly business people coborns exec david best tapped to lead cub food nina roza longquan the dragon spring and dark chocolate scoop prize at locarno pro industry award king luther capital management corp trim stake in exxon mobil corporation nysexom a robot cop named parker spark controversy in wealthy maryland county the washington post inflation fed leadership and other key thing to watch this week blockdag achieves m presale milestone in record time solana hold at bnb near bessent say tariff should melt if trade rebalances nikkei asia </t>
         </is>
       </c>
     </row>
@@ -1515,7 +1515,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>from power plant to the moon the u nuclear revival in dogecoin jump in a week what is going on teenage mutant ninja turtle pizzeria to debut in la thestreet pro analyst tackle tariff crypto and more in market roundtable solar stock outshine sp in despite policy headwind why share of tesla are soaring today time tracking and trust what today employee really think amazon is selling a storage cart for thats great for small place cold wallet m presale entry beat xrps price test and eths resistance goal why many smallbusinesses owner fear even a short recession will sink them creating a load history tracker that improves rate negotiation crypto news today strategy m bitcoin purchase bullish upsizes ipo alt sigma b fundraising move solana price prediction etf approval could help sol overtake xrp but this cheaper token will rally x and outshine their roi bank of america strategist expect fed to lower interest rate benny brown acquires wide open music publishing form new publishing company affirm stock revisits this place a buy now pay later delight shopper demi lovato reunites with exboyfriend joe jonas for a camp rock performance new pickleball kingdom indoor facility coming soon to south brunswick nj nasfm honor fire chief todd parker for excellence in emergency response virginia obamacare premium set to jump sharply scc report virginia obamacare premium set to jump sharply scc report going online in russia can be frustrating complicated and even dangerous chatgpt get smarter with gpt top feature youll love if youd invested in interactive broker ibkr stock year ago here how much youd have today graphene market to grow at cagr by lynch carpenter investigates claim in pandora data breach neptune frozen treat opening in malaga cove plaza top tech news today taylor swift ai scandal iphone price hike tesla dojo shutdown metas talent war siri upgrade stock market party to be ruined by sudden economic slowdown say stifel cnbc bitcoin hovers around whats next lockheed martin could lose major deal after u hit switzerland with tariff top meme coin to invest for maximum gain in xrp news today analyst react to m xrp transfer to coinbase is it routine move ford hit the pedal on ev production with billion overhaul of kentucky plant fed bowman say job data solidifies case for rate cut u consumer to bear brunt of tariff hit goldman economist say u consumer to bear brunt of tariff hit goldman economist say roll royce share price is on a sizzling hot streak but beware of the danger top laptop brand in the usa in ibd live qa stock list for monday aug why good leader ask great question manufacturer urged to act with technologyfirst plan a disruption intensifies say infotech research group in new report philippe cousteau earthecho international announces diverse youth advocate join the blue carbon ambassador program play the perfect game this summer with flightpath golf tee what to expect from tuesday report on inflation investopedia evercommerce to present at third quarter investor conference evercommerce to present at third quarter investor conference comedic multihyphenate matt mathews sign with wme hurry and grab a macbook air for just at back market air india suspends flight to washington dc amid ongoing tension this is what whale are betting on lockheed martin smart money is betting big in ups option aircraft gasket market is forecasted to reach u million in say stratview research best cryptos to invest in that could deliver massive longterm gain blockdag litecoin stellar toncoin solar stock outshine oil and gas benchmark after climate credit cut aerospace pilot control market is forecasted to reach u billion in say stratview research xml announces launch of new xml woman website relaunch of xml woman division aircraft gasket market is forecasted to reach u million in say stratview research aerospace pilot control market is forecasted to reach u billion in say stratview research diversified foodservice supply appoints lev peker a chief executive officer body armor plate market is forecasted to reach u million in say stratview research body armor plate market is forecasted to reach u million in say stratview research best typec hub for macbook in venchi bringing beloved italian chocolate to century city tegna stock rocket on nexstar merger talk fcc appears set to ease local tv rule in order to smooth deal path deadline btc miner stance on cloud mining in if youd invested in zoetis zts stock year ago here how much youd have today fda may not renew pfizers authorization for covid shot in younger child moderna prepares to boost supply ja mining offer fixed usd yield with crypto deposit alphabet inc nasdaqgoog share acquired by gouws capital llc kohmann bosshard financial service llc purchase share of costco wholesale corporation nasdaqcost gouws capital llc boost stock holding in thermo fisher scientific inc nysetmo ana alsharif became the face of the war in gaza for million then israel killed him home condition made rescue effort difficult pfd protect partner with sentin to pioneer aipowered industrial inspection gear up for the new school year with off therabody best seller wall street biggest bear is expecting a stockmarket pullback this year trump say gold import will not face u tariff bloombergcom irobots future isnt looking up russian seeking asylum in u facing new obstacle say usbased activist morse corp awarded m u army ota for uas development morse corp awarded m u army ota for uas development aem united state ag tractor and combine report july aem united state ag tractor and combine report july scientist say they cruised the ocean in a deepsea submersible and came across an undiscovered ecosystem macys is selling a cozy puma hoodie for thats super soft winnebago industry announces strategic leadership change to drive future growth how to stretch backtoschool budget at salvage store openai and google vet periodic lab seek million investment aol dialup got america online in the s it ending next month trump say gold will not be tariffed cnbc how turmeric water fight inflammation aussivo reveals vision to build blockchainverified cloud trust layer a new standard for transparency in the digital world the viral govee floor lamp is still at prime day price silver at doublevibration support ahead of gann time cluster unit building at rockaway reach completion in brownsville fill up your shopping cart with today best target deal including over off outdoor gear headphone kitchen good and more communication service stock whale activity in today session playhouse under construction for popup park in virginia beach aol is finally disconnecting it dialup internet year on barack obamas official portrait moved to nonpublic area in white house western union ceo ice raid tariff no threat to instamex deal video show moment of explosion at u steel plant in pennsylvania trump gross white house makeover reach petty new low crowded north county field vying to replace brian williams in missouri senate how the world most valuable company got caught in the middle of trump spat with china commentary vance right to call out warped partisan representation why is trump attacking intels ceo demi lovato reunites with exboyfriend joe jonas for a camp rock performance mamdani launch tour of new york city with a message linking cuomo to trump nasfm honor fire chief todd parker for excellence in emergency response what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska trump lash out at crockett renews call for cognitive test lynch carpenter investigates claim in pandora data breach president mayor police chief social worker trump is a man of many hat trump say he and putin will discus ukraine future border israel plan to widen coming offensive beyond gaza city into last area not under it control israel plan to widen coming offensive beyond gaza city into last area not under it control israel plan to widen coming offensive beyond gaza city into last area not under it control u senate candidate set the tone for kentucky republican during statewide dinner what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska photo of trump emergency declaration a the national guard is activated in washington photo of trump emergency declaration a the national guard is activated in washington trump mistake alaska for russia and yes there snark surveillance case test chapter a standing and unfairness standard clinton county sheriff office arrest individual involved with multicounty sex trafficking operation a judge brutal rebuke of trump epstein gambit cnn politics what to know about the putintrump summit in alaska local view give ailing minnesota kid a fighting chance philippe cousteau earthecho international announces diverse youth advocate join the blue carbon ambassador program california couple file lawsuit against klp in conway over shortterm rental rule rubio hit medium over gaza narrative say some ally making it harder to achieve peace multiple men have impersonated ice agent to kidnap and assault woman multiple men have impersonated ice agent to kidnap and assault woman doe using ai dumb you down vote to save a historic building from demolition trump promised to fix inflation he doing this instead south carolina lawmaker awaiting trial on child sex abuse material charge resigns from office nvidia to share of revenue from chip sale to china with u government trump say gold wont face tariff trump say gold wont face tariff trump say gold wont face tariff trump say gold wont face tariff trump say gold wont face tariff ana alsharif became the face of the war in gaza for million then israel killed him trump say he placing washington police under federal control and deploying the national guard trump declares crime in dc will be cleaned up real quick during his announcement that he taking over the city police department chinese ship collide on chase in disputed water ap news summary at pm edt trump say he placing washington police under federal control and activating the national guard houlihan financial resource group ltd sell share of international business machine corporation nyseibm meridian wealth management llc ha million position in broadcom inc nasdaqavgo motley fool asset management llc raise stock holding in broadcom inc nasdaqavgo colorado congressional democrat visit aurora ice facility meet with detained activist jeanette vizguerra colorado congressional democrat visit aurora ice facility meet with detained activist jeanette vizguerra colorado congressional democrat visit aurora ice facility meet with detained activist jeanette vizguerra colorado congressional democrat visit aurora ice facility meet with detained activist jeanette vizguerra russian seeking asylum in u facing new obstacle say usbased activist trump warns protester amid dc crime crack down you spit and we hit trump suggests he can send national guard troop into other u city beyond dc scientist say they cruised the ocean in a deepsea submersible and came across an undiscovered ecosystem dillon associate inc increase holding in salesforce inc nysecrm colombian presidential candidate miguel uribe turbay dy two month after assassination attempt live now texas hold legislative session after democrat leave state jeffries hammer trump for seizing control of dc police no basis jeffries hammer trump for seizing control of dc police no basis jeffries hammer trump for seizing control of dc police no basis jeffries hammer trump for seizing control of dc police no basis jeffries hammer trump for seizing control of dc police no basis maga v miga laura loomer block marjorie taylor greene on social medium escalating a feud over america israel policy trump looking at reclassifying marijuana a less dangerous drug trump looking at reclassifying marijuana a less dangerous drug danish zoo asks for donated pet to feed to carnivore trump looking at reclassifying marijuana a less dangerous drug trump looking at reclassifying marijuana a less dangerous drug trump looking at reclassifying marijuana a less dangerous drug el paso police man dy when he hit tree get ejected trump team get blasted by judge for clumsy epstein diversion raw politics is now driving law enforcement at the department of justice civil right division nancy pelosi get all high and mighty lying about trump j and the ntl guard and oh hell no old woman this candidate for california governor ha a potential conflict of interest in her own home ishares core sp etf nysearcaivv share sold by aveo capital partner llc maine state library not victimized a suggested letter maine state library not victimized a suggested letter here are the country that have recognized a palestinian state johnson fistel investigates fairness of proposed sale of meridianlink currently the most dangerous place maia wealth llc purchase share of ishares core u aggregate bond etf nysearcaagg my wife of year just died my grief is so overwhelming i can barely cope</t>
+          <t>from power plant to the moon the u nuclear revival in dogecoin jump in a week what is going on teenage mutant ninja turtle pizzeria to debut in la thestreet pro analyst tackle tariff crypto and more in market roundtable solar stock outshine sp in despite policy headwind why share of tesla are soaring today time tracking and trust what today employee really think amazon is selling a storage cart for thats great for small place cold wallet m presale entry beat xrps price test and eths resistance goal why many smallbusinesses owner fear even a short recession will sink them creating a load history tracker that improves rate negotiation crypto news today strategy m bitcoin purchase bullish upsizes ipo alt sigma b fundraising move solana price prediction etf approval could help sol overtake xrp but this cheaper token will rally x and outshine their roi bank of america strategist expect fed to lower interest rate benny brown acquires wide open music publishing form new publishing company affirm stock revisits this place a buy now pay later delight shopper demi lovato reunites with exboyfriend joe jonas for a camp rock performance new pickleball kingdom indoor facility coming soon to south brunswick nj nasfm honor fire chief todd parker for excellence in emergency response virginia obamacare premium set to jump sharply scc report virginia obamacare premium set to jump sharply scc report going online in russia can be frustrating complicated and even dangerous chatgpt get smarter with gpt top feature youll love if youd invested in interactive broker ibkr stock year ago here how much youd have today graphene market to grow at cagr by lynch carpenter investigates claim in pandora data breach neptune frozen treat opening in malaga cove plaza top tech news today taylor swift ai scandal iphone price hike tesla dojo shutdown metas talent war siri upgrade stock market party to be ruined by sudden economic slowdown say stifel cnbc bitcoin hovers around whats next lockheed martin could lose major deal after u hit switzerland with tariff top meme coin to invest for maximum gain in xrp news today analyst react to m xrp transfer to coinbase is it routine move ford hit the pedal on ev production with billion overhaul of kentucky plant fed bowman say job data solidifies case for rate cut u consumer to bear brunt of tariff hit goldman economist say u consumer to bear brunt of tariff hit goldman economist say roll royce share price is on a sizzling hot streak but beware of the danger top laptop brand in the usa in ibd live qa stock list for monday aug why good leader ask great question manufacturer urged to act with technologyfirst plan a disruption intensifies say infotech research group in new report philippe cousteau earthecho international announces diverse youth advocate join the blue carbon ambassador program play the perfect game this summer with flightpath golf tee what to expect from tuesday report on inflation investopedia evercommerce to present at third quarter investor conference evercommerce to present at third quarter investor conference comedic multihyphenate matt mathews sign with wme hurry and grab a macbook air for just at back market air india suspends flight to washington dc amid ongoing tension this is what whale are betting on lockheed martin smart money is betting big in ups option aircraft gasket market is forecasted to reach u million in say stratview research best cryptos to invest in that could deliver massive longterm gain blockdag litecoin stellar toncoin solar stock outshine oil and gas benchmark after climate credit cut aerospace pilot control market is forecasted to reach u billion in say stratview research xml announces launch of new xml woman website relaunch of xml woman division aircraft gasket market is forecasted to reach u million in say stratview research aerospace pilot control market is forecasted to reach u billion in say stratview research diversified foodservice supply appoints lev peker a chief executive officer body armor plate market is forecasted to reach u million in say stratview research body armor plate market is forecasted to reach u million in say stratview research best typec hub for macbook in venchi bringing beloved italian chocolate to century city tegna stock rocket on nexstar merger talk fcc appears set to ease local tv rule in order to smooth deal path deadline btc miner stance on cloud mining in if youd invested in zoetis zts stock year ago here how much youd have today fda may not renew pfizers authorization for covid shot in younger child moderna prepares to boost supply ja mining offer fixed usd yield with crypto deposit alphabet inc nasdaqgoog share acquired by gouws capital llc kohmann bosshard financial service llc purchase share of costco wholesale corporation nasdaqcost gouws capital llc boost stock holding in thermo fisher scientific inc nysetmo ana alsharif became the face of the war in gaza for million then israel killed him home condition made rescue effort difficult pfd protect partner with sentin to pioneer aipowered industrial inspection gear up for the new school year with off therabody best seller wall street biggest bear is expecting a stockmarket pullback this year trump say gold import will not face u tariff bloombergcom irobots future isnt looking up russian seeking asylum in u facing new obstacle say usbased activist morse corp awarded m u army ota for uas development morse corp awarded m u army ota for uas development aem united state ag tractor and combine report july aem united state ag tractor and combine report july scientist say they cruised the ocean in a deepsea submersible and came across an undiscovered ecosystem macys is selling a cozy puma hoodie for thats super soft winnebago industry announces strategic leadership change to drive future growth how to stretch backtoschool budget at salvage store openai and google vet periodic lab seek million investment aol dialup got america online in the s it ending next month trump say gold will not be tariffed cnbc how turmeric water fight inflammation aussivo reveals vision to build blockchainverified cloud trust layer a new standard for transparency in the digital world the viral govee floor lamp is still at prime day price silver at doublevibration support ahead of gann time cluster unit building at rockaway reach completion in brownsville fill up your shopping cart with today best target deal including over off outdoor gear headphone kitchen good and more communication service stock whale activity in today session playhouse under construction for popup park in virginia beach aol is finally disconnecting it dialup internet year on barack obamas official portrait moved to nonpublic area in white house western union ceo ice raid tariff no threat to instamex deal video show moment of explosion at u steel plant in pennsylvania trump gross white house makeover reach petty new low crowded north county field vying to replace brian williams in missouri senate how the world most valuable company got caught in the middle of trump spat with china commentary vance right to call out warped partisan representation why is trump attacking intels ceo demi lovato reunites with exboyfriend joe jonas for a camp rock performance mamdani launch tour of new york city with a message linking cuomo to trump nasfm honor fire chief todd parker for excellence in emergency response what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska trump lash out at crockett renews call for cognitive test lynch carpenter investigates claim in pandora data breach president mayor police chief social worker trump is a man of many hat trump say he and putin will discus ukraine future border israel plan to widen coming offensive beyond gaza city into last area not under it control israel plan to widen coming offensive beyond gaza city into last area not under it control israel plan to widen coming offensive beyond gaza city into last area not under it control u senate candidate set the tone for kentucky republican during statewide dinner what to know about the putintrump summit in alaska what to know about the putintrump summit in alaska photo of trump emergency declaration a the national guard is activated in washington photo of trump emergency declaration a the national guard is activated in washington trump mistake alaska for russia and yes there snark surveillance case test chapter a standing and unfairness standard clinton county sheriff office arrest individual involved with multicounty sex trafficking operation a judge brutal rebuke of trump epstein gambit cnn politics what to know about the putintrump summit in alaska local view give ailing minnesota kid a fighting chance philippe cousteau earthecho international announces diverse youth advocate join the blue carbon ambassador program california couple file lawsuit against klp in conway over shortterm rental rule rubio hit medium over gaza narrative say some ally making it harder to achieve peace multiple men have impersonated ice agent to kidnap and assault woman multiple men have impersonated ice agent to kidnap and assault woman doe using ai dumb you down vote to save a historic building from demolition trump promised to fix inflation he doing this instead south carolina lawmaker awaiting trial on child sex abuse material charge resigns from office nvidia to share of revenue from chip sale to china with u government trump say gold wont face tariff trump say gold wont face tariff trump say gold wont face tariff trump say gold wont face tariff trump say gold wont face tariff ana alsharif became the face of the war in gaza for million then israel killed him trump say he placing washington police under federal control and deploying the national guard trump declares crime in dc will be cleaned up real quick during his announcement that he taking over the city police department chinese ship collide on chase in disputed water ap news summary at pm edt trump say he placing washington police under federal control and activating the national guard houlihan financial resource group ltd sell share of international business machine corporation nyseibm meridian wealth management llc ha million position in broadcom inc nasdaqavgo motley fool asset management llc raise stock holding in broadcom inc nasdaqavgo colorado congressional democrat visit aurora ice facility meet with detained activist jeanette vizguerra colorado congressional democrat visit aurora ice facility meet with detained activist jeanette vizguerra colorado congressional democrat visit aurora ice facility meet with detained activist jeanette vizguerra colorado congressional democrat visit aurora ice facility meet with detained activist jeanette vizguerra russian seeking asylum in u facing new obstacle say usbased activist trump warns protester amid dc crime crack down you spit and we hit trump suggests he can send national guard troop into other u city beyond dc scientist say they cruised the ocean in a deepsea submersible and came across an undiscovered ecosystem dillon associate inc increase holding in salesforce inc nysecrm colombian presidential candidate miguel uribe turbay dy two month after assassination attempt live now texas hold legislative session after democrat leave state jeffries hammer trump for seizing control of dc police no basis jeffries hammer trump for seizing control of dc police no basis jeffries hammer trump for seizing control of dc police no basis jeffries hammer trump for seizing control of dc police no basis jeffries hammer trump for seizing control of dc police no basis maga v miga laura loomer block marjorie taylor greene on social medium escalating a feud over america israel policy trump looking at reclassifying marijuana a le dangerous drug trump looking at reclassifying marijuana a le dangerous drug danish zoo asks for donated pet to feed to carnivore trump looking at reclassifying marijuana a le dangerous drug trump looking at reclassifying marijuana a le dangerous drug trump looking at reclassifying marijuana a le dangerous drug el paso police man dy when he hit tree get ejected trump team get blasted by judge for clumsy epstein diversion raw politics is now driving law enforcement at the department of justice civil right division nancy pelosi get all high and mighty lying about trump j and the ntl guard and oh hell no old woman this candidate for california governor ha a potential conflict of interest in her own home ishares core sp etf nysearcaivv share sold by aveo capital partner llc maine state library not victimized a suggested letter maine state library not victimized a suggested letter here are the country that have recognized a palestinian state johnson fistel investigates fairness of proposed sale of meridianlink currently the most dangerous place maia wealth llc purchase share of ishares core u aggregate bond etf nysearcaagg my wife of year just died my grief is so overwhelming i can barely cope</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>mp material nysemp stock price up on analyst upgrade affinity bancshares nasdaqafbi v dime community bancshares nasdaqdcom head to head analysis oms energy technology nasdaqomse north american construction group nysenoa headtohead survey reviewing blade air mobility blde and the competition analyzing haverty furniture company nysehvta and brand house collective nasdaqtbhc head to head survey armstrong world industry nyseawi and obayashi otcmktsobycf headtohead review ayro nasdaqayro tesla nasdaqtsla reviewing humana nysehum joint nasdaqjynt financial review kayne anderson bdc nysekbdc hercules capital nysehtgc head to head comparison marui group otcmktsmaury kohl nysekss portillos nasdaqptlo stock rating lowered by wall street zen contrasting bark nysebark and fireman contractor otcmktsfrcn head to head survey southern first bancshares nasdaqsfst v people bancorp of north carolina nasdaqpebk financial comparison city office reit nysecio v lamar advertising nasdaqlamr sadot group nasdaqsdot versus grove collaborative nysegrov headtohead contrast headtohead analysis office property income trust nasdaqopi versus safehold nysesafe financial review ho innovation otcmktsheoff and ho america nasdaqhto lharris technology nyselhx v safran otcmktssafry head to head review orion group nyseorn v mastec nysemtz head to head review headtohead comparison vertiv nysevrt v leidos nyseldos head to head survey hess midstream partner nysehesm v xplr infrastructure nysexifr financial contrast arcutis biotherapeutics nasdaqarqt v novocure nasdaqnvcr contrasting onewater marine nasdaqonew and peloton interactive nasdaqpton critical survey t biosystems nasdaqttoo and perspective therapeutic nysecatx comparing castor maritime nasdaqctrm and united maritime nasdaqusea crypto price today bitcoin price fall to xrp at and solana at riskified ltd nyserskd receives consensus recommendation of hold from brokerage roku inc nasdaqroku given average rating of moderate buy by brokerage financial analysis ameramex international otcmktsammx willis lease finance nasdaqwlfc academy sport and outdoors inc nasdaqaso receives consensus recommendation of moderate buy from analyst brp inc tsedoo given consensus recommendation of hold by brokerage unicredit otcmktsuncry trading down here what happened annaly capital management inc nysenly given average rating of moderate buy by analyst pagseguro digital ltd nysepags receives consensus rating of moderate buy from analyst palantir technology inc nasdaqpltr receives average rating of hold from brokerage travere therapeutic inc nasdaqtvtx given consensus rating of moderate buy by analyst hbo max viu set to offer streaming bundle in asian country sartorius stedim biotech epadim share down should you sell hr real estate investment trust otcmktshruff share up time to buy midnight sun mining cvemma stock price up whats next bmo laddered preferred share index etf tsezpr share down whats next dream industrial real estate investment trust otcmktsdreuf trading down whats next tgs asa otcmktstgsgy trading down whats next doman building material group otcmktscwxzf stock price down should you sell wimi hologram cloud nasdaqwimi trading up still a buy u solar fund lonusfp stock price down whats next titan mining otcmktstnmcf share down whats next china minsheng otcmktscmaky stock price down whats next rational aktiengesellschaft otcmktsrtllf stock price down should you sell intellinetics otcmktsinlxd trading up here what happened melrose industry otcmktsmlspf trading down whats next nippon steel sumitomo metal otcmktsnpscy trading down here what happened barclays etn fi enhanced europe etn series c nysearcaffeu trading up whats next imab nasdaqimab trading higher here why wisdomtree cloud computing fund nasdaqwcld trading down time to sell thai oil public otcmktstoipf trading higher whats next xtrackers international real estate etf nysearcahauz trading down here why fibra uno otcmktsfbasf trading down whats next aimia otcmktsgapff stock price down here what happened camino mineral cvecor share up here what happened sompo otcmktssmpny trading down time to sell foxby otcmktsfxby share up time to buy bmo low volatility canadian equity etf tsezlb trading down time to sell urbana otcmktsubaaf stock price up whats next china citic bank otcmktschcjy stock price down here why biglari nysebha stock price up whats next permrock royalty trust nyseprt trading higher should you buy nufarm otcmktsnufmf trading higher still a buy cascade otcmktscadnf stock price down whats next metaurus u equity exdividend fundseries nysearcaxdiv trading down whats next wisdomtree balanced income fund nysearcawbal share up should you buy midnight sun mining cvemma stock price up whats next uxin nasdaquxin trading up time to buy serica energy otcmktssqzzf trading up whats next bmo laddered preferred share index etf tsezpr share down whats next artis real estate investment trust otcmktsaresf trading down whats next aptus defined risk etf batsdrsk trading down time to sell salmar asa otcmktssalrf share up whats next rpar risk parity etf nysearcarpar share down should you sell sgl carbon otcmktssglff stock price down should you sell overlay share large cap equity etf nysearcaovl share down should you sell boc hong kong otcmktsbhkly share up here what happened amplify alternative harvest etf nysearcamj share up whats next sartorius stedim biotech epadim trading down should you sell manolete partner lonmano stock price down should you sell portfolioplus sp small cap etf nysearcappsc trading higher time to buy vanguard growth etf portfolio tsevgro share down time to sell charlotte web otcmktscwbhf share up here why collplant biotechnology nasdaqclgn trading higher here why iphone pro launch date and price in india revealed check all detail musk grok ai briefly suspended on x for claiming israel commits genocide aersale nasdaqasle raised to strongbuy at wall street zen top tech news nvidias ai chip approved for china meta raise b for ai growth wall street zen downgrade cormedix nasdaqcrmd to buy dragonfly energy dfli expected to announce earnings on thursday mediwound mdwd projected to post quarterly earnings on thursday draftkings nasdaqdkng upgraded at wall street zen palvella therapeutic pvla to release earnings on thursday unusual machine umac expected to announce quarterly earnings on thursday westbow press announces the book answer with truth ha earned exclusive lighthouse recognition portillos nasdaqptlo cut to sell at wall street zen procept biorobotics nasdaqprct rating increased to hold at wall street zen fanatic branded nfl nba mlb nhl apparel sale banned in australia souad m hanna aersale nasdaqasle upgraded at wall street zen donegal group nasdaqdgica stock rating lowered by wall street zen cormedix nasdaqcrmd cut to buy at wall street zen acurx pharmaceutical nasdaqacxp upgraded at wall street zen cricut nasdaqcrct upgraded at wall street zen capital one financial nysecof cut to hold at wall street zen capri nysecpri upgraded at wall street zen citizen nysecia upgraded at wall street zen bwx technology nysebwxt lowered to hold rating by wall street zen vimeo nasdaqvmeo upgraded by wall street zen to buy rating frederick should revisit it district map brehm would be effective leader on council trump say plan to test out putin a europe engages ukraine greg abbott threatens to eliminate democratic district a texas prepares redistricting counterstrike against california map overhaul knightscope nasdaqkscp cut to sell at wall street zen klaviyo nysekvyo upgraded at wall street zen figma nysefig upgraded at wall street zen rxo nyserxo upgraded at wall street zen interactive strength nasdaqtrnr upgraded at wall street zen guardian pharmacy service nysegrdn cut to hold at wall street zen audioeye nasdaqaeye cut to hold at wall street zen biomarin pharmaceutical nasdaqbmrn rating increased to strongbuy at wall street zen banner nasdaqbanr cut to sell at wall street zen alerus financial nasdaqalrs stock rating upgraded by wall street zen ascent solar technology nasdaqasti upgraded at wall street zen ardelyx nasdaqardx upgraded at wall street zen berry nasdaqbry cut to sell at wall street zen applied optoelectronics nasdaqaaoi lowered to sell rating by wall street zen vitesse energy nysevts upgraded at wall street zen amer sport nyseas cut to hold at wall street zen brookdale senior living nysebkd rating increased to hold at wall street zen aflac nyseafl upgraded at wall street zen sapiens international spns expected to announce earnings on wednesday northpointe bancshares inc nysenpb lockup period will expire tomorrow raskin on dc crime do you trust the dems who created the mess or trump who doe the impossible trump back burt jones in republican race for georgia governor in kimmel guest host nicole byer make a dangerous example out of trump dc talk hartselle candidate forum to spotlight local issue u designates baloch separatist a a terror group over role in attack in pakistan eu leader appeal to trump to defend europe security interest at his war summit with putin death notice jean phyllis williams eu leader appeal to trump to defend europe security interest at his war summit with putin the forgotten story of the world deadliest plane crash angler break record after getting green light to reel in harmful fish my fishing pole took a hard hit point coal need to be part of america energy future wdt thought for aug your view constitutional amendment would permit limit on political spending trump back burt jones in republican race for georgia governor in trump back burt jones in republican race for georgia governor in trump back burt jones in republican race for georgia governor in counterpoint america need affordable energy coal doesnt fit the bill u and china extend trade truce another day easing tension between world largest economy u and china extend trade truce another day easing tension between world largest economy at th hour ups bow to teamster strike threat in state nancy pelosi say american know republican ripped away health care will lose midterm unacceptable they want to change rule midgame south korean president lee will travel to washington for aug meeting with trump trump washington police takeover echo history of racist narrative about urban crime hamas hostage video silenced israeli medias talk of gaza aid crisis shareholder action reminder faruqi faruqi llp investigates claim on behalf of investor of lockheed martin fifa move ahead with new human right strategy for world cup game but advocate are skeptical fifa move ahead with new human right strategy for world cup game but advocate are skeptical fifa move ahead with new human right strategy for world cup game but advocate are skeptical inflation likely moved higher last month a tariff bite putting the fed in bind trump washington police takeover echo history of racist narrative about urban crime trump washington police takeover echo history of racist narrative about urban crime trump washington police takeover echo history of racist narrative about urban crime trump washington police takeover echo history of racist narrative about urban crime trump washington police takeover echo history of racist narrative about urban crime federal becomes local the nation capital find itself at the center of a donald trump maelstrom federal becomes local the nation capital find itself at the center of a donald trump maelstrom federal becomes local the nation capital find itself at the center of a donald trump maelstrom letter richard bryan critique donald trump david larson what the dmv can learn from chickfila john hood tariff threat hurt carolina worker letter making my point my turn our right to freedom of conscience and the rowan early voting calendar cartoon what harris campaign memoir should be called editorial hamas steal aid to fund war promote propaganda editorial dallas morning news money role in american politics could get even worse when truth becomes the enemy of the state how to win on immigration go away with leonidas g demas letter stop the hate if you want to up the birth rate scott jennings trigger dems by saying nobody in their right mind think washington dc is safe anna mae midge stellmach trial expose internal tension over trump use of national guard in la photo of mourning for colombian sen miguel uribe who died month after shooting at a rally photo of mourning for colombian sen miguel uribe who died month after shooting at a rally trump unprecedented takeover of dc police come a crime is down figure show application for sd development of affordable housing being accepted library board wont meet in august welcome to south dakota newest news desert with new law city mull election move protest a trump take over dc police deploys national guard in capital dem whistleblower adam schiff okayed leaking of classified info to smear trump in russian collusion hoax letter a reminder from an old friend goodship raise million in series b funding round tesla launch mile model in china a ufc fight at the white house white say it happening a part of deal with paramount cold wallet presale pull in m bonk slip sol breakout loom cenovus indigenous group circle meg energy in possible joint bid pepe coin price prediction at could ozak ai deliver a stronger roi new mexico climate investment center debut energyefficiency loan program for small business nonprofit cardinal health to extend reach by acquiring solaris health dow rally point sp hit new record a cpi report give fed green light to cut rate live update cnbc this best selling jump starter is under for a limited time switzerland could experience unique economic problem from trump tariff bosscattm home service and technology recognized for fourth consecutive year on the inc list of america fastestgrowing private company nuvei tap stablecoins to expand money movement operation fermi americatm name two highly successful nuclear developer mesut and sezin uzman to spearhead nuclear power delivery dow surge point u core inflation rise to meta stock hit new high a thread rocket past million user ai startup perplexity make billion bid for google chrome browser a pause in bitcoin can still be profitable with this option on ibit dutch bros coffee to open th lake houstonarea location in kingwood slqt investor have opportunity to lead selectquote inc security fraud lawsuit with the schall law firm a new chapter for crypto moonshot magax magax bitcoin hyper and aurealone microsoft forecast strong cash flow for fy raising price target to your guide to the top meme coin to invest in trump plan b ipo to privatize fannie mae freddie mac the ally are mostly alright but is that a good thing what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy elon musk threatens apple with lawsuit over openai sparking online feud with sam altman the guardian ibs in america despite advance ibs remains a burden for many million forddirect partner with podium to deliver aipowered conversation to ford and lincoln retailer iconic u film company kodak warns it may go out of business usa today rddt deadline rosen a leading investor right law firm encourages reddit inc investor to crypto entrepreneur who caused market crash pleads guilty to fraud rddt deadline rosen a leading investor right law firm encourages reddit inc investor to secure counsel before important august deadline in security class action rddt gear up for your next project with up to off select tool at the home depot cardinal fiscal q earnings snapshot northern virginia housing market cool slightly a inventory grows resideo technology pop a honeywell indemnity buyout boost growth story iceland eclipse festival to blend music art and space talk hedge fund and insider trading news seth klarman ray dalio ken griffin steve cohen renaissance technology millennium management third point shift payment inc four fastenal co fast and more european auto exporter say tariff stalling business seeing oceanfront property in ukraine trump real estate history shape his presidency spotlight on sezzle analyzing the surge in option activity decoding sofi technologiess option activity whats the big picture peoplesoft how to find own america greatest opportunity why ethereum is rising today rent medical cost drive yearoveryear inflation the magnificent iran and russia vow to block u caucasus ambition best cryptos to buy now in august top crypto opportunity to watch in blockdag xrp stellar solana best dell gaming laptop to buy in abacus insurance and financial service join world insurance associate u july tariff revenue jump fails to halt wider budget deficit bloombergcom best ergonomic gadget for remote worker our view make lasting cut to govguam cost during budget talk why bigbearai stock is cratering today why pubmatic stock fell this morning want to attend world cup game for free fifa need volunteer ai startup perplexity offer to buy google chrome browser for billion the new york time easyfeast unveils new brand identity honoring it mission to make homemade meal easier dow jones leader cisco magnificent seven stock alphabet in new buy zone oryx dental recognized a a top software company on the inc list here why share in united airline took off today advent technology holding inc enhances license to groundbreaking ion pair technology developed at los alamo national laboratory by acquiring exclusivity in marine aviation and portable power field spacex rival ast spacemobile prepares to deploy nearly five dozen satellite signed lanie gardner is on the right track onerpm ink daya g love special sauce generation z saving habit a look at their financial priority and insight zelensky refuse to cede donbas say doing so would give putin springboard for future offensive dorrance planetarium what the cuttingedge led dome at the arizona science center will look like atlantic american corporation report second quarter result for na fallon commander speaks at ceda breakfast atlantic american corporation report second quarter result for gamechange solar rise to third globally and second in u solar tracker market terraform lab founder do kwon pleads guilty to fraud in b terraluna collapse fhlbank san francisco invests million to preserve affordable housing in arizona metro denver inflation hold steady ahead of upcoming tariff keep your toothbrush germfree with the bril uv light toothbrush sanitizer elon musk went from promising tesla unsupervised selfdriving to less nag while los angeles burned rule to protect home from wildfire were on hold spirit airline sound the alarm on it future ability to stay in business what is ai automation and how doe it work official opening of a housing project for adult living with autism spectrum disorder in the gaspe region citizen name barclays executive a it next finance chief worth of labubus headed for black market recovered from socal home los angeles time kucoin first to support ubs umint collateral via digift bridging tokenized rwas and crypto trading bird fan are getting shortchanged reader commentary business spat between daryl hall and john oates ha been resolved in arbitration attorney say desjardins post surplus earnings of million for the second quarter of and surpasses billion in asset family safety stock life surge a parent seek peace of mind bank of america corporation nysebac stock holding decreased by finer wealth management inc tesla inc nasdaqtsla share acquired by saiph capital llc this spy pen secretly record k hd video and audio and it off now the latest national guard arrives in washington dc for trump federal takeover of local police silicon valley lawmaker want to decriminalize homelessness no one is above the law tx ag paxton seek to hold beto orourke in contempt for defying court order ai is reshaping hacking no one agrees how fast trump threatens allowing major lawsuit against fed chair powell over central bank renovation gifford fire grows to more than acre a it shift west in slo county black bear qb embrace life in maine ready to lead football team u teen influencer pilot accused of unauthorized antarctic landing reach deal to leave chile new research discovers the first known latterday saint polygamist with black ancestry israel is in talk to possibly resettle palestinian from gaza in south sudan israel is in talk to possibly resettle palestinian from gaza in south sudan trump takeover of washington law enforcement begin a national guard troop arrive texas senate pass redistricting map despite democrat walkout but house still cant consider bill with no quorum transgender woman sue over jail assault texas republican plan another special session to deliver trump more gop congressional seat texas republican plan another special session to deliver trump more gop congressional seat trump name heritage foundation ej antoni to lead bureau of labor statistic israel is in talk to possibly resettle palestinian from gaza in south sudan israel is in talk to possibly resettle palestinian from gaza in south sudan zelenskyy say putin want the rest of ukraine donetsk region a part of a ceasefire doge land big legal win a appeal court strike down preliminary injunction appeal court remove block on doge data access a familiar name raise democrat spirit in ohio senate race this is how it done here the arrest list from night with trump national guard protecting dc what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy dc top cop clueless on chain of command chief pamela smith deidriven disaster white house say homeless people in dc could be susceptible to jail time white house confirms trumpputin summit in anchorage calling it listening exercise what to know about trump potential change in federal marijuana policy trump use of troop for policing hasnt been seen since america wa ruled by a king trump considering lawsuit against fed a he bash chair jerome powell seeing oceanfront property in ukraine trump real estate history shape his presidency live now u attorney pirro ice and state official announce indictment of haitian gang leader we dont despise the medium enough foreign press association president condemns death of hamas journo how should american college measure merit bank fee for data access threaten the foundation of open banking deja vu another british f just made an emergency landing in japan lima one bill mcdonald honored by housingwire ap news summary at pm edt u citizen detained by ice say she wa denied water for hour israel is in talk to possibly resettle palestinian from gaza in south sudan u designates baloch separatist a a terror group over role in attack in pakistan syria u and jordan say they will work toward a lasting truce in wake of syrian sectarian clash zelensky refuse to cede donbas say doing so would give putin springboard for future offensive paxton urge texas judge to jail beto orourke over fundraising related to redistricting fight more republican join georgia competitive race for lieutenant governor more republican join georgia competitive race for lieutenant governor letter notsofree speech armstrong williams when the bench becomes the battlefield staff commentary takeaway from aps reporting on armed group recruiting child in colombia ashley biden daughter of joe and jill biden file for divorce after year of marriage county call million bond election to build jail live now department of state hold press briefing aug violent guerrilla are taking colombia child unarmed indigenous group are confronting them violent guerrilla are taking colombia child unarmed indigenous group are confronting them boom winsome earlesears just dropped another ad that abigail spanberger will have to answer for watch what to know about the putintrump summit in alaska cdc shooting linked to suspect covid vaccine belief former staff blame rfk jr hostility toward agency the palestinian journalist killed in the war in gaza endured hunger and grief the palestinian journalist killed in the war in gaza endured hunger and grief newsnation cut interview after guest call out trump hypocrisy on live tv newsnation cut interview after guest call out trump hypocrisy on live tv business spat between daryl hall and john oates ha been resolved in arbitration attorney say zelenskyy say putin want the rest of ukraine donetsk region a part of a ceasefire whats at stake a trump prepares to meet putin in alaska shacarri richardson address domestic violence arrest and apologizes to christian coleman musk blow stack after apple snub his racist chatbot texas twostep two additional bill from the texas legislative session that contractor need to know trump want to make the census count a salute to legend like kathy bates jean smart and harrison ford on finally getting their emmy flower inside senate dems summer warpath against trump trump weighs major lawsuit against powell over federal building renovation cost jimmy kimmel obtained italian citizenship in case he need to flee second trump administration it so much worse teen in northfield triple murder to forgo trial and plead guilty teenager in northfield triple murder to plead guilty trump threatens powell with major lawsuit over fed renovation ap news summary at pm edt russian troop advance in ukraine ahead of trumpputin peace summit tinfoil or not you decide damning thread tie nick fuentes to january th in a very troubling way the ncaa is a billiondollar sport behemoth that should not be a nonprofit bosnia serb leader dodik avoids prison term a election loom zelenskyy say russia want a ukrainian withdrawal from ukraine eastern donetsk region a part of a ceasefire deal zelenskyy say russia want a ukrainian withdrawal from ukraine eastern donetsk region a part of a ceasefire deal liar another gop rep face a raucous town hall angered by trump agenda liar another gop rep face a raucous town hall angered by trump agenda poll open in primary election for slain rep melissa hortmans seat pete hegseth belongs to an archconservative church network here what to know cnn slap trump with new nickname accidentally make him sound cooler sherrod brown to launch a comeback attempt for senate in ohio trump v newsom showdown land in court with family tie to the nation highest bench desantis name state sen jay collins a lieutenant governor desantis pick the chuck norris of florida politics a new top deputy allegiant airline to add direct flight from appleton to orlando here what to know bonus editorial cartoon for aug zelenskiy say ukraine wont withdraw troop from donbas first court hearing to take place tuesday in riley strain lawsuit for motion hearing trump washington dc takeover begin a national guard troop arrive</t>
+          <t>mp material nysemp stock price up on analyst upgrade affinity bancshares nasdaqafbi v dime community bancshares nasdaqdcom head to head analysis oms energy technology nasdaqomse north american construction group nysenoa headtohead survey reviewing blade air mobility blde and the competition analyzing haverty furniture company nysehvta and brand house collective nasdaqtbhc head to head survey armstrong world industry nyseawi and obayashi otcmktsobycf headtohead review ayro nasdaqayro tesla nasdaqtsla reviewing humana nysehum joint nasdaqjynt financial review kayne anderson bdc nysekbdc hercules capital nysehtgc head to head comparison marui group otcmktsmaury kohl nysekss portillos nasdaqptlo stock rating lowered by wall street zen contrasting bark nysebark and fireman contractor otcmktsfrcn head to head survey southern first bancshares nasdaqsfst v people bancorp of north carolina nasdaqpebk financial comparison city office reit nysecio v lamar advertising nasdaqlamr sadot group nasdaqsdot versus grove collaborative nysegrov headtohead contrast headtohead analysis office property income trust nasdaqopi versus safehold nysesafe financial review ho innovation otcmktsheoff and ho america nasdaqhto lharris technology nyselhx v safran otcmktssafry head to head review orion group nyseorn v mastec nysemtz head to head review headtohead comparison vertiv nysevrt v leidos nyseldos head to head survey hess midstream partner nysehesm v xplr infrastructure nysexifr financial contrast arcutis biotherapeutics nasdaqarqt v novocure nasdaqnvcr contrasting onewater marine nasdaqonew and peloton interactive nasdaqpton critical survey t biosystems nasdaqttoo and perspective therapeutic nysecatx comparing castor maritime nasdaqctrm and united maritime nasdaqusea crypto price today bitcoin price fall to xrp at and solana at riskified ltd nyserskd receives consensus recommendation of hold from brokerage roku inc nasdaqroku given average rating of moderate buy by brokerage financial analysis ameramex international otcmktsammx willis lease finance nasdaqwlfc academy sport and outdoors inc nasdaqaso receives consensus recommendation of moderate buy from analyst brp inc tsedoo given consensus recommendation of hold by brokerage unicredit otcmktsuncry trading down here what happened annaly capital management inc nysenly given average rating of moderate buy by analyst pagseguro digital ltd nysepags receives consensus rating of moderate buy from analyst palantir technology inc nasdaqpltr receives average rating of hold from brokerage travere therapeutic inc nasdaqtvtx given consensus rating of moderate buy by analyst hbo max viu set to offer streaming bundle in asian country sartorius stedim biotech epadim share down should you sell hr real estate investment trust otcmktshruff share up time to buy midnight sun mining cvemma stock price up whats next bmo laddered preferred share index etf tsezpr share down whats next dream industrial real estate investment trust otcmktsdreuf trading down whats next tgs asa otcmktstgsgy trading down whats next doman building material group otcmktscwxzf stock price down should you sell wimi hologram cloud nasdaqwimi trading up still a buy u solar fund lonusfp stock price down whats next titan mining otcmktstnmcf share down whats next china minsheng otcmktscmaky stock price down whats next rational aktiengesellschaft otcmktsrtllf stock price down should you sell intellinetics otcmktsinlxd trading up here what happened melrose industry otcmktsmlspf trading down whats next nippon steel sumitomo metal otcmktsnpscy trading down here what happened barclays etn fi enhanced europe etn series c nysearcaffeu trading up whats next imab nasdaqimab trading higher here why wisdomtree cloud computing fund nasdaqwcld trading down time to sell thai oil public otcmktstoipf trading higher whats next xtrackers international real estate etf nysearcahauz trading down here why fibra uno otcmktsfbasf trading down whats next aimia otcmktsgapff stock price down here what happened camino mineral cvecor share up here what happened sompo otcmktssmpny trading down time to sell foxby otcmktsfxby share up time to buy bmo low volatility canadian equity etf tsezlb trading down time to sell urbana otcmktsubaaf stock price up whats next china citic bank otcmktschcjy stock price down here why biglari nysebha stock price up whats next permrock royalty trust nyseprt trading higher should you buy nufarm otcmktsnufmf trading higher still a buy cascade otcmktscadnf stock price down whats next metaurus u equity exdividend fundseries nysearcaxdiv trading down whats next wisdomtree balanced income fund nysearcawbal share up should you buy midnight sun mining cvemma stock price up whats next uxin nasdaquxin trading up time to buy serica energy otcmktssqzzf trading up whats next bmo laddered preferred share index etf tsezpr share down whats next artis real estate investment trust otcmktsaresf trading down whats next aptus defined risk etf batsdrsk trading down time to sell salmar asa otcmktssalrf share up whats next rpar risk parity etf nysearcarpar share down should you sell sgl carbon otcmktssglff stock price down should you sell overlay share large cap equity etf nysearcaovl share down should you sell boc hong kong otcmktsbhkly share up here what happened amplify alternative harvest etf nysearcamj share up whats next sartorius stedim biotech epadim trading down should you sell manolete partner lonmano stock price down should you sell portfolioplus sp small cap etf nysearcappsc trading higher time to buy vanguard growth etf portfolio tsevgro share down time to sell charlotte web otcmktscwbhf share up here why collplant biotechnology nasdaqclgn trading higher here why iphone pro launch date and price in india revealed check all detail musk grok ai briefly suspended on x for claiming israel commits genocide aersale nasdaqasle raised to strongbuy at wall street zen top tech news nvidias ai chip approved for china meta raise b for ai growth wall street zen downgrade cormedix nasdaqcrmd to buy dragonfly energy dfli expected to announce earnings on thursday mediwound mdwd projected to post quarterly earnings on thursday draftkings nasdaqdkng upgraded at wall street zen palvella therapeutic pvla to release earnings on thursday unusual machine umac expected to announce quarterly earnings on thursday westbow press announces the book answer with truth ha earned exclusive lighthouse recognition portillos nasdaqptlo cut to sell at wall street zen procept biorobotics nasdaqprct rating increased to hold at wall street zen fanatic branded nfl nba mlb nhl apparel sale banned in australia souad m hanna aersale nasdaqasle upgraded at wall street zen donegal group nasdaqdgica stock rating lowered by wall street zen cormedix nasdaqcrmd cut to buy at wall street zen acurx pharmaceutical nasdaqacxp upgraded at wall street zen cricut nasdaqcrct upgraded at wall street zen capital one financial nysecof cut to hold at wall street zen capri nysecpri upgraded at wall street zen citizen nysecia upgraded at wall street zen bwx technology nysebwxt lowered to hold rating by wall street zen vimeo nasdaqvmeo upgraded by wall street zen to buy rating frederick should revisit it district map brehm would be effective leader on council trump say plan to test out putin a europe engages ukraine greg abbott threatens to eliminate democratic district a texas prepares redistricting counterstrike against california map overhaul knightscope nasdaqkscp cut to sell at wall street zen klaviyo nysekvyo upgraded at wall street zen figma nysefig upgraded at wall street zen rxo nyserxo upgraded at wall street zen interactive strength nasdaqtrnr upgraded at wall street zen guardian pharmacy service nysegrdn cut to hold at wall street zen audioeye nasdaqaeye cut to hold at wall street zen biomarin pharmaceutical nasdaqbmrn rating increased to strongbuy at wall street zen banner nasdaqbanr cut to sell at wall street zen alerus financial nasdaqalrs stock rating upgraded by wall street zen ascent solar technology nasdaqasti upgraded at wall street zen ardelyx nasdaqardx upgraded at wall street zen berry nasdaqbry cut to sell at wall street zen applied optoelectronics nasdaqaaoi lowered to sell rating by wall street zen vitesse energy nysevts upgraded at wall street zen amer sport nyseas cut to hold at wall street zen brookdale senior living nysebkd rating increased to hold at wall street zen aflac nyseafl upgraded at wall street zen sapiens international spns expected to announce earnings on wednesday northpointe bancshares inc nysenpb lockup period will expire tomorrow raskin on dc crime do you trust the dems who created the mess or trump who doe the impossible trump back burt jones in republican race for georgia governor in kimmel guest host nicole byer make a dangerous example out of trump dc talk hartselle candidate forum to spotlight local issue u designates baloch separatist a a terror group over role in attack in pakistan eu leader appeal to trump to defend europe security interest at his war summit with putin death notice jean phyllis williams eu leader appeal to trump to defend europe security interest at his war summit with putin the forgotten story of the world deadliest plane crash angler break record after getting green light to reel in harmful fish my fishing pole took a hard hit point coal need to be part of america energy future wdt thought for aug your view constitutional amendment would permit limit on political spending trump back burt jones in republican race for georgia governor in trump back burt jones in republican race for georgia governor in trump back burt jones in republican race for georgia governor in counterpoint america need affordable energy coal doesnt fit the bill u and china extend trade truce another day easing tension between world largest economy u and china extend trade truce another day easing tension between world largest economy at th hour ups bow to teamster strike threat in state nancy pelosi say american know republican ripped away health care will lose midterm unacceptable they want to change rule midgame south korean president lee will travel to washington for aug meeting with trump trump washington police takeover echo history of racist narrative about urban crime hamas hostage video silenced israeli medias talk of gaza aid crisis shareholder action reminder faruqi faruqi llp investigates claim on behalf of investor of lockheed martin fifa move ahead with new human right strategy for world cup game but advocate are skeptical fifa move ahead with new human right strategy for world cup game but advocate are skeptical fifa move ahead with new human right strategy for world cup game but advocate are skeptical inflation likely moved higher last month a tariff bite putting the fed in bind trump washington police takeover echo history of racist narrative about urban crime trump washington police takeover echo history of racist narrative about urban crime trump washington police takeover echo history of racist narrative about urban crime trump washington police takeover echo history of racist narrative about urban crime trump washington police takeover echo history of racist narrative about urban crime federal becomes local the nation capital find itself at the center of a donald trump maelstrom federal becomes local the nation capital find itself at the center of a donald trump maelstrom federal becomes local the nation capital find itself at the center of a donald trump maelstrom letter richard bryan critique donald trump david larson what the dmv can learn from chickfila john hood tariff threat hurt carolina worker letter making my point my turn our right to freedom of conscience and the rowan early voting calendar cartoon what harris campaign memoir should be called editorial hamas steal aid to fund war promote propaganda editorial dallas morning news money role in american politics could get even worse when truth becomes the enemy of the state how to win on immigration go away with leonidas g demas letter stop the hate if you want to up the birth rate scott jennings trigger dems by saying nobody in their right mind think washington dc is safe anna mae midge stellmach trial expose internal tension over trump use of national guard in la photo of mourning for colombian sen miguel uribe who died month after shooting at a rally photo of mourning for colombian sen miguel uribe who died month after shooting at a rally trump unprecedented takeover of dc police come a crime is down figure show application for sd development of affordable housing being accepted library board wont meet in august welcome to south dakota newest news desert with new law city mull election move protest a trump take over dc police deploys national guard in capital dem whistleblower adam schiff okayed leaking of classified info to smear trump in russian collusion hoax letter a reminder from an old friend goodship raise million in series b funding round tesla launch mile model in china a ufc fight at the white house white say it happening a part of deal with paramount cold wallet presale pull in m bonk slip sol breakout loom cenovus indigenous group circle meg energy in possible joint bid pepe coin price prediction at could ozak ai deliver a stronger roi new mexico climate investment center debut energyefficiency loan program for small business nonprofit cardinal health to extend reach by acquiring solaris health dow rally point sp hit new record a cpi report give fed green light to cut rate live update cnbc this best selling jump starter is under for a limited time switzerland could experience unique economic problem from trump tariff bosscattm home service and technology recognized for fourth consecutive year on the inc list of america fastestgrowing private company nuvei tap stablecoins to expand money movement operation fermi americatm name two highly successful nuclear developer mesut and sezin uzman to spearhead nuclear power delivery dow surge point u core inflation rise to meta stock hit new high a thread rocket past million user ai startup perplexity make billion bid for google chrome browser a pause in bitcoin can still be profitable with this option on ibit dutch bros coffee to open th lake houstonarea location in kingwood slqt investor have opportunity to lead selectquote inc security fraud lawsuit with the schall law firm a new chapter for crypto moonshot magax magax bitcoin hyper and aurealone microsoft forecast strong cash flow for fy raising price target to your guide to the top meme coin to invest in trump plan b ipo to privatize fannie mae freddie mac the ally are mostly alright but is that a good thing what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy elon musk threatens apple with lawsuit over openai sparking online feud with sam altman the guardian ibs in america despite advance ibs remains a burden for many million forddirect partner with podium to deliver aipowered conversation to ford and lincoln retailer iconic u film company kodak warns it may go out of business usa today rddt deadline rosen a leading investor right law firm encourages reddit inc investor to crypto entrepreneur who caused market crash pleads guilty to fraud rddt deadline rosen a leading investor right law firm encourages reddit inc investor to secure counsel before important august deadline in security class action rddt gear up for your next project with up to off select tool at the home depot cardinal fiscal q earnings snapshot northern virginia housing market cool slightly a inventory grows resideo technology pop a honeywell indemnity buyout boost growth story iceland eclipse festival to blend music art and space talk hedge fund and insider trading news seth klarman ray dalio ken griffin steve cohen renaissance technology millennium management third point shift payment inc four fastenal co fast and more european auto exporter say tariff stalling business seeing oceanfront property in ukraine trump real estate history shape his presidency spotlight on sezzle analyzing the surge in option activity decoding sofi technology option activity whats the big picture peoplesoft how to find own america greatest opportunity why ethereum is rising today rent medical cost drive yearoveryear inflation the magnificent iran and russia vow to block u caucasus ambition best cryptos to buy now in august top crypto opportunity to watch in blockdag xrp stellar solana best dell gaming laptop to buy in abacus insurance and financial service join world insurance associate u july tariff revenue jump fails to halt wider budget deficit bloombergcom best ergonomic gadget for remote worker our view make lasting cut to govguam cost during budget talk why bigbearai stock is cratering today why pubmatic stock fell this morning want to attend world cup game for free fifa need volunteer ai startup perplexity offer to buy google chrome browser for billion the new york time easyfeast unveils new brand identity honoring it mission to make homemade meal easier dow jones leader cisco magnificent seven stock alphabet in new buy zone oryx dental recognized a a top software company on the inc list here why share in united airline took off today advent technology holding inc enhances license to groundbreaking ion pair technology developed at los alamo national laboratory by acquiring exclusivity in marine aviation and portable power field spacex rival ast spacemobile prepares to deploy nearly five dozen satellite signed lanie gardner is on the right track onerpm ink daya g love special sauce generation z saving habit a look at their financial priority and insight zelensky refuse to cede donbas say doing so would give putin springboard for future offensive dorrance planetarium what the cuttingedge led dome at the arizona science center will look like atlantic american corporation report second quarter result for na fallon commander speaks at ceda breakfast atlantic american corporation report second quarter result for gamechange solar rise to third globally and second in u solar tracker market terraform lab founder do kwon pleads guilty to fraud in b terraluna collapse fhlbank san francisco invests million to preserve affordable housing in arizona metro denver inflation hold steady ahead of upcoming tariff keep your toothbrush germfree with the bril uv light toothbrush sanitizer elon musk went from promising tesla unsupervised selfdriving to le nag while los angeles burned rule to protect home from wildfire were on hold spirit airline sound the alarm on it future ability to stay in business what is ai automation and how doe it work official opening of a housing project for adult living with autism spectrum disorder in the gaspe region citizen name barclays executive a it next finance chief worth of labubus headed for black market recovered from socal home los angeles time kucoin first to support ubs umint collateral via digift bridging tokenized rwas and crypto trading bird fan are getting shortchanged reader commentary business spat between daryl hall and john oates ha been resolved in arbitration attorney say desjardins post surplus earnings of million for the second quarter of and surpasses billion in asset family safety stock life surge a parent seek peace of mind bank of america corporation nysebac stock holding decreased by finer wealth management inc tesla inc nasdaqtsla share acquired by saiph capital llc this spy pen secretly record k hd video and audio and it off now the latest national guard arrives in washington dc for trump federal takeover of local police silicon valley lawmaker want to decriminalize homelessness no one is above the law tx ag paxton seek to hold beto orourke in contempt for defying court order ai is reshaping hacking no one agrees how fast trump threatens allowing major lawsuit against fed chair powell over central bank renovation gifford fire grows to more than acre a it shift west in slo county black bear qb embrace life in maine ready to lead football team u teen influencer pilot accused of unauthorized antarctic landing reach deal to leave chile new research discovers the first known latterday saint polygamist with black ancestry israel is in talk to possibly resettle palestinian from gaza in south sudan israel is in talk to possibly resettle palestinian from gaza in south sudan trump takeover of washington law enforcement begin a national guard troop arrive texas senate pass redistricting map despite democrat walkout but house still cant consider bill with no quorum transgender woman sue over jail assault texas republican plan another special session to deliver trump more gop congressional seat texas republican plan another special session to deliver trump more gop congressional seat trump name heritage foundation ej antoni to lead bureau of labor statistic israel is in talk to possibly resettle palestinian from gaza in south sudan israel is in talk to possibly resettle palestinian from gaza in south sudan zelenskyy say putin want the rest of ukraine donetsk region a part of a ceasefire doge land big legal win a appeal court strike down preliminary injunction appeal court remove block on doge data access a familiar name raise democrat spirit in ohio senate race this is how it done here the arrest list from night with trump national guard protecting dc what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy what to know about trump potential change in federal marijuana policy dc top cop clueless on chain of command chief pamela smith deidriven disaster white house say homeless people in dc could be susceptible to jail time white house confirms trumpputin summit in anchorage calling it listening exercise what to know about trump potential change in federal marijuana policy trump use of troop for policing hasnt been seen since america wa ruled by a king trump considering lawsuit against fed a he bash chair jerome powell seeing oceanfront property in ukraine trump real estate history shape his presidency live now u attorney pirro ice and state official announce indictment of haitian gang leader we dont despise the medium enough foreign press association president condemns death of hamas journo how should american college measure merit bank fee for data access threaten the foundation of open banking deja vu another british f just made an emergency landing in japan lima one bill mcdonald honored by housingwire ap news summary at pm edt u citizen detained by ice say she wa denied water for hour israel is in talk to possibly resettle palestinian from gaza in south sudan u designates baloch separatist a a terror group over role in attack in pakistan syria u and jordan say they will work toward a lasting truce in wake of syrian sectarian clash zelensky refuse to cede donbas say doing so would give putin springboard for future offensive paxton urge texas judge to jail beto orourke over fundraising related to redistricting fight more republican join georgia competitive race for lieutenant governor more republican join georgia competitive race for lieutenant governor letter notsofree speech armstrong williams when the bench becomes the battlefield staff commentary takeaway from aps reporting on armed group recruiting child in colombia ashley biden daughter of joe and jill biden file for divorce after year of marriage county call million bond election to build jail live now department of state hold press briefing aug violent guerrilla are taking colombia child unarmed indigenous group are confronting them violent guerrilla are taking colombia child unarmed indigenous group are confronting them boom winsome earlesears just dropped another ad that abigail spanberger will have to answer for watch what to know about the putintrump summit in alaska cdc shooting linked to suspect covid vaccine belief former staff blame rfk jr hostility toward agency the palestinian journalist killed in the war in gaza endured hunger and grief the palestinian journalist killed in the war in gaza endured hunger and grief newsnation cut interview after guest call out trump hypocrisy on live tv newsnation cut interview after guest call out trump hypocrisy on live tv business spat between daryl hall and john oates ha been resolved in arbitration attorney say zelenskyy say putin want the rest of ukraine donetsk region a part of a ceasefire whats at stake a trump prepares to meet putin in alaska shacarri richardson address domestic violence arrest and apologizes to christian coleman musk blow stack after apple snub his racist chatbot texas twostep two additional bill from the texas legislative session that contractor need to know trump want to make the census count a salute to legend like kathy bates jean smart and harrison ford on finally getting their emmy flower inside senate dems summer warpath against trump trump weighs major lawsuit against powell over federal building renovation cost jimmy kimmel obtained italian citizenship in case he need to flee second trump administration it so much worse teen in northfield triple murder to forgo trial and plead guilty teenager in northfield triple murder to plead guilty trump threatens powell with major lawsuit over fed renovation ap news summary at pm edt russian troop advance in ukraine ahead of trumpputin peace summit tinfoil or not you decide damning thread tie nick fuentes to january th in a very troubling way the ncaa is a billiondollar sport behemoth that should not be a nonprofit bosnia serb leader dodik avoids prison term a election loom zelenskyy say russia want a ukrainian withdrawal from ukraine eastern donetsk region a part of a ceasefire deal zelenskyy say russia want a ukrainian withdrawal from ukraine eastern donetsk region a part of a ceasefire deal liar another gop rep face a raucous town hall angered by trump agenda liar another gop rep face a raucous town hall angered by trump agenda poll open in primary election for slain rep melissa hortmans seat pete hegseth belongs to an archconservative church network here what to know cnn slap trump with new nickname accidentally make him sound cooler sherrod brown to launch a comeback attempt for senate in ohio trump v newsom showdown land in court with family tie to the nation highest bench desantis name state sen jay collins a lieutenant governor desantis pick the chuck norris of florida politics a new top deputy allegiant airline to add direct flight from appleton to orlando here what to know bonus editorial cartoon for aug zelenskiy say ukraine wont withdraw troop from donbas first court hearing to take place tuesday in riley strain lawsuit for motion hearing trump washington dc takeover begin a national guard troop arrive</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1577,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>invesco ltd acquires share of archrock inc nysearoc invesco ltd lower position in datadog inc nasdaqddog invesco ltd sell share of enbridge inc nyseenb invesco ltd lower stake in datadog inc nasdaqddog palo alto network inc nasdaqpanw share sold by entropy technology lp entropy technology lp sell share of palo alto network inc nasdaqpanw entropy technology lp raise stock holding in plain gp holding lp nysepagp entropy technology lp purchase new share in snap inc nysesnap entropy technology lp purchase share of makemytrip limited nasdaqmmyt entropy technology lp make new investment in coinbase global inc nasdaqcoin entropy technology lp make new investment in spx technology inc nysespxc entropy technology lp invests in makemytrip limited nasdaqmmyt entropy technology lp take position in innodata inc nasdaqinod entropy technology lp sell share of mohawk industry inc nysemhk share in coinbase global inc nasdaqcoin purchased by entropy technology lp entropy technology lp buy new share in innodata inc nasdaqinod share in glacier bancorp inc nasdaqgbci purchased by entropy technology lp entropy technology lp acquires share of biomarin pharmaceutical inc nasdaqbmrn entropy technology lp purchase new stake in integer holding corporation nyseitgr share in glacier bancorp inc nasdaqgbci bought by entropy technology lp share in cellebrite di ltd nasdaqclbt bought by entropy technology lp reason pfizers yielding dividend is getting safer possible reason warren buffett shunned his favorite stock for the fourth straight quarter despite sitting on billion in cash mitsubishi ufj asset management co ltd boost stock position in urban edge property nyseue li auto inc sponsored adr nasdaqli share sold by mitsubishi ufj asset management co ltd swiss national bank ha million stock holding in interpublic group of company inc the nyseipg mitsubishi ufj asset management co ltd purchase share of bwx technology inc nysebwxt medical property trust inc nysempw share purchased by mitsubishi ufj asset management co ltd mitsubishi ufj asset management co ltd raise holding in urban edge property nyseue news corporation nasdaqnwsa share sold by swiss national bank outfront medium inc nyseout share acquired by mitsubishi ufj asset management co ltd mitsubishi ufj asset management co ltd ha million position in sl green realty corporation nyseslg mitsubishi ufj asset management co ltd decrease stake in sprout farmer market inc nasdaqsfm mitsubishi ufj asset management co ltd buy share of millrose property inc nysemrp mitsubishi ufj asset management co ltd cut holding in lucid group inc nasdaqlcid mitsubishi ufj asset management co ltd reduces stock position in liquidia technology inc nasdaqlqda mitsubishi ufj asset management co ltd ha million stock position in sprout farmer market inc nasdaqsfm mitsubishi ufj asset management co ltd increase stock holding in ducommun incorporated nysedco mitsubishi ufj asset management co ltd reduces stake in lucid group inc nasdaqlcid li auto inc sponsored adr nasdaqli share sold by mitsubishi ufj asset management co ltd mitsubishi ufj asset management co ltd ha million stake in sabra healthcare reit inc nasdaqsbra china target lithuanian bank in response to new eu sanction procept biorobotics corporation nasdaqprct share bought by mitsubishi ufj asset management co ltd mitsubishi ufj asset management co ltd buy share of esco technology inc nyseese maryland state retirement pension system reduces position in toast inc nysetost maryland state retirement pension system reduces stock position in rollins inc nyserol mitsubishi ufj asset management co ltd raise stock holding in planet lab pbc nysepl mitsubishi ufj asset management co ltd grows stock holding in caretrust reit inc nasdaqctre mitsubishi ufj asset management co ltd reduces holding in xpeng inc sponsored adr nysexpev headtohead survey metallurgical corp of china mlluy the competition maryland state retirement pension system sell share of toast inc nysetost sun community inc nysesui stock position cut by maryland state retirement pension system maryland state retirement pension system cut stake in burlington store inc nyseburl maryland state retirement pension system sell share of nutanix nasdaqntnx reviewing metallurgical corp of china mlluy and it peer financial contrast nu skin enterprise nysenus and pitanium nasdaqptnm ehang holding limited unsponsored adr nasdaqeh receives average pt from analyst mitsubishi ufj asset management co ltd acquires share of asml holding nv nasdaqasml gold price hover near record high on fed rate cut expectation entain plc otcmktsgmvhf receives average rating of moderate buy from analyst h b fuller company nyseful vp sell in stock swiss re ltd otcmktsssrey receives consensus recommendation of hold from analyst erste group bank ag otcmktsebkdy receives consensus rating of moderate buy from brokerage svenska handelsbanken ab publ otcmktssvnly receives average recommendation of reduce from brokerage april underwood sell share of zillow group inc nasdaqz stock diana sue ferguson acquires share of sally beauty holding inc nysesbh stock jayshree ullal sell share of arista network inc nyseanet stock unity software inc nyseu coo sell in stock joao magalhaes sell share of h b fuller company nyseful stock anglo american otcmktsngloy receives average recommendation of hold from analyst svenska handelsbanken ab publ otcmktssvnly receives consensus rating of reduce from analyst diana sue ferguson acquires share of sally beauty holding inc nysesbh stock centerspace nysecsr ceo purchase in stock nordea bank ab otcmktsnrdby given consensus recommendation of moderate buy by analyst april underwood sell share of zillow group inc nasdaqz stock john f sheridan acquires share of tandem diabetes care inc nasdaqtndm stock idaho strategic resource inc nyseamericanidr director kevin g shiell sell share entain plc otcmktsgmvhf given average recommendation of moderate buy by brokerage alexander blum sell share of unity software inc nyseu stock wgn in chicago hire akemi harrison a news director lumen technology nyselumn grupo televisa nysetv head to head survey a hidden fuel source beneath the midwest scientist are investigating prediction this artificial intelligence ai stock could hit a trillion valuation by top wall street forecaster revamp brinker international expectation ahead of q earnings oi glass inc nyseoi receives average rating of moderate buy from analyst oi glass inc nyseoi given consensus rating of moderate buy by analyst zion bancorporation national association ut take position in charter communication inc nasdaqchtr zion bancorporation national association ut make new investment in mettlertoledo international inc nysemtd share in midamerica apartment community inc nysemaa purchased by zion bancorporation national association ut zion bancorporation national association ut acquires share of halliburton company nysehal zion bancorporation national association ut purchase share of everest group ltd nyseeg perplexity billion dream of buying chrome is never going to happen it also kind of brilliant oscar health inc nyseoscr share bought by connor clark lunn investment management ltd zion bancorporation national association ut take position in evergy inc nasdaqevrg zion bancorporation national association ut take position in garmin ltd nysegrmn connor clark lunn investment management ltd purchase share of commercecom inc nasdaqcmrc zion bancorporation national association ut acquires share of old dominion freight line inc nasdaqodfl zion bancorporation national association ut take position in halliburton company nysehal connor clark lunn investment management ltd increase position in tuya inc sponsored adr nysetuya zion bancorporation national association ut invests in eqt corporation nyseeqt cop cartel and the new drone war on the southern border chris murphy go all in on funding bill boycott a dems seek bipartisanship letter support is plummeting for war on palestine hamas terrorist posing a aid worker taken out by israel japan pokemon happy meal promo end poorly american eagle sydney sweeney ad divide young people poll federal policing take effect in washingtonwhat to know trump cant accept bad news here how that hurt the first amendment opinion nyt chief white house reporter challenged to walk dc at night after mocking trump today in history august east germany close berlin border country once ruled by cleopatra crossword clue partner on a political ticket crossword clue congress must hear from jeffrey epstein victim about ghislaine maxwell role opinion a america navy shrink time is running out to prevent communist china from seizing control of the pacific a fix is needed so candidate wont shun public financing for governor race steve collins presidential order on homelessness push u back in time opinion today in history august east germany close berlin border saving life no more rfk risk u all in targeting mrna vaccine research we have a responsibility to house mainer who live outside opinion letter posting commandment in school is part of learning column coal need to be part of america energy future column america need affordable energy coal doesnt fit the bill more than gop attorney general call on rfk jr fda to reinstate safeguard for abortion drug red state can now protect kid from trans procedure after court victory ap news summary at am edt rural homeowner share how he avoided a hour blackout without a gas generator no one else can do this pax trumpana trump nobel peace prize resume tennessee town approves deal to turn closed prison into immigration detention facility tennessee town approves deal to turn closed prison into immigration detention facility editorial money role in american politics could get even worse white house reviewing all smithsonian museum exhibit content before america celebration in anthony scaramucci share warning about maga going marxist and maoist yale professor alleges assault on freemarket capitalism morning brief low inflation tariff truce wchina dc takeover fallout plan for postwar gaza elizabeth warren say trump promised to slash power bill in half but instead cost rose aid program vanished and ceo cashed in zelenskyy to visit berlin for european virtual meeting ahead of the trumpputin summit german government say reader sound off on investigating tish james troop in dc and hamas culpability donald trump a strongman riling up his base and investigating his enemy out of our past august senegal prime minister move to increase tobacco tax to save life stimulate economic growth paul geisler woman might see themselves in basf planetarium show another viewpoint vaccine decision show rfk jr unfit jungbunzlauer awarded platinum medal from ecovadis for sustainability performance duffy toni marie ppr team preview helix highlander letter for wednesday august dea head say phone call are coming from all over the country from fed agent wanting to help in dc letter green energy is still needed just say no to more marijuana appeal court allows arkansas firstinthenation ban on gender transition care for minor to be enforced chisholm chisholm kilpatrick ltd and national veteran legal service program challenge va denial of benefit to caregiver after veteran death havard getting by with a little help from your friend trump at the kennedy center on the same day recipient of the honor are announced trump unveils nomination for judicial post california and trump spar in court over military deployment in la obituary lois eastman death notice shirley f bennett death notice clifford g foster lewis welcome to american politics without norm this small maine town had school budget trouble then the cost got higher trump official tell census worker congress ha final say over the count not trump san diego resident rally for killed al jazeera journalist dc crime forget issue scott jennings show dems are on the losing side of a one here why trump bls nominee ha ignited a cascade of criticism from economist trump administration threatens fine jail for washington homeless bernie sander say do this instead california governor demand trump abandon texas redistricting push threatens ballot measure response wife of south korea jailed expresident yoon arrested over corruption allegation leaving a top trump administration post the president may have an ambassadorship for you leaving a top trump administration post the president may have an ambassadorship for you judge to hear argument on halting alligator alcatraz construction over environmental concern judge to hear argument on halting alligator alcatraz construction over environmental concern judge to hear argument on halting alligator alcatraz construction over environmental concern judge to hear argument on halting alligator alcatraz construction over environmental concern alligator alcatraz migrant jail could halt construction over environmental concern construction at alligator alcatraz migrant jail could be halted over environmental concern construction at alligator alcatraz migrant jail could be halted over environmental concern judge to hear argument on halting alligator alcatraz construction over environmental concern judge to hear argument on halting alligator alcatraz construction over environmental concern charles gleason lawson ap news in brief at am edt clarence page time for democrat to get serious about their political future seth meyers give trump a failing score after leaving this name out of cognitive brag cartoon democrat are desperate for this letter nevada a sanctuary state trump is making major concession to union boss is it worth it letter gov newsom and the gender confusion club letter natural gas pay off for pa letter right age for sex letter where is our humanity cartoon dont trust him the word of the day letter union leader ignores psycho with hbombs tyler t ray caswell ha nh economy headed in the right direction congressman interacts with local official business leader letter social security now but can it long persist garrison keillor one favor lord if you have a moment editorial reviewjournal socialism lead to worse thing than expensive food can we somehow make backtoschool safe again israel emerging occupation consensus letter voting restriction will do more harm than good in nh len cannon more conservative point of view required fresh grocery arrive in san diego the same day with amazon cisco earnings are imminent these most accurate analyst revise forecast ahead of earnings call stock of the day new alltime high for amd advanced ceramic and nanoceramics lead the way in a market positioned for longterm growth amazon stock gain on big expansion of perishable delivery instacart grocery stock fall investor business daily saga communication inc declares a quarterly cash dividend of per share amazon expands it perishable delivery service putting pressure on traditional grocer ap news alibaba stock soar can ai innovation sustain the growth cold wallet m stage presale offer roi before price move higher in july saga communication inc declares a quarterly cash dividend of per share amazon expands it perishable delivery service putting pressure on traditional grocer tesla diner cut menu and hour amid surging demand in hollywood the nuke race is on energy department tap startup to build a reactor by mid barrons wait the u wind industry is coming back krg baghdad strike another oil deal podcastone post percent gain in q mario paglino and gianni grossi die designer made barbies into art worksport wksp q earnings call transcript apple plot expansion into ai robot home security and smart display bloombergcom south maintains lead in construction backlog driven by population growth new york sue zelle say security lapse led to billion consumer fraud loss reuters wescap management group inc ha position in johnson johnson nysejnj msh capital advisor llc acquires share of johnson johnson nysejnj hurricane owner tom dundon strike tentative deal to buy the portland trail blazer best thriller anime show on crunchyroll amazon roll out sameday perishable grocery delivery to more than u city nvidia face b sale threat a china target h chip over security inventhelp inventor develops new refueling accessory mho pure insurance flip the script on teen driving safetyfocused on education and safety not tracking amazon expands sameday grocery delivery rival stock plunge toll brother announces final opportunity to own a new luxury home at parklynn hill community in fountain inn south carolina connecticut green bank and goodleap partner to create an aipowered virtual power plant initiative to unlock saving for homeowner and enhance grid reliability toll brother announces final opportunity to own a new luxury home at parklynn hill community in fountain inn south carolina nissan cut ariya ev price by over with a new entrylevel model crypto exchange bullish valued at nearly billion in blowout nyse debut reuters deleteme v optery top tool to erase personal data from broker vietnam hightech push to become asia next tiger by leadingre add accounttech to solution group program princeton top linkedins first u college ranking for career rigetti computing stay the course in push for quantum advantage mobile momentum how u consumer and merchant are shaping unified commerce why share of globale online are sinking today well fargo company nysewfc share purchased by financial network wealth advisor llc debt surge past trillion a interest cost eclipse defense spending intellicheck report result tampa ma firm buy naming right to nhl arena the secure mat keep your bathroom clean and safe walmart offer permanent grocery discount to m u worker why cfo must stop treating compensation a a cost twin owner opt to halt the sale and keep the club in the family adding new investor instead ai drive layoff at microsoft and intel for efficiency twin owner opt to halt sale keep club in family public notice greenlight electricity centre project participant funding available costco stock is trading lower wednesday whats going on u housing market frozen by high rate awaits fed cut for thaw what the option market tell u about galaxy digital lowes companiess option a look at what the big money is thinking united airline holdingss option frenzy what you need to know looking into midamerica apartment recent short interest is the market bullish or bearish on insulet a look into borgwarner inc price over earnings what doe the market think about united parcel service best job and career in data science kazakhstan top central asia in digital advancement ecovyst report solid q tightens fullyear guidance new opportunity for business and cooperation are created with the visit to argentina of three central american and caribbean minister and the participation of international expert in a farmer conference way a chatbot will help your customer service team outdoor holding company announces preferred stock dividend top crypto coin to buy blockdag aave link and bnb setting the standard for community strength if you bought worth of shiba inu exactly year ago here what youd have one new coin promise far bigger return sp company see no recession a economy and earnings improve youtube add custom ctas to promote tool for higher ad conversion ap business summarybrief at pm edt this data center play offer fresh buy point but test a moving average boat trader unveils innovation to transform the boatbuying and selling experience u firm stockpile import at la port amid tariff fear att million settlement you could receive up to urban one report revenue drop in q playboy to relocate global headquarters to miami beach plan to develop new playboy club tampa businessman sentenced to federal prison for tax fraud casual dining take a hit stock to watch barrons overlooked stock that are soaring even more than ai save up to on the mindblowing galaxy book pro ai is joining cybersecurity team it could be a bad idea citrin cooperman expands west coast presence with acquisition of bpsd amazon expands sameday grocery delivery to u city secure investment management rank on the inc list of america fastestgrowing private company a leap in national ranking new york ag sue zelle parent over b fraud loss seek reform bolt stock is trading higher wednesday whats going on rigetti revenue drop percent in q little pepe lilpepe presale hit a investor snap up billion token to end stage early no shoe at the startup backtoschool deal alert save when you buy of school supply at amazon tom dundon to buy the portland trail blazer from paul allen estate report blazer find buyer staying in portland coffee sold in state recalled for potential glass fragment aolcom need a boost ankers back to school sale is slashing off charger power bank and more cima selected to lead a unique and major water research project bank of america corporation nysebac share purchased by mondrian investment partner ltd union pacific train derails in texas car off track no injury washington dc police union accuses city of cooking the book with crime stats kiss star say theyre grateful for kennedy center honor stevens democrat need a creative approach to the midterm election ltte frustrated by year of stalled street rotary and tree work fagan the heritage foundation founder legacy is complicated federal court allows doge access to sensitive data on million of american rfk jr is trying to make covid great again why did we build community that discourage walking the ethical life podcast the latest trump warns of very severe consequence if putin continues ukraine war australia punter playing at nebraska break down while discussing homesickness biden admin scrapped bestqualified standard for air traffic controller academy doc show flesheating bacteria found in swimmer who wa at cape cod beach trump shock troop coming to a city near you federal agent will be out on patrol in washington the white house say federal agent will be out on patrol in washington the white house say federal agent will be out on patrol in washington the white house say federal agent will be out on patrol in washington the white house say federal agent will be out on patrol in washington the white house say federal agent will be out on patrol in washington the white house say why democrat have limited power to fight republican redistricting trump real endgame with crime in dc is coming into view national guard presence will grow in dc wednesday night white house say child pregnant woman mistreated in immigration detention sen ossoff say what bangladesh ha achieved in the year since it revolution chesapeake council to allow member virtual participation in some meeting environmental concern could halt construction at florida alligator alcatraz immigration jail environmental concern could halt construction at florida alligator alcatraz immigration jail reporter share eyewitness account from front line of the russiaukraine war federal agent will be out on patrol in washington the white house say trump is engaged in stalinist attempt to rewrite u history axelrod warns live now texas house democrat hold news conference with indiana lawmaker trump visit kennedy center and announces honoree see the full list gaslighter king gavin newsom get ratioed into orbit for attacking stephen miller crime stat truth can public medium survive did india really shoot down an f fighting falcon fighter a freedom caucus target jackson hole housing policy gordon back community solution state leader take on record fee california wa a model for transparency now the capitol operates in the dark california wa a model for transparency now the capitol operates in the dark port a deep dive into how the sausage get made in north dakota trump say he doesnt believe he can convince putin to stop bombing ukrainian civilian att million settlement you could receive up to tulsi gabbard release damning email that put clapper in the hot seat judge is skeptical of justice department lawsuit against federal judge a trump try to limit power of judiciary trump threatens very severe consequence if russia doesnt agree to end ukraine war trump predicts little progress in potential shutdown talk with crazy schumer jeffries zohran mamdani take aim at trump immigration policy in fiery staten island speech we are fighting to keep nyc a sanctuary city auditor california could save million a year by letting state employee work remote trump warns putin of very severe consequence if ukraine war continues trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan new york claim zelles shoddy security enabled a billion dollar in scam wall street journal give trump a stern warning new connection credit union clubhouse coming to riverside golf course judge skeptical of trump administration suit against maryland judge will rule by labor day judge skeptical of trump administration suit against maryland judge will rule by labor day judge skeptical of trump administration suit against maryland judge will rule by labor day judge skeptical of trump administration suit against maryland judge will rule by labor day judge skeptical of trump administration suit against maryland judge will rule by labor day judge skeptical of trump administration suit against maryland judge will rule by labor day he a bit of a mouth local react to vance visit president trump announces sylvester stallone kiss a kennedy center honoree trump name kennedy center honoree say hell host award show brit throw vance a not welcome party on his latest vacation trump tariff are forcing canada to address it money laundering problem trump administration lawsuit against all of maryland federal judge meet skepticism in court u senate approves m to expand willmar veterinary testing lab trump pledged to move homeless people from washington what we know and dont know about his plan allegedly nonpartisan common cause unmasked cheering leftist gerrymandering while condemning the gop pocatello model railroad and historical society open house set for saturday ap news summary at pm edt the latest trump warns of very severe consequence if putin continues ukraine war nyc ramp up effort to remove mentally ill from street subway trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia epa terminates center for rural affair million solar grant trump look to extend dc police takeover beyond day trump look to extend dc police takeover beyond day harvard and the trump administration are nearing a settlement including a million payment harvard and the trump administration are nearing a settlement including a million payment harvard and the trump administration are nearing a settlement including a million payment trump detail expectation for meeting with putin chicago rapper king yella hold chest fall over after drinking crown royal throughout interview a trump turn dc into a fascist laboratory we must mount our own defense what to know about the putintrump summit in alaska maga hang mission accomplished hype on trump tariff jonah goldberg</t>
+          <t>invesco ltd acquires share of archrock inc nysearoc invesco ltd lower position in datadog inc nasdaqddog invesco ltd sell share of enbridge inc nyseenb invesco ltd lower stake in datadog inc nasdaqddog palo alto network inc nasdaqpanw share sold by entropy technology lp entropy technology lp sell share of palo alto network inc nasdaqpanw entropy technology lp raise stock holding in plain gp holding lp nysepagp entropy technology lp purchase new share in snap inc nysesnap entropy technology lp purchase share of makemytrip limited nasdaqmmyt entropy technology lp make new investment in coinbase global inc nasdaqcoin entropy technology lp make new investment in spx technology inc nysespxc entropy technology lp invests in makemytrip limited nasdaqmmyt entropy technology lp take position in innodata inc nasdaqinod entropy technology lp sell share of mohawk industry inc nysemhk share in coinbase global inc nasdaqcoin purchased by entropy technology lp entropy technology lp buy new share in innodata inc nasdaqinod share in glacier bancorp inc nasdaqgbci purchased by entropy technology lp entropy technology lp acquires share of biomarin pharmaceutical inc nasdaqbmrn entropy technology lp purchase new stake in integer holding corporation nyseitgr share in glacier bancorp inc nasdaqgbci bought by entropy technology lp share in cellebrite di ltd nasdaqclbt bought by entropy technology lp reason pfizers yielding dividend is getting safer possible reason warren buffett shunned his favorite stock for the fourth straight quarter despite sitting on billion in cash mitsubishi ufj asset management co ltd boost stock position in urban edge property nyseue li auto inc sponsored adr nasdaqli share sold by mitsubishi ufj asset management co ltd swiss national bank ha million stock holding in interpublic group of company inc the nyseipg mitsubishi ufj asset management co ltd purchase share of bwx technology inc nysebwxt medical property trust inc nysempw share purchased by mitsubishi ufj asset management co ltd mitsubishi ufj asset management co ltd raise holding in urban edge property nyseue news corporation nasdaqnwsa share sold by swiss national bank outfront medium inc nyseout share acquired by mitsubishi ufj asset management co ltd mitsubishi ufj asset management co ltd ha million position in sl green realty corporation nyseslg mitsubishi ufj asset management co ltd decrease stake in sprout farmer market inc nasdaqsfm mitsubishi ufj asset management co ltd buy share of millrose property inc nysemrp mitsubishi ufj asset management co ltd cut holding in lucid group inc nasdaqlcid mitsubishi ufj asset management co ltd reduces stock position in liquidia technology inc nasdaqlqda mitsubishi ufj asset management co ltd ha million stock position in sprout farmer market inc nasdaqsfm mitsubishi ufj asset management co ltd increase stock holding in ducommun incorporated nysedco mitsubishi ufj asset management co ltd reduces stake in lucid group inc nasdaqlcid li auto inc sponsored adr nasdaqli share sold by mitsubishi ufj asset management co ltd mitsubishi ufj asset management co ltd ha million stake in sabra healthcare reit inc nasdaqsbra china target lithuanian bank in response to new eu sanction procept biorobotics corporation nasdaqprct share bought by mitsubishi ufj asset management co ltd mitsubishi ufj asset management co ltd buy share of esco technology inc nyseese maryland state retirement pension system reduces position in toast inc nysetost maryland state retirement pension system reduces stock position in rollins inc nyserol mitsubishi ufj asset management co ltd raise stock holding in planet lab pbc nysepl mitsubishi ufj asset management co ltd grows stock holding in caretrust reit inc nasdaqctre mitsubishi ufj asset management co ltd reduces holding in xpeng inc sponsored adr nysexpev headtohead survey metallurgical corp of china mlluy the competition maryland state retirement pension system sell share of toast inc nysetost sun community inc nysesui stock position cut by maryland state retirement pension system maryland state retirement pension system cut stake in burlington store inc nyseburl maryland state retirement pension system sell share of nutanix nasdaqntnx reviewing metallurgical corp of china mlluy and it peer financial contrast nu skin enterprise nysenus and pitanium nasdaqptnm ehang holding limited unsponsored adr nasdaqeh receives average pt from analyst mitsubishi ufj asset management co ltd acquires share of asml holding nv nasdaqasml gold price hover near record high on fed rate cut expectation entain plc otcmktsgmvhf receives average rating of moderate buy from analyst h b fuller company nyseful vp sell in stock swiss re ltd otcmktsssrey receives consensus recommendation of hold from analyst erste group bank ag otcmktsebkdy receives consensus rating of moderate buy from brokerage svenska handelsbanken ab publ otcmktssvnly receives average recommendation of reduce from brokerage april underwood sell share of zillow group inc nasdaqz stock diana sue ferguson acquires share of sally beauty holding inc nysesbh stock jayshree ullal sell share of arista network inc nyseanet stock unity software inc nyseu coo sell in stock joao magalhaes sell share of h b fuller company nyseful stock anglo american otcmktsngloy receives average recommendation of hold from analyst svenska handelsbanken ab publ otcmktssvnly receives consensus rating of reduce from analyst diana sue ferguson acquires share of sally beauty holding inc nysesbh stock centerspace nysecsr ceo purchase in stock nordea bank ab otcmktsnrdby given consensus recommendation of moderate buy by analyst april underwood sell share of zillow group inc nasdaqz stock john f sheridan acquires share of tandem diabetes care inc nasdaqtndm stock idaho strategic resource inc nyseamericanidr director kevin g shiell sell share entain plc otcmktsgmvhf given average recommendation of moderate buy by brokerage alexander blum sell share of unity software inc nyseu stock wgn in chicago hire akemi harrison a news director lumen technology nyselumn grupo televisa nysetv head to head survey a hidden fuel source beneath the midwest scientist are investigating prediction this artificial intelligence ai stock could hit a trillion valuation by top wall street forecaster revamp brinker international expectation ahead of q earnings oi glass inc nyseoi receives average rating of moderate buy from analyst oi glass inc nyseoi given consensus rating of moderate buy by analyst zion bancorporation national association ut take position in charter communication inc nasdaqchtr zion bancorporation national association ut make new investment in mettlertoledo international inc nysemtd share in midamerica apartment community inc nysemaa purchased by zion bancorporation national association ut zion bancorporation national association ut acquires share of halliburton company nysehal zion bancorporation national association ut purchase share of everest group ltd nyseeg perplexity billion dream of buying chrome is never going to happen it also kind of brilliant oscar health inc nyseoscr share bought by connor clark lunn investment management ltd zion bancorporation national association ut take position in evergy inc nasdaqevrg zion bancorporation national association ut take position in garmin ltd nysegrmn connor clark lunn investment management ltd purchase share of commercecom inc nasdaqcmrc zion bancorporation national association ut acquires share of old dominion freight line inc nasdaqodfl zion bancorporation national association ut take position in halliburton company nysehal connor clark lunn investment management ltd increase position in tuya inc sponsored adr nysetuya zion bancorporation national association ut invests in eqt corporation nyseeqt cop cartel and the new drone war on the southern border chris murphy go all in on funding bill boycott a dems seek bipartisanship letter support is plummeting for war on palestine hamas terrorist posing a aid worker taken out by israel japan pokemon happy meal promo end poorly american eagle sydney sweeney ad divide young people poll federal policing take effect in washingtonwhat to know trump cant accept bad news here how that hurt the first amendment opinion nyt chief white house reporter challenged to walk dc at night after mocking trump today in history august east germany close berlin border country once ruled by cleopatra crossword clue partner on a political ticket crossword clue congress must hear from jeffrey epstein victim about ghislaine maxwell role opinion a america navy shrink time is running out to prevent communist china from seizing control of the pacific a fix is needed so candidate wont shun public financing for governor race steve collins presidential order on homelessness push u back in time opinion today in history august east germany close berlin border saving life no more rfk risk u all in targeting mrna vaccine research we have a responsibility to house mainer who live outside opinion letter posting commandment in school is part of learning column coal need to be part of america energy future column america need affordable energy coal doesnt fit the bill more than gop attorney general call on rfk jr fda to reinstate safeguard for abortion drug red state can now protect kid from trans procedure after court victory ap news summary at am edt rural homeowner share how he avoided a hour blackout without a gas generator no one else can do this pax trumpana trump nobel peace prize resume tennessee town approves deal to turn closed prison into immigration detention facility tennessee town approves deal to turn closed prison into immigration detention facility editorial money role in american politics could get even worse white house reviewing all smithsonian museum exhibit content before america celebration in anthony scaramucci share warning about maga going marxist and maoist yale professor alleges assault on freemarket capitalism morning brief low inflation tariff truce wchina dc takeover fallout plan for postwar gaza elizabeth warren say trump promised to slash power bill in half but instead cost rose aid program vanished and ceo cashed in zelenskyy to visit berlin for european virtual meeting ahead of the trumpputin summit german government say reader sound off on investigating tish james troop in dc and hamas culpability donald trump a strongman riling up his base and investigating his enemy out of our past august senegal prime minister move to increase tobacco tax to save life stimulate economic growth paul geisler woman might see themselves in basf planetarium show another viewpoint vaccine decision show rfk jr unfit jungbunzlauer awarded platinum medal from ecovadis for sustainability performance duffy toni marie ppr team preview helix highlander letter for wednesday august dea head say phone call are coming from all over the country from fed agent wanting to help in dc letter green energy is still needed just say no to more marijuana appeal court allows arkansas firstinthenation ban on gender transition care for minor to be enforced chisholm chisholm kilpatrick ltd and national veteran legal service program challenge va denial of benefit to caregiver after veteran death havard getting by with a little help from your friend trump at the kennedy center on the same day recipient of the honor are announced trump unveils nomination for judicial post california and trump spar in court over military deployment in la obituary lois eastman death notice shirley f bennett death notice clifford g foster lewis welcome to american politics without norm this small maine town had school budget trouble then the cost got higher trump official tell census worker congress ha final say over the count not trump san diego resident rally for killed al jazeera journalist dc crime forget issue scott jennings show dems are on the losing side of a one here why trump bls nominee ha ignited a cascade of criticism from economist trump administration threatens fine jail for washington homeless bernie sander say do this instead california governor demand trump abandon texas redistricting push threatens ballot measure response wife of south korea jailed expresident yoon arrested over corruption allegation leaving a top trump administration post the president may have an ambassadorship for you leaving a top trump administration post the president may have an ambassadorship for you judge to hear argument on halting alligator alcatraz construction over environmental concern judge to hear argument on halting alligator alcatraz construction over environmental concern judge to hear argument on halting alligator alcatraz construction over environmental concern judge to hear argument on halting alligator alcatraz construction over environmental concern alligator alcatraz migrant jail could halt construction over environmental concern construction at alligator alcatraz migrant jail could be halted over environmental concern construction at alligator alcatraz migrant jail could be halted over environmental concern judge to hear argument on halting alligator alcatraz construction over environmental concern judge to hear argument on halting alligator alcatraz construction over environmental concern charles gleason lawson ap news in brief at am edt clarence page time for democrat to get serious about their political future seth meyers give trump a failing score after leaving this name out of cognitive brag cartoon democrat are desperate for this letter nevada a sanctuary state trump is making major concession to union boss is it worth it letter gov newsom and the gender confusion club letter natural gas pay off for pa letter right age for sex letter where is our humanity cartoon dont trust him the word of the day letter union leader ignores psycho with hbombs tyler t ray caswell ha nh economy headed in the right direction congressman interacts with local official business leader letter social security now but can it long persist garrison keillor one favor lord if you have a moment editorial reviewjournal socialism lead to worse thing than expensive food can we somehow make backtoschool safe again israel emerging occupation consensus letter voting restriction will do more harm than good in nh len cannon more conservative point of view required fresh grocery arrive in san diego the same day with amazon cisco earnings are imminent these most accurate analyst revise forecast ahead of earnings call stock of the day new alltime high for amd advanced ceramic and nanoceramics lead the way in a market positioned for longterm growth amazon stock gain on big expansion of perishable delivery instacart grocery stock fall investor business daily saga communication inc declares a quarterly cash dividend of per share amazon expands it perishable delivery service putting pressure on traditional grocer ap news alibaba stock soar can ai innovation sustain the growth cold wallet m stage presale offer roi before price move higher in july saga communication inc declares a quarterly cash dividend of per share amazon expands it perishable delivery service putting pressure on traditional grocer tesla diner cut menu and hour amid surging demand in hollywood the nuke race is on energy department tap startup to build a reactor by mid barrons wait the u wind industry is coming back krg baghdad strike another oil deal podcastone post percent gain in q mario paglino and gianni grossi die designer made barbies into art worksport wksp q earnings call transcript apple plot expansion into ai robot home security and smart display bloombergcom south maintains lead in construction backlog driven by population growth new york sue zelle say security lapse led to billion consumer fraud loss reuters wescap management group inc ha position in johnson johnson nysejnj msh capital advisor llc acquires share of johnson johnson nysejnj hurricane owner tom dundon strike tentative deal to buy the portland trail blazer best thriller anime show on crunchyroll amazon roll out sameday perishable grocery delivery to more than u city nvidia face b sale threat a china target h chip over security inventhelp inventor develops new refueling accessory mho pure insurance flip the script on teen driving safetyfocused on education and safety not tracking amazon expands sameday grocery delivery rival stock plunge toll brother announces final opportunity to own a new luxury home at parklynn hill community in fountain inn south carolina connecticut green bank and goodleap partner to create an aipowered virtual power plant initiative to unlock saving for homeowner and enhance grid reliability toll brother announces final opportunity to own a new luxury home at parklynn hill community in fountain inn south carolina nissan cut ariya ev price by over with a new entrylevel model crypto exchange bullish valued at nearly billion in blowout nyse debut reuters deleteme v optery top tool to erase personal data from broker vietnam hightech push to become asia next tiger by leadingre add accounttech to solution group program princeton top linkedins first u college ranking for career rigetti computing stay the course in push for quantum advantage mobile momentum how u consumer and merchant are shaping unified commerce why share of globale online are sinking today well fargo company nysewfc share purchased by financial network wealth advisor llc debt surge past trillion a interest cost eclipse defense spending intellicheck report result tampa ma firm buy naming right to nhl arena the secure mat keep your bathroom clean and safe walmart offer permanent grocery discount to m u worker why cfo must stop treating compensation a a cost twin owner opt to halt the sale and keep the club in the family adding new investor instead ai drive layoff at microsoft and intel for efficiency twin owner opt to halt sale keep club in family public notice greenlight electricity centre project participant funding available costco stock is trading lower wednesday whats going on u housing market frozen by high rate awaits fed cut for thaw what the option market tell u about galaxy digital lowes company option a look at what the big money is thinking united airline holding option frenzy what you need to know looking into midamerica apartment recent short interest is the market bullish or bearish on insulet a look into borgwarner inc price over earnings what doe the market think about united parcel service best job and career in data science kazakhstan top central asia in digital advancement ecovyst report solid q tightens fullyear guidance new opportunity for business and cooperation are created with the visit to argentina of three central american and caribbean minister and the participation of international expert in a farmer conference way a chatbot will help your customer service team outdoor holding company announces preferred stock dividend top crypto coin to buy blockdag aave link and bnb setting the standard for community strength if you bought worth of shiba inu exactly year ago here what youd have one new coin promise far bigger return sp company see no recession a economy and earnings improve youtube add custom ctas to promote tool for higher ad conversion ap business summarybrief at pm edt this data center play offer fresh buy point but test a moving average boat trader unveils innovation to transform the boatbuying and selling experience u firm stockpile import at la port amid tariff fear att million settlement you could receive up to urban one report revenue drop in q playboy to relocate global headquarters to miami beach plan to develop new playboy club tampa businessman sentenced to federal prison for tax fraud casual dining take a hit stock to watch barrons overlooked stock that are soaring even more than ai save up to on the mindblowing galaxy book pro ai is joining cybersecurity team it could be a bad idea citrin cooperman expands west coast presence with acquisition of bpsd amazon expands sameday grocery delivery to u city secure investment management rank on the inc list of america fastestgrowing private company a leap in national ranking new york ag sue zelle parent over b fraud loss seek reform bolt stock is trading higher wednesday whats going on rigetti revenue drop percent in q little pepe lilpepe presale hit a investor snap up billion token to end stage early no shoe at the startup backtoschool deal alert save when you buy of school supply at amazon tom dundon to buy the portland trail blazer from paul allen estate report blazer find buyer staying in portland coffee sold in state recalled for potential glass fragment aolcom need a boost ankers back to school sale is slashing off charger power bank and more cima selected to lead a unique and major water research project bank of america corporation nysebac share purchased by mondrian investment partner ltd union pacific train derails in texas car off track no injury washington dc police union accuses city of cooking the book with crime stats kiss star say theyre grateful for kennedy center honor stevens democrat need a creative approach to the midterm election ltte frustrated by year of stalled street rotary and tree work fagan the heritage foundation founder legacy is complicated federal court allows doge access to sensitive data on million of american rfk jr is trying to make covid great again why did we build community that discourage walking the ethical life podcast the latest trump warns of very severe consequence if putin continues ukraine war australia punter playing at nebraska break down while discussing homesickness biden admin scrapped bestqualified standard for air traffic controller academy doc show flesheating bacteria found in swimmer who wa at cape cod beach trump shock troop coming to a city near you federal agent will be out on patrol in washington the white house say federal agent will be out on patrol in washington the white house say federal agent will be out on patrol in washington the white house say federal agent will be out on patrol in washington the white house say federal agent will be out on patrol in washington the white house say federal agent will be out on patrol in washington the white house say why democrat have limited power to fight republican redistricting trump real endgame with crime in dc is coming into view national guard presence will grow in dc wednesday night white house say child pregnant woman mistreated in immigration detention sen ossoff say what bangladesh ha achieved in the year since it revolution chesapeake council to allow member virtual participation in some meeting environmental concern could halt construction at florida alligator alcatraz immigration jail environmental concern could halt construction at florida alligator alcatraz immigration jail reporter share eyewitness account from front line of the russiaukraine war federal agent will be out on patrol in washington the white house say trump is engaged in stalinist attempt to rewrite u history axelrod warns live now texas house democrat hold news conference with indiana lawmaker trump visit kennedy center and announces honoree see the full list gaslighter king gavin newsom get ratioed into orbit for attacking stephen miller crime stat truth can public medium survive did india really shoot down an f fighting falcon fighter a freedom caucus target jackson hole housing policy gordon back community solution state leader take on record fee california wa a model for transparency now the capitol operates in the dark california wa a model for transparency now the capitol operates in the dark port a deep dive into how the sausage get made in north dakota trump say he doesnt believe he can convince putin to stop bombing ukrainian civilian att million settlement you could receive up to tulsi gabbard release damning email that put clapper in the hot seat judge is skeptical of justice department lawsuit against federal judge a trump try to limit power of judiciary trump threatens very severe consequence if russia doesnt agree to end ukraine war trump predicts little progress in potential shutdown talk with crazy schumer jeffries zohran mamdani take aim at trump immigration policy in fiery staten island speech we are fighting to keep nyc a sanctuary city auditor california could save million a year by letting state employee work remote trump warns putin of very severe consequence if ukraine war continues trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan trump pledged to move homeless people from washington what we know and dont know about his plan new york claim zelles shoddy security enabled a billion dollar in scam wall street journal give trump a stern warning new connection credit union clubhouse coming to riverside golf course judge skeptical of trump administration suit against maryland judge will rule by labor day judge skeptical of trump administration suit against maryland judge will rule by labor day judge skeptical of trump administration suit against maryland judge will rule by labor day judge skeptical of trump administration suit against maryland judge will rule by labor day judge skeptical of trump administration suit against maryland judge will rule by labor day judge skeptical of trump administration suit against maryland judge will rule by labor day he a bit of a mouth local react to vance visit president trump announces sylvester stallone kiss a kennedy center honoree trump name kennedy center honoree say hell host award show brit throw vance a not welcome party on his latest vacation trump tariff are forcing canada to address it money laundering problem trump administration lawsuit against all of maryland federal judge meet skepticism in court u senate approves m to expand willmar veterinary testing lab trump pledged to move homeless people from washington what we know and dont know about his plan allegedly nonpartisan common cause unmasked cheering leftist gerrymandering while condemning the gop pocatello model railroad and historical society open house set for saturday ap news summary at pm edt the latest trump warns of very severe consequence if putin continues ukraine war nyc ramp up effort to remove mentally ill from street subway trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia trumpputin summit on ukraine is latest chapter in alaska long history and tension with russia epa terminates center for rural affair million solar grant trump look to extend dc police takeover beyond day trump look to extend dc police takeover beyond day harvard and the trump administration are nearing a settlement including a million payment harvard and the trump administration are nearing a settlement including a million payment harvard and the trump administration are nearing a settlement including a million payment trump detail expectation for meeting with putin chicago rapper king yella hold chest fall over after drinking crown royal throughout interview a trump turn dc into a fascist laboratory we must mount our own defense what to know about the putintrump summit in alaska maga hang mission accomplished hype on trump tariff jonah goldberg</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>boring stock offering an over annual dividend yield there a small problem with trump export deal with nvidia and amd the constitution say it illegal fortune trump chief intervened to save rfk jr top vaccine aide politico revisiting carrie bradshaws apartment in sex and the city and and just like that fed face high bar for big cut despite white house pressure the new york time fed face high bar for big cut despite white house pressure bitcoin price soar to a etf inflow surge how trump get what he want from company nbc news wanf in atlanta release new schedule for life after cbs home for sale in manhattan and brooklyn the live music business is booming now rap is getting a piece too there money to be made in maha food company want in cetera investment adviser sell share of camden property trust nysecpt the cost to rebuild a home after a natural disaster is rising pnc financial service group inc acquires share of on holding ag nyseonon pnc financial service group inc raise position in five below inc nasdaqfive pnc financial service group inc purchase share of the madison square garden company nysemsgs tko group holding inc nysetko share acquired by pnc financial service group inc the latest chatgpt is supposed to be phd level smart it cant even label a map crypto presale alert blockchainfx bfx set for explosive growth can it beat bitcoin hyper blockdag big tech ai boom is reordering the u power grid the new york time crisis intervention effort yield impressive result trump is tightening the screw on corporate america and ceo are staying mum titanbay appoints exubs exec a head of switzerland is xrp a buy while it below best spy tv show to watch now on peacock in vipshop report unaudited second quarter financial result instacart is partying like it with third eye blind frosted tip and ring pop new report cleaner manufacturing could save life and prevent million of asthma attack titanbay appoints exubs exec a head of switzerland trump is tightening the screw on corporate america and ceo are staying mum npr weibo announces second quarter unaudited financial result ai development is accelerating vanguard etf to buy right now inside thailand frantic effort to close tariff loophole to the u china offer interest subsidy for loan amid sluggish economy pinterest share just sank time to buy the dip or run for the hill cava group nysecava price target cut to by analyst at morgan stanley nvidia corporation nasdaqnvda share purchased by richard c young co ltd kingsview wealth management llc purchase share of nvidia corporation nasdaqnvda cava group nysecava price target lowered to at citigroup tat technology tatt buy rating reaffirmed at lake street capital summit x llc purchase share of amazoncom inc nasdaqamzn nvidia corporation nasdaqnvda share sold by forum financial management lp repay nasdaqrpay receives neutral rating from ubs group snowflake nysesnow given new price target at ubs group nvidia corporation nasdaqnvda share sold by asset advisor investment management llc rivian automotive nasdaqrivn given new price target at morgan stanley fluence energy nasdaqflnc price target lowered to at royal bank of canada commerzbank aktiengesellschaft fi ha million stock holding in nvidia corporation nasdaqnvda meet the yield dividend stock that could soar in brachioplasty market to surpass usd billion by fueled by rising aesthetic awareness and technological advancement sn insider titanbay appoints paul essen bakery owner say they closed for a mental health break their employee say theyve been ghosted wkmg in orlando give news director autumn jones all the job vanguard group inc trim stock holding in blueprint medicine corporation nasdaqbpmc vanguard group inc ha million stock position in interdigital inc nasdaqidcc charles schwab investment management inc cut stock holding in bright horizon family solution inc nysebfam fluor corporation nyseflr share sold by vanguard group inc charles schwab investment management inc sell share of mattel inc nasdaqmat clearwater analytics holding inc nysecwan share acquired by vanguard group inc agco corporation nyseagco share sold by vanguard group inc vanguard group inc reduces position in ollies bargain outlet holding inc nasdaqolli vanguard group inc sell share of first american financial corporation nysefaf charles schwab investment management inc reduces holding in ally financial inc nyseally u bancorp de acquires share of graphic packaging holding company nysegpk vanguard group inc reduces position in lantheus holding inc nasdaqlnth charles schwab investment management inc boost position in dropbox inc nasdaqdbx vanguard group inc cut position in lincoln national corporation nyselnc vanguard group inc decrease position in itron inc nasdaqitri vanguard group inc trim stake in dropbox inc nasdaqdbx charles schwab investment management inc sell share of spotify technology nysespot chart industry inc nysegtls share purchased by charles schwab investment management inc nov inc nysenov share bought by vanguard group inc charles schwab investment management inc ha million stock position in spx technology inc nysespxc charles schwab investment management inc reduces position in talen energy corporation nasdaqtln curtisswright corporation nysecw position increased by charles schwab investment management inc vanguard group inc sell share of mattel inc nasdaqmat u bancorp de reduces holding in bce inc nysebce vanguard group inc lower stock holding in chart industry inc nysegtls atrium wealth solution inc ha stock position in ppg industry inc nyseppg analyst issue forecast for saputos q earnings tsesap atrium wealth solution inc buy share of vanguard international dividend appreciation etf nasdaqvigi vanguard group inc sell share of antero midstream corporation nyseam atrium wealth solution inc ha stake in southwest gas corporation nyseswx atrium wealth solution inc reduces position in sarepta therapeutic inc nasdaqsrpt vanguard group inc ha million holding in simpson manufacturing company inc nysessd vanguard group inc sell share of universal display corporation nasdaqoled vanguard group inc decrease stock holding in flowserve corporation nysefls share in spdr sp capital market etf nysearcakce bought by atrium wealth solution inc vanguard group inc sell share of credo technology group holding ltd nasdaqcrdo vanguard group inc acquires share of american airline group inc nasdaqaal atrium wealth solution inc invests in ugi corporation nyseugi atrium wealth solution inc decrease position in ingersoll rand inc nyseir home bancshares inc nysehomb share sold by atrium wealth solution inc vanguard group inc sell share of option care health inc nasdaqopch atrium wealth solution inc ha stock holding in rb global inc nyserba sl green realty corporation nyseslg share bought by vanguard group inc atrium wealth solution inc make new investment in crown holding inc nysecck notice regarding uaborkela financial statement for month period ended june nagarro release unaudited q result post yoy revenue growth in constant currency and increase in gross profit despite global macroeconomic challenge parent dont want cell phone ban at school we want smarter rule opinion mexico under pressure from trump sends cartel member to u the key to success at trumpputin alaska summit on ukraine low expectation opinion welcome to the menodivorce why woman arent sweating marriage in a sea of hot flash a tropical storm erin track west palm beach advises resident to stay alert prepared letter new challenge require a new congressman cctv foreign journalist open blind box at shuiting gate america must secure social security now republican pitch trump domestic policy agenda in iowa but some entrepreneur arent yet sold cnn politics the latest chatgpt is supposed to be phd level smart it cant even label a map wfp is leveraging it power in the mayoral race firstofitskind micropathway initiative now help community college build industryaligned training program my legacy is of broken men michael thomas on dream alcoholism and black fatherhood conquistador stolen yearold receipt return to mexico priscilla presley accused of hastening lisa mary death for financial gain memoir on a hill finding the best way to tell the story of america letter why now and why all the surprise eye on art frazier brings lowell to life in all gallery show rosner appointed ferc chair a trump move to reshape regulator u deploys force to take on latin american drug cartel in the southern caribbean today in history august fdr sign social security act now jimmy fallon is using taylor swift to suggest trump had sinister tie to epstein activist amariyanna copenys hometown crossword clue it not just dc republican seem happy to let trump do whatever he want opinion letter wondering if congressman still walk with jesus cincinnati beating suspect face year in prison after new charge from doj no peace without ukraine trumpputin alaska talk call for sober strategy oil city civic center to offer tour of national transit building thompson cosponsors bill to expand k career counseling idea opinion tom durkin come together debence receives grant for kid program grove city college ranked no for most religious student in u year ago aug lucas foley go to bat for bay state ag should too brokerage set cargojet inc tsecjt pt at c brokerage set penn entertainment inc nasdaqpenn target price at cbre group inc nysecbre receives consensus target price from analyst under armour nyseuaa price target lowered to at telsey advisory group john hood german settler helped shape nc rebellion today in historyaug failed gop candidate sentenced to year in connection with shooting spree at democrat official home stage mechanic and hanover in worcester make going out fun prokidney corp nasdaqprok receives average rating of hold from analyst spx technology inc nysespxc given average rating of buy by brokerage adapthealth corp nasdaqahco receives consensus target price from analyst contineum therapeutic inc nasdaqctnm receives consensus price target from brokerage on inc nyseontf receives consensus rating of hold from brokerage ap news summary at am edt douglas cohn and eleanor clift the shamed the shameless and the shirked editorial why is healey hesitating to call for tompkins resignation guest opinion erich menzel sculpture and art in the park event put loveland on the map ap news summary at am edt morning brief arrest since trump dc takeover trumpputin peace talk immigrant exodus social security is the cornerstone of retirement income fbi agent are again pulled from their day job to address a trump priority cnn politics cost of living in california still a discussion at county level propalestinian protester hold demonstration outside ivp reader sound off on turning against israel misusing troop and reckless bikers sbdc guide resident on starting legal homebased food business icf international nasdaqicfi price target raised to hang feng technology innovation co ltd fofo announces august th ipo alaska a source of russian imperial nostalgia powerful sister of north korean leader denies removal of frontline speaker cal thomas washington dc then and now emera tseema price target raised to c expensify nasdaqexfy cut to hold at wall street zen emera tseema price target raised to c rosenblatt security cut hut nasdaqhut price target to irs reportedly confirms stimulus check for eligible american rumor of august payout debunked plan late summer rollout american healthcare reit nyseahr price target raised to trump eas space regulation in boost for elon musk spacex jeff bezos blue origin and more pearson nysepso downgraded to hold rating by wall street zen first interstate bancsystem nasdaqfibk cut to sell at wall street zen morgan stanley cut primo brand nyseprmb price target to speaking out no longer interested in preventing pain and suffering north korea denies removing border loudspeaker ct real estate investment trust tsecrtun price target raised to c national bankshares cut boralex tseblx price target to c constellation software tsecsu price target raised to c share buyback program approved by plus lonplus board of director hong kong lashed with another torrential downpour redwire nyserdw price target lowered to at canaccord genuity group trisura group tsetsu price target raised to c gdi integrated facility service tsegdi downgraded by td security to hold leon furniture tselnf price target raised to c power co of canada tsepow price target raised to c at desjardins savaria tsesis price target raised to c saputo tsesap price target raised to c letter the right betrays every value it claim to hold youngkin order investigation into claim staff at virginia school arranged abortion without parental consent ap news summary at am edt flower food flo expected to announce earnings on friday kodiak gas service nysekgs to repurchase million in outstanding share trump nobel peace prize push gain steam president clinch backing from pakistan cambodia israel ahead of meeting with putin gop senator spill on the illegal measure he take to deal with dc crime fear softcat plc lonsct insider buy in stock jpmorgan global core real asset limited lonjara insider sell in stock fresnillo lonfres stock price expected to rise royal bank of canada analyst say asiamet resource lonars receives house stock rating from shore capital jpmorgan global core real asset limited lonjara insider sell in stock battalion oil post q revenue drop netease stock drop after chinese video game firm miss sale target aebi schmidt group building momentum after merging with the shyft group strong order backlog additional synergy upside and commitment to delever ask a real estate pro how can we stop complaining neighbor harassing behavior ask a real estate pro how can we stop complaining neighbor harassing behavior bessent see nvidia amd china agreement a a model for others nov declares regular quarterly dividend permanent magnet market worth billion by exclusive report by marketsandmarketstm clean energy tax credit market participant remain bullish the wall street journal rare earth rally after department of defense set a price floor aery technology report record q fy result cash flow positive m net income turnaround and strongest start to a fiscal year in company history envirogold global retains cantor fitzgerald a financial advisor p announces dual listing on nyse texas dividendpaying dow jones stock to buy in august u and australia support for nova estelle project realme pro review is it worth a buy shattuck lab report second quarter financial result and recent business highlight medium advisory air canada to hold medium availability with senior executive today aimia report second quarter result reiterates aebitda guidance and lower holdco cost target for the year advance auto part report second quarter result and reaffirms full year sale operating margin and free cash flow guidance calibercos sale drop percent nd century q earnings snapshot aquestive therapeutic announces pricing of million underwritten offering of common stock aquestive therapeutic announces pricing of million underwritten offering of common stock deere report third quarter net income of billion deere report third quarter net income of billion bcg report earnings ap technology summarybrief at am edt ap technology summarybrief at am edt today heloc home equity loan rate august bybit eu tap xion for inaugural launchpool in the eu opening regulated access for m user battalion oil corporation announces second quarter financial and operating result ford next model t moment started in california battalion oil corporation announces second quarter financial and operating result pro kapital council approved consolidated interim report for ii quarter and month of unaudited your guide to the best meme coin for exponential return this year pro kapital council approved consolidated interim report for ii quarter and month of unaudited cd rate today august take home up to u stock future lower a investor await inflation job data tool that have transformed business practice for entrepreneur fennec pharmaceutical report second quarter financial result and provides business update fennec pharmaceutical report second quarter financial result and provides business update kari lake defends voa cut in court after warning from capitol hill hta establishes advisory board want public input for planning highyield saving account rate today august rate are steady money market interest rate today august earn up to down is the worst over for lululemon stock the answer may surprise you lulu announces new credit agreement with white oak commercial finance llc mortgage rate today august rate hold steady spotting a hidden ice flight gold rush hit trumpera washington from price to the oval office xbocom exchange launch native xbo token and staking program ke holding inc to report second quarter financial result on august eastern time aquestive therapeutic announces m strategic funding agreement with rtw to support the potential launch of anaphylmtm epinephrine sublingual film this might be cadillacs craziest concept car ever motorcom big bank show there not just one recipe for success water recycle and reuse market worth billion by exclusive report by marketsandmarketstm ai modelasaservice is rising whats new in ai landscape radware and leading latvian isp tet sign managed security service provider agreement family target toprated school district this moving seasonbut at a price way roadside help harbor insurance see boost in revenue and customer satisfaction true random number generator market to hit usd billion by at a cagr of sn insider some state revenue is down but not the lottery vena receives sixth consecutive trustradius tech care award inception growth acquisition limited announces additional contribution to trust account to extend business combination period zelluna asa invitation to second quarter result webcast presentation aquestive therapeutic announces m strategic funding agreement with rtw to support the potential launch of anaphylmtm epinephrine sublingual film xunlei announces unaudited financial result for the second quarter ended june waterly secures m to power the future of water asset data sample management and more funding from burnt island venture and emerald will multiply the waterly platform reach ke holding inc to report second quarter financial result on august eastern time nd century group report second quarter financial result radware and leading latvian isp tet sign managed security service provider agreement how to enable p console sharing and offline play lulu announces new credit agreement with white oak commercial finance llc tungray technology appoints henry guo a chief financial officer over blizzard worker in irvine join union a gamingindustry labor movement expands xunlei announces unaudited financial result for the second quarter ended june the olympics give sponsor venue naming right for first time letter the city should consider alternative to flawed link plan better buy nike stock v lululemon stock near week low should you buy uipath stock beatendown undervalued growth stock down to buy hand over fist right now in august success of twin ownership deal will come down to how the money is spent the topperforming bank with more than b of asset crewscope raise over m to boost productivity for construction and industrial field crew disney stock buy or sell tyton partner release driving toward a degree career readiness and financial pressure at the forefront of student support best stock to buy novo nordisk stock v unitedhealth stock thing you need to know if you buy medtronic today ambow education sign white house pledge to expand access to aisupported education for america youth world share are mixed ahead of meeting between trump and putin ap news here are today mortgage refinance rate august rate decrease weak production data pours cold water on eurozones hope for industrial recovery charles schwab investment management inc lower stock holding in flowserve corporation nysefls rising rollouts of continuation vehicle signal maturity in private equity fiber reinforced polymer composite market size to surpass usd billion by driven by rising demand in construction automotive and aerospace sn insider china etown claim applied material poached staff misused proprietary chip tech openeden appoints bank of new york police in southern california find worth of labubus stolen from warehouse tech giant spotlight rising opportunity in western new york swalwells shameless flipflop from roleplaying carjacking with wife to shrugging off dc crime surge wisconsin request fema assistance after last weekend storm flooding why would a jew vote for mamdani rabbit in colorado are sprouting horn here why douthat maha like maga populism constrained by complicated marriage to big biz letter republican majority in congress ha sold out letter dl is right place for cruise ship terminal keene man died of multiple gunshot wound after traffic stop standoff trump urging for epstein distraction will lead to shocker at putin summit michael wolff letter christian nationalism richly hypocritical editorial grab hawaii feral cat bane by the scruff new york allowed pot shop to open too close to school now they might have to move alaska to take center stage at trumpputin summit alaska to take center stage at trumpputin summit sherrod brown give democrat jolt of enthusiasm in ohio sherrod brown give democrat jolt of enthusiasm in ohio doe unveils fresh billion funding to boost u critical mineral alaska to take center stage at trumpputin summit sherrod brown give democrat jolt of enthusiasm in ohio couple convicted for harboring illegal alien at texas bakery sheldon h jacobson made in america is alive well and misunderstood spotting a hidden ice flight editorial opposing mayor brandon johnson taxincrease idea is not a criminal act how trump and putin relationship ha evolved since they first met eight year ago cnn politics how trump and putin relationship ha evolved since they first met eight year ago willie wilson even pharaoh knew his limit when it came to tax editorial organ donor should be dead first thomas c bowen why ranked choice is the best cure for gerrymandering california democrat prepare redistricting effort to counter texas gop california democrat prepare redistricting effort to counter texas gop great american medium announces a belle christmas a new original movie starring ash tsai marshall williams and julia reilly family target toprated school district this moving seasonbut at a price chinese climber dy on k after reaching summit letter trump power grab threatens constitutional order letter the city should consider alternative to flawed link plan ice deportation airline avelo relies on bluestate subsidy will dem governor do anything about it trump effect dc police break from sanctuary city policy will cooperate with ice letter mob mentality at it worst ruin a meeting ichthyology is the branch of zoology that involves the study of which animal letter raucous rude and a cause for embarrasment foreign ngo say new israeli rule keep them from delivering gaza aid letter childish attendee ruin an important event father of israeli hostage delivers ringing message destroying hamas must be the main objective reader speak maybe former uconn woman basketball player can buy the connecticut sun kluth the u will regret throwing india under the bus a failed experiment in democracy letter democrat is sickened by town hall behavior israel announces west bank settlement that right group say could imperil palestinian state letter congressman show a lack of accountability zelenskyy meet with uk starmer a europe brace for trumpputin summit letter civility is important but rage is understandable israel announces a settlement that critic say will effectively sever the west bank in two sometimes you just cant put a price on a penny north state voice divided harrisburg house dems reject senate gop transit budget bill newsoms california redistricting push set up a standoff with republicanled opposition california republican are forming plan to oppose newsoms redistricting push cnn politics commentary welcome to american politics without norm commentary bad bunny is loud but puerto rican voter have spoken on statehood letter ugly hostility win out over open conversation ct electric rate to drop in september here why letter civility need to start at the top aid group call on israel to end weaponization of aid in gaza in gaza journalism is a death sentence reader speak trump need only to find answer to one question fit rover popular unconventional local health project awarded by doncaster council n korea accuses south of lying to the public opinion death tax and the nightmare that follows in ct letter town hall just a gigantic temper tantrum arkansas death row inmate sue to stop nitrogen gas execution asks to be next laura loomers attack on rfk jr the latest maga feud explained foton philippine launched a full commercial ev lineup adventure ready how the g tripros bumper cam take offroading to the next level she womens expo to offer health information saturday cisco ai infrastructure order top b why cryptocurrency okb ha more than doubled this week lyme disease is spiking this biotech nears a treatment and a buy point clean truck partnership take another blow with ftc deal in wild week for the beleaguered pact why share of coreweave are plunging this week unlocking the benefit of affordable insurance ace the test how to boost credit score tron flip cardano in market cap but this subm coin could outrun both dogecoin news today dogecoin eye breakout a whale accumulate m doge and golden cross form cold wallet presale hit m bittensor jump dogecoin volume soar best crypto to buy in citgo swing to m profit a bidding war intensifies for parent company israeli and palestinian bridge builder coming together to end the war aramco sign billion jafurah midstream deal with international consortium led by global infrastructure partner ethereum is outpacing cardano price but both are tasting crypto dust when compared to the gain from this presale ace the blue live in this mississippi delta town chicago fact of the day these analyst revise their forecast on coherent rosen leading investor counsel encourages cto realty growth inc investor to secure counsel before important deadline in security class action cto ctopa supreme court allows enforcement of mississippi social medium age verification law texture and franklinwh partner to deliver full control of home energy system ethereum solana lead crypto social medium discussion what about bitcoin doj sec charge two men in million water vending machine ponzi scheme cnbc recycle your electronics in beaufort county aug a car accident in smalltown tennessee lead to u charge against a major mexican drug operation eagle brown come together to gloriously throw down morning beer mississippi may require age verification parental consent for social medium supreme court say joby v archer two air taxi rival race toward but who really ha liftoff can ai cure cancer expert say the answer is complicated romania push nato to step up black sea mine task force eli lilly to raise uk price of mounjaro for outofpocket patient the wall street journal get ultimate allinone digital protection for off from mcafee advent vestment symbolism and tradition in liturgy these analyst increase their forecast on performance food group following strong q earnings how citi and jp morgan blockchain move influence payment philippine first floating solar farm set a national blueprint for clean energy best laptop for accounting in panorama insurance associate endorses california insurance market reform act call on industry to unite behind critical ballot initiative cleanspace continues rapid growth strengthening it concepttocommercialization model supreme court allows enforcement of mississippi social medium age verification law supreme court allows enforcement of mississippi social medium age verification law u dollar bullish structure contrast with softness in precious metal will dogecoin reach in august here the latest doge price forecast brinker international analyst boost their forecast following upbeat q result sonoma pharmaceutical valuation premium hinge on it revenue mix why pagseguro stock plummeted today money is rotating away from big tech stock it a good sign barrons confused trump forgets huge detail of big beautiful bill in cringe oval office moment prsany announces individual award recipient and under honoree ck hutchison profit plunge on oneoff loss from merger canaan report record q profit growth how to navigate the biggest pitfall of a growing business euna solution named government technology management team of the year in stevie award for technology excellence provectus q earnings snapshot auto insurance hike explained how to save without sacrificing coverage fleet electrification is getting easier by the day cisco to rally around here are top analyst forecast for thursday check out what whale are doing with ktos unpacking the latest option trading trend in sweetgreen spotlight on ionq analyzing the surge in option activity looking into domino pizza recent short interest what doe the market think about blackrock a look into mt bank inc price over earnings how is the market feeling about crown holding ozak ai potential may surpass bitcoins high financial trap keeping you stuck frustrated and how to escape past is prologue rising container volume portend falling rate lyno ai early bird presale exceeds k token sold a price increase approach pi coin news today pi coin dip to a investor confidence wane amid bitcoin surge blockdags m presale top trending crypto list despite cosmos positive outlook and k bnb prediction toll brother apartment living and harris realty company llc announce the opening of piper a new luxury apartment community in norwalk connecticut toll brother apartment living and harris realty company llc announce the opening of piper a new luxury apartment community in norwalk connecticut judge dismisses count against u rep cuellar of texas move bribery trial to next year average rate on a year mortgage drop to lowest level since october werner recall ladder due to faulty locking mechanism lm funding america swing to q profit taylor swift economic pull make orange the new green for big brand taylor swift economic pull make orange the new green for big brand connecticut credit union data breach affect verdek rank no on the inc list of america fastestgrowing private company why terawulf stock is skyrocketing today usa reject global carbon tax on global shipping small pacific island are hypocrite for their role in icj climate advisory say friend of science society walmart give employee extra saving on grocery with expanded discount dogecoin price outlook doge might hit however new gaming platform rblk offer bigger longterm upside ease protocol roll out government and enterprisegrade blockchain tool for realworld application fda alert over cookware that may leak lead into food product list todaycom kroger settle with c wholesale after failed billion albertsons merger oscar health face analyst question on path to profitability survey show parent will pay more for packed school lunch this year onfolio holding inc announces second quarter financial result and provides corporate update onfolio holding inc announces second quarter financial result and provides corporate update forget solana sol here are cheaper token to buy for the next gain in analyst predict a x surge for pepe coin but investor are loading up on the new xrp while they still can ibd live qa stock list for thursday aug baltimore face an energy crisis reader commentary best ultrawide camera smartphones to buy in toll brother announces opening of new model home at carrara estate in eagle idaho laura loomers attack on rfk jr the latest maga feud explained supreme court decline to block state law limiting kid use of social medium for now smiling maga man tear down democrat illegal trump hitler sign on highway overpass in iowa watch mayor adam float state bill to involuntarily hospitalize individual for public substance use amid reelection push the ad council and sugar launch ad council entertainment bipartisan solution for afghan ally spark hope israeli and palestinian bridge builder coming together to end the war the blue live in this mississippi delta town rosebud deputy and mhp arrest suspect accused of stealing truck after dodiks historic removal bosnia sovereignty crisis still smolder woman who dumped their manchild partner what wa the final straw live now california governor state l</t>
+          <t>boring stock offering an over annual dividend yield there a small problem with trump export deal with nvidia and amd the constitution say it illegal fortune trump chief intervened to save rfk jr top vaccine aide politico revisiting carrie bradshaws apartment in sex and the city and and just like that fed face high bar for big cut despite white house pressure the new york time fed face high bar for big cut despite white house pressure bitcoin price soar to a etf inflow surge how trump get what he want from company nbc news wanf in atlanta release new schedule for life after cbs home for sale in manhattan and brooklyn the live music business is booming now rap is getting a piece too there money to be made in maha food company want in cetera investment adviser sell share of camden property trust nysecpt the cost to rebuild a home after a natural disaster is rising pnc financial service group inc acquires share of on holding ag nyseonon pnc financial service group inc raise position in five below inc nasdaqfive pnc financial service group inc purchase share of the madison square garden company nysemsgs tko group holding inc nysetko share acquired by pnc financial service group inc the latest chatgpt is supposed to be phd level smart it cant even label a map crypto presale alert blockchainfx bfx set for explosive growth can it beat bitcoin hyper blockdag big tech ai boom is reordering the u power grid the new york time crisis intervention effort yield impressive result trump is tightening the screw on corporate america and ceo are staying mum titanbay appoints exubs exec a head of switzerland is xrp a buy while it below best spy tv show to watch now on peacock in vipshop report unaudited second quarter financial result instacart is partying like it with third eye blind frosted tip and ring pop new report cleaner manufacturing could save life and prevent million of asthma attack titanbay appoints exubs exec a head of switzerland trump is tightening the screw on corporate america and ceo are staying mum npr weibo announces second quarter unaudited financial result ai development is accelerating vanguard etf to buy right now inside thailand frantic effort to close tariff loophole to the u china offer interest subsidy for loan amid sluggish economy pinterest share just sank time to buy the dip or run for the hill cava group nysecava price target cut to by analyst at morgan stanley nvidia corporation nasdaqnvda share purchased by richard c young co ltd kingsview wealth management llc purchase share of nvidia corporation nasdaqnvda cava group nysecava price target lowered to at citigroup tat technology tatt buy rating reaffirmed at lake street capital summit x llc purchase share of amazoncom inc nasdaqamzn nvidia corporation nasdaqnvda share sold by forum financial management lp repay nasdaqrpay receives neutral rating from ubs group snowflake nysesnow given new price target at ubs group nvidia corporation nasdaqnvda share sold by asset advisor investment management llc rivian automotive nasdaqrivn given new price target at morgan stanley fluence energy nasdaqflnc price target lowered to at royal bank of canada commerzbank aktiengesellschaft fi ha million stock holding in nvidia corporation nasdaqnvda meet the yield dividend stock that could soar in brachioplasty market to surpass usd billion by fueled by rising aesthetic awareness and technological advancement sn insider titanbay appoints paul essen bakery owner say they closed for a mental health break their employee say theyve been ghosted wkmg in orlando give news director autumn jones all the job vanguard group inc trim stock holding in blueprint medicine corporation nasdaqbpmc vanguard group inc ha million stock position in interdigital inc nasdaqidcc charles schwab investment management inc cut stock holding in bright horizon family solution inc nysebfam fluor corporation nyseflr share sold by vanguard group inc charles schwab investment management inc sell share of mattel inc nasdaqmat clearwater analytics holding inc nysecwan share acquired by vanguard group inc agco corporation nyseagco share sold by vanguard group inc vanguard group inc reduces position in ollies bargain outlet holding inc nasdaqolli vanguard group inc sell share of first american financial corporation nysefaf charles schwab investment management inc reduces holding in ally financial inc nyseally u bancorp de acquires share of graphic packaging holding company nysegpk vanguard group inc reduces position in lantheus holding inc nasdaqlnth charles schwab investment management inc boost position in dropbox inc nasdaqdbx vanguard group inc cut position in lincoln national corporation nyselnc vanguard group inc decrease position in itron inc nasdaqitri vanguard group inc trim stake in dropbox inc nasdaqdbx charles schwab investment management inc sell share of spotify technology nysespot chart industry inc nysegtls share purchased by charles schwab investment management inc nov inc nysenov share bought by vanguard group inc charles schwab investment management inc ha million stock position in spx technology inc nysespxc charles schwab investment management inc reduces position in talen energy corporation nasdaqtln curtisswright corporation nysecw position increased by charles schwab investment management inc vanguard group inc sell share of mattel inc nasdaqmat u bancorp de reduces holding in bce inc nysebce vanguard group inc lower stock holding in chart industry inc nysegtls atrium wealth solution inc ha stock position in ppg industry inc nyseppg analyst issue forecast for saputos q earnings tsesap atrium wealth solution inc buy share of vanguard international dividend appreciation etf nasdaqvigi vanguard group inc sell share of antero midstream corporation nyseam atrium wealth solution inc ha stake in southwest gas corporation nyseswx atrium wealth solution inc reduces position in sarepta therapeutic inc nasdaqsrpt vanguard group inc ha million holding in simpson manufacturing company inc nysessd vanguard group inc sell share of universal display corporation nasdaqoled vanguard group inc decrease stock holding in flowserve corporation nysefls share in spdr sp capital market etf nysearcakce bought by atrium wealth solution inc vanguard group inc sell share of credo technology group holding ltd nasdaqcrdo vanguard group inc acquires share of american airline group inc nasdaqaal atrium wealth solution inc invests in ugi corporation nyseugi atrium wealth solution inc decrease position in ingersoll rand inc nyseir home bancshares inc nysehomb share sold by atrium wealth solution inc vanguard group inc sell share of option care health inc nasdaqopch atrium wealth solution inc ha stock holding in rb global inc nyserba sl green realty corporation nyseslg share bought by vanguard group inc atrium wealth solution inc make new investment in crown holding inc nysecck notice regarding uaborkela financial statement for month period ended june nagarro release unaudited q result post yoy revenue growth in constant currency and increase in gross profit despite global macroeconomic challenge parent dont want cell phone ban at school we want smarter rule opinion mexico under pressure from trump sends cartel member to u the key to success at trumpputin alaska summit on ukraine low expectation opinion welcome to the menodivorce why woman arent sweating marriage in a sea of hot flash a tropical storm erin track west palm beach advises resident to stay alert prepared letter new challenge require a new congressman cctv foreign journalist open blind box at shuiting gate america must secure social security now republican pitch trump domestic policy agenda in iowa but some entrepreneur arent yet sold cnn politics the latest chatgpt is supposed to be phd level smart it cant even label a map wfp is leveraging it power in the mayoral race firstofitskind micropathway initiative now help community college build industryaligned training program my legacy is of broken men michael thomas on dream alcoholism and black fatherhood conquistador stolen yearold receipt return to mexico priscilla presley accused of hastening lisa mary death for financial gain memoir on a hill finding the best way to tell the story of america letter why now and why all the surprise eye on art frazier brings lowell to life in all gallery show rosner appointed ferc chair a trump move to reshape regulator u deploys force to take on latin american drug cartel in the southern caribbean today in history august fdr sign social security act now jimmy fallon is using taylor swift to suggest trump had sinister tie to epstein activist amariyanna copenys hometown crossword clue it not just dc republican seem happy to let trump do whatever he want opinion letter wondering if congressman still walk with jesus cincinnati beating suspect face year in prison after new charge from doj no peace without ukraine trumpputin alaska talk call for sober strategy oil city civic center to offer tour of national transit building thompson cosponsors bill to expand k career counseling idea opinion tom durkin come together debence receives grant for kid program grove city college ranked no for most religious student in u year ago aug lucas foley go to bat for bay state ag should too brokerage set cargojet inc tsecjt pt at c brokerage set penn entertainment inc nasdaqpenn target price at cbre group inc nysecbre receives consensus target price from analyst under armour nyseuaa price target lowered to at telsey advisory group john hood german settler helped shape nc rebellion today in historyaug failed gop candidate sentenced to year in connection with shooting spree at democrat official home stage mechanic and hanover in worcester make going out fun prokidney corp nasdaqprok receives average rating of hold from analyst spx technology inc nysespxc given average rating of buy by brokerage adapthealth corp nasdaqahco receives consensus target price from analyst contineum therapeutic inc nasdaqctnm receives consensus price target from brokerage on inc nyseontf receives consensus rating of hold from brokerage ap news summary at am edt douglas cohn and eleanor clift the shamed the shameless and the shirked editorial why is healey hesitating to call for tompkins resignation guest opinion erich menzel sculpture and art in the park event put loveland on the map ap news summary at am edt morning brief arrest since trump dc takeover trumpputin peace talk immigrant exodus social security is the cornerstone of retirement income fbi agent are again pulled from their day job to address a trump priority cnn politics cost of living in california still a discussion at county level propalestinian protester hold demonstration outside ivp reader sound off on turning against israel misusing troop and reckless bikers sbdc guide resident on starting legal homebased food business icf international nasdaqicfi price target raised to hang feng technology innovation co ltd fofo announces august th ipo alaska a source of russian imperial nostalgia powerful sister of north korean leader denies removal of frontline speaker cal thomas washington dc then and now emera tseema price target raised to c expensify nasdaqexfy cut to hold at wall street zen emera tseema price target raised to c rosenblatt security cut hut nasdaqhut price target to irs reportedly confirms stimulus check for eligible american rumor of august payout debunked plan late summer rollout american healthcare reit nyseahr price target raised to trump eas space regulation in boost for elon musk spacex jeff bezos blue origin and more pearson nysepso downgraded to hold rating by wall street zen first interstate bancsystem nasdaqfibk cut to sell at wall street zen morgan stanley cut primo brand nyseprmb price target to speaking out no longer interested in preventing pain and suffering north korea denies removing border loudspeaker ct real estate investment trust tsecrtun price target raised to c national bankshares cut boralex tseblx price target to c constellation software tsecsu price target raised to c share buyback program approved by plus lonplus board of director hong kong lashed with another torrential downpour redwire nyserdw price target lowered to at canaccord genuity group trisura group tsetsu price target raised to c gdi integrated facility service tsegdi downgraded by td security to hold leon furniture tselnf price target raised to c power co of canada tsepow price target raised to c at desjardins savaria tsesis price target raised to c saputo tsesap price target raised to c letter the right betrays every value it claim to hold youngkin order investigation into claim staff at virginia school arranged abortion without parental consent ap news summary at am edt flower food flo expected to announce earnings on friday kodiak gas service nysekgs to repurchase million in outstanding share trump nobel peace prize push gain steam president clinch backing from pakistan cambodia israel ahead of meeting with putin gop senator spill on the illegal measure he take to deal with dc crime fear softcat plc lonsct insider buy in stock jpmorgan global core real asset limited lonjara insider sell in stock fresnillo lonfres stock price expected to rise royal bank of canada analyst say asiamet resource lonars receives house stock rating from shore capital jpmorgan global core real asset limited lonjara insider sell in stock battalion oil post q revenue drop netease stock drop after chinese video game firm miss sale target aebi schmidt group building momentum after merging with the shyft group strong order backlog additional synergy upside and commitment to delever ask a real estate pro how can we stop complaining neighbor harassing behavior ask a real estate pro how can we stop complaining neighbor harassing behavior bessent see nvidia amd china agreement a a model for others nov declares regular quarterly dividend permanent magnet market worth billion by exclusive report by marketsandmarketstm clean energy tax credit market participant remain bullish the wall street journal rare earth rally after department of defense set a price floor aery technology report record q fy result cash flow positive m net income turnaround and strongest start to a fiscal year in company history envirogold global retains cantor fitzgerald a financial advisor p announces dual listing on nyse texas dividendpaying dow jones stock to buy in august u and australia support for nova estelle project realme pro review is it worth a buy shattuck lab report second quarter financial result and recent business highlight medium advisory air canada to hold medium availability with senior executive today aimia report second quarter result reiterates aebitda guidance and lower holdco cost target for the year advance auto part report second quarter result and reaffirms full year sale operating margin and free cash flow guidance calibercos sale drop percent nd century q earnings snapshot aquestive therapeutic announces pricing of million underwritten offering of common stock aquestive therapeutic announces pricing of million underwritten offering of common stock deere report third quarter net income of billion deere report third quarter net income of billion bcg report earnings ap technology summarybrief at am edt ap technology summarybrief at am edt today heloc home equity loan rate august bybit eu tap xion for inaugural launchpool in the eu opening regulated access for m user battalion oil corporation announces second quarter financial and operating result ford next model t moment started in california battalion oil corporation announces second quarter financial and operating result pro kapital council approved consolidated interim report for ii quarter and month of unaudited your guide to the best meme coin for exponential return this year pro kapital council approved consolidated interim report for ii quarter and month of unaudited cd rate today august take home up to u stock future lower a investor await inflation job data tool that have transformed business practice for entrepreneur fennec pharmaceutical report second quarter financial result and provides business update fennec pharmaceutical report second quarter financial result and provides business update kari lake defends voa cut in court after warning from capitol hill hta establishes advisory board want public input for planning highyield saving account rate today august rate are steady money market interest rate today august earn up to down is the worst over for lululemon stock the answer may surprise you lulu announces new credit agreement with white oak commercial finance llc mortgage rate today august rate hold steady spotting a hidden ice flight gold rush hit trumpera washington from price to the oval office xbocom exchange launch native xbo token and staking program ke holding inc to report second quarter financial result on august eastern time aquestive therapeutic announces m strategic funding agreement with rtw to support the potential launch of anaphylmtm epinephrine sublingual film this might be cadillacs craziest concept car ever motorcom big bank show there not just one recipe for success water recycle and reuse market worth billion by exclusive report by marketsandmarketstm ai modelasaservice is rising whats new in ai landscape radware and leading latvian isp tet sign managed security service provider agreement family target toprated school district this moving seasonbut at a price way roadside help harbor insurance see boost in revenue and customer satisfaction true random number generator market to hit usd billion by at a cagr of sn insider some state revenue is down but not the lottery vena receives sixth consecutive trustradius tech care award inception growth acquisition limited announces additional contribution to trust account to extend business combination period zelluna asa invitation to second quarter result webcast presentation aquestive therapeutic announces m strategic funding agreement with rtw to support the potential launch of anaphylmtm epinephrine sublingual film xunlei announces unaudited financial result for the second quarter ended june waterly secures m to power the future of water asset data sample management and more funding from burnt island venture and emerald will multiply the waterly platform reach ke holding inc to report second quarter financial result on august eastern time nd century group report second quarter financial result radware and leading latvian isp tet sign managed security service provider agreement how to enable p console sharing and offline play lulu announces new credit agreement with white oak commercial finance llc tungray technology appoints henry guo a chief financial officer over blizzard worker in irvine join union a gamingindustry labor movement expands xunlei announces unaudited financial result for the second quarter ended june the olympics give sponsor venue naming right for first time letter the city should consider alternative to flawed link plan better buy nike stock v lululemon stock near week low should you buy uipath stock beatendown undervalued growth stock down to buy hand over fist right now in august success of twin ownership deal will come down to how the money is spent the topperforming bank with more than b of asset crewscope raise over m to boost productivity for construction and industrial field crew disney stock buy or sell tyton partner release driving toward a degree career readiness and financial pressure at the forefront of student support best stock to buy novo nordisk stock v unitedhealth stock thing you need to know if you buy medtronic today ambow education sign white house pledge to expand access to aisupported education for america youth world share are mixed ahead of meeting between trump and putin ap news here are today mortgage refinance rate august rate decrease weak production data pours cold water on eurozones hope for industrial recovery charles schwab investment management inc lower stock holding in flowserve corporation nysefls rising rollouts of continuation vehicle signal maturity in private equity fiber reinforced polymer composite market size to surpass usd billion by driven by rising demand in construction automotive and aerospace sn insider china etown claim applied material poached staff misused proprietary chip tech openeden appoints bank of new york police in southern california find worth of labubus stolen from warehouse tech giant spotlight rising opportunity in western new york swalwells shameless flipflop from roleplaying carjacking with wife to shrugging off dc crime surge wisconsin request fema assistance after last weekend storm flooding why would a jew vote for mamdani rabbit in colorado are sprouting horn here why douthat maha like maga populism constrained by complicated marriage to big biz letter republican majority in congress ha sold out letter dl is right place for cruise ship terminal keene man died of multiple gunshot wound after traffic stop standoff trump urging for epstein distraction will lead to shocker at putin summit michael wolff letter christian nationalism richly hypocritical editorial grab hawaii feral cat bane by the scruff new york allowed pot shop to open too close to school now they might have to move alaska to take center stage at trumpputin summit alaska to take center stage at trumpputin summit sherrod brown give democrat jolt of enthusiasm in ohio sherrod brown give democrat jolt of enthusiasm in ohio doe unveils fresh billion funding to boost u critical mineral alaska to take center stage at trumpputin summit sherrod brown give democrat jolt of enthusiasm in ohio couple convicted for harboring illegal alien at texas bakery sheldon h jacobson made in america is alive well and misunderstood spotting a hidden ice flight editorial opposing mayor brandon johnson taxincrease idea is not a criminal act how trump and putin relationship ha evolved since they first met eight year ago cnn politics how trump and putin relationship ha evolved since they first met eight year ago willie wilson even pharaoh knew his limit when it came to tax editorial organ donor should be dead first thomas c bowen why ranked choice is the best cure for gerrymandering california democrat prepare redistricting effort to counter texas gop california democrat prepare redistricting effort to counter texas gop great american medium announces a belle christmas a new original movie starring ash tsai marshall williams and julia reilly family target toprated school district this moving seasonbut at a price chinese climber dy on k after reaching summit letter trump power grab threatens constitutional order letter the city should consider alternative to flawed link plan ice deportation airline avelo relies on bluestate subsidy will dem governor do anything about it trump effect dc police break from sanctuary city policy will cooperate with ice letter mob mentality at it worst ruin a meeting ichthyology is the branch of zoology that involves the study of which animal letter raucous rude and a cause for embarrasment foreign ngo say new israeli rule keep them from delivering gaza aid letter childish attendee ruin an important event father of israeli hostage delivers ringing message destroying hamas must be the main objective reader speak maybe former uconn woman basketball player can buy the connecticut sun kluth the u will regret throwing india under the bus a failed experiment in democracy letter democrat is sickened by town hall behavior israel announces west bank settlement that right group say could imperil palestinian state letter congressman show a lack of accountability zelenskyy meet with uk starmer a europe brace for trumpputin summit letter civility is important but rage is understandable israel announces a settlement that critic say will effectively sever the west bank in two sometimes you just cant put a price on a penny north state voice divided harrisburg house dems reject senate gop transit budget bill newsoms california redistricting push set up a standoff with republicanled opposition california republican are forming plan to oppose newsoms redistricting push cnn politics commentary welcome to american politics without norm commentary bad bunny is loud but puerto rican voter have spoken on statehood letter ugly hostility win out over open conversation ct electric rate to drop in september here why letter civility need to start at the top aid group call on israel to end weaponization of aid in gaza in gaza journalism is a death sentence reader speak trump need only to find answer to one question fit rover popular unconventional local health project awarded by doncaster council n korea accuses south of lying to the public opinion death tax and the nightmare that follows in ct letter town hall just a gigantic temper tantrum arkansas death row inmate sue to stop nitrogen gas execution asks to be next laura loomers attack on rfk jr the latest maga feud explained foton philippine launched a full commercial ev lineup adventure ready how the g tripros bumper cam take offroading to the next level she woman expo to offer health information saturday cisco ai infrastructure order top b why cryptocurrency okb ha more than doubled this week lyme disease is spiking this biotech nears a treatment and a buy point clean truck partnership take another blow with ftc deal in wild week for the beleaguered pact why share of coreweave are plunging this week unlocking the benefit of affordable insurance ace the test how to boost credit score tron flip cardano in market cap but this subm coin could outrun both dogecoin news today dogecoin eye breakout a whale accumulate m doge and golden cross form cold wallet presale hit m bittensor jump dogecoin volume soar best crypto to buy in citgo swing to m profit a bidding war intensifies for parent company israeli and palestinian bridge builder coming together to end the war aramco sign billion jafurah midstream deal with international consortium led by global infrastructure partner ethereum is outpacing cardano price but both are tasting crypto dust when compared to the gain from this presale ace the blue live in this mississippi delta town chicago fact of the day these analyst revise their forecast on coherent rosen leading investor counsel encourages cto realty growth inc investor to secure counsel before important deadline in security class action cto ctopa supreme court allows enforcement of mississippi social medium age verification law texture and franklinwh partner to deliver full control of home energy system ethereum solana lead crypto social medium discussion what about bitcoin doj sec charge two men in million water vending machine ponzi scheme cnbc recycle your electronics in beaufort county aug a car accident in smalltown tennessee lead to u charge against a major mexican drug operation eagle brown come together to gloriously throw down morning beer mississippi may require age verification parental consent for social medium supreme court say joby v archer two air taxi rival race toward but who really ha liftoff can ai cure cancer expert say the answer is complicated romania push nato to step up black sea mine task force eli lilly to raise uk price of mounjaro for outofpocket patient the wall street journal get ultimate allinone digital protection for off from mcafee advent vestment symbolism and tradition in liturgy these analyst increase their forecast on performance food group following strong q earnings how citi and jp morgan blockchain move influence payment philippine first floating solar farm set a national blueprint for clean energy best laptop for accounting in panorama insurance associate endorses california insurance market reform act call on industry to unite behind critical ballot initiative cleanspace continues rapid growth strengthening it concepttocommercialization model supreme court allows enforcement of mississippi social medium age verification law supreme court allows enforcement of mississippi social medium age verification law u dollar bullish structure contrast with softness in precious metal will dogecoin reach in august here the latest doge price forecast brinker international analyst boost their forecast following upbeat q result sonoma pharmaceutical valuation premium hinge on it revenue mix why pagseguro stock plummeted today money is rotating away from big tech stock it a good sign barrons confused trump forgets huge detail of big beautiful bill in cringe oval office moment prsany announces individual award recipient and under honoree ck hutchison profit plunge on oneoff loss from merger canaan report record q profit growth how to navigate the biggest pitfall of a growing business euna solution named government technology management team of the year in stevie award for technology excellence provectus q earnings snapshot auto insurance hike explained how to save without sacrificing coverage fleet electrification is getting easier by the day cisco to rally around here are top analyst forecast for thursday check out what whale are doing with ktos unpacking the latest option trading trend in sweetgreen spotlight on ionq analyzing the surge in option activity looking into domino pizza recent short interest what doe the market think about blackrock a look into mt bank inc price over earnings how is the market feeling about crown holding ozak ai potential may surpass bitcoins high financial trap keeping you stuck frustrated and how to escape past is prologue rising container volume portend falling rate lyno ai early bird presale exceeds k token sold a price increase approach pi coin news today pi coin dip to a investor confidence wane amid bitcoin surge blockdags m presale top trending crypto list despite cosmos positive outlook and k bnb prediction toll brother apartment living and harris realty company llc announce the opening of piper a new luxury apartment community in norwalk connecticut toll brother apartment living and harris realty company llc announce the opening of piper a new luxury apartment community in norwalk connecticut judge dismisses count against u rep cuellar of texas move bribery trial to next year average rate on a year mortgage drop to lowest level since october werner recall ladder due to faulty locking mechanism lm funding america swing to q profit taylor swift economic pull make orange the new green for big brand taylor swift economic pull make orange the new green for big brand connecticut credit union data breach affect verdek rank no on the inc list of america fastestgrowing private company why terawulf stock is skyrocketing today usa reject global carbon tax on global shipping small pacific island are hypocrite for their role in icj climate advisory say friend of science society walmart give employee extra saving on grocery with expanded discount dogecoin price outlook doge might hit however new gaming platform rblk offer bigger longterm upside ease protocol roll out government and enterprisegrade blockchain tool for realworld application fda alert over cookware that may leak lead into food product list todaycom kroger settle with c wholesale after failed billion albertsons merger oscar health face analyst question on path to profitability survey show parent will pay more for packed school lunch this year onfolio holding inc announces second quarter financial result and provides corporate update onfolio holding inc announces second quarter financial result and provides corporate update forget solana sol here are cheaper token to buy for the next gain in analyst predict a x surge for pepe coin but investor are loading up on the new xrp while they still can ibd live qa stock list for thursday aug baltimore face an energy crisis reader commentary best ultrawide camera smartphones to buy in toll brother announces opening of new model home at carrara estate in eagle idaho laura loomers attack on rfk jr the latest maga feud explained supreme court decline to block state law limiting kid use of social medium for now smiling maga man tear down democrat illegal trump hitler sign on highway overpass in iowa watch mayor adam float state bill to involuntarily hospitalize individual for public substance use amid reelection push the ad council and sugar launch ad council entertainment bipartisan solution for afghan ally spark hope israeli and palestinian bridge builder coming together to end the war the blue live in this mississippi delta town rosebud deputy and mhp arrest suspect accused of stealing truck after dodiks historic removal bosnia sovereignty crisis still smolder woman who dumped their manchild partner what wa the final straw live now california governor state le</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>poriferous llc achieves coveted eu mdr regulatory certification for porous polyethylene implant warehouse data reveals how shipper managed inventory through tariff nvidia earnings face high bar on datacenter demand china deal newsmax to pay million to settle dominion suit over election fraud claim bmws next big suv is gunning for the top dog but will it go electric jules witcover political reporter and columnist dy at samsung overtakes apple u smartphone market update hint at major shift brent wti edge higher a zelensky arrives in washington for talk with trump top trending coin this week oz presale token gain early momentum best altcoins to buy for september remittix top list over ada pepe and bonk cold wallet offer referral bonus bonk burn t supply ripple eye crypto project set to explode top crypto executive seen accumulating million of token of new meme coin challenging shiba inu shib in walmart is selling a queen mattress topper for only thats soft and cool to the touch best electronic signature apps in judge denies bail to north andover offduty officer shot in home defense file another appeal whale bet big on this new payment token to replace xrp and stellar by carvanas breakout fuel interest in consumer ecommerce etf why are colorado rabbit growing tentacle and horn maluma sign with wme in all area the sky is the limit dow jones today stock tick lower a major index hover near record high after two consecutive week of gain investopedia fake labubu doll pose threat to kid safety watchdog say cbs news court of federal claim side with small business in landmark taa v baa protest employer guidance for new tax deduction for tip and overtime pay terra balcanica intersects gold mineralization over m and start drill program at brezani target in bosnia ap business summarybrief at pm edt conservative network newsmax agrees to pay m in defamation case over bogus election claim invesco qqq qqq share sold by lee financial co bank stock to keep an eye on august th terawulf stock jump more than a google boost stake in data center operator top bse gainer to watch in uncy investor have opportunity to lead unicycive therapeutic inc security fraud lawsuit with the schall law firm cornerstone select advisor llc reduces stock position in pfizer inc pfe southeast toyota finance ranked highest in overall dealer satisfaction by jd power forget ai robotic process automation is healthcare hottest technology warehouse teamster at unfi win lucrative first contract promising retail stock to follow now august th alphabet inc goog share sold by wellington management group llp promising lithium stock to keep an eye on august th insurance stock to watch today august th hydrogen stock to consider august th pwc kunai acquisition to bolster tech enablement for bank cfo the bull case for nvidia just got stronger according to these analyst this curved samsung screen is at one of it lowest price today soho house to be taken private in billion deal the new york time expect fiery outcome from fed jackson hole conference this week financial advisor network inc take position in cocacola company the ko what analyst rating have to say about the campbell mesa laboratory executes previouslyannounced strategic financing plan ibm option trading a deep dive into market sentiment forecasting the future analyst projection for cloudflare a closer look at walmarts option market dynamic flex meal deal return for faculty staff and graduate and professional student paypal holdingss option frenzy what you need to know a glimpse into the expert outlook on jm smucker through analyst assessing microsoft insight from financial analyst this ethereum trader turned into million in month the analyst verdict fedex in the eye of expert ai take apple edge foxconns pivot could spark etf shift where prudential financial stand with analyst mesa laboratory executes previouslyannounced strategic financing plan wired roundup why gpt flopped wired is the market bullish or bearish on royal gold looking into willis tower watson recent short interest a look into pge inc price over earnings how is the market feeling about lumentum holding ozempic creator novo nordisk will sell weight loss drug for cheaper through this new partnership novo nordisk offer ozempic at per month to eligible u cashpaying customer reuters texas may have to shut down data center to protect it energy grid can blockdag reach analyst review of the m presale in dogecoin news today dogecoin price decline but technical indicator suggest potential rebound applied digitals stock apld jump on plan for billion ai campus tipranks worker are job hugging in a stagnant labor market but growing resentment mean they could bail a soon a the next great resignation come yahoocom texas attorney general accuses meta characterai of misleading kid with mental health claim techcrunch worker are job hugging in a stagnant labor market but growing resentment mean they could bail a soon a the next great resignation come fortune conservative network newsmax agrees to pay m in defamation case over bogus election claim skechers named title sponsor of world champion cup shriners childrens announced a official charity partner feather sound country club in clearwater florida to host tournament whats going on with propanc share monday mastercard and worldpay team to streamline uae money movement mcdonalds corporation mcd share sold by community bank trust waco texas granite harbor advisor inc boost holding in mcdonalds corporation mcd walmart ha everything you need to head back to school from backpack to laptop madd join force with law enforcement to prevent impaired driving ahead of labor day with saturation saturday initiative this weekend ibd live qa stock list for monday aug spotlight on fed what powell bowman and waller will say about rate dogecoin rally spark buzz but trader say this sub coin ha more upside fairscale capital llc purchase share of crowdstrike crwd lee financial co sell share of danaher corporation dhr berger montague pc investigates security claim against kindercare learning company inc nyse klc amazon is selling an bluetooth speaker for and it perfect for any setting inventhelp inventor develops new training aid for basketball player chk top data science recruiter in find ai analytics and ml expert gsg advisor llc purchase share of invesco qqq qqq gsg advisor llc ha stock holding in mastercard incorporated ma weekly bankruptcy alert august for the week ending august jackson hole loom a powell speech test september ratecut hope newsmax to pay million to settle dominion defamation lawsuit intel stock drop on report of equity stake via the chip act barrons liquid edge ai platform leap expands support to laptop with bestinclass performance on amd ryzentm and ryzen aitm processor ap business summarybrief at pm edt ap business summarybrief at pm edt texas democrat are back what now froma harrop are parent who dont vaccinate their child guilty of abuse handwritten proof of holocaust theft should compel congress to act ap news summary at pm edt ap news summary at pm edt state and dc sue doj to stop immigration requirement on victim fund trump zelenskyy meeting not end of the road for u support in securing a peace deal editorial roundup united state eric adam roll out nypd expansion say trump dc crackdown not a factor ap trending summarybrief at pm edt texas lawmaker in illinois heading back home following twoweek walkout over remap fight nfl team refuse to back down after facing backlash for hiring male cheerleader stephen miller say trump dc crackdown will also target graffiti ap news summary at pm edt conservative network newsmax agrees to pay m in defamation case over bogus election claim mark hamill say his wife clever thought stopped him from fleeing u after trump won trump zelensky put on the smile at oval office vancouver mayor warns delay on i bridge replacement cost m per day trump zelensky put on the smile at oval office hamas accepts an arab ceasefire proposal on gaza a palestinian death toll pass texas redistricting fight shift a democrat return to austin with a new strategy mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown on putin advice trump launch assault on mailin ballot and voting machine eo seek to expand access to alternative asset investment in retirement plan doj demand sensitive illinois voter registration data mike mcgrew an alternative mindset for patriotic independent commentary ha brian stelter doesnt get that he only making msnbcs rebranding even funnier in his excited thread former attorney general william barr say he didnt see trump implicated in epstein file former attorney general william barr say he didnt see trump implicated in epstein file gavin newsom left fox news speechless with his unexpectedly hilarious woke comeback these state leader might be the last line of defense against trump abuse of power subsidence isnt just an environmental crisis and it can be slowed the latest zelenskyy signal openness to threeway meeting with trump and putin doj wont appeal judge order on concealed carry ban in post office the latest zelenskyy signal openness to threeway meeting with trump and putin letter political treachery versus personal charity what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work bnpl provider ask for extension to nydfs request for information deadline wyoming teen educate youth about human trafficking on social medium congress must correct an injustice facing combatinjured veteran how blessing and disaster shape alabama why is the c galaxy such an iconic aircraft texas attorney general accuses meta characterai of misleading kid with mental health claim texas ag accuses meta characterai of misleading kid with mental health claim european leader join trump zelenskyy at white house conservative network newsmax agrees to pay m in defamation case over bogus election claim what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work twoweek standoff end quorum reached in texas house mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown letter trumpputin photo op accomplished nothing judge weighs detainee legal right at alligator alcatraz in florida everglades judge weighs detainee legal right at alligator alcatraz in florida everglades roblox is locking down sexual content and access to adult location after lawsuit trump say the u would back european security guarantee for ukraine to help end the war with russia good in a crisis dr nirav shah could be a promising candidate for anything steve collins wear a suit bro zelenskyy greeted by banner begging him to dress for the occassion did he hulk hogan couldnt stand gavin newsom exwife say about govs online trolling rightwing reporter brian glenn praise zelenskys attire after shaming him in february texas democrat return ending twoweek walkout over redistricting trump say hell talk to putin after meeting with zelenskyy and european leader at the white house reporter brian glenn brag about dc being safe after walking street with girlfriend marjorie taylor greene zelenskyy trump express hope for trilateral talk with putin to bring end to russiaukraine war oval office meeting again put rocky tense trumpzelenskyy relationship to the test armstrong williams how george washington would end russia war on ukraine staff commentary la habra man charged in fatal whittier shooting of driver texas democrat head home after week in illinois mpo holding first public planning session tuesday at mountain line photo show aftermath of a deadly russian attack in ukraine and the funeral of a fallen soldier now thats a selfown eric swalwell grocery shopping go viral for all the wrong hilarious reason texas democrat return to capitol for republican u house map overhaul a california counter texas democrat return to capitol for republican u house map overhaul a california counter letter time for democrat to play to win volodymyr zelensky wear suit this time for white house meeting with trump tarrant county commissioner again propose cutting voting site ahead of an election this is exactly what technology should be doing man shot injured in parking lot of huntington beach store letter no place for threat violence in politics trump aim to set putinzelenskiy meeting after monday summit obbba creates a cohesive framework for u hydrogen growth top trump lackey demand dc resident kiss the ground for occupation republican look to make a uturn on electric vehicle for the postal service republican look to make a uturn on electric vehicle for the postal service</t>
+          <t>poriferous llc achieves coveted eu mdr regulatory certification for porous polyethylene implant warehouse data reveals how shipper managed inventory through tariff nvidia earnings face high bar on datacenter demand china deal newsmax to pay million to settle dominion suit over election fraud claim bmws next big suv is gunning for the top dog but will it go electric jules witcover political reporter and columnist dy at samsung overtakes apple u smartphone market update hint at major shift brent wti edge higher a zelensky arrives in washington for talk with trump top trending coin this week oz presale token gain early momentum best altcoins to buy for september remittix top list over ada pepe and bonk cold wallet offer referral bonus bonk burn t supply ripple eye crypto project set to explode top crypto executive seen accumulating million of token of new meme coin challenging shiba inu shib in walmart is selling a queen mattress topper for only thats soft and cool to the touch best electronic signature apps in judge denies bail to north andover offduty officer shot in home defense file another appeal whale bet big on this new payment token to replace xrp and stellar by carvanas breakout fuel interest in consumer ecommerce etf why are colorado rabbit growing tentacle and horn maluma sign with wme in all area the sky is the limit dow jones today stock tick lower a major index hover near record high after two consecutive week of gain investopedia fake labubu doll pose threat to kid safety watchdog say cbs news court of federal claim side with small business in landmark taa v baa protest employer guidance for new tax deduction for tip and overtime pay terra balcanica intersects gold mineralization over m and start drill program at brezani target in bosnia ap business summarybrief at pm edt conservative network newsmax agrees to pay m in defamation case over bogus election claim invesco qqq qqq share sold by lee financial co bank stock to keep an eye on august th terawulf stock jump more than a google boost stake in data center operator top bse gainer to watch in uncy investor have opportunity to lead unicycive therapeutic inc security fraud lawsuit with the schall law firm cornerstone select advisor llc reduces stock position in pfizer inc pfe southeast toyota finance ranked highest in overall dealer satisfaction by jd power forget ai robotic process automation is healthcare hottest technology warehouse teamster at unfi win lucrative first contract promising retail stock to follow now august th alphabet inc goog share sold by wellington management group llp promising lithium stock to keep an eye on august th insurance stock to watch today august th hydrogen stock to consider august th pwc kunai acquisition to bolster tech enablement for bank cfo the bull case for nvidia just got stronger according to these analyst this curved samsung screen is at one of it lowest price today soho house to be taken private in billion deal the new york time expect fiery outcome from fed jackson hole conference this week financial advisor network inc take position in cocacola company the ko what analyst rating have to say about the campbell mesa laboratory executes previouslyannounced strategic financing plan ibm option trading a deep dive into market sentiment forecasting the future analyst projection for cloudflare a closer look at walmarts option market dynamic flex meal deal return for faculty staff and graduate and professional student paypal holding option frenzy what you need to know a glimpse into the expert outlook on jm smucker through analyst assessing microsoft insight from financial analyst this ethereum trader turned into million in month the analyst verdict fedex in the eye of expert ai take apple edge foxconns pivot could spark etf shift where prudential financial stand with analyst mesa laboratory executes previouslyannounced strategic financing plan wired roundup why gpt flopped wired is the market bullish or bearish on royal gold looking into willis tower watson recent short interest a look into pge inc price over earnings how is the market feeling about lumentum holding ozempic creator novo nordisk will sell weight loss drug for cheaper through this new partnership novo nordisk offer ozempic at per month to eligible u cashpaying customer reuters texas may have to shut down data center to protect it energy grid can blockdag reach analyst review of the m presale in dogecoin news today dogecoin price decline but technical indicator suggest potential rebound applied digitals stock apld jump on plan for billion ai campus tipranks worker are job hugging in a stagnant labor market but growing resentment mean they could bail a soon a the next great resignation come yahoocom texas attorney general accuses meta characterai of misleading kid with mental health claim techcrunch worker are job hugging in a stagnant labor market but growing resentment mean they could bail a soon a the next great resignation come fortune conservative network newsmax agrees to pay m in defamation case over bogus election claim skechers named title sponsor of world champion cup shriners childrens announced a official charity partner feather sound country club in clearwater florida to host tournament whats going on with propanc share monday mastercard and worldpay team to streamline uae money movement mcdonalds corporation mcd share sold by community bank trust waco texas granite harbor advisor inc boost holding in mcdonalds corporation mcd walmart ha everything you need to head back to school from backpack to laptop madd join force with law enforcement to prevent impaired driving ahead of labor day with saturation saturday initiative this weekend ibd live qa stock list for monday aug spotlight on fed what powell bowman and waller will say about rate dogecoin rally spark buzz but trader say this sub coin ha more upside fairscale capital llc purchase share of crowdstrike crwd lee financial co sell share of danaher corporation dhr berger montague pc investigates security claim against kindercare learning company inc nyse klc amazon is selling an bluetooth speaker for and it perfect for any setting inventhelp inventor develops new training aid for basketball player chk top data science recruiter in find ai analytics and ml expert gsg advisor llc purchase share of invesco qqq qqq gsg advisor llc ha stock holding in mastercard incorporated ma weekly bankruptcy alert august for the week ending august jackson hole loom a powell speech test september ratecut hope newsmax to pay million to settle dominion defamation lawsuit intel stock drop on report of equity stake via the chip act barrons liquid edge ai platform leap expands support to laptop with bestinclass performance on amd ryzentm and ryzen aitm processor ap business summarybrief at pm edt ap business summarybrief at pm edt texas democrat are back what now froma harrop are parent who dont vaccinate their child guilty of abuse handwritten proof of holocaust theft should compel congress to act ap news summary at pm edt ap news summary at pm edt state and dc sue doj to stop immigration requirement on victim fund trump zelenskyy meeting not end of the road for u support in securing a peace deal editorial roundup united state eric adam roll out nypd expansion say trump dc crackdown not a factor ap trending summarybrief at pm edt texas lawmaker in illinois heading back home following twoweek walkout over remap fight nfl team refuse to back down after facing backlash for hiring male cheerleader stephen miller say trump dc crackdown will also target graffiti ap news summary at pm edt conservative network newsmax agrees to pay m in defamation case over bogus election claim mark hamill say his wife clever thought stopped him from fleeing u after trump won trump zelensky put on the smile at oval office vancouver mayor warns delay on i bridge replacement cost m per day trump zelensky put on the smile at oval office hamas accepts an arab ceasefire proposal on gaza a palestinian death toll pass texas redistricting fight shift a democrat return to austin with a new strategy mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown on putin advice trump launch assault on mailin ballot and voting machine eo seek to expand access to alternative asset investment in retirement plan doj demand sensitive illinois voter registration data mike mcgrew an alternative mindset for patriotic independent commentary ha brian stelter doesnt get that he only making msnbcs rebranding even funnier in his excited thread former attorney general william barr say he didnt see trump implicated in epstein file former attorney general william barr say he didnt see trump implicated in epstein file gavin newsom left fox news speechless with his unexpectedly hilarious woke comeback these state leader might be the last line of defense against trump abuse of power subsidence isnt just an environmental crisis and it can be slowed the latest zelenskyy signal openness to threeway meeting with trump and putin doj wont appeal judge order on concealed carry ban in post office the latest zelenskyy signal openness to threeway meeting with trump and putin letter political treachery versus personal charity what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work bnpl provider ask for extension to nydfs request for information deadline wyoming teen educate youth about human trafficking on social medium congress must correct an injustice facing combatinjured veteran how blessing and disaster shape alabama why is the c galaxy such an iconic aircraft texas attorney general accuses meta characterai of misleading kid with mental health claim texas ag accuses meta characterai of misleading kid with mental health claim european leader join trump zelenskyy at white house conservative network newsmax agrees to pay m in defamation case over bogus election claim what to know about redistricting fight a texas democrat return and california start work what to know about redistricting fight a texas democrat return and california start work twoweek standoff end quorum reached in texas house mississippi becomes fourth state to send national guard troop to dc in expanding federal crackdown letter trumpputin photo op accomplished nothing judge weighs detainee legal right at alligator alcatraz in florida everglades judge weighs detainee legal right at alligator alcatraz in florida everglades roblox is locking down sexual content and access to adult location after lawsuit trump say the u would back european security guarantee for ukraine to help end the war with russia good in a crisis dr nirav shah could be a promising candidate for anything steve collins wear a suit bro zelenskyy greeted by banner begging him to dress for the occassion did he hulk hogan couldnt stand gavin newsom exwife say about govs online trolling rightwing reporter brian glenn praise zelenskys attire after shaming him in february texas democrat return ending twoweek walkout over redistricting trump say hell talk to putin after meeting with zelenskyy and european leader at the white house reporter brian glenn brag about dc being safe after walking street with girlfriend marjorie taylor greene zelenskyy trump express hope for trilateral talk with putin to bring end to russiaukraine war oval office meeting again put rocky tense trumpzelenskyy relationship to the test armstrong williams how george washington would end russia war on ukraine staff commentary la habra man charged in fatal whittier shooting of driver texas democrat head home after week in illinois mpo holding first public planning session tuesday at mountain line photo show aftermath of a deadly russian attack in ukraine and the funeral of a fallen soldier now thats a selfown eric swalwell grocery shopping go viral for all the wrong hilarious reason texas democrat return to capitol for republican u house map overhaul a california counter texas democrat return to capitol for republican u house map overhaul a california counter letter time for democrat to play to win volodymyr zelensky wear suit this time for white house meeting with trump tarrant county commissioner again propose cutting voting site ahead of an election this is exactly what technology should be doing man shot injured in parking lot of huntington beach store letter no place for threat violence in politics trump aim to set putinzelenskiy meeting after monday summit obbba creates a cohesive framework for u hydrogen growth top trump lackey demand dc resident kiss the ground for occupation republican look to make a uturn on electric vehicle for the postal service republican look to make a uturn on electric vehicle for the postal service</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>inventhelp inventor develop new thermal capacitor water heater tl council asked to help expand eye on the street program gray medium to produce and air tomorrow new orleans saint preseason game in endtoend native hdr via nextgen tv hidden google search feature that make you a power user jerome powell signal fed may cut rate soon even a inflation risk remain elon musk must face lawsuit for duping trump supporter in million giveaway give your teeth the care they deserve with off an aquasonic ultra whitening toothbrush u supreme court allows nih to cut billion in research grant nature ninepoint partner announces estimated august cash distribution for ninepoint cash management fund etf series clean smarter not harder the best electric spin scrubber make cleaning a breeze federal workforce to lose employee this year trump official say in canada billboard woman in music open nomination for honoree cracker barrel crackup how the culture war are upending corporate branding powell signal fed may cut rate soon even a inflation risk remain canada will match u tariff exemption under usmca trade pact prime minister carney say whats needed to unlock the power and promise of imec new rv provides opioid recovery medical care to underserved minneapolis neighborhood powell signal fed may cut rate soon even a inflation risk remain onlyfans stats that show how massive the platform ha become green space are key to combating record heat in marginalized community familyfriendly workplace gov order budget cut for all state agency except school why xrp is soaring today are you even ready to grow lesson every owneroperator need before adding a truck gen z career catfishing rise ai recruiter a ethical solution trump say canada will drop usmcacompliant retaliatory tariff capital solution hire former caci exec a chief operating officer sunflower elect new board leader director king island tease return of beloved phantom theater ride top evercore analyst boost nvidia nvda stock price target ahead of q earnings tipranks bank lobby for national standard to limit state regulation shareholder alert levi korsinsky llp notifies investor it ha filed a complaint to recover loss suffered by purchaser of cai inc security and set a lead plaintiff deadline of october rosen national investor counsel encourages lockheed martin corporation investor to secure counsel before important deadline in security class action lmt elite express holding inc announces closing of million initial public offering ross benefit from value shopper but tariff challenge continue cvcc board set to review tax implication of new career center best ai writing tool for researcher zumpano patricios welcome sebastian jaramillo a income partner strengthening real estate practice zumpano patricios welcome sebastian jaramillo a income partner strengthening real estate practice canada to ease most retaliatory tariff against united state extrump cfo weisselberg may keep severance pay appellate court rule ethylene buyer could be ruined for their cartel example of unpaid work deal dispatch muskaltman drama ashton kutcher soho house play and we pose question to private equity pro fiserv push embedded payment for health care canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal netskope file for u ipo with m revenue yoy growth walmart q revenue surge to b raise fullyear outlook delta airline offering new direct flight from austin airport why intuit stock intu is sinking today blue bell ice cream recalled due to packaging error trump say hell be very good to canada a it prime minister drop some tariff trump say we want to be very good to canada a it leader drop some tariff canada remove some of it retaliatory tariff on the u canada remove some of it retaliatory tariff on the u canada remove some of it retaliatory tariff on the u npr trump say we want to be very good to canada a it leader drop some tariff canada remove some of it retaliatory tariff on the u weekly commodity wrapup why lucid group stock died today then got better tinley park chamber cancel this year oktoberfest due to cost how market reacted after powell signaled potential rate cut eastgroup property announces dividend increase how nvidias chip became central to the uschina trade war how nvidias chip became central to the uschina trade war how nvidias chip became central to the uschina trade war how nvidias chip became central to the uschina trade war branded legacy inc form strategic partnership with stanford university dr eran bendavid to advance addiction solution stock market surge after jerome powell indicates rate cut may be coming canada remove countertariffs on some u good canada to drop countertariffs on some u good one day after call with trump bitcoin and crypto stock surge a powell ratecut hint revives risk appetite walmart hike discount for shopper amid tariff uncertainty this is what whale are betting on okta starbucks car toy close on broadway in denver coffee giant closing all non drivethrus snap investor with loss in excess of k have opportunity to lead snap inc security lawsuit kirby mcinerney llp announces investigation against avita medical inc on behalf of investor bear alley marketing position itself a a leader in performance marketing for home service trump say hell keep extending tiktok shutdown deadline let talk indianola school business official brian bartz what is credit card forbearance and who qualifies for it this september bet bonus code nypbet bet get in bonus bet win or lose for yankee v red sox on friday sima monthly investment fund statistic july pi down from ath icp volume tank meanwhile blockdags b token sold point to the next x dsw offer discount on brook revel running shoe this week degree capital announces result of special meeting of shareholder to approve the proposed business combination with mount logan capital inc brattleboro parking zone to be relabeled high roller announces nyse acceptance of plan to regain listing compliance degree capital announces result of special meeting of shareholder to approve the proposed business combination with mount logan capital inc canada to remove many retaliatory tariff on u good allegro stock recovery elliott wave structure support fundamental case labubu blind box restocking aug aug here what to know trump say intel ha agreed to give the u a equity stake bloomberg rich lowry trump is wrong about mailin voting cheap drug high stake america risky bet on china trump again give putin a couple of week with no sign of ukraine peace talk underway cnn trump suggests chicago is next for federal crime crackdown followed by new york city cbs news president donald trump plan crime crackdown in chicago similar to dc national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital court ruling clear the way for hundred of cdc staff to be laid off jury selection taking time in randolph csc trial mayor trump president fixates on local crime asphalt and lamppost latest news on fbi searching john boltons home office george mason illegally used race in hiring department of education find george mason illegally used race in hiring department of education find a judge ha ordered alligator alcatraz in florida to wind down operation what happens now world cup draw will be held at washington kennedy center trump say kamala harris will take her day book tour to los angeles california gov gavin newsoms national profile soar with latest trump fight but there are risk california gov gavin newsoms national profile soar with latest trump fight but there are risk california gov gavin newsoms national profile soar with latest trump fight but there are risk newsoms profile soar with trump redistricting fight california gov gavin newsoms national profile soar with latest trump fight but there are risk california gov gavin newsoms national profile soar with latest trump fight but there are risk california gov gavin newsoms national profile soar with latest trump fight but there are risk lake lynn answer ferc question raise possibility of entry fee at cheat lake park people officially became u citizen at the new york state fair funeral home owner who stashed nearly decaying body set to be sentenced new york city to get federal police for crime crackdown after dc chicago trump trump praise missouri republican for considering redistricting bolton investigated over classified document not politics vp vance tell nbc community patrol confronts ice officer at city height elementary school parking lot stitt take aim at tulsa mayor decision to prosecute crime in tribal court trump tariff will reduce deficit by trillion over next decade say cbo report ask rusty how do i apply for s and receive my payment trump say hell keep extending tiktok shutdown deadline trump say hell keep extending tiktok shutdown deadline trump say hell keep extending tiktok shutdown deadline trump say hell keep extending tiktok shutdown deadline uk diplomat receives warning over illegal fishing with jd vance mit global collapse warning revisited humanity enters makeorbreak decade chicago is up next for the national guard theyre screaming for u say trump san carlos and the lastminute commissioner item henderson accepting application for addition to veteran memorial wall trump reacts to canada reversing retaliatory tariff take question at white house erik and lyle menendez can still walk free from prison even if both brother have parole denied a family fight back desantis fire back after dem decries florida move to ditch lgbt rainbow color from crosswalk in orlando hegseth authorizes national guard to carry gun in washington dc ap technology summarybrief at pm edt trump is astonishingly deluded about putin trump official demand apology from george mason president over diversity the new york time the u air force just underwent a massive stress test of how it would fight a highend war in the pacific uk top diplomat get a warning for illegal fishing with u vice president national guard troop in washington will be armed hegseth matt fleming how assembly democrat came to embrace gerrymandering passing the baton in europe could donald trump really win the nobel peace prize asking eric am i wrong for wanting to back out of mexican vacation now that friend included her son beware of the skeeters and malary asking eric am i wrong for backing out of a trip because a friend son is going an energy transition at the crossroad south korea journey toward resilience the u navy drone effort arent going wellbut neither are china pa budget stall again what will it take to break the cycle of delay carney say he will travel to germany next week to deepen tie canada go learn some english customer berates georgian nyc cafe owner now everyones coming to her defense teaching just the fact is not an answer to indoctrination gavin newsoms redistricting gambit a presidential audition not a policy plan fifa world cup draw to take place at kennedy center trump announces tension flare a texas house panel hears a bathroom bill for first time in eight year trump message to dc criminal democrat dont mess with me how some apps are working to solve the epidemic of loneliness what to expect from the ussouth korea summit planned parenthood sue south carolina over medicaid ban certain local voice oppose gov newsoms redistricting campaign cracker barrel new logo sucksand not because of wokeness you idiot ct governor directs flag to halfstaff saturday for state employee fatally injured on job trump say hell ask congress for b for dc improvement letter taxpayer against genocide trump say putin may attend north america world cup it so on after heated back and forth with chris rufo on conservatism jonah goldberg agrees to debate homeowner oppose plan for fencing dune on hollywood beach here why trump say putin may attend north america world cup california ab stall in senate amid parental right opposition trump say putin may attend north america world cup trump say putin may attend north america world cup california governor signed a redistricting plan what happens next trump show off photo putin mailed him from alaska summit but president warns i better be very happy with peace talk after russia ukraine attack policy review committee recap august james jim mcgregor trump say chicago is next for dcstyle federal law enforcement operation a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now shiba inu shib is taking longer than expected to reach new high in pepe coin pepe and this coin to outperform it investing in ozak ai ethereumbased ai token during it under presale could lead to millionaire status by a btc and eth hit ath cadence bank ha million stock holding in texas instrument incorporated txn jpmorgan chase co jpm share sold by rbo co llc hoka ha shoe on sale for a low a right now including bondi and clifton trump administration halt construction of revolution wind farm off mass citing national security new brewery tap into corydons dora ordinance excitement british columbia investment management corp sell share of alphabet inc goog british columbia investment management corp raise holding in broadcom inc avgo air canada say more passenger eligible for reimbursement if flight were cancelled canada grab these safe djia dividend bargain after index hit alltime high nextgen pick best cryptos to buy today a arctic pablos cex listing driving maximum gain potential twothirds of river trash is plastic research fastfood chain lock in meal to fight inflation in newsguild see organizing surge a medium worker fuel grassroots militancy tech ceo urge dignity for billion shift worker amid automation lowes target pro with total home strategy amid sale dip and inflation european postal service halt u shipment over trump tariff china stock surge defies weak economy raising fear of another bust analyst waste management inc nysewm announces quarterly dividend evans city council approves ballot language for permanent road tax bet bonus code orl bonus for seahawks v packer raider v cardinal solana whale rotate capital into layer brett analyst say it could deliver x gain by next year whale are choosing this meme coin a the best crypto to buy in instead of dogecoin doge and shiba sol strengthens on institutional demand xrp jump after whale action and blockdags forecast draw buyer in phoenix wealth advisor sell share of air product and chemical inc apd btc climbed to of global money before fed chair signaled rate cut cointelegraph heritage wealth partner llc buy share of meta platform inc meta palantir technology nasdaqpltr insider ryan taylor sell share palantir technology nasdaqpltr insider ryan taylor sell share of stock promising retail stock to keep an eye on august th jpmorgan chase co jpm is biondo investment advisor llcs th largest position immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say trump appeal in fraud case likely despite his total victory trump appeal in fraud case likely despite his total victory baby boomer turned meme stock trading into a thrilling hobby calling it absolutely gambling trump appeal in fraud case likely despite his total victory this weatherproof storage shed is only during wayfairs labor day blowout sale bank of america nysebac hit new month high whats next invesco qqq qqq share purchased by haverford trust co cardano price prediction ada eye new high yet this lowcap coin ha x more upside beltway buzz august apg asset management nv acquires share of intuitive surgical inc isrg pfizer inc pfe share sold by apg asset management nv what to know about visa for foreign trucker and the politics of a deadly florida crash the best amazon deal to shop right now save up to trump halt work on new england offshore wind project thats nearly complete trump halt work on new england offshore wind project thats nearly complete bitcoin btc price could retrace before a run toward kk but ripple xrp and this coin are aiming high in cryptos next top altcoin why this crypto could shine a xrp fall below best gift for digital artist in trump halt work on nearly complete new england offshore wind project waste management inc wm share acquired by groupe la francaise union pacific corporation unp share purchased by kestra advisory service llc haverford trust co sell share of unitedhealth group incorporated unh waste management inc wm share sold by van hulzen asset management llc groupe la francaise purchase share of walmart inc wmt phoenix wealth advisor trim position in cisco system inc csco bahl gaynor inc increase stake in taiwan semiconductor manufacturing company ltd tsm best of the best bahl gaynor inc sell share of mcdonalds corporation mcd chicago a mess trump vow national guard crackdown layer brett dubbed pepe after early momentum outpaces early doge and shib launch hooter bankruptcy prompt rebrand to tacky familyfriendly are home depot cheapest tool set worth buying here what user say trump halt work on new england offshore wind project thats nearly complete douglas winthrop advisor llc sell share of pepsico inc pep caitlin john llc ha holding in invesco qqq qqq british columbia investment management corp buy share of procter gamble company the pg penticton council willing to work with art gallery after layoff announced penticton get your own steam locomotive how family can save money this backtoschool season northwest minnesota foundation issue over million in grant loan during th quarter why the iea reinstated it business a usual scenario business accelerator academy start in september how u of a help build worldclass entrepreneur dogecoin price target in september but analyst say x gain belong to new lowcaps can solana reach by or is there a better crypto to buy now blockdags m presale and referral reward shift focus from xrp rally and eth market issue trump halt work on new england offshore wind project thats nearly complete yahoocom trump halt work on new england offshore wind project thats nearly complete trump halt work on new england offshore wind project thats nearly complete ai bubble fear spark tech stock slide crash warning rise how and where to bet mlb player prop pick odds for aug garrett crochet among best bet smartleaf asset management llc ha million stock holding in mastercard incorporated ma walmart nysewmt issue fy earnings guidance biondo investment advisor llc ha million stake in unitedhealth group incorporated unh cadence bank sell share of american express company axp forest avenue capital management lp boost holding in vistra corp vst european post suspend u delivery over trumpera tariff biondo investment advisor llc acquires share of amgen inc amgn svb wealth llc lower stock position in blackrock blk svb wealth llc sell share of air product and chemical inc apd air product and chemical inc apd share sold by british columbia investment management corp svb wealth llc sell share of air product and chemical inc apd lionshead wealth management llc ha holding in illinois tool work inc itw biondo investment advisor llc increase stock holding in duke energy corporation duk kruse out a dia director in latest pentagon shakeup cringe watch zohran mamdani plan nyc scavenger hunt is there a prize if youre mugged on the subway cu colorado spring campus thought it could avoid trump education crackdown here what happened cu colorado spring campus thought it could avoid trump education crackdown here what happened cu colorado spring campus thought it could avoid trump education crackdown here what happened u justice department release transcript of interview with ghislaine maxwell kilmar abrego garcia is freed from tennessee jail so he can rejoin family in maryland to await trial greene issue scathing rebuke of condition in gaza i will not be silent about it israel vow to open gate of hell on gaza in chilling warning a famine grip the region u seek to deport kilmar abrego garcia to uganda after he refused plea offer in his smuggling case u seek to deport kilmar abrego garcia to uganda after he refused plea offer in his smuggling case kevin oleary sound alarm on rich kid upbringing they become lost in a sea of mediocrity it a disaster for them former dhs official signal he could be next after bolton fbi raid we expect it the lioness at the center of a city hall battered by scandal dnc vote on israel arm embargo may set democratic party course on palestine trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it u seek to deport abrego garcia to uganda hampton county law enforcement to ramp up duo patrol trump administration considering deporting kilmar abrego garcia to uganda his lawyer say secretariat jockey mourned in maine a well a canada dunkin customer warns to check receipt after spotting wellness fee national guard roll out in state not linked to trump crime crackdown wh say the redistricting war between texas and california is about to jolt the midterm politico asking eric were no longer invited to shared family holiday meal what should we do about upcoming wedding redistricting war poised to explode a california and texas make their move la consequential karen bass earns epic ratio over claim city recovery is fastest in state history the redistricting war between texas and california is about to jolt the midterm texas abbott promise quick signature of redistricting plan following overnight senate vote ghislaine maxwell absolves trump and everyone else in doj interview conservative activist slam cracker barrel a company left reeling after logo redesign south korea japan agree to boost tie a challenge mount kilmar abrego garcia released from ice custody after return from el salvador truck driver in crash at center of trump administration feud with newsom is denied bond when trying to explain low dem party polling look no further than awesome duo of newsom and swalwell immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say u seek to deport kilmar abrego garcia to uganda after he refused plea offer in his smuggling case trump look to chicago next in federal crackdown the wall street journal giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell university of oregon concludes law review discriminated based on perceived national origin against israeli author trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress how redistricting is done and why it could give party an edge in election how redistricting is done and why it could give party an edge in election democrat mock jd vance for having cardboard charisma a he push unpopular budget bill opinion it time for mayo pete buttigieg to find some seasoning what happened to ambition for bay restoration guest commentary kilmar abrego garcia threatened with deportation to uganda larimer county restaurant inspection made aug kilmar abrego garcia threatened with deportation to uganda kilmar abrego garcia threatened with deportation to uganda judge block trump from cutting funding from city and county including denver over sanctuary policy internet tax freedom act preempt new york imposition of tax fbi target john boltons home and office trump he not a smart guy but he could be a very unpatriotic guy inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal rachel bitecofer warns that bolton is just the start and trump will go after the rest of u inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal what we know about china and russia new strategic bomber inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal zelenskyy say security guarantee for ukraine to be ready soon bill maher applauds gavin newsom for mocking donald trump i think it very funny floridarun alligator alcatraz violates u law aclu say russia announces support for venezuela to defend sovereignty amid growing military tension with the united state gianno caldwell mull senate bid a chicagoans are begging for change on crime woe trump threatens chicago with next national guard invasion cnn analyst pinpoint the weirdest part of ghislaine maxwell simply bizarre doj interview cnn analyst pinpoint the weirdest part of ghislaine maxwell simply bizarre doj interview the owl eye liberty and memory from epstein suicide to trump and clinton takeaway from ghislaine maxwell transcript how can israel engineer a famine in gaza in the st century what we learned from the ghislaine maxwell doj interview texas gov abbott say hell swiftly sign redistricting map after lawmaker approve them jeff bezos said he would have felt icky had he taken any more share of amazon i just didnt feel good smart money strategy what the pro buy when the crypto market crash radioactive shrimp update walmart store brand and other brand recalled european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff a winning powerball ticket ha been sold in western new york the sp hasnt yielded this little since the dotcom bubble here what investor can do the motley fool just ranked the biggest financial stock here why the no pick could be your best investment mezcal producer preserve traditional method a demand for liquor grows minute european postal service suspend shipment of package to u over tariff kpop demon hunter give netflix it first boxoffice win curry join the bank holiday sale bonanza with it epic deal event here are the best offer id buy self driving taxi may be coming to nyc a waymo win first av testing permit mashable rosen a leading law firm encourages fiserv inc investor to secure counsel before important rosen a leading law firm encourages fiserv inc investor to secure counsel before important rosen a leading law firm encourages fiserv inc investor to secure counsel before important rosen a leading law firm encourages fiserv inc investor to secure counsel before important rosen a leading law firm encourages fiserv inc investor to secure counsel before important deadline in security class action fi ice cream sold at walmarts across state recalled due to undeclared allergen here how a gamestop purchase turned into a bitcoin jackpot ice cream sold at walmarts across state recalled due to undeclared allergen fox business prediction lucid group sale will soar over the next year if this happens solar executive warn that trump attack on renewables will lead to power crunch that spike electricity price pueblo county home listing asked for less money in july see the current median price here prediction these trilliondollar artificial intelligence ai stock could strike a megadeal that wall street isnt ready for cold wallet cashback utility and presale pricing create a upside case while chainlink and shiba inu struggle maintenance compliance burden viability of hopi water treatment system ethereum in trouble xrp might breakout buyer turn to blockdag to earn referral reward acting a the executor of a will can be a very lucrative job the last word national guard troop to be force multiplier for ice homan little pepe crypto price prediction is lilpepe a good investment for longterm holder here how much you should aim to invest in the invesco qqq etf to get to million or more by retirement state audit question m in federal spending by moses lake school district blockchain stock worth watching august th owner scale back golden mile shopping center redevelopment rosen global investor counsel encourages easterly rocmuni high income municipal bond fund comerica bank lower stake in alphabet inc goog trump tap airbnb cofounder a st government design head to lead huge web overhaul trump tap airbnb cofounder a st government design head to lead huge web overhaul fox business offgrid living next new real estate trend a application for rural mortgage skyrocket rosen global investor counsel encourages altimmune inc investor to secure counsel before rosen global investor counsel encourages altimmune inc investor to secure counsel before rosen global investor counsel encourages altimmune inc investor to secure counsel before epstein accuser virginia giuffre wrote a memoir month after her death it coming out powell warning signal unemployment claim jump to highest in year cardano price outlook can ada reach trumprelated defi platform world liberty financial debut wlfi token on ethereum mainnet rosen global investor counsel encourages altimmune inc investor to secure counsel before important deadline in security class action alt the best meme coin presale stampede is loading whitelist labubull now or watch it moon without you backtoschool deal tellos unlimited plan get you cell service for per month your first month nexus gold cvenxs stock price up whats next mason resource cvellg stock price up here why mason resource cvellg trading up here what happened national guard troop to be force multiplier for ice homan freedom investment management inc purchase share of procter gamble company the pg ascent group llc raise stock holding in ameri</t>
+          <t>inventhelp inventor develop new thermal capacitor water heater tl council asked to help expand eye on the street program gray medium to produce and air tomorrow new orleans saint preseason game in endtoend native hdr via nextgen tv hidden google search feature that make you a power user jerome powell signal fed may cut rate soon even a inflation risk remain elon musk must face lawsuit for duping trump supporter in million giveaway give your teeth the care they deserve with off an aquasonic ultra whitening toothbrush u supreme court allows nih to cut billion in research grant nature ninepoint partner announces estimated august cash distribution for ninepoint cash management fund etf series clean smarter not harder the best electric spin scrubber make cleaning a breeze federal workforce to lose employee this year trump official say in canada billboard woman in music open nomination for honoree cracker barrel crackup how the culture war are upending corporate branding powell signal fed may cut rate soon even a inflation risk remain canada will match u tariff exemption under usmca trade pact prime minister carney say whats needed to unlock the power and promise of imec new rv provides opioid recovery medical care to underserved minneapolis neighborhood powell signal fed may cut rate soon even a inflation risk remain onlyfans stats that show how massive the platform ha become green space are key to combating record heat in marginalized community familyfriendly workplace gov order budget cut for all state agency except school why xrp is soaring today are you even ready to grow lesson every owneroperator need before adding a truck gen z career catfishing rise ai recruiter a ethical solution trump say canada will drop usmcacompliant retaliatory tariff capital solution hire former caci exec a chief operating officer sunflower elect new board leader director king island tease return of beloved phantom theater ride top evercore analyst boost nvidia nvda stock price target ahead of q earnings tipranks bank lobby for national standard to limit state regulation shareholder alert levi korsinsky llp notifies investor it ha filed a complaint to recover loss suffered by purchaser of cai inc security and set a lead plaintiff deadline of october rosen national investor counsel encourages lockheed martin corporation investor to secure counsel before important deadline in security class action lmt elite express holding inc announces closing of million initial public offering ross benefit from value shopper but tariff challenge continue cvcc board set to review tax implication of new career center best ai writing tool for researcher zumpano patricios welcome sebastian jaramillo a income partner strengthening real estate practice zumpano patricios welcome sebastian jaramillo a income partner strengthening real estate practice canada to ease most retaliatory tariff against united state extrump cfo weisselberg may keep severance pay appellate court rule ethylene buyer could be ruined for their cartel example of unpaid work deal dispatch muskaltman drama ashton kutcher soho house play and we pose question to private equity pro fiserv push embedded payment for health care canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal canada removing tariff on u good compliant with free trade deal netskope file for u ipo with m revenue yoy growth walmart q revenue surge to b raise fullyear outlook delta airline offering new direct flight from austin airport why intuit stock intu is sinking today blue bell ice cream recalled due to packaging error trump say hell be very good to canada a it prime minister drop some tariff trump say we want to be very good to canada a it leader drop some tariff canada remove some of it retaliatory tariff on the u canada remove some of it retaliatory tariff on the u canada remove some of it retaliatory tariff on the u npr trump say we want to be very good to canada a it leader drop some tariff canada remove some of it retaliatory tariff on the u weekly commodity wrapup why lucid group stock died today then got better tinley park chamber cancel this year oktoberfest due to cost how market reacted after powell signaled potential rate cut eastgroup property announces dividend increase how nvidias chip became central to the uschina trade war how nvidias chip became central to the uschina trade war how nvidias chip became central to the uschina trade war how nvidias chip became central to the uschina trade war branded legacy inc form strategic partnership with stanford university dr eran bendavid to advance addiction solution stock market surge after jerome powell indicates rate cut may be coming canada remove countertariffs on some u good canada to drop countertariffs on some u good one day after call with trump bitcoin and crypto stock surge a powell ratecut hint revives risk appetite walmart hike discount for shopper amid tariff uncertainty this is what whale are betting on okta starbucks car toy close on broadway in denver coffee giant closing all non drivethrus snap investor with loss in excess of k have opportunity to lead snap inc security lawsuit kirby mcinerney llp announces investigation against avita medical inc on behalf of investor bear alley marketing position itself a a leader in performance marketing for home service trump say hell keep extending tiktok shutdown deadline let talk indianola school business official brian bartz what is credit card forbearance and who qualifies for it this september bet bonus code nypbet bet get in bonus bet win or lose for yankee v red sox on friday sima monthly investment fund statistic july pi down from ath icp volume tank meanwhile blockdags b token sold point to the next x dsw offer discount on brook revel running shoe this week degree capital announces result of special meeting of shareholder to approve the proposed business combination with mount logan capital inc brattleboro parking zone to be relabeled high roller announces nyse acceptance of plan to regain listing compliance degree capital announces result of special meeting of shareholder to approve the proposed business combination with mount logan capital inc canada to remove many retaliatory tariff on u good allegro stock recovery elliott wave structure support fundamental case labubu blind box restocking aug aug here what to know trump say intel ha agreed to give the u a equity stake bloomberg rich lowry trump is wrong about mailin voting cheap drug high stake america risky bet on china trump again give putin a couple of week with no sign of ukraine peace talk underway cnn trump suggests chicago is next for federal crime crackdown followed by new york city cbs news president donald trump plan crime crackdown in chicago similar to dc national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital national guard troop will soon carry weapon in u capital court ruling clear the way for hundred of cdc staff to be laid off jury selection taking time in randolph csc trial mayor trump president fixates on local crime asphalt and lamppost latest news on fbi searching john boltons home office george mason illegally used race in hiring department of education find george mason illegally used race in hiring department of education find a judge ha ordered alligator alcatraz in florida to wind down operation what happens now world cup draw will be held at washington kennedy center trump say kamala harris will take her day book tour to los angeles california gov gavin newsoms national profile soar with latest trump fight but there are risk california gov gavin newsoms national profile soar with latest trump fight but there are risk california gov gavin newsoms national profile soar with latest trump fight but there are risk newsoms profile soar with trump redistricting fight california gov gavin newsoms national profile soar with latest trump fight but there are risk california gov gavin newsoms national profile soar with latest trump fight but there are risk california gov gavin newsoms national profile soar with latest trump fight but there are risk lake lynn answer ferc question raise possibility of entry fee at cheat lake park people officially became u citizen at the new york state fair funeral home owner who stashed nearly decaying body set to be sentenced new york city to get federal police for crime crackdown after dc chicago trump trump praise missouri republican for considering redistricting bolton investigated over classified document not politics vp vance tell nbc community patrol confronts ice officer at city height elementary school parking lot stitt take aim at tulsa mayor decision to prosecute crime in tribal court trump tariff will reduce deficit by trillion over next decade say cbo report ask rusty how do i apply for s and receive my payment trump say hell keep extending tiktok shutdown deadline trump say hell keep extending tiktok shutdown deadline trump say hell keep extending tiktok shutdown deadline trump say hell keep extending tiktok shutdown deadline uk diplomat receives warning over illegal fishing with jd vance mit global collapse warning revisited humanity enters makeorbreak decade chicago is up next for the national guard theyre screaming for u say trump san carlos and the lastminute commissioner item henderson accepting application for addition to veteran memorial wall trump reacts to canada reversing retaliatory tariff take question at white house erik and lyle menendez can still walk free from prison even if both brother have parole denied a family fight back desantis fire back after dem decries florida move to ditch lgbt rainbow color from crosswalk in orlando hegseth authorizes national guard to carry gun in washington dc ap technology summarybrief at pm edt trump is astonishingly deluded about putin trump official demand apology from george mason president over diversity the new york time the u air force just underwent a massive stress test of how it would fight a highend war in the pacific uk top diplomat get a warning for illegal fishing with u vice president national guard troop in washington will be armed hegseth matt fleming how assembly democrat came to embrace gerrymandering passing the baton in europe could donald trump really win the nobel peace prize asking eric am i wrong for wanting to back out of mexican vacation now that friend included her son beware of the skeeters and malary asking eric am i wrong for backing out of a trip because a friend son is going an energy transition at the crossroad south korea journey toward resilience the u navy drone effort arent going wellbut neither are china pa budget stall again what will it take to break the cycle of delay carney say he will travel to germany next week to deepen tie canada go learn some english customer berates georgian nyc cafe owner now everyones coming to her defense teaching just the fact is not an answer to indoctrination gavin newsoms redistricting gambit a presidential audition not a policy plan fifa world cup draw to take place at kennedy center trump announces tension flare a texas house panel hears a bathroom bill for first time in eight year trump message to dc criminal democrat dont mess with me how some apps are working to solve the epidemic of loneliness what to expect from the ussouth korea summit planned parenthood sue south carolina over medicaid ban certain local voice oppose gov newsoms redistricting campaign cracker barrel new logo sucksand not because of wokeness you idiot ct governor directs flag to halfstaff saturday for state employee fatally injured on job trump say hell ask congress for b for dc improvement letter taxpayer against genocide trump say putin may attend north america world cup it so on after heated back and forth with chris rufo on conservatism jonah goldberg agrees to debate homeowner oppose plan for fencing dune on hollywood beach here why trump say putin may attend north america world cup california ab stall in senate amid parental right opposition trump say putin may attend north america world cup trump say putin may attend north america world cup california governor signed a redistricting plan what happens next trump show off photo putin mailed him from alaska summit but president warns i better be very happy with peace talk after russia ukraine attack policy review committee recap august james jim mcgregor trump say chicago is next for dcstyle federal law enforcement operation a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now a judge ha ordered alligator alcatraz in florida to wind down operation what happens now shiba inu shib is taking longer than expected to reach new high in pepe coin pepe and this coin to outperform it investing in ozak ai ethereumbased ai token during it under presale could lead to millionaire status by a btc and eth hit ath cadence bank ha million stock holding in texas instrument incorporated txn jpmorgan chase co jpm share sold by rbo co llc hoka ha shoe on sale for a low a right now including bondi and clifton trump administration halt construction of revolution wind farm off mass citing national security new brewery tap into corydons dora ordinance excitement british columbia investment management corp sell share of alphabet inc goog british columbia investment management corp raise holding in broadcom inc avgo air canada say more passenger eligible for reimbursement if flight were cancelled canada grab these safe djia dividend bargain after index hit alltime high nextgen pick best cryptos to buy today a arctic pablos cex listing driving maximum gain potential twothirds of river trash is plastic research fastfood chain lock in meal to fight inflation in newsguild see organizing surge a medium worker fuel grassroots militancy tech ceo urge dignity for billion shift worker amid automation lowes target pro with total home strategy amid sale dip and inflation european postal service halt u shipment over trump tariff china stock surge defies weak economy raising fear of another bust analyst waste management inc nysewm announces quarterly dividend evans city council approves ballot language for permanent road tax bet bonus code orl bonus for seahawks v packer raider v cardinal solana whale rotate capital into layer brett analyst say it could deliver x gain by next year whale are choosing this meme coin a the best crypto to buy in instead of dogecoin doge and shiba sol strengthens on institutional demand xrp jump after whale action and blockdags forecast draw buyer in phoenix wealth advisor sell share of air product and chemical inc apd btc climbed to of global money before fed chair signaled rate cut cointelegraph heritage wealth partner llc buy share of meta platform inc meta palantir technology nasdaqpltr insider ryan taylor sell share palantir technology nasdaqpltr insider ryan taylor sell share of stock promising retail stock to keep an eye on august th jpmorgan chase co jpm is biondo investment advisor llcs th largest position immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say trump appeal in fraud case likely despite his total victory trump appeal in fraud case likely despite his total victory baby boomer turned meme stock trading into a thrilling hobby calling it absolutely gambling trump appeal in fraud case likely despite his total victory this weatherproof storage shed is only during wayfairs labor day blowout sale bank of america nysebac hit new month high whats next invesco qqq qqq share purchased by haverford trust co cardano price prediction ada eye new high yet this lowcap coin ha x more upside beltway buzz august apg asset management nv acquires share of intuitive surgical inc isrg pfizer inc pfe share sold by apg asset management nv what to know about visa for foreign trucker and the politics of a deadly florida crash the best amazon deal to shop right now save up to trump halt work on new england offshore wind project thats nearly complete trump halt work on new england offshore wind project thats nearly complete bitcoin btc price could retrace before a run toward kk but ripple xrp and this coin are aiming high in cryptos next top altcoin why this crypto could shine a xrp fall below best gift for digital artist in trump halt work on nearly complete new england offshore wind project waste management inc wm share acquired by groupe la francaise union pacific corporation unp share purchased by kestra advisory service llc haverford trust co sell share of unitedhealth group incorporated unh waste management inc wm share sold by van hulzen asset management llc groupe la francaise purchase share of walmart inc wmt phoenix wealth advisor trim position in cisco system inc csco bahl gaynor inc increase stake in taiwan semiconductor manufacturing company ltd tsm best of the best bahl gaynor inc sell share of mcdonalds corporation mcd chicago a mess trump vow national guard crackdown layer brett dubbed pepe after early momentum outpaces early doge and shib launch hooter bankruptcy prompt rebrand to tacky familyfriendly are home depot cheapest tool set worth buying here what user say trump halt work on new england offshore wind project thats nearly complete douglas winthrop advisor llc sell share of pepsico inc pep caitlin john llc ha holding in invesco qqq qqq british columbia investment management corp buy share of procter gamble company the pg penticton council willing to work with art gallery after layoff announced penticton get your own steam locomotive how family can save money this backtoschool season northwest minnesota foundation issue over million in grant loan during th quarter why the iea reinstated it business a usual scenario business accelerator academy start in september how u of a help build worldclass entrepreneur dogecoin price target in september but analyst say x gain belong to new lowcaps can solana reach by or is there a better crypto to buy now blockdags m presale and referral reward shift focus from xrp rally and eth market issue trump halt work on new england offshore wind project thats nearly complete yahoocom trump halt work on new england offshore wind project thats nearly complete trump halt work on new england offshore wind project thats nearly complete ai bubble fear spark tech stock slide crash warning rise how and where to bet mlb player prop pick odds for aug garrett crochet among best bet smartleaf asset management llc ha million stock holding in mastercard incorporated ma walmart nysewmt issue fy earnings guidance biondo investment advisor llc ha million stake in unitedhealth group incorporated unh cadence bank sell share of american express company axp forest avenue capital management lp boost holding in vistra corp vst european post suspend u delivery over trumpera tariff biondo investment advisor llc acquires share of amgen inc amgn svb wealth llc lower stock position in blackrock blk svb wealth llc sell share of air product and chemical inc apd air product and chemical inc apd share sold by british columbia investment management corp svb wealth llc sell share of air product and chemical inc apd lionshead wealth management llc ha holding in illinois tool work inc itw biondo investment advisor llc increase stock holding in duke energy corporation duk kruse out a dia director in latest pentagon shakeup cringe watch zohran mamdani plan nyc scavenger hunt is there a prize if youre mugged on the subway cu colorado spring campus thought it could avoid trump education crackdown here what happened cu colorado spring campus thought it could avoid trump education crackdown here what happened cu colorado spring campus thought it could avoid trump education crackdown here what happened u justice department release transcript of interview with ghislaine maxwell kilmar abrego garcia is freed from tennessee jail so he can rejoin family in maryland to await trial greene issue scathing rebuke of condition in gaza i will not be silent about it israel vow to open gate of hell on gaza in chilling warning a famine grip the region u seek to deport kilmar abrego garcia to uganda after he refused plea offer in his smuggling case u seek to deport kilmar abrego garcia to uganda after he refused plea offer in his smuggling case kevin oleary sound alarm on rich kid upbringing they become lost in a sea of mediocrity it a disaster for them former dhs official signal he could be next after bolton fbi raid we expect it the lioness at the center of a city hall battered by scandal dnc vote on israel arm embargo may set democratic party course on palestine trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it trump ran on a promise of revenge he making good on it u seek to deport abrego garcia to uganda hampton county law enforcement to ramp up duo patrol trump administration considering deporting kilmar abrego garcia to uganda his lawyer say secretariat jockey mourned in maine a well a canada dunkin customer warns to check receipt after spotting wellness fee national guard roll out in state not linked to trump crime crackdown wh say the redistricting war between texas and california is about to jolt the midterm politico asking eric were no longer invited to shared family holiday meal what should we do about upcoming wedding redistricting war poised to explode a california and texas make their move la consequential karen bass earns epic ratio over claim city recovery is fastest in state history the redistricting war between texas and california is about to jolt the midterm texas abbott promise quick signature of redistricting plan following overnight senate vote ghislaine maxwell absolves trump and everyone else in doj interview conservative activist slam cracker barrel a company left reeling after logo redesign south korea japan agree to boost tie a challenge mount kilmar abrego garcia released from ice custody after return from el salvador truck driver in crash at center of trump administration feud with newsom is denied bond when trying to explain low dem party polling look no further than awesome duo of newsom and swalwell immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say immigration boosted europe economy after pandemic ecbs lagarde say u seek to deport kilmar abrego garcia to uganda after he refused plea offer in his smuggling case trump look to chicago next in federal crackdown the wall street journal giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell giuffre family outraged over doj interview with ghislaine maxwell university of oregon concludes law review discriminated based on perceived national origin against israeli author trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress trump hail new texas electoral map aimed at keeping grip on congress how redistricting is done and why it could give party an edge in election how redistricting is done and why it could give party an edge in election democrat mock jd vance for having cardboard charisma a he push unpopular budget bill opinion it time for mayo pete buttigieg to find some seasoning what happened to ambition for bay restoration guest commentary kilmar abrego garcia threatened with deportation to uganda larimer county restaurant inspection made aug kilmar abrego garcia threatened with deportation to uganda kilmar abrego garcia threatened with deportation to uganda judge block trump from cutting funding from city and county including denver over sanctuary policy internet tax freedom act preempt new york imposition of tax fbi target john boltons home and office trump he not a smart guy but he could be a very unpatriotic guy inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal rachel bitecofer warns that bolton is just the start and trump will go after the rest of u inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal what we know about china and russia new strategic bomber inside the facility where ice is training recruit to take on trump deportation goal inside the facility where ice is training recruit to take on trump deportation goal zelenskyy say security guarantee for ukraine to be ready soon bill maher applauds gavin newsom for mocking donald trump i think it very funny floridarun alligator alcatraz violates u law aclu say russia announces support for venezuela to defend sovereignty amid growing military tension with the united state gianno caldwell mull senate bid a chicagoans are begging for change on crime woe trump threatens chicago with next national guard invasion cnn analyst pinpoint the weirdest part of ghislaine maxwell simply bizarre doj interview cnn analyst pinpoint the weirdest part of ghislaine maxwell simply bizarre doj interview the owl eye liberty and memory from epstein suicide to trump and clinton takeaway from ghislaine maxwell transcript how can israel engineer a famine in gaza in the st century what we learned from the ghislaine maxwell doj interview texas gov abbott say hell swiftly sign redistricting map after lawmaker approve them jeff bezos said he would have felt icky had he taken any more share of amazon i just didnt feel good smart money strategy what the pro buy when the crypto market crash radioactive shrimp update walmart store brand and other brand recalled european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff european postal service suspend shipment of package to u over tariff a winning powerball ticket ha been sold in western new york the sp hasnt yielded this little since the dotcom bubble here what investor can do the motley fool just ranked the biggest financial stock here why the no pick could be your best investment mezcal producer preserve traditional method a demand for liquor grows minute european postal service suspend shipment of package to u over tariff kpop demon hunter give netflix it first boxoffice win curry join the bank holiday sale bonanza with it epic deal event here are the best offer id buy self driving taxi may be coming to nyc a waymo win first av testing permit mashable rosen a leading law firm encourages fiserv inc investor to secure counsel before important rosen a leading law firm encourages fiserv inc investor to secure counsel before important rosen a leading law firm encourages fiserv inc investor to secure counsel before important rosen a leading law firm encourages fiserv inc investor to secure counsel before important rosen a leading law firm encourages fiserv inc investor to secure counsel before important deadline in security class action fi ice cream sold at walmarts across state recalled due to undeclared allergen here how a gamestop purchase turned into a bitcoin jackpot ice cream sold at walmarts across state recalled due to undeclared allergen fox business prediction lucid group sale will soar over the next year if this happens solar executive warn that trump attack on renewables will lead to power crunch that spike electricity price pueblo county home listing asked for le money in july see the current median price here prediction these trilliondollar artificial intelligence ai stock could strike a megadeal that wall street isnt ready for cold wallet cashback utility and presale pricing create a upside case while chainlink and shiba inu struggle maintenance compliance burden viability of hopi water treatment system ethereum in trouble xrp might breakout buyer turn to blockdag to earn referral reward acting a the executor of a will can be a very lucrative job the last word national guard troop to be force multiplier for ice homan little pepe crypto price prediction is lilpepe a good investment for longterm holder here how much you should aim to invest in the invesco qqq etf to get to million or more by retirement state audit question m in federal spending by moses lake school district blockchain stock worth watching august th owner scale back golden mile shopping center redevelopment rosen global investor counsel encourages easterly rocmuni high income municipal bond fund comerica bank lower stake in alphabet inc goog trump tap airbnb cofounder a st government design head to lead huge web overhaul trump tap airbnb cofounder a st government design head to lead huge web overhaul fox business offgrid living next new real estate trend a application for rural mortgage skyrocket rosen global investor counsel encourages altimmune inc investor to secure counsel before rosen global investor counsel encourages altimmune inc investor to secure counsel before rosen global investor counsel encourages altimmune inc investor to secure counsel before epstein accuser virginia giuffre wrote a memoir month after her death it coming out powell warning signal unemployment claim jump to highest in year cardano price outlook can ada reach trumprelated defi platform world liberty financial debut wlfi token on ethereum mainnet rosen global investor counsel encourages altimmune inc investor to secure counsel before important deadline in security class action alt the best meme coin presale stampede is loading whitelist labubull now or watch it moon without you backtoschool deal tellos unlimited plan get you cell service for per month your first month nexus gold cvenxs stock price up whats next mason resource cvellg stock price up here why mason resource cvellg trading up here what happened national guard troop to be force multiplier for ice homan freedom investment management inc purchase share of procter gamble company the pg ascent group llc raise stock holding in america</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>silver stabilizes above a mean reversion structure hold ford recall more than pickup truck over instrument display failure on the dashboard ford recall more than pickup truck over instrument display failure on the dashboard ford recall more than pickup truck over instrument display failure on the dashboard fashion model reckon with ai model and digital clone after controversial ad appears in vogue ai profit window is wide open here how to time it from swag to strategy why business are replacing cheap merch with thoughtful luxury gifting experience from swag to strategy why business are replacing cheap merch with thoughtful luxury gifting experience from swag to strategy why business are replacing cheap merch with thoughtful luxury gifting experience from swag to strategy why business are replacing cheap merch with thoughtful luxury gifting experience are workplace relationship the key to finding meaning on the job the ethical life podcast are workplace relationship the key to finding meaning on the job the ethical life podcast safer foundation to host open house at new employment service location in rock island are workplace relationship the key to finding meaning on the job the ethical life podcast the next x crypto to invest in a cardano ada and ripple xrp holder seek stronger bull run play are workplace relationship the key to finding meaning on the job the ethical life podcast xrp news today why investor are choosing this defi utility token over ripple clear creek isd trustee approve over k in capital project are workplace relationship the key to finding meaning on the job the ethical life podcast are workplace relationship the key to finding meaning on the job the ethical life podcast are workplace relationship the key to finding meaning on the job the ethical life podcast america bankruptcy wave ha surpassed the pandemicand it getting worse josh kosnicks five bridge answer whats next when the hustle fails highflying stock set for a pullback sp hit record high a investor await nvidia result reuters these analyst increase their forecast on ncino following betterthanexpected q earnings xrp bitcoin or eth here which coin user predict to perform best until trump critic inside fema put on indefinite leave after blasting cut in dissent letter up fintech share drop after strong q result what you need to know subsea awarded contract offshore turkiye rfk jr make good on promise to end covid vaccine mandate biontech tumble this economic sugar high wont last crfb warns touting analysis predicting longterm stagnation and billion of annual borrowing through the latest trump effort to control u capital expands to union station bytedance target billion valuation a revenue exceed meta sharp technology soar after insider buy and m solana treasury plan water wellness summit offer expert analysis recommendation for waterborne disease prevention the death of reaganomics trump break with longtime gop economic doctrine first commerce credit union donates for student scholarship buffalo diocese abuse settlement increase to million downtown san jose apartment complex land construction loan downtown san jose apartment complex land construction loan bank of montreal analyst boost their forecast after q result fargo agrees to jail rate increase after exhausting discussion building your organization next generation of leader no college degree here are job where can still earn figure no college degree here are job where can still earn figure mdot suspending construction lifting traffic restriction for labor day weekend how coolvu is empowering entrepreneur and protecting small business powell see the light in his final jackson hole talk my husband sold our house behind my back and kept every dime well now it my turn to cut him off uvalde cisd considers new law firm a trust in current agency falter following document issue johnson fistel pllp investigates claim on behalf of alto neuroscience inc longterm shareholder these analyst boost their forecast on echostar delta to pay million to resolve fuel dump lawsuit investigation alert elanco animal health incorporated driven brand holding hasbro and transmedics johnson fistel pllp investigates claim on behalf of investor kelowna councillor wonder if the city should stop density bonusing program kelowna arctic pablo coin raise m in presale one of the top meme coin to invest a dogecoin and shiba inu rally make cracker barrel a winner again trump celebrates logo reversal nprs all thing considered name scott detrow a new fulltime host johnson fistel pllp investigates constellation brand atkore domino pizza and fmc corporation on behalf of longterm shareholder innout primanti bros gone after one year on high street these analyst revise their forecast on okta after upbeat q earnings rbc city national bank is back on front foot ceo say nvidias upstart chinese rival cambricon just showed growth but dont get too excited trump is forcing the economy to bend to his will only one person can stop him the latest trump effort to control u capital expands to union station the latest trump effort to control u capital expands to union station the latest trump effort to control u capital expands to union station the latest trump effort to control u capital expands to union station another power company eyeing northwestern ontario city for solar farm guess investor alert by the former attorney general of louisiana kahn swick foti llc investigates adequacy of price and process in proposed sale of guess inc ge executive order open door to alternative asset in k key consideration for plan fiduciary im rooting for female founder comeback and for the end of branding woman from girlboss to tradwife and all the way down the best walmart labor day deal on kitchen bestseller university of phoenix leadership present at greater phoenix chamber foundation workforce summit university of phoenix leadership present at greater phoenix chamber foundation workforce summit the latest trump effort to control u capital expands to union station mongodb to rally around here are top analyst forecast for wednesday will credit card interest rate finally drop this september cross river and sightline team on gamingfocused debit card tom cotton target tax status of terroristsupporting youth movement vertical aerospace shortinterest collapse signal shifting market sentiment food and chemical unpacked epr you keeping up podcast unpacking the latest option trading trend in carvana decoding bank of america option activity whats the big picture oktas option a look at what the big money is thinking attention cio it is just one week away register now florida csuite executive invited to forecasting the future analyst projection for synopsys crowdstrike likely to report lower q earnings these most accurate analyst revise forecast ahead of earnings call analyst assess lineage cell therapeutic what you need to know analyst expectation for omega healthcare invtss future larkins investigation expands to indianapolis in now offering comprehensive investigative and tscm service what analyst rating have to say about compass let talk indianola mayor steve richardson analyst expectation for eli lillys future texas new proxy advisor disclosure law key detail for shareholder and company ahead of september pe ratio insight for bread finl hldgs analyst expectation for essex property trust future coach tory burch and more designer bag are up to off on amazon save up to on dyson dewalt anker adidas and more during ebays th anniversary sale maga loses it after minneapolis mayor emotional speech on shooting voter lose in redistricting game texas republican are wrong to start this tit for tat fight voter lose in redistricting game texas republican are wrong to start this tit for tat fight trump tell supreme court he shouldnt have to spend foreign aid approved by congress fda rescinds emergency use authorization for covid vaccine rfk jr fda rescinds emergency use authorization for covid vaccine rfk jr federal prosecutor fail to indict sandwich slinger exdoj employee on assault charge report gerrymandering is controversial but the alternative is worse fda rescinds emergency use authorization for covid vaccine rfk jr fda rescinds emergency use authorization for covid vaccine rfk jr attorney for jack smith respond to federal watchdog probe fulton county commissioner risk jail time for not appointing republican to election board dc mayor masked ice agent and outoftown national guard are ineffective axios lehigh valley police department shared driver comical excuse during speed enforcement detail ukraine will allow men to leave country exploring trend how immigration shape our region from cracker barrel to bud light trump weighs in on another corporate controversy un warns gaza famine expanding a aid group decry israeli siege riley push bill for rural hospital funding gop whip time to change senate confirmation rule gop whip time to change senate confirmation rule trouble finding tea global matcha shortage take toll on bay area business white nationalist agenda minority in front line of trump policy target minneapolis mayor jacob frey slammed for mocking prayer after the catholic school shooting gop whip time to change senate confirmation rule gop whip time to change senate confirmation rule gop whip time to change senate confirmation rule gop whip time to change senate confirmation rule johnson fistel pllp investigates claim on behalf of alto neuroscience inc longterm shareholder mixed report of russian force holding ground in dnipropetrovsk ice is suddenly showing up in california hospital worker want more guidance on what to do ice is suddenly showing up in california hospital worker want more guidance on what to do the not so dormant commerce clause watch congressional candidate debate ice other issue watch congressional candidate debate ice other issue congressional candidate in arizona debate ice other issue watch congressional candidate debate ice other issue watch congressional candidate debate ice other issue watch congressional candidate debate ice other issue watch congressional candidate debate ice other issue watch congressional candidate debate ice other issue protester to assemble on labor day magic johnson turned down a deal of a lifetime in boy did i make a mistake im still kicking myself offset vow to never get married again warns men against it too mary spencer youre not too young to make an estate plan commentary why is trump going after the smithsonian museum gov tony evers renews appeal for fema help following milwaukeearea flooding a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know executive order open door to alternative asset in k key consideration for plan fiduciary abrego garcia cannot be deported before october hearing judge say council in burnaby bc call for israel arm embargo metro vancouver south african politician criticized by trump is found guilty of hate speech u envoy cut lebanon trip short amid protest outrage over press comment trump say liberal donor george soros and son should be criminally charged bolivian court order the release of a prominent rightwing opposition leader fema worker put on leave after signing letter warning of trump overhaul of the agency how wes moore can stand up for the national guard guest commentary bengalmc air cushion catamaran aim to be the navy future ultraadaptable combat ship newton is removing italian flag color from street again russian force break into another region of ukraine with peace effort stuck green destry covington table drinking area vote again native american housing advocate urge congress to renew affordable housing law nyc mayor race eric adam label democratic socialist mamdani a communist echoing a frequent trump attack trump military invasion is cleaning up dcliterally denmark summons u envoy over suspected influence campaign in greenland debate over book page pit cultural concern against free access asking eric im a loyal person but my husband emotional affair ha me unable to trust him republican nominated to replace sen darin smith joseph kibler running for wyoming governor credit union deliver big return for community through cdfis new parkingmeter hour added for el cajon boulevard surrounding area top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show majority of voter oppose deploying national guard to dc quinnipiac university national poll find support drop for u military aid to israel a think israel is committing genocide in gaza quinnipiac university poll u federal judge rule wisconsin judge cannot claim immunity in immigration obstruction case jared kushner participates in gaza meeting at the white house source say watch labor leader give trump the business for hurting worker top florida official say alligator alcatraz will likely be empty within day email show morris a a wave of shooting roils minneapolis leave the national guard at home a deadly florida truck crash ha fueled an immigration fight here what to know a deadly florida truck crash ha fueled an immigration fight here what to know</t>
+          <t>silver stabilizes above a mean reversion structure hold ford recall more than pickup truck over instrument display failure on the dashboard ford recall more than pickup truck over instrument display failure on the dashboard ford recall more than pickup truck over instrument display failure on the dashboard fashion model reckon with ai model and digital clone after controversial ad appears in vogue ai profit window is wide open here how to time it from swag to strategy why business are replacing cheap merch with thoughtful luxury gifting experience from swag to strategy why business are replacing cheap merch with thoughtful luxury gifting experience from swag to strategy why business are replacing cheap merch with thoughtful luxury gifting experience from swag to strategy why business are replacing cheap merch with thoughtful luxury gifting experience are workplace relationship the key to finding meaning on the job the ethical life podcast are workplace relationship the key to finding meaning on the job the ethical life podcast safer foundation to host open house at new employment service location in rock island are workplace relationship the key to finding meaning on the job the ethical life podcast the next x crypto to invest in a cardano ada and ripple xrp holder seek stronger bull run play are workplace relationship the key to finding meaning on the job the ethical life podcast xrp news today why investor are choosing this defi utility token over ripple clear creek isd trustee approve over k in capital project are workplace relationship the key to finding meaning on the job the ethical life podcast are workplace relationship the key to finding meaning on the job the ethical life podcast are workplace relationship the key to finding meaning on the job the ethical life podcast america bankruptcy wave ha surpassed the pandemicand it getting worse josh kosnicks five bridge answer whats next when the hustle fails highflying stock set for a pullback sp hit record high a investor await nvidia result reuters these analyst increase their forecast on ncino following betterthanexpected q earnings xrp bitcoin or eth here which coin user predict to perform best until trump critic inside fema put on indefinite leave after blasting cut in dissent letter up fintech share drop after strong q result what you need to know subsea awarded contract offshore turkiye rfk jr make good on promise to end covid vaccine mandate biontech tumble this economic sugar high wont last crfb warns touting analysis predicting longterm stagnation and billion of annual borrowing through the latest trump effort to control u capital expands to union station bytedance target billion valuation a revenue exceed meta sharp technology soar after insider buy and m solana treasury plan water wellness summit offer expert analysis recommendation for waterborne disease prevention the death of reaganomics trump break with longtime gop economic doctrine first commerce credit union donates for student scholarship buffalo diocese abuse settlement increase to million downtown san jose apartment complex land construction loan downtown san jose apartment complex land construction loan bank of montreal analyst boost their forecast after q result fargo agrees to jail rate increase after exhausting discussion building your organization next generation of leader no college degree here are job where can still earn figure no college degree here are job where can still earn figure mdot suspending construction lifting traffic restriction for labor day weekend how coolvu is empowering entrepreneur and protecting small business powell see the light in his final jackson hole talk my husband sold our house behind my back and kept every dime well now it my turn to cut him off uvalde cisd considers new law firm a trust in current agency falter following document issue johnson fistel pllp investigates claim on behalf of alto neuroscience inc longterm shareholder these analyst boost their forecast on echostar delta to pay million to resolve fuel dump lawsuit investigation alert elanco animal health incorporated driven brand holding hasbro and transmedics johnson fistel pllp investigates claim on behalf of investor kelowna councillor wonder if the city should stop density bonusing program kelowna arctic pablo coin raise m in presale one of the top meme coin to invest a dogecoin and shiba inu rally make cracker barrel a winner again trump celebrates logo reversal nprs all thing considered name scott detrow a new fulltime host johnson fistel pllp investigates constellation brand atkore domino pizza and fmc corporation on behalf of longterm shareholder innout primanti bros gone after one year on high street these analyst revise their forecast on okta after upbeat q earnings rbc city national bank is back on front foot ceo say nvidias upstart chinese rival cambricon just showed growth but dont get too excited trump is forcing the economy to bend to his will only one person can stop him the latest trump effort to control u capital expands to union station the latest trump effort to control u capital expands to union station the latest trump effort to control u capital expands to union station the latest trump effort to control u capital expands to union station another power company eyeing northwestern ontario city for solar farm guess investor alert by the former attorney general of louisiana kahn swick foti llc investigates adequacy of price and process in proposed sale of guess inc ge executive order open door to alternative asset in k key consideration for plan fiduciary im rooting for female founder comeback and for the end of branding woman from girlboss to tradwife and all the way down the best walmart labor day deal on kitchen bestseller university of phoenix leadership present at greater phoenix chamber foundation workforce summit university of phoenix leadership present at greater phoenix chamber foundation workforce summit the latest trump effort to control u capital expands to union station mongodb to rally around here are top analyst forecast for wednesday will credit card interest rate finally drop this september cross river and sightline team on gamingfocused debit card tom cotton target tax status of terroristsupporting youth movement vertical aerospace shortinterest collapse signal shifting market sentiment food and chemical unpacked epr you keeping up podcast unpacking the latest option trading trend in carvana decoding bank of america option activity whats the big picture oktas option a look at what the big money is thinking attention cio it is just one week away register now florida csuite executive invited to forecasting the future analyst projection for synopsys crowdstrike likely to report lower q earnings these most accurate analyst revise forecast ahead of earnings call analyst ass lineage cell therapeutic what you need to know analyst expectation for omega healthcare invtss future larkins investigation expands to indianapolis in now offering comprehensive investigative and tscm service what analyst rating have to say about compass let talk indianola mayor steve richardson analyst expectation for eli lillys future texas new proxy advisor disclosure law key detail for shareholder and company ahead of september pe ratio insight for bread finl hldgs analyst expectation for essex property trust future coach tory burch and more designer bag are up to off on amazon save up to on dyson dewalt anker adidas and more during ebays th anniversary sale maga loses it after minneapolis mayor emotional speech on shooting voter lose in redistricting game texas republican are wrong to start this tit for tat fight voter lose in redistricting game texas republican are wrong to start this tit for tat fight trump tell supreme court he shouldnt have to spend foreign aid approved by congress fda rescinds emergency use authorization for covid vaccine rfk jr fda rescinds emergency use authorization for covid vaccine rfk jr federal prosecutor fail to indict sandwich slinger exdoj employee on assault charge report gerrymandering is controversial but the alternative is worse fda rescinds emergency use authorization for covid vaccine rfk jr fda rescinds emergency use authorization for covid vaccine rfk jr attorney for jack smith respond to federal watchdog probe fulton county commissioner risk jail time for not appointing republican to election board dc mayor masked ice agent and outoftown national guard are ineffective axios lehigh valley police department shared driver comical excuse during speed enforcement detail ukraine will allow men to leave country exploring trend how immigration shape our region from cracker barrel to bud light trump weighs in on another corporate controversy un warns gaza famine expanding a aid group decry israeli siege riley push bill for rural hospital funding gop whip time to change senate confirmation rule gop whip time to change senate confirmation rule trouble finding tea global matcha shortage take toll on bay area business white nationalist agenda minority in front line of trump policy target minneapolis mayor jacob frey slammed for mocking prayer after the catholic school shooting gop whip time to change senate confirmation rule gop whip time to change senate confirmation rule gop whip time to change senate confirmation rule gop whip time to change senate confirmation rule johnson fistel pllp investigates claim on behalf of alto neuroscience inc longterm shareholder mixed report of russian force holding ground in dnipropetrovsk ice is suddenly showing up in california hospital worker want more guidance on what to do ice is suddenly showing up in california hospital worker want more guidance on what to do the not so dormant commerce clause watch congressional candidate debate ice other issue watch congressional candidate debate ice other issue congressional candidate in arizona debate ice other issue watch congressional candidate debate ice other issue watch congressional candidate debate ice other issue watch congressional candidate debate ice other issue watch congressional candidate debate ice other issue watch congressional candidate debate ice other issue protester to assemble on labor day magic johnson turned down a deal of a lifetime in boy did i make a mistake im still kicking myself offset vow to never get married again warns men against it too mary spencer youre not too young to make an estate plan commentary why is trump going after the smithsonian museum gov tony evers renews appeal for fema help following milwaukeearea flooding a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know a deadly truck crash in florida ha fueled an immigration fight here what to know executive order open door to alternative asset in k key consideration for plan fiduciary abrego garcia cannot be deported before october hearing judge say council in burnaby bc call for israel arm embargo metro vancouver south african politician criticized by trump is found guilty of hate speech u envoy cut lebanon trip short amid protest outrage over press comment trump say liberal donor george soros and son should be criminally charged bolivian court order the release of a prominent rightwing opposition leader fema worker put on leave after signing letter warning of trump overhaul of the agency how wes moore can stand up for the national guard guest commentary bengalmc air cushion catamaran aim to be the navy future ultraadaptable combat ship newton is removing italian flag color from street again russian force break into another region of ukraine with peace effort stuck green destry covington table drinking area vote again native american housing advocate urge congress to renew affordable housing law nyc mayor race eric adam label democratic socialist mamdani a communist echoing a frequent trump attack trump military invasion is cleaning up dcliterally denmark summons u envoy over suspected influence campaign in greenland debate over book page pit cultural concern against free access asking eric im a loyal person but my husband emotional affair ha me unable to trust him republican nominated to replace sen darin smith joseph kibler running for wyoming governor credit union deliver big return for community through cdfis new parkingmeter hour added for el cajon boulevard surrounding area top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show top florida official say alligator alcatraz will likely be empty within day email show majority of voter oppose deploying national guard to dc quinnipiac university national poll find support drop for u military aid to israel a think israel is committing genocide in gaza quinnipiac university poll u federal judge rule wisconsin judge cannot claim immunity in immigration obstruction case jared kushner participates in gaza meeting at the white house source say watch labor leader give trump the business for hurting worker top florida official say alligator alcatraz will likely be empty within day email show morris a a wave of shooting roils minneapolis leave the national guard at home a deadly florida truck crash ha fueled an immigration fight here what to know a deadly florida truck crash ha fueled an immigration fight here what to know</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>judge block kari lake tasked to dismantle voa from firing it director annunciation mass shooting what we know about the shooter motive stock add a bit to their record on wall street flyw class action reminder flyw investor with large loss should contact robbins llp for information about the lead plaintiff deadline in the flywire corporation class action lawsuit atlas energy report second quarter financial result shareholder notice faruqi faruqi llp investigates claim on behalf of investor of altimmune ehc investor news if you have suffered loss in encompass health corporation nyse ehc you are encouraged to contact the rosen law firm about your right coinbase to monetize bitcointoethereum rotation through trading volume cfo say intel took trump deal to remove uncertainty around chip act billion los gatos property sale twobedroom home sell for million los gatos property sale twobedroom home sell for million raising cane to open more restaurant in september how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained fort smith weighs m in water upgrade a demand grows market expert say ozak ai might outperform ethereum in next bull run food hub planned across treaty territory to combat food insecurity xrp news today analyst warns dont sell xrp yet lawsuit win etf catalyst may lift price california face high pump price a phillips shuts la refinery the federal government is taking over dc union station what doe that mean the federal government is taking over dc union station what doe that mean u put official gdp data on nine blockchains in historic trumpera crypto push is ada price mirroring the breakout pattern a holder look for the next x bet big on remittix missing yearold boy with autism killed by alligator in new orleans police finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service hormel share face worst day on record a pork and other cost surge gbank financial holding inc is pleased to share the press release of boltbetz nike put finishing touch on a corporate overhaul more layoff ahead taco bell reconsiders voice ai after seeing mixed result tesla sale plunge again in europe a anger at musk keep buyer away for th month in a row yahoo finance northwood plaza owner defends work at former great eastern council want action gbank financial holding inc is pleased to share the press release of boltbetz will a reverse mortgage impact your social security or medicare benefit taiwan prosecutor charge people for allegedly stealing tsmc trade secret consumer watchdog public interest group to legislator dont let newsom sell out real utility rate reform in eleventh hour deal for utilitybacked western grid proposal and wildfire fund retail roundup key winner and loser after q earnings gbank financial holding inc is pleased to share the press release of boltbetz guardian officially release million veteran after disappointing season small parcel in limbo a trump move to end u tariff exemption small parcel in limbo a trump move to end u tariff exemption small parcel in limbo a trump move to end u tariff exemption small parcel in limbo a trump move to end u tariff exemption small parcel in limbo a trump move to end u tariff exemption small parcel in limbo a trump move to end u tariff exemption beef and nut price have surged and thats driving hormels stock to it biggest drop ever fresno council to vote on m plan for west fresno affordable housing jcpenneys closing down sale spread to two more location after shutdown continue major airline add route with low flight cost challenging a top rival meta is racing the clock to launch it newest llama ai model this year business insider reykjavik energy green bond auction result fed cook an unintentional clerical error may have been behind the mortgage dispute ap sport summarybrief at pm edt earthwise advertising investor awareness campaign bluerock total income real estate fund shareholder receive iss and glass lewis recommendation to support key proposal in connection with listing of the fund on the nyse a sea war brew off gambia a desperate local fisherman attack foreign vessel and each other labor day deal alert heydude is offering an extra off top style city pivot after apex rescinds rosecrans airport lease agreement best ai chatbots and key statistic of stockton mark oneyear anniversary of staart app with conference powerball player win in texas where wa the lucky ticket sold florida taxpayer may lose m on empty alligator alcatraz a judge order shutdown florida taxpayer may lose m on empty alligator alcatraz a judge order shutdown florida taxpayer may lose m on empty alligator alcatraz a judge order shutdown the probability machine trump ha fired a democrat on a federal railroad board he the latest to refuse to leave his post politico who are the most valuable nfl team cowboy b top forbes list for instacart offer indie grocer ecommerce tool with mdi partnership naples set tax rate at postal service across the world to suspend u delivery after trump end tariff exemption casco set tax rate at credo stock notch record high ahead of earnings report grocery chain to close maryland location campaign finance board again denies matching fund to mayor adam seager marine acquires rk marina on rushford lake u economy grew percent in q beating prior estimate denim trend boost abercrombie a outlook stock climb treasury secretary bessent capital market are roaring back powerball jackpot nears billion ahead of saturday drawing trump pick for un aviation office ha long history donating to dems nikki haley nyseg rge to upgrade high voltage line substation across ny state how michael polk growth culture drove performance at newell brand and beyond trump look to fire transportation regulator ahead of rail merger a closer look at enphase energy option market dynamic stonepeak buy fort worth logistics property freeland to host history walk and cemetery tour for th anniversary rwanda say deportee arrived from the u in august under agreement with washington ap business summarybrief at pm edt cdc crisis triggered by upcoming vaccine meeting leading to director firing former yankee mark teixeira running for congress a republican apparently anyone can be an immigration judge in trump america white house confirms trump fired cdc director after she refused to resign woman at center of viral rochester video say she moved intends to fight charge sunday voting choice given to county by state board trump renews citizenship requirement waived since noem hit back at fema critic reveals vision for disaster relief agency the federal government is taking over dc union station what doe that mean npr former golden triangle development leader conduct would harm every member of this community xi put axis of u enemy on parade with putin kim in beijing former mlb star mark teixeira announces run for texas congressional seat trump administration asks military base near chicago for support on immigration operation whatever happened to the woman in the no sex for fish group whatever happened to the woman in the no sex for fish group minneapolis mayor we need a statewide and a federal ban on assault weapon cdc director arrives at office to find dead deer with fired carved into it what to know after the u deports more migrant to africa the latest trump administration asks military base near chicago for support on immigration gov jared polis order million in spending cut sweep state cash account to help close budget gap gov jared polis order million in spending cut sweep state cash account to help close budget gap gov jared polis order million in spending cut sweep state cash account to help close budget gap gov jared polis order million in spending cut sweep state cash account to help close budget gap gov jared polis order million in spending cut sweep state cash account to help close budget gap gov jared polis order million in spending cut sweep state cash account to help close budget gap at least migrant detained by ice in san francisco a arrest soar iran is facing a return of un sanction what happens now immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started exclusive gop smell blood in water over defeated dem exsens vulnerability karoline leavitt take jen psaki to task over her attack on prayer following tragic catholic school shooting fresno council to vote on m plan for west fresno affordable housing governor pay tribute to buttearea veteran still serving veteran closure of florida alligator alcatraz immigration detention center can proceed judge say mass sen warren launch probe over shuttering of public corruption unit at justice dept fbi leavitt slam insensitive psaki on prayer comment after minnesota shooting montgomery county ready to combat mosquito with targeted spraying in windlestrae park amid west nile concern opinion gov newsom playing for a tie in national redistricting battle leavitt slam insensitive psaki on prayer comment after minnesota shooting leavitt slam insensitive psaki on prayer comment after minnesota shooting leavitt slam insensitive psaki on prayer comment after minnesota shooting congress probe wikipedia over antiisrael prokremlin content manipulation trump administration asks military base near chicago for support on immigration operation trump administration asks military base near chicago for support on immigration operation trump administration asks military base near chicago for support on immigration operation trump administration asks military base near chicago for support on immigration operation leavitt slam insensitive psaki on prayer comment after minnesota shooting fed lisa cook sue trump over move to fire her is it ever legal to pas a school bus in new jersey u to sell ukraine extendedrange missile resident have a chance to weigh in on city chicken sept texas governor greg abbott revise special legislative session agenda to enhance law enforcement privacy election integrity election commission panel call for a shakeup in how hawaii vote ecuadorian man arrested in maine sue immigration official alleging unlawful detention deadeyed travis kelce nod at bow tie option for cat ring bearer trump ha fired a democrat on a federal railroad board he the latest to refuse to leave his post trump federal takeover of dc could do irreparable damage to policecommunity relation rfk jr say cdc must deliver on trump agenda after white house fire director flagging flag burner again wife of greencard holder detained by ice speaks outlots of tear shenandoah to rework park master plan following resident pushback watchdog group sue for record on spying targeting trump associate michael caputo tong warns of recruitment scam targeting ct job seeker white house is not happy with view cohost for her comment on latino trumpers campaign finance board again denies matching fund to mayor adam ap business summarybrief at pm edt hud secretary pursues paradigm shift in administration approach to homelessness hud secretary pursues paradigm shift in administration approach to homelessness hud secretary pursues paradigm shift in administration approach to homelessness hud secretary pursues paradigm shift in administration approach to homelessness hud secretary pursues paradigm shift in administration approach to homelessness hud secretary pursues paradigm shift in administration approach to homelessness hud secretary pursues paradigm shift in administration approach to homelessness schumer jeffries call on gop leader to meet to avoid government shutdown bondi patel to testify before congress amid epstein fallout bondi patel to testify before congress amid epstein fallout european power hit iran with pre sanction a pressure for nuclear negotiation hoosier gop legislative leader break redistricting silence no business a usual public rally monday at shorey park judge frank caprios death leaf mourner remembering his compassion that drew many online fan montgomery county executive celebrates new affordable housing milestone in montgomery village uno study offer firstever look into labor trafficking in nebraska lt governor david wasinger launch missouri state employee charitable campaign in jefferson city trump unprecedented firing of fed governor lisa cook raise untested question</t>
+          <t>judge block kari lake tasked to dismantle voa from firing it director annunciation mass shooting what we know about the shooter motive stock add a bit to their record on wall street flyw class action reminder flyw investor with large loss should contact robbins llp for information about the lead plaintiff deadline in the flywire corporation class action lawsuit atlas energy report second quarter financial result shareholder notice faruqi faruqi llp investigates claim on behalf of investor of altimmune ehc investor news if you have suffered loss in encompass health corporation nyse ehc you are encouraged to contact the rosen law firm about your right coinbase to monetize bitcointoethereum rotation through trading volume cfo say intel took trump deal to remove uncertainty around chip act billion los gatos property sale twobedroom home sell for million los gatos property sale twobedroom home sell for million raising cane to open more restaurant in september how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained how global ecommerce brand can recover u import tariff duty drawback explained fort smith weighs m in water upgrade a demand grows market expert say ozak ai might outperform ethereum in next bull run food hub planned across treaty territory to combat food insecurity xrp news today analyst warns dont sell xrp yet lawsuit win etf catalyst may lift price california face high pump price a phillips shuts la refinery the federal government is taking over dc union station what doe that mean the federal government is taking over dc union station what doe that mean u put official gdp data on nine blockchains in historic trumpera crypto push is ada price mirroring the breakout pattern a holder look for the next x bet big on remittix missing yearold boy with autism killed by alligator in new orleans police finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service finturf and energuy launch incentive program contractor earn for every financed project using energuy service hormel share face worst day on record a pork and other cost surge gbank financial holding inc is pleased to share the press release of boltbetz nike put finishing touch on a corporate overhaul more layoff ahead taco bell reconsiders voice ai after seeing mixed result tesla sale plunge again in europe a anger at musk keep buyer away for th month in a row yahoo finance northwood plaza owner defends work at former great eastern council want action gbank financial holding inc is pleased to share the press release of boltbetz will a reverse mortgage impact your social security or medicare benefit taiwan prosecutor charge people for allegedly stealing tsmc trade secret consumer watchdog public interest group to legislator dont let newsom sell out real utility rate reform in eleventh hour deal for utilitybacked western grid proposal and wildfire fund retail roundup key winner and loser after q earnings gbank financial holding inc is pleased to share the press release of boltbetz guardian officially release million veteran after disappointing season small parcel in limbo a trump move to end u tariff exemption small parcel in limbo a trump move to end u tariff exemption small parcel in limbo a trump move to end u tariff exemption small parcel in limbo a trump move to end u tariff exemption small parcel in limbo a trump move to end u tariff exemption small parcel in limbo a trump move to end u tariff exemption beef and nut price have surged and thats driving hormels stock to it biggest drop ever fresno council to vote on m plan for west fresno affordable housing jcpenneys closing down sale spread to two more location after shutdown continue major airline add route with low flight cost challenging a top rival meta is racing the clock to launch it newest llama ai model this year business insider reykjavik energy green bond auction result fed cook an unintentional clerical error may have been behind the mortgage dispute ap sport summarybrief at pm edt earthwise advertising investor awareness campaign bluerock total income real estate fund shareholder receive i and glass lewis recommendation to support key proposal in connection with listing of the fund on the nyse a sea war brew off gambia a desperate local fisherman attack foreign vessel and each other labor day deal alert heydude is offering an extra off top style city pivot after apex rescinds rosecrans airport lease agreement best ai chatbots and key statistic of stockton mark oneyear anniversary of staart app with conference powerball player win in texas where wa the lucky ticket sold florida taxpayer may lose m on empty alligator alcatraz a judge order shutdown florida taxpayer may lose m on empty alligator alcatraz a judge order shutdown florida taxpayer may lose m on empty alligator alcatraz a judge order shutdown the probability machine trump ha fired a democrat on a federal railroad board he the latest to refuse to leave his post politico who are the most valuable nfl team cowboy b top forbes list for instacart offer indie grocer ecommerce tool with mdi partnership naples set tax rate at postal service across the world to suspend u delivery after trump end tariff exemption casco set tax rate at credo stock notch record high ahead of earnings report grocery chain to close maryland location campaign finance board again denies matching fund to mayor adam seager marine acquires rk marina on rushford lake u economy grew percent in q beating prior estimate denim trend boost abercrombie a outlook stock climb treasury secretary bessent capital market are roaring back powerball jackpot nears billion ahead of saturday drawing trump pick for un aviation office ha long history donating to dems nikki haley nyseg rge to upgrade high voltage line substation across ny state how michael polk growth culture drove performance at newell brand and beyond trump look to fire transportation regulator ahead of rail merger a closer look at enphase energy option market dynamic stonepeak buy fort worth logistics property freeland to host history walk and cemetery tour for th anniversary rwanda say deportee arrived from the u in august under agreement with washington ap business summarybrief at pm edt cdc crisis triggered by upcoming vaccine meeting leading to director firing former yankee mark teixeira running for congress a republican apparently anyone can be an immigration judge in trump america white house confirms trump fired cdc director after she refused to resign woman at center of viral rochester video say she moved intends to fight charge sunday voting choice given to county by state board trump renews citizenship requirement waived since noem hit back at fema critic reveals vision for disaster relief agency the federal government is taking over dc union station what doe that mean npr former golden triangle development leader conduct would harm every member of this community xi put axis of u enemy on parade with putin kim in beijing former mlb star mark teixeira announces run for texas congressional seat trump administration asks military base near chicago for support on immigration operation whatever happened to the woman in the no sex for fish group whatever happened to the woman in the no sex for fish group minneapolis mayor we need a statewide and a federal ban on assault weapon cdc director arrives at office to find dead deer with fired carved into it what to know after the u deports more migrant to africa the latest trump administration asks military base near chicago for support on immigration gov jared polis order million in spending cut sweep state cash account to help close budget gap gov jared polis order million in spending cut sweep state cash account to help close budget gap gov jared polis order million in spending cut sweep state cash account to help close budget gap gov jared polis order million in spending cut sweep state cash account to help close budget gap gov jared polis order million in spending cut sweep state cash account to help close budget gap gov jared polis order million in spending cut sweep state cash account to help close budget gap at least migrant detained by ice in san francisco a arrest soar iran is facing a return of un sanction what happens now immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started immigration agent signed up to recruit at a california university then the protest started exclusive gop smell blood in water over defeated dem exsens vulnerability karoline leavitt take jen psaki to task over her attack on prayer following tragic catholic school shooting fresno council to vote on m plan for west fresno affordable housing governor pay tribute to buttearea veteran still serving veteran closure of florida alligator alcatraz immigration detention center can proceed judge say mass sen warren launch probe over shuttering of public corruption unit at justice dept fbi leavitt slam insensitive psaki on prayer comment after minnesota shooting montgomery county ready to combat mosquito with targeted spraying in windlestrae park amid west nile concern opinion gov newsom playing for a tie in national redistricting battle leavitt slam insensitive psaki on prayer comment after minnesota shooting leavitt slam insensitive psaki on prayer comment after minnesota shooting leavitt slam insensitive psaki on prayer comment after minnesota shooting congress probe wikipedia over antiisrael prokremlin content manipulation trump administration asks military base near chicago for support on immigration operation trump administration asks military base near chicago for support on immigration operation trump administration asks military base near chicago for support on immigration operation trump administration asks military base near chicago for support on immigration operation leavitt slam insensitive psaki on prayer comment after minnesota shooting fed lisa cook sue trump over move to fire her is it ever legal to pas a school bus in new jersey u to sell ukraine extendedrange missile resident have a chance to weigh in on city chicken sept texas governor greg abbott revise special legislative session agenda to enhance law enforcement privacy election integrity election commission panel call for a shakeup in how hawaii vote ecuadorian man arrested in maine sue immigration official alleging unlawful detention deadeyed travis kelce nod at bow tie option for cat ring bearer trump ha fired a democrat on a federal railroad board he the latest to refuse to leave his post trump federal takeover of dc could do irreparable damage to policecommunity relation rfk jr say cdc must deliver on trump agenda after white house fire director flagging flag burner again wife of greencard holder detained by ice speaks outlots of tear shenandoah to rework park master plan following resident pushback watchdog group sue for record on spying targeting trump associate michael caputo tong warns of recruitment scam targeting ct job seeker white house is not happy with view cohost for her comment on latino trumpers campaign finance board again denies matching fund to mayor adam ap business summarybrief at pm edt hud secretary pursues paradigm shift in administration approach to homelessness hud secretary pursues paradigm shift in administration approach to homelessness hud secretary pursues paradigm shift in administration approach to homelessness hud secretary pursues paradigm shift in administration approach to homelessness hud secretary pursues paradigm shift in administration approach to homelessness hud secretary pursues paradigm shift in administration approach to homelessness hud secretary pursues paradigm shift in administration approach to homelessness schumer jeffries call on gop leader to meet to avoid government shutdown bondi patel to testify before congress amid epstein fallout bondi patel to testify before congress amid epstein fallout european power hit iran with pre sanction a pressure for nuclear negotiation hoosier gop legislative leader break redistricting silence no business a usual public rally monday at shorey park judge frank caprios death leaf mourner remembering his compassion that drew many online fan montgomery county executive celebrates new affordable housing milestone in montgomery village uno study offer firstever look into labor trafficking in nebraska lt governor david wasinger launch missouri state employee charitable campaign in jefferson city trump unprecedented firing of fed governor lisa cook raise untested question</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>hows the market doe ownership go past the topsoil fresh stock on jim cramers radar juneteenth organizer get funding to repair modernize building panda express owns other restaurant chain do you know which one fed rate cut still on track no firework after nvidia earnings federal government post billion deficit from april to june canada whats going on with broadcom stock friday oakland unified school district looking to shed nearly million from budget is it a bot or not ticketings next big legal fight could reshape the resale industry a model for understanding with edward kaplan smlr investor have opportunity to lead semler scientific inc security fraud lawsuit first filed by the rosen law firm rock tech lithium announces offering of up to million the persistent pitfall of taxpayer funded campaign berkshire hillsbrookline merger nears completion retailer warn trump tariff will trigger consumer price explosion who will he blame boing boing nvidia ceo say ai will actually make u busier in the future gizmodo is amazon falling behind in the cloud computing battle brutally honest way to finance your startup dmv may owe you s and have no obligation to let you know wa being held in just a single case qgold announces financing to complete acquisition of quartz mountain gold project in oregon usa and advance mine centre camp in ontario canada qgold announces financing to complete acquisition of quartz mountain gold project in oregon usa and advance mine centre camp in ontario canada should the federal reserve cut rate next month should the federal reserve cut rate next month hope gas responds to criticism in it pipeline program ratehike case raising cane to open ann arbor location september th the company second in metro detroit trump administration kill wasteful funding for humboldt bay offshore wind project sunblock charcoal and powerball holiday weekend lottery drawing worth billion sunblock charcoal and powerball holiday weekend lottery drawing worth billion sunblock charcoal and powerball holiday weekend lottery drawing worth billion sunblock charcoal and powerball holiday weekend lottery drawing worth billion ardot seeking public comment on proposed disadvantaged business enterprise goal for why you should think twice before buying private equity in your k nasb financial inc declares cash dividend on common stock sunblock charcoal and powerball holiday weekend lottery drawing worth billion ap news ulta beauty delivers strong quarter investor brush off the glow thought i wa going to die tunisian singer detained for week fight deportation while trying to finish music small business joint venture win coast guard cyber contract dupont to sell kevlar business for billion the manufacturer life insurance company grows position in tesla inc tsla stock market news today market slide a chip stock weigh spsp complete index seeking alpha layoff hit international paper jb hunt hormel and more the orange peel first year put asheville on the map now staffer hope to buy it cv walgreens now require prescription for covid vaccine in colorado the denver post in hong kong eric trump lauds growing influence of crypto the new york time forecasting the future analyst projection for oneok what the option market tell u about mastercard lazr investor have opportunity to lead luminar technology inc security fraud lawsuit sword group availability of the h financial report sword group h report of the liquidity agreement contracted with oddo bhf procter gamble unusual option activity forecasting the future analyst projection for dt midstream dows option frenzy what you need to know pce inflation flat but core sticky implication for fed september meeting analyst expectation for targa resourcess future breaking down karooooo analyst share their view segg medium unveils nextgeneration corporate website showcasing completion of turnaround and launch of growth phase a glimpse into the expert outlook on cheniere energy through analyst is rivian automotive gaining or losing market support peering into extreme networkss recent short interest let talk indianola kwik star ribbon cutting expert outlook snapon through the eye of analyst is flex gaining or losing market support pe ratio insight for bank of nova scotia let talk knoxville planning and zoning administrator nathan parch part two segg medium unveils nextgeneration corporate website showcasing completion of turnaround and launch of growth phase u government publishes gdp data on bitcoin ethereum blockchains home price in okanagan and kamloops area may be levelling housewise chainlink link price movement face hurdle litecoin target rally while cold wallet hold roi edge major discount on outdoor furniture costway dining set off at target bytedance hit b valuation a q revenue surge to b energy exchange electronx earns cftc designated market and clearing approval how senior can borrow home equity without refinancing now crypto news today coinshares profit jump avalanche transaction rise gumi add xrp here why serve robotics surged this week savvy shopper save over k in year by extreme couponing she scored k of jcpenney cookware for just backtoschool sale tax holiday the edmund fitzgerald and a state microbe theyre among state bill in august should you buy lucid stock ahead of it for reverse stock split bitcoin drop below a xrp slide below and eth dogecoin wobble shopping labor day furniture sale tip to bargain for the best price ollies bargain earnings suggest analyst underestimate longterm potential no ruling friday on trump attempt to fire fed official the credit race closing the perception gap to win welcome to the new made in china era and it look a lot different dell struggle to protect margin a supply chain cost mount cracker barrel ditched it new logo but it also got rid of something else labubu doll and affordable latte why chinese brand are betting big on the u business insider mycarrier portal and carrier assure integrate to make carrier vetting easier cracker barrel is still deep in dei despite the return of uncle herschel former trans mountain ceo to head major project office canada cracker barrel did more than just ditch it logo after maga meltdown the daily beast cracker barrel new logo wa pitiful one of chain original executive say anthony brown maryland legal victory show prudent use of resource reader commentary atlanta becomes largest u metro without a printed daily newspaper a journalconstitution go digital techstock skid sends nasdaq sharply lower live stockmarket update understanding the benefit and risk of ai agent university of northern iowa to open finance and real estate analytics lab for business eli lilly is proof that wall street star dont have to be tech titan trump fire democratic member from transportation board just before it considers the largest railroad merger in history marvell sink a weak data center outlook stokes custom ai chip worry reuters mount logan capital inc shareholder approve previously announced business combination with degree capital corp court block trump effort to end protected status for venezuelan mamdani team with sharpton to threaten wall street upcoming upgrade to holocaust museum exhibit spark some staff concern source trump planning immigration crackdown in chicago next week dhs source say gov gretchen whitmer call special election for state senate seat that could split michigan chamber gov gretchen whitmer call special election for state senate seat that could split michigan chamber gov gretchen whitmer call special election for state senate seat that could split michigan chamber gov gretchen whitmer call special election for state senate seat that could split michigan chamber gov gretchen whitmer call special election for state senate seat that could split michigan chamber gov gretchen whitmer call special election for state senate seat that could split michigan chamber migrant defer their american dream to seek asylum in mexico bonus editorial cartoon for aug alabama town first black mayor reelected after being locked out of office lawyer who led karen read defense one step closer to joining team for civil suit trump move to cut bn in foreign aid already approved by congress rubio revoke visa for palestinian official denying address at un meeting alabama town first black mayor reelected year after he say white resident locked him out of office cbs news can tv help prepare for invasion jd vance say there thing dems should learn from trump and critic cant believe he serious jd vance say there thing dems should learn from trump and critic cant believe he serious abrego garcia asks for gag order on bondi noem meet bill pulte the trump housing official at the center of the latest fed controversy abrego garcia asks for gag order on bondi noem judge weighs request to block trump firing of fed governor lisa cook abrego garcia asks for gag order on bondi noem contract talk fail between alberta government and teacher possible strike loom alberta republican joni ernst will not seek reelection source say abrego garcia asks for gag order on bondi noem trump yank kamala harris bidenextended taxpayerfunded secret service protection before book tour susan estrich the epitome of dumbness judge hears argument on lisa cook attempted firing by trump administration psc answer preston county commission objection to marl project corruption allegation impact argentina president mileis popularity trump block b in foreign aid congress okd using maneuver last seen nearly year ago trump block b in foreign aid congress okd using maneuver last seen nearly year ago mackinac island police chief to resign citing ongoing friction with city council a lament for the shrinking middle class reader commentary dear annie unfaithful fiancee tell me to stop living in the past appeal court block trump administration from ending legal protection for venezuelan appeal court block trump administration from ending legal protection for venezuelan appeal court block trump administration from ending legal protection for venezuelan a trumpbrokered peace deal in the south caucasus is hopeful but incomplete many state employeefriendly labor law take effect a nlrb remains quorumless benton county to display in god we trust in all public building by oct everyone on x point and laugh at dingus gungrabber who share pic of bullet scattered on his street democrat some republican cry outrage over trump use of rare tactic to withhold approved foreign aid funding lori falce year of thought and prayer appeal court say uk asylumseekers can stay at hotel dc federal judge to weigh order blocking fed gov lisa cook firing ahead of interest rate meeting let talk knoxville planning and zoning administrator nathan parch part two donald trump war on culture is not a sideshow japan india to deepen security economic tie amid u tariff ai is ummasking ice officer can washington do anything about it politico public trust in election increase with clear fact sen ernst of iowa is expected to announce next month that she wont run for reelection in u revoke visa of palestinian official ahead of un general assembly fox news star call out trump ally over apparent hypocrisy this is the same thing sen ernst of iowa is expected to announce next month that she wont run for reelection in ap news fox news star call out trump ally over apparent hypocrisy this is the same thing free speech unmuted president trump executive order on flag desecration it a joke san jose mayor slam california legislature over lack of prop funding ransomware attack targeting pa attorney general lead to case delay susan collins rip trump unlawful effort to cancel billion in foreign aid susan collins rip trump unlawful effort to cancel billion in foreign aid susan collins rip trump unlawful effort to cancel billion in foreign aid what to know a texas bill let resident sue outofstate abortion pill provider what to know a texas bill let resident sue outofstate abortion pill provider what to know a texas bill let resident sue outofstate abortion pill provider what to know a texas bill let resident sue outofstate abortion pill provider chicago is in the trump administration sight for it next immigration crackdown chicago is in the trump administration sight for it next immigration crackdown trump admin plan immigration enforcement surge in boston politico a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows kilmar abrego garcia asks for gag order against pam bondi kristi noem kilmar abrego garcia asks for gag order against pam bondi kristi noem texas gov greg abbott sign new congressional redistricting map president trump requested kimball shinkoskey explain the law talk for trump riviera in gaza persist a israel push deeper into gaza city france germany vow to up pressure on ogre putin bankruptcy for north dakota and western minnesota published aug trump administration to cut plus job at voice of america best business line of credit in flexible small business funding option for growth and emergency adhesive dowel veneer the industrial choice shaping mass timber verizon down how to fix so modeonly issue in phone amid outage hindustan time hindustan time what would the fed do in a tie vote it not clear and the bank of england had to break a deadlock this month can you use milwaukee battery on harbor freight tool ulster county rail trail study to be contracted to new paltzbased consulting firm tim walz admits vp bid might have hurt him with voter in home state judge delay septum rate increase additional service cut gas price go up in killeen area per gallon at one place kari lake lay off hundred at voa parent agency amid legal battle doesnt surprise memark cuban explains why high school senior care more about making money than any generation in year cnc deadline alert rosen a longstanding law firm encourages centene corporation investor to secure counsel before important september deadline in security class action cnc bet bonus code orl bet on oregon v montana state get in bonus bet bemidji chamber ambassador welcome thrivent financial advisor letter illegal dumping and time to support wastetoenergy how the sound of name can bias hiring decision writer bloc a push for change in the u electoral college give u hope for future climate action strengthening italian finance a new era through takeover consolidation u trading partner dazed and confused after tariff court loss delaware ag other state secure americorps funding in winning suit solana etf buzz fade a investor shift to magacoin finance a rising star best soundbars with wireless rear speaker in cryptos under that could make you x richer mirroring pepe coin pepe run best small business loan option in how owner qualify compare program and secure fast funding with rok financial what happens to trump tariff now that a federal appeal court ha knocked them down cracker barrel or waffle house the south most heated food debate return amid logo saga ai cant install an hvac system why gen z is flocking to job in the trade navigating client conundrum california payday loan online same day no credit check bad credit guaranteed approval radcred launch payday loan platform for immediate financial relief for california borrower usa kari lake lay off more than staff at voice of america parent agency the washington post amazon is selling a laptop for thats nice and responsive how to check for a lien on a car before you buy how an appeal court ruling on trump tariff could upend the bond market barrons how an appeal court ruling on trump tariff could upend the bond market how to check for a lien on a car before you buy sameday business loan in fast approval for owner facing urgent cash flow need how to check for a lien on a car before you buy madison county official think wind farm could impact public safety your money way the new tax bill could impact your wallet ultimate plantbased beet burger mowest to reveal library renovation cuba energy crisis deepens a blackout grip the nation best crypto to invest in why blockdag rtx hyper and snort are gaining attention how europe is redrawing it energy map rosen global investor counsel encourages easterly rocmuni high income municipal bond fund cryptos under to accumulate now ozak ai xdc cro trx and vechain carol saline dy journalist with a story to tell about her dying powerball jackpot rise to billion sixthlargest ever sunblock charcoal and powerball holiday weekend lottery jackpot worth billion is up for grab larimer county restaurant inspection made aug china xi offer backing for myanmar sco membership bid wamco deadline notice rosen trusted investor counsel encourages western asset management company llc mutual fund investor with loss in excess of k to secure counsel before important september deadline in security class action merz promise debt relief for municipality ahead of electoral test burlington store nyseburl announces quarterly earnings result beat estimate by eps u trading partner dazed and confused after tariff court loss bloombergcom u trading partner dazed and confused after tariff court loss shopper can get electronics clothes and school supply worth up to taxfree a u state exemption final hour spirit airline bankruptcy tee up painful cut in survival bid do novelty menu like taco bell yk make investor money southwest airline begin flying first plane with secondary cockpit barrier reuters stock retail wa discussing this week and how they performed open bull mdb nvda baba channel rewind growth spark conflict video vault top wireless printer under r in paige thomason caramel pecan turtle brownie recipe dogecoin price prediction doge alternative for x gain this bull cycle billion powerball jackpot is up for grab saturday here how to play austin americanstatesman baird financial group inc acquires share of qualcomm incorporated qcom best water stock to watch now august th walmart inc wmt share purchased by titleist asset management llc deadline approach for under forty nomination eu to work on using frozen russian asset to aid ukraine after war white house to release m in americorps funding after maryland lawsuit white house to release m in americorps funding after maryland lawsuit groundbreaking of home housing cooperative in upper hammonds plain commentary lawmaker could trim electric bill baird financial group inc acquires share of ishares core sp etf ivv kodai capital management lp invests in honeywell international inc hon haberman call tariff ruling a big blow to trump agenda orange county restaurant shut down by health inspector aug costcos controversial policy change officially take effect costcos controversial policy change officially take effect mcdonalds corporation mcd share sold by baird financial group inc warren buffett warns not to invest in terrible industry because it a rewarding a struggling in quicksand micron boeing lead five stock near buy point yearold retail chain closed dozen of store s at risk in order to become the you must do what the other wont billionaire grant cardone say hard work defines success a court ha ruled most of trump tariff illegal here whats next tesla lawyer ask judge to throw out million verdict saying mention of elon musk misled the jury tesla lawyer ask judge to throw out million verdict saying mention of elon musk misled the jury fortune promising value stock to keep an eye on august th adam thielen take pay cut with viking excited to be back home insight wealth partner llc make new investment in palantir technology inc pltr insight wealth partner llc ha holding in jpmorgan chase co jpm deeply affordable halawa rental tower nearly full best altcoins to buy this week ethereum xrp and magacoin finance highlighted after market dip letter charlotte county ha no goodpaying job young american expect to inherit on average a new survey show how much millennials and gen z are banking on family wealth buford pusser famous tennessee sheriff who inspired hollywood in the s may have killed his wife in authority say mayor brandon johnson executive order ban law enforcement from wearing mask amid impending immigration crackdown mayor brandon johnson executive order ban law enforcement from wearing mask amid impending immigration crackdown a look at the race to replace canada rapidly aging fleet of submarine hilarious antivance demonstrator line up to protest his motorcade a last second turn sends them chasing car trenton raise the ukrainian flag at city hall with help from area organization photo college face financial struggle a trump policy send international enrollment plummeting college face financial struggle a trump policy send international enrollment plummeting election ejection chicago mayor and other dems are warning illegal alien ice will be at the poll we are on the street palestinian flee israel assault on gaza city cal thomas flagging flag burner again ny gov hochul now ha a press office account thats trying to outdo the newsom press office account naomi osaka call out jelena ostapenko over controversial remark toward taylor townsend ukraine exparliamentary speaker is shot dead in lviv dave bossie dnc and mamdani expose the coming disaster for democrat monday is labor day whats open whats closed wisconsin conservative supreme justice rebecca bradley wont seek reelection in fate intervenes family avoids execution in holocaust asking eric since my husband wa killed his family want nothing to do with me or my child salmo to get voter approval for new firetruck nelson trump revenge summer heat up with fed ouster bolton raid trump revenge summer heat up with fed ouster bolton raid new yorkers must fight political manipulation be it by the ccp or the united federation of teacher collegian marlboro rhinebeck resident graduate from university of rhode island tania fernandes anderson asks judge to let her dodge prison time for public corruption israel soon will halt or slow aid to northern gaza a military offensive grows israel soon will halt or slow aid to northern gaza a military offensive grows israel soon will halt or slow aid to northern gaza a military offensive grows doj call for tip on employer favoring foreign worker in hiring practice flag campaignwe cant reclaim that which wa never ours school board member say removing protection doe not give reason to bully trump cast doubt on putinzelensky meeting maybe they have to fight a little longer gaza aid flotilla should not have to exist say thunberg gaza aid flotilla should not have to exist say thunberg gaza aid flotilla should not have to exist say thunberg gaza aid flotilla should not have to exist say thunberg gaza aid flotilla should not have to exist say thunberg gaza aid flotilla should not have to exist say thunberg gaza aid flotilla should not have to exist say thunberg gaza aid flotilla should not have to exist say thunberg thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival nh democrat launch town hall series to promote presidential primary chicago mayor to sign executive order directing city to resist trump immigration raid social security whistleblower who claim doge mishandled american sensitive data resigns from post social security whistleblower who claim doge mishandled american sensitive data resigns from post social security whistleblower who claim doge mishandled american sensitive data resigns from post social security whistleblower who claim doge mishandled american sensitive data resigns from post social security whistleblower who claim doge mishandled american sensitive data resigns from post social security whistleblower who claim doge mishandled american sensitive data resigns from post social security whistleblower who claim doge mishandled american sensitive data resigns from post social security whistleblower who claim doge mishandled american sensitive data resigns from post israel soon will halt or slow aid to northern gaza a military offensive grows israel soon will halt or slow aid to northern gaza a military offensive grows israel soon will halt or slow aid to northern gaza a military offensive grows florida python hunter recount bloody battle with snake she got me son here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza got what it take to be lodis mayor for a day city accepting application from local student border czar say ice ops will ramp up for seattle portland after labor day unofficial election result strike delay start of class in southwest washington school district people are calling this jd vance habit his single most obnoxious characteristic and i have to agree epstein estate to hand over birthday book to lawmaker house dem say saturday morning college face financial struggle a trump policy send international enrollment plummeting letter something to actually feel hopeful about letter far fewer cost with votebymail election dncs summer showdown infighting expose crack in democrat unity narrative against gop agenda law enforcement increasing patrol across new hampshire over labor day weekend when can lawyer be punished for undignified or discourteous criticism of judge kellyanne conway revel in trump insane power grab after cracker barrel fiasco israel soon will halt or slow aid to northern gaza a military offensive grows ice detains somaliamerican activist ramsey county sheriff civilian officer what to know about worker over billionaire protest on labor day axios macron warns world will know by monday if putin played trump again u greenlights million sale of starlink service patriot support to ukraine state top election official balk at doj request for sensitive voter information state top election official balk at doj request for sensitive voter information when did caring for america most vulnerable kid become political opinion assembly bill undermines prop and put public safety at risk chicago plan to maintain peace amid federal deployment bondi fire doj employee over alleged gesture toward guard troop jd vance discusses readiness to be president if god forbid something happens to trump department of defense to conduct training exercise in philly starting sunday summerlins kestrel kestrel common offer unique floor plan whats open whats closed on labor day store hour for walmart costco target publix and more alcom best crypto to buy now magacoin finance gain traction a solana xrp and avax see whale inflow sen rand paul on the national debt let no one say we werent warned magax stage countdown secure your entry before the next wave begin need to save on a new appliance wayfair ha off kitchenaid mixer ninja creami did anyone win the powerball lottery jackpot swell to over billion woodside home open acacia in cadence china xi host modi and putin for summit amid anger over trump tariff daron bland contract cowboy cb agrees to massive extension with hope of returning to pro bowl form surfshark face classaction lawsuit over autorenewal violation final countdown top meme coin to invest before the next x surge hit midhudson people on the move for the week of sept nvidia lean heavily on two undisclosed customer for revenue boom china india pledge partnership ahead of putin joining summit guardian pitcher paid leave extended indefinitely a mlb continues gambling probe rosen top ranked global counsel encourages luminar technology inc investor to secure rosen top ranked global counsel encourages luminar technology inc investor to secure rosen top ranked global counsel encourages luminar technology inc investor to secure grover norquist idea for the next gop reconciliation bill how the fed losing it independence could affect american everyday life social security and medicare cut are coming because the bond market will eventually bring congress to it knee economist say fy energy launch multilevel affiliate program to expand access to cleanpowered crypto infrastructure cardano price support now at a worried holder back altcoins with huge potential like remittix social security and medicare cut are coming because the bond market will force congress economist fortune amazon labor day sale is filled with some surprisingly good deal rosen top ranked global counsel encourages luminar technology inc investor to secure counsel before important deadline in security class action lazr bob on business fort worth ridglea theater look to reel in a buyer nvidia q ai drive growth amid revenue concentration risk lithonias recreation center to get massive renovation and upgrade crypto news ozak ai presale heat up with m raisednext x token tesla unexpectedly end contract at giga texas letting go people tesla unexpectedly end contract at giga texas letting go people electrek gen z shift to aiproof trade like plumbing for job security business brief postal carrier retires after almost year of service intel secures b accelerated chip funding with u equity stake u still working on trade deal despite court ruling ustr say trump tariff spark pricing chaos for u business six month in vintage photo show how the role of woman in the workforce ha evolved in the last year i felt like a dead person former goldman sachs banker said before leaving u to build a startup in seoul which store and restaurant will be open for labor day should you ignore ethereum and buy this surging altcoin instead best samsung phone under r in budget pick that deliver hbar price set for gain in q a one altcoin could make investor over x by november future why trump tariff ruling may not matter for stock investor business daily touted a the teslakiller lucid scramble to stay on the nasdaq kemp jones reaped big money from company with an interest in legislation kemp jones reaped big money from company with an interest in legislation builderais b rise and collapse highlight fragility of ai boom seeking alpha kemp jones reaped big money from company with an interest in legislation final chance to get cash bonus from major u bank putting away a day will secure it for you people still spending on tech despite red flag in july report gizmodo people still spending on tech despite red flag in july report popular weightloss stock make a massive heartsaving claim trump trade counselor peter navarro rebuke politician in black robe over partisan tariff ruling mindanao busine</t>
+          <t>hows the market doe ownership go past the topsoil fresh stock on jim cramers radar juneteenth organizer get funding to repair modernize building panda express owns other restaurant chain do you know which one fed rate cut still on track no firework after nvidia earnings federal government post billion deficit from april to june canada whats going on with broadcom stock friday oakland unified school district looking to shed nearly million from budget is it a bot or not ticketings next big legal fight could reshape the resale industry a model for understanding with edward kaplan smlr investor have opportunity to lead semler scientific inc security fraud lawsuit first filed by the rosen law firm rock tech lithium announces offering of up to million the persistent pitfall of taxpayer funded campaign berkshire hillsbrookline merger nears completion retailer warn trump tariff will trigger consumer price explosion who will he blame boing boing nvidia ceo say ai will actually make u busier in the future gizmodo is amazon falling behind in the cloud computing battle brutally honest way to finance your startup dmv may owe you s and have no obligation to let you know wa being held in just a single case qgold announces financing to complete acquisition of quartz mountain gold project in oregon usa and advance mine centre camp in ontario canada qgold announces financing to complete acquisition of quartz mountain gold project in oregon usa and advance mine centre camp in ontario canada should the federal reserve cut rate next month should the federal reserve cut rate next month hope gas responds to criticism in it pipeline program ratehike case raising cane to open ann arbor location september th the company second in metro detroit trump administration kill wasteful funding for humboldt bay offshore wind project sunblock charcoal and powerball holiday weekend lottery drawing worth billion sunblock charcoal and powerball holiday weekend lottery drawing worth billion sunblock charcoal and powerball holiday weekend lottery drawing worth billion sunblock charcoal and powerball holiday weekend lottery drawing worth billion ardot seeking public comment on proposed disadvantaged business enterprise goal for why you should think twice before buying private equity in your k nasb financial inc declares cash dividend on common stock sunblock charcoal and powerball holiday weekend lottery drawing worth billion ap news ulta beauty delivers strong quarter investor brush off the glow thought i wa going to die tunisian singer detained for week fight deportation while trying to finish music small business joint venture win coast guard cyber contract dupont to sell kevlar business for billion the manufacturer life insurance company grows position in tesla inc tsla stock market news today market slide a chip stock weigh spsp complete index seeking alpha layoff hit international paper jb hunt hormel and more the orange peel first year put asheville on the map now staffer hope to buy it cv walgreens now require prescription for covid vaccine in colorado the denver post in hong kong eric trump lauds growing influence of crypto the new york time forecasting the future analyst projection for oneok what the option market tell u about mastercard lazr investor have opportunity to lead luminar technology inc security fraud lawsuit sword group availability of the h financial report sword group h report of the liquidity agreement contracted with oddo bhf procter gamble unusual option activity forecasting the future analyst projection for dt midstream dows option frenzy what you need to know pce inflation flat but core sticky implication for fed september meeting analyst expectation for targa resource future breaking down karooooo analyst share their view segg medium unveils nextgeneration corporate website showcasing completion of turnaround and launch of growth phase a glimpse into the expert outlook on cheniere energy through analyst is rivian automotive gaining or losing market support peering into extreme network recent short interest let talk indianola kwik star ribbon cutting expert outlook snapon through the eye of analyst is flex gaining or losing market support pe ratio insight for bank of nova scotia let talk knoxville planning and zoning administrator nathan parch part two segg medium unveils nextgeneration corporate website showcasing completion of turnaround and launch of growth phase u government publishes gdp data on bitcoin ethereum blockchains home price in okanagan and kamloops area may be levelling housewise chainlink link price movement face hurdle litecoin target rally while cold wallet hold roi edge major discount on outdoor furniture costway dining set off at target bytedance hit b valuation a q revenue surge to b energy exchange electronx earns cftc designated market and clearing approval how senior can borrow home equity without refinancing now crypto news today coinshares profit jump avalanche transaction rise gumi add xrp here why serve robotics surged this week savvy shopper save over k in year by extreme couponing she scored k of jcpenney cookware for just backtoschool sale tax holiday the edmund fitzgerald and a state microbe theyre among state bill in august should you buy lucid stock ahead of it for reverse stock split bitcoin drop below a xrp slide below and eth dogecoin wobble shopping labor day furniture sale tip to bargain for the best price ollies bargain earnings suggest analyst underestimate longterm potential no ruling friday on trump attempt to fire fed official the credit race closing the perception gap to win welcome to the new made in china era and it look a lot different dell struggle to protect margin a supply chain cost mount cracker barrel ditched it new logo but it also got rid of something else labubu doll and affordable latte why chinese brand are betting big on the u business insider mycarrier portal and carrier assure integrate to make carrier vetting easier cracker barrel is still deep in dei despite the return of uncle herschel former trans mountain ceo to head major project office canada cracker barrel did more than just ditch it logo after maga meltdown the daily beast cracker barrel new logo wa pitiful one of chain original executive say anthony brown maryland legal victory show prudent use of resource reader commentary atlanta becomes largest u metro without a printed daily newspaper a journalconstitution go digital techstock skid sends nasdaq sharply lower live stockmarket update understanding the benefit and risk of ai agent university of northern iowa to open finance and real estate analytics lab for business eli lilly is proof that wall street star dont have to be tech titan trump fire democratic member from transportation board just before it considers the largest railroad merger in history marvell sink a weak data center outlook stokes custom ai chip worry reuters mount logan capital inc shareholder approve previously announced business combination with degree capital corp court block trump effort to end protected status for venezuelan mamdani team with sharpton to threaten wall street upcoming upgrade to holocaust museum exhibit spark some staff concern source trump planning immigration crackdown in chicago next week dhs source say gov gretchen whitmer call special election for state senate seat that could split michigan chamber gov gretchen whitmer call special election for state senate seat that could split michigan chamber gov gretchen whitmer call special election for state senate seat that could split michigan chamber gov gretchen whitmer call special election for state senate seat that could split michigan chamber gov gretchen whitmer call special election for state senate seat that could split michigan chamber gov gretchen whitmer call special election for state senate seat that could split michigan chamber migrant defer their american dream to seek asylum in mexico bonus editorial cartoon for aug alabama town first black mayor reelected after being locked out of office lawyer who led karen read defense one step closer to joining team for civil suit trump move to cut bn in foreign aid already approved by congress rubio revoke visa for palestinian official denying address at un meeting alabama town first black mayor reelected year after he say white resident locked him out of office cbs news can tv help prepare for invasion jd vance say there thing dems should learn from trump and critic cant believe he serious jd vance say there thing dems should learn from trump and critic cant believe he serious abrego garcia asks for gag order on bondi noem meet bill pulte the trump housing official at the center of the latest fed controversy abrego garcia asks for gag order on bondi noem judge weighs request to block trump firing of fed governor lisa cook abrego garcia asks for gag order on bondi noem contract talk fail between alberta government and teacher possible strike loom alberta republican joni ernst will not seek reelection source say abrego garcia asks for gag order on bondi noem trump yank kamala harris bidenextended taxpayerfunded secret service protection before book tour susan estrich the epitome of dumbness judge hears argument on lisa cook attempted firing by trump administration psc answer preston county commission objection to marl project corruption allegation impact argentina president mileis popularity trump block b in foreign aid congress okd using maneuver last seen nearly year ago trump block b in foreign aid congress okd using maneuver last seen nearly year ago mackinac island police chief to resign citing ongoing friction with city council a lament for the shrinking middle class reader commentary dear annie unfaithful fiancee tell me to stop living in the past appeal court block trump administration from ending legal protection for venezuelan appeal court block trump administration from ending legal protection for venezuelan appeal court block trump administration from ending legal protection for venezuelan a trumpbrokered peace deal in the south caucasus is hopeful but incomplete many state employeefriendly labor law take effect a nlrb remains quorumless benton county to display in god we trust in all public building by oct everyone on x point and laugh at dingus gungrabber who share pic of bullet scattered on his street democrat some republican cry outrage over trump use of rare tactic to withhold approved foreign aid funding lori falce year of thought and prayer appeal court say uk asylumseekers can stay at hotel dc federal judge to weigh order blocking fed gov lisa cook firing ahead of interest rate meeting let talk knoxville planning and zoning administrator nathan parch part two donald trump war on culture is not a sideshow japan india to deepen security economic tie amid u tariff ai is ummasking ice officer can washington do anything about it politico public trust in election increase with clear fact sen ernst of iowa is expected to announce next month that she wont run for reelection in u revoke visa of palestinian official ahead of un general assembly fox news star call out trump ally over apparent hypocrisy this is the same thing sen ernst of iowa is expected to announce next month that she wont run for reelection in ap news fox news star call out trump ally over apparent hypocrisy this is the same thing free speech unmuted president trump executive order on flag desecration it a joke san jose mayor slam california legislature over lack of prop funding ransomware attack targeting pa attorney general lead to case delay susan collins rip trump unlawful effort to cancel billion in foreign aid susan collins rip trump unlawful effort to cancel billion in foreign aid susan collins rip trump unlawful effort to cancel billion in foreign aid what to know a texas bill let resident sue outofstate abortion pill provider what to know a texas bill let resident sue outofstate abortion pill provider what to know a texas bill let resident sue outofstate abortion pill provider what to know a texas bill let resident sue outofstate abortion pill provider chicago is in the trump administration sight for it next immigration crackdown chicago is in the trump administration sight for it next immigration crackdown trump admin plan immigration enforcement surge in boston politico a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows a trump threatens more guard troop in u city here what the law allows kilmar abrego garcia asks for gag order against pam bondi kristi noem kilmar abrego garcia asks for gag order against pam bondi kristi noem texas gov greg abbott sign new congressional redistricting map president trump requested kimball shinkoskey explain the law talk for trump riviera in gaza persist a israel push deeper into gaza city france germany vow to up pressure on ogre putin bankruptcy for north dakota and western minnesota published aug trump administration to cut plus job at voice of america best business line of credit in flexible small business funding option for growth and emergency adhesive dowel veneer the industrial choice shaping mass timber verizon down how to fix so modeonly issue in phone amid outage hindustan time hindustan time what would the fed do in a tie vote it not clear and the bank of england had to break a deadlock this month can you use milwaukee battery on harbor freight tool ulster county rail trail study to be contracted to new paltzbased consulting firm tim walz admits vp bid might have hurt him with voter in home state judge delay septum rate increase additional service cut gas price go up in killeen area per gallon at one place kari lake lay off hundred at voa parent agency amid legal battle doesnt surprise memark cuban explains why high school senior care more about making money than any generation in year cnc deadline alert rosen a longstanding law firm encourages centene corporation investor to secure counsel before important september deadline in security class action cnc bet bonus code orl bet on oregon v montana state get in bonus bet bemidji chamber ambassador welcome thrivent financial advisor letter illegal dumping and time to support wastetoenergy how the sound of name can bias hiring decision writer bloc a push for change in the u electoral college give u hope for future climate action strengthening italian finance a new era through takeover consolidation u trading partner dazed and confused after tariff court loss delaware ag other state secure americorps funding in winning suit solana etf buzz fade a investor shift to magacoin finance a rising star best soundbars with wireless rear speaker in cryptos under that could make you x richer mirroring pepe coin pepe run best small business loan option in how owner qualify compare program and secure fast funding with rok financial what happens to trump tariff now that a federal appeal court ha knocked them down cracker barrel or waffle house the south most heated food debate return amid logo saga ai cant install an hvac system why gen z is flocking to job in the trade navigating client conundrum california payday loan online same day no credit check bad credit guaranteed approval radcred launch payday loan platform for immediate financial relief for california borrower usa kari lake lay off more than staff at voice of america parent agency the washington post amazon is selling a laptop for thats nice and responsive how to check for a lien on a car before you buy how an appeal court ruling on trump tariff could upend the bond market barrons how an appeal court ruling on trump tariff could upend the bond market how to check for a lien on a car before you buy sameday business loan in fast approval for owner facing urgent cash flow need how to check for a lien on a car before you buy madison county official think wind farm could impact public safety your money way the new tax bill could impact your wallet ultimate plantbased beet burger mowest to reveal library renovation cuba energy crisis deepens a blackout grip the nation best crypto to invest in why blockdag rtx hyper and snort are gaining attention how europe is redrawing it energy map rosen global investor counsel encourages easterly rocmuni high income municipal bond fund cryptos under to accumulate now ozak ai xdc cro trx and vechain carol saline dy journalist with a story to tell about her dying powerball jackpot rise to billion sixthlargest ever sunblock charcoal and powerball holiday weekend lottery jackpot worth billion is up for grab larimer county restaurant inspection made aug china xi offer backing for myanmar sco membership bid wamco deadline notice rosen trusted investor counsel encourages western asset management company llc mutual fund investor with loss in excess of k to secure counsel before important september deadline in security class action merz promise debt relief for municipality ahead of electoral test burlington store nyseburl announces quarterly earnings result beat estimate by eps u trading partner dazed and confused after tariff court loss bloombergcom u trading partner dazed and confused after tariff court loss shopper can get electronics clothes and school supply worth up to taxfree a u state exemption final hour spirit airline bankruptcy tee up painful cut in survival bid do novelty menu like taco bell yk make investor money southwest airline begin flying first plane with secondary cockpit barrier reuters stock retail wa discussing this week and how they performed open bull mdb nvda baba channel rewind growth spark conflict video vault top wireless printer under r in paige thomason caramel pecan turtle brownie recipe dogecoin price prediction doge alternative for x gain this bull cycle billion powerball jackpot is up for grab saturday here how to play austin americanstatesman baird financial group inc acquires share of qualcomm incorporated qcom best water stock to watch now august th walmart inc wmt share purchased by titleist asset management llc deadline approach for under forty nomination eu to work on using frozen russian asset to aid ukraine after war white house to release m in americorps funding after maryland lawsuit white house to release m in americorps funding after maryland lawsuit groundbreaking of home housing cooperative in upper hammonds plain commentary lawmaker could trim electric bill baird financial group inc acquires share of ishares core sp etf ivv kodai capital management lp invests in honeywell international inc hon haberman call tariff ruling a big blow to trump agenda orange county restaurant shut down by health inspector aug costcos controversial policy change officially take effect costcos controversial policy change officially take effect mcdonalds corporation mcd share sold by baird financial group inc warren buffett warns not to invest in terrible industry because it a rewarding a struggling in quicksand micron boeing lead five stock near buy point yearold retail chain closed dozen of store s at risk in order to become the you must do what the other wont billionaire grant cardone say hard work defines success a court ha ruled most of trump tariff illegal here whats next tesla lawyer ask judge to throw out million verdict saying mention of elon musk misled the jury tesla lawyer ask judge to throw out million verdict saying mention of elon musk misled the jury fortune promising value stock to keep an eye on august th adam thielen take pay cut with viking excited to be back home insight wealth partner llc make new investment in palantir technology inc pltr insight wealth partner llc ha holding in jpmorgan chase co jpm deeply affordable halawa rental tower nearly full best altcoins to buy this week ethereum xrp and magacoin finance highlighted after market dip letter charlotte county ha no goodpaying job young american expect to inherit on average a new survey show how much millennials and gen z are banking on family wealth buford pusser famous tennessee sheriff who inspired hollywood in the s may have killed his wife in authority say mayor brandon johnson executive order ban law enforcement from wearing mask amid impending immigration crackdown mayor brandon johnson executive order ban law enforcement from wearing mask amid impending immigration crackdown a look at the race to replace canada rapidly aging fleet of submarine hilarious antivance demonstrator line up to protest his motorcade a last second turn sends them chasing car trenton raise the ukrainian flag at city hall with help from area organization photo college face financial struggle a trump policy send international enrollment plummeting college face financial struggle a trump policy send international enrollment plummeting election ejection chicago mayor and other dems are warning illegal alien ice will be at the poll we are on the street palestinian flee israel assault on gaza city cal thomas flagging flag burner again ny gov hochul now ha a press office account thats trying to outdo the newsom press office account naomi osaka call out jelena ostapenko over controversial remark toward taylor townsend ukraine exparliamentary speaker is shot dead in lviv dave bossie dnc and mamdani expose the coming disaster for democrat monday is labor day whats open whats closed wisconsin conservative supreme justice rebecca bradley wont seek reelection in fate intervenes family avoids execution in holocaust asking eric since my husband wa killed his family want nothing to do with me or my child salmo to get voter approval for new firetruck nelson trump revenge summer heat up with fed ouster bolton raid trump revenge summer heat up with fed ouster bolton raid new yorkers must fight political manipulation be it by the ccp or the united federation of teacher collegian marlboro rhinebeck resident graduate from university of rhode island tania fernandes anderson asks judge to let her dodge prison time for public corruption israel soon will halt or slow aid to northern gaza a military offensive grows israel soon will halt or slow aid to northern gaza a military offensive grows israel soon will halt or slow aid to northern gaza a military offensive grows doj call for tip on employer favoring foreign worker in hiring practice flag campaignwe cant reclaim that which wa never ours school board member say removing protection doe not give reason to bully trump cast doubt on putinzelensky meeting maybe they have to fight a little longer gaza aid flotilla should not have to exist say thunberg gaza aid flotilla should not have to exist say thunberg gaza aid flotilla should not have to exist say thunberg gaza aid flotilla should not have to exist say thunberg gaza aid flotilla should not have to exist say thunberg gaza aid flotilla should not have to exist say thunberg gaza aid flotilla should not have to exist say thunberg gaza aid flotilla should not have to exist say thunberg thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival thousand protest israeli siege of gaza near venice film festival nh democrat launch town hall series to promote presidential primary chicago mayor to sign executive order directing city to resist trump immigration raid social security whistleblower who claim doge mishandled american sensitive data resigns from post social security whistleblower who claim doge mishandled american sensitive data resigns from post social security whistleblower who claim doge mishandled american sensitive data resigns from post social security whistleblower who claim doge mishandled american sensitive data resigns from post social security whistleblower who claim doge mishandled american sensitive data resigns from post social security whistleblower who claim doge mishandled american sensitive data resigns from post social security whistleblower who claim doge mishandled american sensitive data resigns from post social security whistleblower who claim doge mishandled american sensitive data resigns from post israel soon will halt or slow aid to northern gaza a military offensive grows israel soon will halt or slow aid to northern gaza a military offensive grows israel soon will halt or slow aid to northern gaza a military offensive grows florida python hunter recount bloody battle with snake she got me son here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza here a look at why it is so hard to end the war in gaza got what it take to be lodis mayor for a day city accepting application from local student border czar say ice ops will ramp up for seattle portland after labor day unofficial election result strike delay start of class in southwest washington school district people are calling this jd vance habit his single most obnoxious characteristic and i have to agree epstein estate to hand over birthday book to lawmaker house dem say saturday morning college face financial struggle a trump policy send international enrollment plummeting letter something to actually feel hopeful about letter far fewer cost with votebymail election dncs summer showdown infighting expose crack in democrat unity narrative against gop agenda law enforcement increasing patrol across new hampshire over labor day weekend when can lawyer be punished for undignified or discourteous criticism of judge kellyanne conway revel in trump insane power grab after cracker barrel fiasco israel soon will halt or slow aid to northern gaza a military offensive grows ice detains somaliamerican activist ramsey county sheriff civilian officer what to know about worker over billionaire protest on labor day axios macron warns world will know by monday if putin played trump again u greenlights million sale of starlink service patriot support to ukraine state top election official balk at doj request for sensitive voter information state top election official balk at doj request for sensitive voter information when did caring for america most vulnerable kid become political opinion assembly bill undermines prop and put public safety at risk chicago plan to maintain peace amid federal deployment bondi fire doj employee over alleged gesture toward guard troop jd vance discus readiness to be president if god forbid something happens to trump department of defense to conduct training exercise in philly starting sunday summerlins kestrel kestrel common offer unique floor plan whats open whats closed on labor day store hour for walmart costco target publix and more alcom best crypto to buy now magacoin finance gain traction a solana xrp and avax see whale inflow sen rand paul on the national debt let no one say we werent warned magax stage countdown secure your entry before the next wave begin need to save on a new appliance wayfair ha off kitchenaid mixer ninja creami did anyone win the powerball lottery jackpot swell to over billion woodside home open acacia in cadence china xi host modi and putin for summit amid anger over trump tariff daron bland contract cowboy cb agrees to massive extension with hope of returning to pro bowl form surfshark face classaction lawsuit over autorenewal violation final countdown top meme coin to invest before the next x surge hit midhudson people on the move for the week of sept nvidia lean heavily on two undisclosed customer for revenue boom china india pledge partnership ahead of putin joining summit guardian pitcher paid leave extended indefinitely a mlb continues gambling probe rosen top ranked global counsel encourages luminar technology inc investor to secure rosen top ranked global counsel encourages luminar technology inc investor to secure rosen top ranked global counsel encourages luminar technology inc investor to secure grover norquist idea for the next gop reconciliation bill how the fed losing it independence could affect american everyday life social security and medicare cut are coming because the bond market will eventually bring congress to it knee economist say fy energy launch multilevel affiliate program to expand access to cleanpowered crypto infrastructure cardano price support now at a worried holder back altcoins with huge potential like remittix social security and medicare cut are coming because the bond market will force congress economist fortune amazon labor day sale is filled with some surprisingly good deal rosen top ranked global counsel encourages luminar technology inc investor to secure counsel before important deadline in security class action lazr bob on business fort worth ridglea theater look to reel in a buyer nvidia q ai drive growth amid revenue concentration risk lithonias recreation center to get massive renovation and upgrade crypto news ozak ai presale heat up with m raisednext x token tesla unexpectedly end contract at giga texas letting go people tesla unexpectedly end contract at giga texas letting go people electrek gen z shift to aiproof trade like plumbing for job security business brief postal carrier retires after almost year of service intel secures b accelerated chip funding with u equity stake u still working on trade deal despite court ruling ustr say trump tariff spark pricing chaos for u business six month in vintage photo show how the role of woman in the workforce ha evolved in the last year i felt like a dead person former goldman sachs banker said before leaving u to build a startup in seoul which store and restaurant will be open for labor day should you ignore ethereum and buy this surging altcoin instead best samsung phone under r in budget pick that deliver hbar price set for gain in q a one altcoin could make investor over x by november future why trump tariff ruling may not matter for stock investor business daily touted a the teslakiller lucid scramble to stay on the nasdaq kemp jones reaped big money from company with an interest in legislation kemp jones reaped big money from company with an interest in legislation builderais b rise and collapse highlight fragility of ai boom seeking alpha kemp jones reaped big money from company with an interest in legislation final chance to get cash bonus from major u bank putting away a day will secure it for you people still spending on tech despite red flag in july report gizmodo people still spending on tech despite red flag in july report popular weightloss stock make a massive heartsaving claim trump trade counselor peter navarro rebuke politician in black robe over partisan tariff ruling mindanao business embr</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>the winklevoss twin are eyeing billion crypto ipo trump cant use national guard military in california to enforce law judge breyer rule family of max crash victim push to appoint a special prosecutor saying boeing is trying to buy everyone off gold smash record a ratecut bet policy turmoil fuel haven rush coming price cut at mcdonalds could signal a broader fast food price war coming price cut at mcdonalds could signal a broader fast food price war coming price cut at mcdonalds could signal a broader fast food price war coming price cut at mcdonalds could signal a broader fast food price war coming price cut at mcdonalds could signal a broader fast food price war coming price cut at mcdonalds could signal a broader fast food price war coming price cut at mcdonalds could signal a broader fast food price war palantir stock struggle a valuation criticism and ceo sale weigh on investor coming price cut at mcdonalds could signal a broader fast food price war coming price cut at mcdonalds could signal a broader fast food price war turkiyes huge summer of transfer explained how galatasaray and fenerbahce can outspend europe big club anthropic nearly triple valuation to b with massive new funding disney to pay million over alleged violation of childrens online privacy army pick startup to fasttrack selfdriving squad vehicle ai chatbots for doctor are hot but there plenty of value down the stack too argues corti ceo genesee county architecture firm selects yearold batavia house for new hq hundred of economist defend lisa cook fed independence in open letter against trump effort coming price cut at mcdonalds may signal a broader fast food price war a trump tariff struggle in the court there a simple solution he could consider top trending topic of august the less independent the fed is the more the yield curve will steepen national alliance brenner sap to invest billion in europe sovereign cloud anna wintour tap chloe malle a vogue successor but shes still in charge marcus where you are and where youve been stock are experiencing a healthy reset say citis drew pettit ubs give america a recession checkup and see a probability from the hard data with a soggy economy ahead fortune mcdonalds will launch new value meal on monday sept mcdonalds will launch new value meal on monday sept amazon end a program that let prime member share free shipping perk with user outside household amazon end a program that let prime member share free shipping perk with user outside household general assembly looking to reinvigorate staterun venture capital fund fi deadline rosen leading investor counsel encourages fiserv inc investor with loss in excess of k to secure counsel before important deadline in security class action fi trifork group reporting of transaction made by person discharging managerial responsibility clean any screen or lens with the infinitely reuseable waterbear screen cleaner exbudget staffer weigh in against trump pocket rescission offstrip casino team up with new bookmaker proposed budget for west aurora school district show million surplus save big on top gaming gear from walmart now score headset laptop desktop more company kick off ipo roadshow market rally still ha room to run where to invest what are analytical insight wet strength resin market to reach u million by astute analytica blue apron pivot amid our subscription fatigue coreweave stock crwv sink a insider sell at an alarming pace tipranks kraft heinz to separate into two publicly traded company predoc raise million for aipowered health information management system space stock tracker trump move space command rocket lab open launch complex crocs appoints nike alum to cfo chair coreweave tumble a top shareholder magnetar dial down position put on huge collar trade sherwood news bitcoin buck stock market downtrend but lag gold rally congress return but trump pocket rescission snarl govt funding process congress return but trump pocket rescission snarl govt funding process congress return but trump pocket rescission snarl govt funding process congress return but trump pocket rescission snarl govt funding process solana early investor who bought at and exited at ath belief only new crypto can repeat sol rise congress return but trump pocket rescission snarl govt funding process congress return but trump pocket rescission snarl govt funding process congress return but trump pocket rescission snarl govt funding process congress return but trump pocket rescission snarl govt funding process openai and meta say theyre fixing ai chatbots to better respond to teen in distress openai and meta say theyre fixing ai chatbots to better respond to teen in distress costco told to review footage after store manager blatantly accused shopper of ignoring strict store policy nestle dismisses ceo over undisclosed relationship with subordinate nestle dismisses ceo over undisclosed relationship with subordinate egg milk bread all rising a summer close royce microcap trust nyse rmt a of jul how low will mortgage rate fall with a september fed rate cut here what to know trump and son stake in crypto firm worth bn the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way tesla trillion secret musk say robot could be of it value coming price cut at mcdonalds may signal a broader fast food price war stafford co mull zoning regulation government shutdown on oct seen a increasingly likely exclusive disney will pay m to settle childrens privacy lawsuit with ftc axios ace hardware crave cooky among new business in sugar landmissouri city bet bonus code njcom unlock a guaranteed bonus for mlb u open today syndeo medical announces multiyear exclusive distribution agreement for bearpacs passiotm pump drainage system irbt deadline rosen recognized investor counsel encourages irobot corporation investor with loss in excess of k to secure counsel before important september deadline in security class action irbt the white house premium how washington is creating ai stock rocket openai shuffle executive role acquires statsig for billion openai shuffle executive role acquires statsig for billion the verge salesforce advantage over hubspot and mondaycom highlight relative valuation an expanded version of the dol opinion letter program return what do retail employer need to know jefferies david katz bullish call for cruise maryland man collect his second big lottery prize in two month elliott management look to put fizz back into pepsi with b stake a it press for a turnaround amazon prime signups reportedly lagged in u leading up to annual sale event pennsylvania democrat attract some buzz in the party bid to take back u house turn out trump cant turn activeduty troop into police officer after losing two antiviolence worker to gunfire chicago nonprofit persists we have to be strong why is bangladesh saying it can no longer host rohingya school shouldnt wait for legislature to ban cellphone use the republican editorial pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge why are our church no longer safe annunciation school shooting raise alarming question letter to the editor sen joni ernst will not run for reelection in live now gop hold press conference on federal authority over dc a trump tariff struggle in the court there a simple solution he could consider trump tariff decision an emergency will appeal a soon a wednesday axios what america should know about wes moore guest commentary gov healey slam republic service over stalled trash strike talk kim jong un daughter and possible heir make rare foreign appearance poll what should be the new massachusetts flag the judge who defied trump now face brazil biggest case what is the posse comitatus act yearold law governs military role in local law enforcement voter registration trend unchanged at traditional summer end cimg inc completes the previously announced sale of million of it common stock for bitcoin pentagon authorizes military lawyer to serve a temporary immigration judge pentagon authorizes military lawyer to serve a temporary immigration judge pentagon authorizes military lawyer to serve a temporary immigration judge tim walz appears to tell supporter all is not lost because trump will die soon watch profane rashida tlaib rant target israel backer in wild unhinged tirade how much ha your devon county councillor spent in their community so far british wife of trump voter face deportation after year in u amid immigration crackdown saga education launch tutoring partnership with brooklyn lab to accelerate math learning a life lived herman lyon carried the horror of war with strength and courage harford council district f incumbent jacob bennett run for reelection harford council district f incumbent jacob bennett run for reelection tv writer graham linehans arrest over transgender post spark free speech outcry in the uk tv writer graham linehans arrest over transgender post spark free speech outcry in the uk gop rep thomas massie take first step to force a vote on releasing the epstein file texas dei ban expands to public school face federal lawsuit u drone strike cartel drug boat trump post video for world to see beware uk comedy writer graham linehan arrested over social medium post criticizing trans activist gavin newsom brutally taunt trump after major legal victory trump face new epstein headache a congress return from recess israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive airbnb cofounder share when he lost faith in dem party switched to gop israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive springfield garden could be banned from owning managing property in mass ag campbell say what is a pardon and who is eligible wichita criminal defense lawyer who will replace jerry nadler who will retire in after year in congress repping manhattan looking back on japan surrender in wwii year later trump expected to speak shortly a majority of nevada legislation aimed at government transparency failed during the session in the martian author david baron explores mar mania of the th century israel continues to intensify offensive in gaza city rep jerry nadler announces retirement citing bidens oneterm presidency politico ussfcu win dual honor at broadcom customer achievement award trial of greensboro native accused of attempting to assassinate trump set for sept court annuls istanbul congress of turkey main opposition party dismisses leadership court annuls istanbul congress of turkey main opposition party dismisses leadership ernst wont seek reelection giving democrat opening in battle for senate israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge madness in minneapolis court allows trump admin close in on yanking back bidens gold bar pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge delray beach argues to keep it rainbow intersection at hearing in orlando delray beach argues to keep it rainbow intersection at hearing in orlando judge dismisses lawsuit springfield joined over terminated m epa grant labor day protester across the country demand worker right decry ice labor day protester across the country demand worker right decry ice</t>
+          <t>the winklevoss twin are eyeing billion crypto ipo trump cant use national guard military in california to enforce law judge breyer rule family of max crash victim push to appoint a special prosecutor saying boeing is trying to buy everyone off gold smash record a ratecut bet policy turmoil fuel haven rush coming price cut at mcdonalds could signal a broader fast food price war coming price cut at mcdonalds could signal a broader fast food price war coming price cut at mcdonalds could signal a broader fast food price war coming price cut at mcdonalds could signal a broader fast food price war coming price cut at mcdonalds could signal a broader fast food price war coming price cut at mcdonalds could signal a broader fast food price war coming price cut at mcdonalds could signal a broader fast food price war palantir stock struggle a valuation criticism and ceo sale weigh on investor coming price cut at mcdonalds could signal a broader fast food price war coming price cut at mcdonalds could signal a broader fast food price war turkiyes huge summer of transfer explained how galatasaray and fenerbahce can outspend europe big club anthropic nearly triple valuation to b with massive new funding disney to pay million over alleged violation of childrens online privacy army pick startup to fasttrack selfdriving squad vehicle ai chatbots for doctor are hot but there plenty of value down the stack too argues corti ceo genesee county architecture firm selects yearold batavia house for new hq hundred of economist defend lisa cook fed independence in open letter against trump effort coming price cut at mcdonalds may signal a broader fast food price war a trump tariff struggle in the court there a simple solution he could consider top trending topic of august the le independent the fed is the more the yield curve will steepen national alliance brenner sap to invest billion in europe sovereign cloud anna wintour tap chloe malle a vogue successor but shes still in charge marcus where you are and where youve been stock are experiencing a healthy reset say citis drew pettit ubs give america a recession checkup and see a probability from the hard data with a soggy economy ahead fortune mcdonalds will launch new value meal on monday sept mcdonalds will launch new value meal on monday sept amazon end a program that let prime member share free shipping perk with user outside household amazon end a program that let prime member share free shipping perk with user outside household general assembly looking to reinvigorate staterun venture capital fund fi deadline rosen leading investor counsel encourages fiserv inc investor with loss in excess of k to secure counsel before important deadline in security class action fi trifork group reporting of transaction made by person discharging managerial responsibility clean any screen or lens with the infinitely reuseable waterbear screen cleaner exbudget staffer weigh in against trump pocket rescission offstrip casino team up with new bookmaker proposed budget for west aurora school district show million surplus save big on top gaming gear from walmart now score headset laptop desktop more company kick off ipo roadshow market rally still ha room to run where to invest what are analytical insight wet strength resin market to reach u million by astute analytica blue apron pivot amid our subscription fatigue coreweave stock crwv sink a insider sell at an alarming pace tipranks kraft heinz to separate into two publicly traded company predoc raise million for aipowered health information management system space stock tracker trump move space command rocket lab open launch complex crocs appoints nike alum to cfo chair coreweave tumble a top shareholder magnetar dial down position put on huge collar trade sherwood news bitcoin buck stock market downtrend but lag gold rally congress return but trump pocket rescission snarl govt funding process congress return but trump pocket rescission snarl govt funding process congress return but trump pocket rescission snarl govt funding process congress return but trump pocket rescission snarl govt funding process solana early investor who bought at and exited at ath belief only new crypto can repeat sol rise congress return but trump pocket rescission snarl govt funding process congress return but trump pocket rescission snarl govt funding process congress return but trump pocket rescission snarl govt funding process congress return but trump pocket rescission snarl govt funding process openai and meta say theyre fixing ai chatbots to better respond to teen in distress openai and meta say theyre fixing ai chatbots to better respond to teen in distress costco told to review footage after store manager blatantly accused shopper of ignoring strict store policy nestle dismisses ceo over undisclosed relationship with subordinate nestle dismisses ceo over undisclosed relationship with subordinate egg milk bread all rising a summer close royce microcap trust nyse rmt a of jul how low will mortgage rate fall with a september fed rate cut here what to know trump and son stake in crypto firm worth bn the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way the rule for cash how to manage your money the smart way tesla trillion secret musk say robot could be of it value coming price cut at mcdonalds may signal a broader fast food price war stafford co mull zoning regulation government shutdown on oct seen a increasingly likely exclusive disney will pay m to settle childrens privacy lawsuit with ftc axios ace hardware crave cooky among new business in sugar landmissouri city bet bonus code njcom unlock a guaranteed bonus for mlb u open today syndeo medical announces multiyear exclusive distribution agreement for bearpacs passiotm pump drainage system irbt deadline rosen recognized investor counsel encourages irobot corporation investor with loss in excess of k to secure counsel before important september deadline in security class action irbt the white house premium how washington is creating ai stock rocket openai shuffle executive role acquires statsig for billion openai shuffle executive role acquires statsig for billion the verge salesforce advantage over hubspot and mondaycom highlight relative valuation an expanded version of the dol opinion letter program return what do retail employer need to know jefferies david katz bullish call for cruise maryland man collect his second big lottery prize in two month elliott management look to put fizz back into pepsi with b stake a it press for a turnaround amazon prime signups reportedly lagged in u leading up to annual sale event pennsylvania democrat attract some buzz in the party bid to take back u house turn out trump cant turn activeduty troop into police officer after losing two antiviolence worker to gunfire chicago nonprofit persists we have to be strong why is bangladesh saying it can no longer host rohingya school shouldnt wait for legislature to ban cellphone use the republican editorial pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge why are our church no longer safe annunciation school shooting raise alarming question letter to the editor sen joni ernst will not run for reelection in live now gop hold press conference on federal authority over dc a trump tariff struggle in the court there a simple solution he could consider trump tariff decision an emergency will appeal a soon a wednesday axios what america should know about wes moore guest commentary gov healey slam republic service over stalled trash strike talk kim jong un daughter and possible heir make rare foreign appearance poll what should be the new massachusetts flag the judge who defied trump now face brazil biggest case what is the posse comitatus act yearold law governs military role in local law enforcement voter registration trend unchanged at traditional summer end cimg inc completes the previously announced sale of million of it common stock for bitcoin pentagon authorizes military lawyer to serve a temporary immigration judge pentagon authorizes military lawyer to serve a temporary immigration judge pentagon authorizes military lawyer to serve a temporary immigration judge tim walz appears to tell supporter all is not lost because trump will die soon watch profane rashida tlaib rant target israel backer in wild unhinged tirade how much ha your devon county councillor spent in their community so far british wife of trump voter face deportation after year in u amid immigration crackdown saga education launch tutoring partnership with brooklyn lab to accelerate math learning a life lived herman lyon carried the horror of war with strength and courage harford council district f incumbent jacob bennett run for reelection harford council district f incumbent jacob bennett run for reelection tv writer graham linehans arrest over transgender post spark free speech outcry in the uk tv writer graham linehans arrest over transgender post spark free speech outcry in the uk gop rep thomas massie take first step to force a vote on releasing the epstein file texas dei ban expands to public school face federal lawsuit u drone strike cartel drug boat trump post video for world to see beware uk comedy writer graham linehan arrested over social medium post criticizing trans activist gavin newsom brutally taunt trump after major legal victory trump face new epstein headache a congress return from recess israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive airbnb cofounder share when he lost faith in dem party switched to gop israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive springfield garden could be banned from owning managing property in mass ag campbell say what is a pardon and who is eligible wichita criminal defense lawyer who will replace jerry nadler who will retire in after year in congress repping manhattan looking back on japan surrender in wwii year later trump expected to speak shortly a majority of nevada legislation aimed at government transparency failed during the session in the martian author david baron explores mar mania of the th century israel continues to intensify offensive in gaza city rep jerry nadler announces retirement citing bidens oneterm presidency politico ussfcu win dual honor at broadcom customer achievement award trial of greensboro native accused of attempting to assassinate trump set for sept court annuls istanbul congress of turkey main opposition party dismisses leadership court annuls istanbul congress of turkey main opposition party dismisses leadership ernst wont seek reelection giving democrat opening in battle for senate israel start calling up reservist a it push into initial stage of gaza city offensive israel start calling up reservist a it push into initial stage of gaza city offensive pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge madness in minneapolis court allows trump admin close in on yanking back bidens gold bar pentagon authorizes up to military lawyer to serve a temporary immigration judge pentagon authorizes up to military lawyer to serve a temporary immigration judge delray beach argues to keep it rainbow intersection at hearing in orlando delray beach argues to keep it rainbow intersection at hearing in orlando judge dismisses lawsuit springfield joined over terminated m epa grant labor day protester across the country demand worker right decry ice labor day protester across the country demand worker right decry ice</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>smci nokia deal position it a a fullstack ai solution provider sugar price slip on prospect of higher indian sugar export real estate redux why s housing market feel like penn state to close wpsu radio station this hardhit ai stock is betting big on robotics should you buy share now two meridian hotel up for sale cocoa price fall a the dollar strengthens spot bitcoin etf see strong demand crypto market top trillion a gena shuns gold hamilton leo headshotjpg reconstructing road montrose tirz set sight on west alabama street a latest transportation project ice make rare catastrophically bad call end in retreat with emboldened illegals rioter and sanctuary city placer county planning commission support housing amendment for tahoe basin aim to boost local worker accommodation faa say boeing should pay m in fine over door failure and other safety lapse spesfront highest resolutionjpg report mta lost b to fare and toll scofflaw in report mta lost b to fare and toll scofflaw in coffee price surge on brazil dryness and tighter global supply atlantic settle writer suit over article it retracted rule abandoned crackdown continues the federal trade commission new noncompete strategy thurston county open application period for land use and zoning reform starting september th jurisdictional authority in transnational litigation the greenpeace and energy transfer dispute blackrocks rick rieder climb rank of fed chair contender baton rouge golden deed award winner is leo hamilton giving back to the community brynsontm launch the multifamily industry first fee transparency compliance monitoring tool brynsontm launch the multifamily industry first fee transparency compliance monitoring tool mercks exit highlight uk risk losing pharma investment amid rising cost press release aviatra accelerator launch fall session of fuel your startup income accelerator american shatter fundraising record after charlie kirk tragic death at university event michigan increase power outage bill credit to daily to offset resident inconvenience u and china will discus trade and tiktok in madrid what fed chair powell say next week will be critical for a stock market insistent on cut ukrainian drone hit key russian oil port for the first time cost are down trump declares inflation solved a gas and grocery price soar way cfo are shaking off the finance function department of no label uprgade your cleaning game with off the tineco floor one smart vacuum and mop chewy stock is down after strong fcf result chwy is worth more putnam county legal notice apollo hospital to acquire ifc in health and lifestyle arm consumer sentiment drop to lowest point since may consumer sentiment drop to lowest point since may stock of the day netflix at crossroad can support hold this time rolling the dice board game cafe last place on earth open dumbo location executive turntable ascap add cto to help harness ai plus primary wave hire wmg mainstay tariff tax cut fight each other in latest cbo outlook ap business summarybrief at pm edt ap business summarybrief at pm edt why arista network fell today consumer sentiment drop a american household continue to bear the brunt of trump working family price hike low cost airline struggle while legacy rival soar on global travel rebound figuresiporidesblockchainenthusiasminvestors winklevoss twin gemini stock jump over in nyse debut after pricing ipo above range gemini the winklevoss crypto exchange pop more than in nasdaq debut how to earn money from snapchat in tip trick strategy after year this new orleans nurse gain wisdom best friend working with senior lee county raise tax mill approves budget new exhibit installed at acadiana center for the art take color out of the equation a baton rouge pizzeria moved into the old pluckers wing bar on nicholson see whats new consumer sentiment plummet for lowerincome household nasdaq proposes rule change to enable trading of tokenized security is the jetblue premier credit card worth it annual fee how fibi vacation rental brings an investorfocused approach nationwide tata son board discusses ai future no decision on director appointment update boil water notice lifted for the city of willis boil water notice in effect for the city of willis parento help small business plan to cover parental leave synopsys inc snp share suffer worst day ever amid q result revealing problem with major foundry customer hagens berman wall street coast toward the finish of it best week in the last wall street coast toward the finish of it best week in the last wall street coast toward the finish of it best week in the last construction company zoning change request in gorham town council hand related ross appoints adam mcpherson new vp of residential sale former mar chocolate employee from connecticut admits stealing million from company former mar chocolate employee from connecticut admits stealing million from company wall street coast toward the finish of it best week in the last millionaire trader preferfs dogecoin solana etf over xrp a main catalyst for this explosive meme coin united way raise or of goal fbi reward for info leading to arrest of charlie kirk assassin boosted by private donation brazil prosecutor call for halt on lithium mining in mina gerais striking defense worker reject boeing contract offer bemidji city council discusses budget challenge setting preliminary tax levy jonathan kuminga strongly considering signing m qualifying offer with warrior watchdog trump interior department move to scrap key public land protection in latest giveaway to trump big oil donor polymarket see valuation skyrocket in new funding round taylor swift to be deposed in it end with u fallout mining metric ghalis take on gold silver scarcity fed cut silver price shoot above for fresh year high mentor considers plan for retail residential development project in old village corridor eli lilly loses appeal over medicaid drug pricing fraud case democratic senator call for jpmorgan ceo to testify on bank epstein tie the best amazon deal this week mmgs m nickel deal with anglo american face eu doubt senator jain dc councilmember henderson to discus dc autonomy sept polymarket nears b valuation triple in funding round openai and microsoft seal deal for forprofit shift with b stake sanford bemidji highlight job opportunity at fall frenzy career expo hp board discusses building maintenance challenge britannica and merriamwebster sue perplexity ai over copyright infringement striking defense worker reject boeing contract offer cnbc health union announces winner of social health award elevating healthcare unsung voice italianos restaurant eye fall opening date in new caney flower vendor arrested at launch of trump operation midway blitz deported to mexico parish council debate bus stop signage congressional black caucus demand an investigation into hbcu bomb threat congressional black caucus demand an investigation into hbcu bomb threat congressional black caucus demand an investigation into hbcu bomb threat congressional black caucus demand an investigation into hbcu bomb threat congressional black caucus demand an investigation into hbcu bomb threat congressional black caucus demand an investigation into hbcu bomb threat congressional black caucus demand an investigation into hbcu bomb threat louisiana join multistate push to overturn gun magazine ban protest call for florida dem steve cody to resign after mocking charlie kirk assassination hegseth say pentagon tracking service member civilian who celebrate charlie kirk killing alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege charlie kirk alleged killer wrote meme message on bullet casing alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege legal hurdle persist at alligator alcatraz detention center lawyer say alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege appeal court ruling creates lowerclass citizenship for transgender people judge say social medium erupts over squad dems interview after charlie kirk assassination need to resign eric trump is very sad about charlie kirkand also please buy his book county find temporary solution in idaho for birdtail road bridge northeast of helena placer county planning commission support housing amendment for tahoe basin aim to boost local worker accommodation ohio national guard troop to stay longer in dc gov dewine say former msnbc analyst matthew dowd say channel reacted to right wing medium mob by firing him backlash and firing follow social medium comment on charlie kirk assassination schumer warns of a shutdown if republican dont accept democrat health care demand copy nebraska plan for an immigrant detention center face backlash and uncertainty mamdani if elected mayor pledge to order nypd to arrest netanyahu smithsonian wrestle with independence a white house review pick up press release announcing the release of nky democracy in action a podcast presented by the league of woman voter of nky liberal hype tyler robinson conservative root after maga backlash build bridge depolarize leader to congregate at utah state capitol after charlie kirk assassination immigration agent held a u citizenand veteranfor day without checking his id california bill that say federal officer cant wear facial covering pass jasmine crockett slam maga for blaming kirk killing on dems press release mcdaniel open lifesciky lab at onenky center warns progress depends on free expression and competition of idea trump dismisses catloving nyc republican candidate for mayor a not exactly prime time a israel carried out strike far beyond it border violence surged in the occupied west bank amid quiet mourning some are calling charlie kirk a martyr and want vengeance amid quiet mourning some are calling charlie kirk a martyr and want vengeance amid quiet mourning some are calling charlie kirk a martyr and want vengeance amid quiet mourning some are calling charlie kirk a martyr and want vengeance amid quiet mourning some are calling charlie kirk a martyr and want vengeance marco rubio to address global security during overseas trip historical society set downtown walking tour official fear telling trump harsh truth dynast rule the roost in lok sabha with share show adr analysis ice officer fatally shoot suspect after being dragged by car near chicago official say the girlfriend ending explained who doe daniel side with in the end black student and college across u targeted with racist threat day after charlie kirk killing the guardian ice officer shoot kill suspect who dragged officer with car near chicago say homeland security ice officer shoot kill suspect who dragged officer with car near chicago say homeland security ice officer shoot kill suspect who dragged officer with car near chicago say homeland security ice officer shoot kill suspect who dragged officer with car near chicago say homeland security charlie kirk murder spur firstinthenation state political violence hate crime legislation trump just went on fox and issued an unnerving threat against liberal u and china will discus trade and tiktok in madrid uc berkeley give name in antisemitism investigation pitt college republican hold vigil for activist charlie kirk secret service put agent on leave who wrote negative post about charlie kirk lisa cook bank document appear to contradict trump admins mortgage fraud allegation trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump swipe at sliwa a nyc mayoral candidate poke at plan to use mayor mansion to house cat trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time amid quiet mourning some are calling charlie kirk a martyr and want vengeance teacher put on leave after inflammatory post sauk valley resident gathering in dixon tonight to mourn charlie kirk speak against violence portland mayor refuse trump suggestion of deploying national guard a new crow wing county attorney take oath ohio showdown democrat demand unveiling of epstein file gop hold back amid plead for bipartisan support nyc mayor eric adam admin official fired after calling charlie kirk killing karma nyc mayor eric adam admin official fired after calling charlie kirk killing karma desay sv shine at iaa mobility with in europe with europe for all concept altcoins that could outperform ethereum ozak ai solana and cardano real estate developer gary creagh jr unveils bold symphony park proposal harbor investment advisory llc acquires share of alphabet inc googl walmart inc wmt share sold by norway saving bank doliver advisor lp sell share of walmart inc wmt central pacific bank trust division reduces stock position in alphabet inc googl harbor investment advisory llc purchase share of walmart inc wmt first financial bank trust division purchase share of walmart inc wmt doliver advisor lp cut holding in johnson johnson jnj fiduciary financial group llc ha position in johnson johnson jnj jacob co ca decrease stock holding in exxon mobil corporation xom official break ground on chelmsford water district pfas treatment plant faa seek million in fine from boeing over safety violation midair panel blowout abc news eu reaffirms ice phaseout plan final countdown for arctic pablo coin headline top cryptos to buy this week while cronos rise and cardano hold steady medium advisory important housing announcement faa seek m in fine from boeing over safety violation midair panel blowout broadcom inc avgo position lifted by cullen investment group ltd rosen top ranked investor counsel encourages flye group inc investor to secure counsel rosen top ranked investor counsel encourages flye group inc investor to secure counsel rosen top ranked investor counsel encourages flye group inc investor to secure counsel rosen leading trial attorney encourages cto realty growth inc investor to secure counsel rosen a leading law firm encourage dow inc investor to secure counsel before important rosen leading trial attorney encourages cto realty growth inc investor to secure counsel rosen leading trial attorney encourages cto realty growth inc investor to secure counsel rosen leading trial attorney encourages cto realty growth inc investor to secure counsel taylor morrison kent lay named chair of nevada state contractor board rosen top ranked investor counsel encourages flye group inc investor to secure counsel before important deadline in security class action flye panda express founder join tom dundon in portland trail blazer purchase voya investment management llc increase stock position in pepsico inc pep pepsico inc pep position lessened by lvm capital management ltd mi from rsted to ontario how populist conservative undermine contract sanctity share in ishares core sp etf ivv purchased by jacob co ca american express company axp share bought by jacob co ca marotta asset management take position in ishares core sp etf ivv jacob co ca raise stock position in american express company axp carlisle by tri pointe open in summerlins grand park village bloomington to host public hearing for mndots i corridor expansion on october rosen atrusted and leading law firm encourages pubmatic inc investor to secure counsel before important deadline in security class action pubm xrp and dogecoin observer note magacoin finance announces presale expansion amid growing interest ro khanna seth levine and elizabeth macbride revive america innovation economy before it too late business time big turnout for chamber business showcase mustwatch new movie this weekend dangerous animal friendship more cool season vegetable begin now tony tomeo why strong operational system might be the hidden key to expansion dubuque parking ramp to shift to permit parking only during construction opinion san diego need to build all type of housing not just apartment economic measurement the mirage of exactness first financial bank trust division take position in tesla inc tsla capital market strategy llc ha stake in meta platform inc meta capital market strategy llc cut position in chevron corporation cvx international business machine corporation ibm share sold by investrust capital market strategy llc decrease holding in the home depot inc hd medtronic plc mdt share purchased by first hawaiian bank first financial bank trust division purchase share of the home depot inc hd norway saving bank sell share of chevron corporation cvx first hawaiian bank ha million stake in cisco system inc csco first hawaiian bank grows stock holding in medtronic plc mdt central pacific bank trust division purchase share of chevron corporation cvx investrust reduces stock holding in chevron corporation cvx accountability led to spark improvement next is more rebuilding why andrew friedman october test is looming with dodger moderna share hit a low after report suggests the fda plan to tie covid shot to child death merck co inc mrk share sold by jacob co ca merck co inc mrk is cactus asset management llcs th largest position harbor investment advisory llc acquires share of costco wholesale corporation cost norway saving bank ha million stake in mcdonalds corporation mcd ifc sign million contract with iraq basrah gas for associated gas development of major port mcalister sweet associate inc grows stock holding in alphabet inc googl walmart inc wmt share sold by norway saving bank private client service llc increase position in exxon mobil corporation xom park national corp oh cut stock holding in exxon mobil corporation xom kera capital partner inc increase stock position in exxon mobil corporation xom union pacific corporation unp position lessened by harbor investment advisory llc johnson johnson jnj share sold by park national corp oh realtor interior designer find dream home at arrow peak in northwest valley mass closure of popular grocery chain thats better than walmart to devastate community and threaten snap user journeying towards devcon adventure in ethereum innovation skye canyon present chalk cheer oct faa seek to fine boeing million for safety violation door plug blowout npr ncaaf bet bonus code syracuse secures bonus for tennessee v georgia walmarts pack of extremely useful samsung galaxy smarttags is on sale for only rowlandmiller partnersadv boost holding in united parcel service inc ups round rock city council unanimously pass m budget focused on public safety and infrastructure ahead of growth tariff face legal threat that put trump deficit plan at risk tariff face legal threat that put trump deficit plan at risk dividend stock perfect for gen z investor nobrainer fintech growth stock to buy with right now promising telecom stock to follow today september th broadcom inc avgo share acquired by mclean asset management corp city center advisor llc reduces position in broadcom inc avgo modern wealth management llc ha million stake in broadcom inc avgo tariff face legal threat that put trump deficit plan at risk lvm capital management ltd mi sell share of digital realty trust inc dlr reason to love microsofts dividend goaltender spencer knight sign threeyear extension with blackhawks jacob co ca buy share of abbvie inc abbv oracle corporation orcl holding raised by jacob co ca jpmorgan chase co jpm stake reduced by neville rodie shaw inc lawyer fear child from central america dozen in california are at risk of being deported rubio say qatar strike not going to change usisrael tie university of minnesota teamster reach deal to end strike farm aid concert saved million face skyrocketing health insurance cost unless congress extends subsidy u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie university of minnesota teamster reach deal to end strike farm aid concert saved trump say he want national healing while blaming the radical left a a barrier trump say he want national healing while blaming the radical left a a barrier u farmer head to china a trade strain weigh report pentagon plan national guard troop for louisiana policing washington post report reuters trump defends patel amid scrutiny of fbi director leadership during kirk assassination investigation trump defends patel amid scrutiny of fbi director leadership during kirk assassination investigation politico msnbc ghoul were calling charlie kirk a coward and a baby two week before his assassination london protest organized by farright activist exceeds a small clash break out london protest organized by farright activist exceeds a small clash break out london protest organized by farright activist exceeds a small clash break out london protest organized by farright activist exceeds a small clash break out london protest organized by farright activist exceeds a small clash break out taliban claim an agreement is reached with u envoy on a prisoner swap a they seek better tie texas legislative committee will study freedom of speech on college campus in wake of charlie kirk killing pepsico inc pep share sold by lvm capital management ltd mi dentgroup llc ha million position in vanguard value etf vtv howe rusling inc increase position in spdr gold share gld question linger about alleged shooter motivation for killing charlie kirk question linger about alleged shooter motivation for killing charlie kirk neighbor reeling after nice quiet boy scout arrested for charlie kirk assassination advocate look to statebased immigration program advocate look to statebased immigration program advocate look to statebased immigration program advocate look to statebased immigration program advocate look to statebased immigration program gop bid to oust trump antagonist massie open door for worse outcome report charlie kirk honored a generation greatest at massive london rally where musk condemns left new betmgm bonus code silive secures bonus in pa for eagle v chief ai could use online image a a backdoor into your computer alarming new study suggests live science finovatefall unveiling the future of fintech innovation corp for public broadcasting recipient of governor award wa among early emmy honoree wesbanco bank inc sell share of merck co inc mrk capital asset advisory service llc raise stock position in merck co inc mrk capital asset advisory service llc purchase share of cisco system inc csco wesbanco bank inc boost stock holding in the home depot inc hd capital asset advisory service llc acquires share of the home depot inc hd shotwell rutter baer inc increase holding in vanguard ftse developed market etf vea capital asset advisory service llc sell share of visa inc v accelerate investment advisor llc ha stock holding in visa inc v accelerate investment advisor llc boost stock holding in alphabet inc goog capital asset advisory service llc sell share of mastercard incorporated ma wesbanco bank inc sell share of mastercard incorporated ma rtx corporation rtx share acquired by capital asset advisory service llc capital asset advisory service llc purchase share of merck co inc mrk advanced micro device inc amd stake cut by wesbanco bank inc capital asset advisory service llc acquires share of international business machine corporation ibm capital asset advisory service llc increase holding in rtx corporation rtx wesbanco bank inc ha million holding in mastercard incorporated ma build canada home aim to build housing unit on federal land carney value partner investment inc buy share of unitedhealth group incorporated unh value partner investment inc increase stock position in ge aerospace ge value partner investment inc ha million holding in unitedhealth group incorporated unh central pacific bank trust division purchase share of unitedhealth group incorporated unh greenfield saving bank ha million stock position in oracle corporation orcl vanguard midcap etf vo share acquired by good steward wealth advisor llc salesforce inc crm share sold by roxbury financial llc oracle nyseorcl see strong trading volume here what happened versant capital management inc sell share of exxon mobil corporation xom oracle corporation orcl stake boosted by greenfield saving bank salesforce inc crm share sold by roxbury financial llc greenfield saving bank grows holding in exxon mobil corporation xom greenfield saving bank raise stake in ishares core sp midcap etf ijh walmart inc wmt share bought by greenfield saving bank phillies superstar projected to exceed million in free agency insider legal south winn csd bill frank founder charlie javice accepts responsibility for m fraud ahead of sentencing park edge advisor llc buy share of invesco qqq qqq invesco qqq qqq holding decreased by whitaker myers wealth manager ltd invesco qqq qqq stock position lifted by life line wealth management llc garde capital inc ha stock holding in mcdonalds corporation mcd peak financial advisor llc invests in johnson johnson jnj garde capital inc boost stake in abbvie inc abbv salem investment counselor inc sell share of pepsico inc pep pepsico inc pep share purchased by wealth alliance advisory group llc park edge advisor llc acquires share of invesco qqq qqq johnson johnson jnj share sold by aletheian wealth advisor llc wealth alliance advisory group llc grows stock holding in abbvie inc abbv wealth alliance advisory group llc purchase share of mcdonalds corporation mcd fiduciary financial group llc lower position in pepsico inc pep invesco qqq qqq share sold by whitaker myers wealth manager ltd looking for a job in transit hrt is hosting fall career fair looking for a job in transit hrt is hosting fall career fair datcp weekly livestock market update the final countdown why these best cryptos to buy today could explode soon global wealth strategy associate ha holding in ishares core sp etf ivv retirement wealth solution llc sell share of ishares core sp etf ivv retirement wealth solution llc ha position in vanguard total stock market etf vti ftc investigates amazon google for misleading ad practice eli lilly and company lly share bought by first community trust na modus advisor llc grows stock position in procter gamble company the pg truewealth advisor llc sell share of procter gamble company the pg first community trust na boost stake in eli lilly and company lly yankee predicted to lose cody bellinger a price reach million u china meet for trade talk in madrid somerset trust co sell share of ishares core sp smallcap etf ijr california lawmaker pas measure to expand oil production in central valley restrict offshore drilling s sc law is the reason you wont find playing card at a local bar zevenbergen capital investment llc ha stake in accenture plc acn accenture plc acn stock holding raised by osprey private wealth llc vishria bird financial group llc buy new position in philip morr</t>
+          <t>smci nokia deal position it a a fullstack ai solution provider sugar price slip on prospect of higher indian sugar export real estate redux why s housing market feel like penn state to close wpsu radio station this hardhit ai stock is betting big on robotics should you buy share now two meridian hotel up for sale cocoa price fall a the dollar strengthens spot bitcoin etf see strong demand crypto market top trillion a gena shuns gold hamilton leo headshotjpg reconstructing road montrose tirz set sight on west alabama street a latest transportation project ice make rare catastrophically bad call end in retreat with emboldened illegals rioter and sanctuary city placer county planning commission support housing amendment for tahoe basin aim to boost local worker accommodation faa say boeing should pay m in fine over door failure and other safety lapse spesfront highest resolutionjpg report mta lost b to fare and toll scofflaw in report mta lost b to fare and toll scofflaw in coffee price surge on brazil dryness and tighter global supply atlantic settle writer suit over article it retracted rule abandoned crackdown continues the federal trade commission new noncompete strategy thurston county open application period for land use and zoning reform starting september th jurisdictional authority in transnational litigation the greenpeace and energy transfer dispute blackrocks rick rieder climb rank of fed chair contender baton rouge golden deed award winner is leo hamilton giving back to the community brynsontm launch the multifamily industry first fee transparency compliance monitoring tool brynsontm launch the multifamily industry first fee transparency compliance monitoring tool mercks exit highlight uk risk losing pharma investment amid rising cost press release aviatra accelerator launch fall session of fuel your startup income accelerator american shatter fundraising record after charlie kirk tragic death at university event michigan increase power outage bill credit to daily to offset resident inconvenience u and china will discus trade and tiktok in madrid what fed chair powell say next week will be critical for a stock market insistent on cut ukrainian drone hit key russian oil port for the first time cost are down trump declares inflation solved a gas and grocery price soar way cfo are shaking off the finance function department of no label uprgade your cleaning game with off the tineco floor one smart vacuum and mop chewy stock is down after strong fcf result chwy is worth more putnam county legal notice apollo hospital to acquire ifc in health and lifestyle arm consumer sentiment drop to lowest point since may consumer sentiment drop to lowest point since may stock of the day netflix at crossroad can support hold this time rolling the dice board game cafe last place on earth open dumbo location executive turntable ascap add cto to help harness ai plus primary wave hire wmg mainstay tariff tax cut fight each other in latest cbo outlook ap business summarybrief at pm edt ap business summarybrief at pm edt why arista network fell today consumer sentiment drop a american household continue to bear the brunt of trump working family price hike low cost airline struggle while legacy rival soar on global travel rebound figuresiporidesblockchainenthusiasminvestors winklevoss twin gemini stock jump over in nyse debut after pricing ipo above range gemini the winklevoss crypto exchange pop more than in nasdaq debut how to earn money from snapchat in tip trick strategy after year this new orleans nurse gain wisdom best friend working with senior lee county raise tax mill approves budget new exhibit installed at acadiana center for the art take color out of the equation a baton rouge pizzeria moved into the old pluckers wing bar on nicholson see whats new consumer sentiment plummet for lowerincome household nasdaq proposes rule change to enable trading of tokenized security is the jetblue premier credit card worth it annual fee how fibi vacation rental brings an investorfocused approach nationwide tata son board discus ai future no decision on director appointment update boil water notice lifted for the city of willis boil water notice in effect for the city of willis parento help small business plan to cover parental leave synopsys inc snp share suffer worst day ever amid q result revealing problem with major foundry customer hagens berman wall street coast toward the finish of it best week in the last wall street coast toward the finish of it best week in the last wall street coast toward the finish of it best week in the last construction company zoning change request in gorham town council hand related ross appoints adam mcpherson new vp of residential sale former mar chocolate employee from connecticut admits stealing million from company former mar chocolate employee from connecticut admits stealing million from company wall street coast toward the finish of it best week in the last millionaire trader preferfs dogecoin solana etf over xrp a main catalyst for this explosive meme coin united way raise or of goal fbi reward for info leading to arrest of charlie kirk assassin boosted by private donation brazil prosecutor call for halt on lithium mining in mina gerais striking defense worker reject boeing contract offer bemidji city council discus budget challenge setting preliminary tax levy jonathan kuminga strongly considering signing m qualifying offer with warrior watchdog trump interior department move to scrap key public land protection in latest giveaway to trump big oil donor polymarket see valuation skyrocket in new funding round taylor swift to be deposed in it end with u fallout mining metric ghalis take on gold silver scarcity fed cut silver price shoot above for fresh year high mentor considers plan for retail residential development project in old village corridor eli lilly loses appeal over medicaid drug pricing fraud case democratic senator call for jpmorgan ceo to testify on bank epstein tie the best amazon deal this week mmgs m nickel deal with anglo american face eu doubt senator jain dc councilmember henderson to discus dc autonomy sept polymarket nears b valuation triple in funding round openai and microsoft seal deal for forprofit shift with b stake sanford bemidji highlight job opportunity at fall frenzy career expo hp board discus building maintenance challenge britannica and merriamwebster sue perplexity ai over copyright infringement striking defense worker reject boeing contract offer cnbc health union announces winner of social health award elevating healthcare unsung voice italianos restaurant eye fall opening date in new caney flower vendor arrested at launch of trump operation midway blitz deported to mexico parish council debate bus stop signage congressional black caucus demand an investigation into hbcu bomb threat congressional black caucus demand an investigation into hbcu bomb threat congressional black caucus demand an investigation into hbcu bomb threat congressional black caucus demand an investigation into hbcu bomb threat congressional black caucus demand an investigation into hbcu bomb threat congressional black caucus demand an investigation into hbcu bomb threat congressional black caucus demand an investigation into hbcu bomb threat louisiana join multistate push to overturn gun magazine ban protest call for florida dem steve cody to resign after mocking charlie kirk assassination hegseth say pentagon tracking service member civilian who celebrate charlie kirk killing alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege charlie kirk alleged killer wrote meme message on bullet casing alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege legal hurdle persist at alligator alcatraz detention center lawyer say alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege alligator alcatraz detainee continue to face obstacle to meet with lawyer court paper allege appeal court ruling creates lowerclass citizenship for transgender people judge say social medium erupts over squad dems interview after charlie kirk assassination need to resign eric trump is very sad about charlie kirkand also please buy his book county find temporary solution in idaho for birdtail road bridge northeast of helena placer county planning commission support housing amendment for tahoe basin aim to boost local worker accommodation ohio national guard troop to stay longer in dc gov dewine say former msnbc analyst matthew dowd say channel reacted to right wing medium mob by firing him backlash and firing follow social medium comment on charlie kirk assassination schumer warns of a shutdown if republican dont accept democrat health care demand copy nebraska plan for an immigrant detention center face backlash and uncertainty mamdani if elected mayor pledge to order nypd to arrest netanyahu smithsonian wrestle with independence a white house review pick up press release announcing the release of nky democracy in action a podcast presented by the league of woman voter of nky liberal hype tyler robinson conservative root after maga backlash build bridge depolarize leader to congregate at utah state capitol after charlie kirk assassination immigration agent held a u citizenand veteranfor day without checking his id california bill that say federal officer cant wear facial covering pass jasmine crockett slam maga for blaming kirk killing on dems press release mcdaniel open lifesciky lab at onenky center warns progress depends on free expression and competition of idea trump dismisses catloving nyc republican candidate for mayor a not exactly prime time a israel carried out strike far beyond it border violence surged in the occupied west bank amid quiet mourning some are calling charlie kirk a martyr and want vengeance amid quiet mourning some are calling charlie kirk a martyr and want vengeance amid quiet mourning some are calling charlie kirk a martyr and want vengeance amid quiet mourning some are calling charlie kirk a martyr and want vengeance amid quiet mourning some are calling charlie kirk a martyr and want vengeance marco rubio to address global security during overseas trip historical society set downtown walking tour official fear telling trump harsh truth dynast rule the roost in lok sabha with share show adr analysis ice officer fatally shoot suspect after being dragged by car near chicago official say the girlfriend ending explained who doe daniel side with in the end black student and college across u targeted with racist threat day after charlie kirk killing the guardian ice officer shoot kill suspect who dragged officer with car near chicago say homeland security ice officer shoot kill suspect who dragged officer with car near chicago say homeland security ice officer shoot kill suspect who dragged officer with car near chicago say homeland security ice officer shoot kill suspect who dragged officer with car near chicago say homeland security charlie kirk murder spur firstinthenation state political violence hate crime legislation trump just went on fox and issued an unnerving threat against liberal u and china will discus trade and tiktok in madrid uc berkeley give name in antisemitism investigation pitt college republican hold vigil for activist charlie kirk secret service put agent on leave who wrote negative post about charlie kirk lisa cook bank document appear to contradict trump admins mortgage fraud allegation trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump swipe at sliwa a nyc mayoral candidate poke at plan to use mayor mansion to house cat trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time trump dismisses catloving nyc republican candidate for mayor a not exactly prime time amid quiet mourning some are calling charlie kirk a martyr and want vengeance teacher put on leave after inflammatory post sauk valley resident gathering in dixon tonight to mourn charlie kirk speak against violence portland mayor refuse trump suggestion of deploying national guard a new crow wing county attorney take oath ohio showdown democrat demand unveiling of epstein file gop hold back amid plead for bipartisan support nyc mayor eric adam admin official fired after calling charlie kirk killing karma nyc mayor eric adam admin official fired after calling charlie kirk killing karma desay sv shine at iaa mobility with in europe with europe for all concept altcoins that could outperform ethereum ozak ai solana and cardano real estate developer gary creagh jr unveils bold symphony park proposal harbor investment advisory llc acquires share of alphabet inc googl walmart inc wmt share sold by norway saving bank doliver advisor lp sell share of walmart inc wmt central pacific bank trust division reduces stock position in alphabet inc googl harbor investment advisory llc purchase share of walmart inc wmt first financial bank trust division purchase share of walmart inc wmt doliver advisor lp cut holding in johnson johnson jnj fiduciary financial group llc ha position in johnson johnson jnj jacob co ca decrease stock holding in exxon mobil corporation xom official break ground on chelmsford water district pfas treatment plant faa seek million in fine from boeing over safety violation midair panel blowout abc news eu reaffirms ice phaseout plan final countdown for arctic pablo coin headline top cryptos to buy this week while cronos rise and cardano hold steady medium advisory important housing announcement faa seek m in fine from boeing over safety violation midair panel blowout broadcom inc avgo position lifted by cullen investment group ltd rosen top ranked investor counsel encourages flye group inc investor to secure counsel rosen top ranked investor counsel encourages flye group inc investor to secure counsel rosen top ranked investor counsel encourages flye group inc investor to secure counsel rosen leading trial attorney encourages cto realty growth inc investor to secure counsel rosen a leading law firm encourage dow inc investor to secure counsel before important rosen leading trial attorney encourages cto realty growth inc investor to secure counsel rosen leading trial attorney encourages cto realty growth inc investor to secure counsel rosen leading trial attorney encourages cto realty growth inc investor to secure counsel taylor morrison kent lay named chair of nevada state contractor board rosen top ranked investor counsel encourages flye group inc investor to secure counsel before important deadline in security class action flye panda express founder join tom dundon in portland trail blazer purchase voya investment management llc increase stock position in pepsico inc pep pepsico inc pep position lessened by lvm capital management ltd mi from rsted to ontario how populist conservative undermine contract sanctity share in ishares core sp etf ivv purchased by jacob co ca american express company axp share bought by jacob co ca marotta asset management take position in ishares core sp etf ivv jacob co ca raise stock position in american express company axp carlisle by tri pointe open in summerlins grand park village bloomington to host public hearing for mndots i corridor expansion on october rosen atrusted and leading law firm encourages pubmatic inc investor to secure counsel before important deadline in security class action pubm xrp and dogecoin observer note magacoin finance announces presale expansion amid growing interest ro khanna seth levine and elizabeth macbride revive america innovation economy before it too late business time big turnout for chamber business showcase mustwatch new movie this weekend dangerous animal friendship more cool season vegetable begin now tony tomeo why strong operational system might be the hidden key to expansion dubuque parking ramp to shift to permit parking only during construction opinion san diego need to build all type of housing not just apartment economic measurement the mirage of exactness first financial bank trust division take position in tesla inc tsla capital market strategy llc ha stake in meta platform inc meta capital market strategy llc cut position in chevron corporation cvx international business machine corporation ibm share sold by investrust capital market strategy llc decrease holding in the home depot inc hd medtronic plc mdt share purchased by first hawaiian bank first financial bank trust division purchase share of the home depot inc hd norway saving bank sell share of chevron corporation cvx first hawaiian bank ha million stake in cisco system inc csco first hawaiian bank grows stock holding in medtronic plc mdt central pacific bank trust division purchase share of chevron corporation cvx investrust reduces stock holding in chevron corporation cvx accountability led to spark improvement next is more rebuilding why andrew friedman october test is looming with dodger moderna share hit a low after report suggests the fda plan to tie covid shot to child death merck co inc mrk share sold by jacob co ca merck co inc mrk is cactus asset management llcs th largest position harbor investment advisory llc acquires share of costco wholesale corporation cost norway saving bank ha million stake in mcdonalds corporation mcd ifc sign million contract with iraq basrah gas for associated gas development of major port mcalister sweet associate inc grows stock holding in alphabet inc googl walmart inc wmt share sold by norway saving bank private client service llc increase position in exxon mobil corporation xom park national corp oh cut stock holding in exxon mobil corporation xom kera capital partner inc increase stock position in exxon mobil corporation xom union pacific corporation unp position lessened by harbor investment advisory llc johnson johnson jnj share sold by park national corp oh realtor interior designer find dream home at arrow peak in northwest valley mass closure of popular grocery chain thats better than walmart to devastate community and threaten snap user journeying towards devcon adventure in ethereum innovation skye canyon present chalk cheer oct faa seek to fine boeing million for safety violation door plug blowout npr ncaaf bet bonus code syracuse secures bonus for tennessee v georgia walmarts pack of extremely useful samsung galaxy smarttags is on sale for only rowlandmiller partnersadv boost holding in united parcel service inc ups round rock city council unanimously pass m budget focused on public safety and infrastructure ahead of growth tariff face legal threat that put trump deficit plan at risk tariff face legal threat that put trump deficit plan at risk dividend stock perfect for gen z investor nobrainer fintech growth stock to buy with right now promising telecom stock to follow today september th broadcom inc avgo share acquired by mclean asset management corp city center advisor llc reduces position in broadcom inc avgo modern wealth management llc ha million stake in broadcom inc avgo tariff face legal threat that put trump deficit plan at risk lvm capital management ltd mi sell share of digital realty trust inc dlr reason to love microsofts dividend goaltender spencer knight sign threeyear extension with blackhawks jacob co ca buy share of abbvie inc abbv oracle corporation orcl holding raised by jacob co ca jpmorgan chase co jpm stake reduced by neville rodie shaw inc lawyer fear child from central america dozen in california are at risk of being deported rubio say qatar strike not going to change usisrael tie university of minnesota teamster reach deal to end strike farm aid concert saved million face skyrocketing health insurance cost unless congress extends subsidy u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap u envoy in kabul to discus possible prisoner swap rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie rubio say qatar strike not going to change usisrael tie university of minnesota teamster reach deal to end strike farm aid concert saved trump say he want national healing while blaming the radical left a a barrier trump say he want national healing while blaming the radical left a a barrier u farmer head to china a trade strain weigh report pentagon plan national guard troop for louisiana policing washington post report reuters trump defends patel amid scrutiny of fbi director leadership during kirk assassination investigation trump defends patel amid scrutiny of fbi director leadership during kirk assassination investigation politico msnbc ghoul were calling charlie kirk a coward and a baby two week before his assassination london protest organized by farright activist exceeds a small clash break out london protest organized by farright activist exceeds a small clash break out london protest organized by farright activist exceeds a small clash break out london protest organized by farright activist exceeds a small clash break out london protest organized by farright activist exceeds a small clash break out taliban claim an agreement is reached with u envoy on a prisoner swap a they seek better tie texas legislative committee will study freedom of speech on college campus in wake of charlie kirk killing pepsico inc pep share sold by lvm capital management ltd mi dentgroup llc ha million position in vanguard value etf vtv howe rusling inc increase position in spdr gold share gld question linger about alleged shooter motivation for killing charlie kirk question linger about alleged shooter motivation for killing charlie kirk neighbor reeling after nice quiet boy scout arrested for charlie kirk assassination advocate look to statebased immigration program advocate look to statebased immigration program advocate look to statebased immigration program advocate look to statebased immigration program advocate look to statebased immigration program gop bid to oust trump antagonist massie open door for worse outcome report charlie kirk honored a generation greatest at massive london rally where musk condemns left new betmgm bonus code silive secures bonus in pa for eagle v chief ai could use online image a a backdoor into your computer alarming new study suggests live science finovatefall unveiling the future of fintech innovation corp for public broadcasting recipient of governor award wa among early emmy honoree wesbanco bank inc sell share of merck co inc mrk capital asset advisory service llc raise stock position in merck co inc mrk capital asset advisory service llc purchase share of cisco system inc csco wesbanco bank inc boost stock holding in the home depot inc hd capital asset advisory service llc acquires share of the home depot inc hd shotwell rutter baer inc increase holding in vanguard ftse developed market etf vea capital asset advisory service llc sell share of visa inc v accelerate investment advisor llc ha stock holding in visa inc v accelerate investment advisor llc boost stock holding in alphabet inc goog capital asset advisory service llc sell share of mastercard incorporated ma wesbanco bank inc sell share of mastercard incorporated ma rtx corporation rtx share acquired by capital asset advisory service llc capital asset advisory service llc purchase share of merck co inc mrk advanced micro device inc amd stake cut by wesbanco bank inc capital asset advisory service llc acquires share of international business machine corporation ibm capital asset advisory service llc increase holding in rtx corporation rtx wesbanco bank inc ha million holding in mastercard incorporated ma build canada home aim to build housing unit on federal land carney value partner investment inc buy share of unitedhealth group incorporated unh value partner investment inc increase stock position in ge aerospace ge value partner investment inc ha million holding in unitedhealth group incorporated unh central pacific bank trust division purchase share of unitedhealth group incorporated unh greenfield saving bank ha million stock position in oracle corporation orcl vanguard midcap etf vo share acquired by good steward wealth advisor llc salesforce inc crm share sold by roxbury financial llc oracle nyseorcl see strong trading volume here what happened versant capital management inc sell share of exxon mobil corporation xom oracle corporation orcl stake boosted by greenfield saving bank salesforce inc crm share sold by roxbury financial llc greenfield saving bank grows holding in exxon mobil corporation xom greenfield saving bank raise stake in ishares core sp midcap etf ijh walmart inc wmt share bought by greenfield saving bank phillies superstar projected to exceed million in free agency insider legal south winn csd bill frank founder charlie javice accepts responsibility for m fraud ahead of sentencing park edge advisor llc buy share of invesco qqq qqq invesco qqq qqq holding decreased by whitaker myers wealth manager ltd invesco qqq qqq stock position lifted by life line wealth management llc garde capital inc ha stock holding in mcdonalds corporation mcd peak financial advisor llc invests in johnson johnson jnj garde capital inc boost stake in abbvie inc abbv salem investment counselor inc sell share of pepsico inc pep pepsico inc pep share purchased by wealth alliance advisory group llc park edge advisor llc acquires share of invesco qqq qqq johnson johnson jnj share sold by aletheian wealth advisor llc wealth alliance advisory group llc grows stock holding in abbvie inc abbv wealth alliance advisory group llc purchase share of mcdonalds corporation mcd fiduciary financial group llc lower position in pepsico inc pep invesco qqq qqq share sold by whitaker myers wealth manager ltd looking for a job in transit hrt is hosting fall career fair looking for a job in transit hrt is hosting fall career fair datcp weekly livestock market update the final countdown why these best cryptos to buy today could explode soon global wealth strategy associate ha holding in ishares core sp etf ivv retirement wealth solution llc sell share of ishares core sp etf ivv retirement wealth solution llc ha position in vanguard total stock market etf vti ftc investigates amazon google for misleading ad practice eli lilly and company lly share bought by first community trust na modus advisor llc grows stock position in procter gamble company the pg truewealth advisor llc sell share of procter gamble company the pg first community trust na boost stake in eli lilly and company lly yankee predicted to lose cody bellinger a price reach million u china meet for trade talk in madrid somerset trust co sell share of ishares core sp smallcap etf ijr california lawmaker pas measure to expand oil production in central valley restrict offshore drilling s sc law is the reason you wont find playing card at a local bar zevenbergen capital investment llc ha stake in accenture plc acn accenture plc acn stock holding raised by osprey private wealth llc vishria bird financial group llc buy new position in philip morris intern</t>
         </is>
       </c>
     </row>
@@ -2361,10 +2361,10 @@
         <v>45922</v>
       </c>
       <c r="B63" t="n">
-        <v>6692.02001953125</v>
+        <v>6693.75</v>
       </c>
       <c r="C63" t="n">
-        <v>6694.3701171875</v>
+        <v>6698.8798828125</v>
       </c>
       <c r="D63" t="n">
         <v>6648.06982421875</v>
@@ -2373,10 +2373,10 @@
         <v>6654.27978515625</v>
       </c>
       <c r="F63" t="n">
-        <v>1881121000</v>
+        <v>5642620000</v>
       </c>
       <c r="G63" t="n">
-        <v>0.0041504595816321</v>
+        <v>0.004410046474333</v>
       </c>
       <c r="H63" t="n">
         <v>1</v>
@@ -2386,6 +2386,91 @@
           <t>subnautica lawsuit take a bizarre turn a krafton seemingly change it tune miller receives regional west caring kind award stock to buy a fed rate cut reshape the market kingstone capital partner texas llc acquires new position in abbvie inc abbv procter gamble company the pg share sold by grove bank trust ar wealth advisor group llc ha stock holding in oracle corporation orcl livforsakringsbolaget skandia omsesidigt decrease position in unitedhealth group incorporated unh legacy financial strategy llc purchase share of walmart inc wmt ferguson wellman capital management inc ha million holding in eli lilly and company lly mogy joel r investment counsel inc sell share of oracle corporation orcl bank of america corporation bac holding decreased by ferguson wellman capital management inc grove bank trust ha million stock position in unitedhealth group incorporated unh livforsakringsbolaget skandia omsesidigt ha million stock holding in bank of america corporation bac ferguson wellman capital management inc sell share of unitedhealth group incorporated unh eli lilly and company lly share bought by contravisory investment management inc eli lilly and company lly share sold by ferguson wellman capital management inc bank of america corporation bac share sold by ferguson wellman capital management inc george soros reportedly shell out million for gavin newsoms gerrymandering gambit meridian hold budget hearing set millage rate u household electricity bill expected to rise percent this winter montgomery county planning commission to reveal comprehensive plan montgomery county planning commission to reveal comprehensive plan can lululemon get new life from the amex platinum card dont count on it analyst say oldfather financial service llc reduces stock position in invesco qqq qqq invesco qqq qqq position boosted by baker tilly wealth management llc atticus wealth management llc ha stock holding in taiwan semiconductor manufacturing company ltd tsm white wing wealth management sell share of invesco qqq qqq invesco qqq qqq position lessened by kozak associate inc tripadvisor stock argan and another reach new high and buy point myriad system partner remain ahead of the curve on good faith estimate and the no surprise act jpmorgan chase hire two senior banker to bolster consumer and retail investment team yahoo finance is your baby food on the recall list sugar price settle higher a they consolidate this week loss fanfavorite crocs loungefly backpack and starbucks tumbler or more off at disney store fanfavorite crocs loungefly backpack and starbucks tumbler or more off at disney store climatecontrolled storage facility coming to easton redhawk wealth advisor inc ha million holding in chevron corporation cvx chevron corporation cvx stock position lifted by ar wealth advisor group llc san diego gas price hit fourmonth high tax hike and refinery closure add pressure cocoa price rebound a ice inventory tighten freight rate war engulfs asiaeurope astranspacific rally vanishes trump new york time lawsuit dismissed by federal judge meet the exec taking the helm of blackstones billion real estate fund after the tragic loss of wesley lepatner coffee price plummet a u lawmaker seek tariff exemption on coffee county road work to reduce flow of traffic for two week the gold bull pile back in a it nears prefomc level nx class action notice the law office of frank r cruz file security fraud lawsuit against quanex building product corporation jurassic park of investing why democratized private equity is a dangerous idea selective wealth management inc ha million stock holding in vanguard total stock market etf vti impactfolio llc acquires share of vanguard total stock market etf vti charter oak capital management llc acquires share of tesla inc tsla ap news summary at pm edt ted cruz compare fcc chair carr to mafia bos in jimmy kimmel warning ap news summary at pm edt who qualifies for no tax on tip and what count a a tip here are the new rule who qualifies for no tax on tip and what count a a tip here are the new rule political gridlock continues over pa budget straining finance for county school nonprofit could this new drug be the safer way to fight obesity montpelier subcommittee ponders economic development initiative nextera energy inc nee share purchased by moody national bank trust division outside voice making the case for an end to aluminum tariff new fhwa chief under pressure to fix truck parking unusual machine appoints nathaniel kennedy a vice president of marketing unusual machine appoints nathaniel kennedy a vice president of marketing unusual machine appoints nathaniel kennedy a vice president of marketing unusual machine appoints nathaniel kennedy a vice president of marketing unusual machine appoints nathaniel kennedy a vice president of marketing group join moscow school district in lawsuit over idaho private school tax credit loss of health care tax credit loom for oklahoman foothill chamber of commerce gather local business for after afterhours event inventhelp inventor develops recycle receptacle for contact lens los inventhelp inventor develops recycle receptacle for contact lens los ecopro material and green liion announce loi to establish longterm strategic partnership for recycled ncm hydroxide supply the latest federal judge toss trump b defamation lawsuit against the new york time signal advisor wealth llc boost stake in stryker corporation syk stryker corporation syk share sold by perkins coie trust co signal advisor wealth llc acquires share of philip morris international inc pm federal judge dismisses trump bn defamation lawsuit against nyt al jazeera msft stock look set to rejoin the trillion club a microsoft get more ambitious with ai magic castle could vanish if deal isnt approved exdisney ceo lash company for bowing to trump on kimmel ap business summarybrief at pm edt ap business summarybrief at pm edt pennsylvania budget is nearly three month passed due pennsylvania budget is nearly three month passed due pennsylvania budget is nearly three month passed due pennsylvania budget is nearly three month passed due residential parking permit could be required on some city street under new proposal wall street coast toward the finish of another recordsetting week wall street coast toward the finish of another recordsetting week ap news summary at pm edt ap news summary at pm edt starbucks corporation sbux share sold by brady family wealth llc omni hire new food beverage director lapel reject planned housing development silver technical map point to bullish breakout above iconic coast restaurant with colorful story and elvis presley connection ha closed detroit city distillery open new event space proof elon musk ha trapped tesla shareholder give me trillion or i wont lie for you anymore samsung confirms it will begin showing you advertisement on your plus refrigerator screen mogy joel r investment counsel inc sell share of oracle corporation orcl medical stock to keep an eye on september th federal judge toss trump billion lawsuit against new york time at the forum nine inch nail conjure rage and dread be afraid american concord immigration judge fired a trump administration continues purge ridiculous trump admin ignites another firestorm with passport fight susan collins blast democrat for poison pill that may cause a shutdown george soros reportedly shell out million for gavin newsoms gerrymandering gambit texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor texas am president step down but doesnt say if controversial classroom video wa a factor supreme court upholds decision on cottonwood culdesac a city highway political news mecosta county want to create charlie kirk statue with public money moolenaar raise alarm on tiktok deal meet ailis mccardle russian fighter jet violate nato oil platform safety zone democratic congressional candidate get bodied by ice officer after trying to interfere with them alexandria ocasiocortez smear charlie kirk and his supporter on the house floor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor former ohio state football coach jim tressel a political rookie decides not to run for governor we still have a long road ahead preston lord stepmom speaks ahead of day honoring teen senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay senate confirms mike waltz a trump ambassador to the united nation after month of delay essex saving bank cut stake in unitedhealth group incorporated unh essex saving bank sell share of unitedhealth group incorporated unh diversified trust co ha million holding in chevron corporation cvx seacrest wealth management llc sell share of cocacola company the ko hf advisory group llc buy share of unitedhealth group incorporated unh meme coin to buy now a new forecast say k is not the top for bitcoin price robert kiyosaki blast mutual fund and etf a for loser back trump xo for alternative investment mastercard incorporated ma share sold by cx institutional cx institutional reduces stake in mastercard incorporated ma marshall sullivan inc wa make new investment in procter gamble company the pg silver oak security incorporated raise position in procter gamble company the pg cmh wealth management llc lower holding in procter gamble company the pg procter gamble company the pg share bought by weatherly asset management l p public health alert issued for a seasonal trader joes readytoeat favorite delish ap business summarybrief at pm edt ap technology summarybrief at pm edt emerging tiktok deal with china ensures u control of board and crucial algorithm white house say kaydan wealth management inc ha stake in the home depot inc hd ucloudlinks glocalme tap into u pet boom with petphone after market reentry immediate edge exploring the ai technology behind immediate edge trading platform germany insight india express concern about trump plan to hike fee on hb visa that bring tech worker to u fastselling crocs for dog are back how to get a pair th annual neighborhood market herald end of summer first tucker carlson now ted cruz conservative are talking about an unbelievably dangerous precedent being set by the fcc chair exclusive trump administration cancel annual hunger survey the wall street journal with just day of cash left remote california hospital nears crisis point harbour capital advisor llc ha million stock position in ishares russell etf iwm inside starbucks crackdown on cup note windsor capital management llc ha million position in merck co inc mrk merck co inc mrk share sold by windsor capital management llc bridge creek capital management llc ha million stock position in pepsico inc pep cx institutional ha million holding in salesforce inc crm bridge creek capital management llc ha million holding in salesforce inc crm man killed by falling jet engine identified a inventor david monroe founder of samsat woai u will complete tiktok deal in coming day and control it algorithm white house say cnn business weatherly asset management l p sell share of verizon communication inc vz adirondack trust co acquires share of vanguard total stock market etf vti weatherly asset management l p sell share of cisco system inc csco kingstone capital partner texas llc make new investment in amgen inc amgn cisco system inc csco share sold by diversified trust co diversified trust co boost stake in amgen inc amgn cm set repair deadline after firm exit threat over bluru poor road u administration attack vermont superfund law streamlined task process solana and xrp market report highlight magacoin finance a an early contender gen z is rewriting luxury can klxy and fine etf keep up college football betting promos claim s in week sportsbook offer lowincome american slash spending a worrying sign for the economy the washington post dont ignore this red flag behavior in a relationship social psychologist say it could hurt your selfesteem and sense of self underdog fantasy promo code orlive play get in site credit for oregon state v oregon cfb saturday fear dread and how america got to this point betmgm bonus code oregonmgm feature in bonus for oregon state v oregon betmgm promo code nola claim cfb bet offer sppi deadline sppi investor with loss in excess of k have opportunity to lead spectrum pharmaceutical inc security fraud lawsuit top ai token prediction for x growth ozak ai render and fetch ai sppi deadline sppi investor with loss in excess of k have opportunity to lead spectrum pharmaceutical inc security fraud lawsuit mandy steele bill mckibben and joe morinville ai crypto and pa war on the little guy the walt disney company dis share sold by essex saving bank financiere de professionnels fonds d investissement inc purchase share of costco wholesale corporation cost seacrest wealth management llc sell share of costco wholesale corporation cost diversified trust co grows stake in costco wholesale corporation cost costco wholesale corporation cost share sold by seacrest wealth management llc lowincome american slash spending a worrying sign for the economy sat sep pst yhb investment advisor inc buy share of cocacola company the ko bls silent on reason for postponing new job report after brutal august number out maine receives grant from jonathan stein fund pinnacle bancorp inc sell share of mcdonalds corporation mcd mcdonalds corporation mcd share acquired by butensky cohen financial security inc emerging tiktok deal with china ensures u control of board and crucial algorithm white house say emerging tiktok deal with china ensures u control of board and crucial algorithm white house say emerging tiktok deal with china ensures u control of board and crucial algorithm white house say kaydan wealth management inc ha million stock position in ishares core sp midcap etf ijh kaydan wealth management inc sell share of mastercard incorporated ma silver oak security incorporated purchase share of taiwan semiconductor manufacturing company ltd tsm westwind capital buy new holding in netflix inc nflx rob arnott revolutionized stock investing decade later he still disrupting the market favorite strategy top stock to buy that will likely benefit from declining interest rate top stock to buy that will likely benefit from declining interest rate ap business summarybrief at pm edt you may have never heard of this company but it stock is up over year to date why ford motor company f dividend record appeal to cheap dividend stock investor crisis at nato shipbuilder unsettles europe defense plan better fintech stock robinhood market v interactive broker cyberattack disrupts checkin system at major european airport abc news breaking news latest news and video ishares russell etf iwm share bought by william howard co financial advisor inc my legacy advisor llc invests in oracle corporation orcl bridge creek capital management llc acquires share of ge vernova inc gev cx institutional increase stock holding in ishares core sp smallcap etf ijr the home depot inc hd share sold by marshall sullivan inc wa ishares russell etf iwm stock holding boosted by william howard co financial advisor inc bdf gestion sell share of merck co inc mrk ishares core sp smallcap etf ijr share bought by cx institutional cheap dividend stock with defensive characteristic spotlight on the kraft heinz company khc cyberattack cause delay at heathrow and other airport in europe the new york time cheap dividend stock with consistent payouts where amcor amcr fit in share in pepsico inc pep purchased by kingstone capital partner texas llc weatherly asset management l p reduces stake in abbott laboratory abt yhb investment advisor inc ha stake in verizon communication inc vz weatherly asset management l p ha million position in nextera energy inc nee lantz financial llc buy share of pepsico inc pep fcc threatens abc suspends kimmel cruz warns of chilling effect on political speech cocacola company the ko share sold by seacrest wealth management llc trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact rich miller jim edgar crafted blueprint for illinois leadership trump redistricting push threatens minority representation black voter worry about it impact voice democracy rally to preserve history trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact rich miller jim edgar crafted blueprint for illinois leadership trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact federal government shutdown brinkmanship ha got to go amber gunn trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact trump redistricting push threatens minority representation black voter worry about it impact election supervisor post two town board seat being contested in lloyd after cut to food stamp trump administration end government annual report on hunger in america world tiktoks algorithm and data will be controlled by america white house say tiktoks algorithm and data will be controlled by america white house say russian jet over estonia ignored signal from nato pilot official say russian jet over estonia ignored signal from nato pilot official say colin kaepernick pay for autopsy of black student found hanging from tree pentagon demand journalist allow government to vet information bloombergcom india warns new u hb visa fee will have humanitarian consequence bbc weatherly asset management l p buy share of procter gamble company the pg rage at labour council on birmingham bin worker demo protester ice agent clash at immigrant processing site near chicago india express concern about trump plan to hike fee on hb visa that bring tech worker to u copy india express concern about trump plan to hike fee on hb visa that bring tech worker to u india express concern about trump plan to hike fee on hb visa that bring tech worker to u ap news summary at pm edt ap business summarybrief at pm edt ap business summarybrief at pm edt ap news summary at pm edt ap news summary at pm edt ap news summary at pm edt ap news summary at pm edt ap news summary at pm edt ap news summary at pm edt ap business summarybrief at pm edt ap news summary at pm edt ap news summary at pm edt ap news summary at pm edt ap news summary at pm edt ap news summary at pm edt ap news summary at pm edt ap news summary at pm edt sen alex padilla introduces redistricting measure mull political future emerging tiktok deal with china ensures u control of board and crucial algorithm white house say emerging tiktok deal with china ensures u control of board and crucial algorithm white house say emerging tiktok deal with china ensures u control of board and crucial algorithm white house say emerging tiktok deal with china ensures u control of board and crucial algorithm white house say emerging tiktok deal with china ensures u control of board and crucial algorithm white house say emerging tiktok deal with china ensures u control of board and crucial algorithm white house say emerging tiktok deal with china ensures u control of board and crucial algorithm white house say trump tap new u attorney in eastern virginia amid fallout from siebert resignation politico trump tap new u attorney in eastern virginia amid fallout from siebert resignation klobuchar grassley america cant ignore russia kidnapping ukrainian child oklahoma state fan call for mike gundy to be fired after historic loss to tulsa message of faith focused prayer in this time of crisis message of faith focused prayer in this time of crisis message of faith focused prayer in this time of crisis u roll toward a government shutdown</t>
         </is>
       </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>45923</v>
+      </c>
+      <c r="B64" t="n">
+        <v>6656.919921875</v>
+      </c>
+      <c r="C64" t="n">
+        <v>6699.52001953125</v>
+      </c>
+      <c r="D64" t="n">
+        <v>6645.580078125</v>
+      </c>
+      <c r="E64" t="n">
+        <v>6692.43994140625</v>
+      </c>
+      <c r="F64" t="n">
+        <v>5633620000</v>
+      </c>
+      <c r="G64" t="n">
+        <v>-0.0055021591970121</v>
+      </c>
+      <c r="H64" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>jpmorgan chase co cut fedex nysefdx price target to micron technology nasdaqmu price target raised to servicetitan nasdaqttan price target raised to servicetitan nasdaqttan price target raised to taiwan culture take the stage across europe with event in country europe market set for mixed open a investor ass trump visa crackdown venture firm raise million from tech leader to support new canadian business crypto price today bitcoin price drop to xrp at dogecoin fall climate goal and fossil fuel plan dont add up expert say amazon face u trial over alleged prime subscription trick wall street zen downgrade mind technology nasdaqmind to buy ctrl group nasdaqmctr downgraded to sell rating by wall street zen oculis nasdaqocs downgraded to sell rating by wall street zen fossil group nasdaqfosl downgraded to hold rating by wall street zen gossamer bio nasdaqgoss lowered to sell rating by wall street zen ichor nasdaqichr downgraded by wall street zen to sell laser photonics nasdaqlase upgraded to hold at wall street zen first western financial nasdaqmyfw downgraded to sell rating by wall street zen lite strategy nasdaqlits lowered to sell rating by wall street zen pra group announces proposed offering of million of senior note due pra group announces proposed offering of million of senior note due instagram using ai to detect canadian teen signed up for adult account warren buffett exit byd amid china cutthroat ev market south china morning post mks nasdaqmksi upgraded by wall street zen to strongbuy rating fy eps forecast for costco wholesale boosted by analyst hyundai motor up against issue price should you book profit or hold amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick amazon face u trial over alleged prime subscription trick the risk of a growing passive share in the stock market broker issue forecast for roiv q earnings cormark predicts reduced earnings for sangoma technology capital one financial forecast reduced earnings for mongodb cormark predicts reduced earnings for sangoma technology q earnings estimate for bandwidth issued by zacks research broker issue forecast for roiv q earnings atb cap market boost earnings estimate for capital power desjardins ha negative outlook of capreit fy earnings fy eps estimate for sangoma technology cut by analyst target announces biggest target circle week yet with deeper discount seasonal style member perk and exclusive product drop heineken holding nv report transaction under it current share buyback programme kaldalon hf routine announcement regarding share buyback pursuant to buyback program more than irish pension at risk of costly tax hit without urgent action pm modi interacts with arunachal trader industry leader on gst rate cut graftech international ltd nyseeaf receives average rating of hold from brokerage tpg re finance trust inc nysetrtx receives average target price from analyst trican well service ltd tsetcw given average rating of moderate buy by analyst brokerage set entain plc lonent price target at gbx brokerage set medicus pharma ltd nasdaqmdcx pt at brokerage set cytomx therapeutic inc nasdaqctmx price target at paramount group inc nysepgre receives average pt from analyst opal fuel inc nasdaqopal receives consensus rating of reduce from analyst acv auction nasdaqacva asap nasdaqwtrh headtohead comparison farmer national banc nasdaqfmnb versus huntington bancshares nasdaqhban headtohead contrast comparing braemar hotel resort nysebhr and sba communication nasdaqsbac comparing compass group otcmktscmpgy and cracker barrel old country store nasdaqcbrl xcel energy inc nasdaqxel receives consensus target price from analyst reviewing avient nyseavnt and shinetsu chemical otcmktsshecy foghorn therapeutic inc nasdaqfhtx receives average pt from brokerage sealed air corporation nysesee receives consensus target price from brokerage carvana nysecvna versus artistdirect otcmktsartd financial analysis analyst set tg therapeutic inc nasdaqtgtx pt at tesla nasdaqtsla upgraded at baird r w financial analysis great elm group nasdaqgeg citic otcmktsctpcy comparing meyer burger technology otcmktsmybuf and cslm acquisition nasdaqspwr quaker houghton nysekwr receives average target price from analyst reviewing digital ally incnv nasdaqdgly and dac technology group international otcmktsdaat analyzing fusion acquisition corp ii nysefsnb and blaize nasdaqbzai siyata mobile nasdaqsyta and liberty latin america nasdaqlila head to head contrast head to head review bright horizon family solution nysebfam v legacy education alliance otcmktsleai financial survey bank first national nasdaqbfc valley national bancorp nasdaqvly ukraine us remotecontrolled vehicle for dangerous mission to protect soldier world public disorder housing among the top issue a bcs local politician meet bc extrump white house lawyer crack dark deadpan joke about comedy purge extrump white house lawyer crack dark deadpan joke about comedy purge live israel keep pummeling gaza a support grows for palestinian state ecuador constitutional showdown amid a surge in violence venezuela military loyalty under scrutiny a rumor of highprofile desertion persist new gst reform show pm modis resolve to serve poor farmer amit shah trump speaks to reporter aboard air force one after charlie kirk memorial permapipe international nasdaqppih rating lowered to hold at wall street zen northeast bancorp nasdaqnbn raised to buy at wall street zen sanuwave health nasdaqsnwv downgraded by wall street zen to hold wall street zen upgrade urban outfitter nasdaqurbn to strongbuy national storage affiliate trust nysensa upgraded to hold at wall street zen wall street zen upgrade wisekey international nasdaqwkey to hold wall street zen downgrade zoom communication nasdaqzm to buy benton county marriage license issued sept annual celebration of woman equality day celebration held in august dear abby my husband died month ago is it too soon to start dating msp launch awareness campaign about online sexual predator alabama painter build community through art kindness former ag firm to sue gwa if action not taken on dieldrin nwa editorial fining family a they bury a loved one cemetery policing might be the height of bad timing hb what trump visa mean for india and u industry bbc sab biotherapeutics sabs buy rating reiterated at chardan capital commercial metal nysecmc price target raised to akhilesh question bjp on gst collection seek clarity on usage of money unisys nyseuis raised to buy at wall street zen masimo nasdaqmasi cut to hold at wall street zen easyjet lonezj insider buy in stock hurricane gabrielle is here alliant energy nasdaqlnt rating lowered to sell at wall street zen cemex nysecx rating lowered to hold at wall street zen kinetik nysekntk upgraded at wall street zen aar air projected to post earnings on tuesday corpay nysecpay lowered to hold rating by wall street zen ituran location and control nasdaqitrn raised to buy at wall street zen kinross gold nysekgc downgraded to buy rating by wall street zen france others to recognize palestinian state a un week get underway letter litigation against company for destroying coast justified by science letter coverage of katrina anniversary wa stellar today in historysept brazilian protest against a bill that could lead to a pardon for bolsonaro and ally brazilian protest against a bill that could lead to a pardon for bolsonaro and ally brazilian protest against a bill that could lead to a pardon for bolsonaro and ally brazilian protest against a bill that could lead to a pardon for bolsonaro and ally brazilian protest against a bill that could lead to a pardon for bolsonaro and ally brazilian protest against a bill that could lead to a pardon for bolsonaro and ally brazilian protest against a bill that could lead to a pardon for bolsonaro and ally brazilian protest against a bill that could lead to a pardon for bolsonaro and ally france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway france others to recognize palestinian state a un week get underway after charlie kirk murder conservative hope for a religious revival after charlie kirk murder young conservative are hoping for a religious revival forward air nasdaqfwrd stock rating lowered by wall street zen establishment lab nasdaqesta stock rating upgraded by wall street zen wall street zen downgrade helius medical technology nasdaqhsdt to sell innospec nasdaqiosp stock rating lowered by wall street zen un security council to on russia incursion into estonia airspace capital power tsecpx price target raised to c bandwidth nasdaqband raised to strongbuy at wall street zen autodesk nasdaqadsk upgraded to strongbuy at wall street zen foliage map and timing ahead of schedule fall color appears in new england central garden pet nasdaqcenta upgraded to strongbuy at wall street zen wall street zen downgrade consolidated water nasdaqcwco to hold trump ramp up retribution campaign with push for bondi to pursue case against foe suit against uwec end separate suit against former chancellor continues page free speech under fire again letter dont paint planned parenthood a all abou woman health ukrainian russian attack kill civilian a zelenskyy prepares to meet trump aboriginal centre welcome planning commission rejection of macquarie point sta charlie kirk friend praise slain activist faith indelible mark on conservative movement uk australia and canada recognize palestinian state prompting angry response from israel israeli strike kill more than people in gaza say health official letter why would new orleans turn down help from national guard u lawmaker push for military dialogue in a rare china visit u lawmaker push for military dialogue in a rare china visit hw electro co ltd plan million ipo for september th hwep travere therapeutic tvtx buy rating reiterated at hc wainwright boston scientific nysebsx receives buy rating from needham company llc perspective therapeutic catx buy rating reiterated at hc wainwright perrigo nyseprgo stock rating lowered by wall street zen</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>45924</v>
+      </c>
+      <c r="B65" t="n">
+        <v>6637.97021484375</v>
+      </c>
+      <c r="C65" t="n">
+        <v>6672.66015625</v>
+      </c>
+      <c r="D65" t="n">
+        <v>6621.759765625</v>
+      </c>
+      <c r="E65" t="n">
+        <v>6669.7900390625</v>
+      </c>
+      <c r="F65" t="n">
+        <v>5459180000</v>
+      </c>
+      <c r="G65" t="n">
+        <v>-0.0028466178433332</v>
+      </c>
+      <c r="H65" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>45925</v>
+      </c>
+      <c r="B66" t="n">
+        <v>6602.9501953125</v>
+      </c>
+      <c r="C66" t="n">
+        <v>6619</v>
+      </c>
+      <c r="D66" t="n">
+        <v>6569.22021484375</v>
+      </c>
+      <c r="E66" t="n">
+        <v>6608.18994140625</v>
+      </c>
+      <c r="F66" t="n">
+        <v>2387445000</v>
+      </c>
+      <c r="G66" t="n">
+        <v>-0.0052757120622413</v>
+      </c>
+      <c r="H66" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I66" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>